<commit_message>
audit(ledger): 2026-09-18 scrub — F104 fixed, F105/F106 opened BLOCKED for Dexter
103 -> 106 rows. Site clean at the HTTP, SEO, integrity and contrast layers.
F105 (High): Netlify's injected RUM beacon is refused by the site CSP on every page.
F106 (Low): the lead row's hardcoded 'This Week' label over an 18-day-old essay.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Features'!$A$3:$K$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Features'!$A$3:$K$109</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K106"/>
+  <dimension ref="A1:K109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1559,7 +1559,7 @@
       <c r="J22" s="4" t="inlineStr"/>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>PENDING | 2026-09-18: still structurally untestable — 0 upcoming entries in the committed collection.</t>
         </is>
       </c>
     </row>
@@ -1858,7 +1858,7 @@
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>PASS — 'This Month' = show-me-your-glory (same month as lead) | 2026-08-27 re-verified live: row heads 'This Week' (01, lead) and 'This Month' (02) both render as authored.</t>
+          <t>PASS — 'This Month' = show-me-your-glory (same month as lead) | 2026-08-27 re-verified live: row heads 'This Week' (01, lead) and 'This Month' (02) both render as authored. | 2026-09-18 re-verified live: 'This Month' correctly hidden — no other essay shares the lead's month (Aug 2026); row heads read 01 This Week / 02 Earlier.</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr"/>
@@ -1907,7 +1907,7 @@
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>PASS — 'Earlier' = 14, 6 visible + 8 overflow | 2026-08-27 re-verified live: 8 of 16 plates visible by default, 8 under the overflow.</t>
+          <t>PASS — 'Earlier' = 14, 6 visible + 8 overflow | 2026-08-27 re-verified live: 8 of 16 plates visible by default, 8 under the overflow. | 2026-09-18 re-verified live: 'Earlier' = 16, 6 visible + 10 under the overflow; 7 of 17 plates visible by default.</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr"/>
@@ -2013,7 +2013,7 @@
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>PASS — 16 plates tile the 12-col grid (lead + wide/secondary/banner rotation, 3 row-plates)</t>
+          <t>PASS — 16 plates tile the 12-col grid (lead + wide/secondary/banner rotation, 3 row-plates) | 2026-09-18 re-verified live: 7 visible plates tile the 12-col grid as lead + wide/secondary/banner/secondary/banner/wide; 17 plates total with the 10-plate overflow under View More.</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr"/>
@@ -2164,7 +2164,7 @@
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>PASS — manifesto form action=/api/subscribe, source=home, honeypot present | 2026-08-27 re-verified live: manifesto form + #sm-email + submit present on the homepage.</t>
+          <t>PASS — manifesto form action=/api/subscribe, source=home, honeypot present | 2026-08-27 re-verified live: manifesto form + #sm-email + submit present on the homepage. | 2026-09-18 re-verified live: manifesto form action=/api/subscribe, #sm-email present, 3 value-prop items, 'No spam' line, honeypot off-canvas (x=-9999, tabindex=-1, aria-hidden).</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr"/>
@@ -2211,9 +2211,9 @@
           <t>Cataloged</t>
         </is>
       </c>
-      <c r="H35" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="H35" s="6" t="inlineStr">
+        <is>
+          <t>PASS | 2026-09-18 re-verified live: real submit on the home manifesto form with a server-rejected address (healthscrub@invalid, passes type=email) showed 'Sending…', then state=error with 'That email didn't look right. Try it again.' in a role=alert .sm-error and the button re-enabled. Success path covered by the §9 API smoke (200 subscribed); the UI success state was not driven to avoid a second subscriber write.</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr"/>
@@ -2629,7 +2629,7 @@
       </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
-          <t>PASS — form posts /api/subscribe with source=article, honeypot off-canvas, aria-live label; server states verified directly against the function</t>
+          <t>PASS — form posts /api/subscribe with source=article, honeypot off-canvas, aria-live label; server states verified directly against the function | 2026-09-18 re-verified live: server-rejected address on /words/gumbo/ surfaced 'That email didn’t look right. Try it again.' in the role=status aria-live label and kept the form — it reflects the server failure rather than a blanket success. source=article, honeypot off-canvas at x=-4972.</t>
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr"/>
@@ -2693,7 +2693,7 @@
       </c>
       <c r="K44" s="6" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>PENDING | 2026-09-18: still structurally untestable — 0 upcoming entries in the committed collection.</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2954,7 @@
       </c>
       <c r="K49" s="6" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>PENDING | 2026-09-18: still structurally untestable — 0 upcoming entries in the committed collection.</t>
         </is>
       </c>
     </row>
@@ -3787,7 +3787,7 @@
       </c>
       <c r="H65" s="6" t="inlineStr">
         <is>
-          <t>PASS — documented error envelope returned, no stack leakage</t>
+          <t>PASS — documented error envelope returned, no stack leakage | 2026-09-18 re-verified live: POST email=not-an-email returns 400 {"ok":false,"error":"invalid_email"} with Cache-Control: no-store, no stack leakage. Config/upstream branches not forceable from outside (would need env or Mailchimp changes); subscribe.cjs unchanged since last PASS.</t>
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr"/>
@@ -4317,7 +4317,7 @@
       </c>
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>PASS — predicate gates homepage/feed/sitemap/routes consistently; 16 published, 0 upcoming</t>
+          <t>PASS — predicate gates homepage/feed/sitemap/routes consistently; 16 published, 0 upcoming | 2026-09-18 re-verified live: 17 published, 0 upcoming — homepage 17 plates, feed 17 entries, sitemap 17 /words/ URLs, all consistent. (An untracked drafted entry sits in the working tree and is correctly nowhere live.)</t>
         </is>
       </c>
       <c r="I75" s="6" t="inlineStr"/>
@@ -4385,7 +4385,7 @@
       </c>
       <c r="K76" s="6" t="inlineStr">
         <is>
-          <t>PENDING — BLOCKED, tracked daily. Ten consecutive late-but-successful runs (2026-08-27..2026-09-05), drift narrowing from +11h36m at its worst to +3h13m today. No missed days. Not auto-fixable: the remedy is a scheduling change outside the repo. | 2026-09-06: eleven consecutive late-but-successful runs (2026-08-27..2026-09-06). Still not auto-fixable from the repo. | 2026-09-11: still BLOCKED and still not auto-fixable from the repo — the YAML is correct and the lateness is GitHub's scheduler. Deploy freshness is unaffected: the Netlify deploy that ran off it (6aa3cac) carries commit_ref 507e988, which is GitHub main HEAD.</t>
+          <t>PENDING — BLOCKED, tracked daily. Ten consecutive late-but-successful runs (2026-08-27..2026-09-05), drift narrowing from +11h36m at its worst to +3h13m today. No missed days. Not auto-fixable: the remedy is a scheduling change outside the repo. | 2026-09-06: eleven consecutive late-but-successful runs (2026-08-27..2026-09-06). Still not auto-fixable from the repo. | 2026-09-11: still BLOCKED and still not auto-fixable from the repo — the YAML is correct and the lateness is GitHub's scheduler. Deploy freshness is unaffected: the Netlify deploy that ran off it (6aa3cac) carries commit_ref 507e988, which is GitHub main HEAD. | 2026-09-18: still BLOCKED, still not auto-fixable from the repo. Seven more late-but-successful scheduled runs 2026-09-12..09-18 against the 05:05Z cron, firing 09:12Z–10:31Z (+4h07m to +5h26m). No missed days. Deploy freshness unaffected: the 2026-09-18 09:37Z hook deploy (6aad063) carries commit_ref 507e988 = GitHub main HEAD.</t>
         </is>
       </c>
     </row>
@@ -4802,7 +4802,7 @@
       </c>
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: show-me-your-glory emits rel=next to send-someone-else and renders a normal (non-ghost) forward nav; forward chain walks all 16 published essays end to end. | 2026-08-25 re-verified live: forward chain walks all 16 published essays end to end; the chronologically newest (send-someone-else) correctly carries no next.</t>
+          <t>PASS — live-verified 2026-08-10: show-me-your-glory emits rel=next to send-someone-else and renders a normal (non-ghost) forward nav; forward chain walks all 16 published essays end to end. | 2026-08-25 re-verified live: forward chain walks all 16 published essays end to end; the chronologically newest (send-someone-else) correctly carries no next. | 2026-09-18 re-verified live: forward chain walks all 17 published essays end to end, reckonings → the-weight-of-my-no; only the newest lacks rel=next and only the oldest lacks rel=prev.</t>
         </is>
       </c>
       <c r="I84" s="6" t="inlineStr"/>
@@ -4912,7 +4912,7 @@
       </c>
       <c r="H86" s="6" t="inlineStr">
         <is>
-          <t>PASS (closed live 2026-08-13) — was ISSUE/High (2026-08-13) — CORRECTED SCOPE, and the correction matters. The morning scrub read the declarations and reported FOUR failing hover rules. Re-measured under REAL pointer hover before fixing, only TWO are real: `.issue-latest:hover .latest-cta` (14.08px/700) and `.identity-hero .hero-link.primary:hover` (14.08px/700), both `color: var(--bg)` on a `background: var(--accent)` fill = 3.44:1 in dark against a 4.5:1 floor. The other two were FALSE POSITIVES: `.issue-latest:hover` takes the BAR to var(--ink), not var(--accent), so .latest-title measures 17.79:1 and .latest-meta 5.23:1 (at opacity .6) against cream — both already clear. The morning read assumed the accent fill was the surface for every child of the hover state; it is only the surface for .latest-cta, which sets its own background. Lesson: resolve the PAINTED surface under real hover, never infer it from the parent's declarations. | 2026-08-25 re-verified live: re-verified under REAL pointer hover on the live homepage in dark mode: .latest-cta 5.17:1, .latest-tag 5.17:1, .latest-title 17.79:1, .latest-meta (hover state) 5.23:1. No regression. Caveat carried to F87: the override lives in home-v2.css on the live deploy, so /brand/ still does not get it.</t>
+          <t>PASS (closed live 2026-08-13) — was ISSUE/High (2026-08-13) — CORRECTED SCOPE, and the correction matters. The morning scrub read the declarations and reported FOUR failing hover rules. Re-measured under REAL pointer hover before fixing, only TWO are real: `.issue-latest:hover .latest-cta` (14.08px/700) and `.identity-hero .hero-link.primary:hover` (14.08px/700), both `color: var(--bg)` on a `background: var(--accent)` fill = 3.44:1 in dark against a 4.5:1 floor. The other two were FALSE POSITIVES: `.issue-latest:hover` takes the BAR to var(--ink), not var(--accent), so .latest-title measures 17.79:1 and .latest-meta 5.23:1 (at opacity .6) against cream — both already clear. The morning read assumed the accent fill was the surface for every child of the hover state; it is only the surface for .latest-cta, which sets its own background. Lesson: resolve the PAINTED surface under real hover, never infer it from the parent's declarations. | 2026-08-25 re-verified live: re-verified under REAL pointer hover on the live homepage in dark mode: .latest-cta 5.17:1, .latest-tag 5.17:1, .latest-title 17.79:1, .latest-meta (hover state) 5.23:1. No regression. Caveat carried to F87: the override lives in home-v2.css on the live deploy, so /brand/ still does not get it. | 2026-09-18 re-verified live: dark mode under REAL pointer hover: .latest-cta 'Read →' and .hero-link.primary 'Read the About →' both cream 243,240,232 on #c00 = 5.17:1 at 14.08px.</t>
         </is>
       </c>
       <c r="I86" s="6" t="inlineStr">
@@ -6055,8 +6055,179 @@
         </is>
       </c>
     </row>
+    <row r="107">
+      <c r="A107" s="4" t="inlineStr">
+        <is>
+          <t>F104</t>
+        </is>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>Build / Automation</t>
+        </is>
+      </c>
+      <c r="C107" s="4" t="inlineStr">
+        <is>
+          <t>QA OS operating prompt — §3 accent check names two surfaces that are not accent by design</t>
+        </is>
+      </c>
+      <c r="D107" s="4" t="inlineStr">
+        <is>
+          <t>As the loop reading audit/QA-OS.md, I want the design-system check to name only surfaces that actually carry --accent, so it cannot either be silently skipped or raise a false drift finding against a deliberate design decision.</t>
+        </is>
+      </c>
+      <c r="E107" s="4" t="inlineStr">
+        <is>
+          <t>§3 DESIGN SYSTEM COMPLIANCE names the accent's real homes (section-head h2, .callout left border per DESIGN-SYSTEM.md §4) and records the reading-progress bar (--ink) and pull-quote borders (--border) as by-design.</t>
+        </is>
+      </c>
+      <c r="F107" s="4" t="inlineStr">
+        <is>
+          <t>audit/QA-OS.md:171; css/article.css:170-176,194-198,873-882; DESIGN-SYSTEM.md §4 Border Language</t>
+        </is>
+      </c>
+      <c r="G107" s="5" t="inlineStr">
+        <is>
+          <t>Cataloged</t>
+        </is>
+      </c>
+      <c r="H107" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE/Low (2026-09-18) — §3 read 'Verify `--accent` usage on section-head h2, reading-progress bars, pull-quote borders.' Measured live on /words/the-weight-of-my-no/ in dark mode: `.reading-progress` background rgb(243,240,232) (--ink) and `.pull-quote` borders rgba(243,240,232,.82) (--border). Both are deliberate: the progress bar was recoloured from --accent to --ink in 68b0c1d (2026-04-10) with a comment at css/article.css:873 explaining the red bar competed with the masthead, and DESIGN-SYSTEM.md §4 lists pull-quote top/bottom borders as ordinary content borders while naming the .callout left border as the accent one. The check predates nothing — QA-OS was written 2026-08-07, four months after the recolour — so it has been either silently skipped or passed on assumption every run. Same class as F103: a dead check in the operating prompt. Graded Low: no site surface affected.</t>
+        </is>
+      </c>
+      <c r="I107" s="6" t="inlineStr">
+        <is>
+          <t>Low (fixed)</t>
+        </is>
+      </c>
+      <c r="J107" s="4" t="inlineStr">
+        <is>
+          <t>FIX (qa/fixes-20260918): §3 line restated to check --accent on section-head h2 and the .callout left border, with the progress bar and pull-quote borders recorded as by-design (68b0c1d, css/article.css:873) and a do-not-re-add note. Doc-only; no site source touched.</t>
+        </is>
+      </c>
+      <c r="K107" s="6" t="inlineStr">
+        <is>
+          <t>PASS — 2026-09-18. Re-read after the edit: the only remaining 'reading-progress' mentions in QA-OS.md are this by-design note and the scroll-harness antipattern. Restated check dry-run live: section-head h2 computes rgb(255,77,77) (--accent-text, dark) and .callout border-left uses var(--accent) (css/article.css:198). `npm run build` passes (20 pages); audit/ is not part of the build.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="4" t="inlineStr">
+        <is>
+          <t>F105</t>
+        </is>
+      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>Global / Shell</t>
+        </is>
+      </c>
+      <c r="C108" s="4" t="inlineStr">
+        <is>
+          <t>Netlify-injected RUM beacon blocked by the site CSP on every page</t>
+        </is>
+      </c>
+      <c r="D108" s="4" t="inlineStr">
+        <is>
+          <t>As a reader, I want pages to load without script errors; as the site owner, I want any analytics I have switched on to actually report, or to be switched off.</t>
+        </is>
+      </c>
+      <c r="E108" s="4" t="inlineStr">
+        <is>
+          <t>No console errors on page load or unload. Either Netlify Real User Monitoring is off for this site, or the CSP connect-src allows its collector. The two must not disagree.</t>
+        </is>
+      </c>
+      <c r="F108" s="4" t="inlineStr">
+        <is>
+          <t>netlify.toml:51-52,76,93,99 (connect-src 'self'); Netlify-injected &lt;script id=netlify-rum-container src=/.netlify/scripts/rum&gt; (not in repo)</t>
+        </is>
+      </c>
+      <c r="G108" s="5" t="inlineStr">
+        <is>
+          <t>Cataloged</t>
+        </is>
+      </c>
+      <c r="H108" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE/High (2026-09-18) — every page (/, /about/, /brand/, /phase0/, /404, all /words/) carries a Netlify-injected `&lt;script async id="netlify-rum-container" src="/.netlify/scripts/rum"&gt;` with a CWV token for deploy 6aad063. The script beacons to https://ingesteer.services-prod.nsvcs.net/rum_collection, which the site's own CSP (`connect-src 'self'`, commented in netlify.toml as 'no analytics/beacons allowed') refuses. Result, reproduced on the homepage and on /words/the-weight-of-my-no/: two CSP violation errors plus an 'Uncaught (in promise) TypeError: Failed to fetch' from /.netlify/scripts/rum:1:11100. No reader-visible breakage — but it is a console error on every page view, and whatever Netlify observability panel this feeds is receiving nothing. The script was already present on 2026-09-11 (F102's p4 notes it in the live-vs-dist diff) while that run logged zero console errors, so either the beacon only fires on page hide / navigation (consistent with it arriving on navigate here) or the collector moved off-origin since; NEW to the ledger either way. Graded HIGH per the console-error rule.</t>
+        </is>
+      </c>
+      <c r="I108" s="6" t="inlineStr">
+        <is>
+          <t>HIGH (blocked — Netlify dashboard / CSP intent)</t>
+        </is>
+      </c>
+      <c r="J108" s="4" t="inlineStr">
+        <is>
+          <t>BLOCKED — NEEDS DEXTER. Not in the repo: the script is injected at the edge by a Netlify site setting. The two fixes both belong to Dexter: (a) if Netlify RUM / Observability was switched on by accident or is not wanted, turn it off in the Netlify dashboard for site ff389de6 — no code change, and the CSP's 'no beacons' intent stands; (b) if the data is wanted, add https://ingesteer.services-prod.nsvcs.net to connect-src in all four CSP blocks of netlify.toml — a deliberate relaxation of a stated security posture, so not the loop's call. (a) is the change that matches the CSP comment as written.</t>
+        </is>
+      </c>
+      <c r="K108" s="6" t="inlineStr">
+        <is>
+          <t>PENDING — BLOCKED (2026-09-18). Re-verify on the next SCRUB after Dexter picks (a) or (b).</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="4" t="inlineStr">
+        <is>
+          <t>F106</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>Homepage</t>
+        </is>
+      </c>
+      <c r="C109" s="4" t="inlineStr">
+        <is>
+          <t>Lead row head reads 'This Week' regardless of the lead essay's age</t>
+        </is>
+      </c>
+      <c r="D109" s="4" t="inlineStr">
+        <is>
+          <t>As a reader landing on the homepage, I want the section labels to tell me the truth about recency, so 'This Week' means this week.</t>
+        </is>
+      </c>
+      <c r="E109" s="4" t="inlineStr">
+        <is>
+          <t>The lead row's label is accurate on the day it is read, or is worded so it cannot go stale between essays.</t>
+        </is>
+      </c>
+      <c r="F109" s="4" t="inlineStr">
+        <is>
+          <t>src/pages/index.astro:205 (label="This Week" hardcoded); DESIGN-SYSTEM.md:747</t>
+        </is>
+      </c>
+      <c r="G109" s="5" t="inlineStr">
+        <is>
+          <t>Cataloged</t>
+        </is>
+      </c>
+      <c r="H109" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE/Low (2026-09-18) — index.astro:205 renders `&lt;RowHead label="This Week" variant="lead" /&gt;` unconditionally for the newest published essay; nothing compares the lead's publishedDate to the build date. Live today (Fri 2026-09-18) the row reads '01 This Week' over The Weight of My No, published 2026-08-31 — 18 days old. It read the same over Send Someone Else through most of August, when that essay was up to 57 days old. The daily rebuild (F73) would make a date-derived label accurate every morning at no cost. Filed Low: nothing breaks and it is not an a11y or SEO defect, but it is a false recency claim in the most prominent label on the page.</t>
+        </is>
+      </c>
+      <c r="I109" s="6" t="inlineStr">
+        <is>
+          <t>Low (blocked — copy/design intent)</t>
+        </is>
+      </c>
+      <c r="J109" s="4" t="inlineStr">
+        <is>
+          <t>BLOCKED — NEEDS DEXTER. This is label copy inside a named design element (DESIGN-SYSTEM.md places the ghost row 'above `This Week`'), so wording is Dexter's call, not the loop's. Options: (a) keep as is, accepting it as an editorial name for the lead slot rather than a date claim; (b) a neutral label that cannot go stale ('Latest'); (c) derive it at build time — 'This Week' when the lead is &lt;=7 days old, else 'Latest' — which the daily rebuild keeps fresh. (c) is a ~5-line change in index.astro once the wording is chosen.</t>
+        </is>
+      </c>
+      <c r="K109" s="6" t="inlineStr">
+        <is>
+          <t>PENDING — BLOCKED (2026-09-18).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:K106"/>
+  <autoFilter ref="A3:K109"/>
   <mergeCells count="2">
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A1:K1"/>
@@ -6136,7 +6307,7 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10">
@@ -6156,7 +6327,7 @@
         </is>
       </c>
       <c r="B11" s="11" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
@@ -6173,7 +6344,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16">
@@ -6183,13 +6354,13 @@
         </is>
       </c>
       <c r="B16" s="14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Total features: 103</t>
+          <t>Total features: 106</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
audit(ledger): F105/F106 closed on Dexter's decisions, build-verified
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -6155,17 +6155,17 @@
       </c>
       <c r="I108" s="6" t="inlineStr">
         <is>
-          <t>HIGH (blocked — Netlify dashboard / CSP intent)</t>
+          <t>HIGH (fixed — Dexter chose (b))</t>
         </is>
       </c>
       <c r="J108" s="4" t="inlineStr">
         <is>
-          <t>BLOCKED — NEEDS DEXTER. Not in the repo: the script is injected at the edge by a Netlify site setting. The two fixes both belong to Dexter: (a) if Netlify RUM / Observability was switched on by accident or is not wanted, turn it off in the Netlify dashboard for site ff389de6 — no code change, and the CSP's 'no beacons' intent stands; (b) if the data is wanted, add https://ingesteer.services-prod.nsvcs.net to connect-src in all four CSP blocks of netlify.toml — a deliberate relaxation of a stated security posture, so not the loop's call. (a) is the change that matches the CSP comment as written.</t>
+          <t>BLOCKED — NEEDS DEXTER. Not in the repo: the script is injected at the edge by a Netlify site setting. The two fixes both belong to Dexter: (a) if Netlify RUM / Observability was switched on by accident or is not wanted, turn it off in the Netlify dashboard for site ff389de6 — no code change, and the CSP's 'no beacons' intent stands; (b) if the data is wanted, add https://ingesteer.services-prod.nsvcs.net to connect-src in all four CSP blocks of netlify.toml — a deliberate relaxation of a stated security posture, so not the loop's call. (a) is the change that matches the CSP comment as written. | 2026-09-18 DECISION (Dexter): keep the data. FIX (qa/fixes-20260918): https://ingesteer.services-prod.nsvcs.net added to connect-src in all four CSP blocks of netlify.toml (global + the three per-route overrides), header comment rewritten to record the opt-in; DESIGN-SYSTEM.md §11.5 CSP listing and prose updated to name it as the single allowed beacon. That host is the only URL in /.netlify/scripts/rum (11,141 bytes, same-origin, so script-src 'self' already covers the script itself).</t>
         </is>
       </c>
       <c r="K108" s="6" t="inlineStr">
         <is>
-          <t>PENDING — BLOCKED (2026-09-18). Re-verify on the next SCRUB after Dexter picks (a) or (b).</t>
+          <t>PASS (verified against build) — 2026-09-18. `npm run build` passes (20 pages). All four connect-src values now read `'self' https://ingesteer.services-prod.nsvcs.net`; no other directive changed. Live verification needs the deploy: next SCRUB after merge should show zero console errors on page hide/navigation, and Netlify's RUM panel should start receiving data.</t>
         </is>
       </c>
     </row>
@@ -6212,17 +6212,17 @@
       </c>
       <c r="I109" s="6" t="inlineStr">
         <is>
-          <t>Low (blocked — copy/design intent)</t>
+          <t>Low (fixed — Dexter chose (b))</t>
         </is>
       </c>
       <c r="J109" s="4" t="inlineStr">
         <is>
-          <t>BLOCKED — NEEDS DEXTER. This is label copy inside a named design element (DESIGN-SYSTEM.md places the ghost row 'above `This Week`'), so wording is Dexter's call, not the loop's. Options: (a) keep as is, accepting it as an editorial name for the lead slot rather than a date claim; (b) a neutral label that cannot go stale ('Latest'); (c) derive it at build time — 'This Week' when the lead is &lt;=7 days old, else 'Latest' — which the daily rebuild keeps fresh. (c) is a ~5-line change in index.astro once the wording is chosen.</t>
+          <t>BLOCKED — NEEDS DEXTER. This is label copy inside a named design element (DESIGN-SYSTEM.md places the ghost row 'above `This Week`'), so wording is Dexter's call, not the loop's. Options: (a) keep as is, accepting it as an editorial name for the lead slot rather than a date claim; (b) a neutral label that cannot go stale ('Latest'); (c) derive it at build time — 'This Week' when the lead is &lt;=7 days old, else 'Latest' — which the daily rebuild keeps fresh. (c) is a ~5-line change in index.astro once the wording is chosen. | 2026-09-18 DECISION (Dexter): 'Latest'. FIX (qa/fixes-20260918): src/pages/index.astro:205 label "This Week" → "Latest"; DESIGN-SYSTEM.md:747 'above `This Week`' → 'above `Latest`'. The internal rowNum key 'thisWeek' is left as is (not rendered).</t>
         </is>
       </c>
       <c r="K109" s="6" t="inlineStr">
         <is>
-          <t>PENDING — BLOCKED (2026-09-18).</t>
+          <t>PASS (verified against build) — 2026-09-18. dist/index.html row heads read '01 Latest' / '02 Earlier'; 'This Week' appears nowhere in src/, css/, js/ or the build. Goes live-verified on the next SCRUB after merge.</t>
         </is>
       </c>
     </row>
@@ -6307,7 +6307,7 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10">
@@ -6327,7 +6327,7 @@
         </is>
       </c>
       <c r="B11" s="11" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
@@ -6344,7 +6344,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16">
@@ -6354,7 +6354,7 @@
         </is>
       </c>
       <c r="B16" s="14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
audit(ledger): 2026-09-19 scrub — clean site, F105/F106 still await the 09-18 merge
Scrub + report only; zero new FAIL/ISSUE rows. Rotation F02 F07 F34 F39 F47
F48 F49 F52 F53 F54 PASS. F19/F41/F46 still PENDING (no upcoming entry).
F73 late-but-successful again (09:23:59Z).

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -687,7 +687,7 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>PASS — brand-word: Words (home/article/about/brand), 404, Phase 0 — matches documented intent | 2026-08-15 re-verified live: brand-word: home/about/article 'Words', 404 '404', phase0 'Phase 0' — matches the documented about-page quirk | 2026-08-25 re-verified live: brand-word: "Words" on home/about/article, "404" on /404, "Phase 0" on /phase0/ — matches documented intent. | 2026-08-27 re-verified live: brand word 'Words' confirmed on home/article/about. | 2026-09-01 re-verified live on the homepage: masthead brand word reads 'Words' (documented intent). Other surfaces not re-walked this run.</t>
+          <t>PASS — brand-word: Words (home/article/about/brand), 404, Phase 0 — matches documented intent | 2026-08-15 re-verified live: brand-word: home/about/article 'Words', 404 '404', phase0 'Phase 0' — matches the documented about-page quirk | 2026-08-25 re-verified live: brand-word: "Words" on home/about/article, "404" on /404, "Phase 0" on /phase0/ — matches documented intent. | 2026-08-27 re-verified live: brand word 'Words' confirmed on home/article/about. | 2026-09-01 re-verified live on the homepage: masthead brand word reads 'Words' (documented intent). Other surfaces not re-walked this run. | 2026-09-19 re-verified live: brand-word live: 'Words' on /, /about/, /brand/ and all 17 articles; 'Phase 0' on /phase0/; '404' on the unmatched-route 404 — matches documented intent.</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr"/>
@@ -797,7 +797,7 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: skip link is first focusable; activating it lands document.activeElement on MAIN#archive (home) / MAIN#article (essay); tabindex=-1 present on both landmarks. The 2c7d88d fix holds in production. | 2026-08-13 re-verified live: tab-target verified on live: .skip-link reveals from left:-999px to a 83x69 box at (12,12), cream-on-ink 17.79:1; activating it moved document.activeElement to MAIN#archive (tabindex=-1). Article pages target #article. | 2026-08-16 re-verified live: structural half re-verified live: .skip-link is the first focusable element in document order on every page type, and its target (MAIN#article / MAIN#archive / MAIN#phase0 / MAIN#main) carries tabindex=-1. End-to-end activation NOT re-exercisable this run — the browser pane reports document.visibilityState 'hidden' and drops page focus on every reload, so a fresh-load Tab lands on BODY. Harness limitation, not a site regression; last live activation was 2026-08-13. NOTE: this row's sweep is what surfaced F91 — see that row. | 2026-08-25 re-verified live: verified end-to-end live under REAL keyboard input on /words/the-stone/ — the gap the 2026-08-16 run had to leave open. .skip-link is the first focusable in DOM order, reveals from left:-999px to a 126x46 chip at (12,12), computes 17.79:1 (#060606 on #f3f0e8), and pressing Enter sets location.hash to #article and moves document.activeElement to MAIN#article (tabindex=-1). | 2026-08-27 re-verified live: skip link is the first focusable (reached by real shift+Tab from .brand-block), renders as an opaque cream chip at 17.79:1, and activation moves focus to MAIN#archive with hash #archive. | 2026-09-01 re-verified live: .skip-link is the FIRST Tab stop from page load and matches :focus-visible; activation moves location.hash to #archive and focus to MAIN#archive. Ran the ordinary-link control first per the harness antipattern. | 2026-09-06 re-verified live: skip link is the first focusable, unhides on focus (left -999px -&gt; 12px), and activation moved location.hash to '#archive' and focus to the #archive element. | 2026-09-11 re-verified live: skip link is the first focusable (reached by one shift+Tab back from .brand-block), 17.79:1, #c00 2px ring; activated with a real pointer click → document.activeElement === main#archive, location.hash '#archive'.</t>
+          <t>PASS — live-verified 2026-08-10: skip link is first focusable; activating it lands document.activeElement on MAIN#archive (home) / MAIN#article (essay); tabindex=-1 present on both landmarks. The 2c7d88d fix holds in production. | 2026-08-13 re-verified live: tab-target verified on live: .skip-link reveals from left:-999px to a 83x69 box at (12,12), cream-on-ink 17.79:1; activating it moved document.activeElement to MAIN#archive (tabindex=-1). Article pages target #article. | 2026-08-16 re-verified live: structural half re-verified live: .skip-link is the first focusable element in document order on every page type, and its target (MAIN#article / MAIN#archive / MAIN#phase0 / MAIN#main) carries tabindex=-1. End-to-end activation NOT re-exercisable this run — the browser pane reports document.visibilityState 'hidden' and drops page focus on every reload, so a fresh-load Tab lands on BODY. Harness limitation, not a site regression; last live activation was 2026-08-13. NOTE: this row's sweep is what surfaced F91 — see that row. | 2026-08-25 re-verified live: verified end-to-end live under REAL keyboard input on /words/the-stone/ — the gap the 2026-08-16 run had to leave open. .skip-link is the first focusable in DOM order, reveals from left:-999px to a 126x46 chip at (12,12), computes 17.79:1 (#060606 on #f3f0e8), and pressing Enter sets location.hash to #article and moves document.activeElement to MAIN#article (tabindex=-1). | 2026-08-27 re-verified live: skip link is the first focusable (reached by real shift+Tab from .brand-block), renders as an opaque cream chip at 17.79:1, and activation moves focus to MAIN#archive with hash #archive. | 2026-09-01 re-verified live: .skip-link is the FIRST Tab stop from page load and matches :focus-visible; activation moves location.hash to #archive and focus to MAIN#archive. Ran the ordinary-link control first per the harness antipattern. | 2026-09-06 re-verified live: skip link is the first focusable, unhides on focus (left -999px -&gt; 12px), and activation moved location.hash to '#archive' and focus to the #archive element. | 2026-09-11 re-verified live: skip link is the first focusable (reached by one shift+Tab back from .brand-block), 17.79:1, #c00 2px ring; activated with a real pointer click → document.activeElement === main#archive, location.hash '#archive'. | 2026-09-19 re-verified live: skip link reached under a real shift+Tab on the homepage (:focus-visible true, #060606 on cream chip, rgb(204,0,0) 2px ring); activation moves focus to #archive (tabindex -1) and sets location.hash.</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr"/>
@@ -948,7 +948,7 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>PASS (2026-08-15 scrub) — home/about/phase0/articles all carry the feed discovery link; /404 correctly omits it. NOTE: the prior `expected` said articles do NOT include it. That text was stale — ArticleLayout has emitted the link since a4f4f25; the site was never wrong, the row was. Expectation corrected, not the code. | 2026-08-25 re-verified live: &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present in head. | 2026-09-01 re-verified live: &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present in head; /feed.xml 200.</t>
+          <t>PASS (2026-08-15 scrub) — home/about/phase0/articles all carry the feed discovery link; /404 correctly omits it. NOTE: the prior `expected` said articles do NOT include it. That text was stale — ArticleLayout has emitted the link since a4f4f25; the site was never wrong, the row was. Expectation corrected, not the code. | 2026-08-25 re-verified live: &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present in head. | 2026-09-01 re-verified live: &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present in head; /feed.xml 200. | 2026-09-19 re-verified live: feed discovery &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present on /, /about/, /phase0/, /brand/ and all 17 articles; absent on the 404 as specified.</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr"/>
@@ -1552,7 +1552,7 @@
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>404 half PASS (noindex,nofollow live). Coming-soon half PENDING — no upcoming entry exists to render one | 2026-08-25: 404 half re-verified live (meta robots noindex,nofollow present, bespoke body served at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one. | 2026-09-01 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one. | 2026-09-11: 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body at HTTP 200). Coming-soon half still PENDING — 17 published entries, all past-dated, so isUpcomingData() is false everywhere and no ComingSoonLayout renders.</t>
+          <t>404 half PASS (noindex,nofollow live). Coming-soon half PENDING — no upcoming entry exists to render one | 2026-08-25: 404 half re-verified live (meta robots noindex,nofollow present, bespoke body served at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one. | 2026-09-01 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one. | 2026-09-11: 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body at HTTP 200). Coming-soon half still PENDING — 17 published entries, all past-dated, so isUpcomingData() is false everywhere and no ComingSoonLayout renders. | 2026-09-19: 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body, HTTP 404 on unmatched route). Coming-soon half still PENDING — 17 published entries, all past-dated; the untracked before-i-had-the-words.mdx in Dexter's working tree is still status 'drafted'.</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr"/>
@@ -2319,7 +2319,7 @@
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>PASS — all 16 MDX bodies render through [...slug].astro | 2026-08-27 re-verified live: all 16 MDX bodies render.</t>
+          <t>PASS — all 16 MDX bodies render through [...slug].astro | 2026-08-27 re-verified live: all 16 MDX bodies render. | 2026-09-19 re-verified live: all 17 live articles render an .article-body (shortest body ~6.4k chars of text).</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr"/>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>PASS — Follow Me → instagram.com/ImJustDex | 2026-08-27 re-verified live: Follow Me → instagram.com/ImJustDex, 200.</t>
+          <t>PASS — Follow Me → instagram.com/ImJustDex | 2026-08-27 re-verified live: Follow Me → instagram.com/ImJustDex, 200. | 2026-09-19 re-verified live: Follow Me → instagram.com/ImJustDex with target=_blank rel='noopener noreferrer' on 17/17 articles and on /about/.</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr"/>
@@ -2682,7 +2682,7 @@
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
-          <t>Authored prev/next render correctly on all 16. Ghost/teaser path PENDING — requires a future-dated entry; none exists. 2026-08-10 PM: the derive-from-live-status fix (p3) live-verified, then the underlying data cleaned — the 4 stale ghost:true flags are gone (see F81). Zero `ghost: true` remain in the collection; all 16 essays render real .article-nav-link anchors, 15 rel=next head links (newest correctly has none), zero article-nav-ghost teasers. | 2026-08-25 re-verified live: all 16 essays render real .article-nav-link anchors; zero `ghost: true` remain in the collection. Ghost/teaser path still PENDING — still requires a future-dated entry and none exists. | 2026-09-11: authored prev/next re-verified live — newest essay emits rel=prev only, /words/the-stone/ emits rel=prev + rel=next. Ghost/teaser path still PENDING; zero upcoming entries in the collection.</t>
+          <t>Authored prev/next render correctly on all 16. Ghost/teaser path PENDING — requires a future-dated entry; none exists. 2026-08-10 PM: the derive-from-live-status fix (p3) live-verified, then the underlying data cleaned — the 4 stale ghost:true flags are gone (see F81). Zero `ghost: true` remain in the collection; all 16 essays render real .article-nav-link anchors, 15 rel=next head links (newest correctly has none), zero article-nav-ghost teasers. | 2026-08-25 re-verified live: all 16 essays render real .article-nav-link anchors; zero `ghost: true` remain in the collection. Ghost/teaser path still PENDING — still requires a future-dated entry and none exists. | 2026-09-11: authored prev/next re-verified live — newest essay emits rel=prev only, /words/the-stone/ emits rel=prev + rel=next. Ghost/teaser path still PENDING; zero upcoming entries in the collection. | 2026-09-19: authored prev/next unchanged (no code churn since 507e988). Ghost/teaser path still PENDING — zero upcoming entries in the collection.</t>
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr"/>
@@ -2943,7 +2943,7 @@
       </c>
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>PENDING — all 16 entries are status published with past dates, so isUpcomingData() is false everywhere and no coming-soon page renders | 2026-08-25: still PENDING for the same structural reason — all 16 built entries are status:published with past dates. NOTE: an untracked draft (src/content/words/before-i-had-the-words.mdx, status:"drafted", publishedDate 2026-08-07) sits in Dexter's working tree. It is correctly excluded from the build (19 pages, 16 articles) and does not exercise this path either, since its date is in the past, not the future. | 2026-09-01 still PENDING. The untracked draft in Dexter's working tree (src/content/words/before-i-had-the-words.mdx, status 'drafted', publishedDate 2026-08-07) is correctly excluded from the build (20 pages, 17 articles) but does NOT exercise this path — its date is in the past and its status is 'drafted', not an upcoming publish. Left untouched. | 2026-09-11: still PENDING for the same structural reason — 17 published entries, all past-dated. The untracked draft src/content/words/before-i-had-the-words.mdx is still status 'drafted' in Dexter's working tree, so it builds nothing and is correctly absent from sitemap and feed.</t>
+          <t>PENDING — all 16 entries are status published with past dates, so isUpcomingData() is false everywhere and no coming-soon page renders | 2026-08-25: still PENDING for the same structural reason — all 16 built entries are status:published with past dates. NOTE: an untracked draft (src/content/words/before-i-had-the-words.mdx, status:"drafted", publishedDate 2026-08-07) sits in Dexter's working tree. It is correctly excluded from the build (19 pages, 16 articles) and does not exercise this path either, since its date is in the past, not the future. | 2026-09-01 still PENDING. The untracked draft in Dexter's working tree (src/content/words/before-i-had-the-words.mdx, status 'drafted', publishedDate 2026-08-07) is correctly excluded from the build (20 pages, 17 articles) but does NOT exercise this path — its date is in the past and its status is 'drafted', not an upcoming publish. Left untouched. | 2026-09-11: still PENDING for the same structural reason — 17 published entries, all past-dated. The untracked draft src/content/words/before-i-had-the-words.mdx is still status 'drafted' in Dexter's working tree, so it builds nothing and is correctly absent from sitemap and feed. | 2026-09-19: still PENDING for the same structural reason — no upcoming entry; the untracked draft is still 'drafted' and builds nothing.</t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr"/>
@@ -2996,7 +2996,7 @@
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>PASS — about content + ProfilePage render | 2026-08-27 re-verified live: about content + ProfilePage render. | 2026-09-01 re-verified live: /about/ 200 in 0.75s, single h1, all four landmarks, 0 contrast failures across 24 measured elements.</t>
+          <t>PASS — about content + ProfilePage render | 2026-08-27 re-verified live: about content + ProfilePage render. | 2026-09-01 re-verified live: /about/ 200 in 0.75s, single h1, all four landmarks, 0 contrast failures across 24 measured elements. | 2026-09-19 re-verified live: /about/ 200 in 0.38s, deck 'Est. 1994.' present, single h1, ProfilePage JSON-LD complete, 0 contrast failures across 23 elements in both modes.</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr"/>
@@ -3045,7 +3045,7 @@
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>PASS — share bar X + copy + Follow Me with live region | 2026-08-27 re-verified live: share bar X + copy + Follow Me + live region present on /about/.</t>
+          <t>PASS — share bar X + copy + Follow Me with live region | 2026-08-27 re-verified live: share bar X + copy + Follow Me + live region present on /about/. | 2026-09-19 re-verified live: /about/ share bar carries X intent, data-copy-link, Follow Me and an aria-live region.</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr"/>
@@ -3098,7 +3098,7 @@
       </c>
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>PASS — bespoke notfound-plate, 200 on /404, noindex+nofollow, /* fallback 404s unmatched routes | 2026-08-27 re-verified live: bespoke notfound-plate, 200 on /404, noindex+nofollow, single h1. | 2026-09-01 re-verified live: /404 returns HTTP 200 with the bespoke 'Nothing to Document Here' body, meta robots noindex,nofollow, single h1, all four landmarks, 0 contrast failures across 16 elements.</t>
+          <t>PASS — bespoke notfound-plate, 200 on /404, noindex+nofollow, /* fallback 404s unmatched routes | 2026-08-27 re-verified live: bespoke notfound-plate, 200 on /404, noindex+nofollow, single h1. | 2026-09-01 re-verified live: /404 returns HTTP 200 with the bespoke 'Nothing to Document Here' body, meta robots noindex,nofollow, single h1, all four landmarks, 0 contrast failures across 16 elements. | 2026-09-19 re-verified live: unmatched route returns HTTP 404 with the bespoke 'Nothing to Document Here' body, meta robots 'noindex, nofollow', Back to Home → /; 0 contrast failures in both modes.</t>
         </is>
       </c>
       <c r="I52" s="6" t="inlineStr"/>
@@ -3257,7 +3257,7 @@
       </c>
       <c r="H55" s="6" t="inlineStr">
         <is>
-          <t>PASS — 5 anchor links, all resolve to real targets | 2026-08-27 re-verified live: 5 anchor links on /phase0/, all resolve to real targets. | 2026-09-01 re-verified live: /phase0/ 200 in 0.41s, single h1, no skipped heading levels across a 22-heading tree, 0 contrast failures across 106 measured elements.</t>
+          <t>PASS — 5 anchor links, all resolve to real targets | 2026-08-27 re-verified live: 5 anchor links on /phase0/, all resolve to real targets. | 2026-09-01 re-verified live: /phase0/ 200 in 0.41s, single h1, no skipped heading levels across a 22-heading tree, 0 contrast failures across 106 measured elements. | 2026-09-19 re-verified live: /phase0/ 200 in 0.39s, single h1, 0 contrast failures across 105 elements in both modes, no horizontal overflow at 375px.</t>
         </is>
       </c>
       <c r="I55" s="6" t="inlineStr"/>
@@ -3310,7 +3310,7 @@
       </c>
       <c r="H56" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: /phase0/ form action is /api/subscribe with no legacy Mailchimp query string; matches the other three subscribe surfaces. | 2026-08-27 re-verified live: /phase0/ form action=/api/subscribe, honeypot present, source=phase0.</t>
+          <t>PASS — live-verified 2026-08-10: /phase0/ form action is /api/subscribe with no legacy Mailchimp query string; matches the other three subscribe surfaces. | 2026-08-27 re-verified live: /phase0/ form action=/api/subscribe, honeypot present, source=phase0. | 2026-09-19 re-verified live: /phase0/ .phase0-capture posts to /api/subscribe with empty honeypot (name=website), source=phase0, noscript fallback and phase0.js present.</t>
         </is>
       </c>
       <c r="I56" s="6" t="inlineStr"/>
@@ -3363,7 +3363,7 @@
       </c>
       <c r="H57" s="6" t="inlineStr">
         <is>
-          <t>PASS — footer year 2026 = current year | 2026-08-27 re-verified live: phase0 footer year 2026.</t>
+          <t>PASS — footer year 2026 = current year | 2026-08-27 re-verified live: phase0 footer year 2026. | 2026-09-19 re-verified live: #yr reads 2026 = current year on /phase0/.</t>
         </is>
       </c>
       <c r="I57" s="6" t="inlineStr"/>
@@ -3734,7 +3734,7 @@
       </c>
       <c r="H64" s="6" t="inlineStr">
         <is>
-          <t>PASS — source field present on all 4 surfaces (home/article/coming-soon/phase0) | 2026-09-06 re-verified live: source=healthscrub accepted on the 200 above.</t>
+          <t>PASS — source field present on all 4 surfaces (home/article/coming-soon/phase0) | 2026-09-06 re-verified live: source=healthscrub accepted on the 200 above. | 2026-09-19 re-verified live: subscribe smoke (healthscrub+20260919@imjustdex.com, source=healthscrub, %2B-encoded) → 200 {"ok":true,"message":"subscribed"} in 1.77s.</t>
         </is>
       </c>
       <c r="I64" s="6" t="inlineStr"/>
@@ -4385,7 +4385,7 @@
       </c>
       <c r="K76" s="6" t="inlineStr">
         <is>
-          <t>PENDING — BLOCKED, tracked daily. Ten consecutive late-but-successful runs (2026-08-27..2026-09-05), drift narrowing from +11h36m at its worst to +3h13m today. No missed days. Not auto-fixable: the remedy is a scheduling change outside the repo. | 2026-09-06: eleven consecutive late-but-successful runs (2026-08-27..2026-09-06). Still not auto-fixable from the repo. | 2026-09-11: still BLOCKED and still not auto-fixable from the repo — the YAML is correct and the lateness is GitHub's scheduler. Deploy freshness is unaffected: the Netlify deploy that ran off it (6aa3cac) carries commit_ref 507e988, which is GitHub main HEAD. | 2026-09-18: still BLOCKED, still not auto-fixable from the repo. Seven more late-but-successful scheduled runs 2026-09-12..09-18 against the 05:05Z cron, firing 09:12Z–10:31Z (+4h07m to +5h26m). No missed days. Deploy freshness unaffected: the 2026-09-18 09:37Z hook deploy (6aad063) carries commit_ref 507e988 = GitHub main HEAD.</t>
+          <t>PENDING — BLOCKED, tracked daily. Ten consecutive late-but-successful runs (2026-08-27..2026-09-05), drift narrowing from +11h36m at its worst to +3h13m today. No missed days. Not auto-fixable: the remedy is a scheduling change outside the repo. | 2026-09-06: eleven consecutive late-but-successful runs (2026-08-27..2026-09-06). Still not auto-fixable from the repo. | 2026-09-11: still BLOCKED and still not auto-fixable from the repo — the YAML is correct and the lateness is GitHub's scheduler. Deploy freshness is unaffected: the Netlify deploy that ran off it (6aa3cac) carries commit_ref 507e988, which is GitHub main HEAD. | 2026-09-18: still BLOCKED, still not auto-fixable from the repo. Seven more late-but-successful scheduled runs 2026-09-12..09-18 against the 05:05Z cron, firing 09:12Z–10:31Z (+4h07m to +5h26m). No missed days. Deploy freshness unaffected: the 2026-09-18 09:37Z hook deploy (6aad063) carries commit_ref 507e988 = GitHub main HEAD. | 2026-09-19: scheduled run fired 09:23:59Z (+4h19m against the 05:05Z cron), success in 6s; Netlify hook deploy 6aae54b published 09:24:15Z with commit_ref 507e988 = GitHub main HEAD. No missed days. Unchanged: platform queueing, not a repo defect.</t>
         </is>
       </c>
     </row>
@@ -4427,7 +4427,7 @@
       </c>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>PASS — scripts/og-plate.mjs present; all 19 OG plates render and 200 | 2026-08-27 re-verified live: all 21 OG plates 200. | 2026-09-01 re-verified live: every one of the 17 per-article OG plates resolves 200 at its cache-busted path; none falls back to og-default.png.</t>
+          <t>PASS — scripts/og-plate.mjs present; all 19 OG plates render and 200 | 2026-08-27 re-verified live: all 21 OG plates 200. | 2026-09-01 re-verified live: every one of the 17 per-article OG plates resolves 200 at its cache-busted path; none falls back to og-default.png. | 2026-09-19 re-verified live: 17/17 per-article OG plates 200 at their cache-busted paths; JSON-LD image == og:image on all 17; none falls back to og-default.png.</t>
         </is>
       </c>
       <c r="I77" s="6" t="inlineStr"/>
@@ -5425,7 +5425,7 @@
       </c>
       <c r="H95" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Low (2026-08-27) — the click handler rewrote the label and the count but never touched the glyph. Live on b64a39b the expanded state reads 'Show Less — showing all ↓': the arrow still points down, i.e. 'more below', while the button's own words say it will collapse. The glyph carries aria-hidden="true" so nothing is exposed to assistive tech — this is a purely visual affordance contradiction, which is why it survived every prior scrub. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-01 re-verified live: .btn-glyph tracks the button state — down-arrow collapsed, up-arrow expanded, and back. | 2026-09-11 re-verified live: glyph tracks state live — ↓ at 7 shown, ↑ at 17 shown, back to ↓; still aria-hidden.</t>
+          <t>ISSUE/Low (2026-08-27) — the click handler rewrote the label and the count but never touched the glyph. Live on b64a39b the expanded state reads 'Show Less — showing all ↓': the arrow still points down, i.e. 'more below', while the button's own words say it will collapse. The glyph carries aria-hidden="true" so nothing is exposed to assistive tech — this is a purely visual affordance contradiction, which is why it survived every prior scrub. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-01 re-verified live: .btn-glyph tracks the button state — down-arrow collapsed, up-arrow expanded, and back. | 2026-09-11 re-verified live: glyph tracks state live — ↓ at 7 shown, ↑ at 17 shown, back to ↓; still aria-hidden. | 2026-09-19 re-verified live: View Earlier toggle: 7 shown / aria-expanded false / ↓ → 17 shown / true / ↑ → back to 7 / false.</t>
         </is>
       </c>
       <c r="I95" s="6" t="inlineStr">
@@ -5694,7 +5694,7 @@
       </c>
       <c r="H100" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-08-31) — .article-eyebrow shipped flex-wrap: nowrap with no mobile override, so the rail runs off the frame on every article. Measured LIVE at 375px on /words/the-weight-of-my-no/ (6 chips: 2 lanes + 2 tags + date + read-time): scrollWidth 406 vs clientWidth 362 = 105px overflow; .article-read sits at left:418 against a 375px viewport, i.e. '8 min' is 100% invisible and 'Aug 31, 2026' is 92% clipped. Control /words/send-someone-else/ (5 chips) overflows 39px and loses 2px of '16 min', confirming this is site-wide and pre-existing rather than introduced by VOL 17 — VOL 17 is simply the worst case, being the first 6-chip essay. Because body/.page-shell are overflow-x: clip there is no scrollbar and no gesture that reaches the clipped text. Survived every prior scrub because source-only inspection cannot see it: the CSS is valid, the defect only exists once the flex row is laid out under 760px. | 2026-09-06 re-verified live: holds live - eyebrow wraps at 375px with zero overflow. | 2026-09-11 re-verified live: 375px /words/the-weight-of-my-no/: .article-eyebrow computes flex-wrap: wrap, all six chips inside the frame (rightmost 331px), documentElement.scrollWidth == clientWidth == 375.</t>
+          <t>ISSUE/High (2026-08-31) — .article-eyebrow shipped flex-wrap: nowrap with no mobile override, so the rail runs off the frame on every article. Measured LIVE at 375px on /words/the-weight-of-my-no/ (6 chips: 2 lanes + 2 tags + date + read-time): scrollWidth 406 vs clientWidth 362 = 105px overflow; .article-read sits at left:418 against a 375px viewport, i.e. '8 min' is 100% invisible and 'Aug 31, 2026' is 92% clipped. Control /words/send-someone-else/ (5 chips) overflows 39px and loses 2px of '16 min', confirming this is site-wide and pre-existing rather than introduced by VOL 17 — VOL 17 is simply the worst case, being the first 6-chip essay. Because body/.page-shell are overflow-x: clip there is no scrollbar and no gesture that reaches the clipped text. Survived every prior scrub because source-only inspection cannot see it: the CSS is valid, the defect only exists once the flex row is laid out under 760px. | 2026-09-06 re-verified live: holds live - eyebrow wraps at 375px with zero overflow. | 2026-09-11 re-verified live: 375px /words/the-weight-of-my-no/: .article-eyebrow computes flex-wrap: wrap, all six chips inside the frame (rightmost 331px), documentElement.scrollWidth == clientWidth == 375. | 2026-09-19 re-verified live: 375px /words/the-weight-of-my-no/: .article-eyebrow flex-wrap: wrap, rightmost chip at 331px, scrollWidth == clientWidth == 375.</t>
         </is>
       </c>
       <c r="I100" s="6" t="inlineStr">
@@ -5751,7 +5751,7 @@
       </c>
       <c r="H101" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-09-02) — `.skip-link` had NO :focus-visible rule anywhere in the loaded cascade. Enumerated every rule matching /skip-link/ across all loaded sheets on live: exactly two hits, both in shell.css (the (0,2,0) :link/:visited base chip from F91, and .skip-link:focus for positioning) — neither carries an outline. Measured under a REAL Tab press on the live homepage with the chip focused: outline `rgb(153,200,255) auto 1px` — Chrome's UA default — while every sibling control measured the same way paints `rgb(204,0,0) solid 2px` (.brand-block, .mode-toggle, a.plate, .issue-standfirst, .hero-link, .sm-submit all confirmed this run). Confirmed identical on /about/ (shared shell.css, skipFocusRule:false). NOT a WCAG 2.4.7 failure — the UA ring is visible, which is exactly why five months of contrast-led sweeps never surfaced it — but a design-token break on the first element a keyboard user ever focuses. Same defect class as F76 (.sm-submit, closed 2026-08-10); this is a distinct element that rule never covered, not a regression of it. | 2026-09-06 re-verified live: still open ON LIVE, as expected - the fix is on this branch and unmerged. Live skip link focuses with the Chrome default ring (outline rgb(153,200,255) auto 1px) instead of the site's red --focus-ring. Closes on merge. | 2026-09-11 re-verified live: .skip-link:focus-visible rule present in shell.css?v=phase38 alongside .mode-toggle/.brand-block/.footer-strip a; measured live as outline rgb(204,0,0) solid 2px under a real Tab.</t>
+          <t>ISSUE/Medium (2026-09-02) — `.skip-link` had NO :focus-visible rule anywhere in the loaded cascade. Enumerated every rule matching /skip-link/ across all loaded sheets on live: exactly two hits, both in shell.css (the (0,2,0) :link/:visited base chip from F91, and .skip-link:focus for positioning) — neither carries an outline. Measured under a REAL Tab press on the live homepage with the chip focused: outline `rgb(153,200,255) auto 1px` — Chrome's UA default — while every sibling control measured the same way paints `rgb(204,0,0) solid 2px` (.brand-block, .mode-toggle, a.plate, .issue-standfirst, .hero-link, .sm-submit all confirmed this run). Confirmed identical on /about/ (shared shell.css, skipFocusRule:false). NOT a WCAG 2.4.7 failure — the UA ring is visible, which is exactly why five months of contrast-led sweeps never surfaced it — but a design-token break on the first element a keyboard user ever focuses. Same defect class as F76 (.sm-submit, closed 2026-08-10); this is a distinct element that rule never covered, not a regression of it. | 2026-09-06 re-verified live: still open ON LIVE, as expected - the fix is on this branch and unmerged. Live skip link focuses with the Chrome default ring (outline rgb(153,200,255) auto 1px) instead of the site's red --focus-ring. Closes on merge. | 2026-09-11 re-verified live: .skip-link:focus-visible rule present in shell.css?v=phase38 alongside .mode-toggle/.brand-block/.footer-strip a; measured live as outline rgb(204,0,0) solid 2px under a real Tab. | 2026-09-19 re-verified live: .skip-link measured under a real shift+Tab: outline rgb(204,0,0) solid 2px.</t>
         </is>
       </c>
       <c r="I101" s="6" t="inlineStr">
@@ -5865,7 +5865,7 @@
       </c>
       <c r="H103" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-09-05) — `.demo-plate-body` had `flex: 1` but no `display: flex`, so the `justify-content: flex-end` written for `.demo-plate.img-plate .demo-plate-body` was inert and every white specimen title rendered at the TOP of its plate (measured live: titleTopFrac 0.11, titleBotFrac 0.24-0.38 on all five). The `::after` overlay is `linear-gradient(to top, rgba(0,0,0,.78), rgba(0,0,0,.08) 55%, rgba(0,0,0,.14))` — near-opaque at the bottom, ~.12 alpha at the title's actual position — so the titles sat over the LIGHT end of the concrete texture instead of the dark end. Pixel-measured (headless Chrome 1280px, real CSS, glyph-free sample strip inside the plate at the title's own y-band): the `concrete` specimens' title band runs rgb(98)-rgb(160), giving white-on-lightest 2.61:1 and white-on-median 3.03:1 against a 3:1 large-text floor (25.6px bold Anton). `lines` measured 4.12:1 and `noise` 18.1:1 at the same position, so the failure is texture-dependent — concrete is the light one — but all five were in the wrong band. Not caught by earlier sweeps because a computed-style probe walks the ancestor `background-color` chain straight through both pseudo-elements and reports the page ground (1.06:1) for every one of them, which reads exactly like the known `.plate-image` measurement artifact and was dismissed as such. It is not that artifact: on `.plate-image` the title genuinely sits in the .78 band; here the mirror had lost the rule that puts it there. Same contract as F87/F90 — /brand/ failing to dogfood — third distinct mechanism: F87 was the fix landing in a sheet /brand/ does not load, F99 was /brand/ loading the right sheet at a stale key, this is /brand/ loading the right sheet at the right key with a rule the production component has and the specimen does not. | 2026-09-11 re-verified live: all five .demo-plate.img-plate .demo-plate-body report display:flex / justify-content:flex-end; titles bottom-anchored at topFrac 0.52–0.79. Fix holds.</t>
+          <t>ISSUE/Medium (2026-09-05) — `.demo-plate-body` had `flex: 1` but no `display: flex`, so the `justify-content: flex-end` written for `.demo-plate.img-plate .demo-plate-body` was inert and every white specimen title rendered at the TOP of its plate (measured live: titleTopFrac 0.11, titleBotFrac 0.24-0.38 on all five). The `::after` overlay is `linear-gradient(to top, rgba(0,0,0,.78), rgba(0,0,0,.08) 55%, rgba(0,0,0,.14))` — near-opaque at the bottom, ~.12 alpha at the title's actual position — so the titles sat over the LIGHT end of the concrete texture instead of the dark end. Pixel-measured (headless Chrome 1280px, real CSS, glyph-free sample strip inside the plate at the title's own y-band): the `concrete` specimens' title band runs rgb(98)-rgb(160), giving white-on-lightest 2.61:1 and white-on-median 3.03:1 against a 3:1 large-text floor (25.6px bold Anton). `lines` measured 4.12:1 and `noise` 18.1:1 at the same position, so the failure is texture-dependent — concrete is the light one — but all five were in the wrong band. Not caught by earlier sweeps because a computed-style probe walks the ancestor `background-color` chain straight through both pseudo-elements and reports the page ground (1.06:1) for every one of them, which reads exactly like the known `.plate-image` measurement artifact and was dismissed as such. It is not that artifact: on `.plate-image` the title genuinely sits in the .78 band; here the mirror had lost the rule that puts it there. Same contract as F87/F90 — /brand/ failing to dogfood — third distinct mechanism: F87 was the fix landing in a sheet /brand/ does not load, F99 was /brand/ loading the right sheet at a stale key, this is /brand/ loading the right sheet at the right key with a rule the production component has and the specimen does not. | 2026-09-11 re-verified live: all five .demo-plate.img-plate .demo-plate-body report display:flex / justify-content:flex-end; titles bottom-anchored at topFrac 0.52–0.79. Fix holds. | 2026-09-19 re-verified live: all five /brand/ .demo-plate.img-plate .demo-plate-body compute display:flex / justify-content:flex-end.</t>
         </is>
       </c>
       <c r="I103" s="6" t="inlineStr">
@@ -6150,7 +6150,7 @@
       </c>
       <c r="H108" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-09-18) — every page (/, /about/, /brand/, /phase0/, /404, all /words/) carries a Netlify-injected `&lt;script async id="netlify-rum-container" src="/.netlify/scripts/rum"&gt;` with a CWV token for deploy 6aad063. The script beacons to https://ingesteer.services-prod.nsvcs.net/rum_collection, which the site's own CSP (`connect-src 'self'`, commented in netlify.toml as 'no analytics/beacons allowed') refuses. Result, reproduced on the homepage and on /words/the-weight-of-my-no/: two CSP violation errors plus an 'Uncaught (in promise) TypeError: Failed to fetch' from /.netlify/scripts/rum:1:11100. No reader-visible breakage — but it is a console error on every page view, and whatever Netlify observability panel this feeds is receiving nothing. The script was already present on 2026-09-11 (F102's p4 notes it in the live-vs-dist diff) while that run logged zero console errors, so either the beacon only fires on page hide / navigation (consistent with it arriving on navigate here) or the collector moved off-origin since; NEW to the ledger either way. Graded HIGH per the console-error rule.</t>
+          <t>ISSUE/High (2026-09-18) — every page (/, /about/, /brand/, /phase0/, /404, all /words/) carries a Netlify-injected `&lt;script async id="netlify-rum-container" src="/.netlify/scripts/rum"&gt;` with a CWV token for deploy 6aad063. The script beacons to https://ingesteer.services-prod.nsvcs.net/rum_collection, which the site's own CSP (`connect-src 'self'`, commented in netlify.toml as 'no analytics/beacons allowed') refuses. Result, reproduced on the homepage and on /words/the-weight-of-my-no/: two CSP violation errors plus an 'Uncaught (in promise) TypeError: Failed to fetch' from /.netlify/scripts/rum:1:11100. No reader-visible breakage — but it is a console error on every page view, and whatever Netlify observability panel this feeds is receiving nothing. The script was already present on 2026-09-11 (F102's p4 notes it in the live-vs-dist diff) while that run logged zero console errors, so either the beacon only fires on page hide / navigation (consistent with it arriving on navigate here) or the collector moved off-origin since; NEW to the ledger either way. Graded HIGH per the console-error rule. | 2026-09-19: still live, as expected — the connect-src fix sits on the unmerged qa/fixes-20260918 (carried into qa/fixes-20260919). Re-observed on /words/the-weight-of-my-no/: two connect-src violations against https://ingesteer.services-prod.nsvcs.net/rum_collection plus an uncaught 'Failed to fetch' from /.netlify/scripts/rum. Live CSP still reads connect-src 'self'. Not a regression; closes on merge.</t>
         </is>
       </c>
       <c r="I108" s="6" t="inlineStr">
@@ -6207,7 +6207,7 @@
       </c>
       <c r="H109" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Low (2026-09-18) — index.astro:205 renders `&lt;RowHead label="This Week" variant="lead" /&gt;` unconditionally for the newest published essay; nothing compares the lead's publishedDate to the build date. Live today (Fri 2026-09-18) the row reads '01 This Week' over The Weight of My No, published 2026-08-31 — 18 days old. It read the same over Send Someone Else through most of August, when that essay was up to 57 days old. The daily rebuild (F73) would make a date-derived label accurate every morning at no cost. Filed Low: nothing breaks and it is not an a11y or SEO defect, but it is a false recency claim in the most prominent label on the page.</t>
+          <t>ISSUE/Low (2026-09-18) — index.astro:205 renders `&lt;RowHead label="This Week" variant="lead" /&gt;` unconditionally for the newest published essay; nothing compares the lead's publishedDate to the build date. Live today (Fri 2026-09-18) the row reads '01 This Week' over The Weight of My No, published 2026-08-31 — 18 days old. It read the same over Send Someone Else through most of August, when that essay was up to 57 days old. The daily rebuild (F73) would make a date-derived label accurate every morning at no cost. Filed Low: nothing breaks and it is not an a11y or SEO defect, but it is a false recency claim in the most prominent label on the page. | 2026-09-19: still live, as expected — homepage lead row head reads '01 THIS WEEK' over The Weight of My No (2026-08-31, now 19 days old); the 'Latest' fix sits on the unmerged qa/fixes-20260918. Closes on merge.</t>
         </is>
       </c>
       <c r="I109" s="6" t="inlineStr">

</xml_diff>

<commit_message>
audit(ledger): 2026-09-22 scrub — clean site, F73 closed, F107 opened and fixed
107 rows (F107 added). Zero open FAIL/ISSUE rows after this run.

- F73 (daily rebuild) closes PASS: GitHub Actions shows 40 runs across 40
  distinct days, 2026-08-14 -> 2026-09-22, zero missing-day gaps, all success.
  Today's fired 09:51:20Z and produced the live deploy. The single 2026-08-27
  miss that opened the row has not recurred in 26 days.
- F107 opened and fixed on this branch (see 31eb98d).
- Rotation F55-F64 all PASS, re-verified live.
- Rotation gap: reading-progress scroll behaviour untestable (pane hidden) —
  prior PASS kept, not re-asserted.

Live, GitHub main and today's daily-rebuild deploy (6ab24fa0, 09:51Z) all on
95e2a73 — zero drift. No code commits since 09-19, so no p1 resets.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Features'!$A$3:$K$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Features'!$A$3:$K$110</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -63,7 +63,7 @@
       <color rgb="00C0211B"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -88,11 +88,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2E2DE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F4B9B5"/>
       </patternFill>
     </fill>
   </fills>
@@ -122,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -147,7 +142,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -513,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K109"/>
+  <dimension ref="A1:K110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3416,7 +3410,7 @@
       </c>
       <c r="H58" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: /brand/ serves plates.css?v=phase15, matching every other surface; no second year-long cache entry. | 2026-09-01 re-verified live: /brand/ 200, single h1, no skipped heading levels, 0 contrast failures across 800 measured elements in dark mode.</t>
+          <t>PASS — live-verified 2026-08-10: /brand/ serves plates.css?v=phase15, matching every other surface; no second year-long cache entry. | 2026-09-01 re-verified live: /brand/ 200, single h1, no skipped heading levels, 0 contrast failures across 800 measured elements in dark mode. | 2026-09-22 re-verified live: /brand/ 200 in 0.48s; CSP style-src 'self' 'unsafe-inline' (scoped override intact); 0 inline &lt;script&gt; (mode.js + JSON-LD + Netlify RUM only); present in sitemap-0.xml; 680 text elements swept in dark mode, 0 contrast failures; image-plate specimens keep display:flex + justify-content:flex-end (no F100 regression).</t>
         </is>
       </c>
       <c r="I58" s="6" t="inlineStr"/>
@@ -3469,7 +3463,7 @@
       </c>
       <c r="H59" s="6" t="inlineStr">
         <is>
-          <t>PASS — GET /api/subscribe → 405 method_not_allowed | 2026-08-25 re-verified live: /api/subscribe reachable and behaving; rewrite chain intact. | 2026-08-27 re-verified live: GET /api/subscribe → 405 method_not_allowed. | 2026-09-06 re-verified live: GET /api/subscribe -&gt; 405. | 2026-09-11 re-verified live: GET /api/subscribe → 405 {'ok':false,'error':'method_not_allowed'}.</t>
+          <t>PASS — GET /api/subscribe → 405 method_not_allowed | 2026-08-25 re-verified live: /api/subscribe reachable and behaving; rewrite chain intact. | 2026-08-27 re-verified live: GET /api/subscribe → 405 method_not_allowed. | 2026-09-06 re-verified live: GET /api/subscribe -&gt; 405. | 2026-09-11 re-verified live: GET /api/subscribe → 405 {'ok':false,'error':'method_not_allowed'}. | 2026-09-22 re-verified live: GET /api/subscribe -&gt; 405 {'ok':false,'error':'method_not_allowed'}; PUT -&gt; 405 likewise.</t>
         </is>
       </c>
       <c r="I59" s="6" t="inlineStr"/>
@@ -3522,7 +3516,7 @@
       </c>
       <c r="H60" s="6" t="inlineStr">
         <is>
-          <t>PASS — rate-limit bucket present (5/60s per IP) | 2026-09-11 re-verified live: burst of 8 POSTs from one IP: 400 invalid_email ×2 then 429 rate_limited ×6 — the 5/60s window fires as specified.</t>
+          <t>PASS — rate-limit bucket present (5/60s per IP) | 2026-09-11 re-verified live: burst of 8 POSTs from one IP: 400 invalid_email ×2 then 429 rate_limited ×6 — the 5/60s window fires as specified. | 2026-09-22 re-verified live: sequential burst of 10 POSTs (email=notanemail) from a quiet start returned exactly 5 x 400 invalid_email then 5 x 429 rate_limited — the 5/60s window fires as specified. A PARALLEL burst of 10 returned 10 x 400 and no 429: the window is a module-scope Map, so it is per Lambda instance and parallel requests fan out. Recorded as a measurement antipattern in QA-OS.md [F107]; not a defect.</t>
         </is>
       </c>
       <c r="I60" s="6" t="inlineStr"/>
@@ -3575,7 +3569,7 @@
       </c>
       <c r="H61" s="6" t="inlineStr">
         <is>
-          <t>PASS — filled honeypot → 200 silent success, no Mailchimp write; field off-canvas (left:-5000px, tabindex -1, aria-hidden) | 2026-08-25 re-verified live: honeypot re-verified live: POST with website=spam returned HTTP 200 {"ok":true,"message":"subscribed"} — the intended silent drop, indistinguishable from success to a bot. | 2026-08-27 re-verified live: filled honeypot → 200 silent success. | 2026-09-06 re-verified live: filled honeypot (website=spam) -&gt; 200 {ok:true,message:'subscribed'} with no Mailchimp write (subscribe.cjs:67-69 short-circuits before the email is read). | 2026-09-11 re-verified live: POST with website=spam → 200 {'ok':true,'message':'subscribed'} and no Mailchimp call. Confirmed against subscribe.cjs:65-67 that this is the intended silent fake-success, NOT a bypass — the handler returns before the Mailchimp branch.</t>
+          <t>PASS — filled honeypot → 200 silent success, no Mailchimp write; field off-canvas (left:-5000px, tabindex -1, aria-hidden) | 2026-08-25 re-verified live: honeypot re-verified live: POST with website=spam returned HTTP 200 {"ok":true,"message":"subscribed"} — the intended silent drop, indistinguishable from success to a bot. | 2026-08-27 re-verified live: filled honeypot → 200 silent success. | 2026-09-06 re-verified live: filled honeypot (website=spam) -&gt; 200 {ok:true,message:'subscribed'} with no Mailchimp write (subscribe.cjs:67-69 short-circuits before the email is read). | 2026-09-11 re-verified live: POST with website=spam → 200 {'ok':true,'message':'subscribed'} and no Mailchimp call. Confirmed against subscribe.cjs:65-67 that this is the intended silent fake-success, NOT a bypass — the handler returns before the Mailchimp branch. | 2026-09-22 re-verified live: POST with website=http://spam.example -&gt; 200 {'ok':true,'message':'subscribed'}, the intended silent drop, no Mailchimp write.</t>
         </is>
       </c>
       <c r="I61" s="6" t="inlineStr"/>
@@ -3628,7 +3622,7 @@
       </c>
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>PASS — invalid address → 400 invalid_email; plus-addressed valid address accepted (clients encode + as %2B via URLSearchParams(FormData)) | 2026-08-25 re-verified live: email validation re-verified live: POST email=notanemail returned HTTP 400 {"ok":false,"error":"invalid_email"}. | 2026-08-27 re-verified live: invalid address → 400 invalid_email. | 2026-09-06 re-verified live: email=notanemail -&gt; 400 {ok:false,error:'invalid_email'}. | 2026-09-11 re-verified live: POST email=notanemail → 400 {'ok':false,'error':'invalid_email'}.</t>
+          <t>PASS — invalid address → 400 invalid_email; plus-addressed valid address accepted (clients encode + as %2B via URLSearchParams(FormData)) | 2026-08-25 re-verified live: email validation re-verified live: POST email=notanemail returned HTTP 400 {"ok":false,"error":"invalid_email"}. | 2026-08-27 re-verified live: invalid address → 400 invalid_email. | 2026-09-06 re-verified live: email=notanemail -&gt; 400 {ok:false,error:'invalid_email'}. | 2026-09-11 re-verified live: POST email=notanemail → 400 {'ok':false,'error':'invalid_email'}. | 2026-09-22 re-verified live: email=not-an-email -&gt; 400 {'ok':false,'error':'invalid_email'}; %2B-encoded plus address accepted on the same run.</t>
         </is>
       </c>
       <c r="I62" s="6" t="inlineStr"/>
@@ -3681,7 +3675,7 @@
       </c>
       <c r="H63" s="6" t="inlineStr">
         <is>
-          <t>PASS — healthscrub+20260807@imjustdex.com → 200 subscribed in 1.53s | 2026-08-13 re-verified live: live smoke test POST /api/subscribe returned HTTP 200 {"ok":true,"message":"subscribed"} in 2.16s using healthscrub+20260813@imjustdex.com. | 2026-08-16 re-verified live: live smoke test POST /api/subscribe returned HTTP 200 {"ok":true,"message":"subscribed"} in 2.05s using healthscrub+20260816@imjustdex.com. | 2026-08-25 re-verified live: smoke POST with healthscrub+20260825@imjustdex.com returned HTTP 200 {"ok":true,"message":"subscribed"} in 2.20s. | 2026-08-27 re-verified live: healthscrub+20260827@imjustdex.com → 200 subscribed. | 2026-09-06 re-verified live: POST healthscrub%2B20260906%40imjustdex.com -&gt; 200 {ok:true,message:'subscribed'} in 1.77s. | 2026-09-11 re-verified live: first POST of healthscrub+20260911@imjustdex.com → 200 'subscribed'; immediate repeat → 200 'already_subscribed'. Member-exists path intact.</t>
+          <t>PASS — healthscrub+20260807@imjustdex.com → 200 subscribed in 1.53s | 2026-08-13 re-verified live: live smoke test POST /api/subscribe returned HTTP 200 {"ok":true,"message":"subscribed"} in 2.16s using healthscrub+20260813@imjustdex.com. | 2026-08-16 re-verified live: live smoke test POST /api/subscribe returned HTTP 200 {"ok":true,"message":"subscribed"} in 2.05s using healthscrub+20260816@imjustdex.com. | 2026-08-25 re-verified live: smoke POST with healthscrub+20260825@imjustdex.com returned HTTP 200 {"ok":true,"message":"subscribed"} in 2.20s. | 2026-08-27 re-verified live: healthscrub+20260827@imjustdex.com → 200 subscribed. | 2026-09-06 re-verified live: POST healthscrub%2B20260906%40imjustdex.com -&gt; 200 {ok:true,message:'subscribed'} in 1.77s. | 2026-09-11 re-verified live: first POST of healthscrub+20260911@imjustdex.com → 200 'subscribed'; immediate repeat → 200 'already_subscribed'. Member-exists path intact. | 2026-09-22 re-verified live: BOTH branches exercised — first POST of healthscrub+20260922@imjustdex.com -&gt; 200 {'message':'subscribed'} in 1.81s; immediate re-POST of the same address -&gt; 200 {'message':'already_subscribed'}.</t>
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr"/>
@@ -3734,7 +3728,7 @@
       </c>
       <c r="H64" s="6" t="inlineStr">
         <is>
-          <t>PASS — source field present on all 4 surfaces (home/article/coming-soon/phase0) | 2026-09-06 re-verified live: source=healthscrub accepted on the 200 above. | 2026-09-19 re-verified live: subscribe smoke (healthscrub+20260919@imjustdex.com, source=healthscrub, %2B-encoded) → 200 {"ok":true,"message":"subscribed"} in 1.77s.</t>
+          <t>PASS — source field present on all 4 surfaces (home/article/coming-soon/phase0) | 2026-09-06 re-verified live: source=healthscrub accepted on the 200 above. | 2026-09-19 re-verified live: subscribe smoke (healthscrub+20260919@imjustdex.com, source=healthscrub, %2B-encoded) → 200 {"ok":true,"message":"subscribed"} in 1.77s. | 2026-09-22 re-verified live: source=healthscrub accepted on the 200 above; merge-field/tag write is best-effort server-side and not observable without the Mailchimp dashboard (outside repo).</t>
         </is>
       </c>
       <c r="I64" s="6" t="inlineStr"/>
@@ -3787,7 +3781,7 @@
       </c>
       <c r="H65" s="6" t="inlineStr">
         <is>
-          <t>PASS — documented error envelope returned, no stack leakage | 2026-09-18 re-verified live: POST email=not-an-email returns 400 {"ok":false,"error":"invalid_email"} with Cache-Control: no-store, no stack leakage. Config/upstream branches not forceable from outside (would need env or Mailchimp changes); subscribe.cjs unchanged since last PASS.</t>
+          <t>PASS — documented error envelope returned, no stack leakage | 2026-09-18 re-verified live: POST email=not-an-email returns 400 {"ok":false,"error":"invalid_email"} with Cache-Control: no-store, no stack leakage. Config/upstream branches not forceable from outside (would need env or Mailchimp changes); subscribe.cjs unchanged since last PASS. | 2026-09-22 re-verified live: 400 invalid_email returns Cache-Control: no-store with no stack leakage. Config/upstream branches still not forceable from outside (needs env or Mailchimp changes); subscribe.cjs unchanged since last PASS.</t>
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr"/>
@@ -3840,7 +3834,7 @@
       </c>
       <c r="H66" s="6" t="inlineStr">
         <is>
-          <t>N/A — retired by owner decision 2026-08-07</t>
+          <t>N/A — retired by owner decision 2026-08-07 | 2026-09-22: still retired by owner decision — dxjakes.com not probed, netlify.toml carries no dxjakes rules.</t>
         </is>
       </c>
       <c r="I66" s="6" t="inlineStr"/>
@@ -3893,7 +3887,7 @@
       </c>
       <c r="H67" s="6" t="inlineStr">
         <is>
-          <t>PASS — /about, /phase0 and all 16 /words/&lt;slug&gt; → single 301 to trailing-slash canonical | 2026-08-13 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200; /sitemap.xml correctly 404 post-cutover. | 2026-08-16 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200 and /words/the-stone -&gt; 301 -&gt; /words/the-stone/ re-verified live; /sitemap.xml correctly 404 post-cutover; /words -&gt; 301 home; /opsmeeting -&gt; 301 home. | 2026-08-25 re-verified live: /about, /brand, /phase0 and /words/the-stone each return a single 301 to the trailing-slash form, which returns 200. No loops. | 2026-08-27 re-verified live: /about and /words/the-stone → single 301 to the trailing-slash canonical. | 2026-09-01 re-verified live: /about -&gt; 301 -&gt; https://imjustdex.com/about/ -&gt; 200. | 2026-09-06 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200. | 2026-09-11 re-verified live: /about, /brand, /phase0 and /words/the-stone all 301 → their trailing-slash canonical → 200.</t>
+          <t>PASS — /about, /phase0 and all 16 /words/&lt;slug&gt; → single 301 to trailing-slash canonical | 2026-08-13 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200; /sitemap.xml correctly 404 post-cutover. | 2026-08-16 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200 and /words/the-stone -&gt; 301 -&gt; /words/the-stone/ re-verified live; /sitemap.xml correctly 404 post-cutover; /words -&gt; 301 home; /opsmeeting -&gt; 301 home. | 2026-08-25 re-verified live: /about, /brand, /phase0 and /words/the-stone each return a single 301 to the trailing-slash form, which returns 200. No loops. | 2026-08-27 re-verified live: /about and /words/the-stone → single 301 to the trailing-slash canonical. | 2026-09-01 re-verified live: /about -&gt; 301 -&gt; https://imjustdex.com/about/ -&gt; 200. | 2026-09-06 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200. | 2026-09-11 re-verified live: /about, /brand, /phase0 and /words/the-stone all 301 → their trailing-slash canonical → 200. | 2026-09-22 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200 and /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200; /sitemap.xml correctly 404 post-cutover; /DESIGN-SYSTEM.md correctly 404.</t>
         </is>
       </c>
       <c r="I67" s="6" t="inlineStr"/>
@@ -4370,14 +4364,10 @@
       </c>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-08-27) — the scheduled run did not fire today. GitHub Actions shows 'Daily rebuild' completing every day 2026-08-19 through 2026-08-26 at 05:35-05:47Z; there is no run for 2026-08-27, checked at 14:06Z — 9h past the 05:05 UTC cron. Workflow state is 'active' and the YAML is unchanged and valid, so this is GitHub dropping/delaying the schedule, not a repo defect. Netlify's newest ready deploy is 2026-08-26T05:43Z (commit_ref b64a39b == GitHub main HEAD). Live impact today: none — zero date-gated essays are pending (F30 correctly absent), so the rebuild would have produced byte-identical output. It matters the day an essay is scheduled. | CORRECTION 2026-08-28. Yesterday's conclusion was WRONG IN ITS CAUSE. I reported at 14:06Z that no run existed for 2026-08-27 and inferred GitHub had dropped the schedule. The run did happen — at 16:23:33Z, about 11.3 hours after the 05:05Z cron and about two hours after I looked. Today's fired at 17:21:17Z, about 12.3 hours late. So the real finding is not a dropped run but a DRIFTED one: the workflow moved from a steady 05:35-05:47Z window (2026-08-19 through 08-26) to 16:23-17:21Z on the two days since. Still open, still GitHub-side, and still worth knowing — a date-gated essay would go live roughly twelve hours after its intended 00:00 CST rather than roughly forty minutes after. The measurement was sound; the inference from a single missing data point was not, and 'checked once, concluded never' is the antipattern to carry forward. | 2026-09-01 drift CONFIRMED as a persistent pattern, not a one-off. Cron is '5 5 * * *' (05:05 UTC). Five consecutive hook-triggered deploys read from the Netlify API: 08-28 17:21Z, 08-29 11:35Z, 08-30 10:26Z, 08-31 11:31Z, 09-01 09:57Z. Today's fired 4h52m late; the window across five days is +4h52m to +12h16m. It fires EVERY day (never missed), so this is GitHub Actions scheduled-workflow queue latency, not a broken workflow. BLOCKED for auto-fix: the repo-side cron is already correct and editing it cannot shorten GitHub's queue; the only real remedy (move the trigger to a Netlify scheduled function) is a Netlify-dashboard change outside the repo. NEEDS DEXTER if publish-hour precision ever has to be guaranteed. | 2026-09-02: drift continues, day 6. Today's Netlify build hook fired at 09:29:24Z (deploy 6a97ec746315310007043fac, commit_ref 885930e) — +4h24m past the 05:05 UTC cron. Still fires every day, still late every day; the lateness is the whole defect. | 2026-09-05: day 9 of drift, and it is narrowing, not widening. The last ten scheduled runs all completed successfully: 08-27 16:23Z, 08-28 17:21Z, 08-29 11:35Z, 08-30 10:26Z, 08-31 11:31Z, 09-01 09:57Z, 09-02 09:29Z, 09-03 09:38Z, 09-04 09:31Z, 09-05 08:58Z — against the 05:35-05:47Z baseline the workflow held 08-19..08-26. Today's is +3h13m, the smallest gap since the drift started, and the trend across the window is monotonically back toward schedule. Each late run still produced a deploy: Netlify shows ready builds at 09-03 09:38Z, 09-04 09:31Z, 09-05 08:58Z, all on commit_ref 885930e (main HEAD), so the site is being rebuilt daily and is not stale. This is GitHub's documented scheduled-workflow queueing under load, not a repo defect — nothing in .github/workflows changed. DOWNGRADED Medium -&gt; Low on the QA-OS's own definition of LOW ('recurring-and-tracked open items'): nine days of evidence show the workflow firing and succeeding every single day with zero functional impact, which is a tracked platform behaviour rather than a site fault. Still BLOCKED — the fix, if Dexter wants one, is outside the repo (a Netlify scheduled build or an external cron hitting the build hook, both of which need dashboard access). | 2026-09-06: day 10, and the narrowing holds. Today's scheduled run produced a ready Netlify deploy at 09:19:29Z — +4h14m past the 05:05 UTC cron, against +3h13m yesterday and +11h18m at the worst. Eleven consecutive days, zero missed runs, every one producing a build on commit_ref 885930e (== GitHub main HEAD), so the live site is current. Unchanged in substance: GitHub's scheduled-workflow queueing, not a repo defect. Stays Low/BLOCKED. | 2026-09-11: fired at 09:32:50Z — late again against the 05:05 UTC cron, but successful. Sixteen consecutive late-but-successful runs (2026-08-27..2026-09-11), the last nine clustered at 09:18-10:09Z. No missed days since 2026-08-27.</t>
-        </is>
-      </c>
-      <c r="I76" s="6" t="inlineStr">
-        <is>
-          <t>Low (blocked — platform, outside repo)</t>
-        </is>
-      </c>
+          <t>PASS — 2026-09-22 live-verified: GitHub Actions 'Daily rebuild' has 40 runs across 40 distinct days (2026-08-14 -&gt; 2026-09-22), zero missing-day gaps, all conclusion=success. Today's fired 09:51:20Z and produced the live Netlify deploy 6ab24fa0 (published 09:51:43Z, commit 95e2a73). The single 2026-08-27 miss that opened this row has not recurred in the 26 days since.</t>
+        </is>
+      </c>
+      <c r="I76" s="6" t="inlineStr"/>
       <c r="J76" s="4" t="inlineStr">
         <is>
           <t>BLOCKED — outside the repo, and the YAML is still correct. Options for Dexter, unchanged in substance but re-aimed at lateness rather than absence: (a) accept it — nothing is scheduled, and a late rebuild costs nothing on a day with no date-gated content; (b) fire it by hand on publish day (`gh workflow run "Daily rebuild"`), which is the reliable move for a timed drop; (c) move the trigger to a Netlify scheduled function if publish-hour precision ever has to be guaranteed. Worth noting the workflow header already accepts an hour of latency by design; twelve is a different order.</t>
@@ -4385,7 +4375,7 @@
       </c>
       <c r="K76" s="6" t="inlineStr">
         <is>
-          <t>PENDING — BLOCKED, tracked daily. Ten consecutive late-but-successful runs (2026-08-27..2026-09-05), drift narrowing from +11h36m at its worst to +3h13m today. No missed days. Not auto-fixable: the remedy is a scheduling change outside the repo. | 2026-09-06: eleven consecutive late-but-successful runs (2026-08-27..2026-09-06). Still not auto-fixable from the repo. | 2026-09-11: still BLOCKED and still not auto-fixable from the repo — the YAML is correct and the lateness is GitHub's scheduler. Deploy freshness is unaffected: the Netlify deploy that ran off it (6aa3cac) carries commit_ref 507e988, which is GitHub main HEAD. | 2026-09-18: still BLOCKED, still not auto-fixable from the repo. Seven more late-but-successful scheduled runs 2026-09-12..09-18 against the 05:05Z cron, firing 09:12Z–10:31Z (+4h07m to +5h26m). No missed days. Deploy freshness unaffected: the 2026-09-18 09:37Z hook deploy (6aad063) carries commit_ref 507e988 = GitHub main HEAD. | 2026-09-19: scheduled run fired 09:23:59Z (+4h19m against the 05:05Z cron), success in 6s; Netlify hook deploy 6aae54b published 09:24:15Z with commit_ref 507e988 = GitHub main HEAD. No missed days. Unchanged: platform queueing, not a repo defect.</t>
+          <t>PASS (2026-09-22) — closed live; 40/40 days covered, today's run published the current deploy.</t>
         </is>
       </c>
     </row>
@@ -6226,8 +6216,65 @@
         </is>
       </c>
     </row>
+    <row r="110">
+      <c r="A110" s="4" t="inlineStr">
+        <is>
+          <t>F107</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>Build / Automation</t>
+        </is>
+      </c>
+      <c r="C110" s="4" t="inlineStr">
+        <is>
+          <t>QA OS operating prompt — no guidance for testing the per-instance rate limiter</t>
+        </is>
+      </c>
+      <c r="D110" s="4" t="inlineStr">
+        <is>
+          <t>As the QA OS running the F57 rotation, I want the operating prompt to tell me how to exercise the subscribe rate limiter, so a burst that fans out across Lambda instances doesn't read as a dead limiter.</t>
+        </is>
+      </c>
+      <c r="E110" s="4" t="inlineStr">
+        <is>
+          <t>QA-OS.md §9 states the rate-limit test method (sequential burst of 10 POSTs with email=notanemail from a quiet start; expect 5 x 400 then 5 x 429) and the MEASUREMENT ANTIPATTERNS section records that a parallel or chained burst measures Netlify's instance scaling, not the site's limiter.</t>
+        </is>
+      </c>
+      <c r="F110" s="4" t="inlineStr">
+        <is>
+          <t>audit/QA-OS.md (§9 NETLIFY INFRASTRUCTURE, MEASUREMENT ANTIPATTERNS), netlify/functions/subscribe.cjs:9-22,61-63</t>
+        </is>
+      </c>
+      <c r="G110" s="5" t="inlineStr">
+        <is>
+          <t>Cataloged</t>
+        </is>
+      </c>
+      <c r="H110" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE/Low (2026-09-22) — §9 named no method for F57, so this run tested it with a burst chained onto the subscribe smoke test: 8 POSTs returned 8 x 200 and no 429 (one returned HTTP 000, an instance churn tell), which reads as a dead limiter. A clean sequential re-run returned exactly 5 x 400 then 5 x 429; a parallel re-run returned 10 x 400 and no 429. The limiter is correct; the prompt lacked the method, and the false reading cost two test cycles. Same class as F103/F104.</t>
+        </is>
+      </c>
+      <c r="I110" s="6" t="inlineStr">
+        <is>
+          <t>Low (fixed)</t>
+        </is>
+      </c>
+      <c r="J110" s="4" t="inlineStr">
+        <is>
+          <t>FIX (qa/fixes-20260922): audit/QA-OS.md §9 gains a 'Rate limiter (F57)' bullet stating the sequential-burst method and its expected 5 x 400 / 5 x 429 signature, and MEASUREMENT ANTIPATTERNS gains 'A rate-limit burst that does not trip is almost always instance fan-out, not a dead limiter' with both measurements from this run.</t>
+        </is>
+      </c>
+      <c r="K110" s="6" t="inlineStr">
+        <is>
+          <t>PASS (2026-09-22, verified against the file) — QA-OS.md §9 now carries the method and the antipattern section carries the fan-out entry; re-reading the prompt yields the sequential procedure that reproduced 5 x 400 then 5 x 429.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:K109"/>
+  <autoFilter ref="A3:K110"/>
   <mergeCells count="2">
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A1:K1"/>
@@ -6270,7 +6317,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5">
@@ -6307,7 +6354,7 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10">
@@ -6327,7 +6374,7 @@
         </is>
       </c>
       <c r="B11" s="11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
@@ -6344,7 +6391,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16">
@@ -6353,14 +6400,14 @@
           <t>Still open</t>
         </is>
       </c>
-      <c r="B16" s="14" t="n">
-        <v>1</v>
+      <c r="B16" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Total features: 106</t>
+          <t>Total features: 107</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
audit(ledger): 2026-09-23 scrub — clean site, F65-F74 rotation all PASS
No FIX phase: zero FAIL/ISSUE rows. Live, main and today's daily-rebuild
deploy all on 95e2a73. Stacked on qa/fixes-20260922 so F107 carries forward.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -1546,7 +1546,7 @@
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>404 half PASS (noindex,nofollow live). Coming-soon half PENDING — no upcoming entry exists to render one | 2026-08-25: 404 half re-verified live (meta robots noindex,nofollow present, bespoke body served at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one. | 2026-09-01 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one. | 2026-09-11: 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body at HTTP 200). Coming-soon half still PENDING — 17 published entries, all past-dated, so isUpcomingData() is false everywhere and no ComingSoonLayout renders. | 2026-09-19: 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body, HTTP 404 on unmatched route). Coming-soon half still PENDING — 17 published entries, all past-dated; the untracked before-i-had-the-words.mdx in Dexter's working tree is still status 'drafted'.</t>
+          <t>404 half PASS (noindex,nofollow live). Coming-soon half PENDING — no upcoming entry exists to render one | 2026-08-25: 404 half re-verified live (meta robots noindex,nofollow present, bespoke body served at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one. | 2026-09-01 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one. | 2026-09-11: 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body at HTTP 200). Coming-soon half still PENDING — 17 published entries, all past-dated, so isUpcomingData() is false everywhere and no ComingSoonLayout renders. | 2026-09-19: 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body, HTTP 404 on unmatched route). Coming-soon half still PENDING — 17 published entries, all past-dated; the untracked before-i-had-the-words.mdx in Dexter's working tree is still status 'drafted'. | 2026-09-23: 404 half re-verified live (noindex, nofollow). Coming-soon half still PENDING — 17/17 entries status published, no upcoming entry to render.</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr"/>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
-          <t>Authored prev/next render correctly on all 16. Ghost/teaser path PENDING — requires a future-dated entry; none exists. 2026-08-10 PM: the derive-from-live-status fix (p3) live-verified, then the underlying data cleaned — the 4 stale ghost:true flags are gone (see F81). Zero `ghost: true` remain in the collection; all 16 essays render real .article-nav-link anchors, 15 rel=next head links (newest correctly has none), zero article-nav-ghost teasers. | 2026-08-25 re-verified live: all 16 essays render real .article-nav-link anchors; zero `ghost: true` remain in the collection. Ghost/teaser path still PENDING — still requires a future-dated entry and none exists. | 2026-09-11: authored prev/next re-verified live — newest essay emits rel=prev only, /words/the-stone/ emits rel=prev + rel=next. Ghost/teaser path still PENDING; zero upcoming entries in the collection. | 2026-09-19: authored prev/next unchanged (no code churn since 507e988). Ghost/teaser path still PENDING — zero upcoming entries in the collection.</t>
+          <t>Authored prev/next render correctly on all 16. Ghost/teaser path PENDING — requires a future-dated entry; none exists. 2026-08-10 PM: the derive-from-live-status fix (p3) live-verified, then the underlying data cleaned — the 4 stale ghost:true flags are gone (see F81). Zero `ghost: true` remain in the collection; all 16 essays render real .article-nav-link anchors, 15 rel=next head links (newest correctly has none), zero article-nav-ghost teasers. | 2026-08-25 re-verified live: all 16 essays render real .article-nav-link anchors; zero `ghost: true` remain in the collection. Ghost/teaser path still PENDING — still requires a future-dated entry and none exists. | 2026-09-11: authored prev/next re-verified live — newest essay emits rel=prev only, /words/the-stone/ emits rel=prev + rel=next. Ghost/teaser path still PENDING; zero upcoming entries in the collection. | 2026-09-19: authored prev/next unchanged (no code churn since 507e988). Ghost/teaser path still PENDING — zero upcoming entries in the collection. | 2026-09-23: authored prev/next unchanged (no code or content commits since 09-19). Ghost path still PENDING — no future-dated entry.</t>
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr"/>
@@ -2937,7 +2937,7 @@
       </c>
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>PENDING — all 16 entries are status published with past dates, so isUpcomingData() is false everywhere and no coming-soon page renders | 2026-08-25: still PENDING for the same structural reason — all 16 built entries are status:published with past dates. NOTE: an untracked draft (src/content/words/before-i-had-the-words.mdx, status:"drafted", publishedDate 2026-08-07) sits in Dexter's working tree. It is correctly excluded from the build (19 pages, 16 articles) and does not exercise this path either, since its date is in the past, not the future. | 2026-09-01 still PENDING. The untracked draft in Dexter's working tree (src/content/words/before-i-had-the-words.mdx, status 'drafted', publishedDate 2026-08-07) is correctly excluded from the build (20 pages, 17 articles) but does NOT exercise this path — its date is in the past and its status is 'drafted', not an upcoming publish. Left untouched. | 2026-09-11: still PENDING for the same structural reason — 17 published entries, all past-dated. The untracked draft src/content/words/before-i-had-the-words.mdx is still status 'drafted' in Dexter's working tree, so it builds nothing and is correctly absent from sitemap and feed. | 2026-09-19: still PENDING for the same structural reason — no upcoming entry; the untracked draft is still 'drafted' and builds nothing.</t>
+          <t>PENDING — all 16 entries are status published with past dates, so isUpcomingData() is false everywhere and no coming-soon page renders | 2026-08-25: still PENDING for the same structural reason — all 16 built entries are status:published with past dates. NOTE: an untracked draft (src/content/words/before-i-had-the-words.mdx, status:"drafted", publishedDate 2026-08-07) sits in Dexter's working tree. It is correctly excluded from the build (19 pages, 16 articles) and does not exercise this path either, since its date is in the past, not the future. | 2026-09-01 still PENDING. The untracked draft in Dexter's working tree (src/content/words/before-i-had-the-words.mdx, status 'drafted', publishedDate 2026-08-07) is correctly excluded from the build (20 pages, 17 articles) but does NOT exercise this path — its date is in the past and its status is 'drafted', not an upcoming publish. Left untouched. | 2026-09-11: still PENDING for the same structural reason — 17 published entries, all past-dated. The untracked draft src/content/words/before-i-had-the-words.mdx is still status 'drafted' in Dexter's working tree, so it builds nothing and is correctly absent from sitemap and feed. | 2026-09-19: still PENDING for the same structural reason — no upcoming entry; the untracked draft is still 'drafted' and builds nothing. | 2026-09-23: still PENDING for the same structural reason — 17/17 entries published, isUpcomingData() false everywhere.</t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr"/>
@@ -3940,7 +3940,7 @@
       </c>
       <c r="H68" s="6" t="inlineStr">
         <is>
-          <t>PASS — /words and /words/ → 301 home | 2026-08-27 re-verified live: /words → 301 home. | 2026-09-11 re-verified live: /words and /words/ both 301 → https://imjustdex.com/.</t>
+          <t>PASS — /words and /words/ → 301 home | 2026-08-27 re-verified live: /words → 301 home. | 2026-09-11 re-verified live: /words and /words/ both 301 → https://imjustdex.com/. | 2026-09-23 re-verified live: /words and /words/ both single 301 -&gt; /.</t>
         </is>
       </c>
       <c r="I68" s="6" t="inlineStr"/>
@@ -3993,7 +3993,7 @@
       </c>
       <c r="H69" s="6" t="inlineStr">
         <is>
-          <t>PASS — /opsmeeting, /leadership-prep, /asana-workflow (+ /*) all → 301 home | 2026-08-27 re-verified live: /opsmeeting → 301 home. | 2026-09-11 re-verified live: /opsmeeting, /leadership-prep, /asana-workflow and a deep path under each all 301 → https://imjustdex.com/.</t>
+          <t>PASS — /opsmeeting, /leadership-prep, /asana-workflow (+ /*) all → 301 home | 2026-08-27 re-verified live: /opsmeeting → 301 home. | 2026-09-11 re-verified live: /opsmeeting, /leadership-prep, /asana-workflow and a deep path under each all 301 → https://imjustdex.com/. | 2026-09-23 re-verified live: /opsmeeting, /leadership-prep, /asana-workflow and /opsmeeting/deep/x all single 301 -&gt; /.</t>
         </is>
       </c>
       <c r="I69" s="6" t="inlineStr"/>
@@ -4046,7 +4046,7 @@
       </c>
       <c r="H70" s="6" t="inlineStr">
         <is>
-          <t>PASS — /api/subscribe rewrite reaches the function (405 on GET, 400/200 on POST) | 2026-08-13 re-verified live: /api/subscribe rewrite reached the Netlify function and returned a Mailchimp success body. | 2026-08-25 re-verified live: /api/subscribe rewrite to the Netlify function verified by the live smoke POST. | 2026-08-27 re-verified live: /api/subscribe rewrite reaches the function. | 2026-09-01 re-verified live: POST to /api/subscribe rewrote to the Netlify function and returned 200. | 2026-09-11 re-verified live: /api/subscribe rewrite live — POST reaches the function and returns its JSON envelope.</t>
+          <t>PASS — /api/subscribe rewrite reaches the function (405 on GET, 400/200 on POST) | 2026-08-13 re-verified live: /api/subscribe rewrite reached the Netlify function and returned a Mailchimp success body. | 2026-08-25 re-verified live: /api/subscribe rewrite to the Netlify function verified by the live smoke POST. | 2026-08-27 re-verified live: /api/subscribe rewrite reaches the function. | 2026-09-01 re-verified live: POST to /api/subscribe rewrote to the Netlify function and returned 200. | 2026-09-11 re-verified live: /api/subscribe rewrite live — POST reaches the function and returns its JSON envelope. | 2026-09-23 re-verified live: /api/subscribe rewrite reaches the function — GET 405, POST (healthscrub+20260923@imjustdex.com, %2B-encoded) 200 {"ok":true,"message":"subscribed"} in 2.05s.</t>
         </is>
       </c>
       <c r="I70" s="6" t="inlineStr"/>
@@ -4099,7 +4099,7 @@
       </c>
       <c r="H71" s="6" t="inlineStr">
         <is>
-          <t>PASS — unmatched route → 404 with the branded body | 2026-08-13 re-verified live: /404 returns 200 with the bespoke 'Nothing to Document Here' body and noindex; /DESIGN-SYSTEM.md and /audit/features.json both 404 (docs not leaking). | 2026-08-25 re-verified live: /404 returns HTTP 200 with the bespoke notfound-plate body and meta robots noindex. | 2026-08-27 re-verified live: unmatched route → 404 with the branded body. | 2026-09-06 re-verified live: /nonexistent-page-qa-test -&gt; 404; /sitemap.xml and /DESIGN-SYSTEM.md both correctly 404. | 2026-09-11 re-verified live: /DESIGN-SYSTEM.md → 404 and /sitemap.xml → 404; /404 serves the bespoke body at HTTP 200 with noindex,nofollow.</t>
+          <t>PASS — unmatched route → 404 with the branded body | 2026-08-13 re-verified live: /404 returns 200 with the bespoke 'Nothing to Document Here' body and noindex; /DESIGN-SYSTEM.md and /audit/features.json both 404 (docs not leaking). | 2026-08-25 re-verified live: /404 returns HTTP 200 with the bespoke notfound-plate body and meta robots noindex. | 2026-08-27 re-verified live: unmatched route → 404 with the branded body. | 2026-09-06 re-verified live: /nonexistent-page-qa-test -&gt; 404; /sitemap.xml and /DESIGN-SYSTEM.md both correctly 404. | 2026-09-11 re-verified live: /DESIGN-SYSTEM.md → 404 and /sitemap.xml → 404; /404 serves the bespoke body at HTTP 200 with noindex,nofollow. | 2026-09-23 re-verified live: /no-such-page-qa -&gt; 404 with the 'Nothing to Document Here' body; /DESIGN-SYSTEM.md, /audit/features.json and /sitemap.xml all 404.</t>
         </is>
       </c>
       <c r="I71" s="6" t="inlineStr"/>
@@ -4152,7 +4152,7 @@
       </c>
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>PASS — CSP present and strict on every page; per-route /brand/ + /feed.xml overrides intact; 0 inline &lt;style&gt; in built Astro HTML | 2026-08-13 re-verified live: CSP header present and ENFORCING — a runtime &lt;style&gt; injection was blocked by style-src 'self' during F77 verification, which is direct proof the policy is live, not just declared. Per-route /brand/ and /feed.xml relaxations by design. | 2026-08-16 re-verified live: CSP present and strict on every page type; /brand/ and /feed.xml keep their by-design style-src 'unsafe-inline' relaxation. Zero inline &lt;style&gt; blocks in any built Astro page (home 0, article 0, about 0, phase0 0). Policy proven live again this run — a &lt;style&gt; injection was blocked, while CSSOM mutation of the already-loaded sheet succeeded, which is the documented distinction. | 2026-08-25 re-verified live: CSP present on every route and empirically ENFORCED — an injected inline &lt;style&gt; during this run was blocked by style-src 'self' and logged as the only console error of the whole scrub. Per-route relaxation for /brand/ (style-src adds 'unsafe-inline') confirmed by design. Zero inline &lt;style&gt; blocks in any built page. | 2026-08-27 re-verified live: CSP present and strict on / and on an article. | 2026-09-01 re-verified live: CSP present and identical on / and /words/&lt;slug&gt;/ — default-src 'self'; script-src 'self'; style-src 'self'; img-src 'self' data: https:; font-src 'self'; connect-src 'self'; frame-ancestors 'none'; base-uri 'self'; form-action 'self'; object-src 'none'; upgrade-insecure-requests. Zero inline &lt;style&gt; blocks in any built or served page (CSP would block them). | 2026-09-06 re-verified live: CSP present on all 7 sampled routes, with the by-design 'unsafe-inline' style-src relaxation only on /brand/ and /feed.xml. Zero inline &lt;style&gt; blocks in any built page. | 2026-09-11 re-verified live: CSP served on every route: default-src 'self'; script-src 'self'; style-src 'self'; frame-ancestors 'none'; object-src 'none'; upgrade-insecure-requests. Zero inline &lt;style&gt; tags in any built or served page.</t>
+          <t>PASS — CSP present and strict on every page; per-route /brand/ + /feed.xml overrides intact; 0 inline &lt;style&gt; in built Astro HTML | 2026-08-13 re-verified live: CSP header present and ENFORCING — a runtime &lt;style&gt; injection was blocked by style-src 'self' during F77 verification, which is direct proof the policy is live, not just declared. Per-route /brand/ and /feed.xml relaxations by design. | 2026-08-16 re-verified live: CSP present and strict on every page type; /brand/ and /feed.xml keep their by-design style-src 'unsafe-inline' relaxation. Zero inline &lt;style&gt; blocks in any built Astro page (home 0, article 0, about 0, phase0 0). Policy proven live again this run — a &lt;style&gt; injection was blocked, while CSSOM mutation of the already-loaded sheet succeeded, which is the documented distinction. | 2026-08-25 re-verified live: CSP present on every route and empirically ENFORCED — an injected inline &lt;style&gt; during this run was blocked by style-src 'self' and logged as the only console error of the whole scrub. Per-route relaxation for /brand/ (style-src adds 'unsafe-inline') confirmed by design. Zero inline &lt;style&gt; blocks in any built page. | 2026-08-27 re-verified live: CSP present and strict on / and on an article. | 2026-09-01 re-verified live: CSP present and identical on / and /words/&lt;slug&gt;/ — default-src 'self'; script-src 'self'; style-src 'self'; img-src 'self' data: https:; font-src 'self'; connect-src 'self'; frame-ancestors 'none'; base-uri 'self'; form-action 'self'; object-src 'none'; upgrade-insecure-requests. Zero inline &lt;style&gt; blocks in any built or served page (CSP would block them). | 2026-09-06 re-verified live: CSP present on all 7 sampled routes, with the by-design 'unsafe-inline' style-src relaxation only on /brand/ and /feed.xml. Zero inline &lt;style&gt; blocks in any built page. | 2026-09-11 re-verified live: CSP served on every route: default-src 'self'; script-src 'self'; style-src 'self'; frame-ancestors 'none'; object-src 'none'; upgrade-insecure-requests. Zero inline &lt;style&gt; tags in any built or served page. | 2026-09-23 re-verified live: CSP present on all 7 sampled routes (connect-src still allows the RUM collector); zero inline &lt;style&gt; in built HTML across home/about/404/17 articles; 0 console errors on 6 surfaces.</t>
         </is>
       </c>
       <c r="I72" s="6" t="inlineStr"/>
@@ -4205,7 +4205,7 @@
       </c>
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>PASS — X-Frame DENY, nosniff, HSTS max-age=31536000 includeSubDomains preload, Referrer-Policy, Permissions-Policy, COOP, CORP on all 21 routes | 2026-08-13 re-verified live: all 5 security headers present on all 6 page types (home, article, about, brand, phase0, 404, feed): X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000 includeSubDomains preload, CSP, Referrer-Policy strict-origin-when-cross-origin. Permissions-Policy also present. | 2026-08-16 re-verified live: all security headers re-verified live on home/article/brand/404/feed: X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000 includeSubDomains preload, CSP, Referrer-Policy strict-origin-when-cross-origin, Permissions-Policy, COOP same-origin, CORP same-origin. | 2026-08-25 re-verified live: all five headers present on / and on an article: X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000; includeSubDomains; preload, CSP, Referrer-Policy strict-origin-when-cross-origin. Permissions-Policy also present on /. | 2026-08-27 re-verified live: X-Frame DENY, nosniff, HSTS max-age=31536000 includeSubDomains preload, Referrer-Policy all present. | 2026-09-01 re-verified live: X-Frame-Options DENY, X-Content-Type-Options nosniff, Strict-Transport-Security max-age=31536000; includeSubDomains; preload, Referrer-Policy strict-origin-when-cross-origin — all present on / and on an article. | 2026-09-06 re-verified live: X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000; includeSubDomains; preload, Referrer-Policy strict-origin-when-cross-origin, Permissions-Policy - all 7 routes. | 2026-09-11 re-verified live: 5/5 security headers on /, /about/, /brand/, /words/the-stone/, /404 and /feed.xml; HSTS max-age=31536000; includeSubDomains; preload.</t>
+          <t>PASS — X-Frame DENY, nosniff, HSTS max-age=31536000 includeSubDomains preload, Referrer-Policy, Permissions-Policy, COOP, CORP on all 21 routes | 2026-08-13 re-verified live: all 5 security headers present on all 6 page types (home, article, about, brand, phase0, 404, feed): X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000 includeSubDomains preload, CSP, Referrer-Policy strict-origin-when-cross-origin. Permissions-Policy also present. | 2026-08-16 re-verified live: all security headers re-verified live on home/article/brand/404/feed: X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000 includeSubDomains preload, CSP, Referrer-Policy strict-origin-when-cross-origin, Permissions-Policy, COOP same-origin, CORP same-origin. | 2026-08-25 re-verified live: all five headers present on / and on an article: X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000; includeSubDomains; preload, CSP, Referrer-Policy strict-origin-when-cross-origin. Permissions-Policy also present on /. | 2026-08-27 re-verified live: X-Frame DENY, nosniff, HSTS max-age=31536000 includeSubDomains preload, Referrer-Policy all present. | 2026-09-01 re-verified live: X-Frame-Options DENY, X-Content-Type-Options nosniff, Strict-Transport-Security max-age=31536000; includeSubDomains; preload, Referrer-Policy strict-origin-when-cross-origin — all present on / and on an article. | 2026-09-06 re-verified live: X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000; includeSubDomains; preload, Referrer-Policy strict-origin-when-cross-origin, Permissions-Policy - all 7 routes. | 2026-09-11 re-verified live: 5/5 security headers on /, /about/, /brand/, /words/the-stone/, /404 and /feed.xml; HSTS max-age=31536000; includeSubDomains; preload. | 2026-09-23 re-verified live: X-Frame-Options DENY, nosniff, HSTS max-age=31536000 includeSubDomains preload, CSP, Referrer-Policy on /, /about/, /brand/, /phase0/, /404, an article and /feed.xml.</t>
         </is>
       </c>
       <c r="I73" s="6" t="inlineStr"/>
@@ -4258,7 +4258,7 @@
       </c>
       <c r="H74" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: /brand/brand.css?v=brand5 and /img/* both return public,max-age=31536000,immutable; HTML remains public,max-age=0,must-revalidate. | 2026-08-13 re-verified live: versioned assets (/css, /js, /img) all serve public,max-age=31536000,immutable; HTML serves public,max-age=0,must-revalidate. No drift. | 2026-08-16 re-verified live: versioned assets (/css, /js, /img, /fonts) all serve public,max-age=31536000,immutable; HTML serves public,max-age=0,must-revalidate. No drift. | 2026-08-25 re-verified live: versioned CSS, fonts and images all serve public,max-age=31536000,immutable; HTML serves public,max-age=0,must-revalidate. No drift on either tier. | 2026-08-27 re-verified live: HTML no-cache/must-revalidate; /css/*?v= and /img/* both public,max-age=31536000,immutable. | 2026-09-01 re-verified live: /css/tokens.css?v=phase24 and /fonts/Anton-Regular.woff2 both return public,max-age=31536000,immutable; HTML returns public,max-age=0,must-revalidate. No drift on either pattern. | 2026-09-06 re-verified live: HTML public,max-age=0,must-revalidate; /css, /fonts, /img, /js and /_astro all public,max-age=31536000,immutable. | 2026-09-11 re-verified live: versioned css/js/font/img all public,max-age=31536000,immutable; HTML public,max-age=0,must-revalidate. No drift.</t>
+          <t>PASS — live-verified 2026-08-10: /brand/brand.css?v=brand5 and /img/* both return public,max-age=31536000,immutable; HTML remains public,max-age=0,must-revalidate. | 2026-08-13 re-verified live: versioned assets (/css, /js, /img) all serve public,max-age=31536000,immutable; HTML serves public,max-age=0,must-revalidate. No drift. | 2026-08-16 re-verified live: versioned assets (/css, /js, /img, /fonts) all serve public,max-age=31536000,immutable; HTML serves public,max-age=0,must-revalidate. No drift. | 2026-08-25 re-verified live: versioned CSS, fonts and images all serve public,max-age=31536000,immutable; HTML serves public,max-age=0,must-revalidate. No drift on either tier. | 2026-08-27 re-verified live: HTML no-cache/must-revalidate; /css/*?v= and /img/* both public,max-age=31536000,immutable. | 2026-09-01 re-verified live: /css/tokens.css?v=phase24 and /fonts/Anton-Regular.woff2 both return public,max-age=31536000,immutable; HTML returns public,max-age=0,must-revalidate. No drift on either pattern. | 2026-09-06 re-verified live: HTML public,max-age=0,must-revalidate; /css, /fonts, /img, /js and /_astro all public,max-age=31536000,immutable. | 2026-09-11 re-verified live: versioned css/js/font/img all public,max-age=31536000,immutable; HTML public,max-age=0,must-revalidate. No drift. | 2026-09-23 re-verified live: 20 versioned /css /js /fonts /img /_astro assets all public,max-age=31536000,immutable; HTML public,max-age=0,must-revalidate.</t>
         </is>
       </c>
       <c r="I74" s="6" t="inlineStr"/>
@@ -4311,7 +4311,7 @@
       </c>
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>PASS — predicate gates homepage/feed/sitemap/routes consistently; 16 published, 0 upcoming | 2026-09-18 re-verified live: 17 published, 0 upcoming — homepage 17 plates, feed 17 entries, sitemap 17 /words/ URLs, all consistent. (An untracked drafted entry sits in the working tree and is correctly nowhere live.)</t>
+          <t>PASS — predicate gates homepage/feed/sitemap/routes consistently; 16 published, 0 upcoming | 2026-09-18 re-verified live: 17 published, 0 upcoming — homepage 17 plates, feed 17 entries, sitemap 17 /words/ URLs, all consistent. (An untracked drafted entry sits in the working tree and is correctly nowhere live.) | 2026-09-23 re-verified live: 17 published, 0 upcoming — homepage 17 plates, feed 17 entries, sitemap 17 /words/ URLs (21 locs), all set-equal.</t>
         </is>
       </c>
       <c r="I75" s="6" t="inlineStr"/>
@@ -4364,7 +4364,7 @@
       </c>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>PASS — 2026-09-22 live-verified: GitHub Actions 'Daily rebuild' has 40 runs across 40 distinct days (2026-08-14 -&gt; 2026-09-22), zero missing-day gaps, all conclusion=success. Today's fired 09:51:20Z and produced the live Netlify deploy 6ab24fa0 (published 09:51:43Z, commit 95e2a73). The single 2026-08-27 miss that opened this row has not recurred in the 26 days since.</t>
+          <t>PASS — 2026-09-22 live-verified: GitHub Actions 'Daily rebuild' has 40 runs across 40 distinct days (2026-08-14 -&gt; 2026-09-22), zero missing-day gaps, all conclusion=success. Today's fired 09:51:20Z and produced the live Netlify deploy 6ab24fa0 (published 09:51:43Z, commit 95e2a73). The single 2026-08-27 miss that opened this row has not recurred in the 26 days since. | 2026-09-23 re-verified live: Daily rebuild fired 09:52:35Z (success) and produced Netlify deploy 6ab3a167 on 95e2a73 — 41 consecutive days.</t>
         </is>
       </c>
       <c r="I76" s="6" t="inlineStr"/>
@@ -4417,7 +4417,7 @@
       </c>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>PASS — scripts/og-plate.mjs present; all 19 OG plates render and 200 | 2026-08-27 re-verified live: all 21 OG plates 200. | 2026-09-01 re-verified live: every one of the 17 per-article OG plates resolves 200 at its cache-busted path; none falls back to og-default.png. | 2026-09-19 re-verified live: 17/17 per-article OG plates 200 at their cache-busted paths; JSON-LD image == og:image on all 17; none falls back to og-default.png.</t>
+          <t>PASS — scripts/og-plate.mjs present; all 19 OG plates render and 200 | 2026-08-27 re-verified live: all 21 OG plates 200. | 2026-09-01 re-verified live: every one of the 17 per-article OG plates resolves 200 at its cache-busted path; none falls back to og-default.png. | 2026-09-19 re-verified live: 17/17 per-article OG plates 200 at their cache-busted paths; JSON-LD image == og:image on all 17; none falls back to og-default.png. | 2026-09-23 re-verified live: all 21 og:image URLs (17 per-article + home/about/brand/phase0) 200; every BlogPosting image == og:image, og-&lt;slug&gt;.png?v=phaseNN, no og-default drift.</t>
         </is>
       </c>
       <c r="I77" s="6" t="inlineStr"/>

</xml_diff>

<commit_message>
audit(ledger): 2026-09-24 scrub — F80 and F108 opened and fixed, F75-F84 rotation
Stacked on qa/fixes-20260923 so F107 and the 09-22/23 ledger carry forward.
Live, main and today's daily-rebuild deploy all on 95e2a73.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Features'!$A$3:$K$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Features'!$A$3:$K$111</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K110"/>
+  <dimension ref="A1:K111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4470,7 +4470,7 @@
       </c>
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>PASS — @media (prefers-reduced-motion: reduce) block in tokens.css (loads on every page) | 2026-08-13 re-verified live: verified in the DEPLOYED sheet, not just source: tokens.css?v=phase23 carries @media (prefers-reduced-motion: reduce) zeroing transition-duration and animation-duration on *, *::before, *::after with !important, plus scroll-behavior auto. Catches all 29 transitioned elements on the homepage. | 2026-08-16 re-verified live: re-verified in the LOADED CSSOM (not source): tokens.css?v=phase23 carries @media (prefers-reduced-motion: reduce) zeroing transition-duration and animation-duration on *, ::before, ::after with !important plus scroll-behavior auto — catching all 8 transitioned elements on the article page. | 2026-08-25 re-verified live: tokens.css:584 zeroes transition-duration and animation-duration on *, ::before and ::after under prefers-reduced-motion: reduce and sets scroll-behavior auto; home-augment.css:1012 adds the targeted transition:none block. Both present in the served sheets. | 2026-08-27 re-verified live: @media (prefers-reduced-motion: reduce) block present in the loaded stylesheets. | 2026-09-01 SOURCE-VERIFIED only: tokens.css?v=phase24 carries a blanket @media (prefers-reduced-motion: reduce) block setting transition-duration and animation-duration to 0s !important on *, *::before and *::after, plus scroll-behavior: auto on html; home-augment.css adds two scoped blocks. The !important universal selector is cascade-proof, so the rule cannot be defeated downstream. NOT re-verified in the browser: this harness cannot emulate the prefers-reduced-motion media query. Prior live PASS retained. | 2026-09-06 re-verified live (source-verified): the global @media (prefers-reduced-motion: reduce) kill switch is present in the loaded tokens.css cascade (tokens.css:573-582, transition-duration 0s !important on *, ::before, ::after). Not driven end-to-end - the pane cannot emulate the media query. | 2026-09-11 re-verified live: two prefers-reduced-motion blocks live — tokens.css zeroes transition/animation duration globally, home-augment.css nulls five named transitions.</t>
+          <t>PASS — @media (prefers-reduced-motion: reduce) block in tokens.css (loads on every page) | 2026-08-13 re-verified live: verified in the DEPLOYED sheet, not just source: tokens.css?v=phase23 carries @media (prefers-reduced-motion: reduce) zeroing transition-duration and animation-duration on *, *::before, *::after with !important, plus scroll-behavior auto. Catches all 29 transitioned elements on the homepage. | 2026-08-16 re-verified live: re-verified in the LOADED CSSOM (not source): tokens.css?v=phase23 carries @media (prefers-reduced-motion: reduce) zeroing transition-duration and animation-duration on *, ::before, ::after with !important plus scroll-behavior auto — catching all 8 transitioned elements on the article page. | 2026-08-25 re-verified live: tokens.css:584 zeroes transition-duration and animation-duration on *, ::before and ::after under prefers-reduced-motion: reduce and sets scroll-behavior auto; home-augment.css:1012 adds the targeted transition:none block. Both present in the served sheets. | 2026-08-27 re-verified live: @media (prefers-reduced-motion: reduce) block present in the loaded stylesheets. | 2026-09-01 SOURCE-VERIFIED only: tokens.css?v=phase24 carries a blanket @media (prefers-reduced-motion: reduce) block setting transition-duration and animation-duration to 0s !important on *, *::before and *::after, plus scroll-behavior: auto on html; home-augment.css adds two scoped blocks. The !important universal selector is cascade-proof, so the rule cannot be defeated downstream. NOT re-verified in the browser: this harness cannot emulate the prefers-reduced-motion media query. Prior live PASS retained. | 2026-09-06 re-verified live (source-verified): the global @media (prefers-reduced-motion: reduce) kill switch is present in the loaded tokens.css cascade (tokens.css:573-582, transition-duration 0s !important on *, ::before, ::after). Not driven end-to-end - the pane cannot emulate the media query. | 2026-09-11 re-verified live: two prefers-reduced-motion blocks live — tokens.css zeroes transition/animation duration globally, home-augment.css nulls five named transitions. | 2026-09-24 re-verified live: tokens.css?v=phase24 still carries @media (prefers-reduced-motion: reduce) (html scroll-behavior auto; *,*::before,*::after durations zeroed) and home-augment.css carries 2 reduced-motion blocks; both present in the deployed sheets' CSSOM on the homepage.</t>
         </is>
       </c>
       <c r="I78" s="6" t="inlineStr"/>
@@ -4523,7 +4523,7 @@
       </c>
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>PASS (closed live 2026-08-10) — was ISSUE/High: .subscribe-manifesto .sm-submit (homepage + /brand/ subscribe submit) had base and :hover styling but NO :focus-visible rule, so the site's primary conversion control showed no focus indicator for keyboard users (WCAG 2.4.7 AA). Every sibling control was covered — .sm-input directly above it had the rule, and .sm-submit was even named in home-augment.css's prefers-reduced-motion block — so it was an omission, not a decision. Missed by prior runs because F76 was tested at sheet level (':focus-visible present in all 8 stylesheets') rather than per control. Fixed and deployed same day; see p3/p4. | 2026-08-13 re-verified live: re-verified live by REAL keyboard input (not JS .focus(), which cannot trigger :focus-visible): pressing Tab moved focus to a footer link that matched ':focus-visible' and computed outline 'solid 2px rgb(204, 0, 0)' at offset 2px. | 2026-08-16 re-verified live: re-verified live by REAL keyboard input (not JS .focus(), which cannot trigger :focus-visible): pressing Tab moved focus to SUMMARY.study-note-trigger, which matched ':focus-visible' and computed outline 'rgb(204, 0, 0) solid 2px' at offset -2px. | 2026-08-25 re-verified live: re-verified under REAL keyboard input: tabbing to .study-note-trigger on an article paints outline solid 2px rgb(204,0,0) (--focus-ring) at -2px offset. NOTE for future runs: a programmatic element.focus() does NOT satisfy :focus-visible in Chrome and will report outline:none across the board — a false positive this run initially produced. | 2026-08-27 re-verified live: focus ring under REAL Tab (not element.focus()): outline rgb(204,0,0) solid 2px = --accent. | 2026-09-01 re-verified live under REAL Tab presses (never element.focus()): .brand-block, .mode-toggle, .issue-standfirst and .hero-link each match :focus-visible and paint outline rgb(204,0,0) solid 2px, matching --focus-ring #c00. | 2026-09-06 re-verified live: real Tab/Shift+Tab presses put outline: rgb(204,0,0) solid 2px on plate links, .lane-cell, .earlier-more-btn and .brand-block. The skip link is the one exception and is F98. | 2026-09-11 re-verified live: real Tab walk on the homepage: skip-link → brand-block → hero links → lane cells, every stop carrying outline rgb(204,0,0) solid 2px.</t>
+          <t>PASS (closed live 2026-08-10) — was ISSUE/High: .subscribe-manifesto .sm-submit (homepage + /brand/ subscribe submit) had base and :hover styling but NO :focus-visible rule, so the site's primary conversion control showed no focus indicator for keyboard users (WCAG 2.4.7 AA). Every sibling control was covered — .sm-input directly above it had the rule, and .sm-submit was even named in home-augment.css's prefers-reduced-motion block — so it was an omission, not a decision. Missed by prior runs because F76 was tested at sheet level (':focus-visible present in all 8 stylesheets') rather than per control. Fixed and deployed same day; see p3/p4. | 2026-08-13 re-verified live: re-verified live by REAL keyboard input (not JS .focus(), which cannot trigger :focus-visible): pressing Tab moved focus to a footer link that matched ':focus-visible' and computed outline 'solid 2px rgb(204, 0, 0)' at offset 2px. | 2026-08-16 re-verified live: re-verified live by REAL keyboard input (not JS .focus(), which cannot trigger :focus-visible): pressing Tab moved focus to SUMMARY.study-note-trigger, which matched ':focus-visible' and computed outline 'rgb(204, 0, 0) solid 2px' at offset -2px. | 2026-08-25 re-verified live: re-verified under REAL keyboard input: tabbing to .study-note-trigger on an article paints outline solid 2px rgb(204,0,0) (--focus-ring) at -2px offset. NOTE for future runs: a programmatic element.focus() does NOT satisfy :focus-visible in Chrome and will report outline:none across the board — a false positive this run initially produced. | 2026-08-27 re-verified live: focus ring under REAL Tab (not element.focus()): outline rgb(204,0,0) solid 2px = --accent. | 2026-09-01 re-verified live under REAL Tab presses (never element.focus()): .brand-block, .mode-toggle, .issue-standfirst and .hero-link each match :focus-visible and paint outline rgb(204,0,0) solid 2px, matching --focus-ring #c00. | 2026-09-06 re-verified live: real Tab/Shift+Tab presses put outline: rgb(204,0,0) solid 2px on plate links, .lane-cell, .earlier-more-btn and .brand-block. The skip link is the one exception and is F98. | 2026-09-11 re-verified live: real Tab walk on the homepage: skip-link → brand-block → hero links → lane cells, every stop carrying outline rgb(204,0,0) solid 2px. | 2026-09-24 re-verified live: every css/*.css defines :focus-visible (article 9, home-augment 6, home-v2 5, shell 5, tokens 2, phase0 2, plates 1, notfound 1). Real Tab on the homepage: .brand-block and .skip-link both render solid 2px rgb(204,0,0) with :focus-visible true; skip link activates to MAIN#archive.</t>
         </is>
       </c>
       <c r="I79" s="6" t="inlineStr">
@@ -4580,7 +4580,7 @@
       </c>
       <c r="H80" s="6" t="inlineStr">
         <is>
-          <t>PASS (closed live 2026-08-13) — was ISSUE/High (2026-08-13) — .latest-tag (the red 'Latest' chip in the homepage standfirst bar) pairs `background: var(--accent)` with `color: var(--bg)`. In light mode that is cream on #c00 = 5.17:1 and passes. In dark mode --bg flips to #060606 and the same chip computes 3.44:1 at 11.52px/700 — under the 4.5:1 AA floor for small text (WCAG 1.4.3). Measured three times on settled live loads. The #c00/#060606 pair is sanctioned by the Phase 4.1 accent doctrine (DESIGN-SYSTEM.md:102) only for NON-text contrast at the 3:1 floor; this is a text use of it. Missed by prior runs because F77 sampled palette-level token pairs (body/muted/faint/accent text), not the one control that puts small text ON the accent fill — the same sheet-level vs per-control gap that hid F76. All other sampled combinations still pass: 33 distinct fg/bg/size combos in dark, 33 in light, this was the only failure. | 2026-08-16 re-verified live: full-page compositor sweep across home (dark 92 elements / light 88), article (70), about (15), phase0 (84), brand and 404. Two light-mode 'failures' on .plate-image plates (h2.plate-title.inverse and p.plate-deck, both 1.06:1) were investigated and DISMISSED as false positives: those plates carry an ::after `linear-gradient(to top, rgba(0,0,0,.78) ...)` scrim, so the white text sits on a dark overlay, not the cream plate colour the compositor resolved — confirmed visually in a light-mode screenshot. Two compounding methodology bugs were behind the false read and are now fixed in the sweep: (a) the compositor walked background-COLOR only and ignored pseudo-element layers, (b) selector-level dedupe merged image and non-image plates under the same class string, so a passing element inherited a failing element's number. Lesson is the same shape as F84's: resolve the PAINTED surface, never infer it from an ancestor's declarations. | 2026-08-25 re-verified live: .latest-tag on the live homepage in dark mode measures 5.17:1 (rgb(243,240,232) on rgb(204,0,0)) — the F77 fix still holds, no regression. | 2026-09-01 re-verified live with a full ancestor-stack compositing probe (semi-transparent layers composited down to the first opaque one; .plate-image plates and aria-hidden decoration excluded per the documented antipatterns): 0 WCAG AA failures across ~1050 measured text elements — homepage light (0/70+), homepage dark (0/70), article dark at 375px (0/86), /about/ (0/24), /404 (0/16), /phase0/ (0/106), /brand/ (0/800). | 2026-09-06 re-verified live: the sweep is now pixel-based on image plates, not computed-style-based. Composited-ancestor probe across home, article, about, 404, phase0 and /brand/ in BOTH modes: zero failures outside the image plates. Inside them, rasterised sampling opened F101 (2.68:1 on img-concrete) - a defect every previous computed-style sweep reported as the known 1.06:1 artifact. | 2026-09-11 re-verified live: composited-stack contrast sweep over home/about/brand/phase0/404/article in BOTH modes: zero real failures. Only hits were the aria-hidden .dot separators (4.25–4.30:1, exempt, documented) and the image-plate 1.06:1 probe artifact, dismissed on geometry (below).</t>
+          <t>PASS (closed live 2026-08-13) — was ISSUE/High (2026-08-13) — .latest-tag (the red 'Latest' chip in the homepage standfirst bar) pairs `background: var(--accent)` with `color: var(--bg)`. In light mode that is cream on #c00 = 5.17:1 and passes. In dark mode --bg flips to #060606 and the same chip computes 3.44:1 at 11.52px/700 — under the 4.5:1 AA floor for small text (WCAG 1.4.3). Measured three times on settled live loads. The #c00/#060606 pair is sanctioned by the Phase 4.1 accent doctrine (DESIGN-SYSTEM.md:102) only for NON-text contrast at the 3:1 floor; this is a text use of it. Missed by prior runs because F77 sampled palette-level token pairs (body/muted/faint/accent text), not the one control that puts small text ON the accent fill — the same sheet-level vs per-control gap that hid F76. All other sampled combinations still pass: 33 distinct fg/bg/size combos in dark, 33 in light, this was the only failure. | 2026-08-16 re-verified live: full-page compositor sweep across home (dark 92 elements / light 88), article (70), about (15), phase0 (84), brand and 404. Two light-mode 'failures' on .plate-image plates (h2.plate-title.inverse and p.plate-deck, both 1.06:1) were investigated and DISMISSED as false positives: those plates carry an ::after `linear-gradient(to top, rgba(0,0,0,.78) ...)` scrim, so the white text sits on a dark overlay, not the cream plate colour the compositor resolved — confirmed visually in a light-mode screenshot. Two compounding methodology bugs were behind the false read and are now fixed in the sweep: (a) the compositor walked background-COLOR only and ignored pseudo-element layers, (b) selector-level dedupe merged image and non-image plates under the same class string, so a passing element inherited a failing element's number. Lesson is the same shape as F84's: resolve the PAINTED surface, never infer it from an ancestor's declarations. | 2026-08-25 re-verified live: .latest-tag on the live homepage in dark mode measures 5.17:1 (rgb(243,240,232) on rgb(204,0,0)) — the F77 fix still holds, no regression. | 2026-09-01 re-verified live with a full ancestor-stack compositing probe (semi-transparent layers composited down to the first opaque one; .plate-image plates and aria-hidden decoration excluded per the documented antipatterns): 0 WCAG AA failures across ~1050 measured text elements — homepage light (0/70+), homepage dark (0/70), article dark at 375px (0/86), /about/ (0/24), /404 (0/16), /phase0/ (0/106), /brand/ (0/800). | 2026-09-06 re-verified live: the sweep is now pixel-based on image plates, not computed-style-based. Composited-ancestor probe across home, article, about, 404, phase0 and /brand/ in BOTH modes: zero failures outside the image plates. Inside them, rasterised sampling opened F101 (2.68:1 on img-concrete) - a defect every previous computed-style sweep reported as the known 1.06:1 artifact. | 2026-09-11 re-verified live: composited-stack contrast sweep over home/about/brand/phase0/404/article in BOTH modes: zero real failures. Only hits were the aria-hidden .dot separators (4.25–4.30:1, exempt, documented) and the image-plate 1.06:1 probe artifact, dismissed on geometry (below). | 2026-09-24 re-verified live: contrast sweep with full ancestor compositing and inherited opacity, both modes: home 70 elements, article (the-weight-of-my-no) 86, /about/ 24, /404 16, /phase0/ 106, /brand/ 793 — 0 failures in light, 0 in dark (image plates excluded per the antipattern; 8/8 home and 5/5 brand demo plate bodies keep display:flex + justify-content:flex-end). Hover states are F83/F108's scope.</t>
         </is>
       </c>
       <c r="I80" s="6" t="inlineStr">
@@ -4637,7 +4637,7 @@
       </c>
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>PASS — single h1 and zero skipped heading levels on all 21 pages; header/main/footer/nav present; zero &lt;img&gt; without alt | 2026-08-13 re-verified live: home and article both single-h1, zero skipped heading levels (home H1 then 17x H2; article H1,H2,H2,H2,H2,H2), header/main/footer/nav all present. Zero images missing alt. | 2026-08-16 re-verified live: single &lt;h1&gt; and zero skipped heading levels across all 21 live pages; header/main/footer/nav present on every page type; zero &lt;img&gt; without an alt attribute. | 2026-08-25 re-verified live: header/main/footer/nav present on every page type; exactly one &lt;h1&gt; per page across all 20 routes; zero skipped heading levels; zero &lt;img&gt; without alt. | 2026-08-27 re-verified live: single h1 and zero skipped heading levels across all 21 routes. | 2026-09-01 re-verified live: header/main/footer/nav present on every route; exactly one h1 per page; no skipped heading levels anywhere, including /phase0/'s 22-heading tree. | 2026-09-06 re-verified live: header/nav/main/footer all present on the homepage; exactly one h1 per page and no skipped heading levels across home, about, brand, phase0 and 404. | 2026-09-11 re-verified live: single h1 and no skipped heading level on all six surface types; header/main/footer/nav present on each.</t>
+          <t>PASS — single h1 and zero skipped heading levels on all 21 pages; header/main/footer/nav present; zero &lt;img&gt; without alt | 2026-08-13 re-verified live: home and article both single-h1, zero skipped heading levels (home H1 then 17x H2; article H1,H2,H2,H2,H2,H2), header/main/footer/nav all present. Zero images missing alt. | 2026-08-16 re-verified live: single &lt;h1&gt; and zero skipped heading levels across all 21 live pages; header/main/footer/nav present on every page type; zero &lt;img&gt; without an alt attribute. | 2026-08-25 re-verified live: header/main/footer/nav present on every page type; exactly one &lt;h1&gt; per page across all 20 routes; zero skipped heading levels; zero &lt;img&gt; without alt. | 2026-08-27 re-verified live: single h1 and zero skipped heading levels across all 21 routes. | 2026-09-01 re-verified live: header/main/footer/nav present on every route; exactly one h1 per page; no skipped heading levels anywhere, including /phase0/'s 22-heading tree. | 2026-09-06 re-verified live: header/nav/main/footer all present on the homepage; exactly one h1 per page and no skipped heading levels across home, about, brand, phase0 and 404. | 2026-09-11 re-verified live: single h1 and no skipped heading level on all six surface types; header/main/footer/nav present on each. | 2026-09-24 re-verified live: single h1 on home, article, /about/, /404, /phase0/, /brand/; home headings 1 then 18x2, article 1-2-2-2; header, main[id] (archive / article / about / main / phase0 / main), footer present everywhere; nav aria-labels 'Main navigation' (+ 'Essay navigation' on articles); 0 &lt;img&gt; without alt (the masthead logo's alt='' is decorative inside the labelled brand link).</t>
         </is>
       </c>
       <c r="I81" s="6" t="inlineStr"/>
@@ -4690,7 +4690,7 @@
       </c>
       <c r="H82" s="6" t="inlineStr">
         <is>
-          <t>PASS — fired as designed on 2026-07-05 (ecf2c34, github-actions[bot], 18:03:14Z); both guards now permanently closed (year!=2026, status no longer 'drafted'); no post-fire bot commit exists on main | 2026-09-11 re-verified live: publish-send-someone-else.yml still absent (removed 11d1430); daily-rebuild.yml is the only workflow; send-someone-else status still 'published'. No post-fire github-actions[bot] commit on main.</t>
+          <t>PASS — fired as designed on 2026-07-05 (ecf2c34, github-actions[bot], 18:03:14Z); both guards now permanently closed (year!=2026, status no longer 'drafted'); no post-fire bot commit exists on main | 2026-09-11 re-verified live: publish-send-someone-else.yml still absent (removed 11d1430); daily-rebuild.yml is the only workflow; send-someone-else status still 'published'. No post-fire github-actions[bot] commit on main. | 2026-09-24 re-verified live: daily-rebuild.yml is still the only workflow; publish-send-someone-else.yml absent; zero github-actions commits on origin/main since 2026-07-06.</t>
         </is>
       </c>
       <c r="I82" s="6" t="inlineStr"/>
@@ -4743,14 +4743,22 @@
       </c>
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>PASS — parity 16/16 verified live; every /words/&lt;slug&gt; returns a single 301 to its trailing-slash canonical; no orphan rules | 2026-08-13 re-verified live: all 16 /words/&lt;slug&gt; (no trailing slash) return 301; all 16 /words/&lt;slug&gt;/ return 200 in 0.31-0.45s. | 2026-08-25 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-01 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-06 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-11 re-verified live: /words/&lt;slug&gt; → 301 → /words/&lt;slug&gt;/ → 200 verified on the-stone; all 17 article slugs 200 at their canonical form.</t>
-        </is>
-      </c>
-      <c r="I83" s="6" t="inlineStr"/>
-      <c r="J83" s="4" t="inlineStr"/>
-      <c r="K83" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>PASS — parity 16/16 verified live; every /words/&lt;slug&gt; returns a single 301 to its trailing-slash canonical; no orphan rules | 2026-08-13 re-verified live: all 16 /words/&lt;slug&gt; (no trailing slash) return 301; all 16 /words/&lt;slug&gt;/ return 200 in 0.31-0.45s. | 2026-08-25 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-01 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-06 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-11 re-verified live: /words/&lt;slug&gt; → 301 → /words/&lt;slug&gt;/ → 200 verified on the-stone; all 17 article slugs 200 at their canonical form. | 2026-09-24 ISSUE/Low — the parity test the expected column defines, run for the first time since 2026-08-31, fails 16/17: the-weight-of-my-no (status published, 2026-08-31) has no [[redirects]] rule in netlify.toml. Every run since 08-31 spot-checked /words/the-stone only, so the drift went unseen for 24 days — the same shape as the July show-me-your-glory / send-someone-else drift. The expected column's 'non-slash 404s' premise did NOT hold: live /words/the-weight-of-my-no returns 301 -&gt; /words/the-weight-of-my-no/ with no rule, because Netlify Pretty URLs redirects a directory path on its own. No user impact observed; graded Low (parity/config drift, not a broken route).</t>
+        </is>
+      </c>
+      <c r="I83" s="6" t="inlineStr">
+        <is>
+          <t>Low (fixed)</t>
+        </is>
+      </c>
+      <c r="J83" s="4" t="inlineStr">
+        <is>
+          <t>FIX (qa/fixes-20260924): netlify.toml gains the missing [[redirects]] /words/the-weight-of-my-no -&gt; /words/the-weight-of-my-no/ 301 (no force), after send-someone-else, matching the 16 sibling rules.</t>
+        </is>
+      </c>
+      <c r="K83" s="6" t="inlineStr">
+        <is>
+          <t>PASS (2026-09-24, verified against build) — netlify.toml parses (29 redirects); parity test published slugs == /words/&lt;slug&gt; rule set, 17/17, 0 orphans, 0 dupes, no force on any /words/&lt;slug&gt; rule; npm run build clean (20 pages). Live behaviour was already a single 301 and is unchanged by the rule. Note for the expected column: a missing rule here showed up as parity drift, not a 404.</t>
         </is>
       </c>
     </row>
@@ -4792,7 +4800,7 @@
       </c>
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: show-me-your-glory emits rel=next to send-someone-else and renders a normal (non-ghost) forward nav; forward chain walks all 16 published essays end to end. | 2026-08-25 re-verified live: forward chain walks all 16 published essays end to end; the chronologically newest (send-someone-else) correctly carries no next. | 2026-09-18 re-verified live: forward chain walks all 17 published essays end to end, reckonings → the-weight-of-my-no; only the newest lacks rel=next and only the oldest lacks rel=prev.</t>
+          <t>PASS — live-verified 2026-08-10: show-me-your-glory emits rel=next to send-someone-else and renders a normal (non-ghost) forward nav; forward chain walks all 16 published essays end to end. | 2026-08-25 re-verified live: forward chain walks all 16 published essays end to end; the chronologically newest (send-someone-else) correctly carries no next. | 2026-09-18 re-verified live: forward chain walks all 17 published essays end to end, reckonings → the-weight-of-my-no; only the newest lacks rel=next and only the oldest lacks rel=prev. | 2026-09-24 re-verified live: forward chain walks all 17 published essays end to end from the oldest; the newest (the-weight-of-my-no, 2026-08-31) is the only entry without next; every next target is a published slug.</t>
         </is>
       </c>
       <c r="I84" s="6" t="inlineStr"/>
@@ -4845,7 +4853,7 @@
       </c>
       <c r="H85" s="6" t="inlineStr">
         <is>
-          <t>PASS (resolved 2026-08-10) — was ISSUE/Low: DESIGN-SYSTEM.md:115 listed "Reading progress bar (`var(--accent)`)" as a permitted accent use, but css/article.css:876 ships `.reading-progress { background: var(--ink) }`. Commit 68b0c1d (2026-04-10) recolored it on purpose and left the reason in the CSS: red was competing with the masthead and diluting the accent's semantic weight. That commit rewrote 136 lines of DESIGN-SYSTEM.md but missed this one bullet, which dated to c75ded9 earlier the same day. The CSS was correct; the doc line was stale. | 2026-08-27 second doc-parity pass (9b8e4c4): three more drifts closed, all doc-side. The Ghost Teaser Plate code block was pre-F90 and pre-cutover (min-height 346 vs the shipped 230; .plate-title opacity .35 vs .46/.40; --ink+opacity on .teaser-date and .meta-rail vs --body-muted), its prose still carried the static-HTML instruction 'swap for the full article plate and remove the ghost CSS from index.html', and the prev/next section claimed `next.ghost: true` drives 'the homepage's issue-next ghost CTA' — which conflated .article-nav-ghost with a component that no longer exists and was wrong before any of today's work. Also corrected a stale comment inside plates.css that justified a padding choice against '346px min-height' on a rule setting 230px — the same wrong number that had propagated into the doc. | 2026-09-11 re-verified live: permitted-accent list re-read; diff of css/ and brand/ from 2026-08-13 to HEAD adds ZERO new var(--accent) rules (two removals only). No new doc-vs-implementation drift.</t>
+          <t>PASS (resolved 2026-08-10) — was ISSUE/Low: DESIGN-SYSTEM.md:115 listed "Reading progress bar (`var(--accent)`)" as a permitted accent use, but css/article.css:876 ships `.reading-progress { background: var(--ink) }`. Commit 68b0c1d (2026-04-10) recolored it on purpose and left the reason in the CSS: red was competing with the masthead and diluting the accent's semantic weight. That commit rewrote 136 lines of DESIGN-SYSTEM.md but missed this one bullet, which dated to c75ded9 earlier the same day. The CSS was correct; the doc line was stale. | 2026-08-27 second doc-parity pass (9b8e4c4): three more drifts closed, all doc-side. The Ghost Teaser Plate code block was pre-F90 and pre-cutover (min-height 346 vs the shipped 230; .plate-title opacity .35 vs .46/.40; --ink+opacity on .teaser-date and .meta-rail vs --body-muted), its prose still carried the static-HTML instruction 'swap for the full article plate and remove the ghost CSS from index.html', and the prev/next section claimed `next.ghost: true` drives 'the homepage's issue-next ghost CTA' — which conflated .article-nav-ghost with a component that no longer exists and was wrong before any of today's work. Also corrected a stale comment inside plates.css that justified a padding choice against '346px min-height' on a rule setting 230px — the same wrong number that had propagated into the doc. | 2026-09-11 re-verified live: permitted-accent list re-read; diff of css/ and brand/ from 2026-08-13 to HEAD adds ZERO new var(--accent) rules (two removals only). No new doc-vs-implementation drift. | 2026-09-24 re-verified live: no css/ or DESIGN-SYSTEM.md change on main since the last PASS; the Permitted list still resolves to live accent rules (section-head h2 and rule, callout border, stat bar, plate hover border, focus ring). DESIGN-SYSTEM.md:148 edited today on the fix branch for F108 (names the third hover control and the sheet the override actually lives in, home-augment.css, per F87) — parity improved, not broken.</t>
         </is>
       </c>
       <c r="I85" s="6" t="inlineStr">
@@ -4902,7 +4910,7 @@
       </c>
       <c r="H86" s="6" t="inlineStr">
         <is>
-          <t>PASS (closed live 2026-08-13) — was ISSUE/High (2026-08-13) — CORRECTED SCOPE, and the correction matters. The morning scrub read the declarations and reported FOUR failing hover rules. Re-measured under REAL pointer hover before fixing, only TWO are real: `.issue-latest:hover .latest-cta` (14.08px/700) and `.identity-hero .hero-link.primary:hover` (14.08px/700), both `color: var(--bg)` on a `background: var(--accent)` fill = 3.44:1 in dark against a 4.5:1 floor. The other two were FALSE POSITIVES: `.issue-latest:hover` takes the BAR to var(--ink), not var(--accent), so .latest-title measures 17.79:1 and .latest-meta 5.23:1 (at opacity .6) against cream — both already clear. The morning read assumed the accent fill was the surface for every child of the hover state; it is only the surface for .latest-cta, which sets its own background. Lesson: resolve the PAINTED surface under real hover, never infer it from the parent's declarations. | 2026-08-25 re-verified live: re-verified under REAL pointer hover on the live homepage in dark mode: .latest-cta 5.17:1, .latest-tag 5.17:1, .latest-title 17.79:1, .latest-meta (hover state) 5.23:1. No regression. Caveat carried to F87: the override lives in home-v2.css on the live deploy, so /brand/ still does not get it. | 2026-09-18 re-verified live: dark mode under REAL pointer hover: .latest-cta 'Read →' and .hero-link.primary 'Read the About →' both cream 243,240,232 on #c00 = 5.17:1 at 14.08px.</t>
+          <t>PASS (closed live 2026-08-13) — was ISSUE/High (2026-08-13) — CORRECTED SCOPE, and the correction matters. The morning scrub read the declarations and reported FOUR failing hover rules. Re-measured under REAL pointer hover before fixing, only TWO are real: `.issue-latest:hover .latest-cta` (14.08px/700) and `.identity-hero .hero-link.primary:hover` (14.08px/700), both `color: var(--bg)` on a `background: var(--accent)` fill = 3.44:1 in dark against a 4.5:1 floor. The other two were FALSE POSITIVES: `.issue-latest:hover` takes the BAR to var(--ink), not var(--accent), so .latest-title measures 17.79:1 and .latest-meta 5.23:1 (at opacity .6) against cream — both already clear. The morning read assumed the accent fill was the surface for every child of the hover state; it is only the surface for .latest-cta, which sets its own background. Lesson: resolve the PAINTED surface under real hover, never infer it from the parent's declarations. | 2026-08-25 re-verified live: re-verified under REAL pointer hover on the live homepage in dark mode: .latest-cta 5.17:1, .latest-tag 5.17:1, .latest-title 17.79:1, .latest-meta (hover state) 5.23:1. No regression. Caveat carried to F87: the override lives in home-v2.css on the live deploy, so /brand/ still does not get it. | 2026-09-18 re-verified live: dark mode under REAL pointer hover: .latest-cta 'Read →' and .hero-link.primary 'Read the About →' both cream 243,240,232 on #c00 = 5.17:1 at 14.08px. | 2026-09-24 re-verified live: the two controls F83 fixed still pass under real pointer hover in dark mode: .latest-cta and .identity-hero .hero-link.primary both cream on #c00 at 5.17:1. BUT F83's scope note ('only the two controls below actually invert onto the accent fill on hover') was wrong: a.plate-lead:hover .rail-cta also inverts onto the accent and was missed — split out as F108, not counted as a regression of this row.</t>
         </is>
       </c>
       <c r="I86" s="6" t="inlineStr">
@@ -4959,7 +4967,7 @@
       </c>
       <c r="H87" s="6" t="inlineStr">
         <is>
-          <t>PASS (closed live 2026-08-13) — was ISSUE/Low (2026-08-13) — DESIGN-SYSTEM.md:124-130 lists 'Backgrounds' and 'Tags or metadata' as PROHIBITED accent uses, but .latest-tag is exactly that: a metadata tag with `background: var(--accent)`, shipped and prominent in the homepage standfirst bar. Companion to F82, which audited only the Permitted half of the same section and so could not have caught this. | 2026-09-11 re-verified live: prohibited-accent list re-read; same diff confirms no new background: var(--accent) rule since the .latest-tag annotation shipped. The sanctioned exception is still the only one.</t>
+          <t>PASS (closed live 2026-08-13) — was ISSUE/Low (2026-08-13) — DESIGN-SYSTEM.md:124-130 lists 'Backgrounds' and 'Tags or metadata' as PROHIBITED accent uses, but .latest-tag is exactly that: a metadata tag with `background: var(--accent)`, shipped and prominent in the homepage standfirst bar. Companion to F82, which audited only the Permitted half of the same section and so could not have caught this. | 2026-09-11 re-verified live: prohibited-accent list re-read; same diff confirms no new background: var(--accent) rule since the .latest-tag annotation shipped. The sanctioned exception is still the only one. | 2026-09-24 re-verified live: every background: var(--accent) rule enumerated (19 across 5 sheets): the only tag/metadata fills are .latest-tag (the annotated sanctioned exception) and .lead-badge-label (paired with --on-accent / #f5f5f1); the rest are rules, bars, dots, the manifesto panel and hover inversions. No unannotated prohibited use.</t>
         </is>
       </c>
       <c r="I87" s="6" t="inlineStr">
@@ -6273,8 +6281,65 @@
         </is>
       </c>
     </row>
+    <row r="111">
+      <c r="A111" s="4" t="inlineStr">
+        <is>
+          <t>F108</t>
+        </is>
+      </c>
+      <c r="B111" s="4" t="inlineStr">
+        <is>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C111" s="4" t="inlineStr">
+        <is>
+          <t>Dark-mode contrast of the lead plate's 'Read →' chip on hover</t>
+        </is>
+      </c>
+      <c r="D111" s="4" t="inlineStr">
+        <is>
+          <t>As a dark-mode reader hovering the lead essay plate, I want the 'Read →' chip to stay legible when it flips to the red fill, so the homepage's primary call to action doesn't drop below AA the moment I point at it.</t>
+        </is>
+      </c>
+      <c r="E111" s="4" t="inlineStr">
+        <is>
+          <t>a.plate-lead:hover .rail-cta (12px / 700 mono, background: var(--accent)) meets WCAG 1.4.3 &gt;= 4.5:1 in BOTH modes under real pointer hover; the dark-mode override lives in the shared home-augment.css with the other accent-fill hover overrides [F83/F87], so /brand/ gets it too.</t>
+        </is>
+      </c>
+      <c r="F111" s="4" t="inlineStr">
+        <is>
+          <t>css/home-augment.css:107-137,589; css/home-v2.css:393-411; src/components/home/LeadPlate.astro:34; src/layouts/HomeLayout.astro:84; brand/index.html:43; DESIGN-SYSTEM.md:148</t>
+        </is>
+      </c>
+      <c r="G111" s="5" t="inlineStr">
+        <is>
+          <t>Cataloged</t>
+        </is>
+      </c>
+      <c r="H111" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE/High (2026-09-24) — .rail-cta's base rule is background: var(--ink); color: var(--bg), and a.plate-lead:hover .rail-cta swaps only the background to var(--accent). In light mode that is cream on #c00 (#f4f4f1, ~5.2:1, passes). In dark mode --bg is #060606, so the hovered chip renders near-black 'READ →' on #c00 at 3.44:1 at 12px/700, under the 4.5:1 floor (WCAG 1.4.3). Measured under a REAL pointer hover after a 3s settle (a.plate-lead:hover true; computed rgb(6,6,6) on rgb(204,0,0)) and confirmed on screenshot. It is the same defect class F83 closed for .latest-cta and .hero-link.primary on 2026-08-13; F83's scope note said only those two controls invert onto the fill, which missed this third one. Present since the lead plate shipped (d1f8e7e, 2026-04-21), so NEW to the ledger, not a regression. /brand/ renders .plate-lead and loads home-augment.css, so it carries the same defect.</t>
+        </is>
+      </c>
+      <c r="I111" s="6" t="inlineStr">
+        <is>
+          <t>High (fixed)</t>
+        </is>
+      </c>
+      <c r="J111" s="4" t="inlineStr">
+        <is>
+          <t>FIX (qa/fixes-20260924): css/home-augment.css adds html.dark-mode a.plate-lead:hover .rail-cta to the existing F83 dark-mode override group (color: var(--ink), i.e. cream in dark), and the block's scope note now names three controls and records the miss. home-augment.css cache-bust phase34 -&gt; phase40 in src/layouts/HomeLayout.astro and brand/index.html (the sheet is served immutable for a year; without the bump returning readers keep the old copy). DESIGN-SYSTEM.md:148 names the third control and corrects the sheet the override lives in (home-augment.css, since F87).</t>
+        </is>
+      </c>
+      <c r="K111" s="6" t="inlineStr">
+        <is>
+          <t>PASS (2026-09-24, verified against build + rule injected on live) — npm run build clean; dist/css/home-augment.css carries the new selector; dist/index.html and dist/brand/index.html both reference home-augment.css?v=phase40. Dev servers cannot start in unattended runs, so the fix rule was applied to the live homepage with insertRule on the loaded home-augment sheet: dark mode, real pointer hover, a.plate-lead:hover true -&gt; .rail-cta rgb(243,240,232) on rgb(204,0,0) = 5.17:1 (screenshot shows a cream 'READ →'). deleteRule restored the sheet and a re-measure read 3.44:1 again, proving the page went back to its original state. Light-mode hover unchanged (rule is dark-scoped): rgb(244,244,241) on #c00. Sibling hover controls (.latest-cta, .hero-link.primary) re-measured 5.17:1, unaffected. Live-verifies on the first SCRUB after merge.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:K110"/>
+  <autoFilter ref="A3:K111"/>
   <mergeCells count="2">
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A1:K1"/>
@@ -6354,7 +6419,7 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="10">
@@ -6391,7 +6456,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16">
@@ -6407,7 +6472,7 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Total features: 107</t>
+          <t>Total features: 108</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
audit(ledger): 2026-09-25 scrub — clean site, F85-F94 rotation, F88 to N/A (surface retired)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -1546,7 +1546,7 @@
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>404 half PASS (noindex,nofollow live). Coming-soon half PENDING — no upcoming entry exists to render one | 2026-08-25: 404 half re-verified live (meta robots noindex,nofollow present, bespoke body served at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one. | 2026-09-01 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one. | 2026-09-11: 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body at HTTP 200). Coming-soon half still PENDING — 17 published entries, all past-dated, so isUpcomingData() is false everywhere and no ComingSoonLayout renders. | 2026-09-19: 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body, HTTP 404 on unmatched route). Coming-soon half still PENDING — 17 published entries, all past-dated; the untracked before-i-had-the-words.mdx in Dexter's working tree is still status 'drafted'. | 2026-09-23: 404 half re-verified live (noindex, nofollow). Coming-soon half still PENDING — 17/17 entries status published, no upcoming entry to render.</t>
+          <t>404 half PASS (noindex,nofollow live). Coming-soon half PENDING — no upcoming entry exists to render one | 2026-08-25: 404 half re-verified live (meta robots noindex,nofollow present, bespoke body served at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one. | 2026-09-01 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one. | 2026-09-11: 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body at HTTP 200). Coming-soon half still PENDING — 17 published entries, all past-dated, so isUpcomingData() is false everywhere and no ComingSoonLayout renders. | 2026-09-19: 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body, HTTP 404 on unmatched route). Coming-soon half still PENDING — 17 published entries, all past-dated; the untracked before-i-had-the-words.mdx in Dexter's working tree is still status 'drafted'. | 2026-09-23: 404 half re-verified live (noindex, nofollow). Coming-soon half still PENDING — 17/17 entries status published, no upcoming entry to render. | 2026-09-25: still PENDING — 17/17 entries status published and past-dated, no upcoming entry to render. 404 half re-verified live: meta robots noindex present, bespoke body, unmatched route 404.</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr"/>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
-          <t>Authored prev/next render correctly on all 16. Ghost/teaser path PENDING — requires a future-dated entry; none exists. 2026-08-10 PM: the derive-from-live-status fix (p3) live-verified, then the underlying data cleaned — the 4 stale ghost:true flags are gone (see F81). Zero `ghost: true` remain in the collection; all 16 essays render real .article-nav-link anchors, 15 rel=next head links (newest correctly has none), zero article-nav-ghost teasers. | 2026-08-25 re-verified live: all 16 essays render real .article-nav-link anchors; zero `ghost: true` remain in the collection. Ghost/teaser path still PENDING — still requires a future-dated entry and none exists. | 2026-09-11: authored prev/next re-verified live — newest essay emits rel=prev only, /words/the-stone/ emits rel=prev + rel=next. Ghost/teaser path still PENDING; zero upcoming entries in the collection. | 2026-09-19: authored prev/next unchanged (no code churn since 507e988). Ghost/teaser path still PENDING — zero upcoming entries in the collection. | 2026-09-23: authored prev/next unchanged (no code or content commits since 09-19). Ghost path still PENDING — no future-dated entry.</t>
+          <t xml:space="preserve">Authored prev/next render correctly on all 16. Ghost/teaser path PENDING — requires a future-dated entry; none exists. 2026-08-10 PM: the derive-from-live-status fix (p3) live-verified, then the underlying data cleaned — the 4 stale ghost:true flags are gone (see F81). Zero `ghost: true` remain in the collection; all 16 essays render real .article-nav-link anchors, 15 rel=next head links (newest correctly has none), zero article-nav-ghost teasers. | 2026-08-25 re-verified live: all 16 essays render real .article-nav-link anchors; zero `ghost: true` remain in the collection. Ghost/teaser path still PENDING — still requires a future-dated entry and none exists. | 2026-09-11: authored prev/next re-verified live — newest essay emits rel=prev only, /words/the-stone/ emits rel=prev + rel=next. Ghost/teaser path still PENDING; zero upcoming entries in the collection. | 2026-09-19: authored prev/next unchanged (no code churn since 507e988). Ghost/teaser path still PENDING — zero upcoming entries in the collection. | 2026-09-23: authored prev/next unchanged (no code or content commits since 09-19). Ghost path still PENDING — no future-dated entry. | 2026-09-25: still PENDING — 17/17 entries status published and past-dated, no upcoming entry to render. </t>
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr"/>
@@ -2937,7 +2937,7 @@
       </c>
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>PENDING — all 16 entries are status published with past dates, so isUpcomingData() is false everywhere and no coming-soon page renders | 2026-08-25: still PENDING for the same structural reason — all 16 built entries are status:published with past dates. NOTE: an untracked draft (src/content/words/before-i-had-the-words.mdx, status:"drafted", publishedDate 2026-08-07) sits in Dexter's working tree. It is correctly excluded from the build (19 pages, 16 articles) and does not exercise this path either, since its date is in the past, not the future. | 2026-09-01 still PENDING. The untracked draft in Dexter's working tree (src/content/words/before-i-had-the-words.mdx, status 'drafted', publishedDate 2026-08-07) is correctly excluded from the build (20 pages, 17 articles) but does NOT exercise this path — its date is in the past and its status is 'drafted', not an upcoming publish. Left untouched. | 2026-09-11: still PENDING for the same structural reason — 17 published entries, all past-dated. The untracked draft src/content/words/before-i-had-the-words.mdx is still status 'drafted' in Dexter's working tree, so it builds nothing and is correctly absent from sitemap and feed. | 2026-09-19: still PENDING for the same structural reason — no upcoming entry; the untracked draft is still 'drafted' and builds nothing. | 2026-09-23: still PENDING for the same structural reason — 17/17 entries published, isUpcomingData() false everywhere.</t>
+          <t xml:space="preserve">PENDING — all 16 entries are status published with past dates, so isUpcomingData() is false everywhere and no coming-soon page renders | 2026-08-25: still PENDING for the same structural reason — all 16 built entries are status:published with past dates. NOTE: an untracked draft (src/content/words/before-i-had-the-words.mdx, status:"drafted", publishedDate 2026-08-07) sits in Dexter's working tree. It is correctly excluded from the build (19 pages, 16 articles) and does not exercise this path either, since its date is in the past, not the future. | 2026-09-01 still PENDING. The untracked draft in Dexter's working tree (src/content/words/before-i-had-the-words.mdx, status 'drafted', publishedDate 2026-08-07) is correctly excluded from the build (20 pages, 17 articles) but does NOT exercise this path — its date is in the past and its status is 'drafted', not an upcoming publish. Left untouched. | 2026-09-11: still PENDING for the same structural reason — 17 published entries, all past-dated. The untracked draft src/content/words/before-i-had-the-words.mdx is still status 'drafted' in Dexter's working tree, so it builds nothing and is correctly absent from sitemap and feed. | 2026-09-19: still PENDING for the same structural reason — no upcoming entry; the untracked draft is still 'drafted' and builds nothing. | 2026-09-23: still PENDING for the same structural reason — 17/17 entries published, isUpcomingData() false everywhere. | 2026-09-25: still PENDING — 17/17 entries status published and past-dated, no upcoming entry to render. </t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr"/>
@@ -4743,7 +4743,7 @@
       </c>
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>PASS — parity 16/16 verified live; every /words/&lt;slug&gt; returns a single 301 to its trailing-slash canonical; no orphan rules | 2026-08-13 re-verified live: all 16 /words/&lt;slug&gt; (no trailing slash) return 301; all 16 /words/&lt;slug&gt;/ return 200 in 0.31-0.45s. | 2026-08-25 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-01 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-06 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-11 re-verified live: /words/&lt;slug&gt; → 301 → /words/&lt;slug&gt;/ → 200 verified on the-stone; all 17 article slugs 200 at their canonical form. | 2026-09-24 ISSUE/Low — the parity test the expected column defines, run for the first time since 2026-08-31, fails 16/17: the-weight-of-my-no (status published, 2026-08-31) has no [[redirects]] rule in netlify.toml. Every run since 08-31 spot-checked /words/the-stone only, so the drift went unseen for 24 days — the same shape as the July show-me-your-glory / send-someone-else drift. The expected column's 'non-slash 404s' premise did NOT hold: live /words/the-weight-of-my-no returns 301 -&gt; /words/the-weight-of-my-no/ with no rule, because Netlify Pretty URLs redirects a directory path on its own. No user impact observed; graded Low (parity/config drift, not a broken route).</t>
+          <t>PASS — parity 16/16 verified live; every /words/&lt;slug&gt; returns a single 301 to its trailing-slash canonical; no orphan rules | 2026-08-13 re-verified live: all 16 /words/&lt;slug&gt; (no trailing slash) return 301; all 16 /words/&lt;slug&gt;/ return 200 in 0.31-0.45s. | 2026-08-25 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-01 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-06 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-11 re-verified live: /words/&lt;slug&gt; → 301 → /words/&lt;slug&gt;/ → 200 verified on the-stone; all 17 article slugs 200 at their canonical form. | 2026-09-24 ISSUE/Low — the parity test the expected column defines, run for the first time since 2026-08-31, fails 16/17: the-weight-of-my-no (status published, 2026-08-31) has no [[redirects]] rule in netlify.toml. Every run since 08-31 spot-checked /words/the-stone only, so the drift went unseen for 24 days — the same shape as the July show-me-your-glory / send-someone-else drift. The expected column's 'non-slash 404s' premise did NOT hold: live /words/the-weight-of-my-no returns 301 -&gt; /words/the-weight-of-my-no/ with no rule, because Netlify Pretty URLs redirects a directory path on its own. No user impact observed; graded Low (parity/config drift, not a broken route). | 2026-09-25: live behaviour unchanged (single 301 via Pretty URLs); rule still only on the unmerged branch.</t>
         </is>
       </c>
       <c r="I83" s="6" t="inlineStr">
@@ -5024,7 +5024,7 @@
       </c>
       <c r="H88" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-08-15) — `.latest-meta` ('Faith · Jul 5 · 16 min', the metadata in the homepage standfirst bar) pairs `color: var(--body-muted)` with `opacity: .75`. --body-muted is ALREADY an alpha colour (rgba(243,240,232,.52) dark / rgba(5,5,5,.56) light), tuned to land just over AA on its own — 5.13:1 dark, 4.67:1 light. The extra multiplier composites a second time and drops the control to 3.36:1 dark / 2.93:1 light, under the 4.5:1 floor for 11.52px/400 text. FAILS IN BOTH MODES — the only finding this run that is not dark-mode-specific. Measured on the settled live page with a compositor that resolves the painted surface by walking every ancestor background (flat #0d0d0d here, no image layer to confound it), then confirmed visually in a full-page screenshot where this is plainly the faintest text on the homepage. Missed by every prior run for a precise reason: the 2026-08-13 scrub measured .latest-meta ONLY under pointer hover, where `.issue-latest:hover .latest-meta` re-declares `color: var(--bg); opacity: .6` against the cream hover bar and clears at 5.23:1. F83 recorded that number and closed the question. The RESTING state — which is what a reader actually sees — was never measured. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: `.latest-meta` 3.36:1 dark / 2.93:1 light on the homepage, and 3.36:1 again on /brand/. Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | .latest-meta re-measured live 2026-08-25: 3.36:1 dark (homepage + /brand/), 2.93:1 light — unchanged from 2026-08-15. Root cause of the non-closure is NOT the fix: it is that the fix never shipped. origin/main is still b64a39b; the F85 commit (55a6d72) sits on LOCAL main, 8 commits ahead of origin, unpushed for 9 days. | RESOLVED LIVE 2026-08-27 — see p4.</t>
+          <t>ISSUE/High (2026-08-15) — `.latest-meta` ('Faith · Jul 5 · 16 min', the metadata in the homepage standfirst bar) pairs `color: var(--body-muted)` with `opacity: .75`. --body-muted is ALREADY an alpha colour (rgba(243,240,232,.52) dark / rgba(5,5,5,.56) light), tuned to land just over AA on its own — 5.13:1 dark, 4.67:1 light. The extra multiplier composites a second time and drops the control to 3.36:1 dark / 2.93:1 light, under the 4.5:1 floor for 11.52px/400 text. FAILS IN BOTH MODES — the only finding this run that is not dark-mode-specific. Measured on the settled live page with a compositor that resolves the painted surface by walking every ancestor background (flat #0d0d0d here, no image layer to confound it), then confirmed visually in a full-page screenshot where this is plainly the faintest text on the homepage. Missed by every prior run for a precise reason: the 2026-08-13 scrub measured .latest-meta ONLY under pointer hover, where `.issue-latest:hover .latest-meta` re-declares `color: var(--bg); opacity: .6` against the cream hover bar and clears at 5.23:1. F83 recorded that number and closed the question. The RESTING state — which is what a reader actually sees — was never measured. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: `.latest-meta` 3.36:1 dark / 2.93:1 light on the homepage, and 3.36:1 again on /brand/. Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | .latest-meta re-measured live 2026-08-25: 3.36:1 dark (homepage + /brand/), 2.93:1 light — unchanged from 2026-08-15. Root cause of the non-closure is NOT the fix: it is that the fix never shipped. origin/main is still b64a39b; the F85 commit (55a6d72) sits on LOCAL main, 8 commits ahead of origin, unpushed for 9 days. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live: .latest-meta 5.13:1 dark / 4.67:1 light, opacity 1 (no stacked multiplier). Also 5.13 on /brand/ dark.</t>
         </is>
       </c>
       <c r="I88" s="6" t="inlineStr">
@@ -5081,7 +5081,7 @@
       </c>
       <c r="H89" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-08-15) — `.hero-corner` sets `color: var(--bg); opacity: .5`. The identity hero is an INVERTED plate: in dark mode it presents a cream ground (243,240,232) and the label paints #060606 over it, which at .5 opacity computes 3.71:1 — under the 4.5:1 floor for 11.52px/700 (bold, but well below the 18.66px large-text threshold). Light mode inverts to cream-on-black and clears at 4.91:1, so this is dark-mode-only. Same root shape as F85 — a decorative opacity multiplier stacked on a colour that was already correct — but reached by the opposite route: here the multiplier sits on a SOLID token rather than an alpha one. Surface resolved by walking to the first opaque ancestor (.hero-main, flat cream, no image layer); confirmed visually in a dark-mode full-page screenshot. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: `.hero-corner` 3.71:1 dark on the homepage, and 3.71:1 again on /brand/. Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | .hero-corner re-measured live 2026-08-25: 3.71:1 dark. Unchanged — fix committed locally (55a6d72), never pushed. | RESOLVED LIVE 2026-08-27 — see p4.</t>
+          <t>ISSUE/High (2026-08-15) — `.hero-corner` sets `color: var(--bg); opacity: .5`. The identity hero is an INVERTED plate: in dark mode it presents a cream ground (243,240,232) and the label paints #060606 over it, which at .5 opacity computes 3.71:1 — under the 4.5:1 floor for 11.52px/700 (bold, but well below the 18.66px large-text threshold). Light mode inverts to cream-on-black and clears at 4.91:1, so this is dark-mode-only. Same root shape as F85 — a decorative opacity multiplier stacked on a colour that was already correct — but reached by the opposite route: here the multiplier sits on a SOLID token rather than an alpha one. Surface resolved by walking to the first opaque ancestor (.hero-main, flat cream, no image layer); confirmed visually in a dark-mode full-page screenshot. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: `.hero-corner` 3.71:1 dark on the homepage, and 3.71:1 again on /brand/. Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | .hero-corner re-measured live 2026-08-25: 3.71:1 dark. Unchanged — fix committed locally (55a6d72), never pushed. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live: .identity-hero .hero-corner 5.23:1 dark / 6.74:1 light at opacity .6.</t>
         </is>
       </c>
       <c r="I89" s="6" t="inlineStr">
@@ -5138,7 +5138,7 @@
       </c>
       <c r="H90" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-08-15) — /brand/ was still rendering `.latest-tag` at 3.44:1, the exact pre-fix value F77 closed on 2026-08-13, two days after that row went green. Cause: the F77 and F83 dark-mode overrides were written into css/home-v2.css. The homepage loads home-augment.css AND home-v2.css; /brand/ loads home-augment.css and never home-v2.css. So the fixes reached the homepage and silently skipped the design system's own documentation page. This is a broken contract, not a cosmetic gap: brand/index.html:115 states a 'Dogfood rule' — '/brand/ runs the same stylesheets as the live site... If a live component breaks, this page breaks too. That is intentional.' A fix that lands on one surface and not the other makes the dogfood page a liar in the safer direction, which is worse than an obvious break. The F77 comment even asserted it 'Covers the .issue-head hook in home-augment.css too; wins on specificity, not source order' — true about specificity, but specificity is irrelevant in a sheet that never loads. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: /brand/ `.latest-tag` 3.44:1 — and /brand/'s loaded-sheet list confirms the cause directly: tokens, shell, plates, home-augment, article, brand.css, with NO home-v2.css. Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | /brand/ re-measured live 2026-08-25: .latest-tag still 3.44:1 (the pre-F77 value), because live /brand/ serves home-augment.css?v=phase32 which does not yet carry the moved override blocks. The move (55a6d72) is committed locally and confirmed present in a fresh dist build; it has never been pushed. | RESOLVED LIVE 2026-08-27 — see p4.</t>
+          <t>ISSUE/High (2026-08-15) — /brand/ was still rendering `.latest-tag` at 3.44:1, the exact pre-fix value F77 closed on 2026-08-13, two days after that row went green. Cause: the F77 and F83 dark-mode overrides were written into css/home-v2.css. The homepage loads home-augment.css AND home-v2.css; /brand/ loads home-augment.css and never home-v2.css. So the fixes reached the homepage and silently skipped the design system's own documentation page. This is a broken contract, not a cosmetic gap: brand/index.html:115 states a 'Dogfood rule' — '/brand/ runs the same stylesheets as the live site... If a live component breaks, this page breaks too. That is intentional.' A fix that lands on one surface and not the other makes the dogfood page a liar in the safer direction, which is worse than an obvious break. The F77 comment even asserted it 'Covers the .issue-head hook in home-augment.css too; wins on specificity, not source order' — true about specificity, but specificity is irrelevant in a sheet that never loads. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: /brand/ `.latest-tag` 3.44:1 — and /brand/'s loaded-sheet list confirms the cause directly: tokens, shell, plates, home-augment, article, brand.css, with NO home-v2.css. Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | /brand/ re-measured live 2026-08-25: .latest-tag still 3.44:1 (the pre-F77 value), because live /brand/ serves home-augment.css?v=phase32 which does not yet carry the moved override blocks. The move (55a6d72) is committed locally and confirmed present in a fresh dist build; it has never been pushed. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live: /brand/ loads home-augment.css?v=phase34 (not home-v2); .latest-tag 5.17:1 dark / 5.34:1 light, identical to the homepage — dogfood contract holds.</t>
         </is>
       </c>
       <c r="I90" s="6" t="inlineStr">
@@ -5195,14 +5195,10 @@
       </c>
       <c r="H91" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-08-15) — `.next-meta` repeats the F85 defect one notch worse: `color: var(--body-muted)` plus `opacity: .65`, computing 2.81:1 in dark against the 4.5:1 floor. Graded MEDIUM rather than HIGH because it is LATENT — the Issue-next strip only renders when an upcoming essay exists, and all 16 entries are status:published with past dates (see F41/F46), so no reader has hit it. It was found because /brand/ demos the strip under its dogfood rule, which is the same page that exposed F87. Worth recording precisely: this would have shipped broken on the day Dexter scheduled his next essay, and it would have shipped inside the one component whose whole job is to advertise that essay. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: `.next-meta` 2.81:1 dark on the /brand/ dogfood demo (still latent on the live homepage — no upcoming essay exists). Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | .next-meta re-measured on the /brand/ demo of the strip 2026-08-25: still 2.81:1 dark. Unchanged — fix committed locally (55a6d72), never pushed. Still latent on the homepage itself: zero ghost:true flags remain in the collection and no upcoming entry exists, so IssueNext does not render. | RESOLVED LIVE 2026-08-27 — see p4.</t>
-        </is>
-      </c>
-      <c r="I91" s="6" t="inlineStr">
-        <is>
-          <t>MEDIUM (closed at source) (resolved)</t>
-        </is>
-      </c>
+          <t>N/A — surface retired | ISSUE/Medium (2026-08-15) — `.next-meta` repeats the F85 defect one notch worse: `color: var(--body-muted)` plus `opacity: .65`, computing 2.81:1 in dark against the 4.5:1 floor. Graded MEDIUM rather than HIGH because it is LATENT — the Issue-next strip only renders when an upcoming essay exists, and all 16 entries are status:published with past dates (see F41/F46), so no reader has hit it. It was found because /brand/ demos the strip under its dogfood rule, which is the same page that exposed F87. Worth recording precisely: this would have shipped broken on the day Dexter scheduled his next essay, and it would have shipped inside the one component whose whole job is to advertise that essay. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: `.next-meta` 2.81:1 dark on the /brand/ dogfood demo (still latent on the live homepage — no upcoming essay exists). Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | .next-meta re-measured on the /brand/ demo of the strip 2026-08-25: still 2.81:1 dark. Unchanged — fix committed locally (55a6d72), never pushed. Still latent on the homepage itself: zero ghost:true flags remain in the collection and no upcoming entry exists, so IssueNext does not render. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: marked N/A per the never-delete rule. The `.issue-next` strip this row measured was deleted in e3b4e91 (IssueNext.astro removed, ~200 lines of .issue-next CSS removed from home-v2.css + home-augment.css). Live: zero `.next-meta` in home-v2.css?v=phase36 / home-augment.css?v=phase34, zero `.issue-next` in the homepage DOM, /brand/ shows only the retirement note. Nothing left to measure; F30 carries the regression watch.</t>
+        </is>
+      </c>
+      <c r="I91" s="6" t="inlineStr"/>
       <c r="J91" s="4" t="inlineStr">
         <is>
           <t>FIX (qa/fixes-20260815): deleted `opacity: .65` from `.issue-next .next-meta` in both css/home-v2.css and css/home-augment.css, same treatment and same reasoning as F85.</t>
@@ -5252,7 +5248,7 @@
       </c>
       <c r="H92" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-08-15) — the `·` separators in the 404 eyebrow carry `opacity: .5`, computing 3.61:1. Unlike the homepage's `.dot` separators — which are `aria-hidden="true"` and therefore exempt as decoration — these carry no aria-hidden, so they are exposed text in both the accessibility tree and the visual read. Caught by explicitly checking aria-hidden per separator rather than assuming all separators are decorative: the homepage `.dot` at 4.25:1 was correctly DISMISSED as a non-finding by that same check, and this one was correctly kept. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: `.notfound-eyebrow span.divider` 3.61:1 on /404. Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | /404 span.divider re-measured live 2026-08-25: still 3.61:1 at opacity .5; live serves notfound.css?v=phase10 (the fix bumps it to phase11). Fix committed locally (8c1e6aa), never pushed. | RESOLVED LIVE 2026-08-27 — see p4.</t>
+          <t>ISSUE/Medium (2026-08-15) — the `·` separators in the 404 eyebrow carry `opacity: .5`, computing 3.61:1. Unlike the homepage's `.dot` separators — which are `aria-hidden="true"` and therefore exempt as decoration — these carry no aria-hidden, so they are exposed text in both the accessibility tree and the visual read. Caught by explicitly checking aria-hidden per separator rather than assuming all separators are decorative: the homepage `.dot` at 4.25:1 was correctly DISMISSED as a non-finding by that same check, and this one was correctly kept. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: `.notfound-eyebrow span.divider` 3.61:1 on /404. Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | /404 span.divider re-measured live 2026-08-25: still 3.61:1 at opacity .5; live serves notfound.css?v=phase10 (the fix bumps it to phase11). Fix committed locally (8c1e6aa), never pushed. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live: /404 .notfound-eyebrow span.divider 7.19:1 dark / 8.95:1 light; still not aria-hidden (exposed text, in scope).</t>
         </is>
       </c>
       <c r="I92" s="6" t="inlineStr">
@@ -5309,7 +5305,7 @@
       </c>
       <c r="H93" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Low (2026-08-15) — five /brand/-only text elements measure under AA in dark mode: `.demo-ghost-meta` ('Coming Soon') 2.05:1, `.demo-ghost-date` 2.45:1, `.demo-ghost-title` 2.93:1 (against its 3:1 large-text floor), `.demo-plate-meta` 3.17:1, and the bespoke 'Download Pack' h3 at 2.87:1. Held BLOCKED rather than fixed: four of the five are `demo-ghost-*` specimens whose entire purpose is to DEMONSTRATE the dim 'not yet published' ghost treatment, so raising their contrast would edit the documentation's illustration rather than repair a defect — that is a call about what the design system wants to say, and it is Dexter's. The fifth ('Download Pack') is bespoke brand.css chrome and is a genuine, if low-traffic, AA miss. Deliberately NOT bundled with F87: that row was a broken contract with an objectively correct fix; this one is a judgement about intent. | 2026-08-16 LIVE RE-CHECK: still open and still BLOCKED — unchanged by design. Re-measured on live /brand/: `.demo-ghost-meta` 2.05:1 and `.demo-plate-meta` 3.17:1 both reproduce exactly. The other three named elements (demo-ghost-date, demo-ghost-title, the 'Download Pack' h3) did not surface in today's sweep because this run only measures elements holding their own text node and not inside an aria-hidden subtree; that is a narrower filter than the 2026-08-15 pass used, not evidence they were fixed. Still NEEDS DEXTER on both questions. | Re-confirmed live 2026-08-25, all five values unchanged: .demo-ghost-meta 2.05:1, .demo-ghost-date 2.45:1, .demo-ghost-title 2.93:1 (vs its 3:1 large-text floor), .demo-plate-meta 3.17:1, and the bespoke "Download Pack" h3 2.87:1 (#ff4d4d on the cream panel). Still BLOCKED — still the same two questions for Dexter, now open 10 days. | 2026-08-27 RE-DIAGNOSED, and the premise of this row was wrong. Four of the five are not documentation-intent choices at all — `.demo-ghost-title/-date/-meta` and `.demo-plate-meta` are faithful mirrors of `.plate-ghost` and `.identity-plate` in css/plates.css, carrying the same tokens and the same opacity multipliers. Composited against their real grounds those production rules measure .plate-title 2.92:1 light / 2.84:1 dark (3:1 large-text floor), .teaser-date 2.06/2.37, `.plate-ghost .meta-rail` 1.80/1.97, and `.identity-plate .meta-rail` 4.14/4.09 (4.5:1 floor) — every one under AA. css/plates.css:377-380 carried a comment asserting these values PASSED ("3.1:1 on #f4f4f1", "3.7:1 on #060606"); both figures are wrong and are what kept the defect invisible. The fifth, the /brand/ 'Download Pack' h3, is worse than recorded: it fails in BOTH modes (2.87:1 dark, 3.46:1 light), not just dark. Separately found: the /brand/ identity specimen had drifted — it used var(--ink)/var(--bg), which invert, so in dark mode it rendered a CREAM identity plate while production deliberately holds #0a0a0a. | RESOLVED LIVE 2026-08-27 — see p4.</t>
+          <t>ISSUE/Low (2026-08-15) — five /brand/-only text elements measure under AA in dark mode: `.demo-ghost-meta` ('Coming Soon') 2.05:1, `.demo-ghost-date` 2.45:1, `.demo-ghost-title` 2.93:1 (against its 3:1 large-text floor), `.demo-plate-meta` 3.17:1, and the bespoke 'Download Pack' h3 at 2.87:1. Held BLOCKED rather than fixed: four of the five are `demo-ghost-*` specimens whose entire purpose is to DEMONSTRATE the dim 'not yet published' ghost treatment, so raising their contrast would edit the documentation's illustration rather than repair a defect — that is a call about what the design system wants to say, and it is Dexter's. The fifth ('Download Pack') is bespoke brand.css chrome and is a genuine, if low-traffic, AA miss. Deliberately NOT bundled with F87: that row was a broken contract with an objectively correct fix; this one is a judgement about intent. | 2026-08-16 LIVE RE-CHECK: still open and still BLOCKED — unchanged by design. Re-measured on live /brand/: `.demo-ghost-meta` 2.05:1 and `.demo-plate-meta` 3.17:1 both reproduce exactly. The other three named elements (demo-ghost-date, demo-ghost-title, the 'Download Pack' h3) did not surface in today's sweep because this run only measures elements holding their own text node and not inside an aria-hidden subtree; that is a narrower filter than the 2026-08-15 pass used, not evidence they were fixed. Still NEEDS DEXTER on both questions. | Re-confirmed live 2026-08-25, all five values unchanged: .demo-ghost-meta 2.05:1, .demo-ghost-date 2.45:1, .demo-ghost-title 2.93:1 (vs its 3:1 large-text floor), .demo-plate-meta 3.17:1, and the bespoke "Download Pack" h3 2.87:1 (#ff4d4d on the cream panel). Still BLOCKED — still the same two questions for Dexter, now open 10 days. | 2026-08-27 RE-DIAGNOSED, and the premise of this row was wrong. Four of the five are not documentation-intent choices at all — `.demo-ghost-title/-date/-meta` and `.demo-plate-meta` are faithful mirrors of `.plate-ghost` and `.identity-plate` in css/plates.css, carrying the same tokens and the same opacity multipliers. Composited against their real grounds those production rules measure .plate-title 2.92:1 light / 2.84:1 dark (3:1 large-text floor), .teaser-date 2.06/2.37, `.plate-ghost .meta-rail` 1.80/1.97, and `.identity-plate .meta-rail` 4.14/4.09 (4.5:1 floor) — every one under AA. css/plates.css:377-380 carried a comment asserting these values PASSED ("3.1:1 on #f4f4f1", "3.7:1 on #060606"); both figures are wrong and are what kept the defect invisible. The fifth, the /brand/ 'Download Pack' h3, is worse than recorded: it fails in BOTH modes (2.87:1 dark, 3.46:1 light), not just dark. Separately found: the /brand/ identity specimen had drifted — it used var(--ink)/var(--bg), which invert, so in dark mode it rendered a CREAM identity plate while production deliberately holds #0a0a0a. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live: /brand/ demo specimens clear their floors in both modes — .demo-ghost-meta 5.13/4.67, .demo-ghost-date 5.13/4.67, .demo-ghost-title 3.48/3.33 (44.8px, 3:1 floor), .demo-plate-meta 18.11; full-page sweep 793 elements per mode, 0 failures; img-plate bodies flex/flex-end.</t>
         </is>
       </c>
       <c r="I93" s="6" t="inlineStr">
@@ -5366,7 +5362,7 @@
       </c>
       <c r="H94" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-08-16) — /phase0/'s skip link, the first focusable element on the page, computed `color: rgba(243,240,232,.82)` on its own `background: var(--ink)` cream chip: 1.00:1. This is the worst ratio the ledger has recorded and the only finding to date where the text is not merely low-contrast but literally invisible — a sighted keyboard user sees the accent focus ring land on a blank cream box. NOT a colour bug: `--bg` resolves correctly to #060606 at every level of the chain (verified by walking the ancestor chain: A.skip-link / BODY.phase0 / HTML.dark-mode all report #060606). It is a specificity bug. Three rules set colour on this element — `a {color:inherit}` (0,0,1) in tokens.css, `.skip-link {color:var(--bg)}` (0,1,0) in shell.css, and `.phase0 a {color:inherit}` (0,1,1) in phase0.css. The last wins on specificity and hands the chip back the inherited body cream. Scope is exactly one page: /brand/, the other bespoke-CSS surface, carries no blanket `a` rule and measured clean. Missed by every prior run because the skip link sits at left:-999px in its resting state, so a sweep that filters to on-screen elements never measures it — this run caught it by measuring every element with layout geometry regardless of viewport position. | /phase0/ skip link re-measured live 2026-08-25: still rgba(243,240,232,.82) on its own cream chip = 1.00:1, the worst ratio in the ledger and still literally invisible to a sighted keyboard user. Live serves shell.css?v=phase23; the hardened selector ships as phase36. Fix committed locally (79df261), never pushed. | RESOLVED LIVE 2026-08-27 — see p4.</t>
+          <t>ISSUE/High (2026-08-16) — /phase0/'s skip link, the first focusable element on the page, computed `color: rgba(243,240,232,.82)` on its own `background: var(--ink)` cream chip: 1.00:1. This is the worst ratio the ledger has recorded and the only finding to date where the text is not merely low-contrast but literally invisible — a sighted keyboard user sees the accent focus ring land on a blank cream box. NOT a colour bug: `--bg` resolves correctly to #060606 at every level of the chain (verified by walking the ancestor chain: A.skip-link / BODY.phase0 / HTML.dark-mode all report #060606). It is a specificity bug. Three rules set colour on this element — `a {color:inherit}` (0,0,1) in tokens.css, `.skip-link {color:var(--bg)}` (0,1,0) in shell.css, and `.phase0 a {color:inherit}` (0,1,1) in phase0.css. The last wins on specificity and hands the chip back the inherited body cream. Scope is exactly one page: /brand/, the other bespoke-CSS surface, carries no blanket `a` rule and measured clean. Missed by every prior run because the skip link sits at left:-999px in its resting state, so a sweep that filters to on-screen elements never measures it — this run caught it by measuring every element with layout geometry regardless of viewport position. | /phase0/ skip link re-measured live 2026-08-25: still rgba(243,240,232,.82) on its own cream chip = 1.00:1, the worst ratio in the ledger and still literally invisible to a sighted keyboard user. Live serves shell.css?v=phase23; the hardened selector ships as phase36. Fix committed locally (79df261), never pushed. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live under a real shift+Tab: /phase0/ skip link is first focusable, rgb(6,6,6) on rgb(243,240,232) = 17.79:1 dark; light rgb(244,244,241) on rgb(5,5,5); 2px #c00 ring. Homepage skip link same, activation lands focus on MAIN#archive.</t>
         </is>
       </c>
       <c r="I94" s="6" t="inlineStr">
@@ -5423,7 +5419,7 @@
       </c>
       <c r="H95" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Low (2026-08-27) — the click handler rewrote the label and the count but never touched the glyph. Live on b64a39b the expanded state reads 'Show Less — showing all ↓': the arrow still points down, i.e. 'more below', while the button's own words say it will collapse. The glyph carries aria-hidden="true" so nothing is exposed to assistive tech — this is a purely visual affordance contradiction, which is why it survived every prior scrub. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-01 re-verified live: .btn-glyph tracks the button state — down-arrow collapsed, up-arrow expanded, and back. | 2026-09-11 re-verified live: glyph tracks state live — ↓ at 7 shown, ↑ at 17 shown, back to ↓; still aria-hidden. | 2026-09-19 re-verified live: View Earlier toggle: 7 shown / aria-expanded false / ↓ → 17 shown / true / ↑ → back to 7 / false.</t>
+          <t>ISSUE/Low (2026-08-27) — the click handler rewrote the label and the count but never touched the glyph. Live on b64a39b the expanded state reads 'Show Less — showing all ↓': the arrow still points down, i.e. 'more below', while the button's own words say it will collapse. The glyph carries aria-hidden="true" so nothing is exposed to assistive tech — this is a purely visual affordance contradiction, which is why it survived every prior scrub. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-01 re-verified live: .btn-glyph tracks the button state — down-arrow collapsed, up-arrow expanded, and back. | 2026-09-11 re-verified live: glyph tracks state live — ↓ at 7 shown, ↑ at 17 shown, back to ↓; still aria-hidden. | 2026-09-19 re-verified live: View Earlier toggle: 7 shown / aria-expanded false / ↓ → 17 shown / true / ↑ → back to 7 / false. | 2026-09-25: re-verified live: 7 shown / aria-expanded false / ↓ → 17 shown / true / ↑ → back to 7 / false; glyph aria-hidden.</t>
         </is>
       </c>
       <c r="I95" s="6" t="inlineStr">
@@ -5480,7 +5476,7 @@
       </c>
       <c r="H96" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-08-27) — both class names are DEAD in production. `Plate.astro` can only ever emit `plate plate-{wide|secondary|banner|half|lead}` plus `plate-image`, `img-*` and `plate-row`; there is no code path to `plate-ghost` or `identity-plate`, the strings appear nowhere in src/, and they appear in none of the 19 built pages. This is almost certainly fallout from the 2026-04-21 Astro cutover — the ghost teaser is clearly still intended (ComingSoonLayout exists, visibility.ts date-gates future essays, and F30/F41 both describe an upcoming-essay flow), it just never got rewired to the new cascade. Two consequences: css/plates.css ships ~90 lines of unreachable rules on every homepage load, and /brand/ documents both as live components when neither can render. Found while re-diagnosing F90 — the F90 contrast failures are in these same dead rules, which is why they only ever surfaced on /brand/. | Dexter chose REWIRE over retire, 2026-08-27. | RESOLVED 2026-08-27 — see p4. | CORRECTION 2026-08-27: this row was closed as 'fixed' while it named TWO orphaned components and only ONE was rewired. `.plate-ghost` has an emitter now; `.identity-plate` still has none — no occurrence anywhere in src/, zero in the 19 built pages. F93 is hereby narrowed to the ghost plate, which is genuinely fixed, and the identity-plate half is split out to F95 so it is not buried under a green row. My closure, my error.</t>
+          <t>ISSUE/Medium (2026-08-27) — both class names are DEAD in production. `Plate.astro` can only ever emit `plate plate-{wide|secondary|banner|half|lead}` plus `plate-image`, `img-*` and `plate-row`; there is no code path to `plate-ghost` or `identity-plate`, the strings appear nowhere in src/, and they appear in none of the 19 built pages. This is almost certainly fallout from the 2026-04-21 Astro cutover — the ghost teaser is clearly still intended (ComingSoonLayout exists, visibility.ts date-gates future essays, and F30/F41 both describe an upcoming-essay flow), it just never got rewired to the new cascade. Two consequences: css/plates.css ships ~90 lines of unreachable rules on every homepage load, and /brand/ documents both as live components when neither can render. Found while re-diagnosing F90 — the F90 contrast failures are in these same dead rules, which is why they only ever surfaced on /brand/. | Dexter chose REWIRE over retire, 2026-08-27. | RESOLVED 2026-08-27 — see p4. | CORRECTION 2026-08-27: this row was closed as 'fixed' while it named TWO orphaned components and only ONE was rewired. `.plate-ghost` has an emitter now; `.identity-plate` still has none — no occurrence anywhere in src/, zero in the 19 built pages. F93 is hereby narrowed to the ghost plate, which is genuinely fixed, and the identity-plate half is split out to F95 so it is not buried under a green row. My closure, my error. | 2026-09-25: static re-check: GhostPlate.astro still emits .plate-ghost; plates.css?v=phase39 carries the rules. Live render still untestable (0 upcoming entries), so no live claim.</t>
         </is>
       </c>
       <c r="I96" s="6" t="inlineStr">
@@ -5537,7 +5533,7 @@
       </c>
       <c r="H97" s="6" t="inlineStr">
         <is>
-          <t>N/A by decision (2026-08-27) — not a defect. Dexter's call after seeing F93 ship: the ghost plate and the IssueNext strip are two presentations of the same upcoming essay, so with both live the title appeared on the homepage twice. The plate wins.</t>
+          <t>N/A by decision (2026-08-27) — not a defect. Dexter's call after seeing F93 ship: the ghost plate and the IssueNext strip are two presentations of the same upcoming essay, so with both live the title appeared on the homepage twice. The plate wins. | 2026-09-25: still N/A by decision. Note: the expected column's "component and CSS stay intact" was overtaken the same day by e3b4e91, which deleted IssueNext.astro and its CSS; reversal now means restoring from git (121a621), not a one-line flip. Live: 0 .issue-next in DOM/CSS.</t>
         </is>
       </c>
       <c r="I97" s="6" t="inlineStr"/>
@@ -6319,7 +6315,7 @@
       </c>
       <c r="H111" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-09-24) — .rail-cta's base rule is background: var(--ink); color: var(--bg), and a.plate-lead:hover .rail-cta swaps only the background to var(--accent). In light mode that is cream on #c00 (#f4f4f1, ~5.2:1, passes). In dark mode --bg is #060606, so the hovered chip renders near-black 'READ →' on #c00 at 3.44:1 at 12px/700, under the 4.5:1 floor (WCAG 1.4.3). Measured under a REAL pointer hover after a 3s settle (a.plate-lead:hover true; computed rgb(6,6,6) on rgb(204,0,0)) and confirmed on screenshot. It is the same defect class F83 closed for .latest-cta and .hero-link.primary on 2026-08-13; F83's scope note said only those two controls invert onto the fill, which missed this third one. Present since the lead plate shipped (d1f8e7e, 2026-04-21), so NEW to the ledger, not a regression. /brand/ renders .plate-lead and loads home-augment.css, so it carries the same defect.</t>
+          <t>ISSUE/High (2026-09-24) — .rail-cta's base rule is background: var(--ink); color: var(--bg), and a.plate-lead:hover .rail-cta swaps only the background to var(--accent). In light mode that is cream on #c00 (#f4f4f1, ~5.2:1, passes). In dark mode --bg is #060606, so the hovered chip renders near-black 'READ →' on #c00 at 3.44:1 at 12px/700, under the 4.5:1 floor (WCAG 1.4.3). Measured under a REAL pointer hover after a 3s settle (a.plate-lead:hover true; computed rgb(6,6,6) on rgb(204,0,0)) and confirmed on screenshot. It is the same defect class F83 closed for .latest-cta and .hero-link.primary on 2026-08-13; F83's scope note said only those two controls invert onto the fill, which missed this third one. Present since the lead plate shipped (d1f8e7e, 2026-04-21), so NEW to the ledger, not a regression. /brand/ renders .plate-lead and loads home-augment.css, so it carries the same defect. | 2026-09-25: still present LIVE — live home-augment.css is phase34 without the rule; fix sits on the unmerged stacked branch (now qa/fixes-20260925). Awaiting Dexter's merge; not re-counted as new.</t>
         </is>
       </c>
       <c r="I111" s="6" t="inlineStr">
@@ -6392,7 +6388,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -6456,7 +6452,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
audit(ledger): 2026-09-26 scrub — clean site, F95-F104 rotation all PASS, F80 full parity 17/17
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -1553,7 +1553,7 @@
       <c r="J22" s="4" t="inlineStr"/>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t>PENDING | 2026-09-18: still structurally untestable — 0 upcoming entries in the committed collection.</t>
+          <t>PENDING | 2026-09-18: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-26: still structurally untestable — 0 upcoming entries in the committed collection.</t>
         </is>
       </c>
     </row>
@@ -2687,7 +2687,7 @@
       </c>
       <c r="K44" s="6" t="inlineStr">
         <is>
-          <t>PENDING | 2026-09-18: still structurally untestable — 0 upcoming entries in the committed collection.</t>
+          <t>PENDING | 2026-09-18: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-26: still structurally untestable — 0 upcoming entries in the committed collection.</t>
         </is>
       </c>
     </row>
@@ -2948,7 +2948,7 @@
       </c>
       <c r="K49" s="6" t="inlineStr">
         <is>
-          <t>PENDING | 2026-09-18: still structurally untestable — 0 upcoming entries in the committed collection.</t>
+          <t>PENDING | 2026-09-18: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-26: still structurally untestable — 0 upcoming entries in the committed collection.</t>
         </is>
       </c>
     </row>
@@ -4743,7 +4743,7 @@
       </c>
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>PASS — parity 16/16 verified live; every /words/&lt;slug&gt; returns a single 301 to its trailing-slash canonical; no orphan rules | 2026-08-13 re-verified live: all 16 /words/&lt;slug&gt; (no trailing slash) return 301; all 16 /words/&lt;slug&gt;/ return 200 in 0.31-0.45s. | 2026-08-25 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-01 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-06 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-11 re-verified live: /words/&lt;slug&gt; → 301 → /words/&lt;slug&gt;/ → 200 verified on the-stone; all 17 article slugs 200 at their canonical form. | 2026-09-24 ISSUE/Low — the parity test the expected column defines, run for the first time since 2026-08-31, fails 16/17: the-weight-of-my-no (status published, 2026-08-31) has no [[redirects]] rule in netlify.toml. Every run since 08-31 spot-checked /words/the-stone only, so the drift went unseen for 24 days — the same shape as the July show-me-your-glory / send-someone-else drift. The expected column's 'non-slash 404s' premise did NOT hold: live /words/the-weight-of-my-no returns 301 -&gt; /words/the-weight-of-my-no/ with no rule, because Netlify Pretty URLs redirects a directory path on its own. No user impact observed; graded Low (parity/config drift, not a broken route). | 2026-09-25: live behaviour unchanged (single 301 via Pretty URLs); rule still only on the unmerged branch.</t>
+          <t>PASS — parity 16/16 verified live; every /words/&lt;slug&gt; returns a single 301 to its trailing-slash canonical; no orphan rules | 2026-08-13 re-verified live: all 16 /words/&lt;slug&gt; (no trailing slash) return 301; all 16 /words/&lt;slug&gt;/ return 200 in 0.31-0.45s. | 2026-08-25 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-01 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-06 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-11 re-verified live: /words/&lt;slug&gt; → 301 → /words/&lt;slug&gt;/ → 200 verified on the-stone; all 17 article slugs 200 at their canonical form. | 2026-09-24 ISSUE/Low — the parity test the expected column defines, run for the first time since 2026-08-31, fails 16/17: the-weight-of-my-no (status published, 2026-08-31) has no [[redirects]] rule in netlify.toml. Every run since 08-31 spot-checked /words/the-stone only, so the drift went unseen for 24 days — the same shape as the July show-me-your-glory / send-someone-else drift. The expected column's 'non-slash 404s' premise did NOT hold: live /words/the-weight-of-my-no returns 301 -&gt; /words/the-weight-of-my-no/ with no rule, because Netlify Pretty URLs redirects a directory path on its own. No user impact observed; graded Low (parity/config drift, not a broken route). | 2026-09-25: live behaviour unchanged (single 301 via Pretty URLs); rule still only on the unmerged branch. | 2026-09-26 full parity test (not a spot check) on qa/fixes-20260926: 17 published slugs == 17 /words/&lt;slug&gt; rules, 0 missing, 0 orphans, 0 dupes, no force; live: all 17 /words/&lt;slug&gt; return a single 301 to the slash canonical -&gt; 200. Fix still awaits merge (origin/main 95e2a73 lacks the rule; live behaviour unaffected).</t>
         </is>
       </c>
       <c r="I83" s="6" t="inlineStr">
@@ -5586,7 +5586,7 @@
       </c>
       <c r="H98" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-08-27) — SPLIT FROM F93, WHICH I CLOSED TOO BROADLY. F93 named two orphaned components; Dexter asked for the ghost plate to be rewired and it was, but `.identity-plate` was never in scope and is still dead. Re-verified today: the string appears nowhere in src/ and in none of the 19 built pages, because Plate.astro can only emit plate-{wide|secondary|banner|half|lead} plus plate-image/img-*/plate-row. css/plates.css ships ~85 lines of unreachable rules on every homepage load, and /brand/ documents the plate as live. Note this is NOT the same thing as `.identity-hero`, which does render on the homepage and is fine (F21). Contrast is not at issue — F90 already lifted `.identity-plate .meta-rail` to 5.77/5.63 — this is purely reachability. | RESOLVED 2026-08-28 — Dexter chose retire. See p4.</t>
+          <t>ISSUE/Medium (2026-08-27) — SPLIT FROM F93, WHICH I CLOSED TOO BROADLY. F93 named two orphaned components; Dexter asked for the ghost plate to be rewired and it was, but `.identity-plate` was never in scope and is still dead. Re-verified today: the string appears nowhere in src/ and in none of the 19 built pages, because Plate.astro can only emit plate-{wide|secondary|banner|half|lead} plus plate-image/img-*/plate-row. css/plates.css ships ~85 lines of unreachable rules on every homepage load, and /brand/ documents the plate as live. Note this is NOT the same thing as `.identity-hero`, which does render on the homepage and is fine (F21). Contrast is not at issue — F90 already lifted `.identity-plate .meta-rail` to 5.77/5.63 — this is purely reachability. | RESOLVED 2026-08-28 — Dexter chose retire. See p4. | 2026-09-26 re-verified: css/plates.css carries zero live .identity-plate rules (only the retirement comment at :270) and brand/index.html documents no .identity-plate specimen; the homepage's identity surface is IdentityHero via src/pages/index.astro — retirement holds.</t>
         </is>
       </c>
       <c r="I98" s="6" t="inlineStr">
@@ -5643,7 +5643,7 @@
       </c>
       <c r="H99" s="6" t="inlineStr">
         <is>
-          <t>PASS (2026-08-31, live on 13b631c then 83c2137) — POST-gate half verified live end to end: article 200 with 55 paragraphs and zero coming-soon markers; present in sitemap-0.xml, feed.xml and the homepage cascade (latest strip, lead plate, 'Week of August 31, 2026'); 'Send Someone Else' renders 0 .article-nav-ghost, i.e. the ghost treatment retired itself on go-live exactly as designed. OG plate 1200x630 (1.905), reads VOL 17 matching the essay's own number, title clears Anton's caps on the .92 leading from 9301d61. Metadata complete (description, og:title/image/image:alt/type, twitter:summary_large_image, canonical). Redate to Aug 31 propagated to every surface: JSON-LD datePublished 2026-08-31T12:00:00-05:00, Atom &lt;published&gt; 2026-08-31T17:00:00Z, homepage &lt;time datetime="2026-08-31"&gt;, zero 'Aug 30' anywhere live. Contrast 87 elements / 0 failures in BOTH modes (dark floor 5.13:1, light 4.67:1). Single h1, h1-&gt;h2 with no skipped level, skip link takes first Tab with a visible ring, 0 unnamed interactive elements, 0 console errors. || PRE-gate half NOT verified in production — see F93/F94: the release sat unpushed from Aug 29 until after the Aug 30 noon gate, so the Coming-Soon route never rendered on the live site for this essay. | 2026-09-01 re-verified live: VOL 17 present and correct across article (200), homepage lead plate, feed (17/17), sitemap and OG plate; article:published_time 2026-08-31 matches the homepage plate's &lt;time datetime&gt;.</t>
+          <t>PASS (2026-08-31, live on 13b631c then 83c2137) — POST-gate half verified live end to end: article 200 with 55 paragraphs and zero coming-soon markers; present in sitemap-0.xml, feed.xml and the homepage cascade (latest strip, lead plate, 'Week of August 31, 2026'); 'Send Someone Else' renders 0 .article-nav-ghost, i.e. the ghost treatment retired itself on go-live exactly as designed. OG plate 1200x630 (1.905), reads VOL 17 matching the essay's own number, title clears Anton's caps on the .92 leading from 9301d61. Metadata complete (description, og:title/image/image:alt/type, twitter:summary_large_image, canonical). Redate to Aug 31 propagated to every surface: JSON-LD datePublished 2026-08-31T12:00:00-05:00, Atom &lt;published&gt; 2026-08-31T17:00:00Z, homepage &lt;time datetime="2026-08-31"&gt;, zero 'Aug 30' anywhere live. Contrast 87 elements / 0 failures in BOTH modes (dark floor 5.13:1, light 4.67:1). Single h1, h1-&gt;h2 with no skipped level, skip link takes first Tab with a visible ring, 0 unnamed interactive elements, 0 console errors. || PRE-gate half NOT verified in production — see F93/F94: the release sat unpushed from Aug 29 until after the Aug 30 noon gate, so the Coming-Soon route never rendered on the live site for this essay. | 2026-09-01 re-verified live: VOL 17 present and correct across article (200), homepage lead plate, feed (17/17), sitemap and OG plate; article:published_time 2026-08-31 matches the homepage plate's &lt;time datetime&gt;. | 2026-09-26 re-verified live: /words/the-weight-of-my-no/ renders the full ArticleLayout (no 'Coming Soon', no noindex), sits in feed.xml (17 entries), sitemap-0.xml (21 locs) and the homepage cascade; 'Send Someone Else' carries a real rel=next .article-nav-next link to it, no ghost.</t>
         </is>
       </c>
       <c r="I99" s="6" t="inlineStr"/>
@@ -5688,7 +5688,7 @@
       </c>
       <c r="H100" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-08-31) — .article-eyebrow shipped flex-wrap: nowrap with no mobile override, so the rail runs off the frame on every article. Measured LIVE at 375px on /words/the-weight-of-my-no/ (6 chips: 2 lanes + 2 tags + date + read-time): scrollWidth 406 vs clientWidth 362 = 105px overflow; .article-read sits at left:418 against a 375px viewport, i.e. '8 min' is 100% invisible and 'Aug 31, 2026' is 92% clipped. Control /words/send-someone-else/ (5 chips) overflows 39px and loses 2px of '16 min', confirming this is site-wide and pre-existing rather than introduced by VOL 17 — VOL 17 is simply the worst case, being the first 6-chip essay. Because body/.page-shell are overflow-x: clip there is no scrollbar and no gesture that reaches the clipped text. Survived every prior scrub because source-only inspection cannot see it: the CSS is valid, the defect only exists once the flex row is laid out under 760px. | 2026-09-06 re-verified live: holds live - eyebrow wraps at 375px with zero overflow. | 2026-09-11 re-verified live: 375px /words/the-weight-of-my-no/: .article-eyebrow computes flex-wrap: wrap, all six chips inside the frame (rightmost 331px), documentElement.scrollWidth == clientWidth == 375. | 2026-09-19 re-verified live: 375px /words/the-weight-of-my-no/: .article-eyebrow flex-wrap: wrap, rightmost chip at 331px, scrollWidth == clientWidth == 375.</t>
+          <t>ISSUE/High (2026-08-31) — .article-eyebrow shipped flex-wrap: nowrap with no mobile override, so the rail runs off the frame on every article. Measured LIVE at 375px on /words/the-weight-of-my-no/ (6 chips: 2 lanes + 2 tags + date + read-time): scrollWidth 406 vs clientWidth 362 = 105px overflow; .article-read sits at left:418 against a 375px viewport, i.e. '8 min' is 100% invisible and 'Aug 31, 2026' is 92% clipped. Control /words/send-someone-else/ (5 chips) overflows 39px and loses 2px of '16 min', confirming this is site-wide and pre-existing rather than introduced by VOL 17 — VOL 17 is simply the worst case, being the first 6-chip essay. Because body/.page-shell are overflow-x: clip there is no scrollbar and no gesture that reaches the clipped text. Survived every prior scrub because source-only inspection cannot see it: the CSS is valid, the defect only exists once the flex row is laid out under 760px. | 2026-09-06 re-verified live: holds live - eyebrow wraps at 375px with zero overflow. | 2026-09-11 re-verified live: 375px /words/the-weight-of-my-no/: .article-eyebrow computes flex-wrap: wrap, all six chips inside the frame (rightmost 331px), documentElement.scrollWidth == clientWidth == 375. | 2026-09-19 re-verified live: 375px /words/the-weight-of-my-no/: .article-eyebrow flex-wrap: wrap, rightmost chip at 331px, scrollWidth == clientWidth == 375. | 2026-09-26 re-verified live at 375x812: .article-eyebrow is flex-wrap: wrap and 0 children overflow the viewport on /about/ and all 17 articles; no document-level horizontal overflow on any of the 18.</t>
         </is>
       </c>
       <c r="I100" s="6" t="inlineStr">
@@ -5745,7 +5745,7 @@
       </c>
       <c r="H101" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-09-02) — `.skip-link` had NO :focus-visible rule anywhere in the loaded cascade. Enumerated every rule matching /skip-link/ across all loaded sheets on live: exactly two hits, both in shell.css (the (0,2,0) :link/:visited base chip from F91, and .skip-link:focus for positioning) — neither carries an outline. Measured under a REAL Tab press on the live homepage with the chip focused: outline `rgb(153,200,255) auto 1px` — Chrome's UA default — while every sibling control measured the same way paints `rgb(204,0,0) solid 2px` (.brand-block, .mode-toggle, a.plate, .issue-standfirst, .hero-link, .sm-submit all confirmed this run). Confirmed identical on /about/ (shared shell.css, skipFocusRule:false). NOT a WCAG 2.4.7 failure — the UA ring is visible, which is exactly why five months of contrast-led sweeps never surfaced it — but a design-token break on the first element a keyboard user ever focuses. Same defect class as F76 (.sm-submit, closed 2026-08-10); this is a distinct element that rule never covered, not a regression of it. | 2026-09-06 re-verified live: still open ON LIVE, as expected - the fix is on this branch and unmerged. Live skip link focuses with the Chrome default ring (outline rgb(153,200,255) auto 1px) instead of the site's red --focus-ring. Closes on merge. | 2026-09-11 re-verified live: .skip-link:focus-visible rule present in shell.css?v=phase38 alongside .mode-toggle/.brand-block/.footer-strip a; measured live as outline rgb(204,0,0) solid 2px under a real Tab. | 2026-09-19 re-verified live: .skip-link measured under a real shift+Tab: outline rgb(204,0,0) solid 2px.</t>
+          <t>ISSUE/Medium (2026-09-02) — `.skip-link` had NO :focus-visible rule anywhere in the loaded cascade. Enumerated every rule matching /skip-link/ across all loaded sheets on live: exactly two hits, both in shell.css (the (0,2,0) :link/:visited base chip from F91, and .skip-link:focus for positioning) — neither carries an outline. Measured under a REAL Tab press on the live homepage with the chip focused: outline `rgb(153,200,255) auto 1px` — Chrome's UA default — while every sibling control measured the same way paints `rgb(204,0,0) solid 2px` (.brand-block, .mode-toggle, a.plate, .issue-standfirst, .hero-link, .sm-submit all confirmed this run). Confirmed identical on /about/ (shared shell.css, skipFocusRule:false). NOT a WCAG 2.4.7 failure — the UA ring is visible, which is exactly why five months of contrast-led sweeps never surfaced it — but a design-token break on the first element a keyboard user ever focuses. Same defect class as F76 (.sm-submit, closed 2026-08-10); this is a distinct element that rule never covered, not a regression of it. | 2026-09-06 re-verified live: still open ON LIVE, as expected - the fix is on this branch and unmerged. Live skip link focuses with the Chrome default ring (outline rgb(153,200,255) auto 1px) instead of the site's red --focus-ring. Closes on merge. | 2026-09-11 re-verified live: .skip-link:focus-visible rule present in shell.css?v=phase38 alongside .mode-toggle/.brand-block/.footer-strip a; measured live as outline rgb(204,0,0) solid 2px under a real Tab. | 2026-09-19 re-verified live: .skip-link measured under a real shift+Tab: outline rgb(204,0,0) solid 2px. | 2026-09-26 re-verified live under a REAL shift+Tab on /words/the-stone/: .skip-link matches :focus-visible and paints solid 2px rgb(204,0,0), offset 2px; forward Tab continues to .brand-block and .mode-toggle, both 2px #c00. Skip-link activation (el.click) sets #article and the target exists.</t>
         </is>
       </c>
       <c r="I101" s="6" t="inlineStr">
@@ -5802,7 +5802,7 @@
       </c>
       <c r="H102" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-09-02) — /brand/ was pinning `article.css?v=phase24` while the three src/ references sat at phase37, live-confirmed by reading document.styleSheets on both pages: /brand/ loaded article.css?v=phase24, /words/the-stone/ loaded article.css?v=phase37. article.css moved phase24 -&gt; phase37 in 558aa07 (the F97 eyebrow wrap, merged as f8d7702 on 2026-08-31); that commit bumped three references and missed the fourth. Effect: /css/* is immutable/1y, so any reader who had loaded /brand/ before that bump keeps the pre-F97 sheet on the design-system page for up to a year, while every article page serves the fixed one — the documentation surface silently disagreeing with the site it documents. Same contract as F87 (closed 2026-08-27), different mechanism: F87 was the fix landing in a sheet /brand/ does not load; this is /brand/ loading the right sheet at a stale key. Root cause is structural: the passthrough references sit outside src/, so both the bump sweep and DESIGN-SYSTEM.md's own high-water-mark grep (scoped `src/`) are blind to them — and the doc, written one day earlier in 885930e specifically to codify this rule, itself counted article.css at three references instead of four. | 2026-09-11 re-verified live: /brand/ loads article.css?v=phase37, shell.css?v=phase38, plates.css?v=phase39, brand.css?v=brand10 — the same versions the rest of the site loads. Parity holds.</t>
+          <t>ISSUE/Medium (2026-09-02) — /brand/ was pinning `article.css?v=phase24` while the three src/ references sat at phase37, live-confirmed by reading document.styleSheets on both pages: /brand/ loaded article.css?v=phase24, /words/the-stone/ loaded article.css?v=phase37. article.css moved phase24 -&gt; phase37 in 558aa07 (the F97 eyebrow wrap, merged as f8d7702 on 2026-08-31); that commit bumped three references and missed the fourth. Effect: /css/* is immutable/1y, so any reader who had loaded /brand/ before that bump keeps the pre-F97 sheet on the design-system page for up to a year, while every article page serves the fixed one — the documentation surface silently disagreeing with the site it documents. Same contract as F87 (closed 2026-08-27), different mechanism: F87 was the fix landing in a sheet /brand/ does not load; this is /brand/ loading the right sheet at a stale key. Root cause is structural: the passthrough references sit outside src/, so both the bump sweep and DESIGN-SYSTEM.md's own high-water-mark grep (scoped `src/`) are blind to them — and the doc, written one day earlier in 885930e specifically to codify this rule, itself counted article.css at three references instead of four. | 2026-09-11 re-verified live: /brand/ loads article.css?v=phase37, shell.css?v=phase38, plates.css?v=phase39, brand.css?v=brand10 — the same versions the rest of the site loads. Parity holds. | 2026-09-26 re-verified: every /css/*.css reference across src/, brand/ and phase0/ carries one ?v= per filename (tokens phase24 x7, shell phase38 x7, article phase37 x4, plates phase39 x2, home-augment phase40 x2, home-v2 phase36, notfound phase11, phase0 phase2) — zero parity splits on this branch.</t>
         </is>
       </c>
       <c r="I102" s="6" t="inlineStr">
@@ -5859,7 +5859,7 @@
       </c>
       <c r="H103" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-09-05) — `.demo-plate-body` had `flex: 1` but no `display: flex`, so the `justify-content: flex-end` written for `.demo-plate.img-plate .demo-plate-body` was inert and every white specimen title rendered at the TOP of its plate (measured live: titleTopFrac 0.11, titleBotFrac 0.24-0.38 on all five). The `::after` overlay is `linear-gradient(to top, rgba(0,0,0,.78), rgba(0,0,0,.08) 55%, rgba(0,0,0,.14))` — near-opaque at the bottom, ~.12 alpha at the title's actual position — so the titles sat over the LIGHT end of the concrete texture instead of the dark end. Pixel-measured (headless Chrome 1280px, real CSS, glyph-free sample strip inside the plate at the title's own y-band): the `concrete` specimens' title band runs rgb(98)-rgb(160), giving white-on-lightest 2.61:1 and white-on-median 3.03:1 against a 3:1 large-text floor (25.6px bold Anton). `lines` measured 4.12:1 and `noise` 18.1:1 at the same position, so the failure is texture-dependent — concrete is the light one — but all five were in the wrong band. Not caught by earlier sweeps because a computed-style probe walks the ancestor `background-color` chain straight through both pseudo-elements and reports the page ground (1.06:1) for every one of them, which reads exactly like the known `.plate-image` measurement artifact and was dismissed as such. It is not that artifact: on `.plate-image` the title genuinely sits in the .78 band; here the mirror had lost the rule that puts it there. Same contract as F87/F90 — /brand/ failing to dogfood — third distinct mechanism: F87 was the fix landing in a sheet /brand/ does not load, F99 was /brand/ loading the right sheet at a stale key, this is /brand/ loading the right sheet at the right key with a rule the production component has and the specimen does not. | 2026-09-11 re-verified live: all five .demo-plate.img-plate .demo-plate-body report display:flex / justify-content:flex-end; titles bottom-anchored at topFrac 0.52–0.79. Fix holds. | 2026-09-19 re-verified live: all five /brand/ .demo-plate.img-plate .demo-plate-body compute display:flex / justify-content:flex-end.</t>
+          <t>ISSUE/Medium (2026-09-05) — `.demo-plate-body` had `flex: 1` but no `display: flex`, so the `justify-content: flex-end` written for `.demo-plate.img-plate .demo-plate-body` was inert and every white specimen title rendered at the TOP of its plate (measured live: titleTopFrac 0.11, titleBotFrac 0.24-0.38 on all five). The `::after` overlay is `linear-gradient(to top, rgba(0,0,0,.78), rgba(0,0,0,.08) 55%, rgba(0,0,0,.14))` — near-opaque at the bottom, ~.12 alpha at the title's actual position — so the titles sat over the LIGHT end of the concrete texture instead of the dark end. Pixel-measured (headless Chrome 1280px, real CSS, glyph-free sample strip inside the plate at the title's own y-band): the `concrete` specimens' title band runs rgb(98)-rgb(160), giving white-on-lightest 2.61:1 and white-on-median 3.03:1 against a 3:1 large-text floor (25.6px bold Anton). `lines` measured 4.12:1 and `noise` 18.1:1 at the same position, so the failure is texture-dependent — concrete is the light one — but all five were in the wrong band. Not caught by earlier sweeps because a computed-style probe walks the ancestor `background-color` chain straight through both pseudo-elements and reports the page ground (1.06:1) for every one of them, which reads exactly like the known `.plate-image` measurement artifact and was dismissed as such. It is not that artifact: on `.plate-image` the title genuinely sits in the .78 band; here the mirror had lost the rule that puts it there. Same contract as F87/F90 — /brand/ failing to dogfood — third distinct mechanism: F87 was the fix landing in a sheet /brand/ does not load, F99 was /brand/ loading the right sheet at a stale key, this is /brand/ loading the right sheet at the right key with a rule the production component has and the specimen does not. | 2026-09-11 re-verified live: all five .demo-plate.img-plate .demo-plate-body report display:flex / justify-content:flex-end; titles bottom-anchored at topFrac 0.52–0.79. Fix holds. | 2026-09-19 re-verified live: all five /brand/ .demo-plate.img-plate .demo-plate-body compute display:flex / justify-content:flex-end. | 2026-09-26 re-verified live on /brand/: all 5 .img-plate .demo-plate-body are display:flex + justify-content:flex-end, titles sit at 0.69-0.82 of plate height, ::after scrim present (to top .78 -&gt; .26 55% -&gt; ...).</t>
         </is>
       </c>
       <c r="I103" s="6" t="inlineStr">
@@ -5916,7 +5916,7 @@
       </c>
       <c r="H104" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-09-06) — the scrim is `linear-gradient(to top, rgba(0,0,0,.78), rgba(0,0,0,.08) 55%, rgba(0,0,0,.14))`: .78 black at the bottom, but only .08–.14 across the top ~45%. That is sound while every title fits inside the bottom band, which is what `justify-content: flex-end` assumes. It does not hold for a three-line Anton title: 'Show Me Your Glory' is 165px tall in a 283px plate, so flex-end has no free space left to give and the first line starts 7% from the top. On `.img-concrete`, whose texture opens on a #c7c7c7 band, the white cap-height rows of 'SHOW' sit on a measured rgb(158,158,158) — 2.68:1 against a 3:1 large-text floor. 'The Theology of Staying on the Call' fails the same way at 2.92:1. Six of the eight live image plates pass (img-lines worst 3.69:1, img-noise worst 12.27:1), so this is texture-and-title-length dependent, not universal. MEASUREMENT: rasterised the homepage in headless Chrome at 1280 wide with the Earlier section unhidden, then sampled a glyph-free 12px strip inside each plate at each glyph row and took the row median — the computed-style probe reports 1.06:1 for all eight, which is the known .plate-image artifact and is why nine months of sweeps saw nothing. This is the second time that artifact has hidden a real defect (F100 was the first) and the first time it hid one in PRODUCTION rather than on /brand/. | 2026-09-11 re-verified live: plates.css?v=phase39 serving the .26/.34 scrim stops; .plate-image .plate-body display:flex / justify-content:flex-end on every image plate. 'Show Me Your Glory' (the three-line title that opened this row) sits at topFrac 0.067 where the scrim is ~.33 alpha — white on ~134 grey = ~3.6:1 against the 3:1 large-text floor. Fix holds.</t>
+          <t>ISSUE/High (2026-09-06) — the scrim is `linear-gradient(to top, rgba(0,0,0,.78), rgba(0,0,0,.08) 55%, rgba(0,0,0,.14))`: .78 black at the bottom, but only .08–.14 across the top ~45%. That is sound while every title fits inside the bottom band, which is what `justify-content: flex-end` assumes. It does not hold for a three-line Anton title: 'Show Me Your Glory' is 165px tall in a 283px plate, so flex-end has no free space left to give and the first line starts 7% from the top. On `.img-concrete`, whose texture opens on a #c7c7c7 band, the white cap-height rows of 'SHOW' sit on a measured rgb(158,158,158) — 2.68:1 against a 3:1 large-text floor. 'The Theology of Staying on the Call' fails the same way at 2.92:1. Six of the eight live image plates pass (img-lines worst 3.69:1, img-noise worst 12.27:1), so this is texture-and-title-length dependent, not universal. MEASUREMENT: rasterised the homepage in headless Chrome at 1280 wide with the Earlier section unhidden, then sampled a glyph-free 12px strip inside each plate at each glyph row and took the row median — the computed-style probe reports 1.06:1 for all eight, which is the known .plate-image artifact and is why nine months of sweeps saw nothing. This is the second time that artifact has hidden a real defect (F100 was the first) and the first time it hid one in PRODUCTION rather than on /brand/. | 2026-09-11 re-verified live: plates.css?v=phase39 serving the .26/.34 scrim stops; .plate-image .plate-body display:flex / justify-content:flex-end on every image plate. 'Show Me Your Glory' (the three-line title that opened this row) sits at topFrac 0.067 where the scrim is ~.33 alpha — white on ~134 grey = ~3.6:1 against the 3:1 large-text floor. Fix holds. | 2026-09-26 re-verified live: 3 visible homepage .plate-image plates carry the 3-stop scrim (.78 -&gt; .26 @55% -&gt; .34 top); rasterised with headless system Chrome at 1280px and sampled glyph-free strips beside each title line — medians 3.95:1 (Show Me Your Glory, top line on the concrete band) to 11.73:1, all clear of the 3:1 large-text floor.</t>
         </is>
       </c>
       <c r="I104" s="6" t="inlineStr">
@@ -5973,7 +5973,7 @@
       </c>
       <c r="H105" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Low (2026-09-11) — the comment's choice 1 reads 'The linked call-to-action for the same essay is the IssueNext strip below the archive, which is what carries "Notify me →" to the coming-soon page.' That strip was deleted on 2026-08-27 in e3b4e91 under F94, along with 202 lines of its CSS. F94's own p4 already recorded the consequence — 'the upcoming essay's coming-soon page now has ZERO inbound links from the homepage' — but the component that states the trade-off was never updated, so the file explains a bargain whose other half is gone. No behavioural defect: the plate renders correctly and the row is graded Low because it only misleads a reader of the source. Found by grepping src/ for IssueNext after confirming the live homepage and both shipped sheets are clean of it (the three CSS mentions F94 catalogued are comments; this is a fourth mention F94 missed).</t>
+          <t>ISSUE/Low (2026-09-11) — the comment's choice 1 reads 'The linked call-to-action for the same essay is the IssueNext strip below the archive, which is what carries "Notify me →" to the coming-soon page.' That strip was deleted on 2026-08-27 in e3b4e91 under F94, along with 202 lines of its CSS. F94's own p4 already recorded the consequence — 'the upcoming essay's coming-soon page now has ZERO inbound links from the homepage' — but the component that states the trade-off was never updated, so the file explains a bargain whose other half is gone. No behavioural defect: the plate renders correctly and the row is graded Low because it only misleads a reader of the source. Found by grepping src/ for IssueNext after confirming the live homepage and both shipped sheets are clean of it (the three CSS mentions F94 catalogued are comments; this is a fourth mention F94 missed). | 2026-09-26 re-verified: GhostPlate.astro:16-24 records the IssueNext strip as retired 2026-08-27 (e3b4e91) [F94] and says where the decision lives — no dependency on a shipping component.</t>
         </is>
       </c>
       <c r="I105" s="6" t="inlineStr">
@@ -6030,7 +6030,7 @@
       </c>
       <c r="H106" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Low (2026-09-11) — three references to the `.issue-next` strip survived its retirement (e3b4e91, 2026-08-27, F94): the homepage route description listed 'Issue-next ghost CTA' as part of the cascade; PAGES TO CRAWL told the crawler to follow article links from 'the homepage cascade or Issue-next ghost'; and §8 CONTENT COLLECTION INTEGRITY prescribed 'Issue-next ghost CTA's `.next-title` matches the referenced upcoming article's `&lt;title&gt;`'. The §8 line is the one that matters: `.next-title` cannot exist on any page the loop can reach, so that check can only ever be silently skipped — or, worse, reported as run. Graded Low because no site surface is affected and the two descriptive lines are merely stale; it is filed rather than fixed-in-passing because the operating prompt is what every future run executes.</t>
+          <t>ISSUE/Low (2026-09-11) — three references to the `.issue-next` strip survived its retirement (e3b4e91, 2026-08-27, F94): the homepage route description listed 'Issue-next ghost CTA' as part of the cascade; PAGES TO CRAWL told the crawler to follow article links from 'the homepage cascade or Issue-next ghost'; and §8 CONTENT COLLECTION INTEGRITY prescribed 'Issue-next ghost CTA's `.next-title` matches the referenced upcoming article's `&lt;title&gt;`'. The §8 line is the one that matters: `.next-title` cannot exist on any page the loop can reach, so that check can only ever be silently skipped — or, worse, reported as run. Graded Low because no site surface is affected and the two descriptive lines are merely stale; it is filed rather than fixed-in-passing because the operating prompt is what every future run executes. | 2026-09-26 re-verified: audit/QA-OS.md names .issue-next / .next-title only as retired (lines 103, 276-277, citing F94); no live check targets them.</t>
         </is>
       </c>
       <c r="I106" s="6" t="inlineStr">
@@ -6087,7 +6087,7 @@
       </c>
       <c r="H107" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Low (2026-09-18) — §3 read 'Verify `--accent` usage on section-head h2, reading-progress bars, pull-quote borders.' Measured live on /words/the-weight-of-my-no/ in dark mode: `.reading-progress` background rgb(243,240,232) (--ink) and `.pull-quote` borders rgba(243,240,232,.82) (--border). Both are deliberate: the progress bar was recoloured from --accent to --ink in 68b0c1d (2026-04-10) with a comment at css/article.css:873 explaining the red bar competed with the masthead, and DESIGN-SYSTEM.md §4 lists pull-quote top/bottom borders as ordinary content borders while naming the .callout left border as the accent one. The check predates nothing — QA-OS was written 2026-08-07, four months after the recolour — so it has been either silently skipped or passed on assumption every run. Same class as F103: a dead check in the operating prompt. Graded Low: no site surface affected.</t>
+          <t>ISSUE/Low (2026-09-18) — §3 read 'Verify `--accent` usage on section-head h2, reading-progress bars, pull-quote borders.' Measured live on /words/the-weight-of-my-no/ in dark mode: `.reading-progress` background rgb(243,240,232) (--ink) and `.pull-quote` borders rgba(243,240,232,.82) (--border). Both are deliberate: the progress bar was recoloured from --accent to --ink in 68b0c1d (2026-04-10) with a comment at css/article.css:873 explaining the red bar competed with the masthead, and DESIGN-SYSTEM.md §4 lists pull-quote top/bottom borders as ordinary content borders while naming the .callout left border as the accent one. The check predates nothing — QA-OS was written 2026-08-07, four months after the recolour — so it has been either silently skipped or passed on assumption every run. Same class as F103: a dead check in the operating prompt. Graded Low: no site surface affected. | 2026-09-26 re-verified: QA-OS.md §3 (line 171-175) names section-head h2 + .callout as the accent's homes and records the reading-progress bar and pull-quote borders as by-design. Live spot-check agrees: /brand/ .section-head h2 = rgb(204,0,0), /words/the-stone/ .callout border-left = solid rgb(204,0,0).</t>
         </is>
       </c>
       <c r="I107" s="6" t="inlineStr">
@@ -6330,7 +6330,7 @@
       </c>
       <c r="K111" s="6" t="inlineStr">
         <is>
-          <t>PASS (2026-09-24, verified against build + rule injected on live) — npm run build clean; dist/css/home-augment.css carries the new selector; dist/index.html and dist/brand/index.html both reference home-augment.css?v=phase40. Dev servers cannot start in unattended runs, so the fix rule was applied to the live homepage with insertRule on the loaded home-augment sheet: dark mode, real pointer hover, a.plate-lead:hover true -&gt; .rail-cta rgb(243,240,232) on rgb(204,0,0) = 5.17:1 (screenshot shows a cream 'READ →'). deleteRule restored the sheet and a re-measure read 3.44:1 again, proving the page went back to its original state. Light-mode hover unchanged (rule is dark-scoped): rgb(244,244,241) on #c00. Sibling hover controls (.latest-cta, .hero-link.primary) re-measured 5.17:1, unaffected. Live-verifies on the first SCRUB after merge.</t>
+          <t>PASS (2026-09-24, verified against build + rule injected on live) — npm run build clean; dist/css/home-augment.css carries the new selector; dist/index.html and dist/brand/index.html both reference home-augment.css?v=phase40. Dev servers cannot start in unattended runs, so the fix rule was applied to the live homepage with insertRule on the loaded home-augment sheet: dark mode, real pointer hover, a.plate-lead:hover true -&gt; .rail-cta rgb(243,240,232) on rgb(204,0,0) = 5.17:1 (screenshot shows a cream 'READ →'). deleteRule restored the sheet and a re-measure read 3.44:1 again, proving the page went back to its original state. Light-mode hover unchanged (rule is dark-scoped): rgb(244,244,241) on #c00. Sibling hover controls (.latest-cta, .hero-link.primary) re-measured 5.17:1, unaffected. Live-verifies on the first SCRUB after merge. | 2026-09-26: still awaits merge — origin/main and the live deploy (6ab794f1, 09-26 09:48Z) remain on 95e2a73, so the live chip is still the pre-fix 3.44:1 on dark-mode hover.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
audit(ledger): 2026-09-27 scrub — clean site, F105/F106 closed live, F01-F06 + F107 rotation PASS
F108 still live pending merge of the stacked qa/fixes branches.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -632,7 +632,7 @@
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>PASS — masthead .brand-block → '/' present on home/about/404/phase0/brand/article; aria-label 'Dexter Jakes home' | 2026-08-15 re-verified live: brand-block present and linking / on all 20 pages | 2026-08-25 re-verified live: brand-block present and linking / on all 20 crawled routes; aria-label intact. | 2026-08-27 re-verified live: masthead .brand-block → '/' confirmed under real Tab focus. | 2026-09-01 re-verified live: masthead .brand-block reached under a REAL Tab press (2nd stop), links '/', focus ring #c00 2px. | 2026-09-06 re-verified live: masthead .brand-block reached under a real forward Tab from the skip link and links '/'; present on all 27 crawled routes. | 2026-09-11 re-verified live: masthead .brand-block → '/' reached under a real forward Tab from the skip link on the homepage; present on all 26 crawled routes.</t>
+          <t>PASS — masthead .brand-block → '/' present on home/about/404/phase0/brand/article; aria-label 'Dexter Jakes home' | 2026-08-15 re-verified live: brand-block present and linking / on all 20 pages | 2026-08-25 re-verified live: brand-block present and linking / on all 20 crawled routes; aria-label intact. | 2026-08-27 re-verified live: masthead .brand-block → '/' confirmed under real Tab focus. | 2026-09-01 re-verified live: masthead .brand-block reached under a REAL Tab press (2nd stop), links '/', focus ring #c00 2px. | 2026-09-06 re-verified live: masthead .brand-block reached under a real forward Tab from the skip link and links '/'; present on all 27 crawled routes. | 2026-09-11 re-verified live: masthead .brand-block → '/' reached under a real forward Tab from the skip link on the homepage; present on all 26 crawled routes. | 2026-09-27 re-verified live: masthead .brand-block href '/' (aria-label 'Dexter Jakes home') present on all 22 crawled HTML routes incl. the unmatched-route 404 and /phase0/.</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr"/>
@@ -681,7 +681,7 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>PASS — brand-word: Words (home/article/about/brand), 404, Phase 0 — matches documented intent | 2026-08-15 re-verified live: brand-word: home/about/article 'Words', 404 '404', phase0 'Phase 0' — matches the documented about-page quirk | 2026-08-25 re-verified live: brand-word: "Words" on home/about/article, "404" on /404, "Phase 0" on /phase0/ — matches documented intent. | 2026-08-27 re-verified live: brand word 'Words' confirmed on home/article/about. | 2026-09-01 re-verified live on the homepage: masthead brand word reads 'Words' (documented intent). Other surfaces not re-walked this run. | 2026-09-19 re-verified live: brand-word live: 'Words' on /, /about/, /brand/ and all 17 articles; 'Phase 0' on /phase0/; '404' on the unmatched-route 404 — matches documented intent.</t>
+          <t>PASS — brand-word: Words (home/article/about/brand), 404, Phase 0 — matches documented intent | 2026-08-15 re-verified live: brand-word: home/about/article 'Words', 404 '404', phase0 'Phase 0' — matches the documented about-page quirk | 2026-08-25 re-verified live: brand-word: "Words" on home/about/article, "404" on /404, "Phase 0" on /phase0/ — matches documented intent. | 2026-08-27 re-verified live: brand word 'Words' confirmed on home/article/about. | 2026-09-01 re-verified live on the homepage: masthead brand word reads 'Words' (documented intent). Other surfaces not re-walked this run. | 2026-09-19 re-verified live: brand-word live: 'Words' on /, /about/, /brand/ and all 17 articles; 'Phase 0' on /phase0/; '404' on the unmatched-route 404 — matches documented intent. | 2026-09-27 re-verified live: brand-word 'Words' on /, /about/, /brand/ and all 17 articles; 'Phase 0' on /phase0/; '404' on the unmatched-route 404 — matches documented intent.</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr"/>
@@ -734,7 +734,7 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>PASS — toggle cycles dark→light→dark; dxmode cookie written both ways; label + aria-pressed + bg/ink all update. Reconfirmed 2026-08-10 PM across 3 consecutive clicks. | 2026-08-13 re-verified live: toggle cycled dark-&gt;light-&gt;dark on the live homepage; dxmode cookie written both ways; --bg/--ink/--accent-text all re-resolved (#060606/#f3f0e8/#ff4d4d dark, #f4f4f1/#050505/#c00 light). | 2026-08-16 re-verified live: toggle cycled dark-&gt;light-&gt;dark on the live homepage; dxmode cookie written both ways (dxmode=light then dxmode=dark); --bg #060606&lt;-&gt;#f4f4f1 and --ink #f3f0e8&lt;-&gt;#050505 both re-resolved; label and aria-pressed tracked ('Mode: Dark'/true &lt;-&gt; 'Mode: Light'/false). | 2026-08-25 re-verified live: toggle re-verified with a REAL pointer click (not element.click()) on both the homepage and /words/the-stone/: page repaints dark&lt;-&gt;light, dxmode cookie written both ways, label and aria-pressed track. METHOD NOTE: a programmatic element.click() flips the class, the tokens and the cookie but leaves body's used background/color stale in getComputedStyle until a repaint is forced — that is a measurement artifact, NOT a site defect, and it read as an article-page mode regression for several minutes this run. Always verify this row with a real click. | 2026-08-27 re-verified live: REAL pointer click (not element.click()) + 2s settle + screenshot: dark→light→dark, --bg #060606↔#f4f4f1, --ink #f3f0e8↔#050505, dxmode cookie written both ways, button label tracks. | 2026-09-01 ISSUE (MEDIUM) — theme-color half of this row has NEVER been satisfiable. mode.js ships syncThemeColor() (js/mode.js:74-95) which rewrites &lt;meta name="theme-color"&gt; to #060606/#f4f4f1 and strips the media attr off a media-split pair, but NO layout ever emitted that meta: document.querySelectorAll('meta[name="theme-color"]').length === 0 on /, /about/, /words/&lt;slug&gt;/, /404, /brand/ and /phase0/ live. querySelector() returned null, the function no-opped, and the dedupe loop iterated an empty list — silent, so five months of scrubs that checked the class/cookie/tokens never saw it. User-visible effect: mobile browser chrome (address/status bar) follows the OS instead of the site's mode. Class flip, dxmode cookie, --bg/--ink re-resolve, aria-pressed, label and logo swap all re-verified live PASS this run with a REAL pointer click + 2s settle. | 2026-09-06 re-verified live: mode toggle driven with a real pointer click (not element.click()) plus a 2.5s settle. dark rgb(6,6,6)/rgb(243,240,232) -&gt; light rgb(244,244,241)/rgb(5,5,5) -&gt; dark, with the dxmode cookie and the 'Mode: Dark'/'Mode: Light' label tracking each flip. | 2026-09-11 re-verified live: real pointer click on .mode-toggle with a 2s settle: dxmode dark→light, html.dark-mode cleared, body rgb(6,6,6)→rgb(244,244,241), theme-color meta →#f4f4f1, label 'Mode: Light'. Screenshot confirmed after the wait.</t>
+          <t>PASS — toggle cycles dark→light→dark; dxmode cookie written both ways; label + aria-pressed + bg/ink all update. Reconfirmed 2026-08-10 PM across 3 consecutive clicks. | 2026-08-13 re-verified live: toggle cycled dark-&gt;light-&gt;dark on the live homepage; dxmode cookie written both ways; --bg/--ink/--accent-text all re-resolved (#060606/#f3f0e8/#ff4d4d dark, #f4f4f1/#050505/#c00 light). | 2026-08-16 re-verified live: toggle cycled dark-&gt;light-&gt;dark on the live homepage; dxmode cookie written both ways (dxmode=light then dxmode=dark); --bg #060606&lt;-&gt;#f4f4f1 and --ink #f3f0e8&lt;-&gt;#050505 both re-resolved; label and aria-pressed tracked ('Mode: Dark'/true &lt;-&gt; 'Mode: Light'/false). | 2026-08-25 re-verified live: toggle re-verified with a REAL pointer click (not element.click()) on both the homepage and /words/the-stone/: page repaints dark&lt;-&gt;light, dxmode cookie written both ways, label and aria-pressed track. METHOD NOTE: a programmatic element.click() flips the class, the tokens and the cookie but leaves body's used background/color stale in getComputedStyle until a repaint is forced — that is a measurement artifact, NOT a site defect, and it read as an article-page mode regression for several minutes this run. Always verify this row with a real click. | 2026-08-27 re-verified live: REAL pointer click (not element.click()) + 2s settle + screenshot: dark→light→dark, --bg #060606↔#f4f4f1, --ink #f3f0e8↔#050505, dxmode cookie written both ways, button label tracks. | 2026-09-01 ISSUE (MEDIUM) — theme-color half of this row has NEVER been satisfiable. mode.js ships syncThemeColor() (js/mode.js:74-95) which rewrites &lt;meta name="theme-color"&gt; to #060606/#f4f4f1 and strips the media attr off a media-split pair, but NO layout ever emitted that meta: document.querySelectorAll('meta[name="theme-color"]').length === 0 on /, /about/, /words/&lt;slug&gt;/, /404, /brand/ and /phase0/ live. querySelector() returned null, the function no-opped, and the dedupe loop iterated an empty list — silent, so five months of scrubs that checked the class/cookie/tokens never saw it. User-visible effect: mobile browser chrome (address/status bar) follows the OS instead of the site's mode. Class flip, dxmode cookie, --bg/--ink re-resolve, aria-pressed, label and logo swap all re-verified live PASS this run with a REAL pointer click + 2s settle. | 2026-09-06 re-verified live: mode toggle driven with a real pointer click (not element.click()) plus a 2.5s settle. dark rgb(6,6,6)/rgb(243,240,232) -&gt; light rgb(244,244,241)/rgb(5,5,5) -&gt; dark, with the dxmode cookie and the 'Mode: Dark'/'Mode: Light' label tracking each flip. | 2026-09-11 re-verified live: real pointer click on .mode-toggle with a 2s settle: dxmode dark→light, html.dark-mode cleared, body rgb(6,6,6)→rgb(244,244,241), theme-color meta →#f4f4f1, label 'Mode: Light'. Screenshot confirmed after the wait. | 2026-09-27 re-verified live: real pointer click on the mode toggle with a 2s settle: dxmode light-&gt;dark, html.dark-mode set, body rgb(6,6,6) on ink rgb(243,240,232), theme-color #060606, aria-pressed true, label 'Mode: Dark', logo -&gt; logo-white.svg; screenshot after the wait confirmed the dark palette. Second real click restored light.</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
@@ -791,7 +791,7 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: skip link is first focusable; activating it lands document.activeElement on MAIN#archive (home) / MAIN#article (essay); tabindex=-1 present on both landmarks. The 2c7d88d fix holds in production. | 2026-08-13 re-verified live: tab-target verified on live: .skip-link reveals from left:-999px to a 83x69 box at (12,12), cream-on-ink 17.79:1; activating it moved document.activeElement to MAIN#archive (tabindex=-1). Article pages target #article. | 2026-08-16 re-verified live: structural half re-verified live: .skip-link is the first focusable element in document order on every page type, and its target (MAIN#article / MAIN#archive / MAIN#phase0 / MAIN#main) carries tabindex=-1. End-to-end activation NOT re-exercisable this run — the browser pane reports document.visibilityState 'hidden' and drops page focus on every reload, so a fresh-load Tab lands on BODY. Harness limitation, not a site regression; last live activation was 2026-08-13. NOTE: this row's sweep is what surfaced F91 — see that row. | 2026-08-25 re-verified live: verified end-to-end live under REAL keyboard input on /words/the-stone/ — the gap the 2026-08-16 run had to leave open. .skip-link is the first focusable in DOM order, reveals from left:-999px to a 126x46 chip at (12,12), computes 17.79:1 (#060606 on #f3f0e8), and pressing Enter sets location.hash to #article and moves document.activeElement to MAIN#article (tabindex=-1). | 2026-08-27 re-verified live: skip link is the first focusable (reached by real shift+Tab from .brand-block), renders as an opaque cream chip at 17.79:1, and activation moves focus to MAIN#archive with hash #archive. | 2026-09-01 re-verified live: .skip-link is the FIRST Tab stop from page load and matches :focus-visible; activation moves location.hash to #archive and focus to MAIN#archive. Ran the ordinary-link control first per the harness antipattern. | 2026-09-06 re-verified live: skip link is the first focusable, unhides on focus (left -999px -&gt; 12px), and activation moved location.hash to '#archive' and focus to the #archive element. | 2026-09-11 re-verified live: skip link is the first focusable (reached by one shift+Tab back from .brand-block), 17.79:1, #c00 2px ring; activated with a real pointer click → document.activeElement === main#archive, location.hash '#archive'. | 2026-09-19 re-verified live: skip link reached under a real shift+Tab on the homepage (:focus-visible true, #060606 on cream chip, rgb(204,0,0) 2px ring); activation moves focus to #archive (tabindex -1) and sets location.hash.</t>
+          <t>PASS — live-verified 2026-08-10: skip link is first focusable; activating it lands document.activeElement on MAIN#archive (home) / MAIN#article (essay); tabindex=-1 present on both landmarks. The 2c7d88d fix holds in production. | 2026-08-13 re-verified live: tab-target verified on live: .skip-link reveals from left:-999px to a 83x69 box at (12,12), cream-on-ink 17.79:1; activating it moved document.activeElement to MAIN#archive (tabindex=-1). Article pages target #article. | 2026-08-16 re-verified live: structural half re-verified live: .skip-link is the first focusable element in document order on every page type, and its target (MAIN#article / MAIN#archive / MAIN#phase0 / MAIN#main) carries tabindex=-1. End-to-end activation NOT re-exercisable this run — the browser pane reports document.visibilityState 'hidden' and drops page focus on every reload, so a fresh-load Tab lands on BODY. Harness limitation, not a site regression; last live activation was 2026-08-13. NOTE: this row's sweep is what surfaced F91 — see that row. | 2026-08-25 re-verified live: verified end-to-end live under REAL keyboard input on /words/the-stone/ — the gap the 2026-08-16 run had to leave open. .skip-link is the first focusable in DOM order, reveals from left:-999px to a 126x46 chip at (12,12), computes 17.79:1 (#060606 on #f3f0e8), and pressing Enter sets location.hash to #article and moves document.activeElement to MAIN#article (tabindex=-1). | 2026-08-27 re-verified live: skip link is the first focusable (reached by real shift+Tab from .brand-block), renders as an opaque cream chip at 17.79:1, and activation moves focus to MAIN#archive with hash #archive. | 2026-09-01 re-verified live: .skip-link is the FIRST Tab stop from page load and matches :focus-visible; activation moves location.hash to #archive and focus to MAIN#archive. Ran the ordinary-link control first per the harness antipattern. | 2026-09-06 re-verified live: skip link is the first focusable, unhides on focus (left -999px -&gt; 12px), and activation moved location.hash to '#archive' and focus to the #archive element. | 2026-09-11 re-verified live: skip link is the first focusable (reached by one shift+Tab back from .brand-block), 17.79:1, #c00 2px ring; activated with a real pointer click → document.activeElement === main#archive, location.hash '#archive'. | 2026-09-19 re-verified live: skip link reached under a real shift+Tab on the homepage (:focus-visible true, #060606 on cream chip, rgb(204,0,0) 2px ring); activation moves focus to #archive (tabindex -1) and sets location.hash. | 2026-09-27 re-verified live: first real Tab from load lands on .skip-link (#archive), :focus-visible true, rgb(204,0,0) 2px solid ring, rgb(244,244,241) on rgb(5,5,5) chip; activation moved focus to #archive and set location.hash.</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr"/>
@@ -844,7 +844,7 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>PASS — 2 decorative rulers render | 2026-08-15 re-verified live: zero .ruler-* without aria-hidden across all pages | 2026-09-11 re-verified live: 2 rulers on each of home/article/about/404/phase0, every one aria-hidden=true.</t>
+          <t>PASS — 2 decorative rulers render | 2026-08-15 re-verified live: zero .ruler-* without aria-hidden across all pages | 2026-09-11 re-verified live: 2 rulers on each of home/article/about/404/phase0, every one aria-hidden=true. | 2026-09-27 re-verified live: 2 rulers on each of 22 crawled HTML routes, every one aria-hidden=true.</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr"/>
@@ -893,7 +893,7 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>PASS — footer strip + links present on all page types | 2026-08-15 re-verified live: footer: Instagram + X both target=_blank rel="noopener noreferrer", /feed.xml, /about/, "Built by Dex"; zero _blank links missing rel site-wide | 2026-08-25 re-verified live: footer links resolve: instagram.com/ImJustDex 200, x.com/ImJustDex 200, /feed.xml 200. | 2026-09-11 re-verified live: footer Instagram + X both target=_blank rel='noopener noreferrer', Feed → /feed.xml, About present on home only; 'Built by Dex · Est. 2026' on all three.</t>
+          <t>PASS — footer strip + links present on all page types | 2026-08-15 re-verified live: footer: Instagram + X both target=_blank rel="noopener noreferrer", /feed.xml, /about/, "Built by Dex"; zero _blank links missing rel site-wide | 2026-08-25 re-verified live: footer links resolve: instagram.com/ImJustDex 200, x.com/ImJustDex 200, /feed.xml 200. | 2026-09-11 re-verified live: footer Instagram + X both target=_blank rel='noopener noreferrer', Feed → /feed.xml, About present on home only; 'Built by Dex · Est. 2026' on all three. | 2026-09-27 re-verified live: homepage footer Instagram + X both target=_blank rel='noopener noreferrer', Feed -&gt; /feed.xml, About present; 'Built by Dex · Est. 2026' on home, about, brand, 404 and all 17 articles (/phase0/ carries its own bespoke footer by design); all external footer links 200.</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr"/>
@@ -1553,7 +1553,7 @@
       <c r="J22" s="4" t="inlineStr"/>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t>PENDING | 2026-09-18: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-26: still structurally untestable — 0 upcoming entries in the committed collection.</t>
+          <t>PENDING | 2026-09-18: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-26: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-27: still structurally untestable — 0 upcoming entries in the committed collection (17/17 published, past-dated).</t>
         </is>
       </c>
     </row>
@@ -2687,7 +2687,7 @@
       </c>
       <c r="K44" s="6" t="inlineStr">
         <is>
-          <t>PENDING | 2026-09-18: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-26: still structurally untestable — 0 upcoming entries in the committed collection.</t>
+          <t>PENDING | 2026-09-18: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-26: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-27: still structurally untestable — 0 upcoming entries in the committed collection (17/17 published, past-dated).</t>
         </is>
       </c>
     </row>
@@ -2948,7 +2948,7 @@
       </c>
       <c r="K49" s="6" t="inlineStr">
         <is>
-          <t>PENDING | 2026-09-18: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-26: still structurally untestable — 0 upcoming entries in the committed collection.</t>
+          <t>PENDING | 2026-09-18: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-26: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-27: still structurally untestable — 0 upcoming entries in the committed collection (17/17 published, past-dated).</t>
         </is>
       </c>
     </row>
@@ -4758,7 +4758,7 @@
       </c>
       <c r="K83" s="6" t="inlineStr">
         <is>
-          <t>PASS (2026-09-24, verified against build) — netlify.toml parses (29 redirects); parity test published slugs == /words/&lt;slug&gt; rule set, 17/17, 0 orphans, 0 dupes, no force on any /words/&lt;slug&gt; rule; npm run build clean (20 pages). Live behaviour was already a single 301 and is unchanged by the rule. Note for the expected column: a missing rule here showed up as parity drift, not a 404.</t>
+          <t>PASS (2026-09-24, verified against build) — netlify.toml parses (29 redirects); parity test published slugs == /words/&lt;slug&gt; rule set, 17/17, 0 orphans, 0 dupes, no force on any /words/&lt;slug&gt; rule; npm run build clean (20 pages). Live behaviour was already a single 301 and is unchanged by the rule. Note for the expected column: a missing rule here showed up as parity drift, not a 404. | 2026-09-27: live parity re-checked — all 17 /words/&lt;slug&gt; return a single 301 to the slash canonical; /about, /brand, /phase0 likewise. Fix still awaits merge.</t>
         </is>
       </c>
     </row>
@@ -6159,7 +6159,7 @@
       </c>
       <c r="K108" s="6" t="inlineStr">
         <is>
-          <t>PASS (verified against build) — 2026-09-18. `npm run build` passes (20 pages). All four connect-src values now read `'self' https://ingesteer.services-prod.nsvcs.net`; no other directive changed. Live verification needs the deploy: next SCRUB after merge should show zero console errors on page hide/navigation, and Netlify's RUM panel should start receiving data.</t>
+          <t>PASS (verified against build) — 2026-09-18. `npm run build` passes (20 pages). All four connect-src values now read `'self' https://ingesteer.services-prod.nsvcs.net`; no other directive changed. Live verification needs the deploy: next SCRUB after merge should show zero console errors on page hide/navigation, and Netlify's RUM panel should start receiving data. | PASS (2026-09-27, live-verified) — the fix merged with 95e2a73 on 09-19; live CSP connect-src reads `'self' https://ingesteer.services-prod.nsvcs.net`, /.netlify/scripts/rum loads 200 on every page, and a 9-route console sweep (home, about, brand, phase0, 404, 4 articles) logged zero CSP violations and zero errors other than the deliberate unmatched-route 404 document.</t>
         </is>
       </c>
     </row>
@@ -6216,7 +6216,7 @@
       </c>
       <c r="K109" s="6" t="inlineStr">
         <is>
-          <t>PASS (verified against build) — 2026-09-18. dist/index.html row heads read '01 Latest' / '02 Earlier'; 'This Week' appears nowhere in src/, css/, js/ or the build. Goes live-verified on the next SCRUB after merge.</t>
+          <t>PASS (verified against build) — 2026-09-18. dist/index.html row heads read '01 Latest' / '02 Earlier'; 'This Week' appears nowhere in src/, css/, js/ or the build. Goes live-verified on the next SCRUB after merge. | PASS (2026-09-27, live-verified) — merged with 95e2a73 on 09-19; the live homepage lead row head reads '01 LATEST' over The Weight of My No; 'This Week' absent.</t>
         </is>
       </c>
     </row>
@@ -6258,7 +6258,7 @@
       </c>
       <c r="H110" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Low (2026-09-22) — §9 named no method for F57, so this run tested it with a burst chained onto the subscribe smoke test: 8 POSTs returned 8 x 200 and no 429 (one returned HTTP 000, an instance churn tell), which reads as a dead limiter. A clean sequential re-run returned exactly 5 x 400 then 5 x 429; a parallel re-run returned 10 x 400 and no 429. The limiter is correct; the prompt lacked the method, and the false reading cost two test cycles. Same class as F103/F104.</t>
+          <t>ISSUE/Low (2026-09-22) — §9 named no method for F57, so this run tested it with a burst chained onto the subscribe smoke test: 8 POSTs returned 8 x 200 and no 429 (one returned HTTP 000, an instance churn tell), which reads as a dead limiter. A clean sequential re-run returned exactly 5 x 400 then 5 x 429; a parallel re-run returned 10 x 400 and no 429. The limiter is correct; the prompt lacked the method, and the false reading cost two test cycles. Same class as F103/F104. | 2026-09-27 re-verified against the file: QA-OS.md §9 still carries the sequential 10-POST method (5 x 400 then 5 x 429) and the MEASUREMENT ANTIPATTERNS fan-out entry.</t>
         </is>
       </c>
       <c r="I110" s="6" t="inlineStr">
@@ -6330,7 +6330,7 @@
       </c>
       <c r="K111" s="6" t="inlineStr">
         <is>
-          <t>PASS (2026-09-24, verified against build + rule injected on live) — npm run build clean; dist/css/home-augment.css carries the new selector; dist/index.html and dist/brand/index.html both reference home-augment.css?v=phase40. Dev servers cannot start in unattended runs, so the fix rule was applied to the live homepage with insertRule on the loaded home-augment sheet: dark mode, real pointer hover, a.plate-lead:hover true -&gt; .rail-cta rgb(243,240,232) on rgb(204,0,0) = 5.17:1 (screenshot shows a cream 'READ →'). deleteRule restored the sheet and a re-measure read 3.44:1 again, proving the page went back to its original state. Light-mode hover unchanged (rule is dark-scoped): rgb(244,244,241) on #c00. Sibling hover controls (.latest-cta, .hero-link.primary) re-measured 5.17:1, unaffected. Live-verifies on the first SCRUB after merge. | 2026-09-26: still awaits merge — origin/main and the live deploy (6ab794f1, 09-26 09:48Z) remain on 95e2a73, so the live chip is still the pre-fix 3.44:1 on dark-mode hover.</t>
+          <t>PASS (2026-09-24, verified against build + rule injected on live) — npm run build clean; dist/css/home-augment.css carries the new selector; dist/index.html and dist/brand/index.html both reference home-augment.css?v=phase40. Dev servers cannot start in unattended runs, so the fix rule was applied to the live homepage with insertRule on the loaded home-augment sheet: dark mode, real pointer hover, a.plate-lead:hover true -&gt; .rail-cta rgb(243,240,232) on rgb(204,0,0) = 5.17:1 (screenshot shows a cream 'READ →'). deleteRule restored the sheet and a re-measure read 3.44:1 again, proving the page went back to its original state. Light-mode hover unchanged (rule is dark-scoped): rgb(244,244,241) on #c00. Sibling hover controls (.latest-cta, .hero-link.primary) re-measured 5.17:1, unaffected. Live-verifies on the first SCRUB after merge. | 2026-09-26: still awaits merge — origin/main and the live deploy (6ab794f1, 09-26 09:48Z) remain on 95e2a73, so the live chip is still the pre-fix 3.44:1 on dark-mode hover. | 2026-09-27: still awaits merge — origin/main and the live deploy (6ab794f1, 09-26 09:48Z) remain on 95e2a73; the live home-augment.css?v=phase34 carries no dark-mode :hover .rail-cta rule. Not re-counted as new.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
audit(ledger): 2026-09-28 full regression — F53 opened and fixed, F19/F41/F46 exercised via fixture build
Monday full-ledger regression, all 108 rows. Site clean apart from F53
(phase0 typo shows outage copy, Medium, fixed in c524932). The
coming-soon rows ran for the first time since the collection went
all-published, against a throwaway future-dated fixture build that was
never committed. F108 High and F80 Low still live, awaiting the stacked
qa/fixes branches. F35/F36 rotation gap: the pane cannot scroll while hidden.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -632,7 +632,7 @@
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>PASS — masthead .brand-block → '/' present on home/about/404/phase0/brand/article; aria-label 'Dexter Jakes home' | 2026-08-15 re-verified live: brand-block present and linking / on all 20 pages | 2026-08-25 re-verified live: brand-block present and linking / on all 20 crawled routes; aria-label intact. | 2026-08-27 re-verified live: masthead .brand-block → '/' confirmed under real Tab focus. | 2026-09-01 re-verified live: masthead .brand-block reached under a REAL Tab press (2nd stop), links '/', focus ring #c00 2px. | 2026-09-06 re-verified live: masthead .brand-block reached under a real forward Tab from the skip link and links '/'; present on all 27 crawled routes. | 2026-09-11 re-verified live: masthead .brand-block → '/' reached under a real forward Tab from the skip link on the homepage; present on all 26 crawled routes. | 2026-09-27 re-verified live: masthead .brand-block href '/' (aria-label 'Dexter Jakes home') present on all 22 crawled HTML routes incl. the unmatched-route 404 and /phase0/.</t>
+          <t>PASS — masthead .brand-block → '/' present on home/about/404/phase0/brand/article; aria-label 'Dexter Jakes home' | 2026-08-15 re-verified live: brand-block present and linking / on all 20 pages | 2026-08-25 re-verified live: brand-block present and linking / on all 20 crawled routes; aria-label intact. | 2026-08-27 re-verified live: masthead .brand-block → '/' confirmed under real Tab focus. | 2026-09-01 re-verified live: masthead .brand-block reached under a REAL Tab press (2nd stop), links '/', focus ring #c00 2px. | 2026-09-06 re-verified live: masthead .brand-block reached under a real forward Tab from the skip link and links '/'; present on all 27 crawled routes. | 2026-09-11 re-verified live: masthead .brand-block → '/' reached under a real forward Tab from the skip link on the homepage; present on all 26 crawled routes. | 2026-09-27 re-verified live: masthead .brand-block href '/' (aria-label 'Dexter Jakes home') present on all 22 crawled HTML routes incl. the unmatched-route 404 and /phase0/. | 2026-09-28: live, full regression: .brand-block -&gt; '/' on home/about/article/phase0/404.</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr"/>
@@ -681,7 +681,7 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>PASS — brand-word: Words (home/article/about/brand), 404, Phase 0 — matches documented intent | 2026-08-15 re-verified live: brand-word: home/about/article 'Words', 404 '404', phase0 'Phase 0' — matches the documented about-page quirk | 2026-08-25 re-verified live: brand-word: "Words" on home/about/article, "404" on /404, "Phase 0" on /phase0/ — matches documented intent. | 2026-08-27 re-verified live: brand word 'Words' confirmed on home/article/about. | 2026-09-01 re-verified live on the homepage: masthead brand word reads 'Words' (documented intent). Other surfaces not re-walked this run. | 2026-09-19 re-verified live: brand-word live: 'Words' on /, /about/, /brand/ and all 17 articles; 'Phase 0' on /phase0/; '404' on the unmatched-route 404 — matches documented intent. | 2026-09-27 re-verified live: brand-word 'Words' on /, /about/, /brand/ and all 17 articles; 'Phase 0' on /phase0/; '404' on the unmatched-route 404 — matches documented intent.</t>
+          <t>PASS — brand-word: Words (home/article/about/brand), 404, Phase 0 — matches documented intent | 2026-08-15 re-verified live: brand-word: home/about/article 'Words', 404 '404', phase0 'Phase 0' — matches the documented about-page quirk | 2026-08-25 re-verified live: brand-word: "Words" on home/about/article, "404" on /404, "Phase 0" on /phase0/ — matches documented intent. | 2026-08-27 re-verified live: brand word 'Words' confirmed on home/article/about. | 2026-09-01 re-verified live on the homepage: masthead brand word reads 'Words' (documented intent). Other surfaces not re-walked this run. | 2026-09-19 re-verified live: brand-word live: 'Words' on /, /about/, /brand/ and all 17 articles; 'Phase 0' on /phase0/; '404' on the unmatched-route 404 — matches documented intent. | 2026-09-27 re-verified live: brand-word 'Words' on /, /about/, /brand/ and all 17 articles; 'Phase 0' on /phase0/; '404' on the unmatched-route 404 — matches documented intent. | 2026-09-28: live: brand-word Words (home/about/article), Phase 0 (phase0), 404 (404).</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr"/>
@@ -734,7 +734,7 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>PASS — toggle cycles dark→light→dark; dxmode cookie written both ways; label + aria-pressed + bg/ink all update. Reconfirmed 2026-08-10 PM across 3 consecutive clicks. | 2026-08-13 re-verified live: toggle cycled dark-&gt;light-&gt;dark on the live homepage; dxmode cookie written both ways; --bg/--ink/--accent-text all re-resolved (#060606/#f3f0e8/#ff4d4d dark, #f4f4f1/#050505/#c00 light). | 2026-08-16 re-verified live: toggle cycled dark-&gt;light-&gt;dark on the live homepage; dxmode cookie written both ways (dxmode=light then dxmode=dark); --bg #060606&lt;-&gt;#f4f4f1 and --ink #f3f0e8&lt;-&gt;#050505 both re-resolved; label and aria-pressed tracked ('Mode: Dark'/true &lt;-&gt; 'Mode: Light'/false). | 2026-08-25 re-verified live: toggle re-verified with a REAL pointer click (not element.click()) on both the homepage and /words/the-stone/: page repaints dark&lt;-&gt;light, dxmode cookie written both ways, label and aria-pressed track. METHOD NOTE: a programmatic element.click() flips the class, the tokens and the cookie but leaves body's used background/color stale in getComputedStyle until a repaint is forced — that is a measurement artifact, NOT a site defect, and it read as an article-page mode regression for several minutes this run. Always verify this row with a real click. | 2026-08-27 re-verified live: REAL pointer click (not element.click()) + 2s settle + screenshot: dark→light→dark, --bg #060606↔#f4f4f1, --ink #f3f0e8↔#050505, dxmode cookie written both ways, button label tracks. | 2026-09-01 ISSUE (MEDIUM) — theme-color half of this row has NEVER been satisfiable. mode.js ships syncThemeColor() (js/mode.js:74-95) which rewrites &lt;meta name="theme-color"&gt; to #060606/#f4f4f1 and strips the media attr off a media-split pair, but NO layout ever emitted that meta: document.querySelectorAll('meta[name="theme-color"]').length === 0 on /, /about/, /words/&lt;slug&gt;/, /404, /brand/ and /phase0/ live. querySelector() returned null, the function no-opped, and the dedupe loop iterated an empty list — silent, so five months of scrubs that checked the class/cookie/tokens never saw it. User-visible effect: mobile browser chrome (address/status bar) follows the OS instead of the site's mode. Class flip, dxmode cookie, --bg/--ink re-resolve, aria-pressed, label and logo swap all re-verified live PASS this run with a REAL pointer click + 2s settle. | 2026-09-06 re-verified live: mode toggle driven with a real pointer click (not element.click()) plus a 2.5s settle. dark rgb(6,6,6)/rgb(243,240,232) -&gt; light rgb(244,244,241)/rgb(5,5,5) -&gt; dark, with the dxmode cookie and the 'Mode: Dark'/'Mode: Light' label tracking each flip. | 2026-09-11 re-verified live: real pointer click on .mode-toggle with a 2s settle: dxmode dark→light, html.dark-mode cleared, body rgb(6,6,6)→rgb(244,244,241), theme-color meta →#f4f4f1, label 'Mode: Light'. Screenshot confirmed after the wait. | 2026-09-27 re-verified live: real pointer click on the mode toggle with a 2s settle: dxmode light-&gt;dark, html.dark-mode set, body rgb(6,6,6) on ink rgb(243,240,232), theme-color #060606, aria-pressed true, label 'Mode: Dark', logo -&gt; logo-white.svg; screenshot after the wait confirmed the dark palette. Second real click restored light.</t>
+          <t>PASS — toggle cycles dark→light→dark; dxmode cookie written both ways; label + aria-pressed + bg/ink all update. Reconfirmed 2026-08-10 PM across 3 consecutive clicks. | 2026-08-13 re-verified live: toggle cycled dark-&gt;light-&gt;dark on the live homepage; dxmode cookie written both ways; --bg/--ink/--accent-text all re-resolved (#060606/#f3f0e8/#ff4d4d dark, #f4f4f1/#050505/#c00 light). | 2026-08-16 re-verified live: toggle cycled dark-&gt;light-&gt;dark on the live homepage; dxmode cookie written both ways (dxmode=light then dxmode=dark); --bg #060606&lt;-&gt;#f4f4f1 and --ink #f3f0e8&lt;-&gt;#050505 both re-resolved; label and aria-pressed tracked ('Mode: Dark'/true &lt;-&gt; 'Mode: Light'/false). | 2026-08-25 re-verified live: toggle re-verified with a REAL pointer click (not element.click()) on both the homepage and /words/the-stone/: page repaints dark&lt;-&gt;light, dxmode cookie written both ways, label and aria-pressed track. METHOD NOTE: a programmatic element.click() flips the class, the tokens and the cookie but leaves body's used background/color stale in getComputedStyle until a repaint is forced — that is a measurement artifact, NOT a site defect, and it read as an article-page mode regression for several minutes this run. Always verify this row with a real click. | 2026-08-27 re-verified live: REAL pointer click (not element.click()) + 2s settle + screenshot: dark→light→dark, --bg #060606↔#f4f4f1, --ink #f3f0e8↔#050505, dxmode cookie written both ways, button label tracks. | 2026-09-01 ISSUE (MEDIUM) — theme-color half of this row has NEVER been satisfiable. mode.js ships syncThemeColor() (js/mode.js:74-95) which rewrites &lt;meta name="theme-color"&gt; to #060606/#f4f4f1 and strips the media attr off a media-split pair, but NO layout ever emitted that meta: document.querySelectorAll('meta[name="theme-color"]').length === 0 on /, /about/, /words/&lt;slug&gt;/, /404, /brand/ and /phase0/ live. querySelector() returned null, the function no-opped, and the dedupe loop iterated an empty list — silent, so five months of scrubs that checked the class/cookie/tokens never saw it. User-visible effect: mobile browser chrome (address/status bar) follows the OS instead of the site's mode. Class flip, dxmode cookie, --bg/--ink re-resolve, aria-pressed, label and logo swap all re-verified live PASS this run with a REAL pointer click + 2s settle. | 2026-09-06 re-verified live: mode toggle driven with a real pointer click (not element.click()) plus a 2.5s settle. dark rgb(6,6,6)/rgb(243,240,232) -&gt; light rgb(244,244,241)/rgb(5,5,5) -&gt; dark, with the dxmode cookie and the 'Mode: Dark'/'Mode: Light' label tracking each flip. | 2026-09-11 re-verified live: real pointer click on .mode-toggle with a 2s settle: dxmode dark→light, html.dark-mode cleared, body rgb(6,6,6)→rgb(244,244,241), theme-color meta →#f4f4f1, label 'Mode: Light'. Screenshot confirmed after the wait. | 2026-09-27 re-verified live: real pointer click on the mode toggle with a 2s settle: dxmode light-&gt;dark, html.dark-mode set, body rgb(6,6,6) on ink rgb(243,240,232), theme-color #060606, aria-pressed true, label 'Mode: Dark', logo -&gt; logo-white.svg; screenshot after the wait confirmed the dark palette. Second real click restored light. | 2026-09-28: live: REAL pointer click light-&gt;dark, 2s settle: html.dark-mode, dxmode=dark, label 'Mode: Dark', aria-pressed true, body rgb(6,6,6) / ink rgb(243,240,232); screenshot confirmed.</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
@@ -791,7 +791,7 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: skip link is first focusable; activating it lands document.activeElement on MAIN#archive (home) / MAIN#article (essay); tabindex=-1 present on both landmarks. The 2c7d88d fix holds in production. | 2026-08-13 re-verified live: tab-target verified on live: .skip-link reveals from left:-999px to a 83x69 box at (12,12), cream-on-ink 17.79:1; activating it moved document.activeElement to MAIN#archive (tabindex=-1). Article pages target #article. | 2026-08-16 re-verified live: structural half re-verified live: .skip-link is the first focusable element in document order on every page type, and its target (MAIN#article / MAIN#archive / MAIN#phase0 / MAIN#main) carries tabindex=-1. End-to-end activation NOT re-exercisable this run — the browser pane reports document.visibilityState 'hidden' and drops page focus on every reload, so a fresh-load Tab lands on BODY. Harness limitation, not a site regression; last live activation was 2026-08-13. NOTE: this row's sweep is what surfaced F91 — see that row. | 2026-08-25 re-verified live: verified end-to-end live under REAL keyboard input on /words/the-stone/ — the gap the 2026-08-16 run had to leave open. .skip-link is the first focusable in DOM order, reveals from left:-999px to a 126x46 chip at (12,12), computes 17.79:1 (#060606 on #f3f0e8), and pressing Enter sets location.hash to #article and moves document.activeElement to MAIN#article (tabindex=-1). | 2026-08-27 re-verified live: skip link is the first focusable (reached by real shift+Tab from .brand-block), renders as an opaque cream chip at 17.79:1, and activation moves focus to MAIN#archive with hash #archive. | 2026-09-01 re-verified live: .skip-link is the FIRST Tab stop from page load and matches :focus-visible; activation moves location.hash to #archive and focus to MAIN#archive. Ran the ordinary-link control first per the harness antipattern. | 2026-09-06 re-verified live: skip link is the first focusable, unhides on focus (left -999px -&gt; 12px), and activation moved location.hash to '#archive' and focus to the #archive element. | 2026-09-11 re-verified live: skip link is the first focusable (reached by one shift+Tab back from .brand-block), 17.79:1, #c00 2px ring; activated with a real pointer click → document.activeElement === main#archive, location.hash '#archive'. | 2026-09-19 re-verified live: skip link reached under a real shift+Tab on the homepage (:focus-visible true, #060606 on cream chip, rgb(204,0,0) 2px ring); activation moves focus to #archive (tabindex -1) and sets location.hash. | 2026-09-27 re-verified live: first real Tab from load lands on .skip-link (#archive), :focus-visible true, rgb(204,0,0) 2px solid ring, rgb(244,244,241) on rgb(5,5,5) chip; activation moved focus to #archive and set location.hash.</t>
+          <t>PASS — live-verified 2026-08-10: skip link is first focusable; activating it lands document.activeElement on MAIN#archive (home) / MAIN#article (essay); tabindex=-1 present on both landmarks. The 2c7d88d fix holds in production. | 2026-08-13 re-verified live: tab-target verified on live: .skip-link reveals from left:-999px to a 83x69 box at (12,12), cream-on-ink 17.79:1; activating it moved document.activeElement to MAIN#archive (tabindex=-1). Article pages target #article. | 2026-08-16 re-verified live: structural half re-verified live: .skip-link is the first focusable element in document order on every page type, and its target (MAIN#article / MAIN#archive / MAIN#phase0 / MAIN#main) carries tabindex=-1. End-to-end activation NOT re-exercisable this run — the browser pane reports document.visibilityState 'hidden' and drops page focus on every reload, so a fresh-load Tab lands on BODY. Harness limitation, not a site regression; last live activation was 2026-08-13. NOTE: this row's sweep is what surfaced F91 — see that row. | 2026-08-25 re-verified live: verified end-to-end live under REAL keyboard input on /words/the-stone/ — the gap the 2026-08-16 run had to leave open. .skip-link is the first focusable in DOM order, reveals from left:-999px to a 126x46 chip at (12,12), computes 17.79:1 (#060606 on #f3f0e8), and pressing Enter sets location.hash to #article and moves document.activeElement to MAIN#article (tabindex=-1). | 2026-08-27 re-verified live: skip link is the first focusable (reached by real shift+Tab from .brand-block), renders as an opaque cream chip at 17.79:1, and activation moves focus to MAIN#archive with hash #archive. | 2026-09-01 re-verified live: .skip-link is the FIRST Tab stop from page load and matches :focus-visible; activation moves location.hash to #archive and focus to MAIN#archive. Ran the ordinary-link control first per the harness antipattern. | 2026-09-06 re-verified live: skip link is the first focusable, unhides on focus (left -999px -&gt; 12px), and activation moved location.hash to '#archive' and focus to the #archive element. | 2026-09-11 re-verified live: skip link is the first focusable (reached by one shift+Tab back from .brand-block), 17.79:1, #c00 2px ring; activated with a real pointer click → document.activeElement === main#archive, location.hash '#archive'. | 2026-09-19 re-verified live: skip link reached under a real shift+Tab on the homepage (:focus-visible true, #060606 on cream chip, rgb(204,0,0) 2px ring); activation moves focus to #archive (tabindex -1) and sets location.hash. | 2026-09-27 re-verified live: first real Tab from load lands on .skip-link (#archive), :focus-visible true, rgb(204,0,0) 2px solid ring, rgb(244,244,241) on rgb(5,5,5) chip; activation moved focus to #archive and set location.hash. | 2026-09-28: live: real shift+Tab lands on .skip-link (:focus-visible); activation -&gt; #archive, focus on #archive.</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr"/>
@@ -844,7 +844,7 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>PASS — 2 decorative rulers render | 2026-08-15 re-verified live: zero .ruler-* without aria-hidden across all pages | 2026-09-11 re-verified live: 2 rulers on each of home/article/about/404/phase0, every one aria-hidden=true. | 2026-09-27 re-verified live: 2 rulers on each of 22 crawled HTML routes, every one aria-hidden=true.</t>
+          <t>PASS — 2 decorative rulers render | 2026-08-15 re-verified live: zero .ruler-* without aria-hidden across all pages | 2026-09-11 re-verified live: 2 rulers on each of home/article/about/404/phase0, every one aria-hidden=true. | 2026-09-27 re-verified live: 2 rulers on each of 22 crawled HTML routes, every one aria-hidden=true. | 2026-09-28: live: 2 aria-hidden rulers on all 5 page types.</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr"/>
@@ -893,7 +893,7 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>PASS — footer strip + links present on all page types | 2026-08-15 re-verified live: footer: Instagram + X both target=_blank rel="noopener noreferrer", /feed.xml, /about/, "Built by Dex"; zero _blank links missing rel site-wide | 2026-08-25 re-verified live: footer links resolve: instagram.com/ImJustDex 200, x.com/ImJustDex 200, /feed.xml 200. | 2026-09-11 re-verified live: footer Instagram + X both target=_blank rel='noopener noreferrer', Feed → /feed.xml, About present on home only; 'Built by Dex · Est. 2026' on all three. | 2026-09-27 re-verified live: homepage footer Instagram + X both target=_blank rel='noopener noreferrer', Feed -&gt; /feed.xml, About present; 'Built by Dex · Est. 2026' on home, about, brand, 404 and all 17 articles (/phase0/ carries its own bespoke footer by design); all external footer links 200.</t>
+          <t>PASS — footer strip + links present on all page types | 2026-08-15 re-verified live: footer: Instagram + X both target=_blank rel="noopener noreferrer", /feed.xml, /about/, "Built by Dex"; zero _blank links missing rel site-wide | 2026-08-25 re-verified live: footer links resolve: instagram.com/ImJustDex 200, x.com/ImJustDex 200, /feed.xml 200. | 2026-09-11 re-verified live: footer Instagram + X both target=_blank rel='noopener noreferrer', Feed → /feed.xml, About present on home only; 'Built by Dex · Est. 2026' on all three. | 2026-09-27 re-verified live: homepage footer Instagram + X both target=_blank rel='noopener noreferrer', Feed -&gt; /feed.xml, About present; 'Built by Dex · Est. 2026' on home, about, brand, 404 and all 17 articles (/phase0/ carries its own bespoke footer by design); all external footer links 200. | 2026-09-28: live: footer IG + X target=_blank rel=noopener noreferrer, Feed, 'Est. 2026' on home/about/article/404; About on home only; /phase0/ keeps its bespoke footer (Get Prompt · Essays · year) by design.</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr"/>
@@ -942,7 +942,7 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>PASS (2026-08-15 scrub) — home/about/phase0/articles all carry the feed discovery link; /404 correctly omits it. NOTE: the prior `expected` said articles do NOT include it. That text was stale — ArticleLayout has emitted the link since a4f4f25; the site was never wrong, the row was. Expectation corrected, not the code. | 2026-08-25 re-verified live: &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present in head. | 2026-09-01 re-verified live: &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present in head; /feed.xml 200. | 2026-09-19 re-verified live: feed discovery &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present on /, /about/, /phase0/, /brand/ and all 17 articles; absent on the 404 as specified.</t>
+          <t>PASS (2026-08-15 scrub) — home/about/phase0/articles all carry the feed discovery link; /404 correctly omits it. NOTE: the prior `expected` said articles do NOT include it. That text was stale — ArticleLayout has emitted the link since a4f4f25; the site was never wrong, the row was. Expectation corrected, not the code. | 2026-08-25 re-verified live: &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present in head. | 2026-09-01 re-verified live: &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present in head; /feed.xml 200. | 2026-09-19 re-verified live: feed discovery &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present on /, /about/, /phase0/, /brand/ and all 17 articles; absent on the 404 as specified. | 2026-09-28: live: atom alternate link on home/about/phase0/article; absent on 404 as specified.</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr"/>
@@ -995,7 +995,7 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>PASS — /img/favicon-32.png + /img/apple-touch-icon.png 200 on every referenced path | 2026-08-15 re-verified live: favicon-32.png + apple-touch-icon.png linked on every page; both 200 (1327b / 5729b) | 2026-08-25 re-verified live: /img/favicon-32.png 200, /img/apple-touch-icon.png 200 on every referenced path. | 2026-08-27 re-verified live: /img/favicon-32.png + /img/apple-touch-icon.png 200. | 2026-09-01 re-verified live: /img/favicon-32.png 200, /img/apple-touch-icon.png 200, /img/logo-dark.svg 200. | 2026-09-06 re-verified live: /img/favicon-32.png 200 (1327b), /img/apple-touch-icon.png 200 (5729b), /img/logo-dark.svg 200. | 2026-09-11 re-verified live: /img/favicon-32.png and /img/apple-touch-icon.png both 200, served public,max-age=31536000,immutable.</t>
+          <t>PASS — /img/favicon-32.png + /img/apple-touch-icon.png 200 on every referenced path | 2026-08-15 re-verified live: favicon-32.png + apple-touch-icon.png linked on every page; both 200 (1327b / 5729b) | 2026-08-25 re-verified live: /img/favicon-32.png 200, /img/apple-touch-icon.png 200 on every referenced path. | 2026-08-27 re-verified live: /img/favicon-32.png + /img/apple-touch-icon.png 200. | 2026-09-01 re-verified live: /img/favicon-32.png 200, /img/apple-touch-icon.png 200, /img/logo-dark.svg 200. | 2026-09-06 re-verified live: /img/favicon-32.png 200 (1327b), /img/apple-touch-icon.png 200 (5729b), /img/logo-dark.svg 200. | 2026-09-11 re-verified live: /img/favicon-32.png and /img/apple-touch-icon.png both 200, served public,max-age=31536000,immutable. | 2026-09-28: live: favicon-32 + apple-touch-icon linked on all 5 page types; both 200 immutable.</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr"/>
@@ -1044,7 +1044,7 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>PASS — Anton + IBM Plex Sans self-hosted, preloaded, document.fonts status 'loaded'; CSP font-src intact | 2026-08-15 re-verified live: Anton + IBM Plex Sans preloaded with crossorigin; zero Google Fonts refs; document.fonts reports all 3 faces loaded | 2026-08-16 re-verified live: Anton + IBM Plex Sans (Regular/Bold) all report document.fonts status 'loaded', document.fonts.status 'loaded'; zero Google Fonts references. /brand/ additionally preloads IBMPlexSans-Italic.woff2 and the console warns it is 'not used within a few seconds of load' — investigated and DISMISSED as a non-finding: the italic face is genuinely used by 13 elements on that page and reports status 'loaded'; the warning is a below-the-fold timing artifact. No other page preloads italic, which is correct. | 2026-08-25 re-verified live: document.fonts.status "loaded"; Anton/400, IBM Plex Sans/400 and /700 all report loaded. All three woff2 200. No FOUT observed. | 2026-08-27 re-verified live: document.fonts: Anton 400, IBM Plex Sans 400 + 700 all 'loaded'; fonts.status 'loaded'; no FOUT observed. | 2026-09-01 re-verified live via document.fonts (not the CSS stack): Anton 400 loaded, IBM Plex Sans 400 + 700 loaded; document.fonts.check() true for all three on home and article. No FOUT/FOIT observed. | 2026-09-06 re-verified live: document.fonts reports Anton 400, IBM Plex Sans 400 and 700 all 'loaded' on home and article; all three woff2 files 200 with immutable cache-control. No FOUT observed. | 2026-09-11 re-verified live: document.fonts reports Anton 400 loaded and IBM Plex Sans 400/700 loaded; fonts.check() true for both families. No FOUT observed.</t>
+          <t>PASS — Anton + IBM Plex Sans self-hosted, preloaded, document.fonts status 'loaded'; CSP font-src intact | 2026-08-15 re-verified live: Anton + IBM Plex Sans preloaded with crossorigin; zero Google Fonts refs; document.fonts reports all 3 faces loaded | 2026-08-16 re-verified live: Anton + IBM Plex Sans (Regular/Bold) all report document.fonts status 'loaded', document.fonts.status 'loaded'; zero Google Fonts references. /brand/ additionally preloads IBMPlexSans-Italic.woff2 and the console warns it is 'not used within a few seconds of load' — investigated and DISMISSED as a non-finding: the italic face is genuinely used by 13 elements on that page and reports status 'loaded'; the warning is a below-the-fold timing artifact. No other page preloads italic, which is correct. | 2026-08-25 re-verified live: document.fonts.status "loaded"; Anton/400, IBM Plex Sans/400 and /700 all report loaded. All three woff2 200. No FOUT observed. | 2026-08-27 re-verified live: document.fonts: Anton 400, IBM Plex Sans 400 + 700 all 'loaded'; fonts.status 'loaded'; no FOUT observed. | 2026-09-01 re-verified live via document.fonts (not the CSS stack): Anton 400 loaded, IBM Plex Sans 400 + 700 loaded; document.fonts.check() true for all three on home and article. No FOUT/FOIT observed. | 2026-09-06 re-verified live: document.fonts reports Anton 400, IBM Plex Sans 400 and 700 all 'loaded' on home and article; all three woff2 files 200 with immutable cache-control. No FOUT observed. | 2026-09-11 re-verified live: document.fonts reports Anton 400 loaded and IBM Plex Sans 400/700 loaded; fonts.check() true for both families. No FOUT observed. | 2026-09-28: live: document.fonts loaded Anton 400 + IBM Plex Sans 400/700; font preload with crossorigin on all 5 page types; no Google Fonts.</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr"/>
@@ -1093,7 +1093,7 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>PASS — no horizontal overflow at 390px on home/article/about/phase0/brand/404 | 2026-08-15 re-verified live: viewport width=device-width + viewport-fit=cover on all pages | 2026-09-01 re-verified live at an emulated 375x812: documentElement.scrollWidth == clientWidth == 375 on the article page — zero horizontal overflow. | 2026-09-06 re-verified live at 375x812: homepage and article scrollWidth == clientWidth (no horizontal overflow). | 2026-09-11 re-verified live: 375px homepage and article: scrollWidth == clientWidth == 375, zero elements overflowing the client width, 17 plates intact.</t>
+          <t>PASS — no horizontal overflow at 390px on home/article/about/phase0/brand/404 | 2026-08-15 re-verified live: viewport width=device-width + viewport-fit=cover on all pages | 2026-09-01 re-verified live at an emulated 375x812: documentElement.scrollWidth == clientWidth == 375 on the article page — zero horizontal overflow. | 2026-09-06 re-verified live at 375x812: homepage and article scrollWidth == clientWidth (no horizontal overflow). | 2026-09-11 re-verified live: 375px homepage and article: scrollWidth == clientWidth == 375, zero elements overflowing the client width, 17 plates intact. | 2026-09-28: live: viewport meta (width=device-width, viewport-fit=cover) on all 5 types; at 390px scrollWidth == 390 and 0 overflowing elements on home/article/about/phase0/brand.</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr"/>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>PASS — title/description/canonical on all 21 routes; every canonical on imjustdex.com | 2026-08-15 re-verified live: zero duplicate &lt;title&gt; across 20 pages; /404 canonical is /404 as specified | 2026-08-25 re-verified live: &lt;title&gt;, meta description and canonical present and correct on all 20 routes; every canonical points at imjustdex.com. | 2026-08-27 re-verified live: title/description/canonical present and on-domain across all 21 routes. | 2026-09-01 re-verified live: &lt;title&gt;, meta description and canonical present on all 17 articles plus / and /about/; canonicals all on imjustdex.com. | 2026-09-06 re-verified live: title, meta description and canonical present on all 5 chrome pages and all 17 articles; every canonical on https://imjustdex.com/. | 2026-09-11 re-verified live: title/description/canonical present and imjustdex.com-absolute on all 17 articles + home/about/brand/phase0/404.</t>
+          <t>PASS — title/description/canonical on all 21 routes; every canonical on imjustdex.com | 2026-08-15 re-verified live: zero duplicate &lt;title&gt; across 20 pages; /404 canonical is /404 as specified | 2026-08-25 re-verified live: &lt;title&gt;, meta description and canonical present and correct on all 20 routes; every canonical points at imjustdex.com. | 2026-08-27 re-verified live: title/description/canonical present and on-domain across all 21 routes. | 2026-09-01 re-verified live: &lt;title&gt;, meta description and canonical present on all 17 articles plus / and /about/; canonicals all on imjustdex.com. | 2026-09-06 re-verified live: title, meta description and canonical present on all 5 chrome pages and all 17 articles; every canonical on https://imjustdex.com/. | 2026-09-11 re-verified live: title/description/canonical present and imjustdex.com-absolute on all 17 articles + home/about/brand/phase0/404. | 2026-09-28: live: title + description + canonical on all 21 indexable routes; 404 canonical /404.</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr"/>
@@ -1195,7 +1195,7 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>PASS — og+twitter complete on all 21; all 19 OG images 200 (16 essays + home/about/phase0/brand) | 2026-08-15 re-verified live: twitter:card summary_large_image on every page in scope (404 correctly excluded) | 2026-08-25 re-verified live: og:title / og:description / og:image present on all 20; all 16 og-&lt;slug&gt;.png 200; og:image byte-identical to the JSON-LD image on all 16. | 2026-08-27 re-verified live: og+twitter complete across 21 routes; all 21 distinct OG images 200. | 2026-09-01 re-verified live: og:image resolves 200 on all 17 articles and every one matches the JSON-LD image URL exactly, cache-bust included. | 2026-09-06 re-verified live: og:title / og:description / og:image present on all 5 chrome pages and all 17 articles; og:image matches the JSON-LD image byte-for-byte on 17/17. | 2026-09-11 re-verified live: og:title/og:description/og:image present on all 22 HTML routes; every og:image resolves 200.</t>
+          <t>PASS — og+twitter complete on all 21; all 19 OG images 200 (16 essays + home/about/phase0/brand) | 2026-08-15 re-verified live: twitter:card summary_large_image on every page in scope (404 correctly excluded) | 2026-08-25 re-verified live: og:title / og:description / og:image present on all 20; all 16 og-&lt;slug&gt;.png 200; og:image byte-identical to the JSON-LD image on all 16. | 2026-08-27 re-verified live: og+twitter complete across 21 routes; all 21 distinct OG images 200. | 2026-09-01 re-verified live: og:image resolves 200 on all 17 articles and every one matches the JSON-LD image URL exactly, cache-bust included. | 2026-09-06 re-verified live: og:title / og:description / og:image present on all 5 chrome pages and all 17 articles; og:image matches the JSON-LD image byte-for-byte on 17/17. | 2026-09-11 re-verified live: og:title/og:description/og:image present on all 22 HTML routes; every og:image resolves 200. | 2026-09-28: live: og + twitter complete on 21 routes; all OG images 200. (/phase0/ omits the optional og:image:width/height hints — not flagged.)</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr"/>
@@ -1248,7 +1248,7 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>PASS — WebSite + Person @graph complete (name/url/sameAs/jobTitle/worksFor) | 2026-08-15 re-verified live: home @graph carries WebSite + Person; Person has name/url/sameAs/jobTitle/worksFor — no missing fields | 2026-08-25 re-verified live: WebSite + Person @graph complete on /; Person carries name, url, sameAs, jobTitle, worksFor. | 2026-08-27 re-verified live: WebSite + Person @graph complete (name/url/sameAs/jobTitle/worksFor). | 2026-09-01 re-verified live: homepage @graph carries WebSite + Person; Person has name, url, sameAs, jobTitle, worksFor — zero required fields missing. | 2026-09-06 re-verified live: homepage @graph carries WebSite + Person; Person complete on name/url/sameAs/jobTitle/worksFor. | 2026-09-11 re-verified live: homepage @graph carries WebSite + Person; Person has name, url, sameAs, jobTitle, worksFor.</t>
+          <t>PASS — WebSite + Person @graph complete (name/url/sameAs/jobTitle/worksFor) | 2026-08-15 re-verified live: home @graph carries WebSite + Person; Person has name/url/sameAs/jobTitle/worksFor — no missing fields | 2026-08-25 re-verified live: WebSite + Person @graph complete on /; Person carries name, url, sameAs, jobTitle, worksFor. | 2026-08-27 re-verified live: WebSite + Person @graph complete (name/url/sameAs/jobTitle/worksFor). | 2026-09-01 re-verified live: homepage @graph carries WebSite + Person; Person has name, url, sameAs, jobTitle, worksFor — zero required fields missing. | 2026-09-06 re-verified live: homepage @graph carries WebSite + Person; Person complete on name/url/sameAs/jobTitle/worksFor. | 2026-09-11 re-verified live: homepage @graph carries WebSite + Person; Person has name, url, sameAs, jobTitle, worksFor. | 2026-09-28: live: WebSite + Person @graph; Person has name/url/sameAs/jobTitle/worksFor.</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr"/>
@@ -1297,7 +1297,7 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>PASS — ProfilePage mainEntity Person complete (name/url/jobTitle/worksFor/sameAs/description) | 2026-08-15 re-verified live: about ProfilePage mainEntity Person complete — name/url/jobTitle/worksFor/sameAs/description all present | 2026-08-25 re-verified live: ProfilePage on /about/ with mainEntity @type Person carrying name, url, jobTitle, worksFor, sameAs, description. | 2026-08-27 re-verified live: ProfilePage mainEntity Person complete (name/url/jobTitle/worksFor/sameAs/description). | 2026-09-01 re-verified live: /about/ ProfilePage mainEntity is @type Person with name, url, jobTitle, worksFor, sameAs, description — zero missing. | 2026-09-06 re-verified live: /about/ ProfilePage present, mainEntity @type=Person complete on name/url/jobTitle/worksFor/sameAs/description. | 2026-09-11 re-verified live: /about/ ProfilePage mainEntity is a Person with all six required fields present.</t>
+          <t>PASS — ProfilePage mainEntity Person complete (name/url/jobTitle/worksFor/sameAs/description) | 2026-08-15 re-verified live: about ProfilePage mainEntity Person complete — name/url/jobTitle/worksFor/sameAs/description all present | 2026-08-25 re-verified live: ProfilePage on /about/ with mainEntity @type Person carrying name, url, jobTitle, worksFor, sameAs, description. | 2026-08-27 re-verified live: ProfilePage mainEntity Person complete (name/url/jobTitle/worksFor/sameAs/description). | 2026-09-01 re-verified live: /about/ ProfilePage mainEntity is @type Person with name, url, jobTitle, worksFor, sameAs, description — zero missing. | 2026-09-06 re-verified live: /about/ ProfilePage present, mainEntity @type=Person complete on name/url/jobTitle/worksFor/sameAs/description. | 2026-09-11 re-verified live: /about/ ProfilePage mainEntity is a Person with all six required fields present. | 2026-09-28: live: ProfilePage mainEntity Person with name/url/jobTitle/worksFor/sameAs/description.</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr"/>
@@ -1346,7 +1346,7 @@
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>PASS — BlogPosting complete on all 16 (headline, description, datePublished, dateModified, author Person, publisher Organization+logo, mainEntityOfPage, image, url, inLanguage, wordCount); image == og:image exactly, no og-default drift | 2026-08-13 re-verified live: all 16 BlogPosting blocks carry every required field (headline, description, datePublished, dateModified, author.@type=Person + name, publisher, mainEntityOfPage, image, url, inLanguage, wordCount); zero og-default.png drift. | 2026-08-16 re-verified live: all 16 BlogPosting blocks re-verified live: every required field present (headline, description, datePublished, dateModified, author.@type=Person, publisher, mainEntityOfPage, image, url, inLanguage, wordCount) and JSON-LD image === og:image exactly, cache-bust included, on all 16. Zero og-default.png drift. | 2026-08-25 re-verified live: BlogPosting on all 16 articles; every required field present (headline, description, datePublished, dateModified, author.Person.name, publisher, mainEntityOfPage, image, url, inLanguage, wordCount). Zero og-default.png regressions. | 2026-08-27 re-verified live: BlogPosting complete on all 16 — all 11 required fields, author.@type=Person, og:image == JSON-LD image, image == og-&lt;slug&gt;.png on every one. | 2026-09-01 re-verified live: all 17 BlogPosting blocks carry every required field (headline, description, datePublished, dateModified, author.@type=Person + name, publisher, mainEntityOfPage, image, url, inLanguage, wordCount). Zero on og-default.png. | 2026-09-06 re-verified live: 17/17 BlogPosting blocks complete on all 11 required fields, author @type=Person with name, image per-slug. | 2026-09-11 re-verified live: all 17 BlogPosting blocks carry the full 11-field set; author is Person with a name.</t>
+          <t>PASS — BlogPosting complete on all 16 (headline, description, datePublished, dateModified, author Person, publisher Organization+logo, mainEntityOfPage, image, url, inLanguage, wordCount); image == og:image exactly, no og-default drift | 2026-08-13 re-verified live: all 16 BlogPosting blocks carry every required field (headline, description, datePublished, dateModified, author.@type=Person + name, publisher, mainEntityOfPage, image, url, inLanguage, wordCount); zero og-default.png drift. | 2026-08-16 re-verified live: all 16 BlogPosting blocks re-verified live: every required field present (headline, description, datePublished, dateModified, author.@type=Person, publisher, mainEntityOfPage, image, url, inLanguage, wordCount) and JSON-LD image === og:image exactly, cache-bust included, on all 16. Zero og-default.png drift. | 2026-08-25 re-verified live: BlogPosting on all 16 articles; every required field present (headline, description, datePublished, dateModified, author.Person.name, publisher, mainEntityOfPage, image, url, inLanguage, wordCount). Zero og-default.png regressions. | 2026-08-27 re-verified live: BlogPosting complete on all 16 — all 11 required fields, author.@type=Person, og:image == JSON-LD image, image == og-&lt;slug&gt;.png on every one. | 2026-09-01 re-verified live: all 17 BlogPosting blocks carry every required field (headline, description, datePublished, dateModified, author.@type=Person + name, publisher, mainEntityOfPage, image, url, inLanguage, wordCount). Zero on og-default.png. | 2026-09-06 re-verified live: 17/17 BlogPosting blocks complete on all 11 required fields, author @type=Person with name, image per-slug. | 2026-09-11 re-verified live: all 17 BlogPosting blocks carry the full 11-field set; author is Person with a name. | 2026-09-28: live: BlogPosting complete 17/17 (all 12 required fields, author @type Person).</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr"/>
@@ -1395,7 +1395,7 @@
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>PASS — phase0 WebPage JSON-LD present and parses | 2026-08-27 re-verified live: phase0 WebPage + Person JSON-LD present and parse. | 2026-09-11 re-verified live: /phase0/ @graph = WebPage(#webpage) isPartOf #website, author #person. Valid JSON-LD.</t>
+          <t>PASS — phase0 WebPage JSON-LD present and parses | 2026-08-27 re-verified live: phase0 WebPage + Person JSON-LD present and parse. | 2026-09-11 re-verified live: /phase0/ @graph = WebPage(#webpage) isPartOf #website, author #person. Valid JSON-LD. | 2026-09-28: live: WebPage isPartOf #website, author #person.</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr"/>
@@ -1444,7 +1444,7 @@
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>PASS — robots.txt Allow / + Sitemap → sitemap-index.xml | 2026-08-13 re-verified live: /robots.txt 200, Sitemap directive -&gt; https://imjustdex.com/sitemap-index.xml. | 2026-08-25 re-verified live: robots.txt = "User-agent: *\nAllow: /\n\nSitemap: https://imjustdex.com/sitemap-index.xml". /DESIGN-SYSTEM.md correctly 404s. | 2026-08-27 re-verified live: robots.txt Allow / + Sitemap → sitemap-index.xml. | 2026-09-01 re-verified live: robots.txt is 'User-agent: * / Allow: / / Sitemap: https://imjustdex.com/sitemap-index.xml'. /DESIGN-SYSTEM.md still 404s (the only thing keeping the doc unexposed). | 2026-09-06 re-verified live: robots.txt is 'User-agent: * / Allow: / / Sitemap: https://imjustdex.com/sitemap-index.xml'. | 2026-09-11 re-verified live: robots.txt = 'User-agent: * / Allow: / / Sitemap: https://imjustdex.com/sitemap-index.xml'.</t>
+          <t>PASS — robots.txt Allow / + Sitemap → sitemap-index.xml | 2026-08-13 re-verified live: /robots.txt 200, Sitemap directive -&gt; https://imjustdex.com/sitemap-index.xml. | 2026-08-25 re-verified live: robots.txt = "User-agent: *\nAllow: /\n\nSitemap: https://imjustdex.com/sitemap-index.xml". /DESIGN-SYSTEM.md correctly 404s. | 2026-08-27 re-verified live: robots.txt Allow / + Sitemap → sitemap-index.xml. | 2026-09-01 re-verified live: robots.txt is 'User-agent: * / Allow: / / Sitemap: https://imjustdex.com/sitemap-index.xml'. /DESIGN-SYSTEM.md still 404s (the only thing keeping the doc unexposed). | 2026-09-06 re-verified live: robots.txt is 'User-agent: * / Allow: / / Sitemap: https://imjustdex.com/sitemap-index.xml'. | 2026-09-11 re-verified live: robots.txt = 'User-agent: * / Allow: / / Sitemap: https://imjustdex.com/sitemap-index.xml'. | 2026-09-28: live: Allow / + Sitemap -&gt; sitemap-index.xml.</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr"/>
@@ -1493,7 +1493,7 @@
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>PASS — sitemap-0.xml 20 locs = exactly the published set + about/brand/phase0; no missing, no orphans | 2026-08-13 re-verified live: /sitemap-index.xml -&gt; sitemap-0.xml; sitemap-0 lists 20 URLs covering all 16 articles + /, /about/, /brand/, /phase0/. Zero missing. | 2026-08-25 re-verified live: sitemap-index.xml references sitemap-0.xml; sitemap-0.xml carries exactly 20 locs = 16 articles + /, /about/, /brand/, /phase0/. The drafted essay is correctly absent. | 2026-08-27 re-verified live: sitemap-0.xml 20 locs; every homepage-linked route plus /about/ /brand/ /phase0/ present. | 2026-09-01 re-verified live: /sitemap-index.xml points to sitemap-0.xml; sitemap-0.xml holds exactly 21 URLs — the 17 live articles plus /, /about/, /brand/, /phase0/. Zero missing, zero extra. The drafted entry before-i-had-the-words is correctly absent. | 2026-09-06 re-verified live: sitemap-index.xml points at sitemap-0.xml; sitemap-0.xml carries 21 URLs and includes all 17 articles plus /, /about/, /brand/, /phase0/. | 2026-09-11 re-verified live: sitemap-index → sitemap-0; 21 locs = 17 articles + /, /about/, /brand/, /phase0/. No drafts leaked (before-i-had-the-words absent).</t>
+          <t>PASS — sitemap-0.xml 20 locs = exactly the published set + about/brand/phase0; no missing, no orphans | 2026-08-13 re-verified live: /sitemap-index.xml -&gt; sitemap-0.xml; sitemap-0 lists 20 URLs covering all 16 articles + /, /about/, /brand/, /phase0/. Zero missing. | 2026-08-25 re-verified live: sitemap-index.xml references sitemap-0.xml; sitemap-0.xml carries exactly 20 locs = 16 articles + /, /about/, /brand/, /phase0/. The drafted essay is correctly absent. | 2026-08-27 re-verified live: sitemap-0.xml 20 locs; every homepage-linked route plus /about/ /brand/ /phase0/ present. | 2026-09-01 re-verified live: /sitemap-index.xml points to sitemap-0.xml; sitemap-0.xml holds exactly 21 URLs — the 17 live articles plus /, /about/, /brand/, /phase0/. Zero missing, zero extra. The drafted entry before-i-had-the-words is correctly absent. | 2026-09-06 re-verified live: sitemap-index.xml points at sitemap-0.xml; sitemap-0.xml carries 21 URLs and includes all 17 articles plus /, /about/, /brand/, /phase0/. | 2026-09-11 re-verified live: sitemap-index → sitemap-0; 21 locs = 17 articles + /, /about/, /brand/, /phase0/. No drafts leaked (before-i-had-the-words absent). | 2026-09-28: live: sitemap-0.xml 21 locs = 17 essays + home/about/brand/phase0; throwaway fixture build: a future-dated entry is excluded.</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr"/>
@@ -1546,14 +1546,14 @@
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>404 half PASS (noindex,nofollow live). Coming-soon half PENDING — no upcoming entry exists to render one | 2026-08-25: 404 half re-verified live (meta robots noindex,nofollow present, bespoke body served at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one. | 2026-09-01 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one. | 2026-09-11: 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body at HTTP 200). Coming-soon half still PENDING — 17 published entries, all past-dated, so isUpcomingData() is false everywhere and no ComingSoonLayout renders. | 2026-09-19: 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body, HTTP 404 on unmatched route). Coming-soon half still PENDING — 17 published entries, all past-dated; the untracked before-i-had-the-words.mdx in Dexter's working tree is still status 'drafted'. | 2026-09-23: 404 half re-verified live (noindex, nofollow). Coming-soon half still PENDING — 17/17 entries status published, no upcoming entry to render. | 2026-09-25: still PENDING — 17/17 entries status published and past-dated, no upcoming entry to render. 404 half re-verified live: meta robots noindex present, bespoke body, unmatched route 404.</t>
+          <t>404 half PASS (noindex,nofollow live). Coming-soon half PENDING — no upcoming entry exists to render one | 2026-08-25: 404 half re-verified live (meta robots noindex,nofollow present, bespoke body served at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one. | 2026-09-01 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one. | 2026-09-11: 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body at HTTP 200). Coming-soon half still PENDING — 17 published entries, all past-dated, so isUpcomingData() is false everywhere and no ComingSoonLayout renders. | 2026-09-19: 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body, HTTP 404 on unmatched route). Coming-soon half still PENDING — 17 published entries, all past-dated; the untracked before-i-had-the-words.mdx in Dexter's working tree is still status 'drafted'. | 2026-09-23: 404 half re-verified live (noindex, nofollow). Coming-soon half still PENDING — 17/17 entries status published, no upcoming entry to render. | 2026-09-25: still PENDING — 17/17 entries status published and past-dated, no upcoming entry to render. 404 half re-verified live: meta robots noindex present, bespoke body, unmatched route 404. | 2026-09-28: 404 half re-verified live (noindex, nofollow). Coming-soon half BUILD-VERIFIED via a throwaway future-dated fixture in a scratch copy (never committed): ComingSoonLayout emits &lt;meta name=robots content=noindex&gt;.</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr"/>
       <c r="J22" s="4" t="inlineStr"/>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t>PENDING | 2026-09-18: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-26: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-27: still structurally untestable — 0 upcoming entries in the committed collection (17/17 published, past-dated).</t>
+          <t>PENDING | 2026-09-18: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-26: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-27: still structurally untestable — 0 upcoming entries in the committed collection (17/17 published, past-dated). | 2026-09-28: PASS (404 live + coming-soon verified against a fixture build) — first time the coming-soon half has been exercised since the collection went all-published.</t>
         </is>
       </c>
     </row>
@@ -1595,7 +1595,7 @@
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>PASS — Entry No. 16 / Week of July 5, 2026, LatestBar → newest essay | 2026-08-13 re-verified live: LatestBar reads 'Entry No. 16 / Week of July 5, 2026' and links to /words/send-someone-else/ (the newest). NOTE: its .latest-tag chip is the F77 finding this run. | 2026-08-25 re-verified live: issue head renders "Entry No. 16" / "Week of July 5, 2026" from the lead; standfirst links /words/send-someone-else/. | 2026-08-27 re-verified live: issue head 'Entry No. 16 / Week of July 5, 2026', LatestBar → send-someone-else. | 2026-09-11 re-verified live: LatestBar: 'Entry No. 17' (= 17 published essays), 'Week of August 31, 2026', latest link → /words/the-weight-of-my-no/.</t>
+          <t>PASS — Entry No. 16 / Week of July 5, 2026, LatestBar → newest essay | 2026-08-13 re-verified live: LatestBar reads 'Entry No. 16 / Week of July 5, 2026' and links to /words/send-someone-else/ (the newest). NOTE: its .latest-tag chip is the F77 finding this run. | 2026-08-25 re-verified live: issue head renders "Entry No. 16" / "Week of July 5, 2026" from the lead; standfirst links /words/send-someone-else/. | 2026-08-27 re-verified live: issue head 'Entry No. 16 / Week of July 5, 2026', LatestBar → send-someone-else. | 2026-09-11 re-verified live: LatestBar: 'Entry No. 17' (= 17 published essays), 'Week of August 31, 2026', latest link → /words/the-weight-of-my-no/. | 2026-09-28: live: 'Entry No. 17', 'Week of August 31, 2026', Latest -&gt; the-weight-of-my-no, 'Faith · Aug 31 · 8 min'.</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr"/>
@@ -1648,7 +1648,7 @@
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>PASS — IdentityHero renders; hero copy contrast 5.17:1 (AA large) | 2026-08-27 re-verified live: IdentityHero renders (screenshot-confirmed in both modes). | 2026-09-11 re-verified live: IdentityHero: name + 'ImJustDex' render; hero links → /about/ and #subscribe-manifesto.</t>
+          <t>PASS — IdentityHero renders; hero copy contrast 5.17:1 (AA large) | 2026-08-27 re-verified live: IdentityHero renders (screenshot-confirmed in both modes). | 2026-09-11 re-verified live: IdentityHero: name + 'ImJustDex' render; hero links → /about/ and #subscribe-manifesto. | 2026-09-28: live: hero name/sub/tagline/bio, 'Read the About' -&gt; /about/, 'Subscribe' -&gt; #subscribe-manifesto.</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr"/>
@@ -1697,7 +1697,7 @@
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>PASS — Faith 13 / Identity 09 / Art 03, verified against frontmatter lanes; 16 articles | 2026-08-13 re-verified live: lane-index counts Faith 13 / Identity 09 / Art 03 — non-negative, zero-padded, and consistent with 16 essays counted per lane (15 .plate-lane chips + 1 .lead-badge-lane). | 2026-08-25 re-verified live: lane counts render Faith 13 / Identity 09 / Art 03 — matches the frontmatter tally across the 16 tracked essays exactly (multi-lane counted per lane). | 2026-08-27 re-verified live: lane counts Faith 13 / Identity 09 / Art 03. | 2026-09-01 re-verified live: lane-index reads Faith 14 / Identity 10 / Art 03 — non-negative integers summing to 27 across 17 essays (multi-lane counted per lane). Cross-checked against the filter: selecting Faith reveals exactly 14 articles. | 2026-09-06 re-verified live: lane index reads Faith 14 / Identity 10 / Art 03 (sum 27 across 17 essays, multi-lane counted per lane). | 2026-09-11 re-verified live: lane counts Faith 14 / Identity 10 / Art 03; sum 27 over 17 articles (multi-lane essays count per lane), all non-negative integers.</t>
+          <t>PASS — Faith 13 / Identity 09 / Art 03, verified against frontmatter lanes; 16 articles | 2026-08-13 re-verified live: lane-index counts Faith 13 / Identity 09 / Art 03 — non-negative, zero-padded, and consistent with 16 essays counted per lane (15 .plate-lane chips + 1 .lead-badge-lane). | 2026-08-25 re-verified live: lane counts render Faith 13 / Identity 09 / Art 03 — matches the frontmatter tally across the 16 tracked essays exactly (multi-lane counted per lane). | 2026-08-27 re-verified live: lane counts Faith 13 / Identity 09 / Art 03. | 2026-09-01 re-verified live: lane-index reads Faith 14 / Identity 10 / Art 03 — non-negative integers summing to 27 across 17 essays (multi-lane counted per lane). Cross-checked against the filter: selecting Faith reveals exactly 14 articles. | 2026-09-06 re-verified live: lane index reads Faith 14 / Identity 10 / Art 03 (sum 27 across 17 essays, multi-lane counted per lane). | 2026-09-11 re-verified live: lane counts Faith 14 / Identity 10 / Art 03; sum 27 over 17 articles (multi-lane essays count per lane), all non-negative integers. | 2026-09-28: live: Faith 14 / Identity 10 / Art 03 essays (no zero lane, so the queued state is not exercised).</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr"/>
@@ -1750,7 +1750,7 @@
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: Faith 13/13, Identity 9/9, Art 3/3 with zero non-matching plates in any filtered view; while filtered the .earlier-more-wrap computes display:none, 0 client rects, offsetHeight 0 (unreachable by mouse or keyboard). The ab07b15 fix holds in production. | 2026-08-16 re-verified live: all three lanes re-verified live: Faith 13, Identity 9, Art 3 — exactly matching the lane-index counts. Verified against the real filter key (data-lane, space-separated) rather than the visible chips: all 9 identity plates carry 'identity' in data-lane. While filtered, .earlier-more-wrap computes display:none with 0 client rects; clearing restores display:flex. | 2026-08-27 re-verified live: real pointer clicks: Faith 13, Identity 9, Art 3, re-click clears to the default 8; aria-pressed single-select correct. | 2026-09-01 re-verified live: .lane-cell[data-lane=faith] click sets aria-pressed=true and reveals exactly 14 articles; clicking again returns aria-pressed=false and the default 7-article view. | 2026-09-06 re-verified live: clicking the Art lane cell filtered the cascade 7 -&gt; 3 visible articles (Music That Raised Me, Useful Is Not the Same, Groan Beneath the Song), aria-pressed=true, and a second click restored 7. | 2026-09-11 re-verified live: lane filter 'art' → 3 visible articles, matching its announced count; aria-pressed true→false; clearing restores 7.</t>
+          <t>PASS — live-verified 2026-08-10: Faith 13/13, Identity 9/9, Art 3/3 with zero non-matching plates in any filtered view; while filtered the .earlier-more-wrap computes display:none, 0 client rects, offsetHeight 0 (unreachable by mouse or keyboard). The ab07b15 fix holds in production. | 2026-08-16 re-verified live: all three lanes re-verified live: Faith 13, Identity 9, Art 3 — exactly matching the lane-index counts. Verified against the real filter key (data-lane, space-separated) rather than the visible chips: all 9 identity plates carry 'identity' in data-lane. While filtered, .earlier-more-wrap computes display:none with 0 client rects; clearing restores display:flex. | 2026-08-27 re-verified live: real pointer clicks: Faith 13, Identity 9, Art 3, re-click clears to the default 8; aria-pressed single-select correct. | 2026-09-01 re-verified live: .lane-cell[data-lane=faith] click sets aria-pressed=true and reveals exactly 14 articles; clicking again returns aria-pressed=false and the default 7-article view. | 2026-09-06 re-verified live: clicking the Art lane cell filtered the cascade 7 -&gt; 3 visible articles (Music That Raised Me, Useful Is Not the Same, Groan Beneath the Song), aria-pressed=true, and a second click restored 7. | 2026-09-11 re-verified live: lane filter 'art' → 3 visible articles, matching its announced count; aria-pressed true→false; clearing restores 7. | 2026-09-28: live: Faith -&gt; aria-pressed true, 14 visible, all data-lane faith; re-click clears (7 visible); Art -&gt; 3.</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr"/>
@@ -1803,7 +1803,7 @@
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>PASS — lead plate = send-someone-else (newest published) | 2026-08-25 re-verified live: lead plate renders send-someone-else with correct eyebrow, deck and 16 min read. | 2026-08-27 re-verified live: lead plate = send-someone-else. | 2026-09-11 re-verified live: LeadPlate renders the newest essay with Latest badge and Read CTA, href /words/the-weight-of-my-no/.</t>
+          <t>PASS — lead plate = send-someone-else (newest published) | 2026-08-25 re-verified live: lead plate renders send-someone-else with correct eyebrow, deck and 16 min read. | 2026-08-27 re-verified live: lead plate = send-someone-else. | 2026-09-11 re-verified live: LeadPlate renders the newest essay with Latest badge and Read CTA, href /words/the-weight-of-my-no/. | 2026-09-28: live: lead = the-weight-of-my-no with Latest badge, Faith, &lt;time 2026-08-31&gt;, 8 min, Read -&gt;.</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr"/>
@@ -1852,7 +1852,7 @@
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>PASS — 'This Month' = show-me-your-glory (same month as lead) | 2026-08-27 re-verified live: row heads 'This Week' (01, lead) and 'This Month' (02) both render as authored. | 2026-09-18 re-verified live: 'This Month' correctly hidden — no other essay shares the lead's month (Aug 2026); row heads read 01 This Week / 02 Earlier.</t>
+          <t>PASS — 'This Month' = show-me-your-glory (same month as lead) | 2026-08-27 re-verified live: row heads 'This Week' (01, lead) and 'This Month' (02) both render as authored. | 2026-09-18 re-verified live: 'This Month' correctly hidden — no other essay shares the lead's month (Aug 2026); row heads read 01 This Week / 02 Earlier. | 2026-09-28: live: correctly hidden — no other essay shares the lead's month (Aug 2026); row heads read 'Latest', 'Earlier'.</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr"/>
@@ -1901,7 +1901,7 @@
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>PASS — 'Earlier' = 14, 6 visible + 8 overflow | 2026-08-27 re-verified live: 8 of 16 plates visible by default, 8 under the overflow. | 2026-09-18 re-verified live: 'Earlier' = 16, 6 visible + 10 under the overflow; 7 of 17 plates visible by default.</t>
+          <t>PASS — 'Earlier' = 14, 6 visible + 8 overflow | 2026-08-27 re-verified live: 8 of 16 plates visible by default, 8 under the overflow. | 2026-09-18 re-verified live: 'Earlier' = 16, 6 visible + 10 under the overflow; 7 of 17 plates visible by default. | 2026-09-28: live: 'Earlier' numbered 02 (no This Month), 16 essays: 6 visible + 10 in .earlier-more.</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr"/>
@@ -1954,7 +1954,7 @@
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: expand 8→16, collapse 16→8, aria-expanded false↔true and the button label track; collapse state survives a full filter cycle (clear restores the wrap to display:flex). | 2026-08-16 re-verified live: expand 8-&gt;16 and collapse 16-&gt;8 re-verified live; aria-expanded false&lt;-&gt;true and the label tracked ('View Earlier Essays — 8 more' &lt;-&gt; 'Show Less — showing all'); collapse state survived a full filter cycle. | 2026-08-27 re-verified live: real pointer clicks: 8→16→8, aria-expanded false↔true, label and count track. | 2026-09-01 re-verified live: toggle expands 10 hidden articles to 0 hidden, label 'View Earlier Essays — 10 more' -&gt; 'Show Less — showing all', aria-expanded false-&gt;true; collapse restores all three. | 2026-09-06 re-verified live: View Earlier 7 -&gt; 17 -&gt; 7 with label 'View Earlier Essays - 10 more' &lt;-&gt; 'Show Less - showing all' and aria-expanded true/false. | 2026-09-11 re-verified live: toggle 7↔17 articles, label 'View Earlier Essays — 10 more ↓' ↔ 'Show Less — showing all ↑', aria-expanded false↔true.</t>
+          <t>PASS — live-verified 2026-08-10: expand 8→16, collapse 16→8, aria-expanded false↔true and the button label track; collapse state survives a full filter cycle (clear restores the wrap to display:flex). | 2026-08-16 re-verified live: expand 8-&gt;16 and collapse 16-&gt;8 re-verified live; aria-expanded false&lt;-&gt;true and the label tracked ('View Earlier Essays — 8 more' &lt;-&gt; 'Show Less — showing all'); collapse state survived a full filter cycle. | 2026-08-27 re-verified live: real pointer clicks: 8→16→8, aria-expanded false↔true, label and count track. | 2026-09-01 re-verified live: toggle expands 10 hidden articles to 0 hidden, label 'View Earlier Essays — 10 more' -&gt; 'Show Less — showing all', aria-expanded false-&gt;true; collapse restores all three. | 2026-09-06 re-verified live: View Earlier 7 -&gt; 17 -&gt; 7 with label 'View Earlier Essays - 10 more' &lt;-&gt; 'Show Less - showing all' and aria-expanded true/false. | 2026-09-11 re-verified live: toggle 7↔17 articles, label 'View Earlier Essays — 10 more ↓' ↔ 'Show Less — showing all ↑', aria-expanded false↔true. | 2026-09-28: live: 'View Earlier Essays — 10 more ↓' -&gt; 'Show Less — showing all ↑', aria-expanded false-&gt;true-&gt;false, 7-&gt;17-&gt;7 visible.</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr"/>
@@ -2007,7 +2007,7 @@
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>PASS — 16 plates tile the 12-col grid (lead + wide/secondary/banner rotation, 3 row-plates) | 2026-09-18 re-verified live: 7 visible plates tile the 12-col grid as lead + wide/secondary/banner/secondary/banner/wide; 17 plates total with the 10-plate overflow under View More.</t>
+          <t>PASS — 16 plates tile the 12-col grid (lead + wide/secondary/banner rotation, 3 row-plates) | 2026-09-18 re-verified live: 7 visible plates tile the 12-col grid as lead + wide/secondary/banner/secondary/banner/wide; 17 plates total with the 10-plate overflow under View More. | 2026-09-28: live: 17 .plate elements render in the cascade; packer source unchanged since last PASS.</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr"/>
@@ -2056,7 +2056,7 @@
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>PASS — 7 of 15 archive plates carry .plate-image, interleaved with plain (Texture Alternation Rule) | 2026-09-06 re-verified live: eight image plates alternate concrete/lines/noise as designed. NOTE - this run pixel-measured them rather than reading computed styles and found the scrim, not the alternation, at fault; see F101. | 2026-09-11 re-verified live: three homepage image plates alternate img-concrete / img-lines / img-noise across the cascade.</t>
+          <t>PASS — 7 of 15 archive plates carry .plate-image, interleaved with plain (Texture Alternation Rule) | 2026-09-06 re-verified live: eight image plates alternate concrete/lines/noise as designed. NOTE - this run pixel-measured them rather than reading computed styles and found the scrim, not the alternation, at fault; see F101. | 2026-09-11 re-verified live: three homepage image plates alternate img-concrete / img-lines / img-noise across the cascade. | 2026-09-28: live: 8 of 16 archive plates carry .plate-image; source unchanged.</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr"/>
@@ -2158,7 +2158,7 @@
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>PASS — manifesto form action=/api/subscribe, source=home, honeypot present | 2026-08-27 re-verified live: manifesto form + #sm-email + submit present on the homepage. | 2026-09-18 re-verified live: manifesto form action=/api/subscribe, #sm-email present, 3 value-prop items, 'No spam' line, honeypot off-canvas (x=-9999, tabindex=-1, aria-hidden).</t>
+          <t>PASS — manifesto form action=/api/subscribe, source=home, honeypot present | 2026-08-27 re-verified live: manifesto form + #sm-email + submit present on the homepage. | 2026-09-18 re-verified live: manifesto form action=/api/subscribe, #sm-email present, 3 value-prop items, 'No spam' line, honeypot off-canvas (x=-9999, tabindex=-1, aria-hidden). | 2026-09-28: live: #subscribe-manifesto, 3 value-prop items, 'No spam', action /api/subscribe, source=home.</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr"/>
@@ -2207,7 +2207,7 @@
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>PASS | 2026-09-18 re-verified live: real submit on the home manifesto form with a server-rejected address (healthscrub@invalid, passes type=email) showed 'Sending…', then state=error with 'That email didn't look right. Try it again.' in a role=alert .sm-error and the button re-enabled. Success path covered by the §9 API smoke (200 subscribed); the UI success state was not driven to avoid a second subscriber write.</t>
+          <t>PASS | 2026-09-18 re-verified live: real submit on the home manifesto form with a server-rejected address (healthscrub@invalid, passes type=email) showed 'Sending…', then state=error with 'That email didn't look right. Try it again.' in a role=alert .sm-error and the button re-enabled. Success path covered by the §9 API smoke (200 subscribed); the UI success state was not driven to avoid a second subscriber write. | 2026-09-28: carried: subscribe.js unchanged; endpoint states verified by API tests today (200 subscribed / already_subscribed / 400 invalid_email / 429). Not browser-submitted today to avoid extra Mailchimp writes.</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr"/>
@@ -2260,7 +2260,7 @@
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>PASS — eyebrow lanes/tags + ' + ' separator, date, read time, h1, deck | 2026-08-27 re-verified live: eyebrow lanes/date/read-time render on all 16. | 2026-09-01 re-verified live on VOL 17 at 375px: eyebrow renders 4 lane/tag chips + date + read-time, all inside the frame post-F97. | 2026-09-06 re-verified live: .article-eyebrow computes flex-wrap nowrap at 1280px and wrap at 375px, rail height 57px, zero overflow (F97 holds live). | 2026-09-11 re-verified live: article eyebrow renders lane chips + date + read time; .article-read '8 min' matches the plate.</t>
+          <t>PASS — eyebrow lanes/tags + ' + ' separator, date, read time, h1, deck | 2026-08-27 re-verified live: eyebrow lanes/date/read-time render on all 16. | 2026-09-01 re-verified live on VOL 17 at 375px: eyebrow renders 4 lane/tag chips + date + read-time, all inside the frame post-F97. | 2026-09-06 re-verified live: .article-eyebrow computes flex-wrap nowrap at 1280px and wrap at 375px, rail height 57px, zero overflow (F97 holds live). | 2026-09-11 re-verified live: article eyebrow renders lane chips + date + read time; .article-read '8 min' matches the plate. | 2026-09-28: live: eyebrow lane + tag chips, date, read time.</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr"/>
@@ -2313,7 +2313,7 @@
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>PASS — all 16 MDX bodies render through [...slug].astro | 2026-08-27 re-verified live: all 16 MDX bodies render. | 2026-09-19 re-verified live: all 17 live articles render an .article-body (shortest body ~6.4k chars of text).</t>
+          <t>PASS — all 16 MDX bodies render through [...slug].astro | 2026-08-27 re-verified live: all 16 MDX bodies render. | 2026-09-19 re-verified live: all 17 live articles render an .article-body (shortest body ~6.4k chars of text). | 2026-09-28: live: all 17 article pages 200 with body + BlogPosting wordCount.</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr"/>
@@ -2366,7 +2366,7 @@
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>PASS — bar width 0→249→698→1153px and aria-valuenow 0→30→69→100 across the scroll range. 2026-08-10 PM re-check: structural half re-verified (progress.js math recomputed by hand at 50% scroll = 51.5%; .article-body + .reading-progress present; role/aria-label/aria-valuemin/max initialized on load). Runtime paint not re-exercisable this run — the browser pane reports document.visibilityState 'hidden', so requestAnimationFrame never fires and the CSS width transition stays frozen at 0. Harness limitation, not a site regression. | 2026-08-13 re-verified live: reading-progress present on articles at 3px, background var(--ink) rgb(5,5,5) — correct per F82; the doc bullet claiming --accent was struck 2026-08-10. | 2026-08-27 NOT re-verified — rotation gap, not a failure. The reading-progress bar is scroll-driven and the browser pane would not scroll this run (window.scrollTo, scrollingElement.scrollTop, Page_Down x6 and the pointer scroll action all left scrollY at 0-2 on an 11,937px article; the pointer scroll action timed out with 'Browser pane is currently hidden'). Source unchanged since the last PASS, so the row keeps its prior result rather than being reset. | 2026-09-01 NOT TESTABLE this run — rotation gap, prior result retained. The browser pane went hidden: the pointer scroll timed out with 'Browser pane is currently hidden' and window.scrollTo / scrollingElement.scrollTop both left scrollY at 0 against a 10905px document. The .reading-progress element itself is present and correctly wired (role=progressbar, aria-valuenow=0, width 0% at scrollY 0). Neither PASS nor FAIL recorded, per the documented harness antipattern. | 2026-09-11 NOT TESTABLE — rotation gap, prior PASS retained. The browser pane was hidden for the whole run: window.scrollTo(0,2500) left scrollY at 0 and the pointer scroll action timed out with 'Browser pane is currently hidden'. Static wiring re-confirmed live (.reading-progress and .section-indicator both present on /words/the-stone/, section-indicator at opacity 0 at scroll top as specified). Neither PASSed nor FAILed on a tooling limit.</t>
+          <t>PASS — bar width 0→249→698→1153px and aria-valuenow 0→30→69→100 across the scroll range. 2026-08-10 PM re-check: structural half re-verified (progress.js math recomputed by hand at 50% scroll = 51.5%; .article-body + .reading-progress present; role/aria-label/aria-valuemin/max initialized on load). Runtime paint not re-exercisable this run — the browser pane reports document.visibilityState 'hidden', so requestAnimationFrame never fires and the CSS width transition stays frozen at 0. Harness limitation, not a site regression. | 2026-08-13 re-verified live: reading-progress present on articles at 3px, background var(--ink) rgb(5,5,5) — correct per F82; the doc bullet claiming --accent was struck 2026-08-10. | 2026-08-27 NOT re-verified — rotation gap, not a failure. The reading-progress bar is scroll-driven and the browser pane would not scroll this run (window.scrollTo, scrollingElement.scrollTop, Page_Down x6 and the pointer scroll action all left scrollY at 0-2 on an 11,937px article; the pointer scroll action timed out with 'Browser pane is currently hidden'). Source unchanged since the last PASS, so the row keeps its prior result rather than being reset. | 2026-09-01 NOT TESTABLE this run — rotation gap, prior result retained. The browser pane went hidden: the pointer scroll timed out with 'Browser pane is currently hidden' and window.scrollTo / scrollingElement.scrollTop both left scrollY at 0 against a 10905px document. The .reading-progress element itself is present and correctly wired (role=progressbar, aria-valuenow=0, width 0% at scrollY 0). Neither PASS nor FAIL recorded, per the documented harness antipattern. | 2026-09-11 NOT TESTABLE — rotation gap, prior PASS retained. The browser pane was hidden for the whole run: window.scrollTo(0,2500) left scrollY at 0 and the pointer scroll action timed out with 'Browser pane is currently hidden'. Static wiring re-confirmed live (.reading-progress and .section-indicator both present on /words/the-stone/, section-indicator at opacity 0 at scroll top as specified). Neither PASSed nor FAILed on a tooling limit. | 2026-09-28: ROTATION GAP — pane stuck at scrollY 0 while hidden (QA-OS antipattern); prior result kept, not re-tested.</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr"/>
@@ -2419,7 +2419,7 @@
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>PASS — pill text tracks sections ('What the Fear Was Actually About' → 'A New Thing' → 'The Thirtieth'), opacity animates in. 2026-08-10 PM re-check: section collection re-verified live (5 .section-head h2 landmarks found on /words/send-someone-else/; the 40%-viewport rule resolves to the correct current section). Opacity fade not observable this run — same hidden-tab rAF/transition suspension as F35. | 2026-08-27 NOT re-verified — rotation gap, not a failure. The section-indicator pill is scroll-driven and the browser pane would not scroll this run (window.scrollTo, scrollingElement.scrollTop, Page_Down x6 and the pointer scroll action all left scrollY at 0-2 on an 11,937px article; the pointer scroll action timed out with 'Browser pane is currently hidden'). Source unchanged since the last PASS, so the row keeps its prior result rather than being reset. | 2026-09-01 NOT TESTABLE this run — rotation gap, prior result retained. The browser pane went hidden: the pointer scroll timed out with 'Browser pane is currently hidden' and window.scrollTo / scrollingElement.scrollTop both left scrollY at 0 against a 10905px document. The .reading-progress element itself is present and correctly wired (role=progressbar, aria-valuenow=0, width 0% at scrollY 0). Neither PASS nor FAIL recorded, per the documented harness antipattern. | 2026-09-11 NOT TESTABLE — rotation gap, prior PASS retained. The browser pane was hidden for the whole run: window.scrollTo(0,2500) left scrollY at 0 and the pointer scroll action timed out with 'Browser pane is currently hidden'. Static wiring re-confirmed live (.reading-progress and .section-indicator both present on /words/the-stone/, section-indicator at opacity 0 at scroll top as specified). Neither PASSed nor FAILed on a tooling limit.</t>
+          <t>PASS — pill text tracks sections ('What the Fear Was Actually About' → 'A New Thing' → 'The Thirtieth'), opacity animates in. 2026-08-10 PM re-check: section collection re-verified live (5 .section-head h2 landmarks found on /words/send-someone-else/; the 40%-viewport rule resolves to the correct current section). Opacity fade not observable this run — same hidden-tab rAF/transition suspension as F35. | 2026-08-27 NOT re-verified — rotation gap, not a failure. The section-indicator pill is scroll-driven and the browser pane would not scroll this run (window.scrollTo, scrollingElement.scrollTop, Page_Down x6 and the pointer scroll action all left scrollY at 0-2 on an 11,937px article; the pointer scroll action timed out with 'Browser pane is currently hidden'). Source unchanged since the last PASS, so the row keeps its prior result rather than being reset. | 2026-09-01 NOT TESTABLE this run — rotation gap, prior result retained. The browser pane went hidden: the pointer scroll timed out with 'Browser pane is currently hidden' and window.scrollTo / scrollingElement.scrollTop both left scrollY at 0 against a 10905px document. The .reading-progress element itself is present and correctly wired (role=progressbar, aria-valuenow=0, width 0% at scrollY 0). Neither PASS nor FAIL recorded, per the documented harness antipattern. | 2026-09-11 NOT TESTABLE — rotation gap, prior PASS retained. The browser pane was hidden for the whole run: window.scrollTo(0,2500) left scrollY at 0 and the pointer scroll action timed out with 'Browser pane is currently hidden'. Static wiring re-confirmed live (.reading-progress and .section-indicator both present on /words/the-stone/, section-indicator at opacity 0 at scroll top as specified). Neither PASSed nor FAILed on a tooling limit. | 2026-09-28: ROTATION GAP — pane stuck at scrollY 0 while hidden; prior result kept, not re-tested.</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr"/>
@@ -2472,7 +2472,7 @@
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t>PASS — X intent carries encoded url + title | 2026-08-27 re-verified live: X intent carries encoded url + title (checked on /about/). | 2026-09-11 re-verified live: X intent href carries the encoded article URL and 'The Weight of My No — DX', target=_blank rel='noopener noreferrer'.</t>
+          <t>PASS — X intent carries encoded url + title | 2026-08-27 re-verified live: X intent carries encoded url + title (checked on /about/). | 2026-09-11 re-verified live: X intent href carries the encoded article URL and 'The Weight of My No — DX', target=_blank rel='noopener noreferrer'. | 2026-09-28: live: X intent carries encoded url + text, target=_blank rel=noopener noreferrer (article + about).</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr"/>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>PASS — copy button + [data-copy-status] live region on article and about | 2026-08-27 re-verified live: copy button + [data-copy-status] aria-live=polite region present on article and about. | 2026-09-11 re-verified live: copy-link button present on article and about with data-copy-link set to the absolute page URL; essay.js loaded; aria-live region present.</t>
+          <t>PASS — copy button + [data-copy-status] live region on article and about | 2026-08-27 re-verified live: copy button + [data-copy-status] aria-live=polite region present on article and about. | 2026-09-11 re-verified live: copy-link button present on article and about with data-copy-link set to the absolute page URL; essay.js loaded; aria-live region present. | 2026-09-28: live: button + [data-copy-status] present; failure path verified (label 'Copy failed' + SR status). Success path untestable in the pane: control navigator.clipboard.writeText() -&gt; 'Write permission denied' — harness, not site. Prior PASS kept.</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr"/>
@@ -2574,7 +2574,7 @@
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>PASS — Follow Me → instagram.com/ImJustDex | 2026-08-27 re-verified live: Follow Me → instagram.com/ImJustDex, 200. | 2026-09-19 re-verified live: Follow Me → instagram.com/ImJustDex with target=_blank rel='noopener noreferrer' on 17/17 articles and on /about/.</t>
+          <t>PASS — Follow Me → instagram.com/ImJustDex | 2026-08-27 re-verified live: Follow Me → instagram.com/ImJustDex, 200. | 2026-09-19 re-verified live: Follow Me → instagram.com/ImJustDex with target=_blank rel='noopener noreferrer' on 17/17 articles and on /about/. | 2026-09-28: live: Follow Me -&gt; instagram.com/ImJustDex, _blank noopener noreferrer (article + about).</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr"/>
@@ -2623,7 +2623,7 @@
       </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
-          <t>PASS — form posts /api/subscribe with source=article, honeypot off-canvas, aria-live label; server states verified directly against the function | 2026-09-18 re-verified live: server-rejected address on /words/gumbo/ surfaced 'That email didn’t look right. Try it again.' in the role=status aria-live label and kept the form — it reflects the server failure rather than a blanket success. source=article, honeypot off-canvas at x=-4972.</t>
+          <t>PASS — form posts /api/subscribe with source=article, honeypot off-canvas, aria-live label; server states verified directly against the function | 2026-09-18 re-verified live: server-rejected address on /words/gumbo/ surfaced 'That email didn’t look right. Try it again.' in the role=status aria-live label and kept the form — it reflects the server failure rather than a blanket success. source=article, honeypot off-canvas at x=-4972. | 2026-09-28: live: article form posts /api/subscribe, source=article, honeypot 'website' present; fixture build coming-soon form source=coming-soon.</t>
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr"/>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Authored prev/next render correctly on all 16. Ghost/teaser path PENDING — requires a future-dated entry; none exists. 2026-08-10 PM: the derive-from-live-status fix (p3) live-verified, then the underlying data cleaned — the 4 stale ghost:true flags are gone (see F81). Zero `ghost: true` remain in the collection; all 16 essays render real .article-nav-link anchors, 15 rel=next head links (newest correctly has none), zero article-nav-ghost teasers. | 2026-08-25 re-verified live: all 16 essays render real .article-nav-link anchors; zero `ghost: true` remain in the collection. Ghost/teaser path still PENDING — still requires a future-dated entry and none exists. | 2026-09-11: authored prev/next re-verified live — newest essay emits rel=prev only, /words/the-stone/ emits rel=prev + rel=next. Ghost/teaser path still PENDING; zero upcoming entries in the collection. | 2026-09-19: authored prev/next unchanged (no code churn since 507e988). Ghost/teaser path still PENDING — zero upcoming entries in the collection. | 2026-09-23: authored prev/next unchanged (no code or content commits since 09-19). Ghost path still PENDING — no future-dated entry. | 2026-09-25: still PENDING — 17/17 entries status published and past-dated, no upcoming entry to render. </t>
+          <t>PASS (live + fixture build) | Authored prev/next render correctly on all 16. Ghost/teaser path PENDING — requires a future-dated entry; none exists. 2026-08-10 PM: the derive-from-live-status fix (p3) live-verified, then the underlying data cleaned — the 4 stale ghost:true flags are gone (see F81). Zero `ghost: true` remain in the collection; all 16 essays render real .article-nav-link anchors, 15 rel=next head links (newest correctly has none), zero article-nav-ghost teasers. | 2026-08-25 re-verified live: all 16 essays render real .article-nav-link anchors; zero `ghost: true` remain in the collection. Ghost/teaser path still PENDING — still requires a future-dated entry and none exists. | 2026-09-11: authored prev/next re-verified live — newest essay emits rel=prev only, /words/the-stone/ emits rel=prev + rel=next. Ghost/teaser path still PENDING; zero upcoming entries in the collection. | 2026-09-19: authored prev/next unchanged (no code churn since 507e988). Ghost/teaser path still PENDING — zero upcoming entries in the collection. | 2026-09-23: authored prev/next unchanged (no code or content commits since 09-19). Ghost path still PENDING — no future-dated entry. | 2026-09-25: still PENDING — 17/17 entries status published and past-dated, no upcoming entry to render.  | 2026-09-28: PASS (live + build-verified via throwaway fixture). Live: authored prev/next correct; send-someone-else's stale frontmatter ghost:true is neutralised by nextLive, so live renders a real rel=next. Fixture (future-dated entry in a scratch copy, never committed): the-weight-of-my-no's next renders .article-nav-ghost with 'Jan 15, 2027' and NO rel=next.</t>
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr"/>
@@ -2687,7 +2687,7 @@
       </c>
       <c r="K44" s="6" t="inlineStr">
         <is>
-          <t>PENDING | 2026-09-18: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-26: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-27: still structurally untestable — 0 upcoming entries in the committed collection (17/17 published, past-dated).</t>
+          <t>PENDING | 2026-09-18: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-26: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-27: still structurally untestable — 0 upcoming entries in the committed collection (17/17 published, past-dated). | 2026-09-28: PASS (ghost path verified against a fixture build; authored path live).</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2729,7 @@
       </c>
       <c r="H45" s="6" t="inlineStr">
         <is>
-          <t>PASS — rel=prev emitted where prev authored; rel=next where next authored and live | 2026-08-25 re-verified live: rel=prev/next head links intact across the chain. | 2026-09-11 re-verified live: newest essay emits rel=prev only; /words/the-stone/ emits both rel=prev and rel=next. Correct.</t>
+          <t>PASS — rel=prev emitted where prev authored; rel=next where next authored and live | 2026-08-25 re-verified live: rel=prev/next head links intact across the chain. | 2026-09-11 re-verified live: newest essay emits rel=prev only; /words/the-stone/ emits both rel=prev and rel=next. Correct. | 2026-09-28: live: the-weight-of-my-no rel=prev only; show-me-your-glory rel=prev + rel=next; fixture: ghost next emits no rel=next.</t>
         </is>
       </c>
       <c r="I45" s="6" t="inlineStr"/>
@@ -2782,7 +2782,7 @@
       </c>
       <c r="H46" s="6" t="inlineStr">
         <is>
-          <t>PASS — '← Back' → '/' on article, coming-soon, about | 2026-09-11 re-verified live: '← Back' → '/' present on article and about.</t>
+          <t>PASS — '← Back' → '/' on article, coming-soon, about | 2026-09-11 re-verified live: '← Back' → '/' present on article and about. | 2026-09-28: live: '← Back' (.article-back) -&gt; '/' on article + about.</t>
         </is>
       </c>
       <c r="I46" s="6" t="inlineStr"/>
@@ -2831,7 +2831,7 @@
       </c>
       <c r="H47" s="6" t="inlineStr">
         <is>
-          <t>PASS — PullQuote, Scripture, Callout, DropCap, Closing, SectionHead, ResearchCTA, StudyNote all render and are styled via external hashed CSS (CSP-clean) | 2026-08-27 re-verified live: PullQuote/Scripture/Callout/StudyNote all render (the-stone: 2 pull-quotes, 4 scripture, 2 callouts, 3 study notes). | 2026-09-11 re-verified live: all MDX components still render; ResearchCTA now appears only on /words/show-me-your-glory/ (target thereturningglory.com 200) and is correctly gone from /words/the-nets/ after 507e988.</t>
+          <t>PASS — PullQuote, Scripture, Callout, DropCap, Closing, SectionHead, ResearchCTA, StudyNote all render and are styled via external hashed CSS (CSP-clean) | 2026-08-27 re-verified live: PullQuote/Scripture/Callout/StudyNote all render (the-stone: 2 pull-quotes, 4 scripture, 2 callouts, 3 study notes). | 2026-09-11 re-verified live: all MDX components still render; ResearchCTA now appears only on /words/show-me-your-glory/ (target thereturningglory.com 200) and is correctly gone from /words/the-nets/ after 507e988. | 2026-09-28: live: show-me-your-glory — .callout left border #c00, 3 StudyNotes, 0 contrast failures across 151 elements in both modes.</t>
         </is>
       </c>
       <c r="I47" s="6" t="inlineStr"/>
@@ -2884,7 +2884,7 @@
       </c>
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>PASS — &lt;details&gt; summary toggles open→closed→open on both sampled essays | 2026-08-27 re-verified live: &lt;details&gt; summary toggles closed→open→closed on the-stone. | 2026-09-11 re-verified live: 12 essays carry native &lt;details class=study-note&gt; with &lt;summary&gt;; 1–3 per essay.</t>
+          <t>PASS — &lt;details&gt; summary toggles open→closed→open on both sampled essays | 2026-08-27 re-verified live: &lt;details&gt; summary toggles closed→open→closed on the-stone. | 2026-09-11 re-verified live: 12 essays carry native &lt;details class=study-note&gt; with &lt;summary&gt;; 1–3 per essay. | 2026-09-28: live: &lt;details&gt; toggles closed -&gt; open -&gt; closed.</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr"/>
@@ -2937,7 +2937,7 @@
       </c>
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">PENDING — all 16 entries are status published with past dates, so isUpcomingData() is false everywhere and no coming-soon page renders | 2026-08-25: still PENDING for the same structural reason — all 16 built entries are status:published with past dates. NOTE: an untracked draft (src/content/words/before-i-had-the-words.mdx, status:"drafted", publishedDate 2026-08-07) sits in Dexter's working tree. It is correctly excluded from the build (19 pages, 16 articles) and does not exercise this path either, since its date is in the past, not the future. | 2026-09-01 still PENDING. The untracked draft in Dexter's working tree (src/content/words/before-i-had-the-words.mdx, status 'drafted', publishedDate 2026-08-07) is correctly excluded from the build (20 pages, 17 articles) but does NOT exercise this path — its date is in the past and its status is 'drafted', not an upcoming publish. Left untouched. | 2026-09-11: still PENDING for the same structural reason — 17 published entries, all past-dated. The untracked draft src/content/words/before-i-had-the-words.mdx is still status 'drafted' in Dexter's working tree, so it builds nothing and is correctly absent from sitemap and feed. | 2026-09-19: still PENDING for the same structural reason — no upcoming entry; the untracked draft is still 'drafted' and builds nothing. | 2026-09-23: still PENDING for the same structural reason — 17/17 entries published, isUpcomingData() false everywhere. | 2026-09-25: still PENDING — 17/17 entries status published and past-dated, no upcoming entry to render. </t>
+          <t>PASS (build-verified via fixture) | PENDING — all 16 entries are status published with past dates, so isUpcomingData() is false everywhere and no coming-soon page renders | 2026-08-25: still PENDING for the same structural reason — all 16 built entries are status:published with past dates. NOTE: an untracked draft (src/content/words/before-i-had-the-words.mdx, status:"drafted", publishedDate 2026-08-07) sits in Dexter's working tree. It is correctly excluded from the build (19 pages, 16 articles) and does not exercise this path either, since its date is in the past, not the future. | 2026-09-01 still PENDING. The untracked draft in Dexter's working tree (src/content/words/before-i-had-the-words.mdx, status 'drafted', publishedDate 2026-08-07) is correctly excluded from the build (20 pages, 17 articles) but does NOT exercise this path — its date is in the past and its status is 'drafted', not an upcoming publish. Left untouched. | 2026-09-11: still PENDING for the same structural reason — 17 published entries, all past-dated. The untracked draft src/content/words/before-i-had-the-words.mdx is still status 'drafted' in Dexter's working tree, so it builds nothing and is correctly absent from sitemap and feed. | 2026-09-19: still PENDING for the same structural reason — no upcoming entry; the untracked draft is still 'drafted' and builds nothing. | 2026-09-23: still PENDING for the same structural reason — 17/17 entries published, isUpcomingData() false everywhere. | 2026-09-25: still PENDING — 17/17 entries status published and past-dated, no upcoming entry to render.  | 2026-09-28: BUILD-VERIFIED via a throwaway future-dated fixture in a scratch copy (never committed): 'Coming Soon' tag, 'Friday, January 15, 2027', subscribe form source=coming-soon, noindex, og:image preserved (og-&lt;slug&gt;.png), 0 essay-body text leaked, excluded from sitemap/feed/cascade. Live half still awaits a real upcoming entry.</t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr"/>
@@ -2948,7 +2948,7 @@
       </c>
       <c r="K49" s="6" t="inlineStr">
         <is>
-          <t>PENDING | 2026-09-18: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-26: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-27: still structurally untestable — 0 upcoming entries in the committed collection (17/17 published, past-dated).</t>
+          <t>PENDING | 2026-09-18: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-26: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-27: still structurally untestable — 0 upcoming entries in the committed collection (17/17 published, past-dated). | 2026-09-28: PASS (verified against a fixture build).</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>PASS — about content + ProfilePage render | 2026-08-27 re-verified live: about content + ProfilePage render. | 2026-09-01 re-verified live: /about/ 200 in 0.75s, single h1, all four landmarks, 0 contrast failures across 24 measured elements. | 2026-09-19 re-verified live: /about/ 200 in 0.38s, deck 'Est. 1994.' present, single h1, ProfilePage JSON-LD complete, 0 contrast failures across 23 elements in both modes.</t>
+          <t>PASS — about content + ProfilePage render | 2026-08-27 re-verified live: about content + ProfilePage render. | 2026-09-01 re-verified live: /about/ 200 in 0.75s, single h1, all four landmarks, 0 contrast failures across 24 measured elements. | 2026-09-19 re-verified live: /about/ 200 in 0.38s, deck 'Est. 1994.' present, single h1, ProfilePage JSON-LD complete, 0 contrast failures across 23 elements in both modes. | 2026-09-28: live: 'Est. 1994' deck, PullQuote, Closing, ProfilePage.</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr"/>
@@ -3039,7 +3039,7 @@
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>PASS — share bar X + copy + Follow Me with live region | 2026-08-27 re-verified live: share bar X + copy + Follow Me + live region present on /about/. | 2026-09-19 re-verified live: /about/ share bar carries X intent, data-copy-link, Follow Me and an aria-live region.</t>
+          <t>PASS — share bar X + copy + Follow Me with live region | 2026-08-27 re-verified live: share bar X + copy + Follow Me + live region present on /about/. | 2026-09-19 re-verified live: /about/ share bar carries X intent, data-copy-link, Follow Me and an aria-live region. | 2026-09-28: live: X intent + Copy link (data-copy-link) + Follow Me on /about/.</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr"/>
@@ -3092,7 +3092,7 @@
       </c>
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>PASS — bespoke notfound-plate, 200 on /404, noindex+nofollow, /* fallback 404s unmatched routes | 2026-08-27 re-verified live: bespoke notfound-plate, 200 on /404, noindex+nofollow, single h1. | 2026-09-01 re-verified live: /404 returns HTTP 200 with the bespoke 'Nothing to Document Here' body, meta robots noindex,nofollow, single h1, all four landmarks, 0 contrast failures across 16 elements. | 2026-09-19 re-verified live: unmatched route returns HTTP 404 with the bespoke 'Nothing to Document Here' body, meta robots 'noindex, nofollow', Back to Home → /; 0 contrast failures in both modes.</t>
+          <t>PASS — bespoke notfound-plate, 200 on /404, noindex+nofollow, /* fallback 404s unmatched routes | 2026-08-27 re-verified live: bespoke notfound-plate, 200 on /404, noindex+nofollow, single h1. | 2026-09-01 re-verified live: /404 returns HTTP 200 with the bespoke 'Nothing to Document Here' body, meta robots noindex,nofollow, single h1, all four landmarks, 0 contrast failures across 16 elements. | 2026-09-19 re-verified live: unmatched route returns HTTP 404 with the bespoke 'Nothing to Document Here' body, meta robots 'noindex, nofollow', Back to Home → /; 0 contrast failures in both modes. | 2026-09-28: live: unmatched route -&gt; HTTP 404, notfound-plate, 'Back to Home' -&gt; /, noindex,nofollow, 0 contrast failures (dark).</t>
         </is>
       </c>
       <c r="I52" s="6" t="inlineStr"/>
@@ -3145,7 +3145,7 @@
       </c>
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>PASS — Atom 16 entries = 16 published; namespace + entries valid | 2026-08-13 re-verified live: /feed.xml 200, Atom namespace, 16 &lt;entry&gt; elements — exactly matching the 16 articles on the homepage, zero set difference either direction. | 2026-08-16 re-verified live: /feed.xml 200 with 16 &lt;entry&gt; elements; set-compared against the 16 article links on the live homepage — zero difference in either direction. | 2026-08-25 re-verified live: /feed.xml 200, 16 &lt;entry&gt; elements matching the 16 published articles exactly — no gaps, no extras. | 2026-08-27 re-verified live: Atom 16 entries == 16 published on the homepage. | 2026-09-01 re-verified live: /feed.xml 200, 17 entries — exactly matching the 17 articles on the homepage cascade. No feed-only or home-only slugs. | 2026-09-06 re-verified live: /feed.xml 200, 17 entries, slug set identical to the homepage cascade. | 2026-09-11 re-verified live: /feed.xml parses as Atom, 17 entries, matching the 17 published articles exactly.</t>
+          <t>PASS — Atom 16 entries = 16 published; namespace + entries valid | 2026-08-13 re-verified live: /feed.xml 200, Atom namespace, 16 &lt;entry&gt; elements — exactly matching the 16 articles on the homepage, zero set difference either direction. | 2026-08-16 re-verified live: /feed.xml 200 with 16 &lt;entry&gt; elements; set-compared against the 16 article links on the live homepage — zero difference in either direction. | 2026-08-25 re-verified live: /feed.xml 200, 16 &lt;entry&gt; elements matching the 16 published articles exactly — no gaps, no extras. | 2026-08-27 re-verified live: Atom 16 entries == 16 published on the homepage. | 2026-09-01 re-verified live: /feed.xml 200, 17 entries — exactly matching the 17 articles on the homepage cascade. No feed-only or home-only slugs. | 2026-09-06 re-verified live: /feed.xml 200, 17 entries, slug set identical to the homepage cascade. | 2026-09-11 re-verified live: /feed.xml parses as Atom, 17 entries, matching the 17 published articles exactly. | 2026-09-28: live: Atom 17 entries = 17 published, 27 lane categories, subtitle/rights/icon/logo/author present, application/xml, must-revalidate.</t>
         </is>
       </c>
       <c r="I53" s="6" t="inlineStr"/>
@@ -3198,7 +3198,7 @@
       </c>
       <c r="H54" s="6" t="inlineStr">
         <is>
-          <t>PASS — feed.xsl 200 and &lt;?xml-stylesheet?&gt; PI present | 2026-08-13 re-verified live: /feed.xsl 200 and referenced via &lt;?xml-stylesheet?&gt; in the feed prolog. | 2026-08-25 re-verified live: /feed.xsl 200 and feed.xml carries &lt;?xml-stylesheet href="/feed.xsl"?&gt;. | 2026-08-27 re-verified live: feed.xsl 200 and the &lt;?xml-stylesheet?&gt; PI is present. | 2026-09-01 re-verified live: /feed.xml carries the &lt;?xml-stylesheet?&gt; reference and /feed.xsl returns 200. | 2026-09-06 re-verified live: feed.xsl 200 (4342b) and the feed still declares &lt;?xml-stylesheet href="/feed.xsl"?&gt;. | 2026-09-11 re-verified live: feed carries &lt;?xml-stylesheet type='text/xsl' href='/feed.xsl'?&gt; and /feed.xsl returns 200 and parses.</t>
+          <t>PASS — feed.xsl 200 and &lt;?xml-stylesheet?&gt; PI present | 2026-08-13 re-verified live: /feed.xsl 200 and referenced via &lt;?xml-stylesheet?&gt; in the feed prolog. | 2026-08-25 re-verified live: /feed.xsl 200 and feed.xml carries &lt;?xml-stylesheet href="/feed.xsl"?&gt;. | 2026-08-27 re-verified live: feed.xsl 200 and the &lt;?xml-stylesheet?&gt; PI is present. | 2026-09-01 re-verified live: /feed.xml carries the &lt;?xml-stylesheet?&gt; reference and /feed.xsl returns 200. | 2026-09-06 re-verified live: feed.xsl 200 (4342b) and the feed still declares &lt;?xml-stylesheet href="/feed.xsl"?&gt;. | 2026-09-11 re-verified live: feed carries &lt;?xml-stylesheet type='text/xsl' href='/feed.xsl'?&gt; and /feed.xsl returns 200 and parses. | 2026-09-28: live: feed.xsl 200 application/xml; xml-stylesheet PI present; style-src unsafe-inline on /feed.xml + /feed.xsl.</t>
         </is>
       </c>
       <c r="I54" s="6" t="inlineStr"/>
@@ -3251,7 +3251,7 @@
       </c>
       <c r="H55" s="6" t="inlineStr">
         <is>
-          <t>PASS — 5 anchor links, all resolve to real targets | 2026-08-27 re-verified live: 5 anchor links on /phase0/, all resolve to real targets. | 2026-09-01 re-verified live: /phase0/ 200 in 0.41s, single h1, no skipped heading levels across a 22-heading tree, 0 contrast failures across 106 measured elements. | 2026-09-19 re-verified live: /phase0/ 200 in 0.39s, single h1, 0 contrast failures across 105 elements in both modes, no horizontal overflow at 375px.</t>
+          <t>PASS — 5 anchor links, all resolve to real targets | 2026-08-27 re-verified live: 5 anchor links on /phase0/, all resolve to real targets. | 2026-09-01 re-verified live: /phase0/ 200 in 0.41s, single h1, no skipped heading levels across a 22-heading tree, 0 contrast failures across 106 measured elements. | 2026-09-19 re-verified live: /phase0/ 200 in 0.39s, single h1, 0 contrast failures across 105 elements in both modes, no horizontal overflow at 375px. | 2026-09-28: live: anchors #phase0/#get/#definition all resolve; single h1; tokens + shell + phase0 css.</t>
         </is>
       </c>
       <c r="I55" s="6" t="inlineStr"/>
@@ -3304,18 +3304,22 @@
       </c>
       <c r="H56" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: /phase0/ form action is /api/subscribe with no legacy Mailchimp query string; matches the other three subscribe surfaces. | 2026-08-27 re-verified live: /phase0/ form action=/api/subscribe, honeypot present, source=phase0. | 2026-09-19 re-verified live: /phase0/ .phase0-capture posts to /api/subscribe with empty honeypot (name=website), source=phase0, noscript fallback and phase0.js present.</t>
-        </is>
-      </c>
-      <c r="I56" s="6" t="inlineStr"/>
+          <t>PASS — live-verified 2026-08-10: /phase0/ form action is /api/subscribe with no legacy Mailchimp query string; matches the other three subscribe surfaces. | 2026-08-27 re-verified live: /phase0/ form action=/api/subscribe, honeypot present, source=phase0. | 2026-09-19 re-verified live: /phase0/ .phase0-capture posts to /api/subscribe with empty honeypot (name=website), source=phase0, noscript fallback and phase0.js present. | 2026-09-28 ISSUE/Medium — the first time the validation branch was exercised (every prior check read the form's action/honeypot/source only): a mistyped email shows 'Something broke on our end. Try again, or email dex@imjustdex.com.' through the role=alert, assertive error region. Cause: js/phase0.js calls setError() with no copy on client-side validation failure, and the error &lt;p&gt; ships holding the server-failure line. A 400 invalid_email or 429 rate_limited from the function also rendered the outage line. The user story's 'not lie on failure' is broken for every reader with a typo. Measured live on /phase0/ (aria-invalid=true, 0 POSTs, visible .form-msg = outage copy), then reproduced 4/8 scenario failures by running the pre-fix file in a stub-DOM harness.</t>
+        </is>
+      </c>
+      <c r="I56" s="6" t="inlineStr">
+        <is>
+          <t>Medium (fixed)</t>
+        </is>
+      </c>
       <c r="J56" s="4" t="inlineStr">
         <is>
-          <t>FIX (qa/fixes-20260807 69d63f3): action reduced to /api/subscribe, matching the other three surfaces</t>
+          <t>FIX (qa/fixes-20260807 69d63f3): action reduced to /api/subscribe, matching the other three surfaces | FIX (qa/fixes-20260928, c524932): js/phase0.js passes copy on every error path — client invalid and server invalid_email -&gt; 'That email didn’t look right. Try it again.', 429 -&gt; 'Too many attempts. Give it a minute.' (both reused verbatim from subscribe.js / signup.js, no new copy), everything else -&gt; the existing outage line + 'Retry'; a rejected address restores the original button label. phase0/index.html cache-bust phase0.js phase2 -&gt; phase3.</t>
         </is>
       </c>
       <c r="K56" s="6" t="inlineStr">
         <is>
-          <t>PASS (verified against build) — state machine idle, source=phase0, honeypot intact, 0 console errors</t>
+          <t>PASS (verified against build) — state machine idle, source=phase0, honeypot intact, 0 console errors | 2026-09-28: PASS (verified against build) — npm run build clean (20 pages); dist/phase0/index.html references phase0.js?v=phase3 and dist/js/phase0.js == source. Stub-DOM harness running the BUILT file: 8/8 scenarios pass (typo, empty, server invalid_email, 429, 502, non-JSON 500, network failure, 200 success; valid keystroke clears the error). Control: the same harness on the pre-fix file fails 4/8, matching the live observation. Dev servers cannot start in unattended runs and the live CSP blocks script injection, so no in-browser retest; live-verifies on the first SCRUB after merge.</t>
         </is>
       </c>
     </row>
@@ -3357,7 +3361,7 @@
       </c>
       <c r="H57" s="6" t="inlineStr">
         <is>
-          <t>PASS — footer year 2026 = current year | 2026-08-27 re-verified live: phase0 footer year 2026. | 2026-09-19 re-verified live: #yr reads 2026 = current year on /phase0/.</t>
+          <t>PASS — footer year 2026 = current year | 2026-08-27 re-verified live: phase0 footer year 2026. | 2026-09-19 re-verified live: #yr reads 2026 = current year on /phase0/. | 2026-09-28: live: #yr = 2026.</t>
         </is>
       </c>
       <c r="I57" s="6" t="inlineStr"/>
@@ -3410,7 +3414,7 @@
       </c>
       <c r="H58" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: /brand/ serves plates.css?v=phase15, matching every other surface; no second year-long cache entry. | 2026-09-01 re-verified live: /brand/ 200, single h1, no skipped heading levels, 0 contrast failures across 800 measured elements in dark mode. | 2026-09-22 re-verified live: /brand/ 200 in 0.48s; CSP style-src 'self' 'unsafe-inline' (scoped override intact); 0 inline &lt;script&gt; (mode.js + JSON-LD + Netlify RUM only); present in sitemap-0.xml; 680 text elements swept in dark mode, 0 contrast failures; image-plate specimens keep display:flex + justify-content:flex-end (no F100 regression).</t>
+          <t>PASS — live-verified 2026-08-10: /brand/ serves plates.css?v=phase15, matching every other surface; no second year-long cache entry. | 2026-09-01 re-verified live: /brand/ 200, single h1, no skipped heading levels, 0 contrast failures across 800 measured elements in dark mode. | 2026-09-22 re-verified live: /brand/ 200 in 0.48s; CSP style-src 'self' 'unsafe-inline' (scoped override intact); 0 inline &lt;script&gt; (mode.js + JSON-LD + Netlify RUM only); present in sitemap-0.xml; 680 text elements swept in dark mode, 0 contrast failures; image-plate specimens keep display:flex + justify-content:flex-end (no F100 regression). | 2026-09-28: live: /brand/ 200, scoped CSP style-src unsafe-inline, 0 inline scripts, in sitemap; 776 elements 0 contrast failures in both modes; image-plate specimens flex/flex-end, titles at 0.61-0.81 of plate height. Catalog note: expected cites brand.js, retired with the v2 build (ed10576) — the page ships no scripts; not a defect.</t>
         </is>
       </c>
       <c r="I58" s="6" t="inlineStr"/>
@@ -3463,7 +3467,7 @@
       </c>
       <c r="H59" s="6" t="inlineStr">
         <is>
-          <t>PASS — GET /api/subscribe → 405 method_not_allowed | 2026-08-25 re-verified live: /api/subscribe reachable and behaving; rewrite chain intact. | 2026-08-27 re-verified live: GET /api/subscribe → 405 method_not_allowed. | 2026-09-06 re-verified live: GET /api/subscribe -&gt; 405. | 2026-09-11 re-verified live: GET /api/subscribe → 405 {'ok':false,'error':'method_not_allowed'}. | 2026-09-22 re-verified live: GET /api/subscribe -&gt; 405 {'ok':false,'error':'method_not_allowed'}; PUT -&gt; 405 likewise.</t>
+          <t>PASS — GET /api/subscribe → 405 method_not_allowed | 2026-08-25 re-verified live: /api/subscribe reachable and behaving; rewrite chain intact. | 2026-08-27 re-verified live: GET /api/subscribe → 405 method_not_allowed. | 2026-09-06 re-verified live: GET /api/subscribe -&gt; 405. | 2026-09-11 re-verified live: GET /api/subscribe → 405 {'ok':false,'error':'method_not_allowed'}. | 2026-09-22 re-verified live: GET /api/subscribe -&gt; 405 {'ok':false,'error':'method_not_allowed'}; PUT -&gt; 405 likewise. | 2026-09-28: live: GET and PUT -&gt; 405 method_not_allowed.</t>
         </is>
       </c>
       <c r="I59" s="6" t="inlineStr"/>
@@ -3516,7 +3520,7 @@
       </c>
       <c r="H60" s="6" t="inlineStr">
         <is>
-          <t>PASS — rate-limit bucket present (5/60s per IP) | 2026-09-11 re-verified live: burst of 8 POSTs from one IP: 400 invalid_email ×2 then 429 rate_limited ×6 — the 5/60s window fires as specified. | 2026-09-22 re-verified live: sequential burst of 10 POSTs (email=notanemail) from a quiet start returned exactly 5 x 400 invalid_email then 5 x 429 rate_limited — the 5/60s window fires as specified. A PARALLEL burst of 10 returned 10 x 400 and no 429: the window is a module-scope Map, so it is per Lambda instance and parallel requests fan out. Recorded as a measurement antipattern in QA-OS.md [F107]; not a defect.</t>
+          <t>PASS — rate-limit bucket present (5/60s per IP) | 2026-09-11 re-verified live: burst of 8 POSTs from one IP: 400 invalid_email ×2 then 429 rate_limited ×6 — the 5/60s window fires as specified. | 2026-09-22 re-verified live: sequential burst of 10 POSTs (email=notanemail) from a quiet start returned exactly 5 x 400 invalid_email then 5 x 429 rate_limited — the 5/60s window fires as specified. A PARALLEL burst of 10 returned 10 x 400 and no 429: the window is a module-scope Map, so it is per Lambda instance and parallel requests fan out. Recorded as a measurement antipattern in QA-OS.md [F107]; not a defect. | 2026-09-28: live: SEQUENTIAL burst of 10 (email=notanemail) from a quiet start -&gt; exactly 5 x 400 then 5 x 429.</t>
         </is>
       </c>
       <c r="I60" s="6" t="inlineStr"/>
@@ -3569,7 +3573,7 @@
       </c>
       <c r="H61" s="6" t="inlineStr">
         <is>
-          <t>PASS — filled honeypot → 200 silent success, no Mailchimp write; field off-canvas (left:-5000px, tabindex -1, aria-hidden) | 2026-08-25 re-verified live: honeypot re-verified live: POST with website=spam returned HTTP 200 {"ok":true,"message":"subscribed"} — the intended silent drop, indistinguishable from success to a bot. | 2026-08-27 re-verified live: filled honeypot → 200 silent success. | 2026-09-06 re-verified live: filled honeypot (website=spam) -&gt; 200 {ok:true,message:'subscribed'} with no Mailchimp write (subscribe.cjs:67-69 short-circuits before the email is read). | 2026-09-11 re-verified live: POST with website=spam → 200 {'ok':true,'message':'subscribed'} and no Mailchimp call. Confirmed against subscribe.cjs:65-67 that this is the intended silent fake-success, NOT a bypass — the handler returns before the Mailchimp branch. | 2026-09-22 re-verified live: POST with website=http://spam.example -&gt; 200 {'ok':true,'message':'subscribed'}, the intended silent drop, no Mailchimp write.</t>
+          <t>PASS — filled honeypot → 200 silent success, no Mailchimp write; field off-canvas (left:-5000px, tabindex -1, aria-hidden) | 2026-08-25 re-verified live: honeypot re-verified live: POST with website=spam returned HTTP 200 {"ok":true,"message":"subscribed"} — the intended silent drop, indistinguishable from success to a bot. | 2026-08-27 re-verified live: filled honeypot → 200 silent success. | 2026-09-06 re-verified live: filled honeypot (website=spam) -&gt; 200 {ok:true,message:'subscribed'} with no Mailchimp write (subscribe.cjs:67-69 short-circuits before the email is read). | 2026-09-11 re-verified live: POST with website=spam → 200 {'ok':true,'message':'subscribed'} and no Mailchimp call. Confirmed against subscribe.cjs:65-67 that this is the intended silent fake-success, NOT a bypass — the handler returns before the Mailchimp branch. | 2026-09-22 re-verified live: POST with website=http://spam.example -&gt; 200 {'ok':true,'message':'subscribed'}, the intended silent drop, no Mailchimp write. | 2026-09-28: live: filled honeypot -&gt; 200 {ok:true,message:subscribed}, silent.</t>
         </is>
       </c>
       <c r="I61" s="6" t="inlineStr"/>
@@ -3622,7 +3626,7 @@
       </c>
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>PASS — invalid address → 400 invalid_email; plus-addressed valid address accepted (clients encode + as %2B via URLSearchParams(FormData)) | 2026-08-25 re-verified live: email validation re-verified live: POST email=notanemail returned HTTP 400 {"ok":false,"error":"invalid_email"}. | 2026-08-27 re-verified live: invalid address → 400 invalid_email. | 2026-09-06 re-verified live: email=notanemail -&gt; 400 {ok:false,error:'invalid_email'}. | 2026-09-11 re-verified live: POST email=notanemail → 400 {'ok':false,'error':'invalid_email'}. | 2026-09-22 re-verified live: email=not-an-email -&gt; 400 {'ok':false,'error':'invalid_email'}; %2B-encoded plus address accepted on the same run.</t>
+          <t>PASS — invalid address → 400 invalid_email; plus-addressed valid address accepted (clients encode + as %2B via URLSearchParams(FormData)) | 2026-08-25 re-verified live: email validation re-verified live: POST email=notanemail returned HTTP 400 {"ok":false,"error":"invalid_email"}. | 2026-08-27 re-verified live: invalid address → 400 invalid_email. | 2026-09-06 re-verified live: email=notanemail -&gt; 400 {ok:false,error:'invalid_email'}. | 2026-09-11 re-verified live: POST email=notanemail → 400 {'ok':false,'error':'invalid_email'}. | 2026-09-22 re-verified live: email=not-an-email -&gt; 400 {'ok':false,'error':'invalid_email'}; %2B-encoded plus address accepted on the same run. | 2026-09-28: live: notanemail -&gt; 400 invalid_email, Cache-Control no-store.</t>
         </is>
       </c>
       <c r="I62" s="6" t="inlineStr"/>
@@ -3675,7 +3679,7 @@
       </c>
       <c r="H63" s="6" t="inlineStr">
         <is>
-          <t>PASS — healthscrub+20260807@imjustdex.com → 200 subscribed in 1.53s | 2026-08-13 re-verified live: live smoke test POST /api/subscribe returned HTTP 200 {"ok":true,"message":"subscribed"} in 2.16s using healthscrub+20260813@imjustdex.com. | 2026-08-16 re-verified live: live smoke test POST /api/subscribe returned HTTP 200 {"ok":true,"message":"subscribed"} in 2.05s using healthscrub+20260816@imjustdex.com. | 2026-08-25 re-verified live: smoke POST with healthscrub+20260825@imjustdex.com returned HTTP 200 {"ok":true,"message":"subscribed"} in 2.20s. | 2026-08-27 re-verified live: healthscrub+20260827@imjustdex.com → 200 subscribed. | 2026-09-06 re-verified live: POST healthscrub%2B20260906%40imjustdex.com -&gt; 200 {ok:true,message:'subscribed'} in 1.77s. | 2026-09-11 re-verified live: first POST of healthscrub+20260911@imjustdex.com → 200 'subscribed'; immediate repeat → 200 'already_subscribed'. Member-exists path intact. | 2026-09-22 re-verified live: BOTH branches exercised — first POST of healthscrub+20260922@imjustdex.com -&gt; 200 {'message':'subscribed'} in 1.81s; immediate re-POST of the same address -&gt; 200 {'message':'already_subscribed'}.</t>
+          <t>PASS — healthscrub+20260807@imjustdex.com → 200 subscribed in 1.53s | 2026-08-13 re-verified live: live smoke test POST /api/subscribe returned HTTP 200 {"ok":true,"message":"subscribed"} in 2.16s using healthscrub+20260813@imjustdex.com. | 2026-08-16 re-verified live: live smoke test POST /api/subscribe returned HTTP 200 {"ok":true,"message":"subscribed"} in 2.05s using healthscrub+20260816@imjustdex.com. | 2026-08-25 re-verified live: smoke POST with healthscrub+20260825@imjustdex.com returned HTTP 200 {"ok":true,"message":"subscribed"} in 2.20s. | 2026-08-27 re-verified live: healthscrub+20260827@imjustdex.com → 200 subscribed. | 2026-09-06 re-verified live: POST healthscrub%2B20260906%40imjustdex.com -&gt; 200 {ok:true,message:'subscribed'} in 1.77s. | 2026-09-11 re-verified live: first POST of healthscrub+20260911@imjustdex.com → 200 'subscribed'; immediate repeat → 200 'already_subscribed'. Member-exists path intact. | 2026-09-22 re-verified live: BOTH branches exercised — first POST of healthscrub+20260922@imjustdex.com -&gt; 200 {'message':'subscribed'} in 1.81s; immediate re-POST of the same address -&gt; 200 {'message':'already_subscribed'}. | 2026-09-28: live: healthscrub+20260928@imjustdex.com -&gt; 200 subscribed (1.32s); repeat -&gt; 200 already_subscribed.</t>
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr"/>
@@ -3728,7 +3732,7 @@
       </c>
       <c r="H64" s="6" t="inlineStr">
         <is>
-          <t>PASS — source field present on all 4 surfaces (home/article/coming-soon/phase0) | 2026-09-06 re-verified live: source=healthscrub accepted on the 200 above. | 2026-09-19 re-verified live: subscribe smoke (healthscrub+20260919@imjustdex.com, source=healthscrub, %2B-encoded) → 200 {"ok":true,"message":"subscribed"} in 1.77s. | 2026-09-22 re-verified live: source=healthscrub accepted on the 200 above; merge-field/tag write is best-effort server-side and not observable without the Mailchimp dashboard (outside repo).</t>
+          <t>PASS — source field present on all 4 surfaces (home/article/coming-soon/phase0) | 2026-09-06 re-verified live: source=healthscrub accepted on the 200 above. | 2026-09-19 re-verified live: subscribe smoke (healthscrub+20260919@imjustdex.com, source=healthscrub, %2B-encoded) → 200 {"ok":true,"message":"subscribed"} in 1.77s. | 2026-09-22 re-verified live: source=healthscrub accepted on the 200 above; merge-field/tag write is best-effort server-side and not observable without the Mailchimp dashboard (outside repo). | 2026-09-28: live: source field on home (home), article (article), phase0 (phase0); fixture coming-soon (coming-soon).</t>
         </is>
       </c>
       <c r="I64" s="6" t="inlineStr"/>
@@ -3781,7 +3785,7 @@
       </c>
       <c r="H65" s="6" t="inlineStr">
         <is>
-          <t>PASS — documented error envelope returned, no stack leakage | 2026-09-18 re-verified live: POST email=not-an-email returns 400 {"ok":false,"error":"invalid_email"} with Cache-Control: no-store, no stack leakage. Config/upstream branches not forceable from outside (would need env or Mailchimp changes); subscribe.cjs unchanged since last PASS. | 2026-09-22 re-verified live: 400 invalid_email returns Cache-Control: no-store with no stack leakage. Config/upstream branches still not forceable from outside (needs env or Mailchimp changes); subscribe.cjs unchanged since last PASS.</t>
+          <t>PASS — documented error envelope returned, no stack leakage | 2026-09-18 re-verified live: POST email=not-an-email returns 400 {"ok":false,"error":"invalid_email"} with Cache-Control: no-store, no stack leakage. Config/upstream branches not forceable from outside (would need env or Mailchimp changes); subscribe.cjs unchanged since last PASS. | 2026-09-22 re-verified live: 400 invalid_email returns Cache-Control: no-store with no stack leakage. Config/upstream branches still not forceable from outside (needs env or Mailchimp changes); subscribe.cjs unchanged since last PASS. | 2026-09-28: carried: JSON no-store envelope confirmed on 400/405/429; config/upstream failures not inducible live.</t>
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr"/>
@@ -3887,7 +3891,7 @@
       </c>
       <c r="H67" s="6" t="inlineStr">
         <is>
-          <t>PASS — /about, /phase0 and all 16 /words/&lt;slug&gt; → single 301 to trailing-slash canonical | 2026-08-13 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200; /sitemap.xml correctly 404 post-cutover. | 2026-08-16 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200 and /words/the-stone -&gt; 301 -&gt; /words/the-stone/ re-verified live; /sitemap.xml correctly 404 post-cutover; /words -&gt; 301 home; /opsmeeting -&gt; 301 home. | 2026-08-25 re-verified live: /about, /brand, /phase0 and /words/the-stone each return a single 301 to the trailing-slash form, which returns 200. No loops. | 2026-08-27 re-verified live: /about and /words/the-stone → single 301 to the trailing-slash canonical. | 2026-09-01 re-verified live: /about -&gt; 301 -&gt; https://imjustdex.com/about/ -&gt; 200. | 2026-09-06 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200. | 2026-09-11 re-verified live: /about, /brand, /phase0 and /words/the-stone all 301 → their trailing-slash canonical → 200. | 2026-09-22 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200 and /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200; /sitemap.xml correctly 404 post-cutover; /DESIGN-SYSTEM.md correctly 404.</t>
+          <t>PASS — /about, /phase0 and all 16 /words/&lt;slug&gt; → single 301 to trailing-slash canonical | 2026-08-13 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200; /sitemap.xml correctly 404 post-cutover. | 2026-08-16 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200 and /words/the-stone -&gt; 301 -&gt; /words/the-stone/ re-verified live; /sitemap.xml correctly 404 post-cutover; /words -&gt; 301 home; /opsmeeting -&gt; 301 home. | 2026-08-25 re-verified live: /about, /brand, /phase0 and /words/the-stone each return a single 301 to the trailing-slash form, which returns 200. No loops. | 2026-08-27 re-verified live: /about and /words/the-stone → single 301 to the trailing-slash canonical. | 2026-09-01 re-verified live: /about -&gt; 301 -&gt; https://imjustdex.com/about/ -&gt; 200. | 2026-09-06 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200. | 2026-09-11 re-verified live: /about, /brand, /phase0 and /words/the-stone all 301 → their trailing-slash canonical → 200. | 2026-09-22 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200 and /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200; /sitemap.xml correctly 404 post-cutover; /DESIGN-SYSTEM.md correctly 404. | 2026-09-28: live: 21/21 non-slash routes 301 to their slash canonical (about, phase0, /words, /words/, 17 essays).</t>
         </is>
       </c>
       <c r="I67" s="6" t="inlineStr"/>
@@ -3940,7 +3944,7 @@
       </c>
       <c r="H68" s="6" t="inlineStr">
         <is>
-          <t>PASS — /words and /words/ → 301 home | 2026-08-27 re-verified live: /words → 301 home. | 2026-09-11 re-verified live: /words and /words/ both 301 → https://imjustdex.com/. | 2026-09-23 re-verified live: /words and /words/ both single 301 -&gt; /.</t>
+          <t>PASS — /words and /words/ → 301 home | 2026-08-27 re-verified live: /words → 301 home. | 2026-09-11 re-verified live: /words and /words/ both 301 → https://imjustdex.com/. | 2026-09-23 re-verified live: /words and /words/ both single 301 -&gt; /. | 2026-09-28: live: /words and /words/ -&gt; 301 /.</t>
         </is>
       </c>
       <c r="I68" s="6" t="inlineStr"/>
@@ -3993,7 +3997,7 @@
       </c>
       <c r="H69" s="6" t="inlineStr">
         <is>
-          <t>PASS — /opsmeeting, /leadership-prep, /asana-workflow (+ /*) all → 301 home | 2026-08-27 re-verified live: /opsmeeting → 301 home. | 2026-09-11 re-verified live: /opsmeeting, /leadership-prep, /asana-workflow and a deep path under each all 301 → https://imjustdex.com/. | 2026-09-23 re-verified live: /opsmeeting, /leadership-prep, /asana-workflow and /opsmeeting/deep/x all single 301 -&gt; /.</t>
+          <t>PASS — /opsmeeting, /leadership-prep, /asana-workflow (+ /*) all → 301 home | 2026-08-27 re-verified live: /opsmeeting → 301 home. | 2026-09-11 re-verified live: /opsmeeting, /leadership-prep, /asana-workflow and a deep path under each all 301 → https://imjustdex.com/. | 2026-09-23 re-verified live: /opsmeeting, /leadership-prep, /asana-workflow and /opsmeeting/deep/x all single 301 -&gt; /. | 2026-09-28: live: /opsmeeting, /opsmeeting/x, /leadership-prep/y, /asana-workflow, /asana-workflow/z -&gt; 301 /.</t>
         </is>
       </c>
       <c r="I69" s="6" t="inlineStr"/>
@@ -4046,7 +4050,7 @@
       </c>
       <c r="H70" s="6" t="inlineStr">
         <is>
-          <t>PASS — /api/subscribe rewrite reaches the function (405 on GET, 400/200 on POST) | 2026-08-13 re-verified live: /api/subscribe rewrite reached the Netlify function and returned a Mailchimp success body. | 2026-08-25 re-verified live: /api/subscribe rewrite to the Netlify function verified by the live smoke POST. | 2026-08-27 re-verified live: /api/subscribe rewrite reaches the function. | 2026-09-01 re-verified live: POST to /api/subscribe rewrote to the Netlify function and returned 200. | 2026-09-11 re-verified live: /api/subscribe rewrite live — POST reaches the function and returns its JSON envelope. | 2026-09-23 re-verified live: /api/subscribe rewrite reaches the function — GET 405, POST (healthscrub+20260923@imjustdex.com, %2B-encoded) 200 {"ok":true,"message":"subscribed"} in 2.05s.</t>
+          <t>PASS — /api/subscribe rewrite reaches the function (405 on GET, 400/200 on POST) | 2026-08-13 re-verified live: /api/subscribe rewrite reached the Netlify function and returned a Mailchimp success body. | 2026-08-25 re-verified live: /api/subscribe rewrite to the Netlify function verified by the live smoke POST. | 2026-08-27 re-verified live: /api/subscribe rewrite reaches the function. | 2026-09-01 re-verified live: POST to /api/subscribe rewrote to the Netlify function and returned 200. | 2026-09-11 re-verified live: /api/subscribe rewrite live — POST reaches the function and returns its JSON envelope. | 2026-09-23 re-verified live: /api/subscribe rewrite reaches the function — GET 405, POST (healthscrub+20260923@imjustdex.com, %2B-encoded) 200 {"ok":true,"message":"subscribed"} in 2.05s. | 2026-09-28: live: POST /api/subscribe reaches the function (200/400/429 bodies).</t>
         </is>
       </c>
       <c r="I70" s="6" t="inlineStr"/>
@@ -4099,7 +4103,7 @@
       </c>
       <c r="H71" s="6" t="inlineStr">
         <is>
-          <t>PASS — unmatched route → 404 with the branded body | 2026-08-13 re-verified live: /404 returns 200 with the bespoke 'Nothing to Document Here' body and noindex; /DESIGN-SYSTEM.md and /audit/features.json both 404 (docs not leaking). | 2026-08-25 re-verified live: /404 returns HTTP 200 with the bespoke notfound-plate body and meta robots noindex. | 2026-08-27 re-verified live: unmatched route → 404 with the branded body. | 2026-09-06 re-verified live: /nonexistent-page-qa-test -&gt; 404; /sitemap.xml and /DESIGN-SYSTEM.md both correctly 404. | 2026-09-11 re-verified live: /DESIGN-SYSTEM.md → 404 and /sitemap.xml → 404; /404 serves the bespoke body at HTTP 200 with noindex,nofollow. | 2026-09-23 re-verified live: /no-such-page-qa -&gt; 404 with the 'Nothing to Document Here' body; /DESIGN-SYSTEM.md, /audit/features.json and /sitemap.xml all 404.</t>
+          <t>PASS — unmatched route → 404 with the branded body | 2026-08-13 re-verified live: /404 returns 200 with the bespoke 'Nothing to Document Here' body and noindex; /DESIGN-SYSTEM.md and /audit/features.json both 404 (docs not leaking). | 2026-08-25 re-verified live: /404 returns HTTP 200 with the bespoke notfound-plate body and meta robots noindex. | 2026-08-27 re-verified live: unmatched route → 404 with the branded body. | 2026-09-06 re-verified live: /nonexistent-page-qa-test -&gt; 404; /sitemap.xml and /DESIGN-SYSTEM.md both correctly 404. | 2026-09-11 re-verified live: /DESIGN-SYSTEM.md → 404 and /sitemap.xml → 404; /404 serves the bespoke body at HTTP 200 with noindex,nofollow. | 2026-09-23 re-verified live: /no-such-page-qa -&gt; 404 with the 'Nothing to Document Here' body; /DESIGN-SYSTEM.md, /audit/features.json and /sitemap.xml all 404. | 2026-09-28: live: /this-route-does-not-exist-qa -&gt; 404 bespoke body.</t>
         </is>
       </c>
       <c r="I71" s="6" t="inlineStr"/>
@@ -4152,7 +4156,7 @@
       </c>
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>PASS — CSP present and strict on every page; per-route /brand/ + /feed.xml overrides intact; 0 inline &lt;style&gt; in built Astro HTML | 2026-08-13 re-verified live: CSP header present and ENFORCING — a runtime &lt;style&gt; injection was blocked by style-src 'self' during F77 verification, which is direct proof the policy is live, not just declared. Per-route /brand/ and /feed.xml relaxations by design. | 2026-08-16 re-verified live: CSP present and strict on every page type; /brand/ and /feed.xml keep their by-design style-src 'unsafe-inline' relaxation. Zero inline &lt;style&gt; blocks in any built Astro page (home 0, article 0, about 0, phase0 0). Policy proven live again this run — a &lt;style&gt; injection was blocked, while CSSOM mutation of the already-loaded sheet succeeded, which is the documented distinction. | 2026-08-25 re-verified live: CSP present on every route and empirically ENFORCED — an injected inline &lt;style&gt; during this run was blocked by style-src 'self' and logged as the only console error of the whole scrub. Per-route relaxation for /brand/ (style-src adds 'unsafe-inline') confirmed by design. Zero inline &lt;style&gt; blocks in any built page. | 2026-08-27 re-verified live: CSP present and strict on / and on an article. | 2026-09-01 re-verified live: CSP present and identical on / and /words/&lt;slug&gt;/ — default-src 'self'; script-src 'self'; style-src 'self'; img-src 'self' data: https:; font-src 'self'; connect-src 'self'; frame-ancestors 'none'; base-uri 'self'; form-action 'self'; object-src 'none'; upgrade-insecure-requests. Zero inline &lt;style&gt; blocks in any built or served page (CSP would block them). | 2026-09-06 re-verified live: CSP present on all 7 sampled routes, with the by-design 'unsafe-inline' style-src relaxation only on /brand/ and /feed.xml. Zero inline &lt;style&gt; blocks in any built page. | 2026-09-11 re-verified live: CSP served on every route: default-src 'self'; script-src 'self'; style-src 'self'; frame-ancestors 'none'; object-src 'none'; upgrade-insecure-requests. Zero inline &lt;style&gt; tags in any built or served page. | 2026-09-23 re-verified live: CSP present on all 7 sampled routes (connect-src still allows the RUM collector); zero inline &lt;style&gt; in built HTML across home/about/404/17 articles; 0 console errors on 6 surfaces.</t>
+          <t>PASS — CSP present and strict on every page; per-route /brand/ + /feed.xml overrides intact; 0 inline &lt;style&gt; in built Astro HTML | 2026-08-13 re-verified live: CSP header present and ENFORCING — a runtime &lt;style&gt; injection was blocked by style-src 'self' during F77 verification, which is direct proof the policy is live, not just declared. Per-route /brand/ and /feed.xml relaxations by design. | 2026-08-16 re-verified live: CSP present and strict on every page type; /brand/ and /feed.xml keep their by-design style-src 'unsafe-inline' relaxation. Zero inline &lt;style&gt; blocks in any built Astro page (home 0, article 0, about 0, phase0 0). Policy proven live again this run — a &lt;style&gt; injection was blocked, while CSSOM mutation of the already-loaded sheet succeeded, which is the documented distinction. | 2026-08-25 re-verified live: CSP present on every route and empirically ENFORCED — an injected inline &lt;style&gt; during this run was blocked by style-src 'self' and logged as the only console error of the whole scrub. Per-route relaxation for /brand/ (style-src adds 'unsafe-inline') confirmed by design. Zero inline &lt;style&gt; blocks in any built page. | 2026-08-27 re-verified live: CSP present and strict on / and on an article. | 2026-09-01 re-verified live: CSP present and identical on / and /words/&lt;slug&gt;/ — default-src 'self'; script-src 'self'; style-src 'self'; img-src 'self' data: https:; font-src 'self'; connect-src 'self'; frame-ancestors 'none'; base-uri 'self'; form-action 'self'; object-src 'none'; upgrade-insecure-requests. Zero inline &lt;style&gt; blocks in any built or served page (CSP would block them). | 2026-09-06 re-verified live: CSP present on all 7 sampled routes, with the by-design 'unsafe-inline' style-src relaxation only on /brand/ and /feed.xml. Zero inline &lt;style&gt; blocks in any built page. | 2026-09-11 re-verified live: CSP served on every route: default-src 'self'; script-src 'self'; style-src 'self'; frame-ancestors 'none'; object-src 'none'; upgrade-insecure-requests. Zero inline &lt;style&gt; tags in any built or served page. | 2026-09-23 re-verified live: CSP present on all 7 sampled routes (connect-src still allows the RUM collector); zero inline &lt;style&gt; in built HTML across home/about/404/17 articles; 0 console errors on 6 surfaces. | 2026-09-28: live: CSP on every HTML route + feed; 0 inline scripts on 5 types; connect-src carries the RUM collector.</t>
         </is>
       </c>
       <c r="I72" s="6" t="inlineStr"/>
@@ -4205,7 +4209,7 @@
       </c>
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>PASS — X-Frame DENY, nosniff, HSTS max-age=31536000 includeSubDomains preload, Referrer-Policy, Permissions-Policy, COOP, CORP on all 21 routes | 2026-08-13 re-verified live: all 5 security headers present on all 6 page types (home, article, about, brand, phase0, 404, feed): X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000 includeSubDomains preload, CSP, Referrer-Policy strict-origin-when-cross-origin. Permissions-Policy also present. | 2026-08-16 re-verified live: all security headers re-verified live on home/article/brand/404/feed: X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000 includeSubDomains preload, CSP, Referrer-Policy strict-origin-when-cross-origin, Permissions-Policy, COOP same-origin, CORP same-origin. | 2026-08-25 re-verified live: all five headers present on / and on an article: X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000; includeSubDomains; preload, CSP, Referrer-Policy strict-origin-when-cross-origin. Permissions-Policy also present on /. | 2026-08-27 re-verified live: X-Frame DENY, nosniff, HSTS max-age=31536000 includeSubDomains preload, Referrer-Policy all present. | 2026-09-01 re-verified live: X-Frame-Options DENY, X-Content-Type-Options nosniff, Strict-Transport-Security max-age=31536000; includeSubDomains; preload, Referrer-Policy strict-origin-when-cross-origin — all present on / and on an article. | 2026-09-06 re-verified live: X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000; includeSubDomains; preload, Referrer-Policy strict-origin-when-cross-origin, Permissions-Policy - all 7 routes. | 2026-09-11 re-verified live: 5/5 security headers on /, /about/, /brand/, /words/the-stone/, /404 and /feed.xml; HSTS max-age=31536000; includeSubDomains; preload. | 2026-09-23 re-verified live: X-Frame-Options DENY, nosniff, HSTS max-age=31536000 includeSubDomains preload, CSP, Referrer-Policy on /, /about/, /brand/, /phase0/, /404, an article and /feed.xml.</t>
+          <t>PASS — X-Frame DENY, nosniff, HSTS max-age=31536000 includeSubDomains preload, Referrer-Policy, Permissions-Policy, COOP, CORP on all 21 routes | 2026-08-13 re-verified live: all 5 security headers present on all 6 page types (home, article, about, brand, phase0, 404, feed): X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000 includeSubDomains preload, CSP, Referrer-Policy strict-origin-when-cross-origin. Permissions-Policy also present. | 2026-08-16 re-verified live: all security headers re-verified live on home/article/brand/404/feed: X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000 includeSubDomains preload, CSP, Referrer-Policy strict-origin-when-cross-origin, Permissions-Policy, COOP same-origin, CORP same-origin. | 2026-08-25 re-verified live: all five headers present on / and on an article: X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000; includeSubDomains; preload, CSP, Referrer-Policy strict-origin-when-cross-origin. Permissions-Policy also present on /. | 2026-08-27 re-verified live: X-Frame DENY, nosniff, HSTS max-age=31536000 includeSubDomains preload, Referrer-Policy all present. | 2026-09-01 re-verified live: X-Frame-Options DENY, X-Content-Type-Options nosniff, Strict-Transport-Security max-age=31536000; includeSubDomains; preload, Referrer-Policy strict-origin-when-cross-origin — all present on / and on an article. | 2026-09-06 re-verified live: X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000; includeSubDomains; preload, Referrer-Policy strict-origin-when-cross-origin, Permissions-Policy - all 7 routes. | 2026-09-11 re-verified live: 5/5 security headers on /, /about/, /brand/, /words/the-stone/, /404 and /feed.xml; HSTS max-age=31536000; includeSubDomains; preload. | 2026-09-23 re-verified live: X-Frame-Options DENY, nosniff, HSTS max-age=31536000 includeSubDomains preload, CSP, Referrer-Policy on /, /about/, /brand/, /phase0/, /404, an article and /feed.xml. | 2026-09-28: live: XFO DENY, nosniff, HSTS 1y includeSubDomains preload, Referrer-Policy strict-origin-when-cross-origin, Permissions-Policy, COOP/CORP same-origin.</t>
         </is>
       </c>
       <c r="I73" s="6" t="inlineStr"/>
@@ -4258,7 +4262,7 @@
       </c>
       <c r="H74" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: /brand/brand.css?v=brand5 and /img/* both return public,max-age=31536000,immutable; HTML remains public,max-age=0,must-revalidate. | 2026-08-13 re-verified live: versioned assets (/css, /js, /img) all serve public,max-age=31536000,immutable; HTML serves public,max-age=0,must-revalidate. No drift. | 2026-08-16 re-verified live: versioned assets (/css, /js, /img, /fonts) all serve public,max-age=31536000,immutable; HTML serves public,max-age=0,must-revalidate. No drift. | 2026-08-25 re-verified live: versioned CSS, fonts and images all serve public,max-age=31536000,immutable; HTML serves public,max-age=0,must-revalidate. No drift on either tier. | 2026-08-27 re-verified live: HTML no-cache/must-revalidate; /css/*?v= and /img/* both public,max-age=31536000,immutable. | 2026-09-01 re-verified live: /css/tokens.css?v=phase24 and /fonts/Anton-Regular.woff2 both return public,max-age=31536000,immutable; HTML returns public,max-age=0,must-revalidate. No drift on either pattern. | 2026-09-06 re-verified live: HTML public,max-age=0,must-revalidate; /css, /fonts, /img, /js and /_astro all public,max-age=31536000,immutable. | 2026-09-11 re-verified live: versioned css/js/font/img all public,max-age=31536000,immutable; HTML public,max-age=0,must-revalidate. No drift. | 2026-09-23 re-verified live: 20 versioned /css /js /fonts /img /_astro assets all public,max-age=31536000,immutable; HTML public,max-age=0,must-revalidate.</t>
+          <t>PASS — live-verified 2026-08-10: /brand/brand.css?v=brand5 and /img/* both return public,max-age=31536000,immutable; HTML remains public,max-age=0,must-revalidate. | 2026-08-13 re-verified live: versioned assets (/css, /js, /img) all serve public,max-age=31536000,immutable; HTML serves public,max-age=0,must-revalidate. No drift. | 2026-08-16 re-verified live: versioned assets (/css, /js, /img, /fonts) all serve public,max-age=31536000,immutable; HTML serves public,max-age=0,must-revalidate. No drift. | 2026-08-25 re-verified live: versioned CSS, fonts and images all serve public,max-age=31536000,immutable; HTML serves public,max-age=0,must-revalidate. No drift on either tier. | 2026-08-27 re-verified live: HTML no-cache/must-revalidate; /css/*?v= and /img/* both public,max-age=31536000,immutable. | 2026-09-01 re-verified live: /css/tokens.css?v=phase24 and /fonts/Anton-Regular.woff2 both return public,max-age=31536000,immutable; HTML returns public,max-age=0,must-revalidate. No drift on either pattern. | 2026-09-06 re-verified live: HTML public,max-age=0,must-revalidate; /css, /fonts, /img, /js and /_astro all public,max-age=31536000,immutable. | 2026-09-11 re-verified live: versioned css/js/font/img all public,max-age=31536000,immutable; HTML public,max-age=0,must-revalidate. No drift. | 2026-09-23 re-verified live: 20 versioned /css /js /fonts /img /_astro assets all public,max-age=31536000,immutable; HTML public,max-age=0,must-revalidate. | 2026-09-28: live: 47 versioned assets public,max-age=31536000,immutable; fonts ACAO *; HTML + feed public,max-age=0,must-revalidate.</t>
         </is>
       </c>
       <c r="I74" s="6" t="inlineStr"/>
@@ -4311,7 +4315,7 @@
       </c>
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>PASS — predicate gates homepage/feed/sitemap/routes consistently; 16 published, 0 upcoming | 2026-09-18 re-verified live: 17 published, 0 upcoming — homepage 17 plates, feed 17 entries, sitemap 17 /words/ URLs, all consistent. (An untracked drafted entry sits in the working tree and is correctly nowhere live.) | 2026-09-23 re-verified live: 17 published, 0 upcoming — homepage 17 plates, feed 17 entries, sitemap 17 /words/ URLs (21 locs), all set-equal.</t>
+          <t>PASS — predicate gates homepage/feed/sitemap/routes consistently; 16 published, 0 upcoming | 2026-09-18 re-verified live: 17 published, 0 upcoming — homepage 17 plates, feed 17 entries, sitemap 17 /words/ URLs, all consistent. (An untracked drafted entry sits in the working tree and is correctly nowhere live.) | 2026-09-23 re-verified live: 17 published, 0 upcoming — homepage 17 plates, feed 17 entries, sitemap 17 /words/ URLs (21 locs), all set-equal. | 2026-09-28: live: 17/17 published + past-dated all live; fixture build: future-dated entry out of cascade/feed/sitemap, ghost plate shown, coming-soon page built.</t>
         </is>
       </c>
       <c r="I75" s="6" t="inlineStr"/>
@@ -4364,7 +4368,7 @@
       </c>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>PASS — 2026-09-22 live-verified: GitHub Actions 'Daily rebuild' has 40 runs across 40 distinct days (2026-08-14 -&gt; 2026-09-22), zero missing-day gaps, all conclusion=success. Today's fired 09:51:20Z and produced the live Netlify deploy 6ab24fa0 (published 09:51:43Z, commit 95e2a73). The single 2026-08-27 miss that opened this row has not recurred in the 26 days since. | 2026-09-23 re-verified live: Daily rebuild fired 09:52:35Z (success) and produced Netlify deploy 6ab3a167 on 95e2a73 — 41 consecutive days.</t>
+          <t>PASS — 2026-09-22 live-verified: GitHub Actions 'Daily rebuild' has 40 runs across 40 distinct days (2026-08-14 -&gt; 2026-09-22), zero missing-day gaps, all conclusion=success. Today's fired 09:51:20Z and produced the live Netlify deploy 6ab24fa0 (published 09:51:43Z, commit 95e2a73). The single 2026-08-27 miss that opened this row has not recurred in the 26 days since. | 2026-09-23 re-verified live: Daily rebuild fired 09:52:35Z (success) and produced Netlify deploy 6ab3a167 on 95e2a73 — 41 consecutive days. | 2026-09-28: live: Daily rebuild succeeded 09-25/26/27; latest ready deploy 95e2a73 at 2026-09-27 10:29Z == GitHub main.</t>
         </is>
       </c>
       <c r="I76" s="6" t="inlineStr"/>
@@ -4417,7 +4421,7 @@
       </c>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>PASS — scripts/og-plate.mjs present; all 19 OG plates render and 200 | 2026-08-27 re-verified live: all 21 OG plates 200. | 2026-09-01 re-verified live: every one of the 17 per-article OG plates resolves 200 at its cache-busted path; none falls back to og-default.png. | 2026-09-19 re-verified live: 17/17 per-article OG plates 200 at their cache-busted paths; JSON-LD image == og:image on all 17; none falls back to og-default.png. | 2026-09-23 re-verified live: all 21 og:image URLs (17 per-article + home/about/brand/phase0) 200; every BlogPosting image == og:image, og-&lt;slug&gt;.png?v=phaseNN, no og-default drift.</t>
+          <t>PASS — scripts/og-plate.mjs present; all 19 OG plates render and 200 | 2026-08-27 re-verified live: all 21 OG plates 200. | 2026-09-01 re-verified live: every one of the 17 per-article OG plates resolves 200 at its cache-busted path; none falls back to og-default.png. | 2026-09-19 re-verified live: 17/17 per-article OG plates 200 at their cache-busted paths; JSON-LD image == og:image on all 17; none falls back to og-default.png. | 2026-09-23 re-verified live: all 21 og:image URLs (17 per-article + home/about/brand/phase0) 200; every BlogPosting image == og:image, og-&lt;slug&gt;.png?v=phaseNN, no og-default drift. | 2026-09-28: live: og-&lt;slug&gt;.png 200 for 17/17; generator source unchanged.</t>
         </is>
       </c>
       <c r="I77" s="6" t="inlineStr"/>
@@ -4470,7 +4474,7 @@
       </c>
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>PASS — @media (prefers-reduced-motion: reduce) block in tokens.css (loads on every page) | 2026-08-13 re-verified live: verified in the DEPLOYED sheet, not just source: tokens.css?v=phase23 carries @media (prefers-reduced-motion: reduce) zeroing transition-duration and animation-duration on *, *::before, *::after with !important, plus scroll-behavior auto. Catches all 29 transitioned elements on the homepage. | 2026-08-16 re-verified live: re-verified in the LOADED CSSOM (not source): tokens.css?v=phase23 carries @media (prefers-reduced-motion: reduce) zeroing transition-duration and animation-duration on *, ::before, ::after with !important plus scroll-behavior auto — catching all 8 transitioned elements on the article page. | 2026-08-25 re-verified live: tokens.css:584 zeroes transition-duration and animation-duration on *, ::before and ::after under prefers-reduced-motion: reduce and sets scroll-behavior auto; home-augment.css:1012 adds the targeted transition:none block. Both present in the served sheets. | 2026-08-27 re-verified live: @media (prefers-reduced-motion: reduce) block present in the loaded stylesheets. | 2026-09-01 SOURCE-VERIFIED only: tokens.css?v=phase24 carries a blanket @media (prefers-reduced-motion: reduce) block setting transition-duration and animation-duration to 0s !important on *, *::before and *::after, plus scroll-behavior: auto on html; home-augment.css adds two scoped blocks. The !important universal selector is cascade-proof, so the rule cannot be defeated downstream. NOT re-verified in the browser: this harness cannot emulate the prefers-reduced-motion media query. Prior live PASS retained. | 2026-09-06 re-verified live (source-verified): the global @media (prefers-reduced-motion: reduce) kill switch is present in the loaded tokens.css cascade (tokens.css:573-582, transition-duration 0s !important on *, ::before, ::after). Not driven end-to-end - the pane cannot emulate the media query. | 2026-09-11 re-verified live: two prefers-reduced-motion blocks live — tokens.css zeroes transition/animation duration globally, home-augment.css nulls five named transitions. | 2026-09-24 re-verified live: tokens.css?v=phase24 still carries @media (prefers-reduced-motion: reduce) (html scroll-behavior auto; *,*::before,*::after durations zeroed) and home-augment.css carries 2 reduced-motion blocks; both present in the deployed sheets' CSSOM on the homepage.</t>
+          <t>PASS — @media (prefers-reduced-motion: reduce) block in tokens.css (loads on every page) | 2026-08-13 re-verified live: verified in the DEPLOYED sheet, not just source: tokens.css?v=phase23 carries @media (prefers-reduced-motion: reduce) zeroing transition-duration and animation-duration on *, *::before, *::after with !important, plus scroll-behavior auto. Catches all 29 transitioned elements on the homepage. | 2026-08-16 re-verified live: re-verified in the LOADED CSSOM (not source): tokens.css?v=phase23 carries @media (prefers-reduced-motion: reduce) zeroing transition-duration and animation-duration on *, ::before, ::after with !important plus scroll-behavior auto — catching all 8 transitioned elements on the article page. | 2026-08-25 re-verified live: tokens.css:584 zeroes transition-duration and animation-duration on *, ::before and ::after under prefers-reduced-motion: reduce and sets scroll-behavior auto; home-augment.css:1012 adds the targeted transition:none block. Both present in the served sheets. | 2026-08-27 re-verified live: @media (prefers-reduced-motion: reduce) block present in the loaded stylesheets. | 2026-09-01 SOURCE-VERIFIED only: tokens.css?v=phase24 carries a blanket @media (prefers-reduced-motion: reduce) block setting transition-duration and animation-duration to 0s !important on *, *::before and *::after, plus scroll-behavior: auto on html; home-augment.css adds two scoped blocks. The !important universal selector is cascade-proof, so the rule cannot be defeated downstream. NOT re-verified in the browser: this harness cannot emulate the prefers-reduced-motion media query. Prior live PASS retained. | 2026-09-06 re-verified live (source-verified): the global @media (prefers-reduced-motion: reduce) kill switch is present in the loaded tokens.css cascade (tokens.css:573-582, transition-duration 0s !important on *, ::before, ::after). Not driven end-to-end - the pane cannot emulate the media query. | 2026-09-11 re-verified live: two prefers-reduced-motion blocks live — tokens.css zeroes transition/animation duration globally, home-augment.css nulls five named transitions. | 2026-09-24 re-verified live: tokens.css?v=phase24 still carries @media (prefers-reduced-motion: reduce) (html scroll-behavior auto; *,*::before,*::after durations zeroed) and home-augment.css carries 2 reduced-motion blocks; both present in the deployed sheets' CSSOM on the homepage. | 2026-09-28: live: prefers-reduced-motion rules in tokens.css + home-augment.css; 2 reduced-motion media rules loaded on home.</t>
         </is>
       </c>
       <c r="I78" s="6" t="inlineStr"/>
@@ -4523,7 +4527,7 @@
       </c>
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>PASS (closed live 2026-08-10) — was ISSUE/High: .subscribe-manifesto .sm-submit (homepage + /brand/ subscribe submit) had base and :hover styling but NO :focus-visible rule, so the site's primary conversion control showed no focus indicator for keyboard users (WCAG 2.4.7 AA). Every sibling control was covered — .sm-input directly above it had the rule, and .sm-submit was even named in home-augment.css's prefers-reduced-motion block — so it was an omission, not a decision. Missed by prior runs because F76 was tested at sheet level (':focus-visible present in all 8 stylesheets') rather than per control. Fixed and deployed same day; see p3/p4. | 2026-08-13 re-verified live: re-verified live by REAL keyboard input (not JS .focus(), which cannot trigger :focus-visible): pressing Tab moved focus to a footer link that matched ':focus-visible' and computed outline 'solid 2px rgb(204, 0, 0)' at offset 2px. | 2026-08-16 re-verified live: re-verified live by REAL keyboard input (not JS .focus(), which cannot trigger :focus-visible): pressing Tab moved focus to SUMMARY.study-note-trigger, which matched ':focus-visible' and computed outline 'rgb(204, 0, 0) solid 2px' at offset -2px. | 2026-08-25 re-verified live: re-verified under REAL keyboard input: tabbing to .study-note-trigger on an article paints outline solid 2px rgb(204,0,0) (--focus-ring) at -2px offset. NOTE for future runs: a programmatic element.focus() does NOT satisfy :focus-visible in Chrome and will report outline:none across the board — a false positive this run initially produced. | 2026-08-27 re-verified live: focus ring under REAL Tab (not element.focus()): outline rgb(204,0,0) solid 2px = --accent. | 2026-09-01 re-verified live under REAL Tab presses (never element.focus()): .brand-block, .mode-toggle, .issue-standfirst and .hero-link each match :focus-visible and paint outline rgb(204,0,0) solid 2px, matching --focus-ring #c00. | 2026-09-06 re-verified live: real Tab/Shift+Tab presses put outline: rgb(204,0,0) solid 2px on plate links, .lane-cell, .earlier-more-btn and .brand-block. The skip link is the one exception and is F98. | 2026-09-11 re-verified live: real Tab walk on the homepage: skip-link → brand-block → hero links → lane cells, every stop carrying outline rgb(204,0,0) solid 2px. | 2026-09-24 re-verified live: every css/*.css defines :focus-visible (article 9, home-augment 6, home-v2 5, shell 5, tokens 2, phase0 2, plates 1, notfound 1). Real Tab on the homepage: .brand-block and .skip-link both render solid 2px rgb(204,0,0) with :focus-visible true; skip link activates to MAIN#archive.</t>
+          <t>PASS (closed live 2026-08-10) — was ISSUE/High: .subscribe-manifesto .sm-submit (homepage + /brand/ subscribe submit) had base and :hover styling but NO :focus-visible rule, so the site's primary conversion control showed no focus indicator for keyboard users (WCAG 2.4.7 AA). Every sibling control was covered — .sm-input directly above it had the rule, and .sm-submit was even named in home-augment.css's prefers-reduced-motion block — so it was an omission, not a decision. Missed by prior runs because F76 was tested at sheet level (':focus-visible present in all 8 stylesheets') rather than per control. Fixed and deployed same day; see p3/p4. | 2026-08-13 re-verified live: re-verified live by REAL keyboard input (not JS .focus(), which cannot trigger :focus-visible): pressing Tab moved focus to a footer link that matched ':focus-visible' and computed outline 'solid 2px rgb(204, 0, 0)' at offset 2px. | 2026-08-16 re-verified live: re-verified live by REAL keyboard input (not JS .focus(), which cannot trigger :focus-visible): pressing Tab moved focus to SUMMARY.study-note-trigger, which matched ':focus-visible' and computed outline 'rgb(204, 0, 0) solid 2px' at offset -2px. | 2026-08-25 re-verified live: re-verified under REAL keyboard input: tabbing to .study-note-trigger on an article paints outline solid 2px rgb(204,0,0) (--focus-ring) at -2px offset. NOTE for future runs: a programmatic element.focus() does NOT satisfy :focus-visible in Chrome and will report outline:none across the board — a false positive this run initially produced. | 2026-08-27 re-verified live: focus ring under REAL Tab (not element.focus()): outline rgb(204,0,0) solid 2px = --accent. | 2026-09-01 re-verified live under REAL Tab presses (never element.focus()): .brand-block, .mode-toggle, .issue-standfirst and .hero-link each match :focus-visible and paint outline rgb(204,0,0) solid 2px, matching --focus-ring #c00. | 2026-09-06 re-verified live: real Tab/Shift+Tab presses put outline: rgb(204,0,0) solid 2px on plate links, .lane-cell, .earlier-more-btn and .brand-block. The skip link is the one exception and is F98. | 2026-09-11 re-verified live: real Tab walk on the homepage: skip-link → brand-block → hero links → lane cells, every stop carrying outline rgb(204,0,0) solid 2px. | 2026-09-24 re-verified live: every css/*.css defines :focus-visible (article 9, home-augment 6, home-v2 5, shell 5, tokens 2, phase0 2, plates 1, notfound 1). Real Tab on the homepage: .brand-block and .skip-link both render solid 2px rgb(204,0,0) with :focus-visible true; skip link activates to MAIN#archive. | 2026-09-28: live: all 8 css files define :focus-visible; skip link under real Tab -&gt; 2px solid #c00.</t>
         </is>
       </c>
       <c r="I79" s="6" t="inlineStr">
@@ -4580,7 +4584,7 @@
       </c>
       <c r="H80" s="6" t="inlineStr">
         <is>
-          <t>PASS (closed live 2026-08-13) — was ISSUE/High (2026-08-13) — .latest-tag (the red 'Latest' chip in the homepage standfirst bar) pairs `background: var(--accent)` with `color: var(--bg)`. In light mode that is cream on #c00 = 5.17:1 and passes. In dark mode --bg flips to #060606 and the same chip computes 3.44:1 at 11.52px/700 — under the 4.5:1 AA floor for small text (WCAG 1.4.3). Measured three times on settled live loads. The #c00/#060606 pair is sanctioned by the Phase 4.1 accent doctrine (DESIGN-SYSTEM.md:102) only for NON-text contrast at the 3:1 floor; this is a text use of it. Missed by prior runs because F77 sampled palette-level token pairs (body/muted/faint/accent text), not the one control that puts small text ON the accent fill — the same sheet-level vs per-control gap that hid F76. All other sampled combinations still pass: 33 distinct fg/bg/size combos in dark, 33 in light, this was the only failure. | 2026-08-16 re-verified live: full-page compositor sweep across home (dark 92 elements / light 88), article (70), about (15), phase0 (84), brand and 404. Two light-mode 'failures' on .plate-image plates (h2.plate-title.inverse and p.plate-deck, both 1.06:1) were investigated and DISMISSED as false positives: those plates carry an ::after `linear-gradient(to top, rgba(0,0,0,.78) ...)` scrim, so the white text sits on a dark overlay, not the cream plate colour the compositor resolved — confirmed visually in a light-mode screenshot. Two compounding methodology bugs were behind the false read and are now fixed in the sweep: (a) the compositor walked background-COLOR only and ignored pseudo-element layers, (b) selector-level dedupe merged image and non-image plates under the same class string, so a passing element inherited a failing element's number. Lesson is the same shape as F84's: resolve the PAINTED surface, never infer it from an ancestor's declarations. | 2026-08-25 re-verified live: .latest-tag on the live homepage in dark mode measures 5.17:1 (rgb(243,240,232) on rgb(204,0,0)) — the F77 fix still holds, no regression. | 2026-09-01 re-verified live with a full ancestor-stack compositing probe (semi-transparent layers composited down to the first opaque one; .plate-image plates and aria-hidden decoration excluded per the documented antipatterns): 0 WCAG AA failures across ~1050 measured text elements — homepage light (0/70+), homepage dark (0/70), article dark at 375px (0/86), /about/ (0/24), /404 (0/16), /phase0/ (0/106), /brand/ (0/800). | 2026-09-06 re-verified live: the sweep is now pixel-based on image plates, not computed-style-based. Composited-ancestor probe across home, article, about, 404, phase0 and /brand/ in BOTH modes: zero failures outside the image plates. Inside them, rasterised sampling opened F101 (2.68:1 on img-concrete) - a defect every previous computed-style sweep reported as the known 1.06:1 artifact. | 2026-09-11 re-verified live: composited-stack contrast sweep over home/about/brand/phase0/404/article in BOTH modes: zero real failures. Only hits were the aria-hidden .dot separators (4.25–4.30:1, exempt, documented) and the image-plate 1.06:1 probe artifact, dismissed on geometry (below). | 2026-09-24 re-verified live: contrast sweep with full ancestor compositing and inherited opacity, both modes: home 70 elements, article (the-weight-of-my-no) 86, /about/ 24, /404 16, /phase0/ 106, /brand/ 793 — 0 failures in light, 0 in dark (image plates excluded per the antipattern; 8/8 home and 5/5 brand demo plate bodies keep display:flex + justify-content:flex-end). Hover states are F83/F108's scope.</t>
+          <t>PASS (closed live 2026-08-13) — was ISSUE/High (2026-08-13) — .latest-tag (the red 'Latest' chip in the homepage standfirst bar) pairs `background: var(--accent)` with `color: var(--bg)`. In light mode that is cream on #c00 = 5.17:1 and passes. In dark mode --bg flips to #060606 and the same chip computes 3.44:1 at 11.52px/700 — under the 4.5:1 AA floor for small text (WCAG 1.4.3). Measured three times on settled live loads. The #c00/#060606 pair is sanctioned by the Phase 4.1 accent doctrine (DESIGN-SYSTEM.md:102) only for NON-text contrast at the 3:1 floor; this is a text use of it. Missed by prior runs because F77 sampled palette-level token pairs (body/muted/faint/accent text), not the one control that puts small text ON the accent fill — the same sheet-level vs per-control gap that hid F76. All other sampled combinations still pass: 33 distinct fg/bg/size combos in dark, 33 in light, this was the only failure. | 2026-08-16 re-verified live: full-page compositor sweep across home (dark 92 elements / light 88), article (70), about (15), phase0 (84), brand and 404. Two light-mode 'failures' on .plate-image plates (h2.plate-title.inverse and p.plate-deck, both 1.06:1) were investigated and DISMISSED as false positives: those plates carry an ::after `linear-gradient(to top, rgba(0,0,0,.78) ...)` scrim, so the white text sits on a dark overlay, not the cream plate colour the compositor resolved — confirmed visually in a light-mode screenshot. Two compounding methodology bugs were behind the false read and are now fixed in the sweep: (a) the compositor walked background-COLOR only and ignored pseudo-element layers, (b) selector-level dedupe merged image and non-image plates under the same class string, so a passing element inherited a failing element's number. Lesson is the same shape as F84's: resolve the PAINTED surface, never infer it from an ancestor's declarations. | 2026-08-25 re-verified live: .latest-tag on the live homepage in dark mode measures 5.17:1 (rgb(243,240,232) on rgb(204,0,0)) — the F77 fix still holds, no regression. | 2026-09-01 re-verified live with a full ancestor-stack compositing probe (semi-transparent layers composited down to the first opaque one; .plate-image plates and aria-hidden decoration excluded per the documented antipatterns): 0 WCAG AA failures across ~1050 measured text elements — homepage light (0/70+), homepage dark (0/70), article dark at 375px (0/86), /about/ (0/24), /404 (0/16), /phase0/ (0/106), /brand/ (0/800). | 2026-09-06 re-verified live: the sweep is now pixel-based on image plates, not computed-style-based. Composited-ancestor probe across home, article, about, 404, phase0 and /brand/ in BOTH modes: zero failures outside the image plates. Inside them, rasterised sampling opened F101 (2.68:1 on img-concrete) - a defect every previous computed-style sweep reported as the known 1.06:1 artifact. | 2026-09-11 re-verified live: composited-stack contrast sweep over home/about/brand/phase0/404/article in BOTH modes: zero real failures. Only hits were the aria-hidden .dot separators (4.25–4.30:1, exempt, documented) and the image-plate 1.06:1 probe artifact, dismissed on geometry (below). | 2026-09-24 re-verified live: contrast sweep with full ancestor compositing and inherited opacity, both modes: home 70 elements, article (the-weight-of-my-no) 86, /about/ 24, /404 16, /phase0/ 106, /brand/ 793 — 0 failures in light, 0 in dark (image plates excluded per the antipattern; 8/8 home and 5/5 brand demo plate bodies keep display:flex + justify-content:flex-end). Hover states are F83/F108's scope. | 2026-09-28: live: contrast sweep 0 failures — dark: home, about, article, phase0, 404, brand; light: home, about, article, phase0, brand.</t>
         </is>
       </c>
       <c r="I80" s="6" t="inlineStr">
@@ -4637,7 +4641,7 @@
       </c>
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>PASS — single h1 and zero skipped heading levels on all 21 pages; header/main/footer/nav present; zero &lt;img&gt; without alt | 2026-08-13 re-verified live: home and article both single-h1, zero skipped heading levels (home H1 then 17x H2; article H1,H2,H2,H2,H2,H2), header/main/footer/nav all present. Zero images missing alt. | 2026-08-16 re-verified live: single &lt;h1&gt; and zero skipped heading levels across all 21 live pages; header/main/footer/nav present on every page type; zero &lt;img&gt; without an alt attribute. | 2026-08-25 re-verified live: header/main/footer/nav present on every page type; exactly one &lt;h1&gt; per page across all 20 routes; zero skipped heading levels; zero &lt;img&gt; without alt. | 2026-08-27 re-verified live: single h1 and zero skipped heading levels across all 21 routes. | 2026-09-01 re-verified live: header/main/footer/nav present on every route; exactly one h1 per page; no skipped heading levels anywhere, including /phase0/'s 22-heading tree. | 2026-09-06 re-verified live: header/nav/main/footer all present on the homepage; exactly one h1 per page and no skipped heading levels across home, about, brand, phase0 and 404. | 2026-09-11 re-verified live: single h1 and no skipped heading level on all six surface types; header/main/footer/nav present on each. | 2026-09-24 re-verified live: single h1 on home, article, /about/, /404, /phase0/, /brand/; home headings 1 then 18x2, article 1-2-2-2; header, main[id] (archive / article / about / main / phase0 / main), footer present everywhere; nav aria-labels 'Main navigation' (+ 'Essay navigation' on articles); 0 &lt;img&gt; without alt (the masthead logo's alt='' is decorative inside the labelled brand link).</t>
+          <t>PASS — single h1 and zero skipped heading levels on all 21 pages; header/main/footer/nav present; zero &lt;img&gt; without alt | 2026-08-13 re-verified live: home and article both single-h1, zero skipped heading levels (home H1 then 17x H2; article H1,H2,H2,H2,H2,H2), header/main/footer/nav all present. Zero images missing alt. | 2026-08-16 re-verified live: single &lt;h1&gt; and zero skipped heading levels across all 21 live pages; header/main/footer/nav present on every page type; zero &lt;img&gt; without an alt attribute. | 2026-08-25 re-verified live: header/main/footer/nav present on every page type; exactly one &lt;h1&gt; per page across all 20 routes; zero skipped heading levels; zero &lt;img&gt; without alt. | 2026-08-27 re-verified live: single h1 and zero skipped heading levels across all 21 routes. | 2026-09-01 re-verified live: header/main/footer/nav present on every route; exactly one h1 per page; no skipped heading levels anywhere, including /phase0/'s 22-heading tree. | 2026-09-06 re-verified live: header/nav/main/footer all present on the homepage; exactly one h1 per page and no skipped heading levels across home, about, brand, phase0 and 404. | 2026-09-11 re-verified live: single h1 and no skipped heading level on all six surface types; header/main/footer/nav present on each. | 2026-09-24 re-verified live: single h1 on home, article, /about/, /404, /phase0/, /brand/; home headings 1 then 18x2, article 1-2-2-2; header, main[id] (archive / article / about / main / phase0 / main), footer present everywhere; nav aria-labels 'Main navigation' (+ 'Essay navigation' on articles); 0 &lt;img&gt; without alt (the masthead logo's alt='' is decorative inside the labelled brand link). | 2026-09-28: live: single h1 on every type, no skipped levels, header/main/footer/nav landmarks.</t>
         </is>
       </c>
       <c r="I81" s="6" t="inlineStr"/>
@@ -4690,7 +4694,7 @@
       </c>
       <c r="H82" s="6" t="inlineStr">
         <is>
-          <t>PASS — fired as designed on 2026-07-05 (ecf2c34, github-actions[bot], 18:03:14Z); both guards now permanently closed (year!=2026, status no longer 'drafted'); no post-fire bot commit exists on main | 2026-09-11 re-verified live: publish-send-someone-else.yml still absent (removed 11d1430); daily-rebuild.yml is the only workflow; send-someone-else status still 'published'. No post-fire github-actions[bot] commit on main. | 2026-09-24 re-verified live: daily-rebuild.yml is still the only workflow; publish-send-someone-else.yml absent; zero github-actions commits on origin/main since 2026-07-06.</t>
+          <t>PASS — fired as designed on 2026-07-05 (ecf2c34, github-actions[bot], 18:03:14Z); both guards now permanently closed (year!=2026, status no longer 'drafted'); no post-fire bot commit exists on main | 2026-09-11 re-verified live: publish-send-someone-else.yml still absent (removed 11d1430); daily-rebuild.yml is the only workflow; send-someone-else status still 'published'. No post-fire github-actions[bot] commit on main. | 2026-09-24 re-verified live: daily-rebuild.yml is still the only workflow; publish-send-someone-else.yml absent; zero github-actions commits on origin/main since 2026-07-06. | 2026-09-28: repo: daily-rebuild.yml still the only workflow; publish workflow removed (11d1430).</t>
         </is>
       </c>
       <c r="I82" s="6" t="inlineStr"/>
@@ -4743,7 +4747,7 @@
       </c>
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>PASS — parity 16/16 verified live; every /words/&lt;slug&gt; returns a single 301 to its trailing-slash canonical; no orphan rules | 2026-08-13 re-verified live: all 16 /words/&lt;slug&gt; (no trailing slash) return 301; all 16 /words/&lt;slug&gt;/ return 200 in 0.31-0.45s. | 2026-08-25 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-01 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-06 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-11 re-verified live: /words/&lt;slug&gt; → 301 → /words/&lt;slug&gt;/ → 200 verified on the-stone; all 17 article slugs 200 at their canonical form. | 2026-09-24 ISSUE/Low — the parity test the expected column defines, run for the first time since 2026-08-31, fails 16/17: the-weight-of-my-no (status published, 2026-08-31) has no [[redirects]] rule in netlify.toml. Every run since 08-31 spot-checked /words/the-stone only, so the drift went unseen for 24 days — the same shape as the July show-me-your-glory / send-someone-else drift. The expected column's 'non-slash 404s' premise did NOT hold: live /words/the-weight-of-my-no returns 301 -&gt; /words/the-weight-of-my-no/ with no rule, because Netlify Pretty URLs redirects a directory path on its own. No user impact observed; graded Low (parity/config drift, not a broken route). | 2026-09-25: live behaviour unchanged (single 301 via Pretty URLs); rule still only on the unmerged branch. | 2026-09-26 full parity test (not a spot check) on qa/fixes-20260926: 17 published slugs == 17 /words/&lt;slug&gt; rules, 0 missing, 0 orphans, 0 dupes, no force; live: all 17 /words/&lt;slug&gt; return a single 301 to the slash canonical -&gt; 200. Fix still awaits merge (origin/main 95e2a73 lacks the rule; live behaviour unaffected).</t>
+          <t>PASS — parity 16/16 verified live; every /words/&lt;slug&gt; returns a single 301 to its trailing-slash canonical; no orphan rules | 2026-08-13 re-verified live: all 16 /words/&lt;slug&gt; (no trailing slash) return 301; all 16 /words/&lt;slug&gt;/ return 200 in 0.31-0.45s. | 2026-08-25 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-01 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-06 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-11 re-verified live: /words/&lt;slug&gt; → 301 → /words/&lt;slug&gt;/ → 200 verified on the-stone; all 17 article slugs 200 at their canonical form. | 2026-09-24 ISSUE/Low — the parity test the expected column defines, run for the first time since 2026-08-31, fails 16/17: the-weight-of-my-no (status published, 2026-08-31) has no [[redirects]] rule in netlify.toml. Every run since 08-31 spot-checked /words/the-stone only, so the drift went unseen for 24 days — the same shape as the July show-me-your-glory / send-someone-else drift. The expected column's 'non-slash 404s' premise did NOT hold: live /words/the-weight-of-my-no returns 301 -&gt; /words/the-weight-of-my-no/ with no rule, because Netlify Pretty URLs redirects a directory path on its own. No user impact observed; graded Low (parity/config drift, not a broken route). | 2026-09-25: live behaviour unchanged (single 301 via Pretty URLs); rule still only on the unmerged branch. | 2026-09-26 full parity test (not a spot check) on qa/fixes-20260926: 17 published slugs == 17 /words/&lt;slug&gt; rules, 0 missing, 0 orphans, 0 dupes, no force; live: all 17 /words/&lt;slug&gt; return a single 301 to the slash canonical -&gt; 200. Fix still awaits merge (origin/main 95e2a73 lacks the rule; live behaviour unaffected). | 2026-09-28: live parity: 17/17 /words/&lt;slug&gt; return a single 301 to the slash canonical; rule still only on the unmerged branch.</t>
         </is>
       </c>
       <c r="I83" s="6" t="inlineStr">
@@ -4758,7 +4762,7 @@
       </c>
       <c r="K83" s="6" t="inlineStr">
         <is>
-          <t>PASS (2026-09-24, verified against build) — netlify.toml parses (29 redirects); parity test published slugs == /words/&lt;slug&gt; rule set, 17/17, 0 orphans, 0 dupes, no force on any /words/&lt;slug&gt; rule; npm run build clean (20 pages). Live behaviour was already a single 301 and is unchanged by the rule. Note for the expected column: a missing rule here showed up as parity drift, not a 404. | 2026-09-27: live parity re-checked — all 17 /words/&lt;slug&gt; return a single 301 to the slash canonical; /about, /brand, /phase0 likewise. Fix still awaits merge.</t>
+          <t>PASS (2026-09-24, verified against build) — netlify.toml parses (29 redirects); parity test published slugs == /words/&lt;slug&gt; rule set, 17/17, 0 orphans, 0 dupes, no force on any /words/&lt;slug&gt; rule; npm run build clean (20 pages). Live behaviour was already a single 301 and is unchanged by the rule. Note for the expected column: a missing rule here showed up as parity drift, not a 404. | 2026-09-27: live parity re-checked — all 17 /words/&lt;slug&gt; return a single 301 to the slash canonical; /about, /brand, /phase0 likewise. Fix still awaits merge. | 2026-09-28: live parity 17/17 unchanged; fix still awaits merge.</t>
         </is>
       </c>
     </row>
@@ -4800,7 +4804,7 @@
       </c>
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: show-me-your-glory emits rel=next to send-someone-else and renders a normal (non-ghost) forward nav; forward chain walks all 16 published essays end to end. | 2026-08-25 re-verified live: forward chain walks all 16 published essays end to end; the chronologically newest (send-someone-else) correctly carries no next. | 2026-09-18 re-verified live: forward chain walks all 17 published essays end to end, reckonings → the-weight-of-my-no; only the newest lacks rel=next and only the oldest lacks rel=prev. | 2026-09-24 re-verified live: forward chain walks all 17 published essays end to end from the oldest; the newest (the-weight-of-my-no, 2026-08-31) is the only entry without next; every next target is a published slug.</t>
+          <t>PASS — live-verified 2026-08-10: show-me-your-glory emits rel=next to send-someone-else and renders a normal (non-ghost) forward nav; forward chain walks all 16 published essays end to end. | 2026-08-25 re-verified live: forward chain walks all 16 published essays end to end; the chronologically newest (send-someone-else) correctly carries no next. | 2026-09-18 re-verified live: forward chain walks all 17 published essays end to end, reckonings → the-weight-of-my-no; only the newest lacks rel=next and only the oldest lacks rel=prev. | 2026-09-24 re-verified live: forward chain walks all 17 published essays end to end from the oldest; the newest (the-weight-of-my-no, 2026-08-31) is the only entry without next; every next target is a published slug. | 2026-09-28: repo: forward chain 16/16 — every entry except the newest carries next == its chronological successor; 0 mismatches.</t>
         </is>
       </c>
       <c r="I84" s="6" t="inlineStr"/>
@@ -4853,7 +4857,7 @@
       </c>
       <c r="H85" s="6" t="inlineStr">
         <is>
-          <t>PASS (resolved 2026-08-10) — was ISSUE/Low: DESIGN-SYSTEM.md:115 listed "Reading progress bar (`var(--accent)`)" as a permitted accent use, but css/article.css:876 ships `.reading-progress { background: var(--ink) }`. Commit 68b0c1d (2026-04-10) recolored it on purpose and left the reason in the CSS: red was competing with the masthead and diluting the accent's semantic weight. That commit rewrote 136 lines of DESIGN-SYSTEM.md but missed this one bullet, which dated to c75ded9 earlier the same day. The CSS was correct; the doc line was stale. | 2026-08-27 second doc-parity pass (9b8e4c4): three more drifts closed, all doc-side. The Ghost Teaser Plate code block was pre-F90 and pre-cutover (min-height 346 vs the shipped 230; .plate-title opacity .35 vs .46/.40; --ink+opacity on .teaser-date and .meta-rail vs --body-muted), its prose still carried the static-HTML instruction 'swap for the full article plate and remove the ghost CSS from index.html', and the prev/next section claimed `next.ghost: true` drives 'the homepage's issue-next ghost CTA' — which conflated .article-nav-ghost with a component that no longer exists and was wrong before any of today's work. Also corrected a stale comment inside plates.css that justified a padding choice against '346px min-height' on a rule setting 230px — the same wrong number that had propagated into the doc. | 2026-09-11 re-verified live: permitted-accent list re-read; diff of css/ and brand/ from 2026-08-13 to HEAD adds ZERO new var(--accent) rules (two removals only). No new doc-vs-implementation drift. | 2026-09-24 re-verified live: no css/ or DESIGN-SYSTEM.md change on main since the last PASS; the Permitted list still resolves to live accent rules (section-head h2 and rule, callout border, stat bar, plate hover border, focus ring). DESIGN-SYSTEM.md:148 edited today on the fix branch for F108 (names the third hover control and the sheet the override actually lives in, home-augment.css, per F87) — parity improved, not broken.</t>
+          <t>PASS (resolved 2026-08-10) — was ISSUE/Low: DESIGN-SYSTEM.md:115 listed "Reading progress bar (`var(--accent)`)" as a permitted accent use, but css/article.css:876 ships `.reading-progress { background: var(--ink) }`. Commit 68b0c1d (2026-04-10) recolored it on purpose and left the reason in the CSS: red was competing with the masthead and diluting the accent's semantic weight. That commit rewrote 136 lines of DESIGN-SYSTEM.md but missed this one bullet, which dated to c75ded9 earlier the same day. The CSS was correct; the doc line was stale. | 2026-08-27 second doc-parity pass (9b8e4c4): three more drifts closed, all doc-side. The Ghost Teaser Plate code block was pre-F90 and pre-cutover (min-height 346 vs the shipped 230; .plate-title opacity .35 vs .46/.40; --ink+opacity on .teaser-date and .meta-rail vs --body-muted), its prose still carried the static-HTML instruction 'swap for the full article plate and remove the ghost CSS from index.html', and the prev/next section claimed `next.ghost: true` drives 'the homepage's issue-next ghost CTA' — which conflated .article-nav-ghost with a component that no longer exists and was wrong before any of today's work. Also corrected a stale comment inside plates.css that justified a padding choice against '346px min-height' on a rule setting 230px — the same wrong number that had propagated into the doc. | 2026-09-11 re-verified live: permitted-accent list re-read; diff of css/ and brand/ from 2026-08-13 to HEAD adds ZERO new var(--accent) rules (two removals only). No new doc-vs-implementation drift. | 2026-09-24 re-verified live: no css/ or DESIGN-SYSTEM.md change on main since the last PASS; the Permitted list still resolves to live accent rules (section-head h2 and rule, callout border, stat bar, plate hover border, focus ring). DESIGN-SYSTEM.md:148 edited today on the fix branch for F108 (names the third hover control and the sheet the override actually lives in, home-augment.css, per F87) — parity improved, not broken. | 2026-09-28: carried: DESIGN-SYSTEM.md touched only by the unmerged F108 commit; accent homes verified live (section-head h2 #ff4d4d dark, .callout border #c00).</t>
         </is>
       </c>
       <c r="I85" s="6" t="inlineStr">
@@ -4910,7 +4914,7 @@
       </c>
       <c r="H86" s="6" t="inlineStr">
         <is>
-          <t>PASS (closed live 2026-08-13) — was ISSUE/High (2026-08-13) — CORRECTED SCOPE, and the correction matters. The morning scrub read the declarations and reported FOUR failing hover rules. Re-measured under REAL pointer hover before fixing, only TWO are real: `.issue-latest:hover .latest-cta` (14.08px/700) and `.identity-hero .hero-link.primary:hover` (14.08px/700), both `color: var(--bg)` on a `background: var(--accent)` fill = 3.44:1 in dark against a 4.5:1 floor. The other two were FALSE POSITIVES: `.issue-latest:hover` takes the BAR to var(--ink), not var(--accent), so .latest-title measures 17.79:1 and .latest-meta 5.23:1 (at opacity .6) against cream — both already clear. The morning read assumed the accent fill was the surface for every child of the hover state; it is only the surface for .latest-cta, which sets its own background. Lesson: resolve the PAINTED surface under real hover, never infer it from the parent's declarations. | 2026-08-25 re-verified live: re-verified under REAL pointer hover on the live homepage in dark mode: .latest-cta 5.17:1, .latest-tag 5.17:1, .latest-title 17.79:1, .latest-meta (hover state) 5.23:1. No regression. Caveat carried to F87: the override lives in home-v2.css on the live deploy, so /brand/ still does not get it. | 2026-09-18 re-verified live: dark mode under REAL pointer hover: .latest-cta 'Read →' and .hero-link.primary 'Read the About →' both cream 243,240,232 on #c00 = 5.17:1 at 14.08px. | 2026-09-24 re-verified live: the two controls F83 fixed still pass under real pointer hover in dark mode: .latest-cta and .identity-hero .hero-link.primary both cream on #c00 at 5.17:1. BUT F83's scope note ('only the two controls below actually invert onto the accent fill on hover') was wrong: a.plate-lead:hover .rail-cta also inverts onto the accent and was missed — split out as F108, not counted as a regression of this row.</t>
+          <t>PASS (closed live 2026-08-13) — was ISSUE/High (2026-08-13) — CORRECTED SCOPE, and the correction matters. The morning scrub read the declarations and reported FOUR failing hover rules. Re-measured under REAL pointer hover before fixing, only TWO are real: `.issue-latest:hover .latest-cta` (14.08px/700) and `.identity-hero .hero-link.primary:hover` (14.08px/700), both `color: var(--bg)` on a `background: var(--accent)` fill = 3.44:1 in dark against a 4.5:1 floor. The other two were FALSE POSITIVES: `.issue-latest:hover` takes the BAR to var(--ink), not var(--accent), so .latest-title measures 17.79:1 and .latest-meta 5.23:1 (at opacity .6) against cream — both already clear. The morning read assumed the accent fill was the surface for every child of the hover state; it is only the surface for .latest-cta, which sets its own background. Lesson: resolve the PAINTED surface under real hover, never infer it from the parent's declarations. | 2026-08-25 re-verified live: re-verified under REAL pointer hover on the live homepage in dark mode: .latest-cta 5.17:1, .latest-tag 5.17:1, .latest-title 17.79:1, .latest-meta (hover state) 5.23:1. No regression. Caveat carried to F87: the override lives in home-v2.css on the live deploy, so /brand/ still does not get it. | 2026-09-18 re-verified live: dark mode under REAL pointer hover: .latest-cta 'Read →' and .hero-link.primary 'Read the About →' both cream 243,240,232 on #c00 = 5.17:1 at 14.08px. | 2026-09-24 re-verified live: the two controls F83 fixed still pass under real pointer hover in dark mode: .latest-cta and .identity-hero .hero-link.primary both cream on #c00 at 5.17:1. BUT F83's scope note ('only the two controls below actually invert onto the accent fill on hover') was wrong: a.plate-lead:hover .rail-cta also inverts onto the accent and was missed — split out as F108, not counted as a regression of this row. | 2026-09-28: live: 0 contrast failures in both sweeps; .latest-cta / .hero-link.primary source unchanged. The third control (F108) is still live pending merge.</t>
         </is>
       </c>
       <c r="I86" s="6" t="inlineStr">
@@ -4967,7 +4971,7 @@
       </c>
       <c r="H87" s="6" t="inlineStr">
         <is>
-          <t>PASS (closed live 2026-08-13) — was ISSUE/Low (2026-08-13) — DESIGN-SYSTEM.md:124-130 lists 'Backgrounds' and 'Tags or metadata' as PROHIBITED accent uses, but .latest-tag is exactly that: a metadata tag with `background: var(--accent)`, shipped and prominent in the homepage standfirst bar. Companion to F82, which audited only the Permitted half of the same section and so could not have caught this. | 2026-09-11 re-verified live: prohibited-accent list re-read; same diff confirms no new background: var(--accent) rule since the .latest-tag annotation shipped. The sanctioned exception is still the only one. | 2026-09-24 re-verified live: every background: var(--accent) rule enumerated (19 across 5 sheets): the only tag/metadata fills are .latest-tag (the annotated sanctioned exception) and .lead-badge-label (paired with --on-accent / #f5f5f1); the rest are rules, bars, dots, the manifesto panel and hover inversions. No unannotated prohibited use.</t>
+          <t>PASS (closed live 2026-08-13) — was ISSUE/Low (2026-08-13) — DESIGN-SYSTEM.md:124-130 lists 'Backgrounds' and 'Tags or metadata' as PROHIBITED accent uses, but .latest-tag is exactly that: a metadata tag with `background: var(--accent)`, shipped and prominent in the homepage standfirst bar. Companion to F82, which audited only the Permitted half of the same section and so could not have caught this. | 2026-09-11 re-verified live: prohibited-accent list re-read; same diff confirms no new background: var(--accent) rule since the .latest-tag annotation shipped. The sanctioned exception is still the only one. | 2026-09-24 re-verified live: every background: var(--accent) rule enumerated (19 across 5 sheets): the only tag/metadata fills are .latest-tag (the annotated sanctioned exception) and .lead-badge-label (paired with --on-accent / #f5f5f1); the rest are rules, bars, dots, the manifesto panel and hover inversions. No unannotated prohibited use. | 2026-09-28: carried: no accent rule changes on origin/main since last PASS.</t>
         </is>
       </c>
       <c r="I87" s="6" t="inlineStr">
@@ -5024,7 +5028,7 @@
       </c>
       <c r="H88" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-08-15) — `.latest-meta` ('Faith · Jul 5 · 16 min', the metadata in the homepage standfirst bar) pairs `color: var(--body-muted)` with `opacity: .75`. --body-muted is ALREADY an alpha colour (rgba(243,240,232,.52) dark / rgba(5,5,5,.56) light), tuned to land just over AA on its own — 5.13:1 dark, 4.67:1 light. The extra multiplier composites a second time and drops the control to 3.36:1 dark / 2.93:1 light, under the 4.5:1 floor for 11.52px/400 text. FAILS IN BOTH MODES — the only finding this run that is not dark-mode-specific. Measured on the settled live page with a compositor that resolves the painted surface by walking every ancestor background (flat #0d0d0d here, no image layer to confound it), then confirmed visually in a full-page screenshot where this is plainly the faintest text on the homepage. Missed by every prior run for a precise reason: the 2026-08-13 scrub measured .latest-meta ONLY under pointer hover, where `.issue-latest:hover .latest-meta` re-declares `color: var(--bg); opacity: .6` against the cream hover bar and clears at 5.23:1. F83 recorded that number and closed the question. The RESTING state — which is what a reader actually sees — was never measured. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: `.latest-meta` 3.36:1 dark / 2.93:1 light on the homepage, and 3.36:1 again on /brand/. Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | .latest-meta re-measured live 2026-08-25: 3.36:1 dark (homepage + /brand/), 2.93:1 light — unchanged from 2026-08-15. Root cause of the non-closure is NOT the fix: it is that the fix never shipped. origin/main is still b64a39b; the F85 commit (55a6d72) sits on LOCAL main, 8 commits ahead of origin, unpushed for 9 days. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live: .latest-meta 5.13:1 dark / 4.67:1 light, opacity 1 (no stacked multiplier). Also 5.13 on /brand/ dark.</t>
+          <t>ISSUE/High (2026-08-15) — `.latest-meta` ('Faith · Jul 5 · 16 min', the metadata in the homepage standfirst bar) pairs `color: var(--body-muted)` with `opacity: .75`. --body-muted is ALREADY an alpha colour (rgba(243,240,232,.52) dark / rgba(5,5,5,.56) light), tuned to land just over AA on its own — 5.13:1 dark, 4.67:1 light. The extra multiplier composites a second time and drops the control to 3.36:1 dark / 2.93:1 light, under the 4.5:1 floor for 11.52px/400 text. FAILS IN BOTH MODES — the only finding this run that is not dark-mode-specific. Measured on the settled live page with a compositor that resolves the painted surface by walking every ancestor background (flat #0d0d0d here, no image layer to confound it), then confirmed visually in a full-page screenshot where this is plainly the faintest text on the homepage. Missed by every prior run for a precise reason: the 2026-08-13 scrub measured .latest-meta ONLY under pointer hover, where `.issue-latest:hover .latest-meta` re-declares `color: var(--bg); opacity: .6` against the cream hover bar and clears at 5.23:1. F83 recorded that number and closed the question. The RESTING state — which is what a reader actually sees — was never measured. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: `.latest-meta` 3.36:1 dark / 2.93:1 light on the homepage, and 3.36:1 again on /brand/. Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | .latest-meta re-measured live 2026-08-25: 3.36:1 dark (homepage + /brand/), 2.93:1 light — unchanged from 2026-08-15. Root cause of the non-closure is NOT the fix: it is that the fix never shipped. origin/main is still b64a39b; the F85 commit (55a6d72) sits on LOCAL main, 8 commits ahead of origin, unpushed for 9 days. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live: .latest-meta 5.13:1 dark / 4.67:1 light, opacity 1 (no stacked multiplier). Also 5.13 on /brand/ dark. | 2026-09-28: live: covered by today's sweeps, 0 failures both modes.</t>
         </is>
       </c>
       <c r="I88" s="6" t="inlineStr">
@@ -5081,7 +5085,7 @@
       </c>
       <c r="H89" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-08-15) — `.hero-corner` sets `color: var(--bg); opacity: .5`. The identity hero is an INVERTED plate: in dark mode it presents a cream ground (243,240,232) and the label paints #060606 over it, which at .5 opacity computes 3.71:1 — under the 4.5:1 floor for 11.52px/700 (bold, but well below the 18.66px large-text threshold). Light mode inverts to cream-on-black and clears at 4.91:1, so this is dark-mode-only. Same root shape as F85 — a decorative opacity multiplier stacked on a colour that was already correct — but reached by the opposite route: here the multiplier sits on a SOLID token rather than an alpha one. Surface resolved by walking to the first opaque ancestor (.hero-main, flat cream, no image layer); confirmed visually in a dark-mode full-page screenshot. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: `.hero-corner` 3.71:1 dark on the homepage, and 3.71:1 again on /brand/. Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | .hero-corner re-measured live 2026-08-25: 3.71:1 dark. Unchanged — fix committed locally (55a6d72), never pushed. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live: .identity-hero .hero-corner 5.23:1 dark / 6.74:1 light at opacity .6.</t>
+          <t>ISSUE/High (2026-08-15) — `.hero-corner` sets `color: var(--bg); opacity: .5`. The identity hero is an INVERTED plate: in dark mode it presents a cream ground (243,240,232) and the label paints #060606 over it, which at .5 opacity computes 3.71:1 — under the 4.5:1 floor for 11.52px/700 (bold, but well below the 18.66px large-text threshold). Light mode inverts to cream-on-black and clears at 4.91:1, so this is dark-mode-only. Same root shape as F85 — a decorative opacity multiplier stacked on a colour that was already correct — but reached by the opposite route: here the multiplier sits on a SOLID token rather than an alpha one. Surface resolved by walking to the first opaque ancestor (.hero-main, flat cream, no image layer); confirmed visually in a dark-mode full-page screenshot. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: `.hero-corner` 3.71:1 dark on the homepage, and 3.71:1 again on /brand/. Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | .hero-corner re-measured live 2026-08-25: 3.71:1 dark. Unchanged — fix committed locally (55a6d72), never pushed. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live: .identity-hero .hero-corner 5.23:1 dark / 6.74:1 light at opacity .6. | 2026-09-28: live: covered by today's sweeps, 0 failures both modes.</t>
         </is>
       </c>
       <c r="I89" s="6" t="inlineStr">
@@ -5138,7 +5142,7 @@
       </c>
       <c r="H90" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-08-15) — /brand/ was still rendering `.latest-tag` at 3.44:1, the exact pre-fix value F77 closed on 2026-08-13, two days after that row went green. Cause: the F77 and F83 dark-mode overrides were written into css/home-v2.css. The homepage loads home-augment.css AND home-v2.css; /brand/ loads home-augment.css and never home-v2.css. So the fixes reached the homepage and silently skipped the design system's own documentation page. This is a broken contract, not a cosmetic gap: brand/index.html:115 states a 'Dogfood rule' — '/brand/ runs the same stylesheets as the live site... If a live component breaks, this page breaks too. That is intentional.' A fix that lands on one surface and not the other makes the dogfood page a liar in the safer direction, which is worse than an obvious break. The F77 comment even asserted it 'Covers the .issue-head hook in home-augment.css too; wins on specificity, not source order' — true about specificity, but specificity is irrelevant in a sheet that never loads. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: /brand/ `.latest-tag` 3.44:1 — and /brand/'s loaded-sheet list confirms the cause directly: tokens, shell, plates, home-augment, article, brand.css, with NO home-v2.css. Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | /brand/ re-measured live 2026-08-25: .latest-tag still 3.44:1 (the pre-F77 value), because live /brand/ serves home-augment.css?v=phase32 which does not yet carry the moved override blocks. The move (55a6d72) is committed locally and confirmed present in a fresh dist build; it has never been pushed. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live: /brand/ loads home-augment.css?v=phase34 (not home-v2); .latest-tag 5.17:1 dark / 5.34:1 light, identical to the homepage — dogfood contract holds.</t>
+          <t>ISSUE/High (2026-08-15) — /brand/ was still rendering `.latest-tag` at 3.44:1, the exact pre-fix value F77 closed on 2026-08-13, two days after that row went green. Cause: the F77 and F83 dark-mode overrides were written into css/home-v2.css. The homepage loads home-augment.css AND home-v2.css; /brand/ loads home-augment.css and never home-v2.css. So the fixes reached the homepage and silently skipped the design system's own documentation page. This is a broken contract, not a cosmetic gap: brand/index.html:115 states a 'Dogfood rule' — '/brand/ runs the same stylesheets as the live site... If a live component breaks, this page breaks too. That is intentional.' A fix that lands on one surface and not the other makes the dogfood page a liar in the safer direction, which is worse than an obvious break. The F77 comment even asserted it 'Covers the .issue-head hook in home-augment.css too; wins on specificity, not source order' — true about specificity, but specificity is irrelevant in a sheet that never loads. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: /brand/ `.latest-tag` 3.44:1 — and /brand/'s loaded-sheet list confirms the cause directly: tokens, shell, plates, home-augment, article, brand.css, with NO home-v2.css. Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | /brand/ re-measured live 2026-08-25: .latest-tag still 3.44:1 (the pre-F77 value), because live /brand/ serves home-augment.css?v=phase32 which does not yet carry the moved override blocks. The move (55a6d72) is committed locally and confirmed present in a fresh dist build; it has never been pushed. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live: /brand/ loads home-augment.css?v=phase34 (not home-v2); .latest-tag 5.17:1 dark / 5.34:1 light, identical to the homepage — dogfood contract holds. | 2026-09-28: carried: /brand/ loads home-augment.css; sweep 0 failures.</t>
         </is>
       </c>
       <c r="I90" s="6" t="inlineStr">
@@ -5248,7 +5252,7 @@
       </c>
       <c r="H92" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-08-15) — the `·` separators in the 404 eyebrow carry `opacity: .5`, computing 3.61:1. Unlike the homepage's `.dot` separators — which are `aria-hidden="true"` and therefore exempt as decoration — these carry no aria-hidden, so they are exposed text in both the accessibility tree and the visual read. Caught by explicitly checking aria-hidden per separator rather than assuming all separators are decorative: the homepage `.dot` at 4.25:1 was correctly DISMISSED as a non-finding by that same check, and this one was correctly kept. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: `.notfound-eyebrow span.divider` 3.61:1 on /404. Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | /404 span.divider re-measured live 2026-08-25: still 3.61:1 at opacity .5; live serves notfound.css?v=phase10 (the fix bumps it to phase11). Fix committed locally (8c1e6aa), never pushed. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live: /404 .notfound-eyebrow span.divider 7.19:1 dark / 8.95:1 light; still not aria-hidden (exposed text, in scope).</t>
+          <t>ISSUE/Medium (2026-08-15) — the `·` separators in the 404 eyebrow carry `opacity: .5`, computing 3.61:1. Unlike the homepage's `.dot` separators — which are `aria-hidden="true"` and therefore exempt as decoration — these carry no aria-hidden, so they are exposed text in both the accessibility tree and the visual read. Caught by explicitly checking aria-hidden per separator rather than assuming all separators are decorative: the homepage `.dot` at 4.25:1 was correctly DISMISSED as a non-finding by that same check, and this one was correctly kept. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: `.notfound-eyebrow span.divider` 3.61:1 on /404. Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | /404 span.divider re-measured live 2026-08-25: still 3.61:1 at opacity .5; live serves notfound.css?v=phase10 (the fix bumps it to phase11). Fix committed locally (8c1e6aa), never pushed. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live: /404 .notfound-eyebrow span.divider 7.19:1 dark / 8.95:1 light; still not aria-hidden (exposed text, in scope). | 2026-09-28: live: 404 0 contrast failures.</t>
         </is>
       </c>
       <c r="I92" s="6" t="inlineStr">
@@ -5305,7 +5309,7 @@
       </c>
       <c r="H93" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Low (2026-08-15) — five /brand/-only text elements measure under AA in dark mode: `.demo-ghost-meta` ('Coming Soon') 2.05:1, `.demo-ghost-date` 2.45:1, `.demo-ghost-title` 2.93:1 (against its 3:1 large-text floor), `.demo-plate-meta` 3.17:1, and the bespoke 'Download Pack' h3 at 2.87:1. Held BLOCKED rather than fixed: four of the five are `demo-ghost-*` specimens whose entire purpose is to DEMONSTRATE the dim 'not yet published' ghost treatment, so raising their contrast would edit the documentation's illustration rather than repair a defect — that is a call about what the design system wants to say, and it is Dexter's. The fifth ('Download Pack') is bespoke brand.css chrome and is a genuine, if low-traffic, AA miss. Deliberately NOT bundled with F87: that row was a broken contract with an objectively correct fix; this one is a judgement about intent. | 2026-08-16 LIVE RE-CHECK: still open and still BLOCKED — unchanged by design. Re-measured on live /brand/: `.demo-ghost-meta` 2.05:1 and `.demo-plate-meta` 3.17:1 both reproduce exactly. The other three named elements (demo-ghost-date, demo-ghost-title, the 'Download Pack' h3) did not surface in today's sweep because this run only measures elements holding their own text node and not inside an aria-hidden subtree; that is a narrower filter than the 2026-08-15 pass used, not evidence they were fixed. Still NEEDS DEXTER on both questions. | Re-confirmed live 2026-08-25, all five values unchanged: .demo-ghost-meta 2.05:1, .demo-ghost-date 2.45:1, .demo-ghost-title 2.93:1 (vs its 3:1 large-text floor), .demo-plate-meta 3.17:1, and the bespoke "Download Pack" h3 2.87:1 (#ff4d4d on the cream panel). Still BLOCKED — still the same two questions for Dexter, now open 10 days. | 2026-08-27 RE-DIAGNOSED, and the premise of this row was wrong. Four of the five are not documentation-intent choices at all — `.demo-ghost-title/-date/-meta` and `.demo-plate-meta` are faithful mirrors of `.plate-ghost` and `.identity-plate` in css/plates.css, carrying the same tokens and the same opacity multipliers. Composited against their real grounds those production rules measure .plate-title 2.92:1 light / 2.84:1 dark (3:1 large-text floor), .teaser-date 2.06/2.37, `.plate-ghost .meta-rail` 1.80/1.97, and `.identity-plate .meta-rail` 4.14/4.09 (4.5:1 floor) — every one under AA. css/plates.css:377-380 carried a comment asserting these values PASSED ("3.1:1 on #f4f4f1", "3.7:1 on #060606"); both figures are wrong and are what kept the defect invisible. The fifth, the /brand/ 'Download Pack' h3, is worse than recorded: it fails in BOTH modes (2.87:1 dark, 3.46:1 light), not just dark. Separately found: the /brand/ identity specimen had drifted — it used var(--ink)/var(--bg), which invert, so in dark mode it rendered a CREAM identity plate while production deliberately holds #0a0a0a. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live: /brand/ demo specimens clear their floors in both modes — .demo-ghost-meta 5.13/4.67, .demo-ghost-date 5.13/4.67, .demo-ghost-title 3.48/3.33 (44.8px, 3:1 floor), .demo-plate-meta 18.11; full-page sweep 793 elements per mode, 0 failures; img-plate bodies flex/flex-end.</t>
+          <t>ISSUE/Low (2026-08-15) — five /brand/-only text elements measure under AA in dark mode: `.demo-ghost-meta` ('Coming Soon') 2.05:1, `.demo-ghost-date` 2.45:1, `.demo-ghost-title` 2.93:1 (against its 3:1 large-text floor), `.demo-plate-meta` 3.17:1, and the bespoke 'Download Pack' h3 at 2.87:1. Held BLOCKED rather than fixed: four of the five are `demo-ghost-*` specimens whose entire purpose is to DEMONSTRATE the dim 'not yet published' ghost treatment, so raising their contrast would edit the documentation's illustration rather than repair a defect — that is a call about what the design system wants to say, and it is Dexter's. The fifth ('Download Pack') is bespoke brand.css chrome and is a genuine, if low-traffic, AA miss. Deliberately NOT bundled with F87: that row was a broken contract with an objectively correct fix; this one is a judgement about intent. | 2026-08-16 LIVE RE-CHECK: still open and still BLOCKED — unchanged by design. Re-measured on live /brand/: `.demo-ghost-meta` 2.05:1 and `.demo-plate-meta` 3.17:1 both reproduce exactly. The other three named elements (demo-ghost-date, demo-ghost-title, the 'Download Pack' h3) did not surface in today's sweep because this run only measures elements holding their own text node and not inside an aria-hidden subtree; that is a narrower filter than the 2026-08-15 pass used, not evidence they were fixed. Still NEEDS DEXTER on both questions. | Re-confirmed live 2026-08-25, all five values unchanged: .demo-ghost-meta 2.05:1, .demo-ghost-date 2.45:1, .demo-ghost-title 2.93:1 (vs its 3:1 large-text floor), .demo-plate-meta 3.17:1, and the bespoke "Download Pack" h3 2.87:1 (#ff4d4d on the cream panel). Still BLOCKED — still the same two questions for Dexter, now open 10 days. | 2026-08-27 RE-DIAGNOSED, and the premise of this row was wrong. Four of the five are not documentation-intent choices at all — `.demo-ghost-title/-date/-meta` and `.demo-plate-meta` are faithful mirrors of `.plate-ghost` and `.identity-plate` in css/plates.css, carrying the same tokens and the same opacity multipliers. Composited against their real grounds those production rules measure .plate-title 2.92:1 light / 2.84:1 dark (3:1 large-text floor), .teaser-date 2.06/2.37, `.plate-ghost .meta-rail` 1.80/1.97, and `.identity-plate .meta-rail` 4.14/4.09 (4.5:1 floor) — every one under AA. css/plates.css:377-380 carried a comment asserting these values PASSED ("3.1:1 on #f4f4f1", "3.7:1 on #060606"); both figures are wrong and are what kept the defect invisible. The fifth, the /brand/ 'Download Pack' h3, is worse than recorded: it fails in BOTH modes (2.87:1 dark, 3.46:1 light), not just dark. Separately found: the /brand/ identity specimen had drifted — it used var(--ink)/var(--bg), which invert, so in dark mode it rendered a CREAM identity plate while production deliberately holds #0a0a0a. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live: /brand/ demo specimens clear their floors in both modes — .demo-ghost-meta 5.13/4.67, .demo-ghost-date 5.13/4.67, .demo-ghost-title 3.48/3.33 (44.8px, 3:1 floor), .demo-plate-meta 18.11; full-page sweep 793 elements per mode, 0 failures; img-plate bodies flex/flex-end. | 2026-09-28: live: /brand/ 776 elements, 0 failures both modes.</t>
         </is>
       </c>
       <c r="I93" s="6" t="inlineStr">
@@ -5362,7 +5366,7 @@
       </c>
       <c r="H94" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-08-16) — /phase0/'s skip link, the first focusable element on the page, computed `color: rgba(243,240,232,.82)` on its own `background: var(--ink)` cream chip: 1.00:1. This is the worst ratio the ledger has recorded and the only finding to date where the text is not merely low-contrast but literally invisible — a sighted keyboard user sees the accent focus ring land on a blank cream box. NOT a colour bug: `--bg` resolves correctly to #060606 at every level of the chain (verified by walking the ancestor chain: A.skip-link / BODY.phase0 / HTML.dark-mode all report #060606). It is a specificity bug. Three rules set colour on this element — `a {color:inherit}` (0,0,1) in tokens.css, `.skip-link {color:var(--bg)}` (0,1,0) in shell.css, and `.phase0 a {color:inherit}` (0,1,1) in phase0.css. The last wins on specificity and hands the chip back the inherited body cream. Scope is exactly one page: /brand/, the other bespoke-CSS surface, carries no blanket `a` rule and measured clean. Missed by every prior run because the skip link sits at left:-999px in its resting state, so a sweep that filters to on-screen elements never measures it — this run caught it by measuring every element with layout geometry regardless of viewport position. | /phase0/ skip link re-measured live 2026-08-25: still rgba(243,240,232,.82) on its own cream chip = 1.00:1, the worst ratio in the ledger and still literally invisible to a sighted keyboard user. Live serves shell.css?v=phase23; the hardened selector ships as phase36. Fix committed locally (79df261), never pushed. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live under a real shift+Tab: /phase0/ skip link is first focusable, rgb(6,6,6) on rgb(243,240,232) = 17.79:1 dark; light rgb(244,244,241) on rgb(5,5,5); 2px #c00 ring. Homepage skip link same, activation lands focus on MAIN#archive.</t>
+          <t>ISSUE/High (2026-08-16) — /phase0/'s skip link, the first focusable element on the page, computed `color: rgba(243,240,232,.82)` on its own `background: var(--ink)` cream chip: 1.00:1. This is the worst ratio the ledger has recorded and the only finding to date where the text is not merely low-contrast but literally invisible — a sighted keyboard user sees the accent focus ring land on a blank cream box. NOT a colour bug: `--bg` resolves correctly to #060606 at every level of the chain (verified by walking the ancestor chain: A.skip-link / BODY.phase0 / HTML.dark-mode all report #060606). It is a specificity bug. Three rules set colour on this element — `a {color:inherit}` (0,0,1) in tokens.css, `.skip-link {color:var(--bg)}` (0,1,0) in shell.css, and `.phase0 a {color:inherit}` (0,1,1) in phase0.css. The last wins on specificity and hands the chip back the inherited body cream. Scope is exactly one page: /brand/, the other bespoke-CSS surface, carries no blanket `a` rule and measured clean. Missed by every prior run because the skip link sits at left:-999px in its resting state, so a sweep that filters to on-screen elements never measures it — this run caught it by measuring every element with layout geometry regardless of viewport position. | /phase0/ skip link re-measured live 2026-08-25: still rgba(243,240,232,.82) on its own cream chip = 1.00:1, the worst ratio in the ledger and still literally invisible to a sighted keyboard user. Live serves shell.css?v=phase23; the hardened selector ships as phase36. Fix committed locally (79df261), never pushed. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live under a real shift+Tab: /phase0/ skip link is first focusable, rgb(6,6,6) on rgb(243,240,232) = 17.79:1 dark; light rgb(244,244,241) on rgb(5,5,5); 2px #c00 ring. Homepage skip link same, activation lands focus on MAIN#archive. | 2026-09-28: carried: skip-link rule unchanged; home skip link verified under real Tab.</t>
         </is>
       </c>
       <c r="I94" s="6" t="inlineStr">
@@ -5419,7 +5423,7 @@
       </c>
       <c r="H95" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Low (2026-08-27) — the click handler rewrote the label and the count but never touched the glyph. Live on b64a39b the expanded state reads 'Show Less — showing all ↓': the arrow still points down, i.e. 'more below', while the button's own words say it will collapse. The glyph carries aria-hidden="true" so nothing is exposed to assistive tech — this is a purely visual affordance contradiction, which is why it survived every prior scrub. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-01 re-verified live: .btn-glyph tracks the button state — down-arrow collapsed, up-arrow expanded, and back. | 2026-09-11 re-verified live: glyph tracks state live — ↓ at 7 shown, ↑ at 17 shown, back to ↓; still aria-hidden. | 2026-09-19 re-verified live: View Earlier toggle: 7 shown / aria-expanded false / ↓ → 17 shown / true / ↑ → back to 7 / false. | 2026-09-25: re-verified live: 7 shown / aria-expanded false / ↓ → 17 shown / true / ↑ → back to 7 / false; glyph aria-hidden.</t>
+          <t>ISSUE/Low (2026-08-27) — the click handler rewrote the label and the count but never touched the glyph. Live on b64a39b the expanded state reads 'Show Less — showing all ↓': the arrow still points down, i.e. 'more below', while the button's own words say it will collapse. The glyph carries aria-hidden="true" so nothing is exposed to assistive tech — this is a purely visual affordance contradiction, which is why it survived every prior scrub. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-01 re-verified live: .btn-glyph tracks the button state — down-arrow collapsed, up-arrow expanded, and back. | 2026-09-11 re-verified live: glyph tracks state live — ↓ at 7 shown, ↑ at 17 shown, back to ↓; still aria-hidden. | 2026-09-19 re-verified live: View Earlier toggle: 7 shown / aria-expanded false / ↓ → 17 shown / true / ↑ → back to 7 / false. | 2026-09-25: re-verified live: 7 shown / aria-expanded false / ↓ → 17 shown / true / ↑ → back to 7 / false; glyph aria-hidden. | 2026-09-28: live: glyph ↓ collapsed / ↑ expanded tracks the label.</t>
         </is>
       </c>
       <c r="I95" s="6" t="inlineStr">
@@ -5476,7 +5480,7 @@
       </c>
       <c r="H96" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-08-27) — both class names are DEAD in production. `Plate.astro` can only ever emit `plate plate-{wide|secondary|banner|half|lead}` plus `plate-image`, `img-*` and `plate-row`; there is no code path to `plate-ghost` or `identity-plate`, the strings appear nowhere in src/, and they appear in none of the 19 built pages. This is almost certainly fallout from the 2026-04-21 Astro cutover — the ghost teaser is clearly still intended (ComingSoonLayout exists, visibility.ts date-gates future essays, and F30/F41 both describe an upcoming-essay flow), it just never got rewired to the new cascade. Two consequences: css/plates.css ships ~90 lines of unreachable rules on every homepage load, and /brand/ documents both as live components when neither can render. Found while re-diagnosing F90 — the F90 contrast failures are in these same dead rules, which is why they only ever surfaced on /brand/. | Dexter chose REWIRE over retire, 2026-08-27. | RESOLVED 2026-08-27 — see p4. | CORRECTION 2026-08-27: this row was closed as 'fixed' while it named TWO orphaned components and only ONE was rewired. `.plate-ghost` has an emitter now; `.identity-plate` still has none — no occurrence anywhere in src/, zero in the 19 built pages. F93 is hereby narrowed to the ghost plate, which is genuinely fixed, and the identity-plate half is split out to F95 so it is not buried under a green row. My closure, my error. | 2026-09-25: static re-check: GhostPlate.astro still emits .plate-ghost; plates.css?v=phase39 carries the rules. Live render still untestable (0 upcoming entries), so no live claim.</t>
+          <t>ISSUE/Medium (2026-08-27) — both class names are DEAD in production. `Plate.astro` can only ever emit `plate plate-{wide|secondary|banner|half|lead}` plus `plate-image`, `img-*` and `plate-row`; there is no code path to `plate-ghost` or `identity-plate`, the strings appear nowhere in src/, and they appear in none of the 19 built pages. This is almost certainly fallout from the 2026-04-21 Astro cutover — the ghost teaser is clearly still intended (ComingSoonLayout exists, visibility.ts date-gates future essays, and F30/F41 both describe an upcoming-essay flow), it just never got rewired to the new cascade. Two consequences: css/plates.css ships ~90 lines of unreachable rules on every homepage load, and /brand/ documents both as live components when neither can render. Found while re-diagnosing F90 — the F90 contrast failures are in these same dead rules, which is why they only ever surfaced on /brand/. | Dexter chose REWIRE over retire, 2026-08-27. | RESOLVED 2026-08-27 — see p4. | CORRECTION 2026-08-27: this row was closed as 'fixed' while it named TWO orphaned components and only ONE was rewired. `.plate-ghost` has an emitter now; `.identity-plate` still has none — no occurrence anywhere in src/, zero in the 19 built pages. F93 is hereby narrowed to the ghost plate, which is genuinely fixed, and the identity-plate half is split out to F95 so it is not buried under a green row. My closure, my error. | 2026-09-25: static re-check: GhostPlate.astro still emits .plate-ghost; plates.css?v=phase39 carries the rules. Live render still untestable (0 upcoming entries), so no live claim. | 2026-09-28: build-verified via fixture: .plate-ghost renders with .plate-title == fixture title and .teaser-date &lt;time 2027-01-15&gt; == publishedDate.</t>
         </is>
       </c>
       <c r="I96" s="6" t="inlineStr">
@@ -5533,7 +5537,7 @@
       </c>
       <c r="H97" s="6" t="inlineStr">
         <is>
-          <t>N/A by decision (2026-08-27) — not a defect. Dexter's call after seeing F93 ship: the ghost plate and the IssueNext strip are two presentations of the same upcoming essay, so with both live the title appeared on the homepage twice. The plate wins. | 2026-09-25: still N/A by decision. Note: the expected column's "component and CSS stay intact" was overtaken the same day by e3b4e91, which deleted IssueNext.astro and its CSS; reversal now means restoring from git (121a621), not a one-line flip. Live: 0 .issue-next in DOM/CSS.</t>
+          <t>N/A by decision (2026-08-27) — not a defect. Dexter's call after seeing F93 ship: the ghost plate and the IssueNext strip are two presentations of the same upcoming essay, so with both live the title appeared on the homepage twice. The plate wins. | 2026-09-25: still N/A by decision. Note: the expected column's "component and CSS stay intact" was overtaken the same day by e3b4e91, which deleted IssueNext.astro and its CSS; reversal now means restoring from git (121a621), not a one-line flip. Live: 0 .issue-next in DOM/CSS. | 2026-09-28: build-verified via fixture: ghost plate rendered, .issue-next count 0.</t>
         </is>
       </c>
       <c r="I97" s="6" t="inlineStr"/>
@@ -5586,7 +5590,7 @@
       </c>
       <c r="H98" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-08-27) — SPLIT FROM F93, WHICH I CLOSED TOO BROADLY. F93 named two orphaned components; Dexter asked for the ghost plate to be rewired and it was, but `.identity-plate` was never in scope and is still dead. Re-verified today: the string appears nowhere in src/ and in none of the 19 built pages, because Plate.astro can only emit plate-{wide|secondary|banner|half|lead} plus plate-image/img-*/plate-row. css/plates.css ships ~85 lines of unreachable rules on every homepage load, and /brand/ documents the plate as live. Note this is NOT the same thing as `.identity-hero`, which does render on the homepage and is fine (F21). Contrast is not at issue — F90 already lifted `.identity-plate .meta-rail` to 5.77/5.63 — this is purely reachability. | RESOLVED 2026-08-28 — Dexter chose retire. See p4. | 2026-09-26 re-verified: css/plates.css carries zero live .identity-plate rules (only the retirement comment at :270) and brand/index.html documents no .identity-plate specimen; the homepage's identity surface is IdentityHero via src/pages/index.astro — retirement holds.</t>
+          <t>ISSUE/Medium (2026-08-27) — SPLIT FROM F93, WHICH I CLOSED TOO BROADLY. F93 named two orphaned components; Dexter asked for the ghost plate to be rewired and it was, but `.identity-plate` was never in scope and is still dead. Re-verified today: the string appears nowhere in src/ and in none of the 19 built pages, because Plate.astro can only emit plate-{wide|secondary|banner|half|lead} plus plate-image/img-*/plate-row. css/plates.css ships ~85 lines of unreachable rules on every homepage load, and /brand/ documents the plate as live. Note this is NOT the same thing as `.identity-hero`, which does render on the homepage and is fine (F21). Contrast is not at issue — F90 already lifted `.identity-plate .meta-rail` to 5.77/5.63 — this is purely reachability. | RESOLVED 2026-08-28 — Dexter chose retire. See p4. | 2026-09-26 re-verified: css/plates.css carries zero live .identity-plate rules (only the retirement comment at :270) and brand/index.html documents no .identity-plate specimen; the homepage's identity surface is IdentityHero via src/pages/index.astro — retirement holds. | 2026-09-28: carried: source unchanged.</t>
         </is>
       </c>
       <c r="I98" s="6" t="inlineStr">
@@ -5643,7 +5647,7 @@
       </c>
       <c r="H99" s="6" t="inlineStr">
         <is>
-          <t>PASS (2026-08-31, live on 13b631c then 83c2137) — POST-gate half verified live end to end: article 200 with 55 paragraphs and zero coming-soon markers; present in sitemap-0.xml, feed.xml and the homepage cascade (latest strip, lead plate, 'Week of August 31, 2026'); 'Send Someone Else' renders 0 .article-nav-ghost, i.e. the ghost treatment retired itself on go-live exactly as designed. OG plate 1200x630 (1.905), reads VOL 17 matching the essay's own number, title clears Anton's caps on the .92 leading from 9301d61. Metadata complete (description, og:title/image/image:alt/type, twitter:summary_large_image, canonical). Redate to Aug 31 propagated to every surface: JSON-LD datePublished 2026-08-31T12:00:00-05:00, Atom &lt;published&gt; 2026-08-31T17:00:00Z, homepage &lt;time datetime="2026-08-31"&gt;, zero 'Aug 30' anywhere live. Contrast 87 elements / 0 failures in BOTH modes (dark floor 5.13:1, light 4.67:1). Single h1, h1-&gt;h2 with no skipped level, skip link takes first Tab with a visible ring, 0 unnamed interactive elements, 0 console errors. || PRE-gate half NOT verified in production — see F93/F94: the release sat unpushed from Aug 29 until after the Aug 30 noon gate, so the Coming-Soon route never rendered on the live site for this essay. | 2026-09-01 re-verified live: VOL 17 present and correct across article (200), homepage lead plate, feed (17/17), sitemap and OG plate; article:published_time 2026-08-31 matches the homepage plate's &lt;time datetime&gt;. | 2026-09-26 re-verified live: /words/the-weight-of-my-no/ renders the full ArticleLayout (no 'Coming Soon', no noindex), sits in feed.xml (17 entries), sitemap-0.xml (21 locs) and the homepage cascade; 'Send Someone Else' carries a real rel=next .article-nav-next link to it, no ghost.</t>
+          <t>PASS (2026-08-31, live on 13b631c then 83c2137) — POST-gate half verified live end to end: article 200 with 55 paragraphs and zero coming-soon markers; present in sitemap-0.xml, feed.xml and the homepage cascade (latest strip, lead plate, 'Week of August 31, 2026'); 'Send Someone Else' renders 0 .article-nav-ghost, i.e. the ghost treatment retired itself on go-live exactly as designed. OG plate 1200x630 (1.905), reads VOL 17 matching the essay's own number, title clears Anton's caps on the .92 leading from 9301d61. Metadata complete (description, og:title/image/image:alt/type, twitter:summary_large_image, canonical). Redate to Aug 31 propagated to every surface: JSON-LD datePublished 2026-08-31T12:00:00-05:00, Atom &lt;published&gt; 2026-08-31T17:00:00Z, homepage &lt;time datetime="2026-08-31"&gt;, zero 'Aug 30' anywhere live. Contrast 87 elements / 0 failures in BOTH modes (dark floor 5.13:1, light 4.67:1). Single h1, h1-&gt;h2 with no skipped level, skip link takes first Tab with a visible ring, 0 unnamed interactive elements, 0 console errors. || PRE-gate half NOT verified in production — see F93/F94: the release sat unpushed from Aug 29 until after the Aug 30 noon gate, so the Coming-Soon route never rendered on the live site for this essay. | 2026-09-01 re-verified live: VOL 17 present and correct across article (200), homepage lead plate, feed (17/17), sitemap and OG plate; article:published_time 2026-08-31 matches the homepage plate's &lt;time datetime&gt;. | 2026-09-26 re-verified live: /words/the-weight-of-my-no/ renders the full ArticleLayout (no 'Coming Soon', no noindex), sits in feed.xml (17 entries), sitemap-0.xml (21 locs) and the homepage cascade; 'Send Someone Else' carries a real rel=next .article-nav-next link to it, no ghost. | 2026-09-28: live: the-weight-of-my-no in cascade (lead), feed and sitemap.</t>
         </is>
       </c>
       <c r="I99" s="6" t="inlineStr"/>
@@ -5688,7 +5692,7 @@
       </c>
       <c r="H100" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-08-31) — .article-eyebrow shipped flex-wrap: nowrap with no mobile override, so the rail runs off the frame on every article. Measured LIVE at 375px on /words/the-weight-of-my-no/ (6 chips: 2 lanes + 2 tags + date + read-time): scrollWidth 406 vs clientWidth 362 = 105px overflow; .article-read sits at left:418 against a 375px viewport, i.e. '8 min' is 100% invisible and 'Aug 31, 2026' is 92% clipped. Control /words/send-someone-else/ (5 chips) overflows 39px and loses 2px of '16 min', confirming this is site-wide and pre-existing rather than introduced by VOL 17 — VOL 17 is simply the worst case, being the first 6-chip essay. Because body/.page-shell are overflow-x: clip there is no scrollbar and no gesture that reaches the clipped text. Survived every prior scrub because source-only inspection cannot see it: the CSS is valid, the defect only exists once the flex row is laid out under 760px. | 2026-09-06 re-verified live: holds live - eyebrow wraps at 375px with zero overflow. | 2026-09-11 re-verified live: 375px /words/the-weight-of-my-no/: .article-eyebrow computes flex-wrap: wrap, all six chips inside the frame (rightmost 331px), documentElement.scrollWidth == clientWidth == 375. | 2026-09-19 re-verified live: 375px /words/the-weight-of-my-no/: .article-eyebrow flex-wrap: wrap, rightmost chip at 331px, scrollWidth == clientWidth == 375. | 2026-09-26 re-verified live at 375x812: .article-eyebrow is flex-wrap: wrap and 0 children overflow the viewport on /about/ and all 17 articles; no document-level horizontal overflow on any of the 18.</t>
+          <t>ISSUE/High (2026-08-31) — .article-eyebrow shipped flex-wrap: nowrap with no mobile override, so the rail runs off the frame on every article. Measured LIVE at 375px on /words/the-weight-of-my-no/ (6 chips: 2 lanes + 2 tags + date + read-time): scrollWidth 406 vs clientWidth 362 = 105px overflow; .article-read sits at left:418 against a 375px viewport, i.e. '8 min' is 100% invisible and 'Aug 31, 2026' is 92% clipped. Control /words/send-someone-else/ (5 chips) overflows 39px and loses 2px of '16 min', confirming this is site-wide and pre-existing rather than introduced by VOL 17 — VOL 17 is simply the worst case, being the first 6-chip essay. Because body/.page-shell are overflow-x: clip there is no scrollbar and no gesture that reaches the clipped text. Survived every prior scrub because source-only inspection cannot see it: the CSS is valid, the defect only exists once the flex row is laid out under 760px. | 2026-09-06 re-verified live: holds live - eyebrow wraps at 375px with zero overflow. | 2026-09-11 re-verified live: 375px /words/the-weight-of-my-no/: .article-eyebrow computes flex-wrap: wrap, all six chips inside the frame (rightmost 331px), documentElement.scrollWidth == clientWidth == 375. | 2026-09-19 re-verified live: 375px /words/the-weight-of-my-no/: .article-eyebrow flex-wrap: wrap, rightmost chip at 331px, scrollWidth == clientWidth == 375. | 2026-09-26 re-verified live at 375x812: .article-eyebrow is flex-wrap: wrap and 0 children overflow the viewport on /about/ and all 17 articles; no document-level horizontal overflow on any of the 18. | 2026-09-28: live at 390px: .article-eyebrow wraps inside the frame (right edge 353px of 390), 0 overflow.</t>
         </is>
       </c>
       <c r="I100" s="6" t="inlineStr">
@@ -5745,7 +5749,7 @@
       </c>
       <c r="H101" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-09-02) — `.skip-link` had NO :focus-visible rule anywhere in the loaded cascade. Enumerated every rule matching /skip-link/ across all loaded sheets on live: exactly two hits, both in shell.css (the (0,2,0) :link/:visited base chip from F91, and .skip-link:focus for positioning) — neither carries an outline. Measured under a REAL Tab press on the live homepage with the chip focused: outline `rgb(153,200,255) auto 1px` — Chrome's UA default — while every sibling control measured the same way paints `rgb(204,0,0) solid 2px` (.brand-block, .mode-toggle, a.plate, .issue-standfirst, .hero-link, .sm-submit all confirmed this run). Confirmed identical on /about/ (shared shell.css, skipFocusRule:false). NOT a WCAG 2.4.7 failure — the UA ring is visible, which is exactly why five months of contrast-led sweeps never surfaced it — but a design-token break on the first element a keyboard user ever focuses. Same defect class as F76 (.sm-submit, closed 2026-08-10); this is a distinct element that rule never covered, not a regression of it. | 2026-09-06 re-verified live: still open ON LIVE, as expected - the fix is on this branch and unmerged. Live skip link focuses with the Chrome default ring (outline rgb(153,200,255) auto 1px) instead of the site's red --focus-ring. Closes on merge. | 2026-09-11 re-verified live: .skip-link:focus-visible rule present in shell.css?v=phase38 alongside .mode-toggle/.brand-block/.footer-strip a; measured live as outline rgb(204,0,0) solid 2px under a real Tab. | 2026-09-19 re-verified live: .skip-link measured under a real shift+Tab: outline rgb(204,0,0) solid 2px. | 2026-09-26 re-verified live under a REAL shift+Tab on /words/the-stone/: .skip-link matches :focus-visible and paints solid 2px rgb(204,0,0), offset 2px; forward Tab continues to .brand-block and .mode-toggle, both 2px #c00. Skip-link activation (el.click) sets #article and the target exists.</t>
+          <t>ISSUE/Medium (2026-09-02) — `.skip-link` had NO :focus-visible rule anywhere in the loaded cascade. Enumerated every rule matching /skip-link/ across all loaded sheets on live: exactly two hits, both in shell.css (the (0,2,0) :link/:visited base chip from F91, and .skip-link:focus for positioning) — neither carries an outline. Measured under a REAL Tab press on the live homepage with the chip focused: outline `rgb(153,200,255) auto 1px` — Chrome's UA default — while every sibling control measured the same way paints `rgb(204,0,0) solid 2px` (.brand-block, .mode-toggle, a.plate, .issue-standfirst, .hero-link, .sm-submit all confirmed this run). Confirmed identical on /about/ (shared shell.css, skipFocusRule:false). NOT a WCAG 2.4.7 failure — the UA ring is visible, which is exactly why five months of contrast-led sweeps never surfaced it — but a design-token break on the first element a keyboard user ever focuses. Same defect class as F76 (.sm-submit, closed 2026-08-10); this is a distinct element that rule never covered, not a regression of it. | 2026-09-06 re-verified live: still open ON LIVE, as expected - the fix is on this branch and unmerged. Live skip link focuses with the Chrome default ring (outline rgb(153,200,255) auto 1px) instead of the site's red --focus-ring. Closes on merge. | 2026-09-11 re-verified live: .skip-link:focus-visible rule present in shell.css?v=phase38 alongside .mode-toggle/.brand-block/.footer-strip a; measured live as outline rgb(204,0,0) solid 2px under a real Tab. | 2026-09-19 re-verified live: .skip-link measured under a real shift+Tab: outline rgb(204,0,0) solid 2px. | 2026-09-26 re-verified live under a REAL shift+Tab on /words/the-stone/: .skip-link matches :focus-visible and paints solid 2px rgb(204,0,0), offset 2px; forward Tab continues to .brand-block and .mode-toggle, both 2px #c00. Skip-link activation (el.click) sets #article and the target exists. | 2026-09-28: live: skip link :focus-visible 2px solid #c00 under real Tab.</t>
         </is>
       </c>
       <c r="I101" s="6" t="inlineStr">
@@ -5802,7 +5806,7 @@
       </c>
       <c r="H102" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-09-02) — /brand/ was pinning `article.css?v=phase24` while the three src/ references sat at phase37, live-confirmed by reading document.styleSheets on both pages: /brand/ loaded article.css?v=phase24, /words/the-stone/ loaded article.css?v=phase37. article.css moved phase24 -&gt; phase37 in 558aa07 (the F97 eyebrow wrap, merged as f8d7702 on 2026-08-31); that commit bumped three references and missed the fourth. Effect: /css/* is immutable/1y, so any reader who had loaded /brand/ before that bump keeps the pre-F97 sheet on the design-system page for up to a year, while every article page serves the fixed one — the documentation surface silently disagreeing with the site it documents. Same contract as F87 (closed 2026-08-27), different mechanism: F87 was the fix landing in a sheet /brand/ does not load; this is /brand/ loading the right sheet at a stale key. Root cause is structural: the passthrough references sit outside src/, so both the bump sweep and DESIGN-SYSTEM.md's own high-water-mark grep (scoped `src/`) are blind to them — and the doc, written one day earlier in 885930e specifically to codify this rule, itself counted article.css at three references instead of four. | 2026-09-11 re-verified live: /brand/ loads article.css?v=phase37, shell.css?v=phase38, plates.css?v=phase39, brand.css?v=brand10 — the same versions the rest of the site loads. Parity holds. | 2026-09-26 re-verified: every /css/*.css reference across src/, brand/ and phase0/ carries one ?v= per filename (tokens phase24 x7, shell phase38 x7, article phase37 x4, plates phase39 x2, home-augment phase40 x2, home-v2 phase36, notfound phase11, phase0 phase2) — zero parity splits on this branch.</t>
+          <t>ISSUE/Medium (2026-09-02) — /brand/ was pinning `article.css?v=phase24` while the three src/ references sat at phase37, live-confirmed by reading document.styleSheets on both pages: /brand/ loaded article.css?v=phase24, /words/the-stone/ loaded article.css?v=phase37. article.css moved phase24 -&gt; phase37 in 558aa07 (the F97 eyebrow wrap, merged as f8d7702 on 2026-08-31); that commit bumped three references and missed the fourth. Effect: /css/* is immutable/1y, so any reader who had loaded /brand/ before that bump keeps the pre-F97 sheet on the design-system page for up to a year, while every article page serves the fixed one — the documentation surface silently disagreeing with the site it documents. Same contract as F87 (closed 2026-08-27), different mechanism: F87 was the fix landing in a sheet /brand/ does not load; this is /brand/ loading the right sheet at a stale key. Root cause is structural: the passthrough references sit outside src/, so both the bump sweep and DESIGN-SYSTEM.md's own high-water-mark grep (scoped `src/`) are blind to them — and the doc, written one day earlier in 885930e specifically to codify this rule, itself counted article.css at three references instead of four. | 2026-09-11 re-verified live: /brand/ loads article.css?v=phase37, shell.css?v=phase38, plates.css?v=phase39, brand.css?v=brand10 — the same versions the rest of the site loads. Parity holds. | 2026-09-26 re-verified: every /css/*.css reference across src/, brand/ and phase0/ carries one ?v= per filename (tokens phase24 x7, shell phase38 x7, article phase37 x4, plates phase39 x2, home-augment phase40 x2, home-v2 phase36, notfound phase11, phase0 phase2) — zero parity splits on this branch. | 2026-09-28: repo: one ?v= per sheet across layouts + passthroughs (8 sheets). phase0.js bumped phase2 -&gt; phase3 with today's F53 fix (its only reference).</t>
         </is>
       </c>
       <c r="I102" s="6" t="inlineStr">
@@ -5859,7 +5863,7 @@
       </c>
       <c r="H103" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-09-05) — `.demo-plate-body` had `flex: 1` but no `display: flex`, so the `justify-content: flex-end` written for `.demo-plate.img-plate .demo-plate-body` was inert and every white specimen title rendered at the TOP of its plate (measured live: titleTopFrac 0.11, titleBotFrac 0.24-0.38 on all five). The `::after` overlay is `linear-gradient(to top, rgba(0,0,0,.78), rgba(0,0,0,.08) 55%, rgba(0,0,0,.14))` — near-opaque at the bottom, ~.12 alpha at the title's actual position — so the titles sat over the LIGHT end of the concrete texture instead of the dark end. Pixel-measured (headless Chrome 1280px, real CSS, glyph-free sample strip inside the plate at the title's own y-band): the `concrete` specimens' title band runs rgb(98)-rgb(160), giving white-on-lightest 2.61:1 and white-on-median 3.03:1 against a 3:1 large-text floor (25.6px bold Anton). `lines` measured 4.12:1 and `noise` 18.1:1 at the same position, so the failure is texture-dependent — concrete is the light one — but all five were in the wrong band. Not caught by earlier sweeps because a computed-style probe walks the ancestor `background-color` chain straight through both pseudo-elements and reports the page ground (1.06:1) for every one of them, which reads exactly like the known `.plate-image` measurement artifact and was dismissed as such. It is not that artifact: on `.plate-image` the title genuinely sits in the .78 band; here the mirror had lost the rule that puts it there. Same contract as F87/F90 — /brand/ failing to dogfood — third distinct mechanism: F87 was the fix landing in a sheet /brand/ does not load, F99 was /brand/ loading the right sheet at a stale key, this is /brand/ loading the right sheet at the right key with a rule the production component has and the specimen does not. | 2026-09-11 re-verified live: all five .demo-plate.img-plate .demo-plate-body report display:flex / justify-content:flex-end; titles bottom-anchored at topFrac 0.52–0.79. Fix holds. | 2026-09-19 re-verified live: all five /brand/ .demo-plate.img-plate .demo-plate-body compute display:flex / justify-content:flex-end. | 2026-09-26 re-verified live on /brand/: all 5 .img-plate .demo-plate-body are display:flex + justify-content:flex-end, titles sit at 0.69-0.82 of plate height, ::after scrim present (to top .78 -&gt; .26 55% -&gt; ...).</t>
+          <t>ISSUE/Medium (2026-09-05) — `.demo-plate-body` had `flex: 1` but no `display: flex`, so the `justify-content: flex-end` written for `.demo-plate.img-plate .demo-plate-body` was inert and every white specimen title rendered at the TOP of its plate (measured live: titleTopFrac 0.11, titleBotFrac 0.24-0.38 on all five). The `::after` overlay is `linear-gradient(to top, rgba(0,0,0,.78), rgba(0,0,0,.08) 55%, rgba(0,0,0,.14))` — near-opaque at the bottom, ~.12 alpha at the title's actual position — so the titles sat over the LIGHT end of the concrete texture instead of the dark end. Pixel-measured (headless Chrome 1280px, real CSS, glyph-free sample strip inside the plate at the title's own y-band): the `concrete` specimens' title band runs rgb(98)-rgb(160), giving white-on-lightest 2.61:1 and white-on-median 3.03:1 against a 3:1 large-text floor (25.6px bold Anton). `lines` measured 4.12:1 and `noise` 18.1:1 at the same position, so the failure is texture-dependent — concrete is the light one — but all five were in the wrong band. Not caught by earlier sweeps because a computed-style probe walks the ancestor `background-color` chain straight through both pseudo-elements and reports the page ground (1.06:1) for every one of them, which reads exactly like the known `.plate-image` measurement artifact and was dismissed as such. It is not that artifact: on `.plate-image` the title genuinely sits in the .78 band; here the mirror had lost the rule that puts it there. Same contract as F87/F90 — /brand/ failing to dogfood — third distinct mechanism: F87 was the fix landing in a sheet /brand/ does not load, F99 was /brand/ loading the right sheet at a stale key, this is /brand/ loading the right sheet at the right key with a rule the production component has and the specimen does not. | 2026-09-11 re-verified live: all five .demo-plate.img-plate .demo-plate-body report display:flex / justify-content:flex-end; titles bottom-anchored at topFrac 0.52–0.79. Fix holds. | 2026-09-19 re-verified live: all five /brand/ .demo-plate.img-plate .demo-plate-body compute display:flex / justify-content:flex-end. | 2026-09-26 re-verified live on /brand/: all 5 .img-plate .demo-plate-body are display:flex + justify-content:flex-end, titles sit at 0.69-0.82 of plate height, ::after scrim present (to top .78 -&gt; .26 55% -&gt; ...). | 2026-09-28: live: .demo-plate-body flex / flex-end.</t>
         </is>
       </c>
       <c r="I103" s="6" t="inlineStr">
@@ -5916,7 +5920,7 @@
       </c>
       <c r="H104" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-09-06) — the scrim is `linear-gradient(to top, rgba(0,0,0,.78), rgba(0,0,0,.08) 55%, rgba(0,0,0,.14))`: .78 black at the bottom, but only .08–.14 across the top ~45%. That is sound while every title fits inside the bottom band, which is what `justify-content: flex-end` assumes. It does not hold for a three-line Anton title: 'Show Me Your Glory' is 165px tall in a 283px plate, so flex-end has no free space left to give and the first line starts 7% from the top. On `.img-concrete`, whose texture opens on a #c7c7c7 band, the white cap-height rows of 'SHOW' sit on a measured rgb(158,158,158) — 2.68:1 against a 3:1 large-text floor. 'The Theology of Staying on the Call' fails the same way at 2.92:1. Six of the eight live image plates pass (img-lines worst 3.69:1, img-noise worst 12.27:1), so this is texture-and-title-length dependent, not universal. MEASUREMENT: rasterised the homepage in headless Chrome at 1280 wide with the Earlier section unhidden, then sampled a glyph-free 12px strip inside each plate at each glyph row and took the row median — the computed-style probe reports 1.06:1 for all eight, which is the known .plate-image artifact and is why nine months of sweeps saw nothing. This is the second time that artifact has hidden a real defect (F100 was the first) and the first time it hid one in PRODUCTION rather than on /brand/. | 2026-09-11 re-verified live: plates.css?v=phase39 serving the .26/.34 scrim stops; .plate-image .plate-body display:flex / justify-content:flex-end on every image plate. 'Show Me Your Glory' (the three-line title that opened this row) sits at topFrac 0.067 where the scrim is ~.33 alpha — white on ~134 grey = ~3.6:1 against the 3:1 large-text floor. Fix holds. | 2026-09-26 re-verified live: 3 visible homepage .plate-image plates carry the 3-stop scrim (.78 -&gt; .26 @55% -&gt; .34 top); rasterised with headless system Chrome at 1280px and sampled glyph-free strips beside each title line — medians 3.95:1 (Show Me Your Glory, top line on the concrete band) to 11.73:1, all clear of the 3:1 large-text floor.</t>
+          <t>ISSUE/High (2026-09-06) — the scrim is `linear-gradient(to top, rgba(0,0,0,.78), rgba(0,0,0,.08) 55%, rgba(0,0,0,.14))`: .78 black at the bottom, but only .08–.14 across the top ~45%. That is sound while every title fits inside the bottom band, which is what `justify-content: flex-end` assumes. It does not hold for a three-line Anton title: 'Show Me Your Glory' is 165px tall in a 283px plate, so flex-end has no free space left to give and the first line starts 7% from the top. On `.img-concrete`, whose texture opens on a #c7c7c7 band, the white cap-height rows of 'SHOW' sit on a measured rgb(158,158,158) — 2.68:1 against a 3:1 large-text floor. 'The Theology of Staying on the Call' fails the same way at 2.92:1. Six of the eight live image plates pass (img-lines worst 3.69:1, img-noise worst 12.27:1), so this is texture-and-title-length dependent, not universal. MEASUREMENT: rasterised the homepage in headless Chrome at 1280 wide with the Earlier section unhidden, then sampled a glyph-free 12px strip inside each plate at each glyph row and took the row median — the computed-style probe reports 1.06:1 for all eight, which is the known .plate-image artifact and is why nine months of sweeps saw nothing. This is the second time that artifact has hidden a real defect (F100 was the first) and the first time it hid one in PRODUCTION rather than on /brand/. | 2026-09-11 re-verified live: plates.css?v=phase39 serving the .26/.34 scrim stops; .plate-image .plate-body display:flex / justify-content:flex-end on every image plate. 'Show Me Your Glory' (the three-line title that opened this row) sits at topFrac 0.067 where the scrim is ~.33 alpha — white on ~134 grey = ~3.6:1 against the 3:1 large-text floor. Fix holds. | 2026-09-26 re-verified live: 3 visible homepage .plate-image plates carry the 3-stop scrim (.78 -&gt; .26 @55% -&gt; .34 top); rasterised with headless system Chrome at 1280px and sampled glyph-free strips beside each title line — medians 3.95:1 (Show Me Your Glory, top line on the concrete band) to 11.73:1, all clear of the 3:1 large-text floor. | 2026-09-28: live: every .plate-image ::after = linear-gradient(to top, .78, .26 55%, .34) — the F101 scrim.</t>
         </is>
       </c>
       <c r="I104" s="6" t="inlineStr">
@@ -5973,7 +5977,7 @@
       </c>
       <c r="H105" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Low (2026-09-11) — the comment's choice 1 reads 'The linked call-to-action for the same essay is the IssueNext strip below the archive, which is what carries "Notify me →" to the coming-soon page.' That strip was deleted on 2026-08-27 in e3b4e91 under F94, along with 202 lines of its CSS. F94's own p4 already recorded the consequence — 'the upcoming essay's coming-soon page now has ZERO inbound links from the homepage' — but the component that states the trade-off was never updated, so the file explains a bargain whose other half is gone. No behavioural defect: the plate renders correctly and the row is graded Low because it only misleads a reader of the source. Found by grepping src/ for IssueNext after confirming the live homepage and both shipped sheets are clean of it (the three CSS mentions F94 catalogued are comments; this is a fourth mention F94 missed). | 2026-09-26 re-verified: GhostPlate.astro:16-24 records the IssueNext strip as retired 2026-08-27 (e3b4e91) [F94] and says where the decision lives — no dependency on a shipping component.</t>
+          <t>ISSUE/Low (2026-09-11) — the comment's choice 1 reads 'The linked call-to-action for the same essay is the IssueNext strip below the archive, which is what carries "Notify me →" to the coming-soon page.' That strip was deleted on 2026-08-27 in e3b4e91 under F94, along with 202 lines of its CSS. F94's own p4 already recorded the consequence — 'the upcoming essay's coming-soon page now has ZERO inbound links from the homepage' — but the component that states the trade-off was never updated, so the file explains a bargain whose other half is gone. No behavioural defect: the plate renders correctly and the row is graded Low because it only misleads a reader of the source. Found by grepping src/ for IssueNext after confirming the live homepage and both shipped sheets are clean of it (the three CSS mentions F94 catalogued are comments; this is a fourth mention F94 missed). | 2026-09-26 re-verified: GhostPlate.astro:16-24 records the IssueNext strip as retired 2026-08-27 (e3b4e91) [F94] and says where the decision lives — no dependency on a shipping component. | 2026-09-28: carried: GhostPlate comment unchanged.</t>
         </is>
       </c>
       <c r="I105" s="6" t="inlineStr">
@@ -6030,7 +6034,7 @@
       </c>
       <c r="H106" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Low (2026-09-11) — three references to the `.issue-next` strip survived its retirement (e3b4e91, 2026-08-27, F94): the homepage route description listed 'Issue-next ghost CTA' as part of the cascade; PAGES TO CRAWL told the crawler to follow article links from 'the homepage cascade or Issue-next ghost'; and §8 CONTENT COLLECTION INTEGRITY prescribed 'Issue-next ghost CTA's `.next-title` matches the referenced upcoming article's `&lt;title&gt;`'. The §8 line is the one that matters: `.next-title` cannot exist on any page the loop can reach, so that check can only ever be silently skipped — or, worse, reported as run. Graded Low because no site surface is affected and the two descriptive lines are merely stale; it is filed rather than fixed-in-passing because the operating prompt is what every future run executes. | 2026-09-26 re-verified: audit/QA-OS.md names .issue-next / .next-title only as retired (lines 103, 276-277, citing F94); no live check targets them.</t>
+          <t>ISSUE/Low (2026-09-11) — three references to the `.issue-next` strip survived its retirement (e3b4e91, 2026-08-27, F94): the homepage route description listed 'Issue-next ghost CTA' as part of the cascade; PAGES TO CRAWL told the crawler to follow article links from 'the homepage cascade or Issue-next ghost'; and §8 CONTENT COLLECTION INTEGRITY prescribed 'Issue-next ghost CTA's `.next-title` matches the referenced upcoming article's `&lt;title&gt;`'. The §8 line is the one that matters: `.next-title` cannot exist on any page the loop can reach, so that check can only ever be silently skipped — or, worse, reported as run. Graded Low because no site surface is affected and the two descriptive lines are merely stale; it is filed rather than fixed-in-passing because the operating prompt is what every future run executes. | 2026-09-26 re-verified: audit/QA-OS.md names .issue-next / .next-title only as retired (lines 103, 276-277, citing F94); no live check targets them. | 2026-09-28: carried: QA-OS.md unchanged.</t>
         </is>
       </c>
       <c r="I106" s="6" t="inlineStr">
@@ -6087,7 +6091,7 @@
       </c>
       <c r="H107" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Low (2026-09-18) — §3 read 'Verify `--accent` usage on section-head h2, reading-progress bars, pull-quote borders.' Measured live on /words/the-weight-of-my-no/ in dark mode: `.reading-progress` background rgb(243,240,232) (--ink) and `.pull-quote` borders rgba(243,240,232,.82) (--border). Both are deliberate: the progress bar was recoloured from --accent to --ink in 68b0c1d (2026-04-10) with a comment at css/article.css:873 explaining the red bar competed with the masthead, and DESIGN-SYSTEM.md §4 lists pull-quote top/bottom borders as ordinary content borders while naming the .callout left border as the accent one. The check predates nothing — QA-OS was written 2026-08-07, four months after the recolour — so it has been either silently skipped or passed on assumption every run. Same class as F103: a dead check in the operating prompt. Graded Low: no site surface affected. | 2026-09-26 re-verified: QA-OS.md §3 (line 171-175) names section-head h2 + .callout as the accent's homes and records the reading-progress bar and pull-quote borders as by-design. Live spot-check agrees: /brand/ .section-head h2 = rgb(204,0,0), /words/the-stone/ .callout border-left = solid rgb(204,0,0).</t>
+          <t>ISSUE/Low (2026-09-18) — §3 read 'Verify `--accent` usage on section-head h2, reading-progress bars, pull-quote borders.' Measured live on /words/the-weight-of-my-no/ in dark mode: `.reading-progress` background rgb(243,240,232) (--ink) and `.pull-quote` borders rgba(243,240,232,.82) (--border). Both are deliberate: the progress bar was recoloured from --accent to --ink in 68b0c1d (2026-04-10) with a comment at css/article.css:873 explaining the red bar competed with the masthead, and DESIGN-SYSTEM.md §4 lists pull-quote top/bottom borders as ordinary content borders while naming the .callout left border as the accent one. The check predates nothing — QA-OS was written 2026-08-07, four months after the recolour — so it has been either silently skipped or passed on assumption every run. Same class as F103: a dead check in the operating prompt. Graded Low: no site surface affected. | 2026-09-26 re-verified: QA-OS.md §3 (line 171-175) names section-head h2 + .callout as the accent's homes and records the reading-progress bar and pull-quote borders as by-design. Live spot-check agrees: /brand/ .section-head h2 = rgb(204,0,0), /words/the-stone/ .callout border-left = solid rgb(204,0,0). | 2026-09-28: carried: QA-OS.md unchanged.</t>
         </is>
       </c>
       <c r="I107" s="6" t="inlineStr">
@@ -6144,7 +6148,7 @@
       </c>
       <c r="H108" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-09-18) — every page (/, /about/, /brand/, /phase0/, /404, all /words/) carries a Netlify-injected `&lt;script async id="netlify-rum-container" src="/.netlify/scripts/rum"&gt;` with a CWV token for deploy 6aad063. The script beacons to https://ingesteer.services-prod.nsvcs.net/rum_collection, which the site's own CSP (`connect-src 'self'`, commented in netlify.toml as 'no analytics/beacons allowed') refuses. Result, reproduced on the homepage and on /words/the-weight-of-my-no/: two CSP violation errors plus an 'Uncaught (in promise) TypeError: Failed to fetch' from /.netlify/scripts/rum:1:11100. No reader-visible breakage — but it is a console error on every page view, and whatever Netlify observability panel this feeds is receiving nothing. The script was already present on 2026-09-11 (F102's p4 notes it in the live-vs-dist diff) while that run logged zero console errors, so either the beacon only fires on page hide / navigation (consistent with it arriving on navigate here) or the collector moved off-origin since; NEW to the ledger either way. Graded HIGH per the console-error rule. | 2026-09-19: still live, as expected — the connect-src fix sits on the unmerged qa/fixes-20260918 (carried into qa/fixes-20260919). Re-observed on /words/the-weight-of-my-no/: two connect-src violations against https://ingesteer.services-prod.nsvcs.net/rum_collection plus an uncaught 'Failed to fetch' from /.netlify/scripts/rum. Live CSP still reads connect-src 'self'. Not a regression; closes on merge.</t>
+          <t>ISSUE/High (2026-09-18) — every page (/, /about/, /brand/, /phase0/, /404, all /words/) carries a Netlify-injected `&lt;script async id="netlify-rum-container" src="/.netlify/scripts/rum"&gt;` with a CWV token for deploy 6aad063. The script beacons to https://ingesteer.services-prod.nsvcs.net/rum_collection, which the site's own CSP (`connect-src 'self'`, commented in netlify.toml as 'no analytics/beacons allowed') refuses. Result, reproduced on the homepage and on /words/the-weight-of-my-no/: two CSP violation errors plus an 'Uncaught (in promise) TypeError: Failed to fetch' from /.netlify/scripts/rum:1:11100. No reader-visible breakage — but it is a console error on every page view, and whatever Netlify observability panel this feeds is receiving nothing. The script was already present on 2026-09-11 (F102's p4 notes it in the live-vs-dist diff) while that run logged zero console errors, so either the beacon only fires on page hide / navigation (consistent with it arriving on navigate here) or the collector moved off-origin since; NEW to the ledger either way. Graded HIGH per the console-error rule. | 2026-09-19: still live, as expected — the connect-src fix sits on the unmerged qa/fixes-20260918 (carried into qa/fixes-20260919). Re-observed on /words/the-weight-of-my-no/: two connect-src violations against https://ingesteer.services-prod.nsvcs.net/rum_collection plus an uncaught 'Failed to fetch' from /.netlify/scripts/rum. Live CSP still reads connect-src 'self'. Not a regression; closes on merge. | 2026-09-28: live: 0 site console errors across 9 routes; RUM loads with no CSP violation.</t>
         </is>
       </c>
       <c r="I108" s="6" t="inlineStr">
@@ -6201,7 +6205,7 @@
       </c>
       <c r="H109" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Low (2026-09-18) — index.astro:205 renders `&lt;RowHead label="This Week" variant="lead" /&gt;` unconditionally for the newest published essay; nothing compares the lead's publishedDate to the build date. Live today (Fri 2026-09-18) the row reads '01 This Week' over The Weight of My No, published 2026-08-31 — 18 days old. It read the same over Send Someone Else through most of August, when that essay was up to 57 days old. The daily rebuild (F73) would make a date-derived label accurate every morning at no cost. Filed Low: nothing breaks and it is not an a11y or SEO defect, but it is a false recency claim in the most prominent label on the page. | 2026-09-19: still live, as expected — homepage lead row head reads '01 THIS WEEK' over The Weight of My No (2026-08-31, now 19 days old); the 'Latest' fix sits on the unmerged qa/fixes-20260918. Closes on merge.</t>
+          <t>ISSUE/Low (2026-09-18) — index.astro:205 renders `&lt;RowHead label="This Week" variant="lead" /&gt;` unconditionally for the newest published essay; nothing compares the lead's publishedDate to the build date. Live today (Fri 2026-09-18) the row reads '01 This Week' over The Weight of My No, published 2026-08-31 — 18 days old. It read the same over Send Someone Else through most of August, when that essay was up to 57 days old. The daily rebuild (F73) would make a date-derived label accurate every morning at no cost. Filed Low: nothing breaks and it is not an a11y or SEO defect, but it is a false recency claim in the most prominent label on the page. | 2026-09-19: still live, as expected — homepage lead row head reads '01 THIS WEEK' over The Weight of My No (2026-08-31, now 19 days old); the 'Latest' fix sits on the unmerged qa/fixes-20260918. Closes on merge. | 2026-09-28: live: lead row label 'Latest'.</t>
         </is>
       </c>
       <c r="I109" s="6" t="inlineStr">
@@ -6258,7 +6262,7 @@
       </c>
       <c r="H110" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Low (2026-09-22) — §9 named no method for F57, so this run tested it with a burst chained onto the subscribe smoke test: 8 POSTs returned 8 x 200 and no 429 (one returned HTTP 000, an instance churn tell), which reads as a dead limiter. A clean sequential re-run returned exactly 5 x 400 then 5 x 429; a parallel re-run returned 10 x 400 and no 429. The limiter is correct; the prompt lacked the method, and the false reading cost two test cycles. Same class as F103/F104. | 2026-09-27 re-verified against the file: QA-OS.md §9 still carries the sequential 10-POST method (5 x 400 then 5 x 429) and the MEASUREMENT ANTIPATTERNS fan-out entry.</t>
+          <t>ISSUE/Low (2026-09-22) — §9 named no method for F57, so this run tested it with a burst chained onto the subscribe smoke test: 8 POSTs returned 8 x 200 and no 429 (one returned HTTP 000, an instance churn tell), which reads as a dead limiter. A clean sequential re-run returned exactly 5 x 400 then 5 x 429; a parallel re-run returned 10 x 400 and no 429. The limiter is correct; the prompt lacked the method, and the false reading cost two test cycles. Same class as F103/F104. | 2026-09-27 re-verified against the file: QA-OS.md §9 still carries the sequential 10-POST method (5 x 400 then 5 x 429) and the MEASUREMENT ANTIPATTERNS fan-out entry. | 2026-09-28: carried: QA-OS.md §9 unchanged; method used today (see F57).</t>
         </is>
       </c>
       <c r="I110" s="6" t="inlineStr">
@@ -6315,7 +6319,7 @@
       </c>
       <c r="H111" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-09-24) — .rail-cta's base rule is background: var(--ink); color: var(--bg), and a.plate-lead:hover .rail-cta swaps only the background to var(--accent). In light mode that is cream on #c00 (#f4f4f1, ~5.2:1, passes). In dark mode --bg is #060606, so the hovered chip renders near-black 'READ →' on #c00 at 3.44:1 at 12px/700, under the 4.5:1 floor (WCAG 1.4.3). Measured under a REAL pointer hover after a 3s settle (a.plate-lead:hover true; computed rgb(6,6,6) on rgb(204,0,0)) and confirmed on screenshot. It is the same defect class F83 closed for .latest-cta and .hero-link.primary on 2026-08-13; F83's scope note said only those two controls invert onto the fill, which missed this third one. Present since the lead plate shipped (d1f8e7e, 2026-04-21), so NEW to the ledger, not a regression. /brand/ renders .plate-lead and loads home-augment.css, so it carries the same defect. | 2026-09-25: still present LIVE — live home-augment.css is phase34 without the rule; fix sits on the unmerged stacked branch (now qa/fixes-20260925). Awaiting Dexter's merge; not re-counted as new.</t>
+          <t>ISSUE/High (2026-09-24) — .rail-cta's base rule is background: var(--ink); color: var(--bg), and a.plate-lead:hover .rail-cta swaps only the background to var(--accent). In light mode that is cream on #c00 (#f4f4f1, ~5.2:1, passes). In dark mode --bg is #060606, so the hovered chip renders near-black 'READ →' on #c00 at 3.44:1 at 12px/700, under the 4.5:1 floor (WCAG 1.4.3). Measured under a REAL pointer hover after a 3s settle (a.plate-lead:hover true; computed rgb(6,6,6) on rgb(204,0,0)) and confirmed on screenshot. It is the same defect class F83 closed for .latest-cta and .hero-link.primary on 2026-08-13; F83's scope note said only those two controls invert onto the fill, which missed this third one. Present since the lead plate shipped (d1f8e7e, 2026-04-21), so NEW to the ledger, not a regression. /brand/ renders .plate-lead and loads home-augment.css, so it carries the same defect. | 2026-09-25: still present LIVE — live home-augment.css is phase34 without the rule; fix sits on the unmerged stacked branch (now qa/fixes-20260925). Awaiting Dexter's merge; not re-counted as new. | 2026-09-28: still present LIVE — real pointer hover, dark mode, 3s settle: .rail-cta rgb(6,6,6) on rgb(204,0,0) = 3.44:1 (screenshot). A 1s read caught the chip mid-transition on --ink; re-measured before concluding. Awaiting Dexter's merge; not re-counted as new.</t>
         </is>
       </c>
       <c r="I111" s="6" t="inlineStr">
@@ -6330,7 +6334,7 @@
       </c>
       <c r="K111" s="6" t="inlineStr">
         <is>
-          <t>PASS (2026-09-24, verified against build + rule injected on live) — npm run build clean; dist/css/home-augment.css carries the new selector; dist/index.html and dist/brand/index.html both reference home-augment.css?v=phase40. Dev servers cannot start in unattended runs, so the fix rule was applied to the live homepage with insertRule on the loaded home-augment sheet: dark mode, real pointer hover, a.plate-lead:hover true -&gt; .rail-cta rgb(243,240,232) on rgb(204,0,0) = 5.17:1 (screenshot shows a cream 'READ →'). deleteRule restored the sheet and a re-measure read 3.44:1 again, proving the page went back to its original state. Light-mode hover unchanged (rule is dark-scoped): rgb(244,244,241) on #c00. Sibling hover controls (.latest-cta, .hero-link.primary) re-measured 5.17:1, unaffected. Live-verifies on the first SCRUB after merge. | 2026-09-26: still awaits merge — origin/main and the live deploy (6ab794f1, 09-26 09:48Z) remain on 95e2a73, so the live chip is still the pre-fix 3.44:1 on dark-mode hover. | 2026-09-27: still awaits merge — origin/main and the live deploy (6ab794f1, 09-26 09:48Z) remain on 95e2a73; the live home-augment.css?v=phase34 carries no dark-mode :hover .rail-cta rule. Not re-counted as new.</t>
+          <t>PASS (2026-09-24, verified against build + rule injected on live) — npm run build clean; dist/css/home-augment.css carries the new selector; dist/index.html and dist/brand/index.html both reference home-augment.css?v=phase40. Dev servers cannot start in unattended runs, so the fix rule was applied to the live homepage with insertRule on the loaded home-augment sheet: dark mode, real pointer hover, a.plate-lead:hover true -&gt; .rail-cta rgb(243,240,232) on rgb(204,0,0) = 5.17:1 (screenshot shows a cream 'READ →'). deleteRule restored the sheet and a re-measure read 3.44:1 again, proving the page went back to its original state. Light-mode hover unchanged (rule is dark-scoped): rgb(244,244,241) on #c00. Sibling hover controls (.latest-cta, .hero-link.primary) re-measured 5.17:1, unaffected. Live-verifies on the first SCRUB after merge. | 2026-09-26: still awaits merge — origin/main and the live deploy (6ab794f1, 09-26 09:48Z) remain on 95e2a73, so the live chip is still the pre-fix 3.44:1 on dark-mode hover. | 2026-09-27: still awaits merge — origin/main and the live deploy (6ab794f1, 09-26 09:48Z) remain on 95e2a73; the live home-augment.css?v=phase34 carries no dark-mode :hover .rail-cta rule. Not re-counted as new. | 2026-09-28: still awaits merge — origin/main and the live deploy (2026-09-27 10:29Z) remain on 95e2a73.</t>
         </is>
       </c>
     </row>
@@ -6350,7 +6354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6378,7 +6382,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5">
@@ -6391,82 +6395,72 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="B6" s="11" t="n">
-        <v>1</v>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>— P4 (re-test) —</t>
+        </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>— P4 (re-test) —</t>
-        </is>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>103</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="n">
-        <v>103</v>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="B11" s="11" t="n">
+      <c r="B10" s="11" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>— Issues by severity (found) —</t>
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>Resolved (P4 PASS)</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="n">
+        <v>29</v>
+      </c>
+    </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>Resolved (P4 PASS)</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="n">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>Still open</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B15" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>Total features: 108</t>
         </is>

</xml_diff>

<commit_message>
audit(ledger): 2026-09-29 scrub — clean site, F07-F16 rotation all PASS, F108 re-measured live
Tuesday rotation, scrub-only (no FAIL/ISSUE opened, FIX/RETEST skipped).
Live = GitHub main = 95e2a73, zero drift. F108 (High), F80 (Low) and F53
(Medium) remain fixed on the unmerged qa/fixes-20260924..0928 branches.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>PASS (2026-08-15 scrub) — home/about/phase0/articles all carry the feed discovery link; /404 correctly omits it. NOTE: the prior `expected` said articles do NOT include it. That text was stale — ArticleLayout has emitted the link since a4f4f25; the site was never wrong, the row was. Expectation corrected, not the code. | 2026-08-25 re-verified live: &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present in head. | 2026-09-01 re-verified live: &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present in head; /feed.xml 200. | 2026-09-19 re-verified live: feed discovery &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present on /, /about/, /phase0/, /brand/ and all 17 articles; absent on the 404 as specified. | 2026-09-28: live: atom alternate link on home/about/phase0/article; absent on 404 as specified.</t>
+          <t>PASS (2026-08-15 scrub) — home/about/phase0/articles all carry the feed discovery link; /404 correctly omits it. NOTE: the prior `expected` said articles do NOT include it. That text was stale — ArticleLayout has emitted the link since a4f4f25; the site was never wrong, the row was. Expectation corrected, not the code. | 2026-08-25 re-verified live: &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present in head. | 2026-09-01 re-verified live: &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present in head; /feed.xml 200. | 2026-09-19 re-verified live: feed discovery &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present on /, /about/, /phase0/, /brand/ and all 17 articles; absent on the 404 as specified. | 2026-09-28: live: atom alternate link on home/about/phase0/article; absent on 404 as specified. | 2026-09-29: live: atom alternate link on home/about/phase0/brand + all 17 articles; absent on the 404 as specified.</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr"/>
@@ -995,7 +995,7 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>PASS — /img/favicon-32.png + /img/apple-touch-icon.png 200 on every referenced path | 2026-08-15 re-verified live: favicon-32.png + apple-touch-icon.png linked on every page; both 200 (1327b / 5729b) | 2026-08-25 re-verified live: /img/favicon-32.png 200, /img/apple-touch-icon.png 200 on every referenced path. | 2026-08-27 re-verified live: /img/favicon-32.png + /img/apple-touch-icon.png 200. | 2026-09-01 re-verified live: /img/favicon-32.png 200, /img/apple-touch-icon.png 200, /img/logo-dark.svg 200. | 2026-09-06 re-verified live: /img/favicon-32.png 200 (1327b), /img/apple-touch-icon.png 200 (5729b), /img/logo-dark.svg 200. | 2026-09-11 re-verified live: /img/favicon-32.png and /img/apple-touch-icon.png both 200, served public,max-age=31536000,immutable. | 2026-09-28: live: favicon-32 + apple-touch-icon linked on all 5 page types; both 200 immutable.</t>
+          <t>PASS — /img/favicon-32.png + /img/apple-touch-icon.png 200 on every referenced path | 2026-08-15 re-verified live: favicon-32.png + apple-touch-icon.png linked on every page; both 200 (1327b / 5729b) | 2026-08-25 re-verified live: /img/favicon-32.png 200, /img/apple-touch-icon.png 200 on every referenced path. | 2026-08-27 re-verified live: /img/favicon-32.png + /img/apple-touch-icon.png 200. | 2026-09-01 re-verified live: /img/favicon-32.png 200, /img/apple-touch-icon.png 200, /img/logo-dark.svg 200. | 2026-09-06 re-verified live: /img/favicon-32.png 200 (1327b), /img/apple-touch-icon.png 200 (5729b), /img/logo-dark.svg 200. | 2026-09-11 re-verified live: /img/favicon-32.png and /img/apple-touch-icon.png both 200, served public,max-age=31536000,immutable. | 2026-09-28: live: favicon-32 + apple-touch-icon linked on all 5 page types; both 200 immutable. | 2026-09-29: live: favicon-32 + apple-touch-icon linked on all 22 routes; both 200 immutable.</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr"/>
@@ -1044,7 +1044,7 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>PASS — Anton + IBM Plex Sans self-hosted, preloaded, document.fonts status 'loaded'; CSP font-src intact | 2026-08-15 re-verified live: Anton + IBM Plex Sans preloaded with crossorigin; zero Google Fonts refs; document.fonts reports all 3 faces loaded | 2026-08-16 re-verified live: Anton + IBM Plex Sans (Regular/Bold) all report document.fonts status 'loaded', document.fonts.status 'loaded'; zero Google Fonts references. /brand/ additionally preloads IBMPlexSans-Italic.woff2 and the console warns it is 'not used within a few seconds of load' — investigated and DISMISSED as a non-finding: the italic face is genuinely used by 13 elements on that page and reports status 'loaded'; the warning is a below-the-fold timing artifact. No other page preloads italic, which is correct. | 2026-08-25 re-verified live: document.fonts.status "loaded"; Anton/400, IBM Plex Sans/400 and /700 all report loaded. All three woff2 200. No FOUT observed. | 2026-08-27 re-verified live: document.fonts: Anton 400, IBM Plex Sans 400 + 700 all 'loaded'; fonts.status 'loaded'; no FOUT observed. | 2026-09-01 re-verified live via document.fonts (not the CSS stack): Anton 400 loaded, IBM Plex Sans 400 + 700 loaded; document.fonts.check() true for all three on home and article. No FOUT/FOIT observed. | 2026-09-06 re-verified live: document.fonts reports Anton 400, IBM Plex Sans 400 and 700 all 'loaded' on home and article; all three woff2 files 200 with immutable cache-control. No FOUT observed. | 2026-09-11 re-verified live: document.fonts reports Anton 400 loaded and IBM Plex Sans 400/700 loaded; fonts.check() true for both families. No FOUT observed. | 2026-09-28: live: document.fonts loaded Anton 400 + IBM Plex Sans 400/700; font preload with crossorigin on all 5 page types; no Google Fonts.</t>
+          <t>PASS — Anton + IBM Plex Sans self-hosted, preloaded, document.fonts status 'loaded'; CSP font-src intact | 2026-08-15 re-verified live: Anton + IBM Plex Sans preloaded with crossorigin; zero Google Fonts refs; document.fonts reports all 3 faces loaded | 2026-08-16 re-verified live: Anton + IBM Plex Sans (Regular/Bold) all report document.fonts status 'loaded', document.fonts.status 'loaded'; zero Google Fonts references. /brand/ additionally preloads IBMPlexSans-Italic.woff2 and the console warns it is 'not used within a few seconds of load' — investigated and DISMISSED as a non-finding: the italic face is genuinely used by 13 elements on that page and reports status 'loaded'; the warning is a below-the-fold timing artifact. No other page preloads italic, which is correct. | 2026-08-25 re-verified live: document.fonts.status "loaded"; Anton/400, IBM Plex Sans/400 and /700 all report loaded. All three woff2 200. No FOUT observed. | 2026-08-27 re-verified live: document.fonts: Anton 400, IBM Plex Sans 400 + 700 all 'loaded'; fonts.status 'loaded'; no FOUT observed. | 2026-09-01 re-verified live via document.fonts (not the CSS stack): Anton 400 loaded, IBM Plex Sans 400 + 700 loaded; document.fonts.check() true for all three on home and article. No FOUT/FOIT observed. | 2026-09-06 re-verified live: document.fonts reports Anton 400, IBM Plex Sans 400 and 700 all 'loaded' on home and article; all three woff2 files 200 with immutable cache-control. No FOUT observed. | 2026-09-11 re-verified live: document.fonts reports Anton 400 loaded and IBM Plex Sans 400/700 loaded; fonts.check() true for both families. No FOUT observed. | 2026-09-28: live: document.fonts loaded Anton 400 + IBM Plex Sans 400/700; font preload with crossorigin on all 5 page types; no Google Fonts. | 2026-09-29: live: document.fonts 'loaded' — Anton 400, IBM Plex Sans 400/700; 3 font preloads with crossorigin on every non-/brand/ route; 0 Google Fonts refs.</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr"/>
@@ -1093,7 +1093,7 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>PASS — no horizontal overflow at 390px on home/article/about/phase0/brand/404 | 2026-08-15 re-verified live: viewport width=device-width + viewport-fit=cover on all pages | 2026-09-01 re-verified live at an emulated 375x812: documentElement.scrollWidth == clientWidth == 375 on the article page — zero horizontal overflow. | 2026-09-06 re-verified live at 375x812: homepage and article scrollWidth == clientWidth (no horizontal overflow). | 2026-09-11 re-verified live: 375px homepage and article: scrollWidth == clientWidth == 375, zero elements overflowing the client width, 17 plates intact. | 2026-09-28: live: viewport meta (width=device-width, viewport-fit=cover) on all 5 types; at 390px scrollWidth == 390 and 0 overflowing elements on home/article/about/phase0/brand.</t>
+          <t>PASS — no horizontal overflow at 390px on home/article/about/phase0/brand/404 | 2026-08-15 re-verified live: viewport width=device-width + viewport-fit=cover on all pages | 2026-09-01 re-verified live at an emulated 375x812: documentElement.scrollWidth == clientWidth == 375 on the article page — zero horizontal overflow. | 2026-09-06 re-verified live at 375x812: homepage and article scrollWidth == clientWidth (no horizontal overflow). | 2026-09-11 re-verified live: 375px homepage and article: scrollWidth == clientWidth == 375, zero elements overflowing the client width, 17 plates intact. | 2026-09-28: live: viewport meta (width=device-width, viewport-fit=cover) on all 5 types; at 390px scrollWidth == 390 and 0 overflowing elements on home/article/about/phase0/brand. | 2026-09-29: live: viewport meta width=device-width on all 22 routes; at 390x844 scrollWidth == clientWidth == 390 on home/article/about/phase0/brand/404.</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr"/>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>PASS — title/description/canonical on all 21 routes; every canonical on imjustdex.com | 2026-08-15 re-verified live: zero duplicate &lt;title&gt; across 20 pages; /404 canonical is /404 as specified | 2026-08-25 re-verified live: &lt;title&gt;, meta description and canonical present and correct on all 20 routes; every canonical points at imjustdex.com. | 2026-08-27 re-verified live: title/description/canonical present and on-domain across all 21 routes. | 2026-09-01 re-verified live: &lt;title&gt;, meta description and canonical present on all 17 articles plus / and /about/; canonicals all on imjustdex.com. | 2026-09-06 re-verified live: title, meta description and canonical present on all 5 chrome pages and all 17 articles; every canonical on https://imjustdex.com/. | 2026-09-11 re-verified live: title/description/canonical present and imjustdex.com-absolute on all 17 articles + home/about/brand/phase0/404. | 2026-09-28: live: title + description + canonical on all 21 indexable routes; 404 canonical /404.</t>
+          <t>PASS — title/description/canonical on all 21 routes; every canonical on imjustdex.com | 2026-08-15 re-verified live: zero duplicate &lt;title&gt; across 20 pages; /404 canonical is /404 as specified | 2026-08-25 re-verified live: &lt;title&gt;, meta description and canonical present and correct on all 20 routes; every canonical points at imjustdex.com. | 2026-08-27 re-verified live: title/description/canonical present and on-domain across all 21 routes. | 2026-09-01 re-verified live: &lt;title&gt;, meta description and canonical present on all 17 articles plus / and /about/; canonicals all on imjustdex.com. | 2026-09-06 re-verified live: title, meta description and canonical present on all 5 chrome pages and all 17 articles; every canonical on https://imjustdex.com/. | 2026-09-11 re-verified live: title/description/canonical present and imjustdex.com-absolute on all 17 articles + home/about/brand/phase0/404. | 2026-09-28: live: title + description + canonical on all 21 indexable routes; 404 canonical /404. | 2026-09-29: live: 0 duplicate titles across 21 indexable routes; every canonical is self-referencing on imjustdex.com; 404 canonical /404.</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr"/>
@@ -1195,7 +1195,7 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>PASS — og+twitter complete on all 21; all 19 OG images 200 (16 essays + home/about/phase0/brand) | 2026-08-15 re-verified live: twitter:card summary_large_image on every page in scope (404 correctly excluded) | 2026-08-25 re-verified live: og:title / og:description / og:image present on all 20; all 16 og-&lt;slug&gt;.png 200; og:image byte-identical to the JSON-LD image on all 16. | 2026-08-27 re-verified live: og+twitter complete across 21 routes; all 21 distinct OG images 200. | 2026-09-01 re-verified live: og:image resolves 200 on all 17 articles and every one matches the JSON-LD image URL exactly, cache-bust included. | 2026-09-06 re-verified live: og:title / og:description / og:image present on all 5 chrome pages and all 17 articles; og:image matches the JSON-LD image byte-for-byte on 17/17. | 2026-09-11 re-verified live: og:title/og:description/og:image present on all 22 HTML routes; every og:image resolves 200. | 2026-09-28: live: og + twitter complete on 21 routes; all OG images 200. (/phase0/ omits the optional og:image:width/height hints — not flagged.)</t>
+          <t>PASS — og+twitter complete on all 21; all 19 OG images 200 (16 essays + home/about/phase0/brand) | 2026-08-15 re-verified live: twitter:card summary_large_image on every page in scope (404 correctly excluded) | 2026-08-25 re-verified live: og:title / og:description / og:image present on all 20; all 16 og-&lt;slug&gt;.png 200; og:image byte-identical to the JSON-LD image on all 16. | 2026-08-27 re-verified live: og+twitter complete across 21 routes; all 21 distinct OG images 200. | 2026-09-01 re-verified live: og:image resolves 200 on all 17 articles and every one matches the JSON-LD image URL exactly, cache-bust included. | 2026-09-06 re-verified live: og:title / og:description / og:image present on all 5 chrome pages and all 17 articles; og:image matches the JSON-LD image byte-for-byte on 17/17. | 2026-09-11 re-verified live: og:title/og:description/og:image present on all 22 HTML routes; every og:image resolves 200. | 2026-09-28: live: og + twitter complete on 21 routes; all OG images 200. (/phase0/ omits the optional og:image:width/height hints — not flagged.) | 2026-09-29: live: og + twitter complete on all 21; og-phase0 and og-brand measured 1200x630 (both pages omit the optional og:image:width/height/alt hints — not flagged, expectation is the image size).</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr"/>
@@ -1248,7 +1248,7 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>PASS — WebSite + Person @graph complete (name/url/sameAs/jobTitle/worksFor) | 2026-08-15 re-verified live: home @graph carries WebSite + Person; Person has name/url/sameAs/jobTitle/worksFor — no missing fields | 2026-08-25 re-verified live: WebSite + Person @graph complete on /; Person carries name, url, sameAs, jobTitle, worksFor. | 2026-08-27 re-verified live: WebSite + Person @graph complete (name/url/sameAs/jobTitle/worksFor). | 2026-09-01 re-verified live: homepage @graph carries WebSite + Person; Person has name, url, sameAs, jobTitle, worksFor — zero required fields missing. | 2026-09-06 re-verified live: homepage @graph carries WebSite + Person; Person complete on name/url/sameAs/jobTitle/worksFor. | 2026-09-11 re-verified live: homepage @graph carries WebSite + Person; Person has name, url, sameAs, jobTitle, worksFor. | 2026-09-28: live: WebSite + Person @graph; Person has name/url/sameAs/jobTitle/worksFor.</t>
+          <t>PASS — WebSite + Person @graph complete (name/url/sameAs/jobTitle/worksFor) | 2026-08-15 re-verified live: home @graph carries WebSite + Person; Person has name/url/sameAs/jobTitle/worksFor — no missing fields | 2026-08-25 re-verified live: WebSite + Person @graph complete on /; Person carries name, url, sameAs, jobTitle, worksFor. | 2026-08-27 re-verified live: WebSite + Person @graph complete (name/url/sameAs/jobTitle/worksFor). | 2026-09-01 re-verified live: homepage @graph carries WebSite + Person; Person has name, url, sameAs, jobTitle, worksFor — zero required fields missing. | 2026-09-06 re-verified live: homepage @graph carries WebSite + Person; Person complete on name/url/sameAs/jobTitle/worksFor. | 2026-09-11 re-verified live: homepage @graph carries WebSite + Person; Person has name, url, sameAs, jobTitle, worksFor. | 2026-09-28: live: WebSite + Person @graph; Person has name/url/sameAs/jobTitle/worksFor. | 2026-09-29: live: WebSite + Person @graph; Person has name/url/sameAs/jobTitle/worksFor.</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr"/>
@@ -1297,7 +1297,7 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>PASS — ProfilePage mainEntity Person complete (name/url/jobTitle/worksFor/sameAs/description) | 2026-08-15 re-verified live: about ProfilePage mainEntity Person complete — name/url/jobTitle/worksFor/sameAs/description all present | 2026-08-25 re-verified live: ProfilePage on /about/ with mainEntity @type Person carrying name, url, jobTitle, worksFor, sameAs, description. | 2026-08-27 re-verified live: ProfilePage mainEntity Person complete (name/url/jobTitle/worksFor/sameAs/description). | 2026-09-01 re-verified live: /about/ ProfilePage mainEntity is @type Person with name, url, jobTitle, worksFor, sameAs, description — zero missing. | 2026-09-06 re-verified live: /about/ ProfilePage present, mainEntity @type=Person complete on name/url/jobTitle/worksFor/sameAs/description. | 2026-09-11 re-verified live: /about/ ProfilePage mainEntity is a Person with all six required fields present. | 2026-09-28: live: ProfilePage mainEntity Person with name/url/jobTitle/worksFor/sameAs/description.</t>
+          <t>PASS — ProfilePage mainEntity Person complete (name/url/jobTitle/worksFor/sameAs/description) | 2026-08-15 re-verified live: about ProfilePage mainEntity Person complete — name/url/jobTitle/worksFor/sameAs/description all present | 2026-08-25 re-verified live: ProfilePage on /about/ with mainEntity @type Person carrying name, url, jobTitle, worksFor, sameAs, description. | 2026-08-27 re-verified live: ProfilePage mainEntity Person complete (name/url/jobTitle/worksFor/sameAs/description). | 2026-09-01 re-verified live: /about/ ProfilePage mainEntity is @type Person with name, url, jobTitle, worksFor, sameAs, description — zero missing. | 2026-09-06 re-verified live: /about/ ProfilePage present, mainEntity @type=Person complete on name/url/jobTitle/worksFor/sameAs/description. | 2026-09-11 re-verified live: /about/ ProfilePage mainEntity is a Person with all six required fields present. | 2026-09-28: live: ProfilePage mainEntity Person with name/url/jobTitle/worksFor/sameAs/description. | 2026-09-29: live: ProfilePage mainEntity Person with name/url/jobTitle/worksFor/sameAs/description.</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr"/>
@@ -1346,7 +1346,7 @@
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>PASS — BlogPosting complete on all 16 (headline, description, datePublished, dateModified, author Person, publisher Organization+logo, mainEntityOfPage, image, url, inLanguage, wordCount); image == og:image exactly, no og-default drift | 2026-08-13 re-verified live: all 16 BlogPosting blocks carry every required field (headline, description, datePublished, dateModified, author.@type=Person + name, publisher, mainEntityOfPage, image, url, inLanguage, wordCount); zero og-default.png drift. | 2026-08-16 re-verified live: all 16 BlogPosting blocks re-verified live: every required field present (headline, description, datePublished, dateModified, author.@type=Person, publisher, mainEntityOfPage, image, url, inLanguage, wordCount) and JSON-LD image === og:image exactly, cache-bust included, on all 16. Zero og-default.png drift. | 2026-08-25 re-verified live: BlogPosting on all 16 articles; every required field present (headline, description, datePublished, dateModified, author.Person.name, publisher, mainEntityOfPage, image, url, inLanguage, wordCount). Zero og-default.png regressions. | 2026-08-27 re-verified live: BlogPosting complete on all 16 — all 11 required fields, author.@type=Person, og:image == JSON-LD image, image == og-&lt;slug&gt;.png on every one. | 2026-09-01 re-verified live: all 17 BlogPosting blocks carry every required field (headline, description, datePublished, dateModified, author.@type=Person + name, publisher, mainEntityOfPage, image, url, inLanguage, wordCount). Zero on og-default.png. | 2026-09-06 re-verified live: 17/17 BlogPosting blocks complete on all 11 required fields, author @type=Person with name, image per-slug. | 2026-09-11 re-verified live: all 17 BlogPosting blocks carry the full 11-field set; author is Person with a name. | 2026-09-28: live: BlogPosting complete 17/17 (all 12 required fields, author @type Person).</t>
+          <t>PASS — BlogPosting complete on all 16 (headline, description, datePublished, dateModified, author Person, publisher Organization+logo, mainEntityOfPage, image, url, inLanguage, wordCount); image == og:image exactly, no og-default drift | 2026-08-13 re-verified live: all 16 BlogPosting blocks carry every required field (headline, description, datePublished, dateModified, author.@type=Person + name, publisher, mainEntityOfPage, image, url, inLanguage, wordCount); zero og-default.png drift. | 2026-08-16 re-verified live: all 16 BlogPosting blocks re-verified live: every required field present (headline, description, datePublished, dateModified, author.@type=Person, publisher, mainEntityOfPage, image, url, inLanguage, wordCount) and JSON-LD image === og:image exactly, cache-bust included, on all 16. Zero og-default.png drift. | 2026-08-25 re-verified live: BlogPosting on all 16 articles; every required field present (headline, description, datePublished, dateModified, author.Person.name, publisher, mainEntityOfPage, image, url, inLanguage, wordCount). Zero og-default.png regressions. | 2026-08-27 re-verified live: BlogPosting complete on all 16 — all 11 required fields, author.@type=Person, og:image == JSON-LD image, image == og-&lt;slug&gt;.png on every one. | 2026-09-01 re-verified live: all 17 BlogPosting blocks carry every required field (headline, description, datePublished, dateModified, author.@type=Person + name, publisher, mainEntityOfPage, image, url, inLanguage, wordCount). Zero on og-default.png. | 2026-09-06 re-verified live: 17/17 BlogPosting blocks complete on all 11 required fields, author @type=Person with name, image per-slug. | 2026-09-11 re-verified live: all 17 BlogPosting blocks carry the full 11-field set; author is Person with a name. | 2026-09-28: live: BlogPosting complete 17/17 (all 12 required fields, author @type Person). | 2026-09-29: live: BlogPosting complete 17/17 (12 required fields, author @type Person); LD image == og:image 17/17.</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr"/>
@@ -1395,7 +1395,7 @@
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>PASS — phase0 WebPage JSON-LD present and parses | 2026-08-27 re-verified live: phase0 WebPage + Person JSON-LD present and parse. | 2026-09-11 re-verified live: /phase0/ @graph = WebPage(#webpage) isPartOf #website, author #person. Valid JSON-LD. | 2026-09-28: live: WebPage isPartOf #website, author #person.</t>
+          <t>PASS — phase0 WebPage JSON-LD present and parses | 2026-08-27 re-verified live: phase0 WebPage + Person JSON-LD present and parse. | 2026-09-11 re-verified live: /phase0/ @graph = WebPage(#webpage) isPartOf #website, author #person. Valid JSON-LD. | 2026-09-28: live: WebPage isPartOf #website, author #person. | 2026-09-29: live: WebPage 'Phase 0 — Ministry Marketing OS', url /phase0/, isPartOf #website, author #person.</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr"/>
@@ -3319,7 +3319,7 @@
       </c>
       <c r="K56" s="6" t="inlineStr">
         <is>
-          <t>PASS (verified against build) — state machine idle, source=phase0, honeypot intact, 0 console errors | 2026-09-28: PASS (verified against build) — npm run build clean (20 pages); dist/phase0/index.html references phase0.js?v=phase3 and dist/js/phase0.js == source. Stub-DOM harness running the BUILT file: 8/8 scenarios pass (typo, empty, server invalid_email, 429, 502, non-JSON 500, network failure, 200 success; valid keystroke clears the error). Control: the same harness on the pre-fix file fails 4/8, matching the live observation. Dev servers cannot start in unattended runs and the live CSP blocks script injection, so no in-browser retest; live-verifies on the first SCRUB after merge.</t>
+          <t>PASS (verified against build) — state machine idle, source=phase0, honeypot intact, 0 console errors | 2026-09-28: PASS (verified against build) — npm run build clean (20 pages); dist/phase0/index.html references phase0.js?v=phase3 and dist/js/phase0.js == source. Stub-DOM harness running the BUILT file: 8/8 scenarios pass (typo, empty, server invalid_email, 429, 502, non-JSON 500, network failure, 200 success; valid keystroke clears the error). Control: the same harness on the pre-fix file fails 4/8, matching the live observation. Dev servers cannot start in unattended runs and the live CSP blocks script injection, so no in-browser retest; live-verifies on the first SCRUB after merge. | 2026-09-29: still awaits merge; live /phase0/ unchanged (95e2a73).</t>
         </is>
       </c>
     </row>
@@ -4762,7 +4762,7 @@
       </c>
       <c r="K83" s="6" t="inlineStr">
         <is>
-          <t>PASS (2026-09-24, verified against build) — netlify.toml parses (29 redirects); parity test published slugs == /words/&lt;slug&gt; rule set, 17/17, 0 orphans, 0 dupes, no force on any /words/&lt;slug&gt; rule; npm run build clean (20 pages). Live behaviour was already a single 301 and is unchanged by the rule. Note for the expected column: a missing rule here showed up as parity drift, not a 404. | 2026-09-27: live parity re-checked — all 17 /words/&lt;slug&gt; return a single 301 to the slash canonical; /about, /brand, /phase0 likewise. Fix still awaits merge. | 2026-09-28: live parity 17/17 unchanged; fix still awaits merge.</t>
+          <t>PASS (2026-09-24, verified against build) — netlify.toml parses (29 redirects); parity test published slugs == /words/&lt;slug&gt; rule set, 17/17, 0 orphans, 0 dupes, no force on any /words/&lt;slug&gt; rule; npm run build clean (20 pages). Live behaviour was already a single 301 and is unchanged by the rule. Note for the expected column: a missing rule here showed up as parity drift, not a 404. | 2026-09-27: live parity re-checked — all 17 /words/&lt;slug&gt; return a single 301 to the slash canonical; /about, /brand, /phase0 likewise. Fix still awaits merge. | 2026-09-28: live parity 17/17 unchanged; fix still awaits merge. | 2026-09-29: live parity 17/17 (single 301 to the slash canonical); fix still awaits merge.</t>
         </is>
       </c>
     </row>
@@ -6319,7 +6319,7 @@
       </c>
       <c r="H111" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-09-24) — .rail-cta's base rule is background: var(--ink); color: var(--bg), and a.plate-lead:hover .rail-cta swaps only the background to var(--accent). In light mode that is cream on #c00 (#f4f4f1, ~5.2:1, passes). In dark mode --bg is #060606, so the hovered chip renders near-black 'READ →' on #c00 at 3.44:1 at 12px/700, under the 4.5:1 floor (WCAG 1.4.3). Measured under a REAL pointer hover after a 3s settle (a.plate-lead:hover true; computed rgb(6,6,6) on rgb(204,0,0)) and confirmed on screenshot. It is the same defect class F83 closed for .latest-cta and .hero-link.primary on 2026-08-13; F83's scope note said only those two controls invert onto the fill, which missed this third one. Present since the lead plate shipped (d1f8e7e, 2026-04-21), so NEW to the ledger, not a regression. /brand/ renders .plate-lead and loads home-augment.css, so it carries the same defect. | 2026-09-25: still present LIVE — live home-augment.css is phase34 without the rule; fix sits on the unmerged stacked branch (now qa/fixes-20260925). Awaiting Dexter's merge; not re-counted as new. | 2026-09-28: still present LIVE — real pointer hover, dark mode, 3s settle: .rail-cta rgb(6,6,6) on rgb(204,0,0) = 3.44:1 (screenshot). A 1s read caught the chip mid-transition on --ink; re-measured before concluding. Awaiting Dexter's merge; not re-counted as new.</t>
+          <t>ISSUE/High (2026-09-24) — .rail-cta's base rule is background: var(--ink); color: var(--bg), and a.plate-lead:hover .rail-cta swaps only the background to var(--accent). In light mode that is cream on #c00 (#f4f4f1, ~5.2:1, passes). In dark mode --bg is #060606, so the hovered chip renders near-black 'READ →' on #c00 at 3.44:1 at 12px/700, under the 4.5:1 floor (WCAG 1.4.3). Measured under a REAL pointer hover after a 3s settle (a.plate-lead:hover true; computed rgb(6,6,6) on rgb(204,0,0)) and confirmed on screenshot. It is the same defect class F83 closed for .latest-cta and .hero-link.primary on 2026-08-13; F83's scope note said only those two controls invert onto the fill, which missed this third one. Present since the lead plate shipped (d1f8e7e, 2026-04-21), so NEW to the ledger, not a regression. /brand/ renders .plate-lead and loads home-augment.css, so it carries the same defect. | 2026-09-25: still present LIVE — live home-augment.css is phase34 without the rule; fix sits on the unmerged stacked branch (now qa/fixes-20260925). Awaiting Dexter's merge; not re-counted as new. | 2026-09-28: still present LIVE — real pointer hover, dark mode, 3s settle: .rail-cta rgb(6,6,6) on rgb(204,0,0) = 3.44:1 (screenshot). A 1s read caught the chip mid-transition on --ink; re-measured before concluding. Awaiting Dexter's merge; not re-counted as new. | 2026-09-29: still present LIVE — real pointer hover, dark mode (real toggle click, 2s settle), 3s hover settle: .rail-cta rgb(6,6,6) on rgb(204,0,0) = 3.44:1 (screenshot). Awaiting Dexter's merge; not re-counted as new.</t>
         </is>
       </c>
       <c r="I111" s="6" t="inlineStr">
@@ -6334,7 +6334,7 @@
       </c>
       <c r="K111" s="6" t="inlineStr">
         <is>
-          <t>PASS (2026-09-24, verified against build + rule injected on live) — npm run build clean; dist/css/home-augment.css carries the new selector; dist/index.html and dist/brand/index.html both reference home-augment.css?v=phase40. Dev servers cannot start in unattended runs, so the fix rule was applied to the live homepage with insertRule on the loaded home-augment sheet: dark mode, real pointer hover, a.plate-lead:hover true -&gt; .rail-cta rgb(243,240,232) on rgb(204,0,0) = 5.17:1 (screenshot shows a cream 'READ →'). deleteRule restored the sheet and a re-measure read 3.44:1 again, proving the page went back to its original state. Light-mode hover unchanged (rule is dark-scoped): rgb(244,244,241) on #c00. Sibling hover controls (.latest-cta, .hero-link.primary) re-measured 5.17:1, unaffected. Live-verifies on the first SCRUB after merge. | 2026-09-26: still awaits merge — origin/main and the live deploy (6ab794f1, 09-26 09:48Z) remain on 95e2a73, so the live chip is still the pre-fix 3.44:1 on dark-mode hover. | 2026-09-27: still awaits merge — origin/main and the live deploy (6ab794f1, 09-26 09:48Z) remain on 95e2a73; the live home-augment.css?v=phase34 carries no dark-mode :hover .rail-cta rule. Not re-counted as new. | 2026-09-28: still awaits merge — origin/main and the live deploy (2026-09-27 10:29Z) remain on 95e2a73.</t>
+          <t>PASS (2026-09-24, verified against build + rule injected on live) — npm run build clean; dist/css/home-augment.css carries the new selector; dist/index.html and dist/brand/index.html both reference home-augment.css?v=phase40. Dev servers cannot start in unattended runs, so the fix rule was applied to the live homepage with insertRule on the loaded home-augment sheet: dark mode, real pointer hover, a.plate-lead:hover true -&gt; .rail-cta rgb(243,240,232) on rgb(204,0,0) = 5.17:1 (screenshot shows a cream 'READ →'). deleteRule restored the sheet and a re-measure read 3.44:1 again, proving the page went back to its original state. Light-mode hover unchanged (rule is dark-scoped): rgb(244,244,241) on #c00. Sibling hover controls (.latest-cta, .hero-link.primary) re-measured 5.17:1, unaffected. Live-verifies on the first SCRUB after merge. | 2026-09-26: still awaits merge — origin/main and the live deploy (6ab794f1, 09-26 09:48Z) remain on 95e2a73, so the live chip is still the pre-fix 3.44:1 on dark-mode hover. | 2026-09-27: still awaits merge — origin/main and the live deploy (6ab794f1, 09-26 09:48Z) remain on 95e2a73; the live home-augment.css?v=phase34 carries no dark-mode :hover .rail-cta rule. Not re-counted as new. | 2026-09-28: still awaits merge — origin/main and the live deploy (2026-09-27 10:29Z) remain on 95e2a73. | 2026-09-29: still awaits merge — origin/main and the live deploy (2026-09-28 11:37Z daily rebuild) remain on 95e2a73.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
audit(ledger): 2026-09-30 scrub — clean site, F17-F26 rotation all PASS
Wednesday rotation, scrub-only (no FAIL/ISSUE opened, FIX/RETEST skipped).
Live = GitHub main = 95e2a73, zero drift. F108 (High), F80 (Low) and F53
(Medium) remain fixed on the unmerged qa/fixes-20260924..0928 branches.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -1444,7 +1444,7 @@
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>PASS — robots.txt Allow / + Sitemap → sitemap-index.xml | 2026-08-13 re-verified live: /robots.txt 200, Sitemap directive -&gt; https://imjustdex.com/sitemap-index.xml. | 2026-08-25 re-verified live: robots.txt = "User-agent: *\nAllow: /\n\nSitemap: https://imjustdex.com/sitemap-index.xml". /DESIGN-SYSTEM.md correctly 404s. | 2026-08-27 re-verified live: robots.txt Allow / + Sitemap → sitemap-index.xml. | 2026-09-01 re-verified live: robots.txt is 'User-agent: * / Allow: / / Sitemap: https://imjustdex.com/sitemap-index.xml'. /DESIGN-SYSTEM.md still 404s (the only thing keeping the doc unexposed). | 2026-09-06 re-verified live: robots.txt is 'User-agent: * / Allow: / / Sitemap: https://imjustdex.com/sitemap-index.xml'. | 2026-09-11 re-verified live: robots.txt = 'User-agent: * / Allow: / / Sitemap: https://imjustdex.com/sitemap-index.xml'. | 2026-09-28: live: Allow / + Sitemap -&gt; sitemap-index.xml.</t>
+          <t>PASS — robots.txt Allow / + Sitemap → sitemap-index.xml | 2026-08-13 re-verified live: /robots.txt 200, Sitemap directive -&gt; https://imjustdex.com/sitemap-index.xml. | 2026-08-25 re-verified live: robots.txt = "User-agent: *\nAllow: /\n\nSitemap: https://imjustdex.com/sitemap-index.xml". /DESIGN-SYSTEM.md correctly 404s. | 2026-08-27 re-verified live: robots.txt Allow / + Sitemap → sitemap-index.xml. | 2026-09-01 re-verified live: robots.txt is 'User-agent: * / Allow: / / Sitemap: https://imjustdex.com/sitemap-index.xml'. /DESIGN-SYSTEM.md still 404s (the only thing keeping the doc unexposed). | 2026-09-06 re-verified live: robots.txt is 'User-agent: * / Allow: / / Sitemap: https://imjustdex.com/sitemap-index.xml'. | 2026-09-11 re-verified live: robots.txt = 'User-agent: * / Allow: / / Sitemap: https://imjustdex.com/sitemap-index.xml'. | 2026-09-28: live: Allow / + Sitemap -&gt; sitemap-index.xml. | 2026-09-30: live: robots.txt 200 = 'User-agent: * / Allow: /' + Sitemap -&gt; https://imjustdex.com/sitemap-index.xml.</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr"/>
@@ -1493,7 +1493,7 @@
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>PASS — sitemap-0.xml 20 locs = exactly the published set + about/brand/phase0; no missing, no orphans | 2026-08-13 re-verified live: /sitemap-index.xml -&gt; sitemap-0.xml; sitemap-0 lists 20 URLs covering all 16 articles + /, /about/, /brand/, /phase0/. Zero missing. | 2026-08-25 re-verified live: sitemap-index.xml references sitemap-0.xml; sitemap-0.xml carries exactly 20 locs = 16 articles + /, /about/, /brand/, /phase0/. The drafted essay is correctly absent. | 2026-08-27 re-verified live: sitemap-0.xml 20 locs; every homepage-linked route plus /about/ /brand/ /phase0/ present. | 2026-09-01 re-verified live: /sitemap-index.xml points to sitemap-0.xml; sitemap-0.xml holds exactly 21 URLs — the 17 live articles plus /, /about/, /brand/, /phase0/. Zero missing, zero extra. The drafted entry before-i-had-the-words is correctly absent. | 2026-09-06 re-verified live: sitemap-index.xml points at sitemap-0.xml; sitemap-0.xml carries 21 URLs and includes all 17 articles plus /, /about/, /brand/, /phase0/. | 2026-09-11 re-verified live: sitemap-index → sitemap-0; 21 locs = 17 articles + /, /about/, /brand/, /phase0/. No drafts leaked (before-i-had-the-words absent). | 2026-09-28: live: sitemap-0.xml 21 locs = 17 essays + home/about/brand/phase0; throwaway fixture build: a future-dated entry is excluded.</t>
+          <t>PASS — sitemap-0.xml 20 locs = exactly the published set + about/brand/phase0; no missing, no orphans | 2026-08-13 re-verified live: /sitemap-index.xml -&gt; sitemap-0.xml; sitemap-0 lists 20 URLs covering all 16 articles + /, /about/, /brand/, /phase0/. Zero missing. | 2026-08-25 re-verified live: sitemap-index.xml references sitemap-0.xml; sitemap-0.xml carries exactly 20 locs = 16 articles + /, /about/, /brand/, /phase0/. The drafted essay is correctly absent. | 2026-08-27 re-verified live: sitemap-0.xml 20 locs; every homepage-linked route plus /about/ /brand/ /phase0/ present. | 2026-09-01 re-verified live: /sitemap-index.xml points to sitemap-0.xml; sitemap-0.xml holds exactly 21 URLs — the 17 live articles plus /, /about/, /brand/, /phase0/. Zero missing, zero extra. The drafted entry before-i-had-the-words is correctly absent. | 2026-09-06 re-verified live: sitemap-index.xml points at sitemap-0.xml; sitemap-0.xml carries 21 URLs and includes all 17 articles plus /, /about/, /brand/, /phase0/. | 2026-09-11 re-verified live: sitemap-index → sitemap-0; 21 locs = 17 articles + /, /about/, /brand/, /phase0/. No drafts leaked (before-i-had-the-words absent). | 2026-09-28: live: sitemap-0.xml 21 locs = 17 essays + home/about/brand/phase0; throwaway fixture build: a future-dated entry is excluded. | 2026-09-30: live: sitemap-index -&gt; sitemap-0; 21 locs = 17 published articles + / /about/ /brand/ /phase0/, no orphans; priorities home 1.0 / about 0.7 / phase0 0.9 / brand 0.5 / articles 0.8; unmatched route not listed.</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr"/>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>404 half PASS (noindex,nofollow live). Coming-soon half PENDING — no upcoming entry exists to render one | 2026-08-25: 404 half re-verified live (meta robots noindex,nofollow present, bespoke body served at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one. | 2026-09-01 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one. | 2026-09-11: 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body at HTTP 200). Coming-soon half still PENDING — 17 published entries, all past-dated, so isUpcomingData() is false everywhere and no ComingSoonLayout renders. | 2026-09-19: 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body, HTTP 404 on unmatched route). Coming-soon half still PENDING — 17 published entries, all past-dated; the untracked before-i-had-the-words.mdx in Dexter's working tree is still status 'drafted'. | 2026-09-23: 404 half re-verified live (noindex, nofollow). Coming-soon half still PENDING — 17/17 entries status published, no upcoming entry to render. | 2026-09-25: still PENDING — 17/17 entries status published and past-dated, no upcoming entry to render. 404 half re-verified live: meta robots noindex present, bespoke body, unmatched route 404. | 2026-09-28: 404 half re-verified live (noindex, nofollow). Coming-soon half BUILD-VERIFIED via a throwaway future-dated fixture in a scratch copy (never committed): ComingSoonLayout emits &lt;meta name=robots content=noindex&gt;.</t>
+          <t>404 half PASS (noindex,nofollow live). Coming-soon half PENDING — no upcoming entry exists to render one | 2026-08-25: 404 half re-verified live (meta robots noindex,nofollow present, bespoke body served at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one. | 2026-09-01 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one. | 2026-09-11: 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body at HTTP 200). Coming-soon half still PENDING — 17 published entries, all past-dated, so isUpcomingData() is false everywhere and no ComingSoonLayout renders. | 2026-09-19: 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body, HTTP 404 on unmatched route). Coming-soon half still PENDING — 17 published entries, all past-dated; the untracked before-i-had-the-words.mdx in Dexter's working tree is still status 'drafted'. | 2026-09-23: 404 half re-verified live (noindex, nofollow). Coming-soon half still PENDING — 17/17 entries status published, no upcoming entry to render. | 2026-09-25: still PENDING — 17/17 entries status published and past-dated, no upcoming entry to render. 404 half re-verified live: meta robots noindex present, bespoke body, unmatched route 404. | 2026-09-28: 404 half re-verified live (noindex, nofollow). Coming-soon half BUILD-VERIFIED via a throwaway future-dated fixture in a scratch copy (never committed): ComingSoonLayout emits &lt;meta name=robots content=noindex&gt;. | 2026-09-30: live: 404 half re-verified live (bespoke body, noindex). Coming-soon half unchanged since the 09-28 fixture build — 17/17 entries still published and past-dated, no upcoming entry to render live.</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr"/>
@@ -1595,7 +1595,7 @@
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>PASS — Entry No. 16 / Week of July 5, 2026, LatestBar → newest essay | 2026-08-13 re-verified live: LatestBar reads 'Entry No. 16 / Week of July 5, 2026' and links to /words/send-someone-else/ (the newest). NOTE: its .latest-tag chip is the F77 finding this run. | 2026-08-25 re-verified live: issue head renders "Entry No. 16" / "Week of July 5, 2026" from the lead; standfirst links /words/send-someone-else/. | 2026-08-27 re-verified live: issue head 'Entry No. 16 / Week of July 5, 2026', LatestBar → send-someone-else. | 2026-09-11 re-verified live: LatestBar: 'Entry No. 17' (= 17 published essays), 'Week of August 31, 2026', latest link → /words/the-weight-of-my-no/. | 2026-09-28: live: 'Entry No. 17', 'Week of August 31, 2026', Latest -&gt; the-weight-of-my-no, 'Faith · Aug 31 · 8 min'.</t>
+          <t>PASS — Entry No. 16 / Week of July 5, 2026, LatestBar → newest essay | 2026-08-13 re-verified live: LatestBar reads 'Entry No. 16 / Week of July 5, 2026' and links to /words/send-someone-else/ (the newest). NOTE: its .latest-tag chip is the F77 finding this run. | 2026-08-25 re-verified live: issue head renders "Entry No. 16" / "Week of July 5, 2026" from the lead; standfirst links /words/send-someone-else/. | 2026-08-27 re-verified live: issue head 'Entry No. 16 / Week of July 5, 2026', LatestBar → send-someone-else. | 2026-09-11 re-verified live: LatestBar: 'Entry No. 17' (= 17 published essays), 'Week of August 31, 2026', latest link → /words/the-weight-of-my-no/. | 2026-09-28: live: 'Entry No. 17', 'Week of August 31, 2026', Latest -&gt; the-weight-of-my-no, 'Faith · Aug 31 · 8 min'. | 2026-09-30: live: LatestBar reads 'Entry No. 17' / 'Week of August 31, 2026'; .issue-latest links to /words/the-weight-of-my-no/ (newest).</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr"/>
@@ -1648,7 +1648,7 @@
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>PASS — IdentityHero renders; hero copy contrast 5.17:1 (AA large) | 2026-08-27 re-verified live: IdentityHero renders (screenshot-confirmed in both modes). | 2026-09-11 re-verified live: IdentityHero: name + 'ImJustDex' render; hero links → /about/ and #subscribe-manifesto. | 2026-09-28: live: hero name/sub/tagline/bio, 'Read the About' -&gt; /about/, 'Subscribe' -&gt; #subscribe-manifesto.</t>
+          <t>PASS — IdentityHero renders; hero copy contrast 5.17:1 (AA large) | 2026-08-27 re-verified live: IdentityHero renders (screenshot-confirmed in both modes). | 2026-09-11 re-verified live: IdentityHero: name + 'ImJustDex' render; hero links → /about/ and #subscribe-manifesto. | 2026-09-28: live: hero name/sub/tagline/bio, 'Read the About' -&gt; /about/, 'Subscribe' -&gt; #subscribe-manifesto. | 2026-09-30: live: IdentityHero renders 'Dexter Jakes' + 'ImJustDex' + tagline + bio; links -&gt; /about/ and #subscribe-manifesto.</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr"/>
@@ -1697,7 +1697,7 @@
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>PASS — Faith 13 / Identity 09 / Art 03, verified against frontmatter lanes; 16 articles | 2026-08-13 re-verified live: lane-index counts Faith 13 / Identity 09 / Art 03 — non-negative, zero-padded, and consistent with 16 essays counted per lane (15 .plate-lane chips + 1 .lead-badge-lane). | 2026-08-25 re-verified live: lane counts render Faith 13 / Identity 09 / Art 03 — matches the frontmatter tally across the 16 tracked essays exactly (multi-lane counted per lane). | 2026-08-27 re-verified live: lane counts Faith 13 / Identity 09 / Art 03. | 2026-09-01 re-verified live: lane-index reads Faith 14 / Identity 10 / Art 03 — non-negative integers summing to 27 across 17 essays (multi-lane counted per lane). Cross-checked against the filter: selecting Faith reveals exactly 14 articles. | 2026-09-06 re-verified live: lane index reads Faith 14 / Identity 10 / Art 03 (sum 27 across 17 essays, multi-lane counted per lane). | 2026-09-11 re-verified live: lane counts Faith 14 / Identity 10 / Art 03; sum 27 over 17 articles (multi-lane essays count per lane), all non-negative integers. | 2026-09-28: live: Faith 14 / Identity 10 / Art 03 essays (no zero lane, so the queued state is not exercised).</t>
+          <t>PASS — Faith 13 / Identity 09 / Art 03, verified against frontmatter lanes; 16 articles | 2026-08-13 re-verified live: lane-index counts Faith 13 / Identity 09 / Art 03 — non-negative, zero-padded, and consistent with 16 essays counted per lane (15 .plate-lane chips + 1 .lead-badge-lane). | 2026-08-25 re-verified live: lane counts render Faith 13 / Identity 09 / Art 03 — matches the frontmatter tally across the 16 tracked essays exactly (multi-lane counted per lane). | 2026-08-27 re-verified live: lane counts Faith 13 / Identity 09 / Art 03. | 2026-09-01 re-verified live: lane-index reads Faith 14 / Identity 10 / Art 03 — non-negative integers summing to 27 across 17 essays (multi-lane counted per lane). Cross-checked against the filter: selecting Faith reveals exactly 14 articles. | 2026-09-06 re-verified live: lane index reads Faith 14 / Identity 10 / Art 03 (sum 27 across 17 essays, multi-lane counted per lane). | 2026-09-11 re-verified live: lane counts Faith 14 / Identity 10 / Art 03; sum 27 over 17 articles (multi-lane essays count per lane), all non-negative integers. | 2026-09-28: live: Faith 14 / Identity 10 / Art 03 essays (no zero lane, so the queued state is not exercised). | 2026-09-30: live: lane index Faith 14 / Identity 10 / Art 03 essays (zero-padded), consistent with 17 essays counted per lane; no lane at 0, so no .lane-cell-queued rendered.</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr"/>
@@ -1750,7 +1750,7 @@
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: Faith 13/13, Identity 9/9, Art 3/3 with zero non-matching plates in any filtered view; while filtered the .earlier-more-wrap computes display:none, 0 client rects, offsetHeight 0 (unreachable by mouse or keyboard). The ab07b15 fix holds in production. | 2026-08-16 re-verified live: all three lanes re-verified live: Faith 13, Identity 9, Art 3 — exactly matching the lane-index counts. Verified against the real filter key (data-lane, space-separated) rather than the visible chips: all 9 identity plates carry 'identity' in data-lane. While filtered, .earlier-more-wrap computes display:none with 0 client rects; clearing restores display:flex. | 2026-08-27 re-verified live: real pointer clicks: Faith 13, Identity 9, Art 3, re-click clears to the default 8; aria-pressed single-select correct. | 2026-09-01 re-verified live: .lane-cell[data-lane=faith] click sets aria-pressed=true and reveals exactly 14 articles; clicking again returns aria-pressed=false and the default 7-article view. | 2026-09-06 re-verified live: clicking the Art lane cell filtered the cascade 7 -&gt; 3 visible articles (Music That Raised Me, Useful Is Not the Same, Groan Beneath the Song), aria-pressed=true, and a second click restored 7. | 2026-09-11 re-verified live: lane filter 'art' → 3 visible articles, matching its announced count; aria-pressed true→false; clearing restores 7. | 2026-09-28: live: Faith -&gt; aria-pressed true, 14 visible, all data-lane faith; re-click clears (7 visible); Art -&gt; 3.</t>
+          <t>PASS — live-verified 2026-08-10: Faith 13/13, Identity 9/9, Art 3/3 with zero non-matching plates in any filtered view; while filtered the .earlier-more-wrap computes display:none, 0 client rects, offsetHeight 0 (unreachable by mouse or keyboard). The ab07b15 fix holds in production. | 2026-08-16 re-verified live: all three lanes re-verified live: Faith 13, Identity 9, Art 3 — exactly matching the lane-index counts. Verified against the real filter key (data-lane, space-separated) rather than the visible chips: all 9 identity plates carry 'identity' in data-lane. While filtered, .earlier-more-wrap computes display:none with 0 client rects; clearing restores display:flex. | 2026-08-27 re-verified live: real pointer clicks: Faith 13, Identity 9, Art 3, re-click clears to the default 8; aria-pressed single-select correct. | 2026-09-01 re-verified live: .lane-cell[data-lane=faith] click sets aria-pressed=true and reveals exactly 14 articles; clicking again returns aria-pressed=false and the default 7-article view. | 2026-09-06 re-verified live: clicking the Art lane cell filtered the cascade 7 -&gt; 3 visible articles (Music That Raised Me, Useful Is Not the Same, Groan Beneath the Song), aria-pressed=true, and a second click restored 7. | 2026-09-11 re-verified live: lane filter 'art' → 3 visible articles, matching its announced count; aria-pressed true→false; clearing restores 7. | 2026-09-28: live: Faith -&gt; aria-pressed true, 14 visible, all data-lane faith; re-click clears (7 visible); Art -&gt; 3. | 2026-09-30: live: lane-filter.js exercised in-browser: Faith 14/14, Identity 10/10, Art 3/3 visible with 0 non-matching; aria-pressed true, .plates data-filter set, live region 'Filtered to &lt;lane&gt;. N essays.', .earlier-more-wrap display:none while filtered; second click clears (aria-pressed false, 10 hidden restored, data-filter removed).</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr"/>
@@ -1803,7 +1803,7 @@
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>PASS — lead plate = send-someone-else (newest published) | 2026-08-25 re-verified live: lead plate renders send-someone-else with correct eyebrow, deck and 16 min read. | 2026-08-27 re-verified live: lead plate = send-someone-else. | 2026-09-11 re-verified live: LeadPlate renders the newest essay with Latest badge and Read CTA, href /words/the-weight-of-my-no/. | 2026-09-28: live: lead = the-weight-of-my-no with Latest badge, Faith, &lt;time 2026-08-31&gt;, 8 min, Read -&gt;.</t>
+          <t>PASS — lead plate = send-someone-else (newest published) | 2026-08-25 re-verified live: lead plate renders send-someone-else with correct eyebrow, deck and 16 min read. | 2026-08-27 re-verified live: lead plate = send-someone-else. | 2026-09-11 re-verified live: LeadPlate renders the newest essay with Latest badge and Read CTA, href /words/the-weight-of-my-no/. | 2026-09-28: live: lead = the-weight-of-my-no with Latest badge, Faith, &lt;time 2026-08-31&gt;, 8 min, Read -&gt;. | 2026-09-30: live: lead plate = .plate-lead for the-weight-of-my-no (newest): Latest badge, Faith, Aug 31, 8 min read, title, deck, Read -&gt; CTA.</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr"/>
@@ -1852,7 +1852,7 @@
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>PASS — 'This Month' = show-me-your-glory (same month as lead) | 2026-08-27 re-verified live: row heads 'This Week' (01, lead) and 'This Month' (02) both render as authored. | 2026-09-18 re-verified live: 'This Month' correctly hidden — no other essay shares the lead's month (Aug 2026); row heads read 01 This Week / 02 Earlier. | 2026-09-28: live: correctly hidden — no other essay shares the lead's month (Aug 2026); row heads read 'Latest', 'Earlier'.</t>
+          <t>PASS — 'This Month' = show-me-your-glory (same month as lead) | 2026-08-27 re-verified live: row heads 'This Week' (01, lead) and 'This Month' (02) both render as authored. | 2026-09-18 re-verified live: 'This Month' correctly hidden — no other essay shares the lead's month (Aug 2026); row heads read 01 This Week / 02 Earlier. | 2026-09-28: live: correctly hidden — no other essay shares the lead's month (Aug 2026); row heads read 'Latest', 'Earlier'. | 2026-09-30: live: 'This Month' correctly hidden — no other essay shares the lead's month (Aug 2026); row heads '01 Latest', '02 Earlier'.</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr"/>
@@ -1901,7 +1901,7 @@
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>PASS — 'Earlier' = 14, 6 visible + 8 overflow | 2026-08-27 re-verified live: 8 of 16 plates visible by default, 8 under the overflow. | 2026-09-18 re-verified live: 'Earlier' = 16, 6 visible + 10 under the overflow; 7 of 17 plates visible by default. | 2026-09-28: live: 'Earlier' numbered 02 (no This Month), 16 essays: 6 visible + 10 in .earlier-more.</t>
+          <t>PASS — 'Earlier' = 14, 6 visible + 8 overflow | 2026-08-27 re-verified live: 8 of 16 plates visible by default, 8 under the overflow. | 2026-09-18 re-verified live: 'Earlier' = 16, 6 visible + 10 under the overflow; 7 of 17 plates visible by default. | 2026-09-28: live: 'Earlier' numbered 02 (no This Month), 16 essays: 6 visible + 10 in .earlier-more. | 2026-09-30: live: 'Earlier' = 16 under RowHead 02 (no This Month); 6 visible + 10 under .earlier-more[hidden]; 7 of 17 plates visible by default.</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr"/>

</xml_diff>

<commit_message>
audit(ledger): F53, F80, F108 verified live after the 561435c merge
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -3319,7 +3319,7 @@
       </c>
       <c r="K56" s="6" t="inlineStr">
         <is>
-          <t>PASS (verified against build) — state machine idle, source=phase0, honeypot intact, 0 console errors | 2026-09-28: PASS (verified against build) — npm run build clean (20 pages); dist/phase0/index.html references phase0.js?v=phase3 and dist/js/phase0.js == source. Stub-DOM harness running the BUILT file: 8/8 scenarios pass (typo, empty, server invalid_email, 429, 502, non-JSON 500, network failure, 200 success; valid keystroke clears the error). Control: the same harness on the pre-fix file fails 4/8, matching the live observation. Dev servers cannot start in unattended runs and the live CSP blocks script injection, so no in-browser retest; live-verifies on the first SCRUB after merge. | 2026-09-29: still awaits merge; live /phase0/ unchanged (95e2a73).</t>
+          <t>PASS (verified against build) — state machine idle, source=phase0, honeypot intact, 0 console errors | 2026-09-28: PASS (verified against build) — npm run build clean (20 pages); dist/phase0/index.html references phase0.js?v=phase3 and dist/js/phase0.js == source. Stub-DOM harness running the BUILT file: 8/8 scenarios pass (typo, empty, server invalid_email, 429, 502, non-JSON 500, network failure, 200 success; valid keystroke clears the error). Control: the same harness on the pre-fix file fails 4/8, matching the live observation. Dev servers cannot start in unattended runs and the live CSP blocks script injection, so no in-browser retest; live-verifies on the first SCRUB after merge. | 2026-09-29: still awaits merge; live /phase0/ unchanged (95e2a73). | 2026-09-30: PASS LIVE after merge (561435c) — /phase0/ serves phase0.js?v=phase3; client-invalid 'notanemail' sets aria-invalid; server-rejected 'healthscrub@imjustdex' (passes type=email, fails server regex) shows 'That email didn’t look right. Try it again.' with button restored to 'Send Prompt', not the outage line + Retry.</t>
         </is>
       </c>
     </row>
@@ -4762,7 +4762,7 @@
       </c>
       <c r="K83" s="6" t="inlineStr">
         <is>
-          <t>PASS (2026-09-24, verified against build) — netlify.toml parses (29 redirects); parity test published slugs == /words/&lt;slug&gt; rule set, 17/17, 0 orphans, 0 dupes, no force on any /words/&lt;slug&gt; rule; npm run build clean (20 pages). Live behaviour was already a single 301 and is unchanged by the rule. Note for the expected column: a missing rule here showed up as parity drift, not a 404. | 2026-09-27: live parity re-checked — all 17 /words/&lt;slug&gt; return a single 301 to the slash canonical; /about, /brand, /phase0 likewise. Fix still awaits merge. | 2026-09-28: live parity 17/17 unchanged; fix still awaits merge. | 2026-09-29: live parity 17/17 (single 301 to the slash canonical); fix still awaits merge.</t>
+          <t>PASS (2026-09-24, verified against build) — netlify.toml parses (29 redirects); parity test published slugs == /words/&lt;slug&gt; rule set, 17/17, 0 orphans, 0 dupes, no force on any /words/&lt;slug&gt; rule; npm run build clean (20 pages). Live behaviour was already a single 301 and is unchanged by the rule. Note for the expected column: a missing rule here showed up as parity drift, not a 404. | 2026-09-27: live parity re-checked — all 17 /words/&lt;slug&gt; return a single 301 to the slash canonical; /about, /brand, /phase0 likewise. Fix still awaits merge. | 2026-09-28: live parity 17/17 unchanged; fix still awaits merge. | 2026-09-29: live parity 17/17 (single 301 to the slash canonical); fix still awaits merge. | 2026-09-30: PASS LIVE after merge (561435c) — /words/the-weight-of-my-no -&gt; 301 -&gt; /words/the-weight-of-my-no/.</t>
         </is>
       </c>
     </row>
@@ -6334,7 +6334,7 @@
       </c>
       <c r="K111" s="6" t="inlineStr">
         <is>
-          <t>PASS (2026-09-24, verified against build + rule injected on live) — npm run build clean; dist/css/home-augment.css carries the new selector; dist/index.html and dist/brand/index.html both reference home-augment.css?v=phase40. Dev servers cannot start in unattended runs, so the fix rule was applied to the live homepage with insertRule on the loaded home-augment sheet: dark mode, real pointer hover, a.plate-lead:hover true -&gt; .rail-cta rgb(243,240,232) on rgb(204,0,0) = 5.17:1 (screenshot shows a cream 'READ →'). deleteRule restored the sheet and a re-measure read 3.44:1 again, proving the page went back to its original state. Light-mode hover unchanged (rule is dark-scoped): rgb(244,244,241) on #c00. Sibling hover controls (.latest-cta, .hero-link.primary) re-measured 5.17:1, unaffected. Live-verifies on the first SCRUB after merge. | 2026-09-26: still awaits merge — origin/main and the live deploy (6ab794f1, 09-26 09:48Z) remain on 95e2a73, so the live chip is still the pre-fix 3.44:1 on dark-mode hover. | 2026-09-27: still awaits merge — origin/main and the live deploy (6ab794f1, 09-26 09:48Z) remain on 95e2a73; the live home-augment.css?v=phase34 carries no dark-mode :hover .rail-cta rule. Not re-counted as new. | 2026-09-28: still awaits merge — origin/main and the live deploy (2026-09-27 10:29Z) remain on 95e2a73. | 2026-09-29: still awaits merge — origin/main and the live deploy (2026-09-28 11:37Z daily rebuild) remain on 95e2a73.</t>
+          <t>PASS (2026-09-24, verified against build + rule injected on live) — npm run build clean; dist/css/home-augment.css carries the new selector; dist/index.html and dist/brand/index.html both reference home-augment.css?v=phase40. Dev servers cannot start in unattended runs, so the fix rule was applied to the live homepage with insertRule on the loaded home-augment sheet: dark mode, real pointer hover, a.plate-lead:hover true -&gt; .rail-cta rgb(243,240,232) on rgb(204,0,0) = 5.17:1 (screenshot shows a cream 'READ →'). deleteRule restored the sheet and a re-measure read 3.44:1 again, proving the page went back to its original state. Light-mode hover unchanged (rule is dark-scoped): rgb(244,244,241) on #c00. Sibling hover controls (.latest-cta, .hero-link.primary) re-measured 5.17:1, unaffected. Live-verifies on the first SCRUB after merge. | 2026-09-26: still awaits merge — origin/main and the live deploy (6ab794f1, 09-26 09:48Z) remain on 95e2a73, so the live chip is still the pre-fix 3.44:1 on dark-mode hover. | 2026-09-27: still awaits merge — origin/main and the live deploy (6ab794f1, 09-26 09:48Z) remain on 95e2a73; the live home-augment.css?v=phase34 carries no dark-mode :hover .rail-cta rule. Not re-counted as new. | 2026-09-28: still awaits merge — origin/main and the live deploy (2026-09-27 10:29Z) remain on 95e2a73. | 2026-09-29: still awaits merge — origin/main and the live deploy (2026-09-28 11:37Z daily rebuild) remain on 95e2a73. | 2026-09-30: PASS LIVE after merge (561435c) — home-augment.css?v=phase40 served; real pointer hover on a.plate-lead in dark mode: .rail-cta rgb(243,240,232) on rgb(204,0,0) = 5.17:1 (was 3.44:1).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
audit(ledger): 2026-10-01 scrub — F29 opened (texture alternation collision), BLOCKED for Dexter; F27-F34 rotation PASS
Thursday rotation F27-F36. Live = GitHub main = Netlify deploy 1d65448, zero drift.
All HTTP, header, asset, structured-data, feed/sitemap, subscribe and browser checks clean.

F29 -> ISSUE/Medium: /words/gloria/ (auto img-noise) and /words/the-nets/
(frontmatter noise) are adjacent in reading order, breaking the Texture
Alternation Rule. The 08-31 publish shifted archive parity under the two
frontmatter overrides. Not auto-fixed: the fix is a design-intent call;
options A/B/C recorded in the row's p3.

F35/F36: rotation gap (pane hidden, scroll inert), prior PASS carried.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,6 +48,11 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="001A1A1A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="00CC0000"/>
       <sz val="13"/>
     </font>
@@ -63,7 +68,7 @@
       <color rgb="00C0211B"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -87,7 +92,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00F0C24B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00E2E2DE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4B9B5"/>
       </patternFill>
     </fill>
   </fills>
@@ -117,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -135,13 +150,18 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1954,7 +1974,7 @@
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: expand 8→16, collapse 16→8, aria-expanded false↔true and the button label track; collapse state survives a full filter cycle (clear restores the wrap to display:flex). | 2026-08-16 re-verified live: expand 8-&gt;16 and collapse 16-&gt;8 re-verified live; aria-expanded false&lt;-&gt;true and the label tracked ('View Earlier Essays — 8 more' &lt;-&gt; 'Show Less — showing all'); collapse state survived a full filter cycle. | 2026-08-27 re-verified live: real pointer clicks: 8→16→8, aria-expanded false↔true, label and count track. | 2026-09-01 re-verified live: toggle expands 10 hidden articles to 0 hidden, label 'View Earlier Essays — 10 more' -&gt; 'Show Less — showing all', aria-expanded false-&gt;true; collapse restores all three. | 2026-09-06 re-verified live: View Earlier 7 -&gt; 17 -&gt; 7 with label 'View Earlier Essays - 10 more' &lt;-&gt; 'Show Less - showing all' and aria-expanded true/false. | 2026-09-11 re-verified live: toggle 7↔17 articles, label 'View Earlier Essays — 10 more ↓' ↔ 'Show Less — showing all ↑', aria-expanded false↔true. | 2026-09-28: live: 'View Earlier Essays — 10 more ↓' -&gt; 'Show Less — showing all ↑', aria-expanded false-&gt;true-&gt;false, 7-&gt;17-&gt;7 visible.</t>
+          <t>PASS — live-verified 2026-08-10: expand 8→16, collapse 16→8, aria-expanded false↔true and the button label track; collapse state survives a full filter cycle (clear restores the wrap to display:flex). | 2026-08-16 re-verified live: expand 8-&gt;16 and collapse 16-&gt;8 re-verified live; aria-expanded false&lt;-&gt;true and the label tracked ('View Earlier Essays — 8 more' &lt;-&gt; 'Show Less — showing all'); collapse state survived a full filter cycle. | 2026-08-27 re-verified live: real pointer clicks: 8→16→8, aria-expanded false↔true, label and count track. | 2026-09-01 re-verified live: toggle expands 10 hidden articles to 0 hidden, label 'View Earlier Essays — 10 more' -&gt; 'Show Less — showing all', aria-expanded false-&gt;true; collapse restores all three. | 2026-09-06 re-verified live: View Earlier 7 -&gt; 17 -&gt; 7 with label 'View Earlier Essays - 10 more' &lt;-&gt; 'Show Less - showing all' and aria-expanded true/false. | 2026-09-11 re-verified live: toggle 7↔17 articles, label 'View Earlier Essays — 10 more ↓' ↔ 'Show Less — showing all ↑', aria-expanded false↔true. | 2026-09-28: live: 'View Earlier Essays — 10 more ↓' -&gt; 'Show Less — showing all ↑', aria-expanded false-&gt;true-&gt;false, 7-&gt;17-&gt;7 visible. | 2026-10-01 re-verified live: 'View Earlier Essays — 10 more ↓', aria-expanded=false, 10 .earlier-more hidden; click -&gt; 'Show Less — showing all ↑', expanded=true, 0 hidden; re-click restores all three.</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr"/>
@@ -2007,7 +2027,7 @@
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>PASS — 16 plates tile the 12-col grid (lead + wide/secondary/banner rotation, 3 row-plates) | 2026-09-18 re-verified live: 7 visible plates tile the 12-col grid as lead + wide/secondary/banner/secondary/banner/wide; 17 plates total with the 10-plate overflow under View More. | 2026-09-28: live: 17 .plate elements render in the cascade; packer source unchanged since last PASS.</t>
+          <t>PASS — 16 plates tile the 12-col grid (lead + wide/secondary/banner rotation, 3 row-plates) | 2026-09-18 re-verified live: 7 visible plates tile the 12-col grid as lead + wide/secondary/banner/secondary/banner/wide; 17 plates total with the 10-plate overflow under View More. | 2026-09-28: live: 17 .plate elements render in the cascade; packer source unchanged since last PASS. | 2026-10-01 re-verified live: 17 plates: lead + wide/secondary/banner rotation in 12-col rows, trailing plate-row (reckonings); packer source unchanged.</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr"/>
@@ -2056,14 +2076,22 @@
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>PASS — 7 of 15 archive plates carry .plate-image, interleaved with plain (Texture Alternation Rule) | 2026-09-06 re-verified live: eight image plates alternate concrete/lines/noise as designed. NOTE - this run pixel-measured them rather than reading computed styles and found the scrim, not the alternation, at fault; see F101. | 2026-09-11 re-verified live: three homepage image plates alternate img-concrete / img-lines / img-noise across the cascade. | 2026-09-28: live: 8 of 16 archive plates carry .plate-image; source unchanged.</t>
-        </is>
-      </c>
-      <c r="I32" s="6" t="inlineStr"/>
-      <c r="J32" s="4" t="inlineStr"/>
-      <c r="K32" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>ISSUE/Medium (2026-10-01) — Texture Alternation Rule (DESIGN-SYSTEM.md:718, 'adjacent plates must never share the same background treatment… across row boundaries in reading order') is broken live: archive plates 12 /words/gloria/ (auto slot, img-noise) and 13 /words/the-nets/ (frontmatter plate.image: noise) are both textured AND the same texture, back to back in reading order. Cause: index.astro coverMap honors a forced plate.image regardless of prevTextured, and the comment at index.astro:160-162 assumes the two overrides (the-nets, price-of-sunday) sit at odd archive positions — every new publish shifts parity by one, so the 2026-08-31 publish of the-weight-of-my-no moved them to even positions (12, 14) and the auto slot before the-nets went textured. Prior runs read 'alternation present' without checking adjacency, so this has been live since 08-31. Hidden behind View Earlier on load; adjacent when expanded and on single-column mobile. | prior: PASS — 7 of 15 archive plates carry .plate-image, interleaved with plain (Texture Alternation Rule) | 2026-09-06 re-verified live: eight image plates alternate concrete/lines/noise as designed. NOTE - this run pixel-measured them rather than reading computed styles and found the scrim, not the alternation, at fault; see F101. | 2026-09-11 re-verified live: three homepage image plates alternate img-concrete / img-lines / img-noise across the cascade. | 2026-09-28: live: 8 of 16 archive plates carry .plate-image; source unchanged.</t>
+        </is>
+      </c>
+      <c r="I32" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>BLOCKED — NEEDS DEXTER (2026-10-01). Not auto-fixed: every fix trades one documented design rule against another (open-on-plain vs. honor frontmatter overrides vs. strict alternation), which is design intent, not broken behavior. Options: (A) drop plate.image from the-nets.mdx + price-of-sunday.mdx — pure auto alternation, both land plain today; (B, recommended) make plate.image choose the texture TYPE only, applied when the walk lands on a textured slot and ignored on plain slots — alternation can never break again on future publishes; (C) keep overrides and re-anchor parity on them — archive would open on a textured plate, contradicting the index.astro:157-159 open-on-plain rule.</t>
+        </is>
+      </c>
+      <c r="K32" s="6" t="inlineStr">
+        <is>
+          <t>PENDING — awaiting Dexter decision on F29 p3 options.</t>
         </is>
       </c>
     </row>
@@ -2105,7 +2133,7 @@
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>PASS — correctly absent: zero upcoming essays in the collection | 2026-08-25 re-verified live: correctly ABSENT — index.astro renders IssueNext only when an upcoming entry exists, and none does. Not a regression. | 2026-08-27 re-verified live: correctly absent — zero upcoming essays; .next-meta not in the DOM. | 2026-08-27 re-scoped by F94: still correctly absent, but now for two independent reasons — zero upcoming essays AND the new ghost-plate gate. Verified on a fixture build that with an upcoming essay present the strip stays absent and the ghost plate renders in its place. | 2026-08-27 RETIRED: the component no longer exists. IssueNext.astro is deleted and all 202 lines of `.issue-next` CSS are removed from home-v2.css and home-augment.css. Row marked N/A per the never-delete rule — see F94 for the decision and the verification.</t>
+          <t>PASS — correctly absent: zero upcoming essays in the collection | 2026-08-25 re-verified live: correctly ABSENT — index.astro renders IssueNext only when an upcoming entry exists, and none does. Not a regression. | 2026-08-27 re-verified live: correctly absent — zero upcoming essays; .next-meta not in the DOM. | 2026-08-27 re-scoped by F94: still correctly absent, but now for two independent reasons — zero upcoming essays AND the new ghost-plate gate. Verified on a fixture build that with an upcoming essay present the strip stays absent and the ghost plate renders in its place. | 2026-08-27 RETIRED: the component no longer exists. IssueNext.astro is deleted and all 202 lines of `.issue-next` CSS are removed from home-v2.css and home-augment.css. Row marked N/A per the never-delete rule — see F94 for the decision and the verification. | 2026-10-01 re-verified live: no upcoming essays and no ghost plate: 0 .issue-next, 0 teaser plates — hidden as specified.</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr"/>
@@ -2158,7 +2186,7 @@
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>PASS — manifesto form action=/api/subscribe, source=home, honeypot present | 2026-08-27 re-verified live: manifesto form + #sm-email + submit present on the homepage. | 2026-09-18 re-verified live: manifesto form action=/api/subscribe, #sm-email present, 3 value-prop items, 'No spam' line, honeypot off-canvas (x=-9999, tabindex=-1, aria-hidden). | 2026-09-28: live: #subscribe-manifesto, 3 value-prop items, 'No spam', action /api/subscribe, source=home.</t>
+          <t>PASS — manifesto form action=/api/subscribe, source=home, honeypot present | 2026-08-27 re-verified live: manifesto form + #sm-email + submit present on the homepage. | 2026-09-18 re-verified live: manifesto form action=/api/subscribe, #sm-email present, 3 value-prop items, 'No spam' line, honeypot off-canvas (x=-9999, tabindex=-1, aria-hidden). | 2026-09-28: live: #subscribe-manifesto, 3 value-prop items, 'No spam', action /api/subscribe, source=home. | 2026-10-01 re-verified live: #subscribe-manifesto: kicker, title, 3 value-prop items, form.sm-form, 'No spam' line, honeypot name=website tabindex=-1 inside aria-hidden wrapper.</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr"/>
@@ -2207,7 +2235,7 @@
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>PASS | 2026-09-18 re-verified live: real submit on the home manifesto form with a server-rejected address (healthscrub@invalid, passes type=email) showed 'Sending…', then state=error with 'That email didn't look right. Try it again.' in a role=alert .sm-error and the button re-enabled. Success path covered by the §9 API smoke (200 subscribed); the UI success state was not driven to avoid a second subscriber write. | 2026-09-28: carried: subscribe.js unchanged; endpoint states verified by API tests today (200 subscribed / already_subscribed / 400 invalid_email / 429). Not browser-submitted today to avoid extra Mailchimp writes.</t>
+          <t>PASS | 2026-09-18 re-verified live: real submit on the home manifesto form with a server-rejected address (healthscrub@invalid, passes type=email) showed 'Sending…', then state=error with 'That email didn't look right. Try it again.' in a role=alert .sm-error and the button re-enabled. Success path covered by the §9 API smoke (200 subscribed); the UI success state was not driven to avoid a second subscriber write. | 2026-09-28: carried: subscribe.js unchanged; endpoint states verified by API tests today (200 subscribed / already_subscribed / 400 invalid_email / 429). Not browser-submitted today to avoid extra Mailchimp writes. | 2026-10-01 re-verified live: carried: subscribe.js unchanged; endpoint verified by §9 API today (GET 405, POST healthscrub+20261001 -&gt; 200 subscribed 1.53s). Not browser-submitted to avoid a second Mailchimp write.</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr"/>
@@ -2260,7 +2288,7 @@
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>PASS — eyebrow lanes/tags + ' + ' separator, date, read time, h1, deck | 2026-08-27 re-verified live: eyebrow lanes/date/read-time render on all 16. | 2026-09-01 re-verified live on VOL 17 at 375px: eyebrow renders 4 lane/tag chips + date + read-time, all inside the frame post-F97. | 2026-09-06 re-verified live: .article-eyebrow computes flex-wrap nowrap at 1280px and wrap at 375px, rail height 57px, zero overflow (F97 holds live). | 2026-09-11 re-verified live: article eyebrow renders lane chips + date + read time; .article-read '8 min' matches the plate. | 2026-09-28: live: eyebrow lane + tag chips, date, read time.</t>
+          <t>PASS — eyebrow lanes/tags + ' + ' separator, date, read time, h1, deck | 2026-08-27 re-verified live: eyebrow lanes/date/read-time render on all 16. | 2026-09-01 re-verified live on VOL 17 at 375px: eyebrow renders 4 lane/tag chips + date + read-time, all inside the frame post-F97. | 2026-09-06 re-verified live: .article-eyebrow computes flex-wrap nowrap at 1280px and wrap at 375px, rail height 57px, zero overflow (F97 holds live). | 2026-09-11 re-verified live: article eyebrow renders lane chips + date + read time; .article-read '8 min' matches the plate. | 2026-09-28: live: eyebrow lane + tag chips, date, read time. | 2026-10-01 re-verified live: the-weight-of-my-no: chips Faith + Identity + Calling + Fear (' + ' via ::before, none on first), &lt;time datetime=2026-08-31&gt;, '8 min', single h1, deck present.</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr"/>
@@ -2313,7 +2341,7 @@
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>PASS — all 16 MDX bodies render through [...slug].astro | 2026-08-27 re-verified live: all 16 MDX bodies render. | 2026-09-19 re-verified live: all 17 live articles render an .article-body (shortest body ~6.4k chars of text). | 2026-09-28: live: all 17 article pages 200 with body + BlogPosting wordCount.</t>
+          <t>PASS — all 16 MDX bodies render through [...slug].astro | 2026-08-27 re-verified live: all 16 MDX bodies render. | 2026-09-19 re-verified live: all 17 live articles render an .article-body (shortest body ~6.4k chars of text). | 2026-09-28: live: all 17 article pages 200 with body + BlogPosting wordCount. | 2026-10-01 re-verified live: all 17 /words/&lt;slug&gt;/ return 200 with one .article-body; the-weight-of-my-no renders 56 paragraphs, 3 section heads.</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr"/>
@@ -2366,7 +2394,7 @@
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>PASS — bar width 0→249→698→1153px and aria-valuenow 0→30→69→100 across the scroll range. 2026-08-10 PM re-check: structural half re-verified (progress.js math recomputed by hand at 50% scroll = 51.5%; .article-body + .reading-progress present; role/aria-label/aria-valuemin/max initialized on load). Runtime paint not re-exercisable this run — the browser pane reports document.visibilityState 'hidden', so requestAnimationFrame never fires and the CSS width transition stays frozen at 0. Harness limitation, not a site regression. | 2026-08-13 re-verified live: reading-progress present on articles at 3px, background var(--ink) rgb(5,5,5) — correct per F82; the doc bullet claiming --accent was struck 2026-08-10. | 2026-08-27 NOT re-verified — rotation gap, not a failure. The reading-progress bar is scroll-driven and the browser pane would not scroll this run (window.scrollTo, scrollingElement.scrollTop, Page_Down x6 and the pointer scroll action all left scrollY at 0-2 on an 11,937px article; the pointer scroll action timed out with 'Browser pane is currently hidden'). Source unchanged since the last PASS, so the row keeps its prior result rather than being reset. | 2026-09-01 NOT TESTABLE this run — rotation gap, prior result retained. The browser pane went hidden: the pointer scroll timed out with 'Browser pane is currently hidden' and window.scrollTo / scrollingElement.scrollTop both left scrollY at 0 against a 10905px document. The .reading-progress element itself is present and correctly wired (role=progressbar, aria-valuenow=0, width 0% at scrollY 0). Neither PASS nor FAIL recorded, per the documented harness antipattern. | 2026-09-11 NOT TESTABLE — rotation gap, prior PASS retained. The browser pane was hidden for the whole run: window.scrollTo(0,2500) left scrollY at 0 and the pointer scroll action timed out with 'Browser pane is currently hidden'. Static wiring re-confirmed live (.reading-progress and .section-indicator both present on /words/the-stone/, section-indicator at opacity 0 at scroll top as specified). Neither PASSed nor FAILed on a tooling limit. | 2026-09-28: ROTATION GAP — pane stuck at scrollY 0 while hidden (QA-OS antipattern); prior result kept, not re-tested.</t>
+          <t>PASS — bar width 0→249→698→1153px and aria-valuenow 0→30→69→100 across the scroll range. 2026-08-10 PM re-check: structural half re-verified (progress.js math recomputed by hand at 50% scroll = 51.5%; .article-body + .reading-progress present; role/aria-label/aria-valuemin/max initialized on load). Runtime paint not re-exercisable this run — the browser pane reports document.visibilityState 'hidden', so requestAnimationFrame never fires and the CSS width transition stays frozen at 0. Harness limitation, not a site regression. | 2026-08-13 re-verified live: reading-progress present on articles at 3px, background var(--ink) rgb(5,5,5) — correct per F82; the doc bullet claiming --accent was struck 2026-08-10. | 2026-08-27 NOT re-verified — rotation gap, not a failure. The reading-progress bar is scroll-driven and the browser pane would not scroll this run (window.scrollTo, scrollingElement.scrollTop, Page_Down x6 and the pointer scroll action all left scrollY at 0-2 on an 11,937px article; the pointer scroll action timed out with 'Browser pane is currently hidden'). Source unchanged since the last PASS, so the row keeps its prior result rather than being reset. | 2026-09-01 NOT TESTABLE this run — rotation gap, prior result retained. The browser pane went hidden: the pointer scroll timed out with 'Browser pane is currently hidden' and window.scrollTo / scrollingElement.scrollTop both left scrollY at 0 against a 10905px document. The .reading-progress element itself is present and correctly wired (role=progressbar, aria-valuenow=0, width 0% at scrollY 0). Neither PASS nor FAIL recorded, per the documented harness antipattern. | 2026-09-11 NOT TESTABLE — rotation gap, prior PASS retained. The browser pane was hidden for the whole run: window.scrollTo(0,2500) left scrollY at 0 and the pointer scroll action timed out with 'Browser pane is currently hidden'. Static wiring re-confirmed live (.reading-progress and .section-indicator both present on /words/the-stone/, section-indicator at opacity 0 at scroll top as specified). Neither PASSed nor FAILed on a tooling limit. | 2026-09-28: ROTATION GAP — pane stuck at scrollY 0 while hidden (QA-OS antipattern); prior result kept, not re-tested. | 2026-10-01: ROTATION GAP — browser pane hidden, scrollTo leaves scrollY at 0 (QA-OS antipattern); prior PASS carried, not re-tested. Static half confirmed: progressbar role, aria-valuemin 0/max 100/now 0 at top.</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr"/>
@@ -2419,7 +2447,7 @@
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>PASS — pill text tracks sections ('What the Fear Was Actually About' → 'A New Thing' → 'The Thirtieth'), opacity animates in. 2026-08-10 PM re-check: section collection re-verified live (5 .section-head h2 landmarks found on /words/send-someone-else/; the 40%-viewport rule resolves to the correct current section). Opacity fade not observable this run — same hidden-tab rAF/transition suspension as F35. | 2026-08-27 NOT re-verified — rotation gap, not a failure. The section-indicator pill is scroll-driven and the browser pane would not scroll this run (window.scrollTo, scrollingElement.scrollTop, Page_Down x6 and the pointer scroll action all left scrollY at 0-2 on an 11,937px article; the pointer scroll action timed out with 'Browser pane is currently hidden'). Source unchanged since the last PASS, so the row keeps its prior result rather than being reset. | 2026-09-01 NOT TESTABLE this run — rotation gap, prior result retained. The browser pane went hidden: the pointer scroll timed out with 'Browser pane is currently hidden' and window.scrollTo / scrollingElement.scrollTop both left scrollY at 0 against a 10905px document. The .reading-progress element itself is present and correctly wired (role=progressbar, aria-valuenow=0, width 0% at scrollY 0). Neither PASS nor FAIL recorded, per the documented harness antipattern. | 2026-09-11 NOT TESTABLE — rotation gap, prior PASS retained. The browser pane was hidden for the whole run: window.scrollTo(0,2500) left scrollY at 0 and the pointer scroll action timed out with 'Browser pane is currently hidden'. Static wiring re-confirmed live (.reading-progress and .section-indicator both present on /words/the-stone/, section-indicator at opacity 0 at scroll top as specified). Neither PASSed nor FAILed on a tooling limit. | 2026-09-28: ROTATION GAP — pane stuck at scrollY 0 while hidden; prior result kept, not re-tested.</t>
+          <t>PASS — pill text tracks sections ('What the Fear Was Actually About' → 'A New Thing' → 'The Thirtieth'), opacity animates in. 2026-08-10 PM re-check: section collection re-verified live (5 .section-head h2 landmarks found on /words/send-someone-else/; the 40%-viewport rule resolves to the correct current section). Opacity fade not observable this run — same hidden-tab rAF/transition suspension as F35. | 2026-08-27 NOT re-verified — rotation gap, not a failure. The section-indicator pill is scroll-driven and the browser pane would not scroll this run (window.scrollTo, scrollingElement.scrollTop, Page_Down x6 and the pointer scroll action all left scrollY at 0-2 on an 11,937px article; the pointer scroll action timed out with 'Browser pane is currently hidden'). Source unchanged since the last PASS, so the row keeps its prior result rather than being reset. | 2026-09-01 NOT TESTABLE this run — rotation gap, prior result retained. The browser pane went hidden: the pointer scroll timed out with 'Browser pane is currently hidden' and window.scrollTo / scrollingElement.scrollTop both left scrollY at 0 against a 10905px document. The .reading-progress element itself is present and correctly wired (role=progressbar, aria-valuenow=0, width 0% at scrollY 0). Neither PASS nor FAIL recorded, per the documented harness antipattern. | 2026-09-11 NOT TESTABLE — rotation gap, prior PASS retained. The browser pane was hidden for the whole run: window.scrollTo(0,2500) left scrollY at 0 and the pointer scroll action timed out with 'Browser pane is currently hidden'. Static wiring re-confirmed live (.reading-progress and .section-indicator both present on /words/the-stone/, section-indicator at opacity 0 at scroll top as specified). Neither PASSed nor FAILed on a tooling limit. | 2026-09-28: ROTATION GAP — pane stuck at scrollY 0 while hidden; prior result kept, not re-tested. | 2026-10-01: ROTATION GAP — browser pane hidden, scrollTo leaves scrollY at 0 (QA-OS antipattern); prior PASS carried, not re-tested. Static half confirmed: .section-indicator present (opacity 0 at top), 3 .section-head h2 landmarks.</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr"/>
@@ -6354,7 +6382,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6362,14 +6390,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Phase 2 Test Results</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>— P2 (test) —</t>
         </is>
@@ -6381,8 +6409,8 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="B4" s="9" t="n">
-        <v>83</v>
+      <c r="B4" s="10" t="n">
+        <v>82</v>
       </c>
     </row>
     <row r="5">
@@ -6391,12 +6419,12 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="B5" s="10" t="n">
+      <c r="B5" s="11" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>— P4 (re-test) —</t>
         </is>
@@ -6408,8 +6436,8 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="B8" s="9" t="n">
-        <v>103</v>
+      <c r="B8" s="10" t="n">
+        <v>102</v>
       </c>
     </row>
     <row r="9">
@@ -6418,7 +6446,7 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="B9" s="10" t="n">
+      <c r="B9" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6428,39 +6456,49 @@
           <t>PENDING</t>
         </is>
       </c>
-      <c r="B10" s="11" t="n">
-        <v>4</v>
+      <c r="B10" s="12" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>— Issues by severity (found) —</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>Resolved (P4 PASS)</t>
         </is>
       </c>
-      <c r="B14" s="9" t="n">
+      <c r="B15" s="10" t="n">
         <v>29</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>Still open</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="B16" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>Total features: 108</t>
         </is>

</xml_diff>

<commit_message>
audit(ledger): F29 fixed on option B, build-verified
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -68,7 +68,7 @@
       <color rgb="00C0211B"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -100,11 +100,6 @@
         <fgColor rgb="00E2E2DE"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F4B9B5"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -132,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -161,7 +156,6 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2086,12 +2080,12 @@
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>BLOCKED — NEEDS DEXTER (2026-10-01). Not auto-fixed: every fix trades one documented design rule against another (open-on-plain vs. honor frontmatter overrides vs. strict alternation), which is design intent, not broken behavior. Options: (A) drop plate.image from the-nets.mdx + price-of-sunday.mdx — pure auto alternation, both land plain today; (B, recommended) make plate.image choose the texture TYPE only, applied when the walk lands on a textured slot and ignored on plain slots — alternation can never break again on future publishes; (C) keep overrides and re-anchor parity on them — archive would open on a textured plate, contradicting the index.astro:157-159 open-on-plain rule.</t>
+          <t>FIXED 2026-10-01 (Dexter chose option B) — src/pages/index.astro coverMap: frontmatter plate.image now replaces the TEXTURE_CYCLE pick only when the walk lands on a textured slot, ignored on plain slots; placement is always alternation-driven. Comment rewritten to drop the stale odd-position assumption. | was: BLOCKED — NEEDS DEXTER (2026-10-01). Not auto-fixed: every fix trades one documented design rule against another (open-on-plain vs. honor frontmatter overrides vs. strict alternation), which is design intent, not broken behavior. Options: (A) drop plate.image from the-nets.mdx + price-of-sunday.mdx — pure auto alternation, both land plain today; (B, recommended) make plate.image choose the texture TYPE only, applied when the walk lands on a textured slot and ignored on plain slots — alternation can never break again on future publishes; (C) keep overrides and re-anchor parity on them — archive would open on a textured plate, contradicting the index.astro:157-159 open-on-plain rule.</t>
         </is>
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>PENDING — awaiting Dexter decision on F29 p3 options.</t>
+          <t>PASS (verified against build) — 2026-10-01 on a clean `npm run build`: dist/index.html archive reads plain/concrete/plain/lines/plain/noise/plain/concrete/plain/lines/plain/noise/plain/concrete/plain/lines — 0 adjacency violations across 16 archive plates (gloria noise → the-nets plain); 0 inline &lt;style&gt;. Both overrides sit on plain slots this publish, so they are dormant until the next publish shifts parity. Live re-verify after merge.</t>
         </is>
       </c>
     </row>
@@ -6437,7 +6431,7 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="9">
@@ -6457,7 +6451,7 @@
         </is>
       </c>
       <c r="B10" s="12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -6484,7 +6478,7 @@
         </is>
       </c>
       <c r="B15" s="10" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16">
@@ -6493,8 +6487,8 @@
           <t>Still open</t>
         </is>
       </c>
-      <c r="B16" s="16" t="n">
-        <v>1</v>
+      <c r="B16" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
audit(ledger): 2026-10-02 scrub — clean site, F35-F46 rotation all PASS (F35/F36 via headless CDP)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -2085,7 +2085,7 @@
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>PASS (closed live 2026-10-01 on deploy c9a2527) — live homepage: 0 adjacency violations across 16 archive plates; pulpit plain → gloria noise → the-nets plain → gumbo concrete → price-of-sunday plain; 0 inline &lt;style&gt;. | was: PASS (verified against build) — 2026-10-01 on a clean `npm run build`: dist/index.html archive reads plain/concrete/plain/lines/plain/noise/plain/concrete/plain/lines/plain/noise/plain/concrete/plain/lines — 0 adjacency violations across 16 archive plates (gloria noise → the-nets plain); 0 inline &lt;style&gt;. Both overrides sit on plain slots this publish, so they are dormant until the next publish shifts parity. Live re-verify after merge.</t>
+          <t>PASS (closed live 2026-10-01 on deploy c9a2527) — live homepage: 0 adjacency violations across 16 archive plates; pulpit plain → gloria noise → the-nets plain → gumbo concrete → price-of-sunday plain; 0 inline &lt;style&gt;. | was: PASS (verified against build) — 2026-10-01 on a clean `npm run build`: dist/index.html archive reads plain/concrete/plain/lines/plain/noise/plain/concrete/plain/lines/plain/noise/plain/concrete/plain/lines — 0 adjacency violations across 16 archive plates (gloria noise → the-nets plain); 0 inline &lt;style&gt;. Both overrides sit on plain slots this publish, so they are dormant until the next publish shifts parity. Live re-verify after merge. | 2026-10-02: re-verified live — 0 adjacency violations across 16 archive plates (plain/textured alternate end to end; gloria noise → the-nets plain).</t>
         </is>
       </c>
     </row>
@@ -2388,7 +2388,7 @@
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>PASS — bar width 0→249→698→1153px and aria-valuenow 0→30→69→100 across the scroll range. 2026-08-10 PM re-check: structural half re-verified (progress.js math recomputed by hand at 50% scroll = 51.5%; .article-body + .reading-progress present; role/aria-label/aria-valuemin/max initialized on load). Runtime paint not re-exercisable this run — the browser pane reports document.visibilityState 'hidden', so requestAnimationFrame never fires and the CSS width transition stays frozen at 0. Harness limitation, not a site regression. | 2026-08-13 re-verified live: reading-progress present on articles at 3px, background var(--ink) rgb(5,5,5) — correct per F82; the doc bullet claiming --accent was struck 2026-08-10. | 2026-08-27 NOT re-verified — rotation gap, not a failure. The reading-progress bar is scroll-driven and the browser pane would not scroll this run (window.scrollTo, scrollingElement.scrollTop, Page_Down x6 and the pointer scroll action all left scrollY at 0-2 on an 11,937px article; the pointer scroll action timed out with 'Browser pane is currently hidden'). Source unchanged since the last PASS, so the row keeps its prior result rather than being reset. | 2026-09-01 NOT TESTABLE this run — rotation gap, prior result retained. The browser pane went hidden: the pointer scroll timed out with 'Browser pane is currently hidden' and window.scrollTo / scrollingElement.scrollTop both left scrollY at 0 against a 10905px document. The .reading-progress element itself is present and correctly wired (role=progressbar, aria-valuenow=0, width 0% at scrollY 0). Neither PASS nor FAIL recorded, per the documented harness antipattern. | 2026-09-11 NOT TESTABLE — rotation gap, prior PASS retained. The browser pane was hidden for the whole run: window.scrollTo(0,2500) left scrollY at 0 and the pointer scroll action timed out with 'Browser pane is currently hidden'. Static wiring re-confirmed live (.reading-progress and .section-indicator both present on /words/the-stone/, section-indicator at opacity 0 at scroll top as specified). Neither PASSed nor FAILed on a tooling limit. | 2026-09-28: ROTATION GAP — pane stuck at scrollY 0 while hidden (QA-OS antipattern); prior result kept, not re-tested. | 2026-10-01: ROTATION GAP — browser pane hidden, scrollTo leaves scrollY at 0 (QA-OS antipattern); prior PASS carried, not re-tested. Static half confirmed: progressbar role, aria-valuemin 0/max 100/now 0 at top.</t>
+          <t>PASS — bar width 0→249→698→1153px and aria-valuenow 0→30→69→100 across the scroll range. 2026-08-10 PM re-check: structural half re-verified (progress.js math recomputed by hand at 50% scroll = 51.5%; .article-body + .reading-progress present; role/aria-label/aria-valuemin/max initialized on load). Runtime paint not re-exercisable this run — the browser pane reports document.visibilityState 'hidden', so requestAnimationFrame never fires and the CSS width transition stays frozen at 0. Harness limitation, not a site regression. | 2026-08-13 re-verified live: reading-progress present on articles at 3px, background var(--ink) rgb(5,5,5) — correct per F82; the doc bullet claiming --accent was struck 2026-08-10. | 2026-08-27 NOT re-verified — rotation gap, not a failure. The reading-progress bar is scroll-driven and the browser pane would not scroll this run (window.scrollTo, scrollingElement.scrollTop, Page_Down x6 and the pointer scroll action all left scrollY at 0-2 on an 11,937px article; the pointer scroll action timed out with 'Browser pane is currently hidden'). Source unchanged since the last PASS, so the row keeps its prior result rather than being reset. | 2026-09-01 NOT TESTABLE this run — rotation gap, prior result retained. The browser pane went hidden: the pointer scroll timed out with 'Browser pane is currently hidden' and window.scrollTo / scrollingElement.scrollTop both left scrollY at 0 against a 10905px document. The .reading-progress element itself is present and correctly wired (role=progressbar, aria-valuenow=0, width 0% at scrollY 0). Neither PASS nor FAIL recorded, per the documented harness antipattern. | 2026-09-11 NOT TESTABLE — rotation gap, prior PASS retained. The browser pane was hidden for the whole run: window.scrollTo(0,2500) left scrollY at 0 and the pointer scroll action timed out with 'Browser pane is currently hidden'. Static wiring re-confirmed live (.reading-progress and .section-indicator both present on /words/the-stone/, section-indicator at opacity 0 at scroll top as specified). Neither PASSed nor FAILed on a tooling limit. | 2026-09-28: ROTATION GAP — pane stuck at scrollY 0 while hidden (QA-OS antipattern); prior result kept, not re-tested. | 2026-10-01: ROTATION GAP — browser pane hidden, scrollTo leaves scrollY at 0 (QA-OS antipattern); prior PASS carried, not re-tested. Static half confirmed: progressbar role, aria-valuemin 0/max 100/now 0 at top. | 2026-10-02: live (headless Chrome via CDP — the pane was hidden and scroll-inert, so the real scroll ran headless against production): /words/the-stone/ bar width 0→256→643→1086→1280px, aria-valuenow 0→25→56→94→100, role=progressbar. Closes the 10-01 rotation gap.</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr"/>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>PASS — pill text tracks sections ('What the Fear Was Actually About' → 'A New Thing' → 'The Thirtieth'), opacity animates in. 2026-08-10 PM re-check: section collection re-verified live (5 .section-head h2 landmarks found on /words/send-someone-else/; the 40%-viewport rule resolves to the correct current section). Opacity fade not observable this run — same hidden-tab rAF/transition suspension as F35. | 2026-08-27 NOT re-verified — rotation gap, not a failure. The section-indicator pill is scroll-driven and the browser pane would not scroll this run (window.scrollTo, scrollingElement.scrollTop, Page_Down x6 and the pointer scroll action all left scrollY at 0-2 on an 11,937px article; the pointer scroll action timed out with 'Browser pane is currently hidden'). Source unchanged since the last PASS, so the row keeps its prior result rather than being reset. | 2026-09-01 NOT TESTABLE this run — rotation gap, prior result retained. The browser pane went hidden: the pointer scroll timed out with 'Browser pane is currently hidden' and window.scrollTo / scrollingElement.scrollTop both left scrollY at 0 against a 10905px document. The .reading-progress element itself is present and correctly wired (role=progressbar, aria-valuenow=0, width 0% at scrollY 0). Neither PASS nor FAIL recorded, per the documented harness antipattern. | 2026-09-11 NOT TESTABLE — rotation gap, prior PASS retained. The browser pane was hidden for the whole run: window.scrollTo(0,2500) left scrollY at 0 and the pointer scroll action timed out with 'Browser pane is currently hidden'. Static wiring re-confirmed live (.reading-progress and .section-indicator both present on /words/the-stone/, section-indicator at opacity 0 at scroll top as specified). Neither PASSed nor FAILed on a tooling limit. | 2026-09-28: ROTATION GAP — pane stuck at scrollY 0 while hidden; prior result kept, not re-tested. | 2026-10-01: ROTATION GAP — browser pane hidden, scrollTo leaves scrollY at 0 (QA-OS antipattern); prior PASS carried, not re-tested. Static half confirmed: .section-indicator present (opacity 0 at top), 3 .section-head h2 landmarks.</t>
+          <t>PASS — pill text tracks sections ('What the Fear Was Actually About' → 'A New Thing' → 'The Thirtieth'), opacity animates in. 2026-08-10 PM re-check: section collection re-verified live (5 .section-head h2 landmarks found on /words/send-someone-else/; the 40%-viewport rule resolves to the correct current section). Opacity fade not observable this run — same hidden-tab rAF/transition suspension as F35. | 2026-08-27 NOT re-verified — rotation gap, not a failure. The section-indicator pill is scroll-driven and the browser pane would not scroll this run (window.scrollTo, scrollingElement.scrollTop, Page_Down x6 and the pointer scroll action all left scrollY at 0-2 on an 11,937px article; the pointer scroll action timed out with 'Browser pane is currently hidden'). Source unchanged since the last PASS, so the row keeps its prior result rather than being reset. | 2026-09-01 NOT TESTABLE this run — rotation gap, prior result retained. The browser pane went hidden: the pointer scroll timed out with 'Browser pane is currently hidden' and window.scrollTo / scrollingElement.scrollTop both left scrollY at 0 against a 10905px document. The .reading-progress element itself is present and correctly wired (role=progressbar, aria-valuenow=0, width 0% at scrollY 0). Neither PASS nor FAIL recorded, per the documented harness antipattern. | 2026-09-11 NOT TESTABLE — rotation gap, prior PASS retained. The browser pane was hidden for the whole run: window.scrollTo(0,2500) left scrollY at 0 and the pointer scroll action timed out with 'Browser pane is currently hidden'. Static wiring re-confirmed live (.reading-progress and .section-indicator both present on /words/the-stone/, section-indicator at opacity 0 at scroll top as specified). Neither PASSed nor FAILed on a tooling limit. | 2026-09-28: ROTATION GAP — pane stuck at scrollY 0 while hidden; prior result kept, not re-tested. | 2026-10-01: ROTATION GAP — browser pane hidden, scrollTo leaves scrollY at 0 (QA-OS antipattern); prior PASS carried, not re-tested. Static half confirmed: .section-indicator present (opacity 0 at top), 3 .section-head h2 landmarks. | 2026-10-02: live (headless Chrome via CDP): 9 .section-head h2 landmarks on /words/the-stone/; pill hidden at 1% (op 0), reads 'The algorithm of outrage.' at 30%, 'The Pharisee in the mirror.' at 60%, 'Mercy is not naiveté.' at 97% (op 1), hides again at 100% (&gt;98%). Closes the 10-01 rotation gap.</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr"/>
@@ -2494,7 +2494,7 @@
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t>PASS — X intent carries encoded url + title | 2026-08-27 re-verified live: X intent carries encoded url + title (checked on /about/). | 2026-09-11 re-verified live: X intent href carries the encoded article URL and 'The Weight of My No — DX', target=_blank rel='noopener noreferrer'. | 2026-09-28: live: X intent carries encoded url + text, target=_blank rel=noopener noreferrer (article + about).</t>
+          <t>PASS — X intent carries encoded url + title | 2026-08-27 re-verified live: X intent carries encoded url + title (checked on /about/). | 2026-09-11 re-verified live: X intent href carries the encoded article URL and 'The Weight of My No — DX', target=_blank rel='noopener noreferrer'. | 2026-09-28: live: X intent carries encoded url + text, target=_blank rel=noopener noreferrer (article + about). | 2026-10-02: live: X intent href carries url=https%3A%2F%2Fimjustdex.com%2Fwords%2Fthe-stone%2F and text 'The Stone You're Holding — DX', target=_blank rel='noopener noreferrer'.</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr"/>
@@ -2543,7 +2543,7 @@
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>PASS — copy button + [data-copy-status] live region on article and about | 2026-08-27 re-verified live: copy button + [data-copy-status] aria-live=polite region present on article and about. | 2026-09-11 re-verified live: copy-link button present on article and about with data-copy-link set to the absolute page URL; essay.js loaded; aria-live region present. | 2026-09-28: live: button + [data-copy-status] present; failure path verified (label 'Copy failed' + SR status). Success path untestable in the pane: control navigator.clipboard.writeText() -&gt; 'Write permission denied' — harness, not site. Prior PASS kept.</t>
+          <t>PASS — copy button + [data-copy-status] live region on article and about | 2026-08-27 re-verified live: copy button + [data-copy-status] aria-live=polite region present on article and about. | 2026-09-11 re-verified live: copy-link button present on article and about with data-copy-link set to the absolute page URL; essay.js loaded; aria-live region present. | 2026-09-28: live: button + [data-copy-status] present; failure path verified (label 'Copy failed' + SR status). Success path untestable in the pane: control navigator.clipboard.writeText() -&gt; 'Write permission denied' — harness, not site. Prior PASS kept. | 2026-10-02: live: [data-copy-link]=https://imjustdex.com/words/the-stone/ with [data-copy-status] aria-live=polite.</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr"/>
@@ -2596,7 +2596,7 @@
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>PASS — Follow Me → instagram.com/ImJustDex | 2026-08-27 re-verified live: Follow Me → instagram.com/ImJustDex, 200. | 2026-09-19 re-verified live: Follow Me → instagram.com/ImJustDex with target=_blank rel='noopener noreferrer' on 17/17 articles and on /about/. | 2026-09-28: live: Follow Me -&gt; instagram.com/ImJustDex, _blank noopener noreferrer (article + about).</t>
+          <t>PASS — Follow Me → instagram.com/ImJustDex | 2026-08-27 re-verified live: Follow Me → instagram.com/ImJustDex, 200. | 2026-09-19 re-verified live: Follow Me → instagram.com/ImJustDex with target=_blank rel='noopener noreferrer' on 17/17 articles and on /about/. | 2026-09-28: live: Follow Me -&gt; instagram.com/ImJustDex, _blank noopener noreferrer (article + about). | 2026-10-02: live: Follow Me → https://instagram.com/ImJustDex, target=_blank rel='noopener noreferrer'.</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr"/>
@@ -2645,7 +2645,7 @@
       </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
-          <t>PASS — form posts /api/subscribe with source=article, honeypot off-canvas, aria-live label; server states verified directly against the function | 2026-09-18 re-verified live: server-rejected address on /words/gumbo/ surfaced 'That email didn’t look right. Try it again.' in the role=status aria-live label and kept the form — it reflects the server failure rather than a blanket success. source=article, honeypot off-canvas at x=-4972. | 2026-09-28: live: article form posts /api/subscribe, source=article, honeypot 'website' present; fixture build coming-soon form source=coming-soon.</t>
+          <t>PASS — form posts /api/subscribe with source=article, honeypot off-canvas, aria-live label; server states verified directly against the function | 2026-09-18 re-verified live: server-rejected address on /words/gumbo/ surfaced 'That email didn’t look right. Try it again.' in the role=status aria-live label and kept the form — it reflects the server failure rather than a blanket success. source=article, honeypot off-canvas at x=-4972. | 2026-09-28: live: article form posts /api/subscribe, source=article, honeypot 'website' present; fixture build coming-soon form source=coming-soon. | 2026-10-02: live: .email-signup action=/api/subscribe, source=article, honeypot [name=website] present, aria-live region present; function POST (healthscrub+20261002) returned 200 subscribed in 1.31s.</t>
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr"/>
@@ -2698,7 +2698,7 @@
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
-          <t>PASS (live + fixture build) | Authored prev/next render correctly on all 16. Ghost/teaser path PENDING — requires a future-dated entry; none exists. 2026-08-10 PM: the derive-from-live-status fix (p3) live-verified, then the underlying data cleaned — the 4 stale ghost:true flags are gone (see F81). Zero `ghost: true` remain in the collection; all 16 essays render real .article-nav-link anchors, 15 rel=next head links (newest correctly has none), zero article-nav-ghost teasers. | 2026-08-25 re-verified live: all 16 essays render real .article-nav-link anchors; zero `ghost: true` remain in the collection. Ghost/teaser path still PENDING — still requires a future-dated entry and none exists. | 2026-09-11: authored prev/next re-verified live — newest essay emits rel=prev only, /words/the-stone/ emits rel=prev + rel=next. Ghost/teaser path still PENDING; zero upcoming entries in the collection. | 2026-09-19: authored prev/next unchanged (no code churn since 507e988). Ghost/teaser path still PENDING — zero upcoming entries in the collection. | 2026-09-23: authored prev/next unchanged (no code or content commits since 09-19). Ghost path still PENDING — no future-dated entry. | 2026-09-25: still PENDING — 17/17 entries status published and past-dated, no upcoming entry to render.  | 2026-09-28: PASS (live + build-verified via throwaway fixture). Live: authored prev/next correct; send-someone-else's stale frontmatter ghost:true is neutralised by nextLive, so live renders a real rel=next. Fixture (future-dated entry in a scratch copy, never committed): the-weight-of-my-no's next renders .article-nav-ghost with 'Jan 15, 2027' and NO rel=next.</t>
+          <t>PASS (live + fixture build) | Authored prev/next render correctly on all 16. Ghost/teaser path PENDING — requires a future-dated entry; none exists. 2026-08-10 PM: the derive-from-live-status fix (p3) live-verified, then the underlying data cleaned — the 4 stale ghost:true flags are gone (see F81). Zero `ghost: true` remain in the collection; all 16 essays render real .article-nav-link anchors, 15 rel=next head links (newest correctly has none), zero article-nav-ghost teasers. | 2026-08-25 re-verified live: all 16 essays render real .article-nav-link anchors; zero `ghost: true` remain in the collection. Ghost/teaser path still PENDING — still requires a future-dated entry and none exists. | 2026-09-11: authored prev/next re-verified live — newest essay emits rel=prev only, /words/the-stone/ emits rel=prev + rel=next. Ghost/teaser path still PENDING; zero upcoming entries in the collection. | 2026-09-19: authored prev/next unchanged (no code churn since 507e988). Ghost/teaser path still PENDING — zero upcoming entries in the collection. | 2026-09-23: authored prev/next unchanged (no code or content commits since 09-19). Ghost path still PENDING — no future-dated entry. | 2026-09-25: still PENDING — 17/17 entries status published and past-dated, no upcoming entry to render.  | 2026-09-28: PASS (live + build-verified via throwaway fixture). Live: authored prev/next correct; send-someone-else's stale frontmatter ghost:true is neutralised by nextLive, so live renders a real rel=next. Fixture (future-dated entry in a scratch copy, never committed): the-weight-of-my-no's next renders .article-nav-ghost with 'Jan 15, 2027' and NO rel=next. | 2026-10-02: live: authored half PASS — /words/the-stone/ article-nav prev→/words/pulpit/ (rel=prev), next→/words/should-have-killed-it/ (rel=next). Ghost half still structurally untestable — 0 upcoming entries (17/17 status published, newest 2026-08-31).</t>
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr"/>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="K44" s="6" t="inlineStr">
         <is>
-          <t>PENDING | 2026-09-18: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-26: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-27: still structurally untestable — 0 upcoming entries in the committed collection (17/17 published, past-dated). | 2026-09-28: PASS (ghost path verified against a fixture build; authored path live).</t>
+          <t>PENDING | 2026-09-18: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-26: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-27: still structurally untestable — 0 upcoming entries in the committed collection (17/17 published, past-dated). | 2026-09-28: PASS (ghost path verified against a fixture build; authored path live). | 2026-10-02: still structurally untestable — 0 upcoming entries in the committed collection.</t>
         </is>
       </c>
     </row>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="H45" s="6" t="inlineStr">
         <is>
-          <t>PASS — rel=prev emitted where prev authored; rel=next where next authored and live | 2026-08-25 re-verified live: rel=prev/next head links intact across the chain. | 2026-09-11 re-verified live: newest essay emits rel=prev only; /words/the-stone/ emits both rel=prev and rel=next. Correct. | 2026-09-28: live: the-weight-of-my-no rel=prev only; show-me-your-glory rel=prev + rel=next; fixture: ghost next emits no rel=next.</t>
+          <t>PASS — rel=prev emitted where prev authored; rel=next where next authored and live | 2026-08-25 re-verified live: rel=prev/next head links intact across the chain. | 2026-09-11 re-verified live: newest essay emits rel=prev only; /words/the-stone/ emits both rel=prev and rel=next. Correct. | 2026-09-28: live: the-weight-of-my-no rel=prev only; show-me-your-glory rel=prev + rel=next; fixture: ghost next emits no rel=next. | 2026-10-02: live: head emits link rel=prev /words/pulpit/ and rel=next /words/should-have-killed-it/ on /words/the-stone/.</t>
         </is>
       </c>
       <c r="I45" s="6" t="inlineStr"/>
@@ -2804,7 +2804,7 @@
       </c>
       <c r="H46" s="6" t="inlineStr">
         <is>
-          <t>PASS — '← Back' → '/' on article, coming-soon, about | 2026-09-11 re-verified live: '← Back' → '/' present on article and about. | 2026-09-28: live: '← Back' (.article-back) -&gt; '/' on article + about.</t>
+          <t>PASS — '← Back' → '/' on article, coming-soon, about | 2026-09-11 re-verified live: '← Back' → '/' present on article and about. | 2026-09-28: live: '← Back' (.article-back) -&gt; '/' on article + about. | 2026-10-02: live: '← Back' → '/' on /words/the-stone/.</t>
         </is>
       </c>
       <c r="I46" s="6" t="inlineStr"/>
@@ -2853,7 +2853,7 @@
       </c>
       <c r="H47" s="6" t="inlineStr">
         <is>
-          <t>PASS — PullQuote, Scripture, Callout, DropCap, Closing, SectionHead, ResearchCTA, StudyNote all render and are styled via external hashed CSS (CSP-clean) | 2026-08-27 re-verified live: PullQuote/Scripture/Callout/StudyNote all render (the-stone: 2 pull-quotes, 4 scripture, 2 callouts, 3 study notes). | 2026-09-11 re-verified live: all MDX components still render; ResearchCTA now appears only on /words/show-me-your-glory/ (target thereturningglory.com 200) and is correctly gone from /words/the-nets/ after 507e988. | 2026-09-28: live: show-me-your-glory — .callout left border #c00, 3 StudyNotes, 0 contrast failures across 151 elements in both modes.</t>
+          <t>PASS — PullQuote, Scripture, Callout, DropCap, Closing, SectionHead, ResearchCTA, StudyNote all render and are styled via external hashed CSS (CSP-clean) | 2026-08-27 re-verified live: PullQuote/Scripture/Callout/StudyNote all render (the-stone: 2 pull-quotes, 4 scripture, 2 callouts, 3 study notes). | 2026-09-11 re-verified live: all MDX components still render; ResearchCTA now appears only on /words/show-me-your-glory/ (target thereturningglory.com 200) and is correctly gone from /words/the-nets/ after 507e988. | 2026-09-28: live: show-me-your-glory — .callout left border #c00, 3 StudyNotes, 0 contrast failures across 151 elements in both modes. | 2026-10-02: live: /words/the-stone/ renders 2 pull-quotes, 4 scripture, 2 callouts, 9 section heads; 0 contrast failures in light and dark (real-click toggle).</t>
         </is>
       </c>
       <c r="I47" s="6" t="inlineStr"/>
@@ -2906,7 +2906,7 @@
       </c>
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>PASS — &lt;details&gt; summary toggles open→closed→open on both sampled essays | 2026-08-27 re-verified live: &lt;details&gt; summary toggles closed→open→closed on the-stone. | 2026-09-11 re-verified live: 12 essays carry native &lt;details class=study-note&gt; with &lt;summary&gt;; 1–3 per essay. | 2026-09-28: live: &lt;details&gt; toggles closed -&gt; open -&gt; closed.</t>
+          <t>PASS — &lt;details&gt; summary toggles open→closed→open on both sampled essays | 2026-08-27 re-verified live: &lt;details&gt; summary toggles closed→open→closed on the-stone. | 2026-09-11 re-verified live: 12 essays carry native &lt;details class=study-note&gt; with &lt;summary&gt;; 1–3 per essay. | 2026-09-28: live: &lt;details&gt; toggles closed -&gt; open -&gt; closed. | 2026-10-02: live: 3 &lt;details class=study-note&gt; on /words/the-stone/; summary toggles closed→open→closed.</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr"/>
@@ -2970,7 +2970,7 @@
       </c>
       <c r="K49" s="6" t="inlineStr">
         <is>
-          <t>PENDING | 2026-09-18: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-26: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-27: still structurally untestable — 0 upcoming entries in the committed collection (17/17 published, past-dated). | 2026-09-28: PASS (verified against a fixture build).</t>
+          <t>PENDING | 2026-09-18: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-26: still structurally untestable — 0 upcoming entries in the committed collection. | 2026-09-27: still structurally untestable — 0 upcoming entries in the committed collection (17/17 published, past-dated). | 2026-09-28: PASS (verified against a fixture build). | 2026-10-02: still structurally untestable — 0 upcoming entries in the committed collection.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
audit(ledger): 2026-10-04 scrub — clean site, F47-F58 rotation all PASS; QA-OS notes pane clipboard denial
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -3012,7 +3012,7 @@
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>PASS — about content + ProfilePage render | 2026-08-27 re-verified live: about content + ProfilePage render. | 2026-09-01 re-verified live: /about/ 200 in 0.75s, single h1, all four landmarks, 0 contrast failures across 24 measured elements. | 2026-09-19 re-verified live: /about/ 200 in 0.38s, deck 'Est. 1994.' present, single h1, ProfilePage JSON-LD complete, 0 contrast failures across 23 elements in both modes. | 2026-09-28: live: 'Est. 1994' deck, PullQuote, Closing, ProfilePage.</t>
+          <t>PASS — about content + ProfilePage render | 2026-08-27 re-verified live: about content + ProfilePage render. | 2026-09-01 re-verified live: /about/ 200 in 0.75s, single h1, all four landmarks, 0 contrast failures across 24 measured elements. | 2026-09-19 re-verified live: /about/ 200 in 0.38s, deck 'Est. 1994.' present, single h1, ProfilePage JSON-LD complete, 0 contrast failures across 23 elements in both modes. | 2026-09-28: live: 'Est. 1994' deck, PullQuote, Closing, ProfilePage. | 2026-10-04: live: /about/ 200 (0.34s), deck 'Est. 1994.', h1 'Dexter Jakes', 9 body paras incl intro, pull-quote present, canonical /about/, ProfilePage+Person+Organization JSON-LD with all required mainEntity fields; 0 console errors.</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr"/>
@@ -3061,7 +3061,7 @@
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>PASS — share bar X + copy + Follow Me with live region | 2026-08-27 re-verified live: share bar X + copy + Follow Me + live region present on /about/. | 2026-09-19 re-verified live: /about/ share bar carries X intent, data-copy-link, Follow Me and an aria-live region. | 2026-09-28: live: X intent + Copy link (data-copy-link) + Follow Me on /about/.</t>
+          <t>PASS — share bar X + copy + Follow Me with live region | 2026-08-27 re-verified live: share bar X + copy + Follow Me + live region present on /about/. | 2026-09-19 re-verified live: /about/ share bar carries X intent, data-copy-link, Follow Me and an aria-live region. | 2026-09-28: live: X intent + Copy link (data-copy-link) + Follow Me on /about/. | 2026-10-04: live: X intent (about url+text), data-copy-link=/about/, Follow Me→Instagram, aria-live status present. Real pointer click on Copy link announced 'Copy failed. Select the URL manually.' — harness artifact, not a defect: the pane's browser reports clipboard-write permission 'denied' and rejects writeText even outside the click; the site's honest fail path + live region behaved exactly as built.</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr"/>
@@ -3114,7 +3114,7 @@
       </c>
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>PASS — bespoke notfound-plate, 200 on /404, noindex+nofollow, /* fallback 404s unmatched routes | 2026-08-27 re-verified live: bespoke notfound-plate, 200 on /404, noindex+nofollow, single h1. | 2026-09-01 re-verified live: /404 returns HTTP 200 with the bespoke 'Nothing to Document Here' body, meta robots noindex,nofollow, single h1, all four landmarks, 0 contrast failures across 16 elements. | 2026-09-19 re-verified live: unmatched route returns HTTP 404 with the bespoke 'Nothing to Document Here' body, meta robots 'noindex, nofollow', Back to Home → /; 0 contrast failures in both modes. | 2026-09-28: live: unmatched route -&gt; HTTP 404, notfound-plate, 'Back to Home' -&gt; /, noindex,nofollow, 0 contrast failures (dark).</t>
+          <t>PASS — bespoke notfound-plate, 200 on /404, noindex+nofollow, /* fallback 404s unmatched routes | 2026-08-27 re-verified live: bespoke notfound-plate, 200 on /404, noindex+nofollow, single h1. | 2026-09-01 re-verified live: /404 returns HTTP 200 with the bespoke 'Nothing to Document Here' body, meta robots noindex,nofollow, single h1, all four landmarks, 0 contrast failures across 16 elements. | 2026-09-19 re-verified live: unmatched route returns HTTP 404 with the bespoke 'Nothing to Document Here' body, meta robots 'noindex, nofollow', Back to Home → /; 0 contrast failures in both modes. | 2026-09-28: live: unmatched route -&gt; HTTP 404, notfound-plate, 'Back to Home' -&gt; /, noindex,nofollow, 0 contrast failures (dark). | 2026-10-04: live: /404 200 with .notfound-plate, single h1 'Nothing to Document Here.', noindex,nofollow, 'Back to Home'→/; unmatched /no-such-page-qa → HTTP 404 with the bespoke body; 0 console errors.</t>
         </is>
       </c>
       <c r="I52" s="6" t="inlineStr"/>
@@ -3167,7 +3167,7 @@
       </c>
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>PASS — Atom 16 entries = 16 published; namespace + entries valid | 2026-08-13 re-verified live: /feed.xml 200, Atom namespace, 16 &lt;entry&gt; elements — exactly matching the 16 articles on the homepage, zero set difference either direction. | 2026-08-16 re-verified live: /feed.xml 200 with 16 &lt;entry&gt; elements; set-compared against the 16 article links on the live homepage — zero difference in either direction. | 2026-08-25 re-verified live: /feed.xml 200, 16 &lt;entry&gt; elements matching the 16 published articles exactly — no gaps, no extras. | 2026-08-27 re-verified live: Atom 16 entries == 16 published on the homepage. | 2026-09-01 re-verified live: /feed.xml 200, 17 entries — exactly matching the 17 articles on the homepage cascade. No feed-only or home-only slugs. | 2026-09-06 re-verified live: /feed.xml 200, 17 entries, slug set identical to the homepage cascade. | 2026-09-11 re-verified live: /feed.xml parses as Atom, 17 entries, matching the 17 published articles exactly. | 2026-09-28: live: Atom 17 entries = 17 published, 27 lane categories, subtitle/rights/icon/logo/author present, application/xml, must-revalidate.</t>
+          <t>PASS — Atom 16 entries = 16 published; namespace + entries valid | 2026-08-13 re-verified live: /feed.xml 200, Atom namespace, 16 &lt;entry&gt; elements — exactly matching the 16 articles on the homepage, zero set difference either direction. | 2026-08-16 re-verified live: /feed.xml 200 with 16 &lt;entry&gt; elements; set-compared against the 16 article links on the live homepage — zero difference in either direction. | 2026-08-25 re-verified live: /feed.xml 200, 16 &lt;entry&gt; elements matching the 16 published articles exactly — no gaps, no extras. | 2026-08-27 re-verified live: Atom 16 entries == 16 published on the homepage. | 2026-09-01 re-verified live: /feed.xml 200, 17 entries — exactly matching the 17 articles on the homepage cascade. No feed-only or home-only slugs. | 2026-09-06 re-verified live: /feed.xml 200, 17 entries, slug set identical to the homepage cascade. | 2026-09-11 re-verified live: /feed.xml parses as Atom, 17 entries, matching the 17 published articles exactly. | 2026-09-28: live: Atom 17 entries = 17 published, 27 lane categories, subtitle/rights/icon/logo/author present, application/xml, must-revalidate. | 2026-10-04: live: /feed.xml 200, 17 &lt;entry&gt; = 17 homepage essays, 5/5 security headers.</t>
         </is>
       </c>
       <c r="I53" s="6" t="inlineStr"/>
@@ -3220,7 +3220,7 @@
       </c>
       <c r="H54" s="6" t="inlineStr">
         <is>
-          <t>PASS — feed.xsl 200 and &lt;?xml-stylesheet?&gt; PI present | 2026-08-13 re-verified live: /feed.xsl 200 and referenced via &lt;?xml-stylesheet?&gt; in the feed prolog. | 2026-08-25 re-verified live: /feed.xsl 200 and feed.xml carries &lt;?xml-stylesheet href="/feed.xsl"?&gt;. | 2026-08-27 re-verified live: feed.xsl 200 and the &lt;?xml-stylesheet?&gt; PI is present. | 2026-09-01 re-verified live: /feed.xml carries the &lt;?xml-stylesheet?&gt; reference and /feed.xsl returns 200. | 2026-09-06 re-verified live: feed.xsl 200 (4342b) and the feed still declares &lt;?xml-stylesheet href="/feed.xsl"?&gt;. | 2026-09-11 re-verified live: feed carries &lt;?xml-stylesheet type='text/xsl' href='/feed.xsl'?&gt; and /feed.xsl returns 200 and parses. | 2026-09-28: live: feed.xsl 200 application/xml; xml-stylesheet PI present; style-src unsafe-inline on /feed.xml + /feed.xsl.</t>
+          <t>PASS — feed.xsl 200 and &lt;?xml-stylesheet?&gt; PI present | 2026-08-13 re-verified live: /feed.xsl 200 and referenced via &lt;?xml-stylesheet?&gt; in the feed prolog. | 2026-08-25 re-verified live: /feed.xsl 200 and feed.xml carries &lt;?xml-stylesheet href="/feed.xsl"?&gt;. | 2026-08-27 re-verified live: feed.xsl 200 and the &lt;?xml-stylesheet?&gt; PI is present. | 2026-09-01 re-verified live: /feed.xml carries the &lt;?xml-stylesheet?&gt; reference and /feed.xsl returns 200. | 2026-09-06 re-verified live: feed.xsl 200 (4342b) and the feed still declares &lt;?xml-stylesheet href="/feed.xsl"?&gt;. | 2026-09-11 re-verified live: feed carries &lt;?xml-stylesheet type='text/xsl' href='/feed.xsl'?&gt; and /feed.xsl returns 200 and parses. | 2026-09-28: live: feed.xsl 200 application/xml; xml-stylesheet PI present; style-src unsafe-inline on /feed.xml + /feed.xsl. | 2026-10-04: live: /feed.xsl 200 and referenced by the &lt;?xml-stylesheet?&gt; PI.</t>
         </is>
       </c>
       <c r="I54" s="6" t="inlineStr"/>
@@ -3273,7 +3273,7 @@
       </c>
       <c r="H55" s="6" t="inlineStr">
         <is>
-          <t>PASS — 5 anchor links, all resolve to real targets | 2026-08-27 re-verified live: 5 anchor links on /phase0/, all resolve to real targets. | 2026-09-01 re-verified live: /phase0/ 200 in 0.41s, single h1, no skipped heading levels across a 22-heading tree, 0 contrast failures across 106 measured elements. | 2026-09-19 re-verified live: /phase0/ 200 in 0.39s, single h1, 0 contrast failures across 105 elements in both modes, no horizontal overflow at 375px. | 2026-09-28: live: anchors #phase0/#get/#definition all resolve; single h1; tokens + shell + phase0 css.</t>
+          <t>PASS — 5 anchor links, all resolve to real targets | 2026-08-27 re-verified live: 5 anchor links on /phase0/, all resolve to real targets. | 2026-09-01 re-verified live: /phase0/ 200 in 0.41s, single h1, no skipped heading levels across a 22-heading tree, 0 contrast failures across 106 measured elements. | 2026-09-19 re-verified live: /phase0/ 200 in 0.39s, single h1, 0 contrast failures across 105 elements in both modes, no horizontal overflow at 375px. | 2026-09-28: live: anchors #phase0/#get/#definition all resolve; single h1; tokens + shell + phase0 css. | 2026-10-04: live: /phase0/ 200 (0.50s), 10 sections, CTAs 'Get The Prompt'→#get / 'Read The System'→#definition, 5 anchor links all resolve, tokens+shell+phase0 CSS, single h1, 0 console errors.</t>
         </is>
       </c>
       <c r="I55" s="6" t="inlineStr"/>
@@ -3326,7 +3326,7 @@
       </c>
       <c r="H56" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: /phase0/ form action is /api/subscribe with no legacy Mailchimp query string; matches the other three subscribe surfaces. | 2026-08-27 re-verified live: /phase0/ form action=/api/subscribe, honeypot present, source=phase0. | 2026-09-19 re-verified live: /phase0/ .phase0-capture posts to /api/subscribe with empty honeypot (name=website), source=phase0, noscript fallback and phase0.js present. | 2026-09-28 ISSUE/Medium — the first time the validation branch was exercised (every prior check read the form's action/honeypot/source only): a mistyped email shows 'Something broke on our end. Try again, or email dex@imjustdex.com.' through the role=alert, assertive error region. Cause: js/phase0.js calls setError() with no copy on client-side validation failure, and the error &lt;p&gt; ships holding the server-failure line. A 400 invalid_email or 429 rate_limited from the function also rendered the outage line. The user story's 'not lie on failure' is broken for every reader with a typo. Measured live on /phase0/ (aria-invalid=true, 0 POSTs, visible .form-msg = outage copy), then reproduced 4/8 scenario failures by running the pre-fix file in a stub-DOM harness.</t>
+          <t>PASS — live-verified 2026-08-10: /phase0/ form action is /api/subscribe with no legacy Mailchimp query string; matches the other three subscribe surfaces. | 2026-08-27 re-verified live: /phase0/ form action=/api/subscribe, honeypot present, source=phase0. | 2026-09-19 re-verified live: /phase0/ .phase0-capture posts to /api/subscribe with empty honeypot (name=website), source=phase0, noscript fallback and phase0.js present. | 2026-09-28 ISSUE/Medium — the first time the validation branch was exercised (every prior check read the form's action/honeypot/source only): a mistyped email shows 'Something broke on our end. Try again, or email dex@imjustdex.com.' through the role=alert, assertive error region. Cause: js/phase0.js calls setError() with no copy on client-side validation failure, and the error &lt;p&gt; ships holding the server-failure line. A 400 invalid_email or 429 rate_limited from the function also rendered the outage line. The user story's 'not lie on failure' is broken for every reader with a typo. Measured live on /phase0/ (aria-invalid=true, 0 POSTs, visible .form-msg = outage copy), then reproduced 4/8 scenario failures by running the pre-fix file in a stub-DOM harness. | 2026-10-04: live: form action /api/subscribe, data-no-signup-js, source=phase0, honeypot present, noscript present. Invalid email → aria-invalid=true + 'That email didn’t look right.' with zero fetches; valid keystroke clears aria-invalid and hides the msg (state idle).</t>
         </is>
       </c>
       <c r="I56" s="6" t="inlineStr">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="H57" s="6" t="inlineStr">
         <is>
-          <t>PASS — footer year 2026 = current year | 2026-08-27 re-verified live: phase0 footer year 2026. | 2026-09-19 re-verified live: #yr reads 2026 = current year on /phase0/. | 2026-09-28: live: #yr = 2026.</t>
+          <t>PASS — footer year 2026 = current year | 2026-08-27 re-verified live: phase0 footer year 2026. | 2026-09-19 re-verified live: #yr reads 2026 = current year on /phase0/. | 2026-09-28: live: #yr = 2026. | 2026-10-04: live: #yr = 2026 = current year.</t>
         </is>
       </c>
       <c r="I57" s="6" t="inlineStr"/>
@@ -3436,7 +3436,7 @@
       </c>
       <c r="H58" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: /brand/ serves plates.css?v=phase15, matching every other surface; no second year-long cache entry. | 2026-09-01 re-verified live: /brand/ 200, single h1, no skipped heading levels, 0 contrast failures across 800 measured elements in dark mode. | 2026-09-22 re-verified live: /brand/ 200 in 0.48s; CSP style-src 'self' 'unsafe-inline' (scoped override intact); 0 inline &lt;script&gt; (mode.js + JSON-LD + Netlify RUM only); present in sitemap-0.xml; 680 text elements swept in dark mode, 0 contrast failures; image-plate specimens keep display:flex + justify-content:flex-end (no F100 regression). | 2026-09-28: live: /brand/ 200, scoped CSP style-src unsafe-inline, 0 inline scripts, in sitemap; 776 elements 0 contrast failures in both modes; image-plate specimens flex/flex-end, titles at 0.61-0.81 of plate height. Catalog note: expected cites brand.js, retired with the v2 build (ed10576) — the page ships no scripts; not a defect.</t>
+          <t>PASS — live-verified 2026-08-10: /brand/ serves plates.css?v=phase15, matching every other surface; no second year-long cache entry. | 2026-09-01 re-verified live: /brand/ 200, single h1, no skipped heading levels, 0 contrast failures across 800 measured elements in dark mode. | 2026-09-22 re-verified live: /brand/ 200 in 0.48s; CSP style-src 'self' 'unsafe-inline' (scoped override intact); 0 inline &lt;script&gt; (mode.js + JSON-LD + Netlify RUM only); present in sitemap-0.xml; 680 text elements swept in dark mode, 0 contrast failures; image-plate specimens keep display:flex + justify-content:flex-end (no F100 regression). | 2026-09-28: live: /brand/ 200, scoped CSP style-src unsafe-inline, 0 inline scripts, in sitemap; 776 elements 0 contrast failures in both modes; image-plate specimens flex/flex-end, titles at 0.61-0.81 of plate height. Catalog note: expected cites brand.js, retired with the v2 build (ed10576) — the page ships no scripts; not a defect. | 2026-10-04: live: /brand/ 200, single h1, no skipped heading levels, 41 swatches / 115 demo nodes, 0 inline scripts (mode.js + Netlify RUM only), .demo-plate-body flex/flex-end (no F100 regression), in sitemap-0.xml, 0 console errors. brand.js retired (see 09-28 note).</t>
         </is>
       </c>
       <c r="I58" s="6" t="inlineStr"/>
@@ -3489,7 +3489,7 @@
       </c>
       <c r="H59" s="6" t="inlineStr">
         <is>
-          <t>PASS — GET /api/subscribe → 405 method_not_allowed | 2026-08-25 re-verified live: /api/subscribe reachable and behaving; rewrite chain intact. | 2026-08-27 re-verified live: GET /api/subscribe → 405 method_not_allowed. | 2026-09-06 re-verified live: GET /api/subscribe -&gt; 405. | 2026-09-11 re-verified live: GET /api/subscribe → 405 {'ok':false,'error':'method_not_allowed'}. | 2026-09-22 re-verified live: GET /api/subscribe -&gt; 405 {'ok':false,'error':'method_not_allowed'}; PUT -&gt; 405 likewise. | 2026-09-28: live: GET and PUT -&gt; 405 method_not_allowed.</t>
+          <t>PASS — GET /api/subscribe → 405 method_not_allowed | 2026-08-25 re-verified live: /api/subscribe reachable and behaving; rewrite chain intact. | 2026-08-27 re-verified live: GET /api/subscribe → 405 method_not_allowed. | 2026-09-06 re-verified live: GET /api/subscribe -&gt; 405. | 2026-09-11 re-verified live: GET /api/subscribe → 405 {'ok':false,'error':'method_not_allowed'}. | 2026-09-22 re-verified live: GET /api/subscribe -&gt; 405 {'ok':false,'error':'method_not_allowed'}; PUT -&gt; 405 likewise. | 2026-09-28: live: GET and PUT -&gt; 405 method_not_allowed. | 2026-10-04: live: GET /api/subscribe → 405 {ok:false,error:method_not_allowed}.</t>
         </is>
       </c>
       <c r="I59" s="6" t="inlineStr"/>
@@ -3542,7 +3542,7 @@
       </c>
       <c r="H60" s="6" t="inlineStr">
         <is>
-          <t>PASS — rate-limit bucket present (5/60s per IP) | 2026-09-11 re-verified live: burst of 8 POSTs from one IP: 400 invalid_email ×2 then 429 rate_limited ×6 — the 5/60s window fires as specified. | 2026-09-22 re-verified live: sequential burst of 10 POSTs (email=notanemail) from a quiet start returned exactly 5 x 400 invalid_email then 5 x 429 rate_limited — the 5/60s window fires as specified. A PARALLEL burst of 10 returned 10 x 400 and no 429: the window is a module-scope Map, so it is per Lambda instance and parallel requests fan out. Recorded as a measurement antipattern in QA-OS.md [F107]; not a defect. | 2026-09-28: live: SEQUENTIAL burst of 10 (email=notanemail) from a quiet start -&gt; exactly 5 x 400 then 5 x 429.</t>
+          <t>PASS — rate-limit bucket present (5/60s per IP) | 2026-09-11 re-verified live: burst of 8 POSTs from one IP: 400 invalid_email ×2 then 429 rate_limited ×6 — the 5/60s window fires as specified. | 2026-09-22 re-verified live: sequential burst of 10 POSTs (email=notanemail) from a quiet start returned exactly 5 x 400 invalid_email then 5 x 429 rate_limited — the 5/60s window fires as specified. A PARALLEL burst of 10 returned 10 x 400 and no 429: the window is a module-scope Map, so it is per Lambda instance and parallel requests fan out. Recorded as a measurement antipattern in QA-OS.md [F107]; not a defect. | 2026-09-28: live: SEQUENTIAL burst of 10 (email=notanemail) from a quiet start -&gt; exactly 5 x 400 then 5 x 429. | 2026-10-04: live: SEQUENTIAL burst of 10 × email=notanemail from a quiet start → exactly 400×5 then 429×5 (rate_limited), as specified.</t>
         </is>
       </c>
       <c r="I60" s="6" t="inlineStr"/>
@@ -3595,7 +3595,7 @@
       </c>
       <c r="H61" s="6" t="inlineStr">
         <is>
-          <t>PASS — filled honeypot → 200 silent success, no Mailchimp write; field off-canvas (left:-5000px, tabindex -1, aria-hidden) | 2026-08-25 re-verified live: honeypot re-verified live: POST with website=spam returned HTTP 200 {"ok":true,"message":"subscribed"} — the intended silent drop, indistinguishable from success to a bot. | 2026-08-27 re-verified live: filled honeypot → 200 silent success. | 2026-09-06 re-verified live: filled honeypot (website=spam) -&gt; 200 {ok:true,message:'subscribed'} with no Mailchimp write (subscribe.cjs:67-69 short-circuits before the email is read). | 2026-09-11 re-verified live: POST with website=spam → 200 {'ok':true,'message':'subscribed'} and no Mailchimp call. Confirmed against subscribe.cjs:65-67 that this is the intended silent fake-success, NOT a bypass — the handler returns before the Mailchimp branch. | 2026-09-22 re-verified live: POST with website=http://spam.example -&gt; 200 {'ok':true,'message':'subscribed'}, the intended silent drop, no Mailchimp write. | 2026-09-28: live: filled honeypot -&gt; 200 {ok:true,message:subscribed}, silent.</t>
+          <t>PASS — filled honeypot → 200 silent success, no Mailchimp write; field off-canvas (left:-5000px, tabindex -1, aria-hidden) | 2026-08-25 re-verified live: honeypot re-verified live: POST with website=spam returned HTTP 200 {"ok":true,"message":"subscribed"} — the intended silent drop, indistinguishable from success to a bot. | 2026-08-27 re-verified live: filled honeypot → 200 silent success. | 2026-09-06 re-verified live: filled honeypot (website=spam) -&gt; 200 {ok:true,message:'subscribed'} with no Mailchimp write (subscribe.cjs:67-69 short-circuits before the email is read). | 2026-09-11 re-verified live: POST with website=spam → 200 {'ok':true,'message':'subscribed'} and no Mailchimp call. Confirmed against subscribe.cjs:65-67 that this is the intended silent fake-success, NOT a bypass — the handler returns before the Mailchimp branch. | 2026-09-22 re-verified live: POST with website=http://spam.example -&gt; 200 {'ok':true,'message':'subscribed'}, the intended silent drop, no Mailchimp write. | 2026-09-28: live: filled honeypot -&gt; 200 {ok:true,message:subscribed}, silent. | 2026-10-04: live: POST with website filled → 200 {ok:true,message:subscribed} in 0.64s vs 2.15s for the real smoke subscribe — consistent with the short-circuit before Mailchimp.</t>
         </is>
       </c>
       <c r="I61" s="6" t="inlineStr"/>

</xml_diff>

<commit_message>
audit(ledger): 2026-10-05 full regression — F109 opened + fixed, F01-F108 PASS
Monday full-ledger regression. 109 rows. F109 (new, ISSUE/Medium) is the
backward-nav stitch: send-someone-else's prev skipped four essays. It is
fixed in c0479c8 and verified against the build. Every other row holds:
PASS, or N/A by decision.

QA-OS.md gains two measurement antipatterns: hover transitions freeze
in the hidden pane, and resetting a form's innerHTML between stubbed
submits leaves the form to submit natively.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Features'!$A$3:$K$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Features'!$A$3:$K$112</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K111"/>
+  <dimension ref="A1:K112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -646,7 +646,7 @@
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>PASS — masthead .brand-block → '/' present on home/about/404/phase0/brand/article; aria-label 'Dexter Jakes home' | 2026-08-15 re-verified live: brand-block present and linking / on all 20 pages | 2026-08-25 re-verified live: brand-block present and linking / on all 20 crawled routes; aria-label intact. | 2026-08-27 re-verified live: masthead .brand-block → '/' confirmed under real Tab focus. | 2026-09-01 re-verified live: masthead .brand-block reached under a REAL Tab press (2nd stop), links '/', focus ring #c00 2px. | 2026-09-06 re-verified live: masthead .brand-block reached under a real forward Tab from the skip link and links '/'; present on all 27 crawled routes. | 2026-09-11 re-verified live: masthead .brand-block → '/' reached under a real forward Tab from the skip link on the homepage; present on all 26 crawled routes. | 2026-09-27 re-verified live: masthead .brand-block href '/' (aria-label 'Dexter Jakes home') present on all 22 crawled HTML routes incl. the unmatched-route 404 and /phase0/. | 2026-09-28: live, full regression: .brand-block -&gt; '/' on home/about/article/phase0/404.</t>
+          <t>PASS — masthead .brand-block → '/' present on home/about/404/phase0/brand/article; aria-label 'Dexter Jakes home' | 2026-08-15 re-verified live: brand-block present and linking / on all 20 pages | 2026-08-25 re-verified live: brand-block present and linking / on all 20 crawled routes; aria-label intact. | 2026-08-27 re-verified live: masthead .brand-block → '/' confirmed under real Tab focus. | 2026-09-01 re-verified live: masthead .brand-block reached under a REAL Tab press (2nd stop), links '/', focus ring #c00 2px. | 2026-09-06 re-verified live: masthead .brand-block reached under a real forward Tab from the skip link and links '/'; present on all 27 crawled routes. | 2026-09-11 re-verified live: masthead .brand-block → '/' reached under a real forward Tab from the skip link on the homepage; present on all 26 crawled routes. | 2026-09-27 re-verified live: masthead .brand-block href '/' (aria-label 'Dexter Jakes home') present on all 22 crawled HTML routes incl. the unmatched-route 404 and /phase0/. | 2026-09-28: live, full regression: .brand-block -&gt; '/' on home/about/article/phase0/404. | 2026-10-05: live, full regression: .brand-block -&gt; "/" on home/about/404/phase0/brand/articles; reached under a real Tab from the skip link (2px #c00 ring).</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>PASS — brand-word: Words (home/article/about/brand), 404, Phase 0 — matches documented intent | 2026-08-15 re-verified live: brand-word: home/about/article 'Words', 404 '404', phase0 'Phase 0' — matches the documented about-page quirk | 2026-08-25 re-verified live: brand-word: "Words" on home/about/article, "404" on /404, "Phase 0" on /phase0/ — matches documented intent. | 2026-08-27 re-verified live: brand word 'Words' confirmed on home/article/about. | 2026-09-01 re-verified live on the homepage: masthead brand word reads 'Words' (documented intent). Other surfaces not re-walked this run. | 2026-09-19 re-verified live: brand-word live: 'Words' on /, /about/, /brand/ and all 17 articles; 'Phase 0' on /phase0/; '404' on the unmatched-route 404 — matches documented intent. | 2026-09-27 re-verified live: brand-word 'Words' on /, /about/, /brand/ and all 17 articles; 'Phase 0' on /phase0/; '404' on the unmatched-route 404 — matches documented intent. | 2026-09-28: live: brand-word Words (home/about/article), Phase 0 (phase0), 404 (404).</t>
+          <t>PASS — brand-word: Words (home/article/about/brand), 404, Phase 0 — matches documented intent | 2026-08-15 re-verified live: brand-word: home/about/article 'Words', 404 '404', phase0 'Phase 0' — matches the documented about-page quirk | 2026-08-25 re-verified live: brand-word: "Words" on home/about/article, "404" on /404, "Phase 0" on /phase0/ — matches documented intent. | 2026-08-27 re-verified live: brand word 'Words' confirmed on home/article/about. | 2026-09-01 re-verified live on the homepage: masthead brand word reads 'Words' (documented intent). Other surfaces not re-walked this run. | 2026-09-19 re-verified live: brand-word live: 'Words' on /, /about/, /brand/ and all 17 articles; 'Phase 0' on /phase0/; '404' on the unmatched-route 404 — matches documented intent. | 2026-09-27 re-verified live: brand-word 'Words' on /, /about/, /brand/ and all 17 articles; 'Phase 0' on /phase0/; '404' on the unmatched-route 404 — matches documented intent. | 2026-09-28: live: brand-word Words (home/about/article), Phase 0 (phase0), 404 (404). | 2026-10-05: live: brand-word "Words" on home/about/brand/articles, "404" on /404, "Phase 0" on /phase0/.</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr"/>
@@ -748,7 +748,7 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>PASS — toggle cycles dark→light→dark; dxmode cookie written both ways; label + aria-pressed + bg/ink all update. Reconfirmed 2026-08-10 PM across 3 consecutive clicks. | 2026-08-13 re-verified live: toggle cycled dark-&gt;light-&gt;dark on the live homepage; dxmode cookie written both ways; --bg/--ink/--accent-text all re-resolved (#060606/#f3f0e8/#ff4d4d dark, #f4f4f1/#050505/#c00 light). | 2026-08-16 re-verified live: toggle cycled dark-&gt;light-&gt;dark on the live homepage; dxmode cookie written both ways (dxmode=light then dxmode=dark); --bg #060606&lt;-&gt;#f4f4f1 and --ink #f3f0e8&lt;-&gt;#050505 both re-resolved; label and aria-pressed tracked ('Mode: Dark'/true &lt;-&gt; 'Mode: Light'/false). | 2026-08-25 re-verified live: toggle re-verified with a REAL pointer click (not element.click()) on both the homepage and /words/the-stone/: page repaints dark&lt;-&gt;light, dxmode cookie written both ways, label and aria-pressed track. METHOD NOTE: a programmatic element.click() flips the class, the tokens and the cookie but leaves body's used background/color stale in getComputedStyle until a repaint is forced — that is a measurement artifact, NOT a site defect, and it read as an article-page mode regression for several minutes this run. Always verify this row with a real click. | 2026-08-27 re-verified live: REAL pointer click (not element.click()) + 2s settle + screenshot: dark→light→dark, --bg #060606↔#f4f4f1, --ink #f3f0e8↔#050505, dxmode cookie written both ways, button label tracks. | 2026-09-01 ISSUE (MEDIUM) — theme-color half of this row has NEVER been satisfiable. mode.js ships syncThemeColor() (js/mode.js:74-95) which rewrites &lt;meta name="theme-color"&gt; to #060606/#f4f4f1 and strips the media attr off a media-split pair, but NO layout ever emitted that meta: document.querySelectorAll('meta[name="theme-color"]').length === 0 on /, /about/, /words/&lt;slug&gt;/, /404, /brand/ and /phase0/ live. querySelector() returned null, the function no-opped, and the dedupe loop iterated an empty list — silent, so five months of scrubs that checked the class/cookie/tokens never saw it. User-visible effect: mobile browser chrome (address/status bar) follows the OS instead of the site's mode. Class flip, dxmode cookie, --bg/--ink re-resolve, aria-pressed, label and logo swap all re-verified live PASS this run with a REAL pointer click + 2s settle. | 2026-09-06 re-verified live: mode toggle driven with a real pointer click (not element.click()) plus a 2.5s settle. dark rgb(6,6,6)/rgb(243,240,232) -&gt; light rgb(244,244,241)/rgb(5,5,5) -&gt; dark, with the dxmode cookie and the 'Mode: Dark'/'Mode: Light' label tracking each flip. | 2026-09-11 re-verified live: real pointer click on .mode-toggle with a 2s settle: dxmode dark→light, html.dark-mode cleared, body rgb(6,6,6)→rgb(244,244,241), theme-color meta →#f4f4f1, label 'Mode: Light'. Screenshot confirmed after the wait. | 2026-09-27 re-verified live: real pointer click on the mode toggle with a 2s settle: dxmode light-&gt;dark, html.dark-mode set, body rgb(6,6,6) on ink rgb(243,240,232), theme-color #060606, aria-pressed true, label 'Mode: Dark', logo -&gt; logo-white.svg; screenshot after the wait confirmed the dark palette. Second real click restored light. | 2026-09-28: live: REAL pointer click light-&gt;dark, 2s settle: html.dark-mode, dxmode=dark, label 'Mode: Dark', aria-pressed true, body rgb(6,6,6) / ink rgb(243,240,232); screenshot confirmed.</t>
+          <t>PASS — toggle cycles dark→light→dark; dxmode cookie written both ways; label + aria-pressed + bg/ink all update. Reconfirmed 2026-08-10 PM across 3 consecutive clicks. | 2026-08-13 re-verified live: toggle cycled dark-&gt;light-&gt;dark on the live homepage; dxmode cookie written both ways; --bg/--ink/--accent-text all re-resolved (#060606/#f3f0e8/#ff4d4d dark, #f4f4f1/#050505/#c00 light). | 2026-08-16 re-verified live: toggle cycled dark-&gt;light-&gt;dark on the live homepage; dxmode cookie written both ways (dxmode=light then dxmode=dark); --bg #060606&lt;-&gt;#f4f4f1 and --ink #f3f0e8&lt;-&gt;#050505 both re-resolved; label and aria-pressed tracked ('Mode: Dark'/true &lt;-&gt; 'Mode: Light'/false). | 2026-08-25 re-verified live: toggle re-verified with a REAL pointer click (not element.click()) on both the homepage and /words/the-stone/: page repaints dark&lt;-&gt;light, dxmode cookie written both ways, label and aria-pressed track. METHOD NOTE: a programmatic element.click() flips the class, the tokens and the cookie but leaves body's used background/color stale in getComputedStyle until a repaint is forced — that is a measurement artifact, NOT a site defect, and it read as an article-page mode regression for several minutes this run. Always verify this row with a real click. | 2026-08-27 re-verified live: REAL pointer click (not element.click()) + 2s settle + screenshot: dark→light→dark, --bg #060606↔#f4f4f1, --ink #f3f0e8↔#050505, dxmode cookie written both ways, button label tracks. | 2026-09-01 ISSUE (MEDIUM) — theme-color half of this row has NEVER been satisfiable. mode.js ships syncThemeColor() (js/mode.js:74-95) which rewrites &lt;meta name="theme-color"&gt; to #060606/#f4f4f1 and strips the media attr off a media-split pair, but NO layout ever emitted that meta: document.querySelectorAll('meta[name="theme-color"]').length === 0 on /, /about/, /words/&lt;slug&gt;/, /404, /brand/ and /phase0/ live. querySelector() returned null, the function no-opped, and the dedupe loop iterated an empty list — silent, so five months of scrubs that checked the class/cookie/tokens never saw it. User-visible effect: mobile browser chrome (address/status bar) follows the OS instead of the site's mode. Class flip, dxmode cookie, --bg/--ink re-resolve, aria-pressed, label and logo swap all re-verified live PASS this run with a REAL pointer click + 2s settle. | 2026-09-06 re-verified live: mode toggle driven with a real pointer click (not element.click()) plus a 2.5s settle. dark rgb(6,6,6)/rgb(243,240,232) -&gt; light rgb(244,244,241)/rgb(5,5,5) -&gt; dark, with the dxmode cookie and the 'Mode: Dark'/'Mode: Light' label tracking each flip. | 2026-09-11 re-verified live: real pointer click on .mode-toggle with a 2s settle: dxmode dark→light, html.dark-mode cleared, body rgb(6,6,6)→rgb(244,244,241), theme-color meta →#f4f4f1, label 'Mode: Light'. Screenshot confirmed after the wait. | 2026-09-27 re-verified live: real pointer click on the mode toggle with a 2s settle: dxmode light-&gt;dark, html.dark-mode set, body rgb(6,6,6) on ink rgb(243,240,232), theme-color #060606, aria-pressed true, label 'Mode: Dark', logo -&gt; logo-white.svg; screenshot after the wait confirmed the dark palette. Second real click restored light. | 2026-09-28: live: REAL pointer click light-&gt;dark, 2s settle: html.dark-mode, dxmode=dark, label 'Mode: Dark', aria-pressed true, body rgb(6,6,6) / ink rgb(243,240,232); screenshot confirmed. | 2026-10-05: live: real pointer click flipped html.dark-mode, cookie dxmode=dark, label "Mode: Dark", aria-pressed true; after 2.5s settle body rgb(6,6,6). Reload kept dark (cookie wins); dxmode=light cookie + reload returned light.</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
@@ -805,7 +805,7 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: skip link is first focusable; activating it lands document.activeElement on MAIN#archive (home) / MAIN#article (essay); tabindex=-1 present on both landmarks. The 2c7d88d fix holds in production. | 2026-08-13 re-verified live: tab-target verified on live: .skip-link reveals from left:-999px to a 83x69 box at (12,12), cream-on-ink 17.79:1; activating it moved document.activeElement to MAIN#archive (tabindex=-1). Article pages target #article. | 2026-08-16 re-verified live: structural half re-verified live: .skip-link is the first focusable element in document order on every page type, and its target (MAIN#article / MAIN#archive / MAIN#phase0 / MAIN#main) carries tabindex=-1. End-to-end activation NOT re-exercisable this run — the browser pane reports document.visibilityState 'hidden' and drops page focus on every reload, so a fresh-load Tab lands on BODY. Harness limitation, not a site regression; last live activation was 2026-08-13. NOTE: this row's sweep is what surfaced F91 — see that row. | 2026-08-25 re-verified live: verified end-to-end live under REAL keyboard input on /words/the-stone/ — the gap the 2026-08-16 run had to leave open. .skip-link is the first focusable in DOM order, reveals from left:-999px to a 126x46 chip at (12,12), computes 17.79:1 (#060606 on #f3f0e8), and pressing Enter sets location.hash to #article and moves document.activeElement to MAIN#article (tabindex=-1). | 2026-08-27 re-verified live: skip link is the first focusable (reached by real shift+Tab from .brand-block), renders as an opaque cream chip at 17.79:1, and activation moves focus to MAIN#archive with hash #archive. | 2026-09-01 re-verified live: .skip-link is the FIRST Tab stop from page load and matches :focus-visible; activation moves location.hash to #archive and focus to MAIN#archive. Ran the ordinary-link control first per the harness antipattern. | 2026-09-06 re-verified live: skip link is the first focusable, unhides on focus (left -999px -&gt; 12px), and activation moved location.hash to '#archive' and focus to the #archive element. | 2026-09-11 re-verified live: skip link is the first focusable (reached by one shift+Tab back from .brand-block), 17.79:1, #c00 2px ring; activated with a real pointer click → document.activeElement === main#archive, location.hash '#archive'. | 2026-09-19 re-verified live: skip link reached under a real shift+Tab on the homepage (:focus-visible true, #060606 on cream chip, rgb(204,0,0) 2px ring); activation moves focus to #archive (tabindex -1) and sets location.hash. | 2026-09-27 re-verified live: first real Tab from load lands on .skip-link (#archive), :focus-visible true, rgb(204,0,0) 2px solid ring, rgb(244,244,241) on rgb(5,5,5) chip; activation moved focus to #archive and set location.hash. | 2026-09-28: live: real shift+Tab lands on .skip-link (:focus-visible); activation -&gt; #archive, focus on #archive.</t>
+          <t>PASS — live-verified 2026-08-10: skip link is first focusable; activating it lands document.activeElement on MAIN#archive (home) / MAIN#article (essay); tabindex=-1 present on both landmarks. The 2c7d88d fix holds in production. | 2026-08-13 re-verified live: tab-target verified on live: .skip-link reveals from left:-999px to a 83x69 box at (12,12), cream-on-ink 17.79:1; activating it moved document.activeElement to MAIN#archive (tabindex=-1). Article pages target #article. | 2026-08-16 re-verified live: structural half re-verified live: .skip-link is the first focusable element in document order on every page type, and its target (MAIN#article / MAIN#archive / MAIN#phase0 / MAIN#main) carries tabindex=-1. End-to-end activation NOT re-exercisable this run — the browser pane reports document.visibilityState 'hidden' and drops page focus on every reload, so a fresh-load Tab lands on BODY. Harness limitation, not a site regression; last live activation was 2026-08-13. NOTE: this row's sweep is what surfaced F91 — see that row. | 2026-08-25 re-verified live: verified end-to-end live under REAL keyboard input on /words/the-stone/ — the gap the 2026-08-16 run had to leave open. .skip-link is the first focusable in DOM order, reveals from left:-999px to a 126x46 chip at (12,12), computes 17.79:1 (#060606 on #f3f0e8), and pressing Enter sets location.hash to #article and moves document.activeElement to MAIN#article (tabindex=-1). | 2026-08-27 re-verified live: skip link is the first focusable (reached by real shift+Tab from .brand-block), renders as an opaque cream chip at 17.79:1, and activation moves focus to MAIN#archive with hash #archive. | 2026-09-01 re-verified live: .skip-link is the FIRST Tab stop from page load and matches :focus-visible; activation moves location.hash to #archive and focus to MAIN#archive. Ran the ordinary-link control first per the harness antipattern. | 2026-09-06 re-verified live: skip link is the first focusable, unhides on focus (left -999px -&gt; 12px), and activation moved location.hash to '#archive' and focus to the #archive element. | 2026-09-11 re-verified live: skip link is the first focusable (reached by one shift+Tab back from .brand-block), 17.79:1, #c00 2px ring; activated with a real pointer click → document.activeElement === main#archive, location.hash '#archive'. | 2026-09-19 re-verified live: skip link reached under a real shift+Tab on the homepage (:focus-visible true, #060606 on cream chip, rgb(204,0,0) 2px ring); activation moves focus to #archive (tabindex -1) and sets location.hash. | 2026-09-27 re-verified live: first real Tab from load lands on .skip-link (#archive), :focus-visible true, rgb(204,0,0) 2px solid ring, rgb(244,244,241) on rgb(5,5,5) chip; activation moved focus to #archive and set location.hash. | 2026-09-28: live: real shift+Tab lands on .skip-link (:focus-visible); activation -&gt; #archive, focus on #archive. | 2026-10-05: live: shift+Tab from a neutral click lands on .skip-link (#archive) inside the viewport; activation sets #archive and focus.</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr"/>
@@ -858,7 +858,7 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>PASS — 2 decorative rulers render | 2026-08-15 re-verified live: zero .ruler-* without aria-hidden across all pages | 2026-09-11 re-verified live: 2 rulers on each of home/article/about/404/phase0, every one aria-hidden=true. | 2026-09-27 re-verified live: 2 rulers on each of 22 crawled HTML routes, every one aria-hidden=true. | 2026-09-28: live: 2 aria-hidden rulers on all 5 page types.</t>
+          <t>PASS — 2 decorative rulers render | 2026-08-15 re-verified live: zero .ruler-* without aria-hidden across all pages | 2026-09-11 re-verified live: 2 rulers on each of home/article/about/404/phase0, every one aria-hidden=true. | 2026-09-27 re-verified live: 2 rulers on each of 22 crawled HTML routes, every one aria-hidden=true. | 2026-09-28: live: 2 aria-hidden rulers on all 5 page types. | 2026-10-05: live: .ruler-top/.ruler-left aria-hidden="true" on all 7 page types.</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr"/>
@@ -907,7 +907,7 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>PASS — footer strip + links present on all page types | 2026-08-15 re-verified live: footer: Instagram + X both target=_blank rel="noopener noreferrer", /feed.xml, /about/, "Built by Dex"; zero _blank links missing rel site-wide | 2026-08-25 re-verified live: footer links resolve: instagram.com/ImJustDex 200, x.com/ImJustDex 200, /feed.xml 200. | 2026-09-11 re-verified live: footer Instagram + X both target=_blank rel='noopener noreferrer', Feed → /feed.xml, About present on home only; 'Built by Dex · Est. 2026' on all three. | 2026-09-27 re-verified live: homepage footer Instagram + X both target=_blank rel='noopener noreferrer', Feed -&gt; /feed.xml, About present; 'Built by Dex · Est. 2026' on home, about, brand, 404 and all 17 articles (/phase0/ carries its own bespoke footer by design); all external footer links 200. | 2026-09-28: live: footer IG + X target=_blank rel=noopener noreferrer, Feed, 'Est. 2026' on home/about/article/404; About on home only; /phase0/ keeps its bespoke footer (Get Prompt · Essays · year) by design.</t>
+          <t>PASS — footer strip + links present on all page types | 2026-08-15 re-verified live: footer: Instagram + X both target=_blank rel="noopener noreferrer", /feed.xml, /about/, "Built by Dex"; zero _blank links missing rel site-wide | 2026-08-25 re-verified live: footer links resolve: instagram.com/ImJustDex 200, x.com/ImJustDex 200, /feed.xml 200. | 2026-09-11 re-verified live: footer Instagram + X both target=_blank rel='noopener noreferrer', Feed → /feed.xml, About present on home only; 'Built by Dex · Est. 2026' on all three. | 2026-09-27 re-verified live: homepage footer Instagram + X both target=_blank rel='noopener noreferrer', Feed -&gt; /feed.xml, About present; 'Built by Dex · Est. 2026' on home, about, brand, 404 and all 17 articles (/phase0/ carries its own bespoke footer by design); all external footer links 200. | 2026-09-28: live: footer IG + X target=_blank rel=noopener noreferrer, Feed, 'Est. 2026' on home/about/article/404; About on home only; /phase0/ keeps its bespoke footer (Get Prompt · Essays · year) by design. | 2026-10-05: live: footer Instagram + X (_blank, noopener noreferrer), Feed, About (home); "Built by Dex · Est. 2026".</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr"/>
@@ -956,7 +956,7 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>PASS (2026-08-15 scrub) — home/about/phase0/articles all carry the feed discovery link; /404 correctly omits it. NOTE: the prior `expected` said articles do NOT include it. That text was stale — ArticleLayout has emitted the link since a4f4f25; the site was never wrong, the row was. Expectation corrected, not the code. | 2026-08-25 re-verified live: &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present in head. | 2026-09-01 re-verified live: &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present in head; /feed.xml 200. | 2026-09-19 re-verified live: feed discovery &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present on /, /about/, /phase0/, /brand/ and all 17 articles; absent on the 404 as specified. | 2026-09-28: live: atom alternate link on home/about/phase0/article; absent on 404 as specified. | 2026-09-29: live: atom alternate link on home/about/phase0/brand + all 17 articles; absent on the 404 as specified.</t>
+          <t>PASS (2026-08-15 scrub) — home/about/phase0/articles all carry the feed discovery link; /404 correctly omits it. NOTE: the prior `expected` said articles do NOT include it. That text was stale — ArticleLayout has emitted the link since a4f4f25; the site was never wrong, the row was. Expectation corrected, not the code. | 2026-08-25 re-verified live: &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present in head. | 2026-09-01 re-verified live: &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present in head; /feed.xml 200. | 2026-09-19 re-verified live: feed discovery &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present on /, /about/, /phase0/, /brand/ and all 17 articles; absent on the 404 as specified. | 2026-09-28: live: atom alternate link on home/about/phase0/article; absent on 404 as specified. | 2026-09-29: live: atom alternate link on home/about/phase0/brand + all 17 articles; absent on the 404 as specified. | 2026-10-05: live: atom alternate link on home/about/phase0/brand/articles; absent on /404 as specified.</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr"/>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>PASS — /img/favicon-32.png + /img/apple-touch-icon.png 200 on every referenced path | 2026-08-15 re-verified live: favicon-32.png + apple-touch-icon.png linked on every page; both 200 (1327b / 5729b) | 2026-08-25 re-verified live: /img/favicon-32.png 200, /img/apple-touch-icon.png 200 on every referenced path. | 2026-08-27 re-verified live: /img/favicon-32.png + /img/apple-touch-icon.png 200. | 2026-09-01 re-verified live: /img/favicon-32.png 200, /img/apple-touch-icon.png 200, /img/logo-dark.svg 200. | 2026-09-06 re-verified live: /img/favicon-32.png 200 (1327b), /img/apple-touch-icon.png 200 (5729b), /img/logo-dark.svg 200. | 2026-09-11 re-verified live: /img/favicon-32.png and /img/apple-touch-icon.png both 200, served public,max-age=31536000,immutable. | 2026-09-28: live: favicon-32 + apple-touch-icon linked on all 5 page types; both 200 immutable. | 2026-09-29: live: favicon-32 + apple-touch-icon linked on all 22 routes; both 200 immutable.</t>
+          <t>PASS — /img/favicon-32.png + /img/apple-touch-icon.png 200 on every referenced path | 2026-08-15 re-verified live: favicon-32.png + apple-touch-icon.png linked on every page; both 200 (1327b / 5729b) | 2026-08-25 re-verified live: /img/favicon-32.png 200, /img/apple-touch-icon.png 200 on every referenced path. | 2026-08-27 re-verified live: /img/favicon-32.png + /img/apple-touch-icon.png 200. | 2026-09-01 re-verified live: /img/favicon-32.png 200, /img/apple-touch-icon.png 200, /img/logo-dark.svg 200. | 2026-09-06 re-verified live: /img/favicon-32.png 200 (1327b), /img/apple-touch-icon.png 200 (5729b), /img/logo-dark.svg 200. | 2026-09-11 re-verified live: /img/favicon-32.png and /img/apple-touch-icon.png both 200, served public,max-age=31536000,immutable. | 2026-09-28: live: favicon-32 + apple-touch-icon linked on all 5 page types; both 200 immutable. | 2026-09-29: live: favicon-32 + apple-touch-icon linked on all 22 routes; both 200 immutable. | 2026-10-05: live: favicon-32 + apple-touch-icon linked on all page types; both 200.</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr"/>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>PASS — Anton + IBM Plex Sans self-hosted, preloaded, document.fonts status 'loaded'; CSP font-src intact | 2026-08-15 re-verified live: Anton + IBM Plex Sans preloaded with crossorigin; zero Google Fonts refs; document.fonts reports all 3 faces loaded | 2026-08-16 re-verified live: Anton + IBM Plex Sans (Regular/Bold) all report document.fonts status 'loaded', document.fonts.status 'loaded'; zero Google Fonts references. /brand/ additionally preloads IBMPlexSans-Italic.woff2 and the console warns it is 'not used within a few seconds of load' — investigated and DISMISSED as a non-finding: the italic face is genuinely used by 13 elements on that page and reports status 'loaded'; the warning is a below-the-fold timing artifact. No other page preloads italic, which is correct. | 2026-08-25 re-verified live: document.fonts.status "loaded"; Anton/400, IBM Plex Sans/400 and /700 all report loaded. All three woff2 200. No FOUT observed. | 2026-08-27 re-verified live: document.fonts: Anton 400, IBM Plex Sans 400 + 700 all 'loaded'; fonts.status 'loaded'; no FOUT observed. | 2026-09-01 re-verified live via document.fonts (not the CSS stack): Anton 400 loaded, IBM Plex Sans 400 + 700 loaded; document.fonts.check() true for all three on home and article. No FOUT/FOIT observed. | 2026-09-06 re-verified live: document.fonts reports Anton 400, IBM Plex Sans 400 and 700 all 'loaded' on home and article; all three woff2 files 200 with immutable cache-control. No FOUT observed. | 2026-09-11 re-verified live: document.fonts reports Anton 400 loaded and IBM Plex Sans 400/700 loaded; fonts.check() true for both families. No FOUT observed. | 2026-09-28: live: document.fonts loaded Anton 400 + IBM Plex Sans 400/700; font preload with crossorigin on all 5 page types; no Google Fonts. | 2026-09-29: live: document.fonts 'loaded' — Anton 400, IBM Plex Sans 400/700; 3 font preloads with crossorigin on every non-/brand/ route; 0 Google Fonts refs.</t>
+          <t>PASS — Anton + IBM Plex Sans self-hosted, preloaded, document.fonts status 'loaded'; CSP font-src intact | 2026-08-15 re-verified live: Anton + IBM Plex Sans preloaded with crossorigin; zero Google Fonts refs; document.fonts reports all 3 faces loaded | 2026-08-16 re-verified live: Anton + IBM Plex Sans (Regular/Bold) all report document.fonts status 'loaded', document.fonts.status 'loaded'; zero Google Fonts references. /brand/ additionally preloads IBMPlexSans-Italic.woff2 and the console warns it is 'not used within a few seconds of load' — investigated and DISMISSED as a non-finding: the italic face is genuinely used by 13 elements on that page and reports status 'loaded'; the warning is a below-the-fold timing artifact. No other page preloads italic, which is correct. | 2026-08-25 re-verified live: document.fonts.status "loaded"; Anton/400, IBM Plex Sans/400 and /700 all report loaded. All three woff2 200. No FOUT observed. | 2026-08-27 re-verified live: document.fonts: Anton 400, IBM Plex Sans 400 + 700 all 'loaded'; fonts.status 'loaded'; no FOUT observed. | 2026-09-01 re-verified live via document.fonts (not the CSS stack): Anton 400 loaded, IBM Plex Sans 400 + 700 loaded; document.fonts.check() true for all three on home and article. No FOUT/FOIT observed. | 2026-09-06 re-verified live: document.fonts reports Anton 400, IBM Plex Sans 400 and 700 all 'loaded' on home and article; all three woff2 files 200 with immutable cache-control. No FOUT observed. | 2026-09-11 re-verified live: document.fonts reports Anton 400 loaded and IBM Plex Sans 400/700 loaded; fonts.check() true for both families. No FOUT observed. | 2026-09-28: live: document.fonts loaded Anton 400 + IBM Plex Sans 400/700; font preload with crossorigin on all 5 page types; no Google Fonts. | 2026-09-29: live: document.fonts 'loaded' — Anton 400, IBM Plex Sans 400/700; 3 font preloads with crossorigin on every non-/brand/ route; 0 Google Fonts refs. | 2026-10-05: live: Anton 400, Plex 400/700 (+400 italic on articles) loaded via document.fonts; font preloads carry crossorigin; no Google Fonts; font ACAO *.</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr"/>
@@ -1107,7 +1107,7 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>PASS — no horizontal overflow at 390px on home/article/about/phase0/brand/404 | 2026-08-15 re-verified live: viewport width=device-width + viewport-fit=cover on all pages | 2026-09-01 re-verified live at an emulated 375x812: documentElement.scrollWidth == clientWidth == 375 on the article page — zero horizontal overflow. | 2026-09-06 re-verified live at 375x812: homepage and article scrollWidth == clientWidth (no horizontal overflow). | 2026-09-11 re-verified live: 375px homepage and article: scrollWidth == clientWidth == 375, zero elements overflowing the client width, 17 plates intact. | 2026-09-28: live: viewport meta (width=device-width, viewport-fit=cover) on all 5 types; at 390px scrollWidth == 390 and 0 overflowing elements on home/article/about/phase0/brand. | 2026-09-29: live: viewport meta width=device-width on all 22 routes; at 390x844 scrollWidth == clientWidth == 390 on home/article/about/phase0/brand/404.</t>
+          <t>PASS — no horizontal overflow at 390px on home/article/about/phase0/brand/404 | 2026-08-15 re-verified live: viewport width=device-width + viewport-fit=cover on all pages | 2026-09-01 re-verified live at an emulated 375x812: documentElement.scrollWidth == clientWidth == 375 on the article page — zero horizontal overflow. | 2026-09-06 re-verified live at 375x812: homepage and article scrollWidth == clientWidth (no horizontal overflow). | 2026-09-11 re-verified live: 375px homepage and article: scrollWidth == clientWidth == 375, zero elements overflowing the client width, 17 plates intact. | 2026-09-28: live: viewport meta (width=device-width, viewport-fit=cover) on all 5 types; at 390px scrollWidth == 390 and 0 overflowing elements on home/article/about/phase0/brand. | 2026-09-29: live: viewport meta width=device-width on all 22 routes; at 390x844 scrollWidth == clientWidth == 390 on home/article/about/phase0/brand/404. | 2026-10-05: live: viewport width=device-width, viewport-fit=cover everywhere; at 375px home/article/about/phase0 scrollWidth == 375, 0 elements past the edge.</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr"/>
@@ -1160,7 +1160,7 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>PASS — title/description/canonical on all 21 routes; every canonical on imjustdex.com | 2026-08-15 re-verified live: zero duplicate &lt;title&gt; across 20 pages; /404 canonical is /404 as specified | 2026-08-25 re-verified live: &lt;title&gt;, meta description and canonical present and correct on all 20 routes; every canonical points at imjustdex.com. | 2026-08-27 re-verified live: title/description/canonical present and on-domain across all 21 routes. | 2026-09-01 re-verified live: &lt;title&gt;, meta description and canonical present on all 17 articles plus / and /about/; canonicals all on imjustdex.com. | 2026-09-06 re-verified live: title, meta description and canonical present on all 5 chrome pages and all 17 articles; every canonical on https://imjustdex.com/. | 2026-09-11 re-verified live: title/description/canonical present and imjustdex.com-absolute on all 17 articles + home/about/brand/phase0/404. | 2026-09-28: live: title + description + canonical on all 21 indexable routes; 404 canonical /404. | 2026-09-29: live: 0 duplicate titles across 21 indexable routes; every canonical is self-referencing on imjustdex.com; 404 canonical /404.</t>
+          <t>PASS — title/description/canonical on all 21 routes; every canonical on imjustdex.com | 2026-08-15 re-verified live: zero duplicate &lt;title&gt; across 20 pages; /404 canonical is /404 as specified | 2026-08-25 re-verified live: &lt;title&gt;, meta description and canonical present and correct on all 20 routes; every canonical points at imjustdex.com. | 2026-08-27 re-verified live: title/description/canonical present and on-domain across all 21 routes. | 2026-09-01 re-verified live: &lt;title&gt;, meta description and canonical present on all 17 articles plus / and /about/; canonicals all on imjustdex.com. | 2026-09-06 re-verified live: title, meta description and canonical present on all 5 chrome pages and all 17 articles; every canonical on https://imjustdex.com/. | 2026-09-11 re-verified live: title/description/canonical present and imjustdex.com-absolute on all 17 articles + home/about/brand/phase0/404. | 2026-09-28: live: title + description + canonical on all 21 indexable routes; 404 canonical /404. | 2026-09-29: live: 0 duplicate titles across 21 indexable routes; every canonical is self-referencing on imjustdex.com; 404 canonical /404. | 2026-10-05: live: 22 HTML routes with unique titles, descriptions and imjustdex.com canonicals; 0 findings.</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr"/>
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>PASS — og+twitter complete on all 21; all 19 OG images 200 (16 essays + home/about/phase0/brand) | 2026-08-15 re-verified live: twitter:card summary_large_image on every page in scope (404 correctly excluded) | 2026-08-25 re-verified live: og:title / og:description / og:image present on all 20; all 16 og-&lt;slug&gt;.png 200; og:image byte-identical to the JSON-LD image on all 16. | 2026-08-27 re-verified live: og+twitter complete across 21 routes; all 21 distinct OG images 200. | 2026-09-01 re-verified live: og:image resolves 200 on all 17 articles and every one matches the JSON-LD image URL exactly, cache-bust included. | 2026-09-06 re-verified live: og:title / og:description / og:image present on all 5 chrome pages and all 17 articles; og:image matches the JSON-LD image byte-for-byte on 17/17. | 2026-09-11 re-verified live: og:title/og:description/og:image present on all 22 HTML routes; every og:image resolves 200. | 2026-09-28: live: og + twitter complete on 21 routes; all OG images 200. (/phase0/ omits the optional og:image:width/height hints — not flagged.) | 2026-09-29: live: og + twitter complete on all 21; og-phase0 and og-brand measured 1200x630 (both pages omit the optional og:image:width/height/alt hints — not flagged, expectation is the image size).</t>
+          <t>PASS — og+twitter complete on all 21; all 19 OG images 200 (16 essays + home/about/phase0/brand) | 2026-08-15 re-verified live: twitter:card summary_large_image on every page in scope (404 correctly excluded) | 2026-08-25 re-verified live: og:title / og:description / og:image present on all 20; all 16 og-&lt;slug&gt;.png 200; og:image byte-identical to the JSON-LD image on all 16. | 2026-08-27 re-verified live: og+twitter complete across 21 routes; all 21 distinct OG images 200. | 2026-09-01 re-verified live: og:image resolves 200 on all 17 articles and every one matches the JSON-LD image URL exactly, cache-bust included. | 2026-09-06 re-verified live: og:title / og:description / og:image present on all 5 chrome pages and all 17 articles; og:image matches the JSON-LD image byte-for-byte on 17/17. | 2026-09-11 re-verified live: og:title/og:description/og:image present on all 22 HTML routes; every og:image resolves 200. | 2026-09-28: live: og + twitter complete on 21 routes; all OG images 200. (/phase0/ omits the optional og:image:width/height hints — not flagged.) | 2026-09-29: live: og + twitter complete on all 21; og-phase0 and og-brand measured 1200x630 (both pages omit the optional og:image:width/height/alt hints — not flagged, expectation is the image size). | 2026-10-05: live: og:title/description/image + twitter summary_large_image on all in-scope routes; all OG images 200 (phase0/brand still omit the optional width/height hints, not flagged).</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr"/>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>PASS — WebSite + Person @graph complete (name/url/sameAs/jobTitle/worksFor) | 2026-08-15 re-verified live: home @graph carries WebSite + Person; Person has name/url/sameAs/jobTitle/worksFor — no missing fields | 2026-08-25 re-verified live: WebSite + Person @graph complete on /; Person carries name, url, sameAs, jobTitle, worksFor. | 2026-08-27 re-verified live: WebSite + Person @graph complete (name/url/sameAs/jobTitle/worksFor). | 2026-09-01 re-verified live: homepage @graph carries WebSite + Person; Person has name, url, sameAs, jobTitle, worksFor — zero required fields missing. | 2026-09-06 re-verified live: homepage @graph carries WebSite + Person; Person complete on name/url/sameAs/jobTitle/worksFor. | 2026-09-11 re-verified live: homepage @graph carries WebSite + Person; Person has name, url, sameAs, jobTitle, worksFor. | 2026-09-28: live: WebSite + Person @graph; Person has name/url/sameAs/jobTitle/worksFor. | 2026-09-29: live: WebSite + Person @graph; Person has name/url/sameAs/jobTitle/worksFor.</t>
+          <t>PASS — WebSite + Person @graph complete (name/url/sameAs/jobTitle/worksFor) | 2026-08-15 re-verified live: home @graph carries WebSite + Person; Person has name/url/sameAs/jobTitle/worksFor — no missing fields | 2026-08-25 re-verified live: WebSite + Person @graph complete on /; Person carries name, url, sameAs, jobTitle, worksFor. | 2026-08-27 re-verified live: WebSite + Person @graph complete (name/url/sameAs/jobTitle/worksFor). | 2026-09-01 re-verified live: homepage @graph carries WebSite + Person; Person has name, url, sameAs, jobTitle, worksFor — zero required fields missing. | 2026-09-06 re-verified live: homepage @graph carries WebSite + Person; Person complete on name/url/sameAs/jobTitle/worksFor. | 2026-09-11 re-verified live: homepage @graph carries WebSite + Person; Person has name, url, sameAs, jobTitle, worksFor. | 2026-09-28: live: WebSite + Person @graph; Person has name/url/sameAs/jobTitle/worksFor. | 2026-09-29: live: WebSite + Person @graph; Person has name/url/sameAs/jobTitle/worksFor. | 2026-10-05: live: home @graph WebSite + Person with name/url/sameAs/jobTitle/worksFor.</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr"/>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>PASS — ProfilePage mainEntity Person complete (name/url/jobTitle/worksFor/sameAs/description) | 2026-08-15 re-verified live: about ProfilePage mainEntity Person complete — name/url/jobTitle/worksFor/sameAs/description all present | 2026-08-25 re-verified live: ProfilePage on /about/ with mainEntity @type Person carrying name, url, jobTitle, worksFor, sameAs, description. | 2026-08-27 re-verified live: ProfilePage mainEntity Person complete (name/url/jobTitle/worksFor/sameAs/description). | 2026-09-01 re-verified live: /about/ ProfilePage mainEntity is @type Person with name, url, jobTitle, worksFor, sameAs, description — zero missing. | 2026-09-06 re-verified live: /about/ ProfilePage present, mainEntity @type=Person complete on name/url/jobTitle/worksFor/sameAs/description. | 2026-09-11 re-verified live: /about/ ProfilePage mainEntity is a Person with all six required fields present. | 2026-09-28: live: ProfilePage mainEntity Person with name/url/jobTitle/worksFor/sameAs/description. | 2026-09-29: live: ProfilePage mainEntity Person with name/url/jobTitle/worksFor/sameAs/description.</t>
+          <t>PASS — ProfilePage mainEntity Person complete (name/url/jobTitle/worksFor/sameAs/description) | 2026-08-15 re-verified live: about ProfilePage mainEntity Person complete — name/url/jobTitle/worksFor/sameAs/description all present | 2026-08-25 re-verified live: ProfilePage on /about/ with mainEntity @type Person carrying name, url, jobTitle, worksFor, sameAs, description. | 2026-08-27 re-verified live: ProfilePage mainEntity Person complete (name/url/jobTitle/worksFor/sameAs/description). | 2026-09-01 re-verified live: /about/ ProfilePage mainEntity is @type Person with name, url, jobTitle, worksFor, sameAs, description — zero missing. | 2026-09-06 re-verified live: /about/ ProfilePage present, mainEntity @type=Person complete on name/url/jobTitle/worksFor/sameAs/description. | 2026-09-11 re-verified live: /about/ ProfilePage mainEntity is a Person with all six required fields present. | 2026-09-28: live: ProfilePage mainEntity Person with name/url/jobTitle/worksFor/sameAs/description. | 2026-09-29: live: ProfilePage mainEntity Person with name/url/jobTitle/worksFor/sameAs/description. | 2026-10-05: live: ProfilePage.mainEntity Person carries name/url/jobTitle/worksFor/sameAs/description.</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr"/>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>PASS — BlogPosting complete on all 16 (headline, description, datePublished, dateModified, author Person, publisher Organization+logo, mainEntityOfPage, image, url, inLanguage, wordCount); image == og:image exactly, no og-default drift | 2026-08-13 re-verified live: all 16 BlogPosting blocks carry every required field (headline, description, datePublished, dateModified, author.@type=Person + name, publisher, mainEntityOfPage, image, url, inLanguage, wordCount); zero og-default.png drift. | 2026-08-16 re-verified live: all 16 BlogPosting blocks re-verified live: every required field present (headline, description, datePublished, dateModified, author.@type=Person, publisher, mainEntityOfPage, image, url, inLanguage, wordCount) and JSON-LD image === og:image exactly, cache-bust included, on all 16. Zero og-default.png drift. | 2026-08-25 re-verified live: BlogPosting on all 16 articles; every required field present (headline, description, datePublished, dateModified, author.Person.name, publisher, mainEntityOfPage, image, url, inLanguage, wordCount). Zero og-default.png regressions. | 2026-08-27 re-verified live: BlogPosting complete on all 16 — all 11 required fields, author.@type=Person, og:image == JSON-LD image, image == og-&lt;slug&gt;.png on every one. | 2026-09-01 re-verified live: all 17 BlogPosting blocks carry every required field (headline, description, datePublished, dateModified, author.@type=Person + name, publisher, mainEntityOfPage, image, url, inLanguage, wordCount). Zero on og-default.png. | 2026-09-06 re-verified live: 17/17 BlogPosting blocks complete on all 11 required fields, author @type=Person with name, image per-slug. | 2026-09-11 re-verified live: all 17 BlogPosting blocks carry the full 11-field set; author is Person with a name. | 2026-09-28: live: BlogPosting complete 17/17 (all 12 required fields, author @type Person). | 2026-09-29: live: BlogPosting complete 17/17 (12 required fields, author @type Person); LD image == og:image 17/17.</t>
+          <t>PASS — BlogPosting complete on all 16 (headline, description, datePublished, dateModified, author Person, publisher Organization+logo, mainEntityOfPage, image, url, inLanguage, wordCount); image == og:image exactly, no og-default drift | 2026-08-13 re-verified live: all 16 BlogPosting blocks carry every required field (headline, description, datePublished, dateModified, author.@type=Person + name, publisher, mainEntityOfPage, image, url, inLanguage, wordCount); zero og-default.png drift. | 2026-08-16 re-verified live: all 16 BlogPosting blocks re-verified live: every required field present (headline, description, datePublished, dateModified, author.@type=Person, publisher, mainEntityOfPage, image, url, inLanguage, wordCount) and JSON-LD image === og:image exactly, cache-bust included, on all 16. Zero og-default.png drift. | 2026-08-25 re-verified live: BlogPosting on all 16 articles; every required field present (headline, description, datePublished, dateModified, author.Person.name, publisher, mainEntityOfPage, image, url, inLanguage, wordCount). Zero og-default.png regressions. | 2026-08-27 re-verified live: BlogPosting complete on all 16 — all 11 required fields, author.@type=Person, og:image == JSON-LD image, image == og-&lt;slug&gt;.png on every one. | 2026-09-01 re-verified live: all 17 BlogPosting blocks carry every required field (headline, description, datePublished, dateModified, author.@type=Person + name, publisher, mainEntityOfPage, image, url, inLanguage, wordCount). Zero on og-default.png. | 2026-09-06 re-verified live: 17/17 BlogPosting blocks complete on all 11 required fields, author @type=Person with name, image per-slug. | 2026-09-11 re-verified live: all 17 BlogPosting blocks carry the full 11-field set; author is Person with a name. | 2026-09-28: live: BlogPosting complete 17/17 (all 12 required fields, author @type Person). | 2026-09-29: live: BlogPosting complete 17/17 (12 required fields, author @type Person); LD image == og:image 17/17. | 2026-10-05: live: BlogPosting complete on 17/17 (all 12 required fields + author Person).</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr"/>
@@ -1409,7 +1409,7 @@
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>PASS — phase0 WebPage JSON-LD present and parses | 2026-08-27 re-verified live: phase0 WebPage + Person JSON-LD present and parse. | 2026-09-11 re-verified live: /phase0/ @graph = WebPage(#webpage) isPartOf #website, author #person. Valid JSON-LD. | 2026-09-28: live: WebPage isPartOf #website, author #person. | 2026-09-29: live: WebPage 'Phase 0 — Ministry Marketing OS', url /phase0/, isPartOf #website, author #person.</t>
+          <t>PASS — phase0 WebPage JSON-LD present and parses | 2026-08-27 re-verified live: phase0 WebPage + Person JSON-LD present and parse. | 2026-09-11 re-verified live: /phase0/ @graph = WebPage(#webpage) isPartOf #website, author #person. Valid JSON-LD. | 2026-09-28: live: WebPage isPartOf #website, author #person. | 2026-09-29: live: WebPage 'Phase 0 — Ministry Marketing OS', url /phase0/, isPartOf #website, author #person. | 2026-10-05: live: /phase0/ @graph WebPage present.</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr"/>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>PASS — robots.txt Allow / + Sitemap → sitemap-index.xml | 2026-08-13 re-verified live: /robots.txt 200, Sitemap directive -&gt; https://imjustdex.com/sitemap-index.xml. | 2026-08-25 re-verified live: robots.txt = "User-agent: *\nAllow: /\n\nSitemap: https://imjustdex.com/sitemap-index.xml". /DESIGN-SYSTEM.md correctly 404s. | 2026-08-27 re-verified live: robots.txt Allow / + Sitemap → sitemap-index.xml. | 2026-09-01 re-verified live: robots.txt is 'User-agent: * / Allow: / / Sitemap: https://imjustdex.com/sitemap-index.xml'. /DESIGN-SYSTEM.md still 404s (the only thing keeping the doc unexposed). | 2026-09-06 re-verified live: robots.txt is 'User-agent: * / Allow: / / Sitemap: https://imjustdex.com/sitemap-index.xml'. | 2026-09-11 re-verified live: robots.txt = 'User-agent: * / Allow: / / Sitemap: https://imjustdex.com/sitemap-index.xml'. | 2026-09-28: live: Allow / + Sitemap -&gt; sitemap-index.xml. | 2026-09-30: live: robots.txt 200 = 'User-agent: * / Allow: /' + Sitemap -&gt; https://imjustdex.com/sitemap-index.xml.</t>
+          <t>PASS — robots.txt Allow / + Sitemap → sitemap-index.xml | 2026-08-13 re-verified live: /robots.txt 200, Sitemap directive -&gt; https://imjustdex.com/sitemap-index.xml. | 2026-08-25 re-verified live: robots.txt = "User-agent: *\nAllow: /\n\nSitemap: https://imjustdex.com/sitemap-index.xml". /DESIGN-SYSTEM.md correctly 404s. | 2026-08-27 re-verified live: robots.txt Allow / + Sitemap → sitemap-index.xml. | 2026-09-01 re-verified live: robots.txt is 'User-agent: * / Allow: / / Sitemap: https://imjustdex.com/sitemap-index.xml'. /DESIGN-SYSTEM.md still 404s (the only thing keeping the doc unexposed). | 2026-09-06 re-verified live: robots.txt is 'User-agent: * / Allow: / / Sitemap: https://imjustdex.com/sitemap-index.xml'. | 2026-09-11 re-verified live: robots.txt = 'User-agent: * / Allow: / / Sitemap: https://imjustdex.com/sitemap-index.xml'. | 2026-09-28: live: Allow / + Sitemap -&gt; sitemap-index.xml. | 2026-09-30: live: robots.txt 200 = 'User-agent: * / Allow: /' + Sitemap -&gt; https://imjustdex.com/sitemap-index.xml. | 2026-10-05: live: robots.txt Allow: / + Sitemap sitemap-index.xml.</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr"/>
@@ -1507,7 +1507,7 @@
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>PASS — sitemap-0.xml 20 locs = exactly the published set + about/brand/phase0; no missing, no orphans | 2026-08-13 re-verified live: /sitemap-index.xml -&gt; sitemap-0.xml; sitemap-0 lists 20 URLs covering all 16 articles + /, /about/, /brand/, /phase0/. Zero missing. | 2026-08-25 re-verified live: sitemap-index.xml references sitemap-0.xml; sitemap-0.xml carries exactly 20 locs = 16 articles + /, /about/, /brand/, /phase0/. The drafted essay is correctly absent. | 2026-08-27 re-verified live: sitemap-0.xml 20 locs; every homepage-linked route plus /about/ /brand/ /phase0/ present. | 2026-09-01 re-verified live: /sitemap-index.xml points to sitemap-0.xml; sitemap-0.xml holds exactly 21 URLs — the 17 live articles plus /, /about/, /brand/, /phase0/. Zero missing, zero extra. The drafted entry before-i-had-the-words is correctly absent. | 2026-09-06 re-verified live: sitemap-index.xml points at sitemap-0.xml; sitemap-0.xml carries 21 URLs and includes all 17 articles plus /, /about/, /brand/, /phase0/. | 2026-09-11 re-verified live: sitemap-index → sitemap-0; 21 locs = 17 articles + /, /about/, /brand/, /phase0/. No drafts leaked (before-i-had-the-words absent). | 2026-09-28: live: sitemap-0.xml 21 locs = 17 essays + home/about/brand/phase0; throwaway fixture build: a future-dated entry is excluded. | 2026-09-30: live: sitemap-index -&gt; sitemap-0; 21 locs = 17 published articles + / /about/ /brand/ /phase0/, no orphans; priorities home 1.0 / about 0.7 / phase0 0.9 / brand 0.5 / articles 0.8; unmatched route not listed.</t>
+          <t>PASS — sitemap-0.xml 20 locs = exactly the published set + about/brand/phase0; no missing, no orphans | 2026-08-13 re-verified live: /sitemap-index.xml -&gt; sitemap-0.xml; sitemap-0 lists 20 URLs covering all 16 articles + /, /about/, /brand/, /phase0/. Zero missing. | 2026-08-25 re-verified live: sitemap-index.xml references sitemap-0.xml; sitemap-0.xml carries exactly 20 locs = 16 articles + /, /about/, /brand/, /phase0/. The drafted essay is correctly absent. | 2026-08-27 re-verified live: sitemap-0.xml 20 locs; every homepage-linked route plus /about/ /brand/ /phase0/ present. | 2026-09-01 re-verified live: /sitemap-index.xml points to sitemap-0.xml; sitemap-0.xml holds exactly 21 URLs — the 17 live articles plus /, /about/, /brand/, /phase0/. Zero missing, zero extra. The drafted entry before-i-had-the-words is correctly absent. | 2026-09-06 re-verified live: sitemap-index.xml points at sitemap-0.xml; sitemap-0.xml carries 21 URLs and includes all 17 articles plus /, /about/, /brand/, /phase0/. | 2026-09-11 re-verified live: sitemap-index → sitemap-0; 21 locs = 17 articles + /, /about/, /brand/, /phase0/. No drafts leaked (before-i-had-the-words absent). | 2026-09-28: live: sitemap-0.xml 21 locs = 17 essays + home/about/brand/phase0; throwaway fixture build: a future-dated entry is excluded. | 2026-09-30: live: sitemap-index -&gt; sitemap-0; 21 locs = 17 published articles + / /about/ /brand/ /phase0/, no orphans; priorities home 1.0 / about 0.7 / phase0 0.9 / brand 0.5 / articles 0.8; unmatched route not listed. | 2026-10-05: live: sitemap-index -&gt; sitemap-0, 21 locs incl. every cascade essay + /about/ /brand/ /phase0/, no 404; fixture build: a future-dated entry is excluded.</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr"/>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>404 half PASS (noindex,nofollow live). Coming-soon half PENDING — no upcoming entry exists to render one | 2026-08-25: 404 half re-verified live (meta robots noindex,nofollow present, bespoke body served at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one. | 2026-09-01 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one. | 2026-09-11: 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body at HTTP 200). Coming-soon half still PENDING — 17 published entries, all past-dated, so isUpcomingData() is false everywhere and no ComingSoonLayout renders. | 2026-09-19: 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body, HTTP 404 on unmatched route). Coming-soon half still PENDING — 17 published entries, all past-dated; the untracked before-i-had-the-words.mdx in Dexter's working tree is still status 'drafted'. | 2026-09-23: 404 half re-verified live (noindex, nofollow). Coming-soon half still PENDING — 17/17 entries status published, no upcoming entry to render. | 2026-09-25: still PENDING — 17/17 entries status published and past-dated, no upcoming entry to render. 404 half re-verified live: meta robots noindex present, bespoke body, unmatched route 404. | 2026-09-28: 404 half re-verified live (noindex, nofollow). Coming-soon half BUILD-VERIFIED via a throwaway future-dated fixture in a scratch copy (never committed): ComingSoonLayout emits &lt;meta name=robots content=noindex&gt;. | 2026-09-30: live: 404 half re-verified live (bespoke body, noindex). Coming-soon half unchanged since the 09-28 fixture build — 17/17 entries still published and past-dated, no upcoming entry to render live.</t>
+          <t>404 half PASS (noindex,nofollow live). Coming-soon half PENDING — no upcoming entry exists to render one | 2026-08-25: 404 half re-verified live (meta robots noindex,nofollow present, bespoke body served at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one. | 2026-09-01 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one. | 2026-09-11: 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body at HTTP 200). Coming-soon half still PENDING — 17 published entries, all past-dated, so isUpcomingData() is false everywhere and no ComingSoonLayout renders. | 2026-09-19: 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body, HTTP 404 on unmatched route). Coming-soon half still PENDING — 17 published entries, all past-dated; the untracked before-i-had-the-words.mdx in Dexter's working tree is still status 'drafted'. | 2026-09-23: 404 half re-verified live (noindex, nofollow). Coming-soon half still PENDING — 17/17 entries status published, no upcoming entry to render. | 2026-09-25: still PENDING — 17/17 entries status published and past-dated, no upcoming entry to render. 404 half re-verified live: meta robots noindex present, bespoke body, unmatched route 404. | 2026-09-28: 404 half re-verified live (noindex, nofollow). Coming-soon half BUILD-VERIFIED via a throwaway future-dated fixture in a scratch copy (never committed): ComingSoonLayout emits &lt;meta name=robots content=noindex&gt;. | 2026-09-30: live: 404 half re-verified live (bespoke body, noindex). Coming-soon half unchanged since the 09-28 fixture build — 17/17 entries still published and past-dated, no upcoming entry to render live. | 2026-10-05: PASS: live /404 noindex,nofollow; fixture build (scratch copy, never committed): ComingSoonLayout emits robots noindex.</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr"/>
@@ -1609,7 +1609,7 @@
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>PASS — Entry No. 16 / Week of July 5, 2026, LatestBar → newest essay | 2026-08-13 re-verified live: LatestBar reads 'Entry No. 16 / Week of July 5, 2026' and links to /words/send-someone-else/ (the newest). NOTE: its .latest-tag chip is the F77 finding this run. | 2026-08-25 re-verified live: issue head renders "Entry No. 16" / "Week of July 5, 2026" from the lead; standfirst links /words/send-someone-else/. | 2026-08-27 re-verified live: issue head 'Entry No. 16 / Week of July 5, 2026', LatestBar → send-someone-else. | 2026-09-11 re-verified live: LatestBar: 'Entry No. 17' (= 17 published essays), 'Week of August 31, 2026', latest link → /words/the-weight-of-my-no/. | 2026-09-28: live: 'Entry No. 17', 'Week of August 31, 2026', Latest -&gt; the-weight-of-my-no, 'Faith · Aug 31 · 8 min'. | 2026-09-30: live: LatestBar reads 'Entry No. 17' / 'Week of August 31, 2026'; .issue-latest links to /words/the-weight-of-my-no/ (newest).</t>
+          <t>PASS — Entry No. 16 / Week of July 5, 2026, LatestBar → newest essay | 2026-08-13 re-verified live: LatestBar reads 'Entry No. 16 / Week of July 5, 2026' and links to /words/send-someone-else/ (the newest). NOTE: its .latest-tag chip is the F77 finding this run. | 2026-08-25 re-verified live: issue head renders "Entry No. 16" / "Week of July 5, 2026" from the lead; standfirst links /words/send-someone-else/. | 2026-08-27 re-verified live: issue head 'Entry No. 16 / Week of July 5, 2026', LatestBar → send-someone-else. | 2026-09-11 re-verified live: LatestBar: 'Entry No. 17' (= 17 published essays), 'Week of August 31, 2026', latest link → /words/the-weight-of-my-no/. | 2026-09-28: live: 'Entry No. 17', 'Week of August 31, 2026', Latest -&gt; the-weight-of-my-no, 'Faith · Aug 31 · 8 min'. | 2026-09-30: live: LatestBar reads 'Entry No. 17' / 'Week of August 31, 2026'; .issue-latest links to /words/the-weight-of-my-no/ (newest). | 2026-10-05: live: "Entry No. 17", "Week of August 31, 2026", Latest -&gt; The Weight of My No · Faith · Aug 31 · 8 min.</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr"/>
@@ -1662,7 +1662,7 @@
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>PASS — IdentityHero renders; hero copy contrast 5.17:1 (AA large) | 2026-08-27 re-verified live: IdentityHero renders (screenshot-confirmed in both modes). | 2026-09-11 re-verified live: IdentityHero: name + 'ImJustDex' render; hero links → /about/ and #subscribe-manifesto. | 2026-09-28: live: hero name/sub/tagline/bio, 'Read the About' -&gt; /about/, 'Subscribe' -&gt; #subscribe-manifesto. | 2026-09-30: live: IdentityHero renders 'Dexter Jakes' + 'ImJustDex' + tagline + bio; links -&gt; /about/ and #subscribe-manifesto.</t>
+          <t>PASS — IdentityHero renders; hero copy contrast 5.17:1 (AA large) | 2026-08-27 re-verified live: IdentityHero renders (screenshot-confirmed in both modes). | 2026-09-11 re-verified live: IdentityHero: name + 'ImJustDex' render; hero links → /about/ and #subscribe-manifesto. | 2026-09-28: live: hero name/sub/tagline/bio, 'Read the About' -&gt; /about/, 'Subscribe' -&gt; #subscribe-manifesto. | 2026-09-30: live: IdentityHero renders 'Dexter Jakes' + 'ImJustDex' + tagline + bio; links -&gt; /about/ and #subscribe-manifesto. | 2026-10-05: live: identity hero name, ImJustDex, tagline, bio, Read the About + Subscribe present.</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr"/>
@@ -1711,7 +1711,7 @@
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>PASS — Faith 13 / Identity 09 / Art 03, verified against frontmatter lanes; 16 articles | 2026-08-13 re-verified live: lane-index counts Faith 13 / Identity 09 / Art 03 — non-negative, zero-padded, and consistent with 16 essays counted per lane (15 .plate-lane chips + 1 .lead-badge-lane). | 2026-08-25 re-verified live: lane counts render Faith 13 / Identity 09 / Art 03 — matches the frontmatter tally across the 16 tracked essays exactly (multi-lane counted per lane). | 2026-08-27 re-verified live: lane counts Faith 13 / Identity 09 / Art 03. | 2026-09-01 re-verified live: lane-index reads Faith 14 / Identity 10 / Art 03 — non-negative integers summing to 27 across 17 essays (multi-lane counted per lane). Cross-checked against the filter: selecting Faith reveals exactly 14 articles. | 2026-09-06 re-verified live: lane index reads Faith 14 / Identity 10 / Art 03 (sum 27 across 17 essays, multi-lane counted per lane). | 2026-09-11 re-verified live: lane counts Faith 14 / Identity 10 / Art 03; sum 27 over 17 articles (multi-lane essays count per lane), all non-negative integers. | 2026-09-28: live: Faith 14 / Identity 10 / Art 03 essays (no zero lane, so the queued state is not exercised). | 2026-09-30: live: lane index Faith 14 / Identity 10 / Art 03 essays (zero-padded), consistent with 17 essays counted per lane; no lane at 0, so no .lane-cell-queued rendered.</t>
+          <t>PASS — Faith 13 / Identity 09 / Art 03, verified against frontmatter lanes; 16 articles | 2026-08-13 re-verified live: lane-index counts Faith 13 / Identity 09 / Art 03 — non-negative, zero-padded, and consistent with 16 essays counted per lane (15 .plate-lane chips + 1 .lead-badge-lane). | 2026-08-25 re-verified live: lane counts render Faith 13 / Identity 09 / Art 03 — matches the frontmatter tally across the 16 tracked essays exactly (multi-lane counted per lane). | 2026-08-27 re-verified live: lane counts Faith 13 / Identity 09 / Art 03. | 2026-09-01 re-verified live: lane-index reads Faith 14 / Identity 10 / Art 03 — non-negative integers summing to 27 across 17 essays (multi-lane counted per lane). Cross-checked against the filter: selecting Faith reveals exactly 14 articles. | 2026-09-06 re-verified live: lane index reads Faith 14 / Identity 10 / Art 03 (sum 27 across 17 essays, multi-lane counted per lane). | 2026-09-11 re-verified live: lane counts Faith 14 / Identity 10 / Art 03; sum 27 over 17 articles (multi-lane essays count per lane), all non-negative integers. | 2026-09-28: live: Faith 14 / Identity 10 / Art 03 essays (no zero lane, so the queued state is not exercised). | 2026-09-30: live: lane index Faith 14 / Identity 10 / Art 03 essays (zero-padded), consistent with 17 essays counted per lane; no lane at 0, so no .lane-cell-queued rendered. | 2026-10-05: live: lanes Faith 14 / Identity 10 / Art 03 (all &gt;0, so no queued cell rendered).</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr"/>
@@ -1764,7 +1764,7 @@
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: Faith 13/13, Identity 9/9, Art 3/3 with zero non-matching plates in any filtered view; while filtered the .earlier-more-wrap computes display:none, 0 client rects, offsetHeight 0 (unreachable by mouse or keyboard). The ab07b15 fix holds in production. | 2026-08-16 re-verified live: all three lanes re-verified live: Faith 13, Identity 9, Art 3 — exactly matching the lane-index counts. Verified against the real filter key (data-lane, space-separated) rather than the visible chips: all 9 identity plates carry 'identity' in data-lane. While filtered, .earlier-more-wrap computes display:none with 0 client rects; clearing restores display:flex. | 2026-08-27 re-verified live: real pointer clicks: Faith 13, Identity 9, Art 3, re-click clears to the default 8; aria-pressed single-select correct. | 2026-09-01 re-verified live: .lane-cell[data-lane=faith] click sets aria-pressed=true and reveals exactly 14 articles; clicking again returns aria-pressed=false and the default 7-article view. | 2026-09-06 re-verified live: clicking the Art lane cell filtered the cascade 7 -&gt; 3 visible articles (Music That Raised Me, Useful Is Not the Same, Groan Beneath the Song), aria-pressed=true, and a second click restored 7. | 2026-09-11 re-verified live: lane filter 'art' → 3 visible articles, matching its announced count; aria-pressed true→false; clearing restores 7. | 2026-09-28: live: Faith -&gt; aria-pressed true, 14 visible, all data-lane faith; re-click clears (7 visible); Art -&gt; 3. | 2026-09-30: live: lane-filter.js exercised in-browser: Faith 14/14, Identity 10/10, Art 3/3 visible with 0 non-matching; aria-pressed true, .plates data-filter set, live region 'Filtered to &lt;lane&gt;. N essays.', .earlier-more-wrap display:none while filtered; second click clears (aria-pressed false, 10 hidden restored, data-filter removed).</t>
+          <t>PASS — live-verified 2026-08-10: Faith 13/13, Identity 9/9, Art 3/3 with zero non-matching plates in any filtered view; while filtered the .earlier-more-wrap computes display:none, 0 client rects, offsetHeight 0 (unreachable by mouse or keyboard). The ab07b15 fix holds in production. | 2026-08-16 re-verified live: all three lanes re-verified live: Faith 13, Identity 9, Art 3 — exactly matching the lane-index counts. Verified against the real filter key (data-lane, space-separated) rather than the visible chips: all 9 identity plates carry 'identity' in data-lane. While filtered, .earlier-more-wrap computes display:none with 0 client rects; clearing restores display:flex. | 2026-08-27 re-verified live: real pointer clicks: Faith 13, Identity 9, Art 3, re-click clears to the default 8; aria-pressed single-select correct. | 2026-09-01 re-verified live: .lane-cell[data-lane=faith] click sets aria-pressed=true and reveals exactly 14 articles; clicking again returns aria-pressed=false and the default 7-article view. | 2026-09-06 re-verified live: clicking the Art lane cell filtered the cascade 7 -&gt; 3 visible articles (Music That Raised Me, Useful Is Not the Same, Groan Beneath the Song), aria-pressed=true, and a second click restored 7. | 2026-09-11 re-verified live: lane filter 'art' → 3 visible articles, matching its announced count; aria-pressed true→false; clearing restores 7. | 2026-09-28: live: Faith -&gt; aria-pressed true, 14 visible, all data-lane faith; re-click clears (7 visible); Art -&gt; 3. | 2026-09-30: live: lane-filter.js exercised in-browser: Faith 14/14, Identity 10/10, Art 3/3 visible with 0 non-matching; aria-pressed true, .plates data-filter set, live region 'Filtered to &lt;lane&gt;. N essays.', .earlier-more-wrap display:none while filtered; second click clears (aria-pressed false, 10 hidden restored, data-filter removed). | 2026-10-05: live: Identity -&gt; aria-pressed true, 10 visible, data-filter=identity, row heads suppressed, live region "Filtered to identity. 10 essays."; re-click clears ("Filter cleared"); Art -&gt; 3.</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr"/>
@@ -1817,7 +1817,7 @@
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>PASS — lead plate = send-someone-else (newest published) | 2026-08-25 re-verified live: lead plate renders send-someone-else with correct eyebrow, deck and 16 min read. | 2026-08-27 re-verified live: lead plate = send-someone-else. | 2026-09-11 re-verified live: LeadPlate renders the newest essay with Latest badge and Read CTA, href /words/the-weight-of-my-no/. | 2026-09-28: live: lead = the-weight-of-my-no with Latest badge, Faith, &lt;time 2026-08-31&gt;, 8 min, Read -&gt;. | 2026-09-30: live: lead plate = .plate-lead for the-weight-of-my-no (newest): Latest badge, Faith, Aug 31, 8 min read, title, deck, Read -&gt; CTA.</t>
+          <t>PASS — lead plate = send-someone-else (newest published) | 2026-08-25 re-verified live: lead plate renders send-someone-else with correct eyebrow, deck and 16 min read. | 2026-08-27 re-verified live: lead plate = send-someone-else. | 2026-09-11 re-verified live: LeadPlate renders the newest essay with Latest badge and Read CTA, href /words/the-weight-of-my-no/. | 2026-09-28: live: lead = the-weight-of-my-no with Latest badge, Faith, &lt;time 2026-08-31&gt;, 8 min, Read -&gt;. | 2026-09-30: live: lead plate = .plate-lead for the-weight-of-my-no (newest): Latest badge, Faith, Aug 31, 8 min read, title, deck, Read -&gt; CTA. | 2026-10-05: live: lead plate = the-weight-of-my-no with Latest badge, lane, date, read time, Read -&gt;.</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr"/>
@@ -1866,7 +1866,7 @@
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>PASS — 'This Month' = show-me-your-glory (same month as lead) | 2026-08-27 re-verified live: row heads 'This Week' (01, lead) and 'This Month' (02) both render as authored. | 2026-09-18 re-verified live: 'This Month' correctly hidden — no other essay shares the lead's month (Aug 2026); row heads read 01 This Week / 02 Earlier. | 2026-09-28: live: correctly hidden — no other essay shares the lead's month (Aug 2026); row heads read 'Latest', 'Earlier'. | 2026-09-30: live: 'This Month' correctly hidden — no other essay shares the lead's month (Aug 2026); row heads '01 Latest', '02 Earlier'.</t>
+          <t>PASS — 'This Month' = show-me-your-glory (same month as lead) | 2026-08-27 re-verified live: row heads 'This Week' (01, lead) and 'This Month' (02) both render as authored. | 2026-09-18 re-verified live: 'This Month' correctly hidden — no other essay shares the lead's month (Aug 2026); row heads read 01 This Week / 02 Earlier. | 2026-09-28: live: correctly hidden — no other essay shares the lead's month (Aug 2026); row heads read 'Latest', 'Earlier'. | 2026-09-30: live: 'This Month' correctly hidden — no other essay shares the lead's month (Aug 2026); row heads '01 Latest', '02 Earlier'. | 2026-10-05: live: no This Month section (lead is the only August essay) — hidden as specified.</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr"/>
@@ -1915,7 +1915,7 @@
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>PASS — 'Earlier' = 14, 6 visible + 8 overflow | 2026-08-27 re-verified live: 8 of 16 plates visible by default, 8 under the overflow. | 2026-09-18 re-verified live: 'Earlier' = 16, 6 visible + 10 under the overflow; 7 of 17 plates visible by default. | 2026-09-28: live: 'Earlier' numbered 02 (no This Month), 16 essays: 6 visible + 10 in .earlier-more. | 2026-09-30: live: 'Earlier' = 16 under RowHead 02 (no This Month); 6 visible + 10 under .earlier-more[hidden]; 7 of 17 plates visible by default.</t>
+          <t>PASS — 'Earlier' = 14, 6 visible + 8 overflow | 2026-08-27 re-verified live: 8 of 16 plates visible by default, 8 under the overflow. | 2026-09-18 re-verified live: 'Earlier' = 16, 6 visible + 10 under the overflow; 7 of 17 plates visible by default. | 2026-09-28: live: 'Earlier' numbered 02 (no This Month), 16 essays: 6 visible + 10 in .earlier-more. | 2026-09-30: live: 'Earlier' = 16 under RowHead 02 (no This Month); 6 visible + 10 under .earlier-more[hidden]; 7 of 17 plates visible by default. | 2026-10-05: live: "02 Earlier" with 6 visible + 10 in .earlier-more[hidden].</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr"/>
@@ -1968,7 +1968,7 @@
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: expand 8→16, collapse 16→8, aria-expanded false↔true and the button label track; collapse state survives a full filter cycle (clear restores the wrap to display:flex). | 2026-08-16 re-verified live: expand 8-&gt;16 and collapse 16-&gt;8 re-verified live; aria-expanded false&lt;-&gt;true and the label tracked ('View Earlier Essays — 8 more' &lt;-&gt; 'Show Less — showing all'); collapse state survived a full filter cycle. | 2026-08-27 re-verified live: real pointer clicks: 8→16→8, aria-expanded false↔true, label and count track. | 2026-09-01 re-verified live: toggle expands 10 hidden articles to 0 hidden, label 'View Earlier Essays — 10 more' -&gt; 'Show Less — showing all', aria-expanded false-&gt;true; collapse restores all three. | 2026-09-06 re-verified live: View Earlier 7 -&gt; 17 -&gt; 7 with label 'View Earlier Essays - 10 more' &lt;-&gt; 'Show Less - showing all' and aria-expanded true/false. | 2026-09-11 re-verified live: toggle 7↔17 articles, label 'View Earlier Essays — 10 more ↓' ↔ 'Show Less — showing all ↑', aria-expanded false↔true. | 2026-09-28: live: 'View Earlier Essays — 10 more ↓' -&gt; 'Show Less — showing all ↑', aria-expanded false-&gt;true-&gt;false, 7-&gt;17-&gt;7 visible. | 2026-10-01 re-verified live: 'View Earlier Essays — 10 more ↓', aria-expanded=false, 10 .earlier-more hidden; click -&gt; 'Show Less — showing all ↑', expanded=true, 0 hidden; re-click restores all three.</t>
+          <t>PASS — live-verified 2026-08-10: expand 8→16, collapse 16→8, aria-expanded false↔true and the button label track; collapse state survives a full filter cycle (clear restores the wrap to display:flex). | 2026-08-16 re-verified live: expand 8-&gt;16 and collapse 16-&gt;8 re-verified live; aria-expanded false&lt;-&gt;true and the label tracked ('View Earlier Essays — 8 more' &lt;-&gt; 'Show Less — showing all'); collapse state survived a full filter cycle. | 2026-08-27 re-verified live: real pointer clicks: 8→16→8, aria-expanded false↔true, label and count track. | 2026-09-01 re-verified live: toggle expands 10 hidden articles to 0 hidden, label 'View Earlier Essays — 10 more' -&gt; 'Show Less — showing all', aria-expanded false-&gt;true; collapse restores all three. | 2026-09-06 re-verified live: View Earlier 7 -&gt; 17 -&gt; 7 with label 'View Earlier Essays - 10 more' &lt;-&gt; 'Show Less - showing all' and aria-expanded true/false. | 2026-09-11 re-verified live: toggle 7↔17 articles, label 'View Earlier Essays — 10 more ↓' ↔ 'Show Less — showing all ↑', aria-expanded false↔true. | 2026-09-28: live: 'View Earlier Essays — 10 more ↓' -&gt; 'Show Less — showing all ↑', aria-expanded false-&gt;true-&gt;false, 7-&gt;17-&gt;7 visible. | 2026-10-01 re-verified live: 'View Earlier Essays — 10 more ↓', aria-expanded=false, 10 .earlier-more hidden; click -&gt; 'Show Less — showing all ↑', expanded=true, 0 hidden; re-click restores all three. | 2026-10-05: live: "View Earlier Essays — 10 more" -&gt; click: aria-expanded true, all revealed, "Show Less — showing all"; re-click restores.</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr"/>
@@ -2021,7 +2021,7 @@
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>PASS — 16 plates tile the 12-col grid (lead + wide/secondary/banner rotation, 3 row-plates) | 2026-09-18 re-verified live: 7 visible plates tile the 12-col grid as lead + wide/secondary/banner/secondary/banner/wide; 17 plates total with the 10-plate overflow under View More. | 2026-09-28: live: 17 .plate elements render in the cascade; packer source unchanged since last PASS. | 2026-10-01 re-verified live: 17 plates: lead + wide/secondary/banner rotation in 12-col rows, trailing plate-row (reckonings); packer source unchanged.</t>
+          <t>PASS — 16 plates tile the 12-col grid (lead + wide/secondary/banner rotation, 3 row-plates) | 2026-09-18 re-verified live: 7 visible plates tile the 12-col grid as lead + wide/secondary/banner/secondary/banner/wide; 17 plates total with the 10-plate overflow under View More. | 2026-09-28: live: 17 .plate elements render in the cascade; packer source unchanged since last PASS. | 2026-10-01 re-verified live: 17 plates: lead + wide/secondary/banner rotation in 12-col rows, trailing plate-row (reckonings); packer source unchanged. | 2026-10-05: live: cascade classes rotate wide/secondary/banner; 17 plates, no orphan rows.</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr"/>
@@ -2070,7 +2070,7 @@
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-10-01) — Texture Alternation Rule (DESIGN-SYSTEM.md:718, 'adjacent plates must never share the same background treatment… across row boundaries in reading order') is broken live: archive plates 12 /words/gloria/ (auto slot, img-noise) and 13 /words/the-nets/ (frontmatter plate.image: noise) are both textured AND the same texture, back to back in reading order. Cause: index.astro coverMap honors a forced plate.image regardless of prevTextured, and the comment at index.astro:160-162 assumes the two overrides (the-nets, price-of-sunday) sit at odd archive positions — every new publish shifts parity by one, so the 2026-08-31 publish of the-weight-of-my-no moved them to even positions (12, 14) and the auto slot before the-nets went textured. Prior runs read 'alternation present' without checking adjacency, so this has been live since 08-31. Hidden behind View Earlier on load; adjacent when expanded and on single-column mobile. | prior: PASS — 7 of 15 archive plates carry .plate-image, interleaved with plain (Texture Alternation Rule) | 2026-09-06 re-verified live: eight image plates alternate concrete/lines/noise as designed. NOTE - this run pixel-measured them rather than reading computed styles and found the scrim, not the alternation, at fault; see F101. | 2026-09-11 re-verified live: three homepage image plates alternate img-concrete / img-lines / img-noise across the cascade. | 2026-09-28: live: 8 of 16 archive plates carry .plate-image; source unchanged.</t>
+          <t>ISSUE/Medium (2026-10-01) — Texture Alternation Rule (DESIGN-SYSTEM.md:718, 'adjacent plates must never share the same background treatment… across row boundaries in reading order') is broken live: archive plates 12 /words/gloria/ (auto slot, img-noise) and 13 /words/the-nets/ (frontmatter plate.image: noise) are both textured AND the same texture, back to back in reading order. Cause: index.astro coverMap honors a forced plate.image regardless of prevTextured, and the comment at index.astro:160-162 assumes the two overrides (the-nets, price-of-sunday) sit at odd archive positions — every new publish shifts parity by one, so the 2026-08-31 publish of the-weight-of-my-no moved them to even positions (12, 14) and the auto slot before the-nets went textured. Prior runs read 'alternation present' without checking adjacency, so this has been live since 08-31. Hidden behind View Earlier on load; adjacent when expanded and on single-column mobile. | prior: PASS — 7 of 15 archive plates carry .plate-image, interleaved with plain (Texture Alternation Rule) | 2026-09-06 re-verified live: eight image plates alternate concrete/lines/noise as designed. NOTE - this run pixel-measured them rather than reading computed styles and found the scrim, not the alternation, at fault; see F101. | 2026-09-11 re-verified live: three homepage image plates alternate img-concrete / img-lines / img-noise across the cascade. | 2026-09-28: live: 8 of 16 archive plates carry .plate-image; source unchanged. | 2026-10-05: live: cover order after the lead alternates plain / textured with concrete -&gt; lines -&gt; noise cycling; no adjacent textured pair.</t>
         </is>
       </c>
       <c r="I32" s="7" t="inlineStr">
@@ -2127,7 +2127,7 @@
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>PASS — correctly absent: zero upcoming essays in the collection | 2026-08-25 re-verified live: correctly ABSENT — index.astro renders IssueNext only when an upcoming entry exists, and none does. Not a regression. | 2026-08-27 re-verified live: correctly absent — zero upcoming essays; .next-meta not in the DOM. | 2026-08-27 re-scoped by F94: still correctly absent, but now for two independent reasons — zero upcoming essays AND the new ghost-plate gate. Verified on a fixture build that with an upcoming essay present the strip stays absent and the ghost plate renders in its place. | 2026-08-27 RETIRED: the component no longer exists. IssueNext.astro is deleted and all 202 lines of `.issue-next` CSS are removed from home-v2.css and home-augment.css. Row marked N/A per the never-delete rule — see F94 for the decision and the verification. | 2026-10-01 re-verified live: no upcoming essays and no ghost plate: 0 .issue-next, 0 teaser plates — hidden as specified.</t>
+          <t>PASS — correctly absent: zero upcoming essays in the collection | 2026-08-25 re-verified live: correctly ABSENT — index.astro renders IssueNext only when an upcoming entry exists, and none does. Not a regression. | 2026-08-27 re-verified live: correctly absent — zero upcoming essays; .next-meta not in the DOM. | 2026-08-27 re-scoped by F94: still correctly absent, but now for two independent reasons — zero upcoming essays AND the new ghost-plate gate. Verified on a fixture build that with an upcoming essay present the strip stays absent and the ghost plate renders in its place. | 2026-08-27 RETIRED: the component no longer exists. IssueNext.astro is deleted and all 202 lines of `.issue-next` CSS are removed from home-v2.css and home-augment.css. Row marked N/A per the never-delete rule — see F94 for the decision and the verification. | 2026-10-01 re-verified live: no upcoming essays and no ghost plate: 0 .issue-next, 0 teaser plates — hidden as specified. | 2026-10-05: N/A by F94 decision; 0 .issue-next live and in the fixture build.</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr"/>
@@ -2180,7 +2180,7 @@
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>PASS — manifesto form action=/api/subscribe, source=home, honeypot present | 2026-08-27 re-verified live: manifesto form + #sm-email + submit present on the homepage. | 2026-09-18 re-verified live: manifesto form action=/api/subscribe, #sm-email present, 3 value-prop items, 'No spam' line, honeypot off-canvas (x=-9999, tabindex=-1, aria-hidden). | 2026-09-28: live: #subscribe-manifesto, 3 value-prop items, 'No spam', action /api/subscribe, source=home. | 2026-10-01 re-verified live: #subscribe-manifesto: kicker, title, 3 value-prop items, form.sm-form, 'No spam' line, honeypot name=website tabindex=-1 inside aria-hidden wrapper.</t>
+          <t>PASS — manifesto form action=/api/subscribe, source=home, honeypot present | 2026-08-27 re-verified live: manifesto form + #sm-email + submit present on the homepage. | 2026-09-18 re-verified live: manifesto form action=/api/subscribe, #sm-email present, 3 value-prop items, 'No spam' line, honeypot off-canvas (x=-9999, tabindex=-1, aria-hidden). | 2026-09-28: live: #subscribe-manifesto, 3 value-prop items, 'No spam', action /api/subscribe, source=home. | 2026-10-01 re-verified live: #subscribe-manifesto: kicker, title, 3 value-prop items, form.sm-form, 'No spam' line, honeypot name=website tabindex=-1 inside aria-hidden wrapper. | 2026-10-05: live: manifesto block, #subscribe-manifesto anchor, form action /api/subscribe POST, honeypot off-screen.</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr"/>
@@ -2229,7 +2229,7 @@
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>PASS | 2026-09-18 re-verified live: real submit on the home manifesto form with a server-rejected address (healthscrub@invalid, passes type=email) showed 'Sending…', then state=error with 'That email didn't look right. Try it again.' in a role=alert .sm-error and the button re-enabled. Success path covered by the §9 API smoke (200 subscribed); the UI success state was not driven to avoid a second subscriber write. | 2026-09-28: carried: subscribe.js unchanged; endpoint states verified by API tests today (200 subscribed / already_subscribed / 400 invalid_email / 429). Not browser-submitted today to avoid extra Mailchimp writes. | 2026-10-01 re-verified live: carried: subscribe.js unchanged; endpoint verified by §9 API today (GET 405, POST healthscrub+20261001 -&gt; 200 subscribed 1.53s). Not browser-submitted to avoid a second Mailchimp write.</t>
+          <t>PASS | 2026-09-18 re-verified live: real submit on the home manifesto form with a server-rejected address (healthscrub@invalid, passes type=email) showed 'Sending…', then state=error with 'That email didn't look right. Try it again.' in a role=alert .sm-error and the button re-enabled. Success path covered by the §9 API smoke (200 subscribed); the UI success state was not driven to avoid a second subscriber write. | 2026-09-28: carried: subscribe.js unchanged; endpoint states verified by API tests today (200 subscribed / already_subscribed / 400 invalid_email / 429). Not browser-submitted today to avoid extra Mailchimp writes. | 2026-10-01 re-verified live: carried: subscribe.js unchanged; endpoint verified by §9 API today (GET 405, POST healthscrub+20261001 -&gt; 200 subscribed 1.53s). Not browser-submitted to avoid a second Mailchimp write. | 2026-10-05: live with stubbed fetch (no network): button "Sending…" disabled; subscribed -&gt; "You're in."; already_subscribed -&gt; "Already on the list."; invalid_email -&gt; "That email didn't look right"; rate_limited -&gt; "Too many attempts".</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr"/>
@@ -2282,7 +2282,7 @@
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>PASS — eyebrow lanes/tags + ' + ' separator, date, read time, h1, deck | 2026-08-27 re-verified live: eyebrow lanes/date/read-time render on all 16. | 2026-09-01 re-verified live on VOL 17 at 375px: eyebrow renders 4 lane/tag chips + date + read-time, all inside the frame post-F97. | 2026-09-06 re-verified live: .article-eyebrow computes flex-wrap nowrap at 1280px and wrap at 375px, rail height 57px, zero overflow (F97 holds live). | 2026-09-11 re-verified live: article eyebrow renders lane chips + date + read time; .article-read '8 min' matches the plate. | 2026-09-28: live: eyebrow lane + tag chips, date, read time. | 2026-10-01 re-verified live: the-weight-of-my-no: chips Faith + Identity + Calling + Fear (' + ' via ::before, none on first), &lt;time datetime=2026-08-31&gt;, '8 min', single h1, deck present.</t>
+          <t>PASS — eyebrow lanes/tags + ' + ' separator, date, read time, h1, deck | 2026-08-27 re-verified live: eyebrow lanes/date/read-time render on all 16. | 2026-09-01 re-verified live on VOL 17 at 375px: eyebrow renders 4 lane/tag chips + date + read-time, all inside the frame post-F97. | 2026-09-06 re-verified live: .article-eyebrow computes flex-wrap nowrap at 1280px and wrap at 375px, rail height 57px, zero overflow (F97 holds live). | 2026-09-11 re-verified live: article eyebrow renders lane chips + date + read time; .article-read '8 min' matches the plate. | 2026-09-28: live: eyebrow lane + tag chips, date, read time. | 2026-10-01 re-verified live: the-weight-of-my-no: chips Faith + Identity + Calling + Fear (' + ' via ::before, none on first), &lt;time datetime=2026-08-31&gt;, '8 min', single h1, deck present. | 2026-10-05: live: eyebrow lanes + tags chips, time, read time, single h1, deck on 17/17.</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr"/>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>PASS — all 16 MDX bodies render through [...slug].astro | 2026-08-27 re-verified live: all 16 MDX bodies render. | 2026-09-19 re-verified live: all 17 live articles render an .article-body (shortest body ~6.4k chars of text). | 2026-09-28: live: all 17 article pages 200 with body + BlogPosting wordCount. | 2026-10-01 re-verified live: all 17 /words/&lt;slug&gt;/ return 200 with one .article-body; the-weight-of-my-no renders 56 paragraphs, 3 section heads.</t>
+          <t>PASS — all 16 MDX bodies render through [...slug].astro | 2026-08-27 re-verified live: all 16 MDX bodies render. | 2026-09-19 re-verified live: all 17 live articles render an .article-body (shortest body ~6.4k chars of text). | 2026-09-28: live: all 17 article pages 200 with body + BlogPosting wordCount. | 2026-10-01 re-verified live: all 17 /words/&lt;slug&gt;/ return 200 with one .article-body; the-weight-of-my-no renders 56 paragraphs, 3 section heads. | 2026-10-05: live: 17/17 articles 200 with .article-body rendered.</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr"/>
@@ -2388,7 +2388,7 @@
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>PASS — bar width 0→249→698→1153px and aria-valuenow 0→30→69→100 across the scroll range. 2026-08-10 PM re-check: structural half re-verified (progress.js math recomputed by hand at 50% scroll = 51.5%; .article-body + .reading-progress present; role/aria-label/aria-valuemin/max initialized on load). Runtime paint not re-exercisable this run — the browser pane reports document.visibilityState 'hidden', so requestAnimationFrame never fires and the CSS width transition stays frozen at 0. Harness limitation, not a site regression. | 2026-08-13 re-verified live: reading-progress present on articles at 3px, background var(--ink) rgb(5,5,5) — correct per F82; the doc bullet claiming --accent was struck 2026-08-10. | 2026-08-27 NOT re-verified — rotation gap, not a failure. The reading-progress bar is scroll-driven and the browser pane would not scroll this run (window.scrollTo, scrollingElement.scrollTop, Page_Down x6 and the pointer scroll action all left scrollY at 0-2 on an 11,937px article; the pointer scroll action timed out with 'Browser pane is currently hidden'). Source unchanged since the last PASS, so the row keeps its prior result rather than being reset. | 2026-09-01 NOT TESTABLE this run — rotation gap, prior result retained. The browser pane went hidden: the pointer scroll timed out with 'Browser pane is currently hidden' and window.scrollTo / scrollingElement.scrollTop both left scrollY at 0 against a 10905px document. The .reading-progress element itself is present and correctly wired (role=progressbar, aria-valuenow=0, width 0% at scrollY 0). Neither PASS nor FAIL recorded, per the documented harness antipattern. | 2026-09-11 NOT TESTABLE — rotation gap, prior PASS retained. The browser pane was hidden for the whole run: window.scrollTo(0,2500) left scrollY at 0 and the pointer scroll action timed out with 'Browser pane is currently hidden'. Static wiring re-confirmed live (.reading-progress and .section-indicator both present on /words/the-stone/, section-indicator at opacity 0 at scroll top as specified). Neither PASSed nor FAILed on a tooling limit. | 2026-09-28: ROTATION GAP — pane stuck at scrollY 0 while hidden (QA-OS antipattern); prior result kept, not re-tested. | 2026-10-01: ROTATION GAP — browser pane hidden, scrollTo leaves scrollY at 0 (QA-OS antipattern); prior PASS carried, not re-tested. Static half confirmed: progressbar role, aria-valuemin 0/max 100/now 0 at top. | 2026-10-02: live (headless Chrome via CDP — the pane was hidden and scroll-inert, so the real scroll ran headless against production): /words/the-stone/ bar width 0→256→643→1086→1280px, aria-valuenow 0→25→56→94→100, role=progressbar. Closes the 10-01 rotation gap.</t>
+          <t>PASS — bar width 0→249→698→1153px and aria-valuenow 0→30→69→100 across the scroll range. 2026-08-10 PM re-check: structural half re-verified (progress.js math recomputed by hand at 50% scroll = 51.5%; .article-body + .reading-progress present; role/aria-label/aria-valuemin/max initialized on load). Runtime paint not re-exercisable this run — the browser pane reports document.visibilityState 'hidden', so requestAnimationFrame never fires and the CSS width transition stays frozen at 0. Harness limitation, not a site regression. | 2026-08-13 re-verified live: reading-progress present on articles at 3px, background var(--ink) rgb(5,5,5) — correct per F82; the doc bullet claiming --accent was struck 2026-08-10. | 2026-08-27 NOT re-verified — rotation gap, not a failure. The reading-progress bar is scroll-driven and the browser pane would not scroll this run (window.scrollTo, scrollingElement.scrollTop, Page_Down x6 and the pointer scroll action all left scrollY at 0-2 on an 11,937px article; the pointer scroll action timed out with 'Browser pane is currently hidden'). Source unchanged since the last PASS, so the row keeps its prior result rather than being reset. | 2026-09-01 NOT TESTABLE this run — rotation gap, prior result retained. The browser pane went hidden: the pointer scroll timed out with 'Browser pane is currently hidden' and window.scrollTo / scrollingElement.scrollTop both left scrollY at 0 against a 10905px document. The .reading-progress element itself is present and correctly wired (role=progressbar, aria-valuenow=0, width 0% at scrollY 0). Neither PASS nor FAIL recorded, per the documented harness antipattern. | 2026-09-11 NOT TESTABLE — rotation gap, prior PASS retained. The browser pane was hidden for the whole run: window.scrollTo(0,2500) left scrollY at 0 and the pointer scroll action timed out with 'Browser pane is currently hidden'. Static wiring re-confirmed live (.reading-progress and .section-indicator both present on /words/the-stone/, section-indicator at opacity 0 at scroll top as specified). Neither PASSed nor FAILed on a tooling limit. | 2026-09-28: ROTATION GAP — pane stuck at scrollY 0 while hidden (QA-OS antipattern); prior result kept, not re-tested. | 2026-10-01: ROTATION GAP — browser pane hidden, scrollTo leaves scrollY at 0 (QA-OS antipattern); prior PASS carried, not re-tested. Static half confirmed: progressbar role, aria-valuemin 0/max 100/now 0 at top. | 2026-10-02: live (headless Chrome via CDP — the pane was hidden and scroll-inert, so the real scroll ran headless against production): /words/the-stone/ bar width 0→256→643→1086→1280px, aria-valuenow 0→25→56→94→100, role=progressbar. Closes the 10-01 rotation gap. | 2026-10-05: PASS via headless Chrome over CDP (pane cannot scroll): /words/the-stone/ aria-valuenow 0 -&gt; 6 -&gt; 24 -&gt; 44 -&gt; 65 -&gt; 87 -&gt; 100 with matching width %.</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr"/>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>PASS — pill text tracks sections ('What the Fear Was Actually About' → 'A New Thing' → 'The Thirtieth'), opacity animates in. 2026-08-10 PM re-check: section collection re-verified live (5 .section-head h2 landmarks found on /words/send-someone-else/; the 40%-viewport rule resolves to the correct current section). Opacity fade not observable this run — same hidden-tab rAF/transition suspension as F35. | 2026-08-27 NOT re-verified — rotation gap, not a failure. The section-indicator pill is scroll-driven and the browser pane would not scroll this run (window.scrollTo, scrollingElement.scrollTop, Page_Down x6 and the pointer scroll action all left scrollY at 0-2 on an 11,937px article; the pointer scroll action timed out with 'Browser pane is currently hidden'). Source unchanged since the last PASS, so the row keeps its prior result rather than being reset. | 2026-09-01 NOT TESTABLE this run — rotation gap, prior result retained. The browser pane went hidden: the pointer scroll timed out with 'Browser pane is currently hidden' and window.scrollTo / scrollingElement.scrollTop both left scrollY at 0 against a 10905px document. The .reading-progress element itself is present and correctly wired (role=progressbar, aria-valuenow=0, width 0% at scrollY 0). Neither PASS nor FAIL recorded, per the documented harness antipattern. | 2026-09-11 NOT TESTABLE — rotation gap, prior PASS retained. The browser pane was hidden for the whole run: window.scrollTo(0,2500) left scrollY at 0 and the pointer scroll action timed out with 'Browser pane is currently hidden'. Static wiring re-confirmed live (.reading-progress and .section-indicator both present on /words/the-stone/, section-indicator at opacity 0 at scroll top as specified). Neither PASSed nor FAILed on a tooling limit. | 2026-09-28: ROTATION GAP — pane stuck at scrollY 0 while hidden; prior result kept, not re-tested. | 2026-10-01: ROTATION GAP — browser pane hidden, scrollTo leaves scrollY at 0 (QA-OS antipattern); prior PASS carried, not re-tested. Static half confirmed: .section-indicator present (opacity 0 at top), 3 .section-head h2 landmarks. | 2026-10-02: live (headless Chrome via CDP): 9 .section-head h2 landmarks on /words/the-stone/; pill hidden at 1% (op 0), reads 'The algorithm of outrage.' at 30%, 'The Pharisee in the mirror.' at 60%, 'Mercy is not naiveté.' at 97% (op 1), hides again at 100% (&gt;98%). Closes the 10-01 rotation gap.</t>
+          <t>PASS — pill text tracks sections ('What the Fear Was Actually About' → 'A New Thing' → 'The Thirtieth'), opacity animates in. 2026-08-10 PM re-check: section collection re-verified live (5 .section-head h2 landmarks found on /words/send-someone-else/; the 40%-viewport rule resolves to the correct current section). Opacity fade not observable this run — same hidden-tab rAF/transition suspension as F35. | 2026-08-27 NOT re-verified — rotation gap, not a failure. The section-indicator pill is scroll-driven and the browser pane would not scroll this run (window.scrollTo, scrollingElement.scrollTop, Page_Down x6 and the pointer scroll action all left scrollY at 0-2 on an 11,937px article; the pointer scroll action timed out with 'Browser pane is currently hidden'). Source unchanged since the last PASS, so the row keeps its prior result rather than being reset. | 2026-09-01 NOT TESTABLE this run — rotation gap, prior result retained. The browser pane went hidden: the pointer scroll timed out with 'Browser pane is currently hidden' and window.scrollTo / scrollingElement.scrollTop both left scrollY at 0 against a 10905px document. The .reading-progress element itself is present and correctly wired (role=progressbar, aria-valuenow=0, width 0% at scrollY 0). Neither PASS nor FAIL recorded, per the documented harness antipattern. | 2026-09-11 NOT TESTABLE — rotation gap, prior PASS retained. The browser pane was hidden for the whole run: window.scrollTo(0,2500) left scrollY at 0 and the pointer scroll action timed out with 'Browser pane is currently hidden'. Static wiring re-confirmed live (.reading-progress and .section-indicator both present on /words/the-stone/, section-indicator at opacity 0 at scroll top as specified). Neither PASSed nor FAILed on a tooling limit. | 2026-09-28: ROTATION GAP — pane stuck at scrollY 0 while hidden; prior result kept, not re-tested. | 2026-10-01: ROTATION GAP — browser pane hidden, scrollTo leaves scrollY at 0 (QA-OS antipattern); prior PASS carried, not re-tested. Static half confirmed: .section-indicator present (opacity 0 at top), 3 .section-head h2 landmarks. | 2026-10-02: live (headless Chrome via CDP): 9 .section-head h2 landmarks on /words/the-stone/; pill hidden at 1% (op 0), reads 'The algorithm of outrage.' at 30%, 'The Pharisee in the mirror.' at 60%, 'Mercy is not naiveté.' at 97% (op 1), hides again at 100% (&gt;98%). Closes the 10-01 rotation gap. | 2026-10-05: PASS via headless CDP: pill hidden at top, shows the current section from 10% to 90% ("The courtyard." … "Restoration is the point."), hides again at the end.</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr"/>
@@ -2494,7 +2494,7 @@
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t>PASS — X intent carries encoded url + title | 2026-08-27 re-verified live: X intent carries encoded url + title (checked on /about/). | 2026-09-11 re-verified live: X intent href carries the encoded article URL and 'The Weight of My No — DX', target=_blank rel='noopener noreferrer'. | 2026-09-28: live: X intent carries encoded url + text, target=_blank rel=noopener noreferrer (article + about). | 2026-10-02: live: X intent href carries url=https%3A%2F%2Fimjustdex.com%2Fwords%2Fthe-stone%2F and text 'The Stone You're Holding — DX', target=_blank rel='noopener noreferrer'.</t>
+          <t>PASS — X intent carries encoded url + title | 2026-08-27 re-verified live: X intent carries encoded url + title (checked on /about/). | 2026-09-11 re-verified live: X intent href carries the encoded article URL and 'The Weight of My No — DX', target=_blank rel='noopener noreferrer'. | 2026-09-28: live: X intent carries encoded url + text, target=_blank rel=noopener noreferrer (article + about). | 2026-10-02: live: X intent href carries url=https%3A%2F%2Fimjustdex.com%2Fwords%2Fthe-stone%2F and text 'The Stone You're Holding — DX', target=_blank rel='noopener noreferrer'. | 2026-10-05: live: X intent carries the encoded article URL, target _blank, noopener noreferrer on 17/17.</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr"/>
@@ -2543,7 +2543,7 @@
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>PASS — copy button + [data-copy-status] live region on article and about | 2026-08-27 re-verified live: copy button + [data-copy-status] aria-live=polite region present on article and about. | 2026-09-11 re-verified live: copy-link button present on article and about with data-copy-link set to the absolute page URL; essay.js loaded; aria-live region present. | 2026-09-28: live: button + [data-copy-status] present; failure path verified (label 'Copy failed' + SR status). Success path untestable in the pane: control navigator.clipboard.writeText() -&gt; 'Write permission denied' — harness, not site. Prior PASS kept. | 2026-10-02: live: [data-copy-link]=https://imjustdex.com/words/the-stone/ with [data-copy-status] aria-live=polite.</t>
+          <t>PASS — copy button + [data-copy-status] live region on article and about | 2026-08-27 re-verified live: copy button + [data-copy-status] aria-live=polite region present on article and about. | 2026-09-11 re-verified live: copy-link button present on article and about with data-copy-link set to the absolute page URL; essay.js loaded; aria-live region present. | 2026-09-28: live: button + [data-copy-status] present; failure path verified (label 'Copy failed' + SR status). Success path untestable in the pane: control navigator.clipboard.writeText() -&gt; 'Write permission denied' — harness, not site. Prior PASS kept. | 2026-10-02: live: [data-copy-link]=https://imjustdex.com/words/the-stone/ with [data-copy-status] aria-live=polite. | 2026-10-05: live: fail path only — the pane denies clipboard-write (permission "denied"); label -&gt; "Copy failed" + live region announcement. Harness limit, as documented.</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr"/>
@@ -2596,7 +2596,7 @@
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>PASS — Follow Me → instagram.com/ImJustDex | 2026-08-27 re-verified live: Follow Me → instagram.com/ImJustDex, 200. | 2026-09-19 re-verified live: Follow Me → instagram.com/ImJustDex with target=_blank rel='noopener noreferrer' on 17/17 articles and on /about/. | 2026-09-28: live: Follow Me -&gt; instagram.com/ImJustDex, _blank noopener noreferrer (article + about). | 2026-10-02: live: Follow Me → https://instagram.com/ImJustDex, target=_blank rel='noopener noreferrer'.</t>
+          <t>PASS — Follow Me → instagram.com/ImJustDex | 2026-08-27 re-verified live: Follow Me → instagram.com/ImJustDex, 200. | 2026-09-19 re-verified live: Follow Me → instagram.com/ImJustDex with target=_blank rel='noopener noreferrer' on 17/17 articles and on /about/. | 2026-09-28: live: Follow Me -&gt; instagram.com/ImJustDex, _blank noopener noreferrer (article + about). | 2026-10-02: live: Follow Me → https://instagram.com/ImJustDex, target=_blank rel='noopener noreferrer'. | 2026-10-05: live: Follow Me -&gt; instagram.com/ImJustDex (_blank, noopener noreferrer) on articles + about.</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr"/>
@@ -2645,7 +2645,7 @@
       </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
-          <t>PASS — form posts /api/subscribe with source=article, honeypot off-canvas, aria-live label; server states verified directly against the function | 2026-09-18 re-verified live: server-rejected address on /words/gumbo/ surfaced 'That email didn’t look right. Try it again.' in the role=status aria-live label and kept the form — it reflects the server failure rather than a blanket success. source=article, honeypot off-canvas at x=-4972. | 2026-09-28: live: article form posts /api/subscribe, source=article, honeypot 'website' present; fixture build coming-soon form source=coming-soon. | 2026-10-02: live: .email-signup action=/api/subscribe, source=article, honeypot [name=website] present, aria-live region present; function POST (healthscrub+20261002) returned 200 subscribed in 1.31s.</t>
+          <t>PASS — form posts /api/subscribe with source=article, honeypot off-canvas, aria-live label; server states verified directly against the function | 2026-09-18 re-verified live: server-rejected address on /words/gumbo/ surfaced 'That email didn’t look right. Try it again.' in the role=status aria-live label and kept the form — it reflects the server failure rather than a blanket success. source=article, honeypot off-canvas at x=-4972. | 2026-09-28: live: article form posts /api/subscribe, source=article, honeypot 'website' present; fixture build coming-soon form source=coming-soon. | 2026-10-02: live: .email-signup action=/api/subscribe, source=article, honeypot [name=website] present, aria-live region present; function POST (healthscrub+20261002) returned 200 subscribed in 1.31s. | 2026-10-05: live: native constraint validation blocks a malformed address (0 fetches); a forced network failure shows "Network hiccup. Try again." (no blanket success); source=article; honeypot off-screen, aria-hidden, tabindex -1.</t>
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr"/>
@@ -2698,7 +2698,7 @@
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
-          <t>PASS (live + fixture build) | Authored prev/next render correctly on all 16. Ghost/teaser path PENDING — requires a future-dated entry; none exists. 2026-08-10 PM: the derive-from-live-status fix (p3) live-verified, then the underlying data cleaned — the 4 stale ghost:true flags are gone (see F81). Zero `ghost: true` remain in the collection; all 16 essays render real .article-nav-link anchors, 15 rel=next head links (newest correctly has none), zero article-nav-ghost teasers. | 2026-08-25 re-verified live: all 16 essays render real .article-nav-link anchors; zero `ghost: true` remain in the collection. Ghost/teaser path still PENDING — still requires a future-dated entry and none exists. | 2026-09-11: authored prev/next re-verified live — newest essay emits rel=prev only, /words/the-stone/ emits rel=prev + rel=next. Ghost/teaser path still PENDING; zero upcoming entries in the collection. | 2026-09-19: authored prev/next unchanged (no code churn since 507e988). Ghost/teaser path still PENDING — zero upcoming entries in the collection. | 2026-09-23: authored prev/next unchanged (no code or content commits since 09-19). Ghost path still PENDING — no future-dated entry. | 2026-09-25: still PENDING — 17/17 entries status published and past-dated, no upcoming entry to render.  | 2026-09-28: PASS (live + build-verified via throwaway fixture). Live: authored prev/next correct; send-someone-else's stale frontmatter ghost:true is neutralised by nextLive, so live renders a real rel=next. Fixture (future-dated entry in a scratch copy, never committed): the-weight-of-my-no's next renders .article-nav-ghost with 'Jan 15, 2027' and NO rel=next. | 2026-10-02: live: authored half PASS — /words/the-stone/ article-nav prev→/words/pulpit/ (rel=prev), next→/words/should-have-killed-it/ (rel=next). Ghost half still structurally untestable — 0 upcoming entries (17/17 status published, newest 2026-08-31).</t>
+          <t>PASS (live + fixture build) | Authored prev/next render correctly on all 16. Ghost/teaser path PENDING — requires a future-dated entry; none exists. 2026-08-10 PM: the derive-from-live-status fix (p3) live-verified, then the underlying data cleaned — the 4 stale ghost:true flags are gone (see F81). Zero `ghost: true` remain in the collection; all 16 essays render real .article-nav-link anchors, 15 rel=next head links (newest correctly has none), zero article-nav-ghost teasers. | 2026-08-25 re-verified live: all 16 essays render real .article-nav-link anchors; zero `ghost: true` remain in the collection. Ghost/teaser path still PENDING — still requires a future-dated entry and none exists. | 2026-09-11: authored prev/next re-verified live — newest essay emits rel=prev only, /words/the-stone/ emits rel=prev + rel=next. Ghost/teaser path still PENDING; zero upcoming entries in the collection. | 2026-09-19: authored prev/next unchanged (no code churn since 507e988). Ghost/teaser path still PENDING — zero upcoming entries in the collection. | 2026-09-23: authored prev/next unchanged (no code or content commits since 09-19). Ghost path still PENDING — no future-dated entry. | 2026-09-25: still PENDING — 17/17 entries status published and past-dated, no upcoming entry to render.  | 2026-09-28: PASS (live + build-verified via throwaway fixture). Live: authored prev/next correct; send-someone-else's stale frontmatter ghost:true is neutralised by nextLive, so live renders a real rel=next. Fixture (future-dated entry in a scratch copy, never committed): the-weight-of-my-no's next renders .article-nav-ghost with 'Jan 15, 2027' and NO rel=next. | 2026-10-02: live: authored half PASS — /words/the-stone/ article-nav prev→/words/pulpit/ (rel=prev), next→/words/should-have-killed-it/ (rel=next). Ghost half still structurally untestable — 0 upcoming entries (17/17 status published, newest 2026-08-31). | 2026-10-05: live: authored prev/next correct across all 17 after the F109 fix (build-verified); fixture: the newest essay's ghost next renders .article-nav-ghost with "Jan 15, 2027" and no rel=next.</t>
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr"/>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="H45" s="6" t="inlineStr">
         <is>
-          <t>PASS — rel=prev emitted where prev authored; rel=next where next authored and live | 2026-08-25 re-verified live: rel=prev/next head links intact across the chain. | 2026-09-11 re-verified live: newest essay emits rel=prev only; /words/the-stone/ emits both rel=prev and rel=next. Correct. | 2026-09-28: live: the-weight-of-my-no rel=prev only; show-me-your-glory rel=prev + rel=next; fixture: ghost next emits no rel=next. | 2026-10-02: live: head emits link rel=prev /words/pulpit/ and rel=next /words/should-have-killed-it/ on /words/the-stone/.</t>
+          <t>PASS — rel=prev emitted where prev authored; rel=next where next authored and live | 2026-08-25 re-verified live: rel=prev/next head links intact across the chain. | 2026-09-11 re-verified live: newest essay emits rel=prev only; /words/the-stone/ emits both rel=prev and rel=next. Correct. | 2026-09-28: live: the-weight-of-my-no rel=prev only; show-me-your-glory rel=prev + rel=next; fixture: ghost next emits no rel=next. | 2026-10-02: live: head emits link rel=prev /words/pulpit/ and rel=next /words/should-have-killed-it/ on /words/the-stone/. | 2026-10-05: live: rel=prev/next on every article; the newest has prev only; fixture ghost emits no rel=next.</t>
         </is>
       </c>
       <c r="I45" s="6" t="inlineStr"/>
@@ -2804,7 +2804,7 @@
       </c>
       <c r="H46" s="6" t="inlineStr">
         <is>
-          <t>PASS — '← Back' → '/' on article, coming-soon, about | 2026-09-11 re-verified live: '← Back' → '/' present on article and about. | 2026-09-28: live: '← Back' (.article-back) -&gt; '/' on article + about. | 2026-10-02: live: '← Back' → '/' on /words/the-stone/.</t>
+          <t>PASS — '← Back' → '/' on article, coming-soon, about | 2026-09-11 re-verified live: '← Back' → '/' present on article and about. | 2026-09-28: live: '← Back' (.article-back) -&gt; '/' on article + about. | 2026-10-02: live: '← Back' → '/' on /words/the-stone/. | 2026-10-05: live: "← Back" -&gt; "/" on articles and about.</t>
         </is>
       </c>
       <c r="I46" s="6" t="inlineStr"/>
@@ -2853,7 +2853,7 @@
       </c>
       <c r="H47" s="6" t="inlineStr">
         <is>
-          <t>PASS — PullQuote, Scripture, Callout, DropCap, Closing, SectionHead, ResearchCTA, StudyNote all render and are styled via external hashed CSS (CSP-clean) | 2026-08-27 re-verified live: PullQuote/Scripture/Callout/StudyNote all render (the-stone: 2 pull-quotes, 4 scripture, 2 callouts, 3 study notes). | 2026-09-11 re-verified live: all MDX components still render; ResearchCTA now appears only on /words/show-me-your-glory/ (target thereturningglory.com 200) and is correctly gone from /words/the-nets/ after 507e988. | 2026-09-28: live: show-me-your-glory — .callout left border #c00, 3 StudyNotes, 0 contrast failures across 151 elements in both modes. | 2026-10-02: live: /words/the-stone/ renders 2 pull-quotes, 4 scripture, 2 callouts, 9 section heads; 0 contrast failures in light and dark (real-click toggle).</t>
+          <t>PASS — PullQuote, Scripture, Callout, DropCap, Closing, SectionHead, ResearchCTA, StudyNote all render and are styled via external hashed CSS (CSP-clean) | 2026-08-27 re-verified live: PullQuote/Scripture/Callout/StudyNote all render (the-stone: 2 pull-quotes, 4 scripture, 2 callouts, 3 study notes). | 2026-09-11 re-verified live: all MDX components still render; ResearchCTA now appears only on /words/show-me-your-glory/ (target thereturningglory.com 200) and is correctly gone from /words/the-nets/ after 507e988. | 2026-09-28: live: show-me-your-glory — .callout left border #c00, 3 StudyNotes, 0 contrast failures across 151 elements in both modes. | 2026-10-02: live: /words/the-stone/ renders 2 pull-quotes, 4 scripture, 2 callouts, 9 section heads; 0 contrast failures in light and dark (real-click toggle). | 2026-10-05: live: /words/the-stone/ renders PullQuote x2, Scripture x4, Callout x2, StatBlock, SectionHead x9, StudyNote x3; contrast sweep 0 failures in both modes.</t>
         </is>
       </c>
       <c r="I47" s="6" t="inlineStr"/>
@@ -2906,7 +2906,7 @@
       </c>
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>PASS — &lt;details&gt; summary toggles open→closed→open on both sampled essays | 2026-08-27 re-verified live: &lt;details&gt; summary toggles closed→open→closed on the-stone. | 2026-09-11 re-verified live: 12 essays carry native &lt;details class=study-note&gt; with &lt;summary&gt;; 1–3 per essay. | 2026-09-28: live: &lt;details&gt; toggles closed -&gt; open -&gt; closed. | 2026-10-02: live: 3 &lt;details class=study-note&gt; on /words/the-stone/; summary toggles closed→open→closed.</t>
+          <t>PASS — &lt;details&gt; summary toggles open→closed→open on both sampled essays | 2026-08-27 re-verified live: &lt;details&gt; summary toggles closed→open→closed on the-stone. | 2026-09-11 re-verified live: 12 essays carry native &lt;details class=study-note&gt; with &lt;summary&gt;; 1–3 per essay. | 2026-09-28: live: &lt;details&gt; toggles closed -&gt; open -&gt; closed. | 2026-10-02: live: 3 &lt;details class=study-note&gt; on /words/the-stone/; summary toggles closed→open→closed. | 2026-10-05: live: StudyNote &lt;details&gt; toggles open and closed on click.</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr"/>
@@ -2959,7 +2959,7 @@
       </c>
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>PASS (build-verified via fixture) | PENDING — all 16 entries are status published with past dates, so isUpcomingData() is false everywhere and no coming-soon page renders | 2026-08-25: still PENDING for the same structural reason — all 16 built entries are status:published with past dates. NOTE: an untracked draft (src/content/words/before-i-had-the-words.mdx, status:"drafted", publishedDate 2026-08-07) sits in Dexter's working tree. It is correctly excluded from the build (19 pages, 16 articles) and does not exercise this path either, since its date is in the past, not the future. | 2026-09-01 still PENDING. The untracked draft in Dexter's working tree (src/content/words/before-i-had-the-words.mdx, status 'drafted', publishedDate 2026-08-07) is correctly excluded from the build (20 pages, 17 articles) but does NOT exercise this path — its date is in the past and its status is 'drafted', not an upcoming publish. Left untouched. | 2026-09-11: still PENDING for the same structural reason — 17 published entries, all past-dated. The untracked draft src/content/words/before-i-had-the-words.mdx is still status 'drafted' in Dexter's working tree, so it builds nothing and is correctly absent from sitemap and feed. | 2026-09-19: still PENDING for the same structural reason — no upcoming entry; the untracked draft is still 'drafted' and builds nothing. | 2026-09-23: still PENDING for the same structural reason — 17/17 entries published, isUpcomingData() false everywhere. | 2026-09-25: still PENDING — 17/17 entries status published and past-dated, no upcoming entry to render.  | 2026-09-28: BUILD-VERIFIED via a throwaway future-dated fixture in a scratch copy (never committed): 'Coming Soon' tag, 'Friday, January 15, 2027', subscribe form source=coming-soon, noindex, og:image preserved (og-&lt;slug&gt;.png), 0 essay-body text leaked, excluded from sitemap/feed/cascade. Live half still awaits a real upcoming entry.</t>
+          <t>PASS (build-verified via fixture) | PENDING — all 16 entries are status published with past dates, so isUpcomingData() is false everywhere and no coming-soon page renders | 2026-08-25: still PENDING for the same structural reason — all 16 built entries are status:published with past dates. NOTE: an untracked draft (src/content/words/before-i-had-the-words.mdx, status:"drafted", publishedDate 2026-08-07) sits in Dexter's working tree. It is correctly excluded from the build (19 pages, 16 articles) and does not exercise this path either, since its date is in the past, not the future. | 2026-09-01 still PENDING. The untracked draft in Dexter's working tree (src/content/words/before-i-had-the-words.mdx, status 'drafted', publishedDate 2026-08-07) is correctly excluded from the build (20 pages, 17 articles) but does NOT exercise this path — its date is in the past and its status is 'drafted', not an upcoming publish. Left untouched. | 2026-09-11: still PENDING for the same structural reason — 17 published entries, all past-dated. The untracked draft src/content/words/before-i-had-the-words.mdx is still status 'drafted' in Dexter's working tree, so it builds nothing and is correctly absent from sitemap and feed. | 2026-09-19: still PENDING for the same structural reason — no upcoming entry; the untracked draft is still 'drafted' and builds nothing. | 2026-09-23: still PENDING for the same structural reason — 17/17 entries published, isUpcomingData() false everywhere. | 2026-09-25: still PENDING — 17/17 entries status published and past-dated, no upcoming entry to render.  | 2026-09-28: BUILD-VERIFIED via a throwaway future-dated fixture in a scratch copy (never committed): 'Coming Soon' tag, 'Friday, January 15, 2027', subscribe form source=coming-soon, noindex, og:image preserved (og-&lt;slug&gt;.png), 0 essay-body text leaked, excluded from sitemap/feed/cascade. Live half still awaits a real upcoming entry. | 2026-10-05: PASS (fixture build, never committed): "Coming Soon", "Friday, January 15, 2027", source=coming-soon, noindex, og-&lt;slug&gt;.png preserved, 0 body text leaked, absent from sitemap/feed.</t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr"/>
@@ -3012,7 +3012,7 @@
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>PASS — about content + ProfilePage render | 2026-08-27 re-verified live: about content + ProfilePage render. | 2026-09-01 re-verified live: /about/ 200 in 0.75s, single h1, all four landmarks, 0 contrast failures across 24 measured elements. | 2026-09-19 re-verified live: /about/ 200 in 0.38s, deck 'Est. 1994.' present, single h1, ProfilePage JSON-LD complete, 0 contrast failures across 23 elements in both modes. | 2026-09-28: live: 'Est. 1994' deck, PullQuote, Closing, ProfilePage. | 2026-10-04: live: /about/ 200 (0.34s), deck 'Est. 1994.', h1 'Dexter Jakes', 9 body paras incl intro, pull-quote present, canonical /about/, ProfilePage+Person+Organization JSON-LD with all required mainEntity fields; 0 console errors.</t>
+          <t>PASS — about content + ProfilePage render | 2026-08-27 re-verified live: about content + ProfilePage render. | 2026-09-01 re-verified live: /about/ 200 in 0.75s, single h1, all four landmarks, 0 contrast failures across 24 measured elements. | 2026-09-19 re-verified live: /about/ 200 in 0.38s, deck 'Est. 1994.' present, single h1, ProfilePage JSON-LD complete, 0 contrast failures across 23 elements in both modes. | 2026-09-28: live: 'Est. 1994' deck, PullQuote, Closing, ProfilePage. | 2026-10-04: live: /about/ 200 (0.34s), deck 'Est. 1994.', h1 'Dexter Jakes', 9 body paras incl intro, pull-quote present, canonical /about/, ProfilePage+Person+Organization JSON-LD with all required mainEntity fields; 0 console errors. | 2026-10-05: live: about header, deck "Est. 1994.", pull quote, closing, single h1, canonical /about/, ProfilePage LD.</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr"/>
@@ -3061,7 +3061,7 @@
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>PASS — share bar X + copy + Follow Me with live region | 2026-08-27 re-verified live: share bar X + copy + Follow Me + live region present on /about/. | 2026-09-19 re-verified live: /about/ share bar carries X intent, data-copy-link, Follow Me and an aria-live region. | 2026-09-28: live: X intent + Copy link (data-copy-link) + Follow Me on /about/. | 2026-10-04: live: X intent (about url+text), data-copy-link=/about/, Follow Me→Instagram, aria-live status present. Real pointer click on Copy link announced 'Copy failed. Select the URL manually.' — harness artifact, not a defect: the pane's browser reports clipboard-write permission 'denied' and rejects writeText even outside the click; the site's honest fail path + live region behaved exactly as built.</t>
+          <t>PASS — share bar X + copy + Follow Me with live region | 2026-08-27 re-verified live: share bar X + copy + Follow Me + live region present on /about/. | 2026-09-19 re-verified live: /about/ share bar carries X intent, data-copy-link, Follow Me and an aria-live region. | 2026-09-28: live: X intent + Copy link (data-copy-link) + Follow Me on /about/. | 2026-10-04: live: X intent (about url+text), data-copy-link=/about/, Follow Me→Instagram, aria-live status present. Real pointer click on Copy link announced 'Copy failed. Select the URL manually.' — harness artifact, not a defect: the pane's browser reports clipboard-write permission 'denied' and rejects writeText even outside the click; the site's honest fail path + live region behaved exactly as built. | 2026-10-05: live: about share bar X intent (about URL), Copy link (data-copy-link), Follow Me.</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr"/>
@@ -3114,7 +3114,7 @@
       </c>
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>PASS — bespoke notfound-plate, 200 on /404, noindex+nofollow, /* fallback 404s unmatched routes | 2026-08-27 re-verified live: bespoke notfound-plate, 200 on /404, noindex+nofollow, single h1. | 2026-09-01 re-verified live: /404 returns HTTP 200 with the bespoke 'Nothing to Document Here' body, meta robots noindex,nofollow, single h1, all four landmarks, 0 contrast failures across 16 elements. | 2026-09-19 re-verified live: unmatched route returns HTTP 404 with the bespoke 'Nothing to Document Here' body, meta robots 'noindex, nofollow', Back to Home → /; 0 contrast failures in both modes. | 2026-09-28: live: unmatched route -&gt; HTTP 404, notfound-plate, 'Back to Home' -&gt; /, noindex,nofollow, 0 contrast failures (dark). | 2026-10-04: live: /404 200 with .notfound-plate, single h1 'Nothing to Document Here.', noindex,nofollow, 'Back to Home'→/; unmatched /no-such-page-qa → HTTP 404 with the bespoke body; 0 console errors.</t>
+          <t>PASS — bespoke notfound-plate, 200 on /404, noindex+nofollow, /* fallback 404s unmatched routes | 2026-08-27 re-verified live: bespoke notfound-plate, 200 on /404, noindex+nofollow, single h1. | 2026-09-01 re-verified live: /404 returns HTTP 200 with the bespoke 'Nothing to Document Here' body, meta robots noindex,nofollow, single h1, all four landmarks, 0 contrast failures across 16 elements. | 2026-09-19 re-verified live: unmatched route returns HTTP 404 with the bespoke 'Nothing to Document Here' body, meta robots 'noindex, nofollow', Back to Home → /; 0 contrast failures in both modes. | 2026-09-28: live: unmatched route -&gt; HTTP 404, notfound-plate, 'Back to Home' -&gt; /, noindex,nofollow, 0 contrast failures (dark). | 2026-10-04: live: /404 200 with .notfound-plate, single h1 'Nothing to Document Here.', noindex,nofollow, 'Back to Home'→/; unmatched /no-such-page-qa → HTTP 404 with the bespoke body; 0 console errors. | 2026-10-05: live: unmatched route -&gt; HTTP 404 with the bespoke "Nothing to Document Here" body; Back to Home -&gt; /; noindex,nofollow.</t>
         </is>
       </c>
       <c r="I52" s="6" t="inlineStr"/>
@@ -3167,7 +3167,7 @@
       </c>
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>PASS — Atom 16 entries = 16 published; namespace + entries valid | 2026-08-13 re-verified live: /feed.xml 200, Atom namespace, 16 &lt;entry&gt; elements — exactly matching the 16 articles on the homepage, zero set difference either direction. | 2026-08-16 re-verified live: /feed.xml 200 with 16 &lt;entry&gt; elements; set-compared against the 16 article links on the live homepage — zero difference in either direction. | 2026-08-25 re-verified live: /feed.xml 200, 16 &lt;entry&gt; elements matching the 16 published articles exactly — no gaps, no extras. | 2026-08-27 re-verified live: Atom 16 entries == 16 published on the homepage. | 2026-09-01 re-verified live: /feed.xml 200, 17 entries — exactly matching the 17 articles on the homepage cascade. No feed-only or home-only slugs. | 2026-09-06 re-verified live: /feed.xml 200, 17 entries, slug set identical to the homepage cascade. | 2026-09-11 re-verified live: /feed.xml parses as Atom, 17 entries, matching the 17 published articles exactly. | 2026-09-28: live: Atom 17 entries = 17 published, 27 lane categories, subtitle/rights/icon/logo/author present, application/xml, must-revalidate. | 2026-10-04: live: /feed.xml 200, 17 &lt;entry&gt; = 17 homepage essays, 5/5 security headers.</t>
+          <t>PASS — Atom 16 entries = 16 published; namespace + entries valid | 2026-08-13 re-verified live: /feed.xml 200, Atom namespace, 16 &lt;entry&gt; elements — exactly matching the 16 articles on the homepage, zero set difference either direction. | 2026-08-16 re-verified live: /feed.xml 200 with 16 &lt;entry&gt; elements; set-compared against the 16 article links on the live homepage — zero difference in either direction. | 2026-08-25 re-verified live: /feed.xml 200, 16 &lt;entry&gt; elements matching the 16 published articles exactly — no gaps, no extras. | 2026-08-27 re-verified live: Atom 16 entries == 16 published on the homepage. | 2026-09-01 re-verified live: /feed.xml 200, 17 entries — exactly matching the 17 articles on the homepage cascade. No feed-only or home-only slugs. | 2026-09-06 re-verified live: /feed.xml 200, 17 entries, slug set identical to the homepage cascade. | 2026-09-11 re-verified live: /feed.xml parses as Atom, 17 entries, matching the 17 published articles exactly. | 2026-09-28: live: Atom 17 entries = 17 published, 27 lane categories, subtitle/rights/icon/logo/author present, application/xml, must-revalidate. | 2026-10-04: live: /feed.xml 200, 17 &lt;entry&gt; = 17 homepage essays, 5/5 security headers. | 2026-10-05: live: Atom feed, 17 entries == homepage cascade.</t>
         </is>
       </c>
       <c r="I53" s="6" t="inlineStr"/>
@@ -3220,7 +3220,7 @@
       </c>
       <c r="H54" s="6" t="inlineStr">
         <is>
-          <t>PASS — feed.xsl 200 and &lt;?xml-stylesheet?&gt; PI present | 2026-08-13 re-verified live: /feed.xsl 200 and referenced via &lt;?xml-stylesheet?&gt; in the feed prolog. | 2026-08-25 re-verified live: /feed.xsl 200 and feed.xml carries &lt;?xml-stylesheet href="/feed.xsl"?&gt;. | 2026-08-27 re-verified live: feed.xsl 200 and the &lt;?xml-stylesheet?&gt; PI is present. | 2026-09-01 re-verified live: /feed.xml carries the &lt;?xml-stylesheet?&gt; reference and /feed.xsl returns 200. | 2026-09-06 re-verified live: feed.xsl 200 (4342b) and the feed still declares &lt;?xml-stylesheet href="/feed.xsl"?&gt;. | 2026-09-11 re-verified live: feed carries &lt;?xml-stylesheet type='text/xsl' href='/feed.xsl'?&gt; and /feed.xsl returns 200 and parses. | 2026-09-28: live: feed.xsl 200 application/xml; xml-stylesheet PI present; style-src unsafe-inline on /feed.xml + /feed.xsl. | 2026-10-04: live: /feed.xsl 200 and referenced by the &lt;?xml-stylesheet?&gt; PI.</t>
+          <t>PASS — feed.xsl 200 and &lt;?xml-stylesheet?&gt; PI present | 2026-08-13 re-verified live: /feed.xsl 200 and referenced via &lt;?xml-stylesheet?&gt; in the feed prolog. | 2026-08-25 re-verified live: /feed.xsl 200 and feed.xml carries &lt;?xml-stylesheet href="/feed.xsl"?&gt;. | 2026-08-27 re-verified live: feed.xsl 200 and the &lt;?xml-stylesheet?&gt; PI is present. | 2026-09-01 re-verified live: /feed.xml carries the &lt;?xml-stylesheet?&gt; reference and /feed.xsl returns 200. | 2026-09-06 re-verified live: feed.xsl 200 (4342b) and the feed still declares &lt;?xml-stylesheet href="/feed.xsl"?&gt;. | 2026-09-11 re-verified live: feed carries &lt;?xml-stylesheet type='text/xsl' href='/feed.xsl'?&gt; and /feed.xsl returns 200 and parses. | 2026-09-28: live: feed.xsl 200 application/xml; xml-stylesheet PI present; style-src unsafe-inline on /feed.xml + /feed.xsl. | 2026-10-04: live: /feed.xsl 200 and referenced by the &lt;?xml-stylesheet?&gt; PI. | 2026-10-05: live: xml-stylesheet PI -&gt; /feed.xsl renders the human feed; /feed.xml CSP allows unsafe-inline style. Chrome now logs "XSLTProcessor and XSLT Processing Instructions have been deprecated" here — watch item, not a defect today.</t>
         </is>
       </c>
       <c r="I54" s="6" t="inlineStr"/>
@@ -3273,7 +3273,7 @@
       </c>
       <c r="H55" s="6" t="inlineStr">
         <is>
-          <t>PASS — 5 anchor links, all resolve to real targets | 2026-08-27 re-verified live: 5 anchor links on /phase0/, all resolve to real targets. | 2026-09-01 re-verified live: /phase0/ 200 in 0.41s, single h1, no skipped heading levels across a 22-heading tree, 0 contrast failures across 106 measured elements. | 2026-09-19 re-verified live: /phase0/ 200 in 0.39s, single h1, 0 contrast failures across 105 elements in both modes, no horizontal overflow at 375px. | 2026-09-28: live: anchors #phase0/#get/#definition all resolve; single h1; tokens + shell + phase0 css. | 2026-10-04: live: /phase0/ 200 (0.50s), 10 sections, CTAs 'Get The Prompt'→#get / 'Read The System'→#definition, 5 anchor links all resolve, tokens+shell+phase0 CSS, single h1, 0 console errors.</t>
+          <t>PASS — 5 anchor links, all resolve to real targets | 2026-08-27 re-verified live: 5 anchor links on /phase0/, all resolve to real targets. | 2026-09-01 re-verified live: /phase0/ 200 in 0.41s, single h1, no skipped heading levels across a 22-heading tree, 0 contrast failures across 106 measured elements. | 2026-09-19 re-verified live: /phase0/ 200 in 0.39s, single h1, 0 contrast failures across 105 elements in both modes, no horizontal overflow at 375px. | 2026-09-28: live: anchors #phase0/#get/#definition all resolve; single h1; tokens + shell + phase0 css. | 2026-10-04: live: /phase0/ 200 (0.50s), 10 sections, CTAs 'Get The Prompt'→#get / 'Read The System'→#definition, 5 anchor links all resolve, tokens+shell+phase0 CSS, single h1, 0 console errors. | 2026-10-05: live: 10 sections, Get The Prompt -&gt; #get, Read The System -&gt; #definition, tokens + shell + phase0 CSS.</t>
         </is>
       </c>
       <c r="I55" s="6" t="inlineStr"/>
@@ -3326,7 +3326,7 @@
       </c>
       <c r="H56" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: /phase0/ form action is /api/subscribe with no legacy Mailchimp query string; matches the other three subscribe surfaces. | 2026-08-27 re-verified live: /phase0/ form action=/api/subscribe, honeypot present, source=phase0. | 2026-09-19 re-verified live: /phase0/ .phase0-capture posts to /api/subscribe with empty honeypot (name=website), source=phase0, noscript fallback and phase0.js present. | 2026-09-28 ISSUE/Medium — the first time the validation branch was exercised (every prior check read the form's action/honeypot/source only): a mistyped email shows 'Something broke on our end. Try again, or email dex@imjustdex.com.' through the role=alert, assertive error region. Cause: js/phase0.js calls setError() with no copy on client-side validation failure, and the error &lt;p&gt; ships holding the server-failure line. A 400 invalid_email or 429 rate_limited from the function also rendered the outage line. The user story's 'not lie on failure' is broken for every reader with a typo. Measured live on /phase0/ (aria-invalid=true, 0 POSTs, visible .form-msg = outage copy), then reproduced 4/8 scenario failures by running the pre-fix file in a stub-DOM harness. | 2026-10-04: live: form action /api/subscribe, data-no-signup-js, source=phase0, honeypot present, noscript present. Invalid email → aria-invalid=true + 'That email didn’t look right.' with zero fetches; valid keystroke clears aria-invalid and hides the msg (state idle).</t>
+          <t>PASS — live-verified 2026-08-10: /phase0/ form action is /api/subscribe with no legacy Mailchimp query string; matches the other three subscribe surfaces. | 2026-08-27 re-verified live: /phase0/ form action=/api/subscribe, honeypot present, source=phase0. | 2026-09-19 re-verified live: /phase0/ .phase0-capture posts to /api/subscribe with empty honeypot (name=website), source=phase0, noscript fallback and phase0.js present. | 2026-09-28 ISSUE/Medium — the first time the validation branch was exercised (every prior check read the form's action/honeypot/source only): a mistyped email shows 'Something broke on our end. Try again, or email dex@imjustdex.com.' through the role=alert, assertive error region. Cause: js/phase0.js calls setError() with no copy on client-side validation failure, and the error &lt;p&gt; ships holding the server-failure line. A 400 invalid_email or 429 rate_limited from the function also rendered the outage line. The user story's 'not lie on failure' is broken for every reader with a typo. Measured live on /phase0/ (aria-invalid=true, 0 POSTs, visible .form-msg = outage copy), then reproduced 4/8 scenario failures by running the pre-fix file in a stub-DOM harness. | 2026-10-04: live: form action /api/subscribe, data-no-signup-js, source=phase0, honeypot present, noscript present. Invalid email → aria-invalid=true + 'That email didn’t look right.' with zero fetches; valid keystroke clears aria-invalid and hides the msg (state idle). | 2026-10-05: live: "bad@" -&gt; aria-invalid true + error, 0 fetches; a valid keystroke clears both; forced network failure -&gt; outage copy + Retry.</t>
         </is>
       </c>
       <c r="I56" s="6" t="inlineStr">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="H57" s="6" t="inlineStr">
         <is>
-          <t>PASS — footer year 2026 = current year | 2026-08-27 re-verified live: phase0 footer year 2026. | 2026-09-19 re-verified live: #yr reads 2026 = current year on /phase0/. | 2026-09-28: live: #yr = 2026. | 2026-10-04: live: #yr = 2026 = current year.</t>
+          <t>PASS — footer year 2026 = current year | 2026-08-27 re-verified live: phase0 footer year 2026. | 2026-09-19 re-verified live: #yr reads 2026 = current year on /phase0/. | 2026-09-28: live: #yr = 2026. | 2026-10-04: live: #yr = 2026 = current year. | 2026-10-05: live: #yr = 2026.</t>
         </is>
       </c>
       <c r="I57" s="6" t="inlineStr"/>
@@ -3436,7 +3436,7 @@
       </c>
       <c r="H58" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: /brand/ serves plates.css?v=phase15, matching every other surface; no second year-long cache entry. | 2026-09-01 re-verified live: /brand/ 200, single h1, no skipped heading levels, 0 contrast failures across 800 measured elements in dark mode. | 2026-09-22 re-verified live: /brand/ 200 in 0.48s; CSP style-src 'self' 'unsafe-inline' (scoped override intact); 0 inline &lt;script&gt; (mode.js + JSON-LD + Netlify RUM only); present in sitemap-0.xml; 680 text elements swept in dark mode, 0 contrast failures; image-plate specimens keep display:flex + justify-content:flex-end (no F100 regression). | 2026-09-28: live: /brand/ 200, scoped CSP style-src unsafe-inline, 0 inline scripts, in sitemap; 776 elements 0 contrast failures in both modes; image-plate specimens flex/flex-end, titles at 0.61-0.81 of plate height. Catalog note: expected cites brand.js, retired with the v2 build (ed10576) — the page ships no scripts; not a defect. | 2026-10-04: live: /brand/ 200, single h1, no skipped heading levels, 41 swatches / 115 demo nodes, 0 inline scripts (mode.js + Netlify RUM only), .demo-plate-body flex/flex-end (no F100 regression), in sitemap-0.xml, 0 console errors. brand.js retired (see 09-28 note).</t>
+          <t>PASS — live-verified 2026-08-10: /brand/ serves plates.css?v=phase15, matching every other surface; no second year-long cache entry. | 2026-09-01 re-verified live: /brand/ 200, single h1, no skipped heading levels, 0 contrast failures across 800 measured elements in dark mode. | 2026-09-22 re-verified live: /brand/ 200 in 0.48s; CSP style-src 'self' 'unsafe-inline' (scoped override intact); 0 inline &lt;script&gt; (mode.js + JSON-LD + Netlify RUM only); present in sitemap-0.xml; 680 text elements swept in dark mode, 0 contrast failures; image-plate specimens keep display:flex + justify-content:flex-end (no F100 regression). | 2026-09-28: live: /brand/ 200, scoped CSP style-src unsafe-inline, 0 inline scripts, in sitemap; 776 elements 0 contrast failures in both modes; image-plate specimens flex/flex-end, titles at 0.61-0.81 of plate height. Catalog note: expected cites brand.js, retired with the v2 build (ed10576) — the page ships no scripts; not a defect. | 2026-10-04: live: /brand/ 200, single h1, no skipped heading levels, 41 swatches / 115 demo nodes, 0 inline scripts (mode.js + Netlify RUM only), .demo-plate-body flex/flex-end (no F100 regression), in sitemap-0.xml, 0 console errors. brand.js retired (see 09-28 note). | 2026-10-05: live: /brand/ 200, style-src unsafe-inline scoped to it, in sitemap; sweep 0 failures dark; light-mode image-plate titles are the documented probe artifact (flex-end, titles in the bottom 52-93%).</t>
         </is>
       </c>
       <c r="I58" s="6" t="inlineStr"/>
@@ -3489,7 +3489,7 @@
       </c>
       <c r="H59" s="6" t="inlineStr">
         <is>
-          <t>PASS — GET /api/subscribe → 405 method_not_allowed | 2026-08-25 re-verified live: /api/subscribe reachable and behaving; rewrite chain intact. | 2026-08-27 re-verified live: GET /api/subscribe → 405 method_not_allowed. | 2026-09-06 re-verified live: GET /api/subscribe -&gt; 405. | 2026-09-11 re-verified live: GET /api/subscribe → 405 {'ok':false,'error':'method_not_allowed'}. | 2026-09-22 re-verified live: GET /api/subscribe -&gt; 405 {'ok':false,'error':'method_not_allowed'}; PUT -&gt; 405 likewise. | 2026-09-28: live: GET and PUT -&gt; 405 method_not_allowed. | 2026-10-04: live: GET /api/subscribe → 405 {ok:false,error:method_not_allowed}.</t>
+          <t>PASS — GET /api/subscribe → 405 method_not_allowed | 2026-08-25 re-verified live: /api/subscribe reachable and behaving; rewrite chain intact. | 2026-08-27 re-verified live: GET /api/subscribe → 405 method_not_allowed. | 2026-09-06 re-verified live: GET /api/subscribe -&gt; 405. | 2026-09-11 re-verified live: GET /api/subscribe → 405 {'ok':false,'error':'method_not_allowed'}. | 2026-09-22 re-verified live: GET /api/subscribe -&gt; 405 {'ok':false,'error':'method_not_allowed'}; PUT -&gt; 405 likewise. | 2026-09-28: live: GET and PUT -&gt; 405 method_not_allowed. | 2026-10-04: live: GET /api/subscribe → 405 {ok:false,error:method_not_allowed}. | 2026-10-05: live: GET -&gt; 405 method_not_allowed.</t>
         </is>
       </c>
       <c r="I59" s="6" t="inlineStr"/>
@@ -3542,7 +3542,7 @@
       </c>
       <c r="H60" s="6" t="inlineStr">
         <is>
-          <t>PASS — rate-limit bucket present (5/60s per IP) | 2026-09-11 re-verified live: burst of 8 POSTs from one IP: 400 invalid_email ×2 then 429 rate_limited ×6 — the 5/60s window fires as specified. | 2026-09-22 re-verified live: sequential burst of 10 POSTs (email=notanemail) from a quiet start returned exactly 5 x 400 invalid_email then 5 x 429 rate_limited — the 5/60s window fires as specified. A PARALLEL burst of 10 returned 10 x 400 and no 429: the window is a module-scope Map, so it is per Lambda instance and parallel requests fan out. Recorded as a measurement antipattern in QA-OS.md [F107]; not a defect. | 2026-09-28: live: SEQUENTIAL burst of 10 (email=notanemail) from a quiet start -&gt; exactly 5 x 400 then 5 x 429. | 2026-10-04: live: SEQUENTIAL burst of 10 × email=notanemail from a quiet start → exactly 400×5 then 429×5 (rate_limited), as specified.</t>
+          <t>PASS — rate-limit bucket present (5/60s per IP) | 2026-09-11 re-verified live: burst of 8 POSTs from one IP: 400 invalid_email ×2 then 429 rate_limited ×6 — the 5/60s window fires as specified. | 2026-09-22 re-verified live: sequential burst of 10 POSTs (email=notanemail) from a quiet start returned exactly 5 x 400 invalid_email then 5 x 429 rate_limited — the 5/60s window fires as specified. A PARALLEL burst of 10 returned 10 x 400 and no 429: the window is a module-scope Map, so it is per Lambda instance and parallel requests fan out. Recorded as a measurement antipattern in QA-OS.md [F107]; not a defect. | 2026-09-28: live: SEQUENTIAL burst of 10 (email=notanemail) from a quiet start -&gt; exactly 5 x 400 then 5 x 429. | 2026-10-04: live: SEQUENTIAL burst of 10 × email=notanemail from a quiet start → exactly 400×5 then 429×5 (rate_limited), as specified. | 2026-10-05: live: sequential burst of 10 from a quiet start -&gt; 400 x5 then 429 x5. (An earlier burst read 400 x3 then 429 x7 because the smoke + honeypot POSTs had already used 2 of the 5 slots on the warm instance — expected, not a failure.)</t>
         </is>
       </c>
       <c r="I60" s="6" t="inlineStr"/>
@@ -3595,7 +3595,7 @@
       </c>
       <c r="H61" s="6" t="inlineStr">
         <is>
-          <t>PASS — filled honeypot → 200 silent success, no Mailchimp write; field off-canvas (left:-5000px, tabindex -1, aria-hidden) | 2026-08-25 re-verified live: honeypot re-verified live: POST with website=spam returned HTTP 200 {"ok":true,"message":"subscribed"} — the intended silent drop, indistinguishable from success to a bot. | 2026-08-27 re-verified live: filled honeypot → 200 silent success. | 2026-09-06 re-verified live: filled honeypot (website=spam) -&gt; 200 {ok:true,message:'subscribed'} with no Mailchimp write (subscribe.cjs:67-69 short-circuits before the email is read). | 2026-09-11 re-verified live: POST with website=spam → 200 {'ok':true,'message':'subscribed'} and no Mailchimp call. Confirmed against subscribe.cjs:65-67 that this is the intended silent fake-success, NOT a bypass — the handler returns before the Mailchimp branch. | 2026-09-22 re-verified live: POST with website=http://spam.example -&gt; 200 {'ok':true,'message':'subscribed'}, the intended silent drop, no Mailchimp write. | 2026-09-28: live: filled honeypot -&gt; 200 {ok:true,message:subscribed}, silent. | 2026-10-04: live: POST with website filled → 200 {ok:true,message:subscribed} in 0.64s vs 2.15s for the real smoke subscribe — consistent with the short-circuit before Mailchimp.</t>
+          <t>PASS — filled honeypot → 200 silent success, no Mailchimp write; field off-canvas (left:-5000px, tabindex -1, aria-hidden) | 2026-08-25 re-verified live: honeypot re-verified live: POST with website=spam returned HTTP 200 {"ok":true,"message":"subscribed"} — the intended silent drop, indistinguishable from success to a bot. | 2026-08-27 re-verified live: filled honeypot → 200 silent success. | 2026-09-06 re-verified live: filled honeypot (website=spam) -&gt; 200 {ok:true,message:'subscribed'} with no Mailchimp write (subscribe.cjs:67-69 short-circuits before the email is read). | 2026-09-11 re-verified live: POST with website=spam → 200 {'ok':true,'message':'subscribed'} and no Mailchimp call. Confirmed against subscribe.cjs:65-67 that this is the intended silent fake-success, NOT a bypass — the handler returns before the Mailchimp branch. | 2026-09-22 re-verified live: POST with website=http://spam.example -&gt; 200 {'ok':true,'message':'subscribed'}, the intended silent drop, no Mailchimp write. | 2026-09-28: live: filled honeypot -&gt; 200 {ok:true,message:subscribed}, silent. | 2026-10-04: live: POST with website filled → 200 {ok:true,message:subscribed} in 0.64s vs 2.15s for the real smoke subscribe — consistent with the short-circuit before Mailchimp. | 2026-10-05: live: honeypot website=x -&gt; 200 subscribed in 0.42s (no Mailchimp call).</t>
         </is>
       </c>
       <c r="I61" s="6" t="inlineStr"/>
@@ -3648,7 +3648,7 @@
       </c>
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>PASS — invalid address → 400 invalid_email; plus-addressed valid address accepted (clients encode + as %2B via URLSearchParams(FormData)) | 2026-08-25 re-verified live: email validation re-verified live: POST email=notanemail returned HTTP 400 {"ok":false,"error":"invalid_email"}. | 2026-08-27 re-verified live: invalid address → 400 invalid_email. | 2026-09-06 re-verified live: email=notanemail -&gt; 400 {ok:false,error:'invalid_email'}. | 2026-09-11 re-verified live: POST email=notanemail → 400 {'ok':false,'error':'invalid_email'}. | 2026-09-22 re-verified live: email=not-an-email -&gt; 400 {'ok':false,'error':'invalid_email'}; %2B-encoded plus address accepted on the same run. | 2026-09-28: live: notanemail -&gt; 400 invalid_email, Cache-Control no-store.</t>
+          <t>PASS — invalid address → 400 invalid_email; plus-addressed valid address accepted (clients encode + as %2B via URLSearchParams(FormData)) | 2026-08-25 re-verified live: email validation re-verified live: POST email=notanemail returned HTTP 400 {"ok":false,"error":"invalid_email"}. | 2026-08-27 re-verified live: invalid address → 400 invalid_email. | 2026-09-06 re-verified live: email=notanemail -&gt; 400 {ok:false,error:'invalid_email'}. | 2026-09-11 re-verified live: POST email=notanemail → 400 {'ok':false,'error':'invalid_email'}. | 2026-09-22 re-verified live: email=not-an-email -&gt; 400 {'ok':false,'error':'invalid_email'}; %2B-encoded plus address accepted on the same run. | 2026-09-28: live: notanemail -&gt; 400 invalid_email, Cache-Control no-store. | 2026-10-05: live: email=notanemail -&gt; 400 invalid_email.</t>
         </is>
       </c>
       <c r="I62" s="6" t="inlineStr"/>
@@ -3701,7 +3701,7 @@
       </c>
       <c r="H63" s="6" t="inlineStr">
         <is>
-          <t>PASS — healthscrub+20260807@imjustdex.com → 200 subscribed in 1.53s | 2026-08-13 re-verified live: live smoke test POST /api/subscribe returned HTTP 200 {"ok":true,"message":"subscribed"} in 2.16s using healthscrub+20260813@imjustdex.com. | 2026-08-16 re-verified live: live smoke test POST /api/subscribe returned HTTP 200 {"ok":true,"message":"subscribed"} in 2.05s using healthscrub+20260816@imjustdex.com. | 2026-08-25 re-verified live: smoke POST with healthscrub+20260825@imjustdex.com returned HTTP 200 {"ok":true,"message":"subscribed"} in 2.20s. | 2026-08-27 re-verified live: healthscrub+20260827@imjustdex.com → 200 subscribed. | 2026-09-06 re-verified live: POST healthscrub%2B20260906%40imjustdex.com -&gt; 200 {ok:true,message:'subscribed'} in 1.77s. | 2026-09-11 re-verified live: first POST of healthscrub+20260911@imjustdex.com → 200 'subscribed'; immediate repeat → 200 'already_subscribed'. Member-exists path intact. | 2026-09-22 re-verified live: BOTH branches exercised — first POST of healthscrub+20260922@imjustdex.com -&gt; 200 {'message':'subscribed'} in 1.81s; immediate re-POST of the same address -&gt; 200 {'message':'already_subscribed'}. | 2026-09-28: live: healthscrub+20260928@imjustdex.com -&gt; 200 subscribed (1.32s); repeat -&gt; 200 already_subscribed.</t>
+          <t>PASS — healthscrub+20260807@imjustdex.com → 200 subscribed in 1.53s | 2026-08-13 re-verified live: live smoke test POST /api/subscribe returned HTTP 200 {"ok":true,"message":"subscribed"} in 2.16s using healthscrub+20260813@imjustdex.com. | 2026-08-16 re-verified live: live smoke test POST /api/subscribe returned HTTP 200 {"ok":true,"message":"subscribed"} in 2.05s using healthscrub+20260816@imjustdex.com. | 2026-08-25 re-verified live: smoke POST with healthscrub+20260825@imjustdex.com returned HTTP 200 {"ok":true,"message":"subscribed"} in 2.20s. | 2026-08-27 re-verified live: healthscrub+20260827@imjustdex.com → 200 subscribed. | 2026-09-06 re-verified live: POST healthscrub%2B20260906%40imjustdex.com -&gt; 200 {ok:true,message:'subscribed'} in 1.77s. | 2026-09-11 re-verified live: first POST of healthscrub+20260911@imjustdex.com → 200 'subscribed'; immediate repeat → 200 'already_subscribed'. Member-exists path intact. | 2026-09-22 re-verified live: BOTH branches exercised — first POST of healthscrub+20260922@imjustdex.com -&gt; 200 {'message':'subscribed'} in 1.81s; immediate re-POST of the same address -&gt; 200 {'message':'already_subscribed'}. | 2026-09-28: live: healthscrub+20260928@imjustdex.com -&gt; 200 subscribed (1.32s); repeat -&gt; 200 already_subscribed. | 2026-10-05: live: healthscrub+20261005@imjustdex.com -&gt; 200 {"ok":true,"message":"subscribed"} in 1.19s.</t>
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr"/>
@@ -3754,7 +3754,7 @@
       </c>
       <c r="H64" s="6" t="inlineStr">
         <is>
-          <t>PASS — source field present on all 4 surfaces (home/article/coming-soon/phase0) | 2026-09-06 re-verified live: source=healthscrub accepted on the 200 above. | 2026-09-19 re-verified live: subscribe smoke (healthscrub+20260919@imjustdex.com, source=healthscrub, %2B-encoded) → 200 {"ok":true,"message":"subscribed"} in 1.77s. | 2026-09-22 re-verified live: source=healthscrub accepted on the 200 above; merge-field/tag write is best-effort server-side and not observable without the Mailchimp dashboard (outside repo). | 2026-09-28: live: source field on home (home), article (article), phase0 (phase0); fixture coming-soon (coming-soon).</t>
+          <t>PASS — source field present on all 4 surfaces (home/article/coming-soon/phase0) | 2026-09-06 re-verified live: source=healthscrub accepted on the 200 above. | 2026-09-19 re-verified live: subscribe smoke (healthscrub+20260919@imjustdex.com, source=healthscrub, %2B-encoded) → 200 {"ok":true,"message":"subscribed"} in 1.77s. | 2026-09-22 re-verified live: source=healthscrub accepted on the 200 above; merge-field/tag write is best-effort server-side and not observable without the Mailchimp dashboard (outside repo). | 2026-09-28: live: source field on home (home), article (article), phase0 (phase0); fixture coming-soon (coming-soon). | 2026-10-05: carried: subscribe.cjs unchanged on origin/main; source tagging not observable without the Mailchimp dashboard.</t>
         </is>
       </c>
       <c r="I64" s="6" t="inlineStr"/>
@@ -3807,7 +3807,7 @@
       </c>
       <c r="H65" s="6" t="inlineStr">
         <is>
-          <t>PASS — documented error envelope returned, no stack leakage | 2026-09-18 re-verified live: POST email=not-an-email returns 400 {"ok":false,"error":"invalid_email"} with Cache-Control: no-store, no stack leakage. Config/upstream branches not forceable from outside (would need env or Mailchimp changes); subscribe.cjs unchanged since last PASS. | 2026-09-22 re-verified live: 400 invalid_email returns Cache-Control: no-store with no stack leakage. Config/upstream branches still not forceable from outside (needs env or Mailchimp changes); subscribe.cjs unchanged since last PASS. | 2026-09-28: carried: JSON no-store envelope confirmed on 400/405/429; config/upstream failures not inducible live.</t>
+          <t>PASS — documented error envelope returned, no stack leakage | 2026-09-18 re-verified live: POST email=not-an-email returns 400 {"ok":false,"error":"invalid_email"} with Cache-Control: no-store, no stack leakage. Config/upstream branches not forceable from outside (would need env or Mailchimp changes); subscribe.cjs unchanged since last PASS. | 2026-09-22 re-verified live: 400 invalid_email returns Cache-Control: no-store with no stack leakage. Config/upstream branches still not forceable from outside (needs env or Mailchimp changes); subscribe.cjs unchanged since last PASS. | 2026-09-28: carried: JSON no-store envelope confirmed on 400/405/429; config/upstream failures not inducible live. | 2026-10-05: live: responses are JSON with Cache-Control no-store.</t>
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr"/>
@@ -3860,7 +3860,7 @@
       </c>
       <c r="H66" s="6" t="inlineStr">
         <is>
-          <t>N/A — retired by owner decision 2026-08-07 | 2026-09-22: still retired by owner decision — dxjakes.com not probed, netlify.toml carries no dxjakes rules.</t>
+          <t>N/A — retired by owner decision 2026-08-07 | 2026-09-22: still retired by owner decision — dxjakes.com not probed, netlify.toml carries no dxjakes rules. | 2026-10-05: still N/A (dxjakes.com out of scope, not probed).</t>
         </is>
       </c>
       <c r="I66" s="6" t="inlineStr"/>
@@ -3913,7 +3913,7 @@
       </c>
       <c r="H67" s="6" t="inlineStr">
         <is>
-          <t>PASS — /about, /phase0 and all 16 /words/&lt;slug&gt; → single 301 to trailing-slash canonical | 2026-08-13 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200; /sitemap.xml correctly 404 post-cutover. | 2026-08-16 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200 and /words/the-stone -&gt; 301 -&gt; /words/the-stone/ re-verified live; /sitemap.xml correctly 404 post-cutover; /words -&gt; 301 home; /opsmeeting -&gt; 301 home. | 2026-08-25 re-verified live: /about, /brand, /phase0 and /words/the-stone each return a single 301 to the trailing-slash form, which returns 200. No loops. | 2026-08-27 re-verified live: /about and /words/the-stone → single 301 to the trailing-slash canonical. | 2026-09-01 re-verified live: /about -&gt; 301 -&gt; https://imjustdex.com/about/ -&gt; 200. | 2026-09-06 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200. | 2026-09-11 re-verified live: /about, /brand, /phase0 and /words/the-stone all 301 → their trailing-slash canonical → 200. | 2026-09-22 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200 and /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200; /sitemap.xml correctly 404 post-cutover; /DESIGN-SYSTEM.md correctly 404. | 2026-09-28: live: 21/21 non-slash routes 301 to their slash canonical (about, phase0, /words, /words/, 17 essays).</t>
+          <t>PASS — /about, /phase0 and all 16 /words/&lt;slug&gt; → single 301 to trailing-slash canonical | 2026-08-13 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200; /sitemap.xml correctly 404 post-cutover. | 2026-08-16 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200 and /words/the-stone -&gt; 301 -&gt; /words/the-stone/ re-verified live; /sitemap.xml correctly 404 post-cutover; /words -&gt; 301 home; /opsmeeting -&gt; 301 home. | 2026-08-25 re-verified live: /about, /brand, /phase0 and /words/the-stone each return a single 301 to the trailing-slash form, which returns 200. No loops. | 2026-08-27 re-verified live: /about and /words/the-stone → single 301 to the trailing-slash canonical. | 2026-09-01 re-verified live: /about -&gt; 301 -&gt; https://imjustdex.com/about/ -&gt; 200. | 2026-09-06 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200. | 2026-09-11 re-verified live: /about, /brand, /phase0 and /words/the-stone all 301 → their trailing-slash canonical → 200. | 2026-09-22 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200 and /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200; /sitemap.xml correctly 404 post-cutover; /DESIGN-SYSTEM.md correctly 404. | 2026-09-28: live: 21/21 non-slash routes 301 to their slash canonical (about, phase0, /words, /words/, 17 essays). | 2026-10-05: live: /about, /phase0 and all 17 /words/&lt;slug&gt; -&gt; 301 to the slashed form.</t>
         </is>
       </c>
       <c r="I67" s="6" t="inlineStr"/>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="H68" s="6" t="inlineStr">
         <is>
-          <t>PASS — /words and /words/ → 301 home | 2026-08-27 re-verified live: /words → 301 home. | 2026-09-11 re-verified live: /words and /words/ both 301 → https://imjustdex.com/. | 2026-09-23 re-verified live: /words and /words/ both single 301 -&gt; /. | 2026-09-28: live: /words and /words/ -&gt; 301 /.</t>
+          <t>PASS — /words and /words/ → 301 home | 2026-08-27 re-verified live: /words → 301 home. | 2026-09-11 re-verified live: /words and /words/ both 301 → https://imjustdex.com/. | 2026-09-23 re-verified live: /words and /words/ both single 301 -&gt; /. | 2026-09-28: live: /words and /words/ -&gt; 301 /. | 2026-10-05: live: /words and /words/ -&gt; 301 /.</t>
         </is>
       </c>
       <c r="I68" s="6" t="inlineStr"/>
@@ -4019,7 +4019,7 @@
       </c>
       <c r="H69" s="6" t="inlineStr">
         <is>
-          <t>PASS — /opsmeeting, /leadership-prep, /asana-workflow (+ /*) all → 301 home | 2026-08-27 re-verified live: /opsmeeting → 301 home. | 2026-09-11 re-verified live: /opsmeeting, /leadership-prep, /asana-workflow and a deep path under each all 301 → https://imjustdex.com/. | 2026-09-23 re-verified live: /opsmeeting, /leadership-prep, /asana-workflow and /opsmeeting/deep/x all single 301 -&gt; /. | 2026-09-28: live: /opsmeeting, /opsmeeting/x, /leadership-prep/y, /asana-workflow, /asana-workflow/z -&gt; 301 /.</t>
+          <t>PASS — /opsmeeting, /leadership-prep, /asana-workflow (+ /*) all → 301 home | 2026-08-27 re-verified live: /opsmeeting → 301 home. | 2026-09-11 re-verified live: /opsmeeting, /leadership-prep, /asana-workflow and a deep path under each all 301 → https://imjustdex.com/. | 2026-09-23 re-verified live: /opsmeeting, /leadership-prep, /asana-workflow and /opsmeeting/deep/x all single 301 -&gt; /. | 2026-09-28: live: /opsmeeting, /opsmeeting/x, /leadership-prep/y, /asana-workflow, /asana-workflow/z -&gt; 301 /. | 2026-10-05: live: /opsmeeting, /opsmeeting/x, /leadership-prep, /asana-workflow/x -&gt; 301 /.</t>
         </is>
       </c>
       <c r="I69" s="6" t="inlineStr"/>
@@ -4072,7 +4072,7 @@
       </c>
       <c r="H70" s="6" t="inlineStr">
         <is>
-          <t>PASS — /api/subscribe rewrite reaches the function (405 on GET, 400/200 on POST) | 2026-08-13 re-verified live: /api/subscribe rewrite reached the Netlify function and returned a Mailchimp success body. | 2026-08-25 re-verified live: /api/subscribe rewrite to the Netlify function verified by the live smoke POST. | 2026-08-27 re-verified live: /api/subscribe rewrite reaches the function. | 2026-09-01 re-verified live: POST to /api/subscribe rewrote to the Netlify function and returned 200. | 2026-09-11 re-verified live: /api/subscribe rewrite live — POST reaches the function and returns its JSON envelope. | 2026-09-23 re-verified live: /api/subscribe rewrite reaches the function — GET 405, POST (healthscrub+20260923@imjustdex.com, %2B-encoded) 200 {"ok":true,"message":"subscribed"} in 2.05s. | 2026-09-28: live: POST /api/subscribe reaches the function (200/400/429 bodies).</t>
+          <t>PASS — /api/subscribe rewrite reaches the function (405 on GET, 400/200 on POST) | 2026-08-13 re-verified live: /api/subscribe rewrite reached the Netlify function and returned a Mailchimp success body. | 2026-08-25 re-verified live: /api/subscribe rewrite to the Netlify function verified by the live smoke POST. | 2026-08-27 re-verified live: /api/subscribe rewrite reaches the function. | 2026-09-01 re-verified live: POST to /api/subscribe rewrote to the Netlify function and returned 200. | 2026-09-11 re-verified live: /api/subscribe rewrite live — POST reaches the function and returns its JSON envelope. | 2026-09-23 re-verified live: /api/subscribe rewrite reaches the function — GET 405, POST (healthscrub+20260923@imjustdex.com, %2B-encoded) 200 {"ok":true,"message":"subscribed"} in 2.05s. | 2026-09-28: live: POST /api/subscribe reaches the function (200/400/429 bodies). | 2026-10-05: live: /api/subscribe answers as the function (405/200/400/429), not a redirect.</t>
         </is>
       </c>
       <c r="I70" s="6" t="inlineStr"/>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="H71" s="6" t="inlineStr">
         <is>
-          <t>PASS — unmatched route → 404 with the branded body | 2026-08-13 re-verified live: /404 returns 200 with the bespoke 'Nothing to Document Here' body and noindex; /DESIGN-SYSTEM.md and /audit/features.json both 404 (docs not leaking). | 2026-08-25 re-verified live: /404 returns HTTP 200 with the bespoke notfound-plate body and meta robots noindex. | 2026-08-27 re-verified live: unmatched route → 404 with the branded body. | 2026-09-06 re-verified live: /nonexistent-page-qa-test -&gt; 404; /sitemap.xml and /DESIGN-SYSTEM.md both correctly 404. | 2026-09-11 re-verified live: /DESIGN-SYSTEM.md → 404 and /sitemap.xml → 404; /404 serves the bespoke body at HTTP 200 with noindex,nofollow. | 2026-09-23 re-verified live: /no-such-page-qa -&gt; 404 with the 'Nothing to Document Here' body; /DESIGN-SYSTEM.md, /audit/features.json and /sitemap.xml all 404. | 2026-09-28: live: /this-route-does-not-exist-qa -&gt; 404 bespoke body.</t>
+          <t>PASS — unmatched route → 404 with the branded body | 2026-08-13 re-verified live: /404 returns 200 with the bespoke 'Nothing to Document Here' body and noindex; /DESIGN-SYSTEM.md and /audit/features.json both 404 (docs not leaking). | 2026-08-25 re-verified live: /404 returns HTTP 200 with the bespoke notfound-plate body and meta robots noindex. | 2026-08-27 re-verified live: unmatched route → 404 with the branded body. | 2026-09-06 re-verified live: /nonexistent-page-qa-test -&gt; 404; /sitemap.xml and /DESIGN-SYSTEM.md both correctly 404. | 2026-09-11 re-verified live: /DESIGN-SYSTEM.md → 404 and /sitemap.xml → 404; /404 serves the bespoke body at HTTP 200 with noindex,nofollow. | 2026-09-23 re-verified live: /no-such-page-qa -&gt; 404 with the 'Nothing to Document Here' body; /DESIGN-SYSTEM.md, /audit/features.json and /sitemap.xml all 404. | 2026-09-28: live: /this-route-does-not-exist-qa -&gt; 404 bespoke body. | 2026-10-05: live: unmatched route -&gt; 404 bespoke body; /sitemap.xml and /DESIGN-SYSTEM.md 404.</t>
         </is>
       </c>
       <c r="I71" s="6" t="inlineStr"/>
@@ -4178,7 +4178,7 @@
       </c>
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>PASS — CSP present and strict on every page; per-route /brand/ + /feed.xml overrides intact; 0 inline &lt;style&gt; in built Astro HTML | 2026-08-13 re-verified live: CSP header present and ENFORCING — a runtime &lt;style&gt; injection was blocked by style-src 'self' during F77 verification, which is direct proof the policy is live, not just declared. Per-route /brand/ and /feed.xml relaxations by design. | 2026-08-16 re-verified live: CSP present and strict on every page type; /brand/ and /feed.xml keep their by-design style-src 'unsafe-inline' relaxation. Zero inline &lt;style&gt; blocks in any built Astro page (home 0, article 0, about 0, phase0 0). Policy proven live again this run — a &lt;style&gt; injection was blocked, while CSSOM mutation of the already-loaded sheet succeeded, which is the documented distinction. | 2026-08-25 re-verified live: CSP present on every route and empirically ENFORCED — an injected inline &lt;style&gt; during this run was blocked by style-src 'self' and logged as the only console error of the whole scrub. Per-route relaxation for /brand/ (style-src adds 'unsafe-inline') confirmed by design. Zero inline &lt;style&gt; blocks in any built page. | 2026-08-27 re-verified live: CSP present and strict on / and on an article. | 2026-09-01 re-verified live: CSP present and identical on / and /words/&lt;slug&gt;/ — default-src 'self'; script-src 'self'; style-src 'self'; img-src 'self' data: https:; font-src 'self'; connect-src 'self'; frame-ancestors 'none'; base-uri 'self'; form-action 'self'; object-src 'none'; upgrade-insecure-requests. Zero inline &lt;style&gt; blocks in any built or served page (CSP would block them). | 2026-09-06 re-verified live: CSP present on all 7 sampled routes, with the by-design 'unsafe-inline' style-src relaxation only on /brand/ and /feed.xml. Zero inline &lt;style&gt; blocks in any built page. | 2026-09-11 re-verified live: CSP served on every route: default-src 'self'; script-src 'self'; style-src 'self'; frame-ancestors 'none'; object-src 'none'; upgrade-insecure-requests. Zero inline &lt;style&gt; tags in any built or served page. | 2026-09-23 re-verified live: CSP present on all 7 sampled routes (connect-src still allows the RUM collector); zero inline &lt;style&gt; in built HTML across home/about/404/17 articles; 0 console errors on 6 surfaces. | 2026-09-28: live: CSP on every HTML route + feed; 0 inline scripts on 5 types; connect-src carries the RUM collector.</t>
+          <t>PASS — CSP present and strict on every page; per-route /brand/ + /feed.xml overrides intact; 0 inline &lt;style&gt; in built Astro HTML | 2026-08-13 re-verified live: CSP header present and ENFORCING — a runtime &lt;style&gt; injection was blocked by style-src 'self' during F77 verification, which is direct proof the policy is live, not just declared. Per-route /brand/ and /feed.xml relaxations by design. | 2026-08-16 re-verified live: CSP present and strict on every page type; /brand/ and /feed.xml keep their by-design style-src 'unsafe-inline' relaxation. Zero inline &lt;style&gt; blocks in any built Astro page (home 0, article 0, about 0, phase0 0). Policy proven live again this run — a &lt;style&gt; injection was blocked, while CSSOM mutation of the already-loaded sheet succeeded, which is the documented distinction. | 2026-08-25 re-verified live: CSP present on every route and empirically ENFORCED — an injected inline &lt;style&gt; during this run was blocked by style-src 'self' and logged as the only console error of the whole scrub. Per-route relaxation for /brand/ (style-src adds 'unsafe-inline') confirmed by design. Zero inline &lt;style&gt; blocks in any built page. | 2026-08-27 re-verified live: CSP present and strict on / and on an article. | 2026-09-01 re-verified live: CSP present and identical on / and /words/&lt;slug&gt;/ — default-src 'self'; script-src 'self'; style-src 'self'; img-src 'self' data: https:; font-src 'self'; connect-src 'self'; frame-ancestors 'none'; base-uri 'self'; form-action 'self'; object-src 'none'; upgrade-insecure-requests. Zero inline &lt;style&gt; blocks in any built or served page (CSP would block them). | 2026-09-06 re-verified live: CSP present on all 7 sampled routes, with the by-design 'unsafe-inline' style-src relaxation only on /brand/ and /feed.xml. Zero inline &lt;style&gt; blocks in any built page. | 2026-09-11 re-verified live: CSP served on every route: default-src 'self'; script-src 'self'; style-src 'self'; frame-ancestors 'none'; object-src 'none'; upgrade-insecure-requests. Zero inline &lt;style&gt; tags in any built or served page. | 2026-09-23 re-verified live: CSP present on all 7 sampled routes (connect-src still allows the RUM collector); zero inline &lt;style&gt; in built HTML across home/about/404/17 articles; 0 console errors on 6 surfaces. | 2026-09-28: live: CSP on every HTML route + feed; 0 inline scripts on 5 types; connect-src carries the RUM collector. | 2026-10-05: live: global CSP self-only + RUM collector in connect-src; /brand/ + /feed.xml relax style-src; 0 inline &lt;style&gt; in built HTML.</t>
         </is>
       </c>
       <c r="I72" s="6" t="inlineStr"/>
@@ -4231,7 +4231,7 @@
       </c>
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>PASS — X-Frame DENY, nosniff, HSTS max-age=31536000 includeSubDomains preload, Referrer-Policy, Permissions-Policy, COOP, CORP on all 21 routes | 2026-08-13 re-verified live: all 5 security headers present on all 6 page types (home, article, about, brand, phase0, 404, feed): X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000 includeSubDomains preload, CSP, Referrer-Policy strict-origin-when-cross-origin. Permissions-Policy also present. | 2026-08-16 re-verified live: all security headers re-verified live on home/article/brand/404/feed: X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000 includeSubDomains preload, CSP, Referrer-Policy strict-origin-when-cross-origin, Permissions-Policy, COOP same-origin, CORP same-origin. | 2026-08-25 re-verified live: all five headers present on / and on an article: X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000; includeSubDomains; preload, CSP, Referrer-Policy strict-origin-when-cross-origin. Permissions-Policy also present on /. | 2026-08-27 re-verified live: X-Frame DENY, nosniff, HSTS max-age=31536000 includeSubDomains preload, Referrer-Policy all present. | 2026-09-01 re-verified live: X-Frame-Options DENY, X-Content-Type-Options nosniff, Strict-Transport-Security max-age=31536000; includeSubDomains; preload, Referrer-Policy strict-origin-when-cross-origin — all present on / and on an article. | 2026-09-06 re-verified live: X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000; includeSubDomains; preload, Referrer-Policy strict-origin-when-cross-origin, Permissions-Policy - all 7 routes. | 2026-09-11 re-verified live: 5/5 security headers on /, /about/, /brand/, /words/the-stone/, /404 and /feed.xml; HSTS max-age=31536000; includeSubDomains; preload. | 2026-09-23 re-verified live: X-Frame-Options DENY, nosniff, HSTS max-age=31536000 includeSubDomains preload, CSP, Referrer-Policy on /, /about/, /brand/, /phase0/, /404, an article and /feed.xml. | 2026-09-28: live: XFO DENY, nosniff, HSTS 1y includeSubDomains preload, Referrer-Policy strict-origin-when-cross-origin, Permissions-Policy, COOP/CORP same-origin.</t>
+          <t>PASS — X-Frame DENY, nosniff, HSTS max-age=31536000 includeSubDomains preload, Referrer-Policy, Permissions-Policy, COOP, CORP on all 21 routes | 2026-08-13 re-verified live: all 5 security headers present on all 6 page types (home, article, about, brand, phase0, 404, feed): X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000 includeSubDomains preload, CSP, Referrer-Policy strict-origin-when-cross-origin. Permissions-Policy also present. | 2026-08-16 re-verified live: all security headers re-verified live on home/article/brand/404/feed: X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000 includeSubDomains preload, CSP, Referrer-Policy strict-origin-when-cross-origin, Permissions-Policy, COOP same-origin, CORP same-origin. | 2026-08-25 re-verified live: all five headers present on / and on an article: X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000; includeSubDomains; preload, CSP, Referrer-Policy strict-origin-when-cross-origin. Permissions-Policy also present on /. | 2026-08-27 re-verified live: X-Frame DENY, nosniff, HSTS max-age=31536000 includeSubDomains preload, Referrer-Policy all present. | 2026-09-01 re-verified live: X-Frame-Options DENY, X-Content-Type-Options nosniff, Strict-Transport-Security max-age=31536000; includeSubDomains; preload, Referrer-Policy strict-origin-when-cross-origin — all present on / and on an article. | 2026-09-06 re-verified live: X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000; includeSubDomains; preload, Referrer-Policy strict-origin-when-cross-origin, Permissions-Policy - all 7 routes. | 2026-09-11 re-verified live: 5/5 security headers on /, /about/, /brand/, /words/the-stone/, /404 and /feed.xml; HSTS max-age=31536000; includeSubDomains; preload. | 2026-09-23 re-verified live: X-Frame-Options DENY, nosniff, HSTS max-age=31536000 includeSubDomains preload, CSP, Referrer-Policy on /, /about/, /brand/, /phase0/, /404, an article and /feed.xml. | 2026-09-28: live: XFO DENY, nosniff, HSTS 1y includeSubDomains preload, Referrer-Policy strict-origin-when-cross-origin, Permissions-Policy, COOP/CORP same-origin. | 2026-10-05: live: XFO DENY, nosniff, Referrer-Policy, Permissions-Policy, HSTS 1yr includeSubDomains preload, COOP/CORP same-origin on every HTML route + feed.</t>
         </is>
       </c>
       <c r="I73" s="6" t="inlineStr"/>
@@ -4284,7 +4284,7 @@
       </c>
       <c r="H74" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: /brand/brand.css?v=brand5 and /img/* both return public,max-age=31536000,immutable; HTML remains public,max-age=0,must-revalidate. | 2026-08-13 re-verified live: versioned assets (/css, /js, /img) all serve public,max-age=31536000,immutable; HTML serves public,max-age=0,must-revalidate. No drift. | 2026-08-16 re-verified live: versioned assets (/css, /js, /img, /fonts) all serve public,max-age=31536000,immutable; HTML serves public,max-age=0,must-revalidate. No drift. | 2026-08-25 re-verified live: versioned CSS, fonts and images all serve public,max-age=31536000,immutable; HTML serves public,max-age=0,must-revalidate. No drift on either tier. | 2026-08-27 re-verified live: HTML no-cache/must-revalidate; /css/*?v= and /img/* both public,max-age=31536000,immutable. | 2026-09-01 re-verified live: /css/tokens.css?v=phase24 and /fonts/Anton-Regular.woff2 both return public,max-age=31536000,immutable; HTML returns public,max-age=0,must-revalidate. No drift on either pattern. | 2026-09-06 re-verified live: HTML public,max-age=0,must-revalidate; /css, /fonts, /img, /js and /_astro all public,max-age=31536000,immutable. | 2026-09-11 re-verified live: versioned css/js/font/img all public,max-age=31536000,immutable; HTML public,max-age=0,must-revalidate. No drift. | 2026-09-23 re-verified live: 20 versioned /css /js /fonts /img /_astro assets all public,max-age=31536000,immutable; HTML public,max-age=0,must-revalidate. | 2026-09-28: live: 47 versioned assets public,max-age=31536000,immutable; fonts ACAO *; HTML + feed public,max-age=0,must-revalidate.</t>
+          <t>PASS — live-verified 2026-08-10: /brand/brand.css?v=brand5 and /img/* both return public,max-age=31536000,immutable; HTML remains public,max-age=0,must-revalidate. | 2026-08-13 re-verified live: versioned assets (/css, /js, /img) all serve public,max-age=31536000,immutable; HTML serves public,max-age=0,must-revalidate. No drift. | 2026-08-16 re-verified live: versioned assets (/css, /js, /img, /fonts) all serve public,max-age=31536000,immutable; HTML serves public,max-age=0,must-revalidate. No drift. | 2026-08-25 re-verified live: versioned CSS, fonts and images all serve public,max-age=31536000,immutable; HTML serves public,max-age=0,must-revalidate. No drift on either tier. | 2026-08-27 re-verified live: HTML no-cache/must-revalidate; /css/*?v= and /img/* both public,max-age=31536000,immutable. | 2026-09-01 re-verified live: /css/tokens.css?v=phase24 and /fonts/Anton-Regular.woff2 both return public,max-age=31536000,immutable; HTML returns public,max-age=0,must-revalidate. No drift on either pattern. | 2026-09-06 re-verified live: HTML public,max-age=0,must-revalidate; /css, /fonts, /img, /js and /_astro all public,max-age=31536000,immutable. | 2026-09-11 re-verified live: versioned css/js/font/img all public,max-age=31536000,immutable; HTML public,max-age=0,must-revalidate. No drift. | 2026-09-23 re-verified live: 20 versioned /css /js /fonts /img /_astro assets all public,max-age=31536000,immutable; HTML public,max-age=0,must-revalidate. | 2026-09-28: live: 47 versioned assets public,max-age=31536000,immutable; fonts ACAO *; HTML + feed public,max-age=0,must-revalidate. | 2026-10-05: live: 47 assets 200 with public,max-age=31536000,immutable; HTML public,max-age=0,must-revalidate; fonts ACAO *.</t>
         </is>
       </c>
       <c r="I74" s="6" t="inlineStr"/>
@@ -4337,7 +4337,7 @@
       </c>
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>PASS — predicate gates homepage/feed/sitemap/routes consistently; 16 published, 0 upcoming | 2026-09-18 re-verified live: 17 published, 0 upcoming — homepage 17 plates, feed 17 entries, sitemap 17 /words/ URLs, all consistent. (An untracked drafted entry sits in the working tree and is correctly nowhere live.) | 2026-09-23 re-verified live: 17 published, 0 upcoming — homepage 17 plates, feed 17 entries, sitemap 17 /words/ URLs (21 locs), all set-equal. | 2026-09-28: live: 17/17 published + past-dated all live; fixture build: future-dated entry out of cascade/feed/sitemap, ghost plate shown, coming-soon page built.</t>
+          <t>PASS — predicate gates homepage/feed/sitemap/routes consistently; 16 published, 0 upcoming | 2026-09-18 re-verified live: 17 published, 0 upcoming — homepage 17 plates, feed 17 entries, sitemap 17 /words/ URLs, all consistent. (An untracked drafted entry sits in the working tree and is correctly nowhere live.) | 2026-09-23 re-verified live: 17 published, 0 upcoming — homepage 17 plates, feed 17 entries, sitemap 17 /words/ URLs (21 locs), all set-equal. | 2026-09-28: live: 17/17 published + past-dated all live; fixture build: future-dated entry out of cascade/feed/sitemap, ghost plate shown, coming-soon page built. | 2026-10-05: repo: index/feed/sitemap/routes all consume isPubliclyLiveData/isUpcomingData from src/utils/published.mjs; fixture build gated the future entry everywhere.</t>
         </is>
       </c>
       <c r="I75" s="6" t="inlineStr"/>
@@ -4390,7 +4390,7 @@
       </c>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>PASS — 2026-09-22 live-verified: GitHub Actions 'Daily rebuild' has 40 runs across 40 distinct days (2026-08-14 -&gt; 2026-09-22), zero missing-day gaps, all conclusion=success. Today's fired 09:51:20Z and produced the live Netlify deploy 6ab24fa0 (published 09:51:43Z, commit 95e2a73). The single 2026-08-27 miss that opened this row has not recurred in the 26 days since. | 2026-09-23 re-verified live: Daily rebuild fired 09:52:35Z (success) and produced Netlify deploy 6ab3a167 on 95e2a73 — 41 consecutive days. | 2026-09-28: live: Daily rebuild succeeded 09-25/26/27; latest ready deploy 95e2a73 at 2026-09-27 10:29Z == GitHub main.</t>
+          <t>PASS — 2026-09-22 live-verified: GitHub Actions 'Daily rebuild' has 40 runs across 40 distinct days (2026-08-14 -&gt; 2026-09-22), zero missing-day gaps, all conclusion=success. Today's fired 09:51:20Z and produced the live Netlify deploy 6ab24fa0 (published 09:51:43Z, commit 95e2a73). The single 2026-08-27 miss that opened this row has not recurred in the 26 days since. | 2026-09-23 re-verified live: Daily rebuild fired 09:52:35Z (success) and produced Netlify deploy 6ab3a167 on 95e2a73 — 41 consecutive days. | 2026-09-28: live: Daily rebuild succeeded 09-25/26/27; latest ready deploy 95e2a73 at 2026-09-27 10:29Z == GitHub main. | 2026-10-05: live: Daily rebuild Action succeeded every day 09-29..10-04 (GitHub fires it 10:20-11:30Z); Netlify ready deploy 5129f69 built 2026-10-04 11:04Z by hook. Today's run had not fired yet at scrub time — normal GitHub cron lag.</t>
         </is>
       </c>
       <c r="I76" s="6" t="inlineStr"/>
@@ -4443,7 +4443,7 @@
       </c>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>PASS — scripts/og-plate.mjs present; all 19 OG plates render and 200 | 2026-08-27 re-verified live: all 21 OG plates 200. | 2026-09-01 re-verified live: every one of the 17 per-article OG plates resolves 200 at its cache-busted path; none falls back to og-default.png. | 2026-09-19 re-verified live: 17/17 per-article OG plates 200 at their cache-busted paths; JSON-LD image == og:image on all 17; none falls back to og-default.png. | 2026-09-23 re-verified live: all 21 og:image URLs (17 per-article + home/about/brand/phase0) 200; every BlogPosting image == og:image, og-&lt;slug&gt;.png?v=phaseNN, no og-default drift. | 2026-09-28: live: og-&lt;slug&gt;.png 200 for 17/17; generator source unchanged.</t>
+          <t>PASS — scripts/og-plate.mjs present; all 19 OG plates render and 200 | 2026-08-27 re-verified live: all 21 OG plates 200. | 2026-09-01 re-verified live: every one of the 17 per-article OG plates resolves 200 at its cache-busted path; none falls back to og-default.png. | 2026-09-19 re-verified live: 17/17 per-article OG plates 200 at their cache-busted paths; JSON-LD image == og:image on all 17; none falls back to og-default.png. | 2026-09-23 re-verified live: all 21 og:image URLs (17 per-article + home/about/brand/phase0) 200; every BlogPosting image == og:image, og-&lt;slug&gt;.png?v=phaseNN, no og-default drift. | 2026-09-28: live: og-&lt;slug&gt;.png 200 for 17/17; generator source unchanged. | 2026-10-05: repo: scripts/og-plate.mjs present; 17/17 og-&lt;slug&gt;.png 200.</t>
         </is>
       </c>
       <c r="I77" s="6" t="inlineStr"/>
@@ -4496,7 +4496,7 @@
       </c>
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>PASS — @media (prefers-reduced-motion: reduce) block in tokens.css (loads on every page) | 2026-08-13 re-verified live: verified in the DEPLOYED sheet, not just source: tokens.css?v=phase23 carries @media (prefers-reduced-motion: reduce) zeroing transition-duration and animation-duration on *, *::before, *::after with !important, plus scroll-behavior auto. Catches all 29 transitioned elements on the homepage. | 2026-08-16 re-verified live: re-verified in the LOADED CSSOM (not source): tokens.css?v=phase23 carries @media (prefers-reduced-motion: reduce) zeroing transition-duration and animation-duration on *, ::before, ::after with !important plus scroll-behavior auto — catching all 8 transitioned elements on the article page. | 2026-08-25 re-verified live: tokens.css:584 zeroes transition-duration and animation-duration on *, ::before and ::after under prefers-reduced-motion: reduce and sets scroll-behavior auto; home-augment.css:1012 adds the targeted transition:none block. Both present in the served sheets. | 2026-08-27 re-verified live: @media (prefers-reduced-motion: reduce) block present in the loaded stylesheets. | 2026-09-01 SOURCE-VERIFIED only: tokens.css?v=phase24 carries a blanket @media (prefers-reduced-motion: reduce) block setting transition-duration and animation-duration to 0s !important on *, *::before and *::after, plus scroll-behavior: auto on html; home-augment.css adds two scoped blocks. The !important universal selector is cascade-proof, so the rule cannot be defeated downstream. NOT re-verified in the browser: this harness cannot emulate the prefers-reduced-motion media query. Prior live PASS retained. | 2026-09-06 re-verified live (source-verified): the global @media (prefers-reduced-motion: reduce) kill switch is present in the loaded tokens.css cascade (tokens.css:573-582, transition-duration 0s !important on *, ::before, ::after). Not driven end-to-end - the pane cannot emulate the media query. | 2026-09-11 re-verified live: two prefers-reduced-motion blocks live — tokens.css zeroes transition/animation duration globally, home-augment.css nulls five named transitions. | 2026-09-24 re-verified live: tokens.css?v=phase24 still carries @media (prefers-reduced-motion: reduce) (html scroll-behavior auto; *,*::before,*::after durations zeroed) and home-augment.css carries 2 reduced-motion blocks; both present in the deployed sheets' CSSOM on the homepage. | 2026-09-28: live: prefers-reduced-motion rules in tokens.css + home-augment.css; 2 reduced-motion media rules loaded on home.</t>
+          <t>PASS — @media (prefers-reduced-motion: reduce) block in tokens.css (loads on every page) | 2026-08-13 re-verified live: verified in the DEPLOYED sheet, not just source: tokens.css?v=phase23 carries @media (prefers-reduced-motion: reduce) zeroing transition-duration and animation-duration on *, *::before, *::after with !important, plus scroll-behavior auto. Catches all 29 transitioned elements on the homepage. | 2026-08-16 re-verified live: re-verified in the LOADED CSSOM (not source): tokens.css?v=phase23 carries @media (prefers-reduced-motion: reduce) zeroing transition-duration and animation-duration on *, ::before, ::after with !important plus scroll-behavior auto — catching all 8 transitioned elements on the article page. | 2026-08-25 re-verified live: tokens.css:584 zeroes transition-duration and animation-duration on *, ::before and ::after under prefers-reduced-motion: reduce and sets scroll-behavior auto; home-augment.css:1012 adds the targeted transition:none block. Both present in the served sheets. | 2026-08-27 re-verified live: @media (prefers-reduced-motion: reduce) block present in the loaded stylesheets. | 2026-09-01 SOURCE-VERIFIED only: tokens.css?v=phase24 carries a blanket @media (prefers-reduced-motion: reduce) block setting transition-duration and animation-duration to 0s !important on *, *::before and *::after, plus scroll-behavior: auto on html; home-augment.css adds two scoped blocks. The !important universal selector is cascade-proof, so the rule cannot be defeated downstream. NOT re-verified in the browser: this harness cannot emulate the prefers-reduced-motion media query. Prior live PASS retained. | 2026-09-06 re-verified live (source-verified): the global @media (prefers-reduced-motion: reduce) kill switch is present in the loaded tokens.css cascade (tokens.css:573-582, transition-duration 0s !important on *, ::before, ::after). Not driven end-to-end - the pane cannot emulate the media query. | 2026-09-11 re-verified live: two prefers-reduced-motion blocks live — tokens.css zeroes transition/animation duration globally, home-augment.css nulls five named transitions. | 2026-09-24 re-verified live: tokens.css?v=phase24 still carries @media (prefers-reduced-motion: reduce) (html scroll-behavior auto; *,*::before,*::after durations zeroed) and home-augment.css carries 2 reduced-motion blocks; both present in the deployed sheets' CSSOM on the homepage. | 2026-09-28: live: prefers-reduced-motion rules in tokens.css + home-augment.css; 2 reduced-motion media rules loaded on home. | 2026-10-05: live: prefers-reduced-motion blocks in tokens.css (global) and home-augment.css (hover controls).</t>
         </is>
       </c>
       <c r="I78" s="6" t="inlineStr"/>
@@ -4549,7 +4549,7 @@
       </c>
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>PASS (closed live 2026-08-10) — was ISSUE/High: .subscribe-manifesto .sm-submit (homepage + /brand/ subscribe submit) had base and :hover styling but NO :focus-visible rule, so the site's primary conversion control showed no focus indicator for keyboard users (WCAG 2.4.7 AA). Every sibling control was covered — .sm-input directly above it had the rule, and .sm-submit was even named in home-augment.css's prefers-reduced-motion block — so it was an omission, not a decision. Missed by prior runs because F76 was tested at sheet level (':focus-visible present in all 8 stylesheets') rather than per control. Fixed and deployed same day; see p3/p4. | 2026-08-13 re-verified live: re-verified live by REAL keyboard input (not JS .focus(), which cannot trigger :focus-visible): pressing Tab moved focus to a footer link that matched ':focus-visible' and computed outline 'solid 2px rgb(204, 0, 0)' at offset 2px. | 2026-08-16 re-verified live: re-verified live by REAL keyboard input (not JS .focus(), which cannot trigger :focus-visible): pressing Tab moved focus to SUMMARY.study-note-trigger, which matched ':focus-visible' and computed outline 'rgb(204, 0, 0) solid 2px' at offset -2px. | 2026-08-25 re-verified live: re-verified under REAL keyboard input: tabbing to .study-note-trigger on an article paints outline solid 2px rgb(204,0,0) (--focus-ring) at -2px offset. NOTE for future runs: a programmatic element.focus() does NOT satisfy :focus-visible in Chrome and will report outline:none across the board — a false positive this run initially produced. | 2026-08-27 re-verified live: focus ring under REAL Tab (not element.focus()): outline rgb(204,0,0) solid 2px = --accent. | 2026-09-01 re-verified live under REAL Tab presses (never element.focus()): .brand-block, .mode-toggle, .issue-standfirst and .hero-link each match :focus-visible and paint outline rgb(204,0,0) solid 2px, matching --focus-ring #c00. | 2026-09-06 re-verified live: real Tab/Shift+Tab presses put outline: rgb(204,0,0) solid 2px on plate links, .lane-cell, .earlier-more-btn and .brand-block. The skip link is the one exception and is F98. | 2026-09-11 re-verified live: real Tab walk on the homepage: skip-link → brand-block → hero links → lane cells, every stop carrying outline rgb(204,0,0) solid 2px. | 2026-09-24 re-verified live: every css/*.css defines :focus-visible (article 9, home-augment 6, home-v2 5, shell 5, tokens 2, phase0 2, plates 1, notfound 1). Real Tab on the homepage: .brand-block and .skip-link both render solid 2px rgb(204,0,0) with :focus-visible true; skip link activates to MAIN#archive. | 2026-09-28: live: all 8 css files define :focus-visible; skip link under real Tab -&gt; 2px solid #c00.</t>
+          <t>PASS (closed live 2026-08-10) — was ISSUE/High: .subscribe-manifesto .sm-submit (homepage + /brand/ subscribe submit) had base and :hover styling but NO :focus-visible rule, so the site's primary conversion control showed no focus indicator for keyboard users (WCAG 2.4.7 AA). Every sibling control was covered — .sm-input directly above it had the rule, and .sm-submit was even named in home-augment.css's prefers-reduced-motion block — so it was an omission, not a decision. Missed by prior runs because F76 was tested at sheet level (':focus-visible present in all 8 stylesheets') rather than per control. Fixed and deployed same day; see p3/p4. | 2026-08-13 re-verified live: re-verified live by REAL keyboard input (not JS .focus(), which cannot trigger :focus-visible): pressing Tab moved focus to a footer link that matched ':focus-visible' and computed outline 'solid 2px rgb(204, 0, 0)' at offset 2px. | 2026-08-16 re-verified live: re-verified live by REAL keyboard input (not JS .focus(), which cannot trigger :focus-visible): pressing Tab moved focus to SUMMARY.study-note-trigger, which matched ':focus-visible' and computed outline 'rgb(204, 0, 0) solid 2px' at offset -2px. | 2026-08-25 re-verified live: re-verified under REAL keyboard input: tabbing to .study-note-trigger on an article paints outline solid 2px rgb(204,0,0) (--focus-ring) at -2px offset. NOTE for future runs: a programmatic element.focus() does NOT satisfy :focus-visible in Chrome and will report outline:none across the board — a false positive this run initially produced. | 2026-08-27 re-verified live: focus ring under REAL Tab (not element.focus()): outline rgb(204,0,0) solid 2px = --accent. | 2026-09-01 re-verified live under REAL Tab presses (never element.focus()): .brand-block, .mode-toggle, .issue-standfirst and .hero-link each match :focus-visible and paint outline rgb(204,0,0) solid 2px, matching --focus-ring #c00. | 2026-09-06 re-verified live: real Tab/Shift+Tab presses put outline: rgb(204,0,0) solid 2px on plate links, .lane-cell, .earlier-more-btn and .brand-block. The skip link is the one exception and is F98. | 2026-09-11 re-verified live: real Tab walk on the homepage: skip-link → brand-block → hero links → lane cells, every stop carrying outline rgb(204,0,0) solid 2px. | 2026-09-24 re-verified live: every css/*.css defines :focus-visible (article 9, home-augment 6, home-v2 5, shell 5, tokens 2, phase0 2, plates 1, notfound 1). Real Tab on the homepage: .brand-block and .skip-link both render solid 2px rgb(204,0,0) with :focus-visible true; skip link activates to MAIN#archive. | 2026-09-28: live: all 8 css files define :focus-visible; skip link under real Tab -&gt; 2px solid #c00. | 2026-10-05: live: :focus-visible rules in shell/plates/home-augment/home-v2; real Tab shows 2px #c00 rings on skip link, brand block, mode toggle.</t>
         </is>
       </c>
       <c r="I79" s="6" t="inlineStr">
@@ -4606,7 +4606,7 @@
       </c>
       <c r="H80" s="6" t="inlineStr">
         <is>
-          <t>PASS (closed live 2026-08-13) — was ISSUE/High (2026-08-13) — .latest-tag (the red 'Latest' chip in the homepage standfirst bar) pairs `background: var(--accent)` with `color: var(--bg)`. In light mode that is cream on #c00 = 5.17:1 and passes. In dark mode --bg flips to #060606 and the same chip computes 3.44:1 at 11.52px/700 — under the 4.5:1 AA floor for small text (WCAG 1.4.3). Measured three times on settled live loads. The #c00/#060606 pair is sanctioned by the Phase 4.1 accent doctrine (DESIGN-SYSTEM.md:102) only for NON-text contrast at the 3:1 floor; this is a text use of it. Missed by prior runs because F77 sampled palette-level token pairs (body/muted/faint/accent text), not the one control that puts small text ON the accent fill — the same sheet-level vs per-control gap that hid F76. All other sampled combinations still pass: 33 distinct fg/bg/size combos in dark, 33 in light, this was the only failure. | 2026-08-16 re-verified live: full-page compositor sweep across home (dark 92 elements / light 88), article (70), about (15), phase0 (84), brand and 404. Two light-mode 'failures' on .plate-image plates (h2.plate-title.inverse and p.plate-deck, both 1.06:1) were investigated and DISMISSED as false positives: those plates carry an ::after `linear-gradient(to top, rgba(0,0,0,.78) ...)` scrim, so the white text sits on a dark overlay, not the cream plate colour the compositor resolved — confirmed visually in a light-mode screenshot. Two compounding methodology bugs were behind the false read and are now fixed in the sweep: (a) the compositor walked background-COLOR only and ignored pseudo-element layers, (b) selector-level dedupe merged image and non-image plates under the same class string, so a passing element inherited a failing element's number. Lesson is the same shape as F84's: resolve the PAINTED surface, never infer it from an ancestor's declarations. | 2026-08-25 re-verified live: .latest-tag on the live homepage in dark mode measures 5.17:1 (rgb(243,240,232) on rgb(204,0,0)) — the F77 fix still holds, no regression. | 2026-09-01 re-verified live with a full ancestor-stack compositing probe (semi-transparent layers composited down to the first opaque one; .plate-image plates and aria-hidden decoration excluded per the documented antipatterns): 0 WCAG AA failures across ~1050 measured text elements — homepage light (0/70+), homepage dark (0/70), article dark at 375px (0/86), /about/ (0/24), /404 (0/16), /phase0/ (0/106), /brand/ (0/800). | 2026-09-06 re-verified live: the sweep is now pixel-based on image plates, not computed-style-based. Composited-ancestor probe across home, article, about, 404, phase0 and /brand/ in BOTH modes: zero failures outside the image plates. Inside them, rasterised sampling opened F101 (2.68:1 on img-concrete) - a defect every previous computed-style sweep reported as the known 1.06:1 artifact. | 2026-09-11 re-verified live: composited-stack contrast sweep over home/about/brand/phase0/404/article in BOTH modes: zero real failures. Only hits were the aria-hidden .dot separators (4.25–4.30:1, exempt, documented) and the image-plate 1.06:1 probe artifact, dismissed on geometry (below). | 2026-09-24 re-verified live: contrast sweep with full ancestor compositing and inherited opacity, both modes: home 70 elements, article (the-weight-of-my-no) 86, /about/ 24, /404 16, /phase0/ 106, /brand/ 793 — 0 failures in light, 0 in dark (image plates excluded per the antipattern; 8/8 home and 5/5 brand demo plate bodies keep display:flex + justify-content:flex-end). Hover states are F83/F108's scope. | 2026-09-28: live: contrast sweep 0 failures — dark: home, about, article, phase0, 404, brand; light: home, about, article, phase0, brand.</t>
+          <t>PASS (closed live 2026-08-13) — was ISSUE/High (2026-08-13) — .latest-tag (the red 'Latest' chip in the homepage standfirst bar) pairs `background: var(--accent)` with `color: var(--bg)`. In light mode that is cream on #c00 = 5.17:1 and passes. In dark mode --bg flips to #060606 and the same chip computes 3.44:1 at 11.52px/700 — under the 4.5:1 AA floor for small text (WCAG 1.4.3). Measured three times on settled live loads. The #c00/#060606 pair is sanctioned by the Phase 4.1 accent doctrine (DESIGN-SYSTEM.md:102) only for NON-text contrast at the 3:1 floor; this is a text use of it. Missed by prior runs because F77 sampled palette-level token pairs (body/muted/faint/accent text), not the one control that puts small text ON the accent fill — the same sheet-level vs per-control gap that hid F76. All other sampled combinations still pass: 33 distinct fg/bg/size combos in dark, 33 in light, this was the only failure. | 2026-08-16 re-verified live: full-page compositor sweep across home (dark 92 elements / light 88), article (70), about (15), phase0 (84), brand and 404. Two light-mode 'failures' on .plate-image plates (h2.plate-title.inverse and p.plate-deck, both 1.06:1) were investigated and DISMISSED as false positives: those plates carry an ::after `linear-gradient(to top, rgba(0,0,0,.78) ...)` scrim, so the white text sits on a dark overlay, not the cream plate colour the compositor resolved — confirmed visually in a light-mode screenshot. Two compounding methodology bugs were behind the false read and are now fixed in the sweep: (a) the compositor walked background-COLOR only and ignored pseudo-element layers, (b) selector-level dedupe merged image and non-image plates under the same class string, so a passing element inherited a failing element's number. Lesson is the same shape as F84's: resolve the PAINTED surface, never infer it from an ancestor's declarations. | 2026-08-25 re-verified live: .latest-tag on the live homepage in dark mode measures 5.17:1 (rgb(243,240,232) on rgb(204,0,0)) — the F77 fix still holds, no regression. | 2026-09-01 re-verified live with a full ancestor-stack compositing probe (semi-transparent layers composited down to the first opaque one; .plate-image plates and aria-hidden decoration excluded per the documented antipatterns): 0 WCAG AA failures across ~1050 measured text elements — homepage light (0/70+), homepage dark (0/70), article dark at 375px (0/86), /about/ (0/24), /404 (0/16), /phase0/ (0/106), /brand/ (0/800). | 2026-09-06 re-verified live: the sweep is now pixel-based on image plates, not computed-style-based. Composited-ancestor probe across home, article, about, 404, phase0 and /brand/ in BOTH modes: zero failures outside the image plates. Inside them, rasterised sampling opened F101 (2.68:1 on img-concrete) - a defect every previous computed-style sweep reported as the known 1.06:1 artifact. | 2026-09-11 re-verified live: composited-stack contrast sweep over home/about/brand/phase0/404/article in BOTH modes: zero real failures. Only hits were the aria-hidden .dot separators (4.25–4.30:1, exempt, documented) and the image-plate 1.06:1 probe artifact, dismissed on geometry (below). | 2026-09-24 re-verified live: contrast sweep with full ancestor compositing and inherited opacity, both modes: home 70 elements, article (the-weight-of-my-no) 86, /about/ 24, /404 16, /phase0/ 106, /brand/ 793 — 0 failures in light, 0 in dark (image plates excluded per the antipattern; 8/8 home and 5/5 brand demo plate bodies keep display:flex + justify-content:flex-end). Hover states are F83/F108's scope. | 2026-09-28: live: contrast sweep 0 failures — dark: home, about, article, phase0, 404, brand; light: home, about, article, phase0, brand. | 2026-10-05: live: composite contrast sweep 0 failures on home, about, 404, phase0, brand (dark) and article, in both modes.</t>
         </is>
       </c>
       <c r="I80" s="6" t="inlineStr">
@@ -4663,7 +4663,7 @@
       </c>
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>PASS — single h1 and zero skipped heading levels on all 21 pages; header/main/footer/nav present; zero &lt;img&gt; without alt | 2026-08-13 re-verified live: home and article both single-h1, zero skipped heading levels (home H1 then 17x H2; article H1,H2,H2,H2,H2,H2), header/main/footer/nav all present. Zero images missing alt. | 2026-08-16 re-verified live: single &lt;h1&gt; and zero skipped heading levels across all 21 live pages; header/main/footer/nav present on every page type; zero &lt;img&gt; without an alt attribute. | 2026-08-25 re-verified live: header/main/footer/nav present on every page type; exactly one &lt;h1&gt; per page across all 20 routes; zero skipped heading levels; zero &lt;img&gt; without alt. | 2026-08-27 re-verified live: single h1 and zero skipped heading levels across all 21 routes. | 2026-09-01 re-verified live: header/main/footer/nav present on every route; exactly one h1 per page; no skipped heading levels anywhere, including /phase0/'s 22-heading tree. | 2026-09-06 re-verified live: header/nav/main/footer all present on the homepage; exactly one h1 per page and no skipped heading levels across home, about, brand, phase0 and 404. | 2026-09-11 re-verified live: single h1 and no skipped heading level on all six surface types; header/main/footer/nav present on each. | 2026-09-24 re-verified live: single h1 on home, article, /about/, /404, /phase0/, /brand/; home headings 1 then 18x2, article 1-2-2-2; header, main[id] (archive / article / about / main / phase0 / main), footer present everywhere; nav aria-labels 'Main navigation' (+ 'Essay navigation' on articles); 0 &lt;img&gt; without alt (the masthead logo's alt='' is decorative inside the labelled brand link). | 2026-09-28: live: single h1 on every type, no skipped levels, header/main/footer/nav landmarks.</t>
+          <t>PASS — single h1 and zero skipped heading levels on all 21 pages; header/main/footer/nav present; zero &lt;img&gt; without alt | 2026-08-13 re-verified live: home and article both single-h1, zero skipped heading levels (home H1 then 17x H2; article H1,H2,H2,H2,H2,H2), header/main/footer/nav all present. Zero images missing alt. | 2026-08-16 re-verified live: single &lt;h1&gt; and zero skipped heading levels across all 21 live pages; header/main/footer/nav present on every page type; zero &lt;img&gt; without an alt attribute. | 2026-08-25 re-verified live: header/main/footer/nav present on every page type; exactly one &lt;h1&gt; per page across all 20 routes; zero skipped heading levels; zero &lt;img&gt; without alt. | 2026-08-27 re-verified live: single h1 and zero skipped heading levels across all 21 routes. | 2026-09-01 re-verified live: header/main/footer/nav present on every route; exactly one h1 per page; no skipped heading levels anywhere, including /phase0/'s 22-heading tree. | 2026-09-06 re-verified live: header/nav/main/footer all present on the homepage; exactly one h1 per page and no skipped heading levels across home, about, brand, phase0 and 404. | 2026-09-11 re-verified live: single h1 and no skipped heading level on all six surface types; header/main/footer/nav present on each. | 2026-09-24 re-verified live: single h1 on home, article, /about/, /404, /phase0/, /brand/; home headings 1 then 18x2, article 1-2-2-2; header, main[id] (archive / article / about / main / phase0 / main), footer present everywhere; nav aria-labels 'Main navigation' (+ 'Essay navigation' on articles); 0 &lt;img&gt; without alt (the masthead logo's alt='' is decorative inside the labelled brand link). | 2026-09-28: live: single h1 on every type, no skipped levels, header/main/footer/nav landmarks. | 2026-10-05: live: header, nav[aria-label="Main navigation"], main#archive, footer[aria-label]; single h1, no skipped heading levels.</t>
         </is>
       </c>
       <c r="I81" s="6" t="inlineStr"/>
@@ -4716,7 +4716,7 @@
       </c>
       <c r="H82" s="6" t="inlineStr">
         <is>
-          <t>PASS — fired as designed on 2026-07-05 (ecf2c34, github-actions[bot], 18:03:14Z); both guards now permanently closed (year!=2026, status no longer 'drafted'); no post-fire bot commit exists on main | 2026-09-11 re-verified live: publish-send-someone-else.yml still absent (removed 11d1430); daily-rebuild.yml is the only workflow; send-someone-else status still 'published'. No post-fire github-actions[bot] commit on main. | 2026-09-24 re-verified live: daily-rebuild.yml is still the only workflow; publish-send-someone-else.yml absent; zero github-actions commits on origin/main since 2026-07-06. | 2026-09-28: repo: daily-rebuild.yml still the only workflow; publish workflow removed (11d1430).</t>
+          <t>PASS — fired as designed on 2026-07-05 (ecf2c34, github-actions[bot], 18:03:14Z); both guards now permanently closed (year!=2026, status no longer 'drafted'); no post-fire bot commit exists on main | 2026-09-11 re-verified live: publish-send-someone-else.yml still absent (removed 11d1430); daily-rebuild.yml is the only workflow; send-someone-else status still 'published'. No post-fire github-actions[bot] commit on main. | 2026-09-24 re-verified live: daily-rebuild.yml is still the only workflow; publish-send-someone-else.yml absent; zero github-actions commits on origin/main since 2026-07-06. | 2026-09-28: repo: daily-rebuild.yml still the only workflow; publish workflow removed (11d1430). | 2026-10-05: repo: daily-rebuild.yml is the only workflow; publish workflow stays removed.</t>
         </is>
       </c>
       <c r="I82" s="6" t="inlineStr"/>
@@ -4769,7 +4769,7 @@
       </c>
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>PASS — parity 16/16 verified live; every /words/&lt;slug&gt; returns a single 301 to its trailing-slash canonical; no orphan rules | 2026-08-13 re-verified live: all 16 /words/&lt;slug&gt; (no trailing slash) return 301; all 16 /words/&lt;slug&gt;/ return 200 in 0.31-0.45s. | 2026-08-25 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-01 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-06 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-11 re-verified live: /words/&lt;slug&gt; → 301 → /words/&lt;slug&gt;/ → 200 verified on the-stone; all 17 article slugs 200 at their canonical form. | 2026-09-24 ISSUE/Low — the parity test the expected column defines, run for the first time since 2026-08-31, fails 16/17: the-weight-of-my-no (status published, 2026-08-31) has no [[redirects]] rule in netlify.toml. Every run since 08-31 spot-checked /words/the-stone only, so the drift went unseen for 24 days — the same shape as the July show-me-your-glory / send-someone-else drift. The expected column's 'non-slash 404s' premise did NOT hold: live /words/the-weight-of-my-no returns 301 -&gt; /words/the-weight-of-my-no/ with no rule, because Netlify Pretty URLs redirects a directory path on its own. No user impact observed; graded Low (parity/config drift, not a broken route). | 2026-09-25: live behaviour unchanged (single 301 via Pretty URLs); rule still only on the unmerged branch. | 2026-09-26 full parity test (not a spot check) on qa/fixes-20260926: 17 published slugs == 17 /words/&lt;slug&gt; rules, 0 missing, 0 orphans, 0 dupes, no force; live: all 17 /words/&lt;slug&gt; return a single 301 to the slash canonical -&gt; 200. Fix still awaits merge (origin/main 95e2a73 lacks the rule; live behaviour unaffected). | 2026-09-28: live parity: 17/17 /words/&lt;slug&gt; return a single 301 to the slash canonical; rule still only on the unmerged branch.</t>
+          <t>PASS — parity 16/16 verified live; every /words/&lt;slug&gt; returns a single 301 to its trailing-slash canonical; no orphan rules | 2026-08-13 re-verified live: all 16 /words/&lt;slug&gt; (no trailing slash) return 301; all 16 /words/&lt;slug&gt;/ return 200 in 0.31-0.45s. | 2026-08-25 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-01 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-06 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-11 re-verified live: /words/&lt;slug&gt; → 301 → /words/&lt;slug&gt;/ → 200 verified on the-stone; all 17 article slugs 200 at their canonical form. | 2026-09-24 ISSUE/Low — the parity test the expected column defines, run for the first time since 2026-08-31, fails 16/17: the-weight-of-my-no (status published, 2026-08-31) has no [[redirects]] rule in netlify.toml. Every run since 08-31 spot-checked /words/the-stone only, so the drift went unseen for 24 days — the same shape as the July show-me-your-glory / send-someone-else drift. The expected column's 'non-slash 404s' premise did NOT hold: live /words/the-weight-of-my-no returns 301 -&gt; /words/the-weight-of-my-no/ with no rule, because Netlify Pretty URLs redirects a directory path on its own. No user impact observed; graded Low (parity/config drift, not a broken route). | 2026-09-25: live behaviour unchanged (single 301 via Pretty URLs); rule still only on the unmerged branch. | 2026-09-26 full parity test (not a spot check) on qa/fixes-20260926: 17 published slugs == 17 /words/&lt;slug&gt; rules, 0 missing, 0 orphans, 0 dupes, no force; live: all 17 /words/&lt;slug&gt; return a single 301 to the slash canonical -&gt; 200. Fix still awaits merge (origin/main 95e2a73 lacks the rule; live behaviour unaffected). | 2026-09-28: live parity: 17/17 /words/&lt;slug&gt; return a single 301 to the slash canonical; rule still only on the unmerged branch. | 2026-10-05: repo: parity holds — 17 per-article 301 redirects (none forced) == 17 published slugs.</t>
         </is>
       </c>
       <c r="I83" s="6" t="inlineStr">
@@ -4826,7 +4826,7 @@
       </c>
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: show-me-your-glory emits rel=next to send-someone-else and renders a normal (non-ghost) forward nav; forward chain walks all 16 published essays end to end. | 2026-08-25 re-verified live: forward chain walks all 16 published essays end to end; the chronologically newest (send-someone-else) correctly carries no next. | 2026-09-18 re-verified live: forward chain walks all 17 published essays end to end, reckonings → the-weight-of-my-no; only the newest lacks rel=next and only the oldest lacks rel=prev. | 2026-09-24 re-verified live: forward chain walks all 17 published essays end to end from the oldest; the newest (the-weight-of-my-no, 2026-08-31) is the only entry without next; every next target is a published slug. | 2026-09-28: repo: forward chain 16/16 — every entry except the newest carries next == its chronological successor; 0 mismatches.</t>
+          <t>PASS — live-verified 2026-08-10: show-me-your-glory emits rel=next to send-someone-else and renders a normal (non-ghost) forward nav; forward chain walks all 16 published essays end to end. | 2026-08-25 re-verified live: forward chain walks all 16 published essays end to end; the chronologically newest (send-someone-else) correctly carries no next. | 2026-09-18 re-verified live: forward chain walks all 17 published essays end to end, reckonings → the-weight-of-my-no; only the newest lacks rel=next and only the oldest lacks rel=prev. | 2026-09-24 re-verified live: forward chain walks all 17 published essays end to end from the oldest; the newest (the-weight-of-my-no, 2026-08-31) is the only entry without next; every next target is a published slug. | 2026-09-28: repo: forward chain 16/16 — every entry except the newest carries next == its chronological successor; 0 mismatches. | 2026-10-05: repo + live: forward chain 16/16 matches chronological order. Backward half was broken (send-someone-else prev -&gt; some); filed and fixed as F109.</t>
         </is>
       </c>
       <c r="I84" s="6" t="inlineStr"/>
@@ -4879,7 +4879,7 @@
       </c>
       <c r="H85" s="6" t="inlineStr">
         <is>
-          <t>PASS (resolved 2026-08-10) — was ISSUE/Low: DESIGN-SYSTEM.md:115 listed "Reading progress bar (`var(--accent)`)" as a permitted accent use, but css/article.css:876 ships `.reading-progress { background: var(--ink) }`. Commit 68b0c1d (2026-04-10) recolored it on purpose and left the reason in the CSS: red was competing with the masthead and diluting the accent's semantic weight. That commit rewrote 136 lines of DESIGN-SYSTEM.md but missed this one bullet, which dated to c75ded9 earlier the same day. The CSS was correct; the doc line was stale. | 2026-08-27 second doc-parity pass (9b8e4c4): three more drifts closed, all doc-side. The Ghost Teaser Plate code block was pre-F90 and pre-cutover (min-height 346 vs the shipped 230; .plate-title opacity .35 vs .46/.40; --ink+opacity on .teaser-date and .meta-rail vs --body-muted), its prose still carried the static-HTML instruction 'swap for the full article plate and remove the ghost CSS from index.html', and the prev/next section claimed `next.ghost: true` drives 'the homepage's issue-next ghost CTA' — which conflated .article-nav-ghost with a component that no longer exists and was wrong before any of today's work. Also corrected a stale comment inside plates.css that justified a padding choice against '346px min-height' on a rule setting 230px — the same wrong number that had propagated into the doc. | 2026-09-11 re-verified live: permitted-accent list re-read; diff of css/ and brand/ from 2026-08-13 to HEAD adds ZERO new var(--accent) rules (two removals only). No new doc-vs-implementation drift. | 2026-09-24 re-verified live: no css/ or DESIGN-SYSTEM.md change on main since the last PASS; the Permitted list still resolves to live accent rules (section-head h2 and rule, callout border, stat bar, plate hover border, focus ring). DESIGN-SYSTEM.md:148 edited today on the fix branch for F108 (names the third hover control and the sheet the override actually lives in, home-augment.css, per F87) — parity improved, not broken. | 2026-09-28: carried: DESIGN-SYSTEM.md touched only by the unmerged F108 commit; accent homes verified live (section-head h2 #ff4d4d dark, .callout border #c00).</t>
+          <t>PASS (resolved 2026-08-10) — was ISSUE/Low: DESIGN-SYSTEM.md:115 listed "Reading progress bar (`var(--accent)`)" as a permitted accent use, but css/article.css:876 ships `.reading-progress { background: var(--ink) }`. Commit 68b0c1d (2026-04-10) recolored it on purpose and left the reason in the CSS: red was competing with the masthead and diluting the accent's semantic weight. That commit rewrote 136 lines of DESIGN-SYSTEM.md but missed this one bullet, which dated to c75ded9 earlier the same day. The CSS was correct; the doc line was stale. | 2026-08-27 second doc-parity pass (9b8e4c4): three more drifts closed, all doc-side. The Ghost Teaser Plate code block was pre-F90 and pre-cutover (min-height 346 vs the shipped 230; .plate-title opacity .35 vs .46/.40; --ink+opacity on .teaser-date and .meta-rail vs --body-muted), its prose still carried the static-HTML instruction 'swap for the full article plate and remove the ghost CSS from index.html', and the prev/next section claimed `next.ghost: true` drives 'the homepage's issue-next ghost CTA' — which conflated .article-nav-ghost with a component that no longer exists and was wrong before any of today's work. Also corrected a stale comment inside plates.css that justified a padding choice against '346px min-height' on a rule setting 230px — the same wrong number that had propagated into the doc. | 2026-09-11 re-verified live: permitted-accent list re-read; diff of css/ and brand/ from 2026-08-13 to HEAD adds ZERO new var(--accent) rules (two removals only). No new doc-vs-implementation drift. | 2026-09-24 re-verified live: no css/ or DESIGN-SYSTEM.md change on main since the last PASS; the Permitted list still resolves to live accent rules (section-head h2 and rule, callout border, stat bar, plate hover border, focus ring). DESIGN-SYSTEM.md:148 edited today on the fix branch for F108 (names the third hover control and the sheet the override actually lives in, home-augment.css, per F87) — parity improved, not broken. | 2026-09-28: carried: DESIGN-SYSTEM.md touched only by the unmerged F108 commit; accent homes verified live (section-head h2 #ff4d4d dark, .callout border #c00). | 2026-10-05: carried: no accent rule or DESIGN-SYSTEM.md change on origin/main; accent homes live (section-head h2 #c00 light / #ff4d4d dark, .callout border #c00).</t>
         </is>
       </c>
       <c r="I85" s="6" t="inlineStr">
@@ -4936,7 +4936,7 @@
       </c>
       <c r="H86" s="6" t="inlineStr">
         <is>
-          <t>PASS (closed live 2026-08-13) — was ISSUE/High (2026-08-13) — CORRECTED SCOPE, and the correction matters. The morning scrub read the declarations and reported FOUR failing hover rules. Re-measured under REAL pointer hover before fixing, only TWO are real: `.issue-latest:hover .latest-cta` (14.08px/700) and `.identity-hero .hero-link.primary:hover` (14.08px/700), both `color: var(--bg)` on a `background: var(--accent)` fill = 3.44:1 in dark against a 4.5:1 floor. The other two were FALSE POSITIVES: `.issue-latest:hover` takes the BAR to var(--ink), not var(--accent), so .latest-title measures 17.79:1 and .latest-meta 5.23:1 (at opacity .6) against cream — both already clear. The morning read assumed the accent fill was the surface for every child of the hover state; it is only the surface for .latest-cta, which sets its own background. Lesson: resolve the PAINTED surface under real hover, never infer it from the parent's declarations. | 2026-08-25 re-verified live: re-verified under REAL pointer hover on the live homepage in dark mode: .latest-cta 5.17:1, .latest-tag 5.17:1, .latest-title 17.79:1, .latest-meta (hover state) 5.23:1. No regression. Caveat carried to F87: the override lives in home-v2.css on the live deploy, so /brand/ still does not get it. | 2026-09-18 re-verified live: dark mode under REAL pointer hover: .latest-cta 'Read →' and .hero-link.primary 'Read the About →' both cream 243,240,232 on #c00 = 5.17:1 at 14.08px. | 2026-09-24 re-verified live: the two controls F83 fixed still pass under real pointer hover in dark mode: .latest-cta and .identity-hero .hero-link.primary both cream on #c00 at 5.17:1. BUT F83's scope note ('only the two controls below actually invert onto the accent fill on hover') was wrong: a.plate-lead:hover .rail-cta also inverts onto the accent and was missed — split out as F108, not counted as a regression of this row. | 2026-09-28: live: 0 contrast failures in both sweeps; .latest-cta / .hero-link.primary source unchanged. The third control (F108) is still live pending merge.</t>
+          <t>PASS (closed live 2026-08-13) — was ISSUE/High (2026-08-13) — CORRECTED SCOPE, and the correction matters. The morning scrub read the declarations and reported FOUR failing hover rules. Re-measured under REAL pointer hover before fixing, only TWO are real: `.issue-latest:hover .latest-cta` (14.08px/700) and `.identity-hero .hero-link.primary:hover` (14.08px/700), both `color: var(--bg)` on a `background: var(--accent)` fill = 3.44:1 in dark against a 4.5:1 floor. The other two were FALSE POSITIVES: `.issue-latest:hover` takes the BAR to var(--ink), not var(--accent), so .latest-title measures 17.79:1 and .latest-meta 5.23:1 (at opacity .6) against cream — both already clear. The morning read assumed the accent fill was the surface for every child of the hover state; it is only the surface for .latest-cta, which sets its own background. Lesson: resolve the PAINTED surface under real hover, never infer it from the parent's declarations. | 2026-08-25 re-verified live: re-verified under REAL pointer hover on the live homepage in dark mode: .latest-cta 5.17:1, .latest-tag 5.17:1, .latest-title 17.79:1, .latest-meta (hover state) 5.23:1. No regression. Caveat carried to F87: the override lives in home-v2.css on the live deploy, so /brand/ still does not get it. | 2026-09-18 re-verified live: dark mode under REAL pointer hover: .latest-cta 'Read →' and .hero-link.primary 'Read the About →' both cream 243,240,232 on #c00 = 5.17:1 at 14.08px. | 2026-09-24 re-verified live: the two controls F83 fixed still pass under real pointer hover in dark mode: .latest-cta and .identity-hero .hero-link.primary both cream on #c00 at 5.17:1. BUT F83's scope note ('only the two controls below actually invert onto the accent fill on hover') was wrong: a.plate-lead:hover .rail-cta also inverts onto the accent and was missed — split out as F108, not counted as a regression of this row. | 2026-09-28: live: 0 contrast failures in both sweeps; .latest-cta / .hero-link.primary source unchanged. The third control (F108) is still live pending merge. | 2026-10-05: live: dark-mode accent hover fills hold (F108 measured 5.17:1 with transitions neutralised).</t>
         </is>
       </c>
       <c r="I86" s="6" t="inlineStr">
@@ -4993,7 +4993,7 @@
       </c>
       <c r="H87" s="6" t="inlineStr">
         <is>
-          <t>PASS (closed live 2026-08-13) — was ISSUE/Low (2026-08-13) — DESIGN-SYSTEM.md:124-130 lists 'Backgrounds' and 'Tags or metadata' as PROHIBITED accent uses, but .latest-tag is exactly that: a metadata tag with `background: var(--accent)`, shipped and prominent in the homepage standfirst bar. Companion to F82, which audited only the Permitted half of the same section and so could not have caught this. | 2026-09-11 re-verified live: prohibited-accent list re-read; same diff confirms no new background: var(--accent) rule since the .latest-tag annotation shipped. The sanctioned exception is still the only one. | 2026-09-24 re-verified live: every background: var(--accent) rule enumerated (19 across 5 sheets): the only tag/metadata fills are .latest-tag (the annotated sanctioned exception) and .lead-badge-label (paired with --on-accent / #f5f5f1); the rest are rules, bars, dots, the manifesto panel and hover inversions. No unannotated prohibited use. | 2026-09-28: carried: no accent rule changes on origin/main since last PASS.</t>
+          <t>PASS (closed live 2026-08-13) — was ISSUE/Low (2026-08-13) — DESIGN-SYSTEM.md:124-130 lists 'Backgrounds' and 'Tags or metadata' as PROHIBITED accent uses, but .latest-tag is exactly that: a metadata tag with `background: var(--accent)`, shipped and prominent in the homepage standfirst bar. Companion to F82, which audited only the Permitted half of the same section and so could not have caught this. | 2026-09-11 re-verified live: prohibited-accent list re-read; same diff confirms no new background: var(--accent) rule since the .latest-tag annotation shipped. The sanctioned exception is still the only one. | 2026-09-24 re-verified live: every background: var(--accent) rule enumerated (19 across 5 sheets): the only tag/metadata fills are .latest-tag (the annotated sanctioned exception) and .lead-badge-label (paired with --on-accent / #f5f5f1); the rest are rules, bars, dots, the manifesto panel and hover inversions. No unannotated prohibited use. | 2026-09-28: carried: no accent rule changes on origin/main since last PASS. | 2026-10-05: carried: no accent rule changes on origin/main since last PASS.</t>
         </is>
       </c>
       <c r="I87" s="6" t="inlineStr">
@@ -5050,7 +5050,7 @@
       </c>
       <c r="H88" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-08-15) — `.latest-meta` ('Faith · Jul 5 · 16 min', the metadata in the homepage standfirst bar) pairs `color: var(--body-muted)` with `opacity: .75`. --body-muted is ALREADY an alpha colour (rgba(243,240,232,.52) dark / rgba(5,5,5,.56) light), tuned to land just over AA on its own — 5.13:1 dark, 4.67:1 light. The extra multiplier composites a second time and drops the control to 3.36:1 dark / 2.93:1 light, under the 4.5:1 floor for 11.52px/400 text. FAILS IN BOTH MODES — the only finding this run that is not dark-mode-specific. Measured on the settled live page with a compositor that resolves the painted surface by walking every ancestor background (flat #0d0d0d here, no image layer to confound it), then confirmed visually in a full-page screenshot where this is plainly the faintest text on the homepage. Missed by every prior run for a precise reason: the 2026-08-13 scrub measured .latest-meta ONLY under pointer hover, where `.issue-latest:hover .latest-meta` re-declares `color: var(--bg); opacity: .6` against the cream hover bar and clears at 5.23:1. F83 recorded that number and closed the question. The RESTING state — which is what a reader actually sees — was never measured. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: `.latest-meta` 3.36:1 dark / 2.93:1 light on the homepage, and 3.36:1 again on /brand/. Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | .latest-meta re-measured live 2026-08-25: 3.36:1 dark (homepage + /brand/), 2.93:1 light — unchanged from 2026-08-15. Root cause of the non-closure is NOT the fix: it is that the fix never shipped. origin/main is still b64a39b; the F85 commit (55a6d72) sits on LOCAL main, 8 commits ahead of origin, unpushed for 9 days. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live: .latest-meta 5.13:1 dark / 4.67:1 light, opacity 1 (no stacked multiplier). Also 5.13 on /brand/ dark. | 2026-09-28: live: covered by today's sweeps, 0 failures both modes.</t>
+          <t>ISSUE/High (2026-08-15) — `.latest-meta` ('Faith · Jul 5 · 16 min', the metadata in the homepage standfirst bar) pairs `color: var(--body-muted)` with `opacity: .75`. --body-muted is ALREADY an alpha colour (rgba(243,240,232,.52) dark / rgba(5,5,5,.56) light), tuned to land just over AA on its own — 5.13:1 dark, 4.67:1 light. The extra multiplier composites a second time and drops the control to 3.36:1 dark / 2.93:1 light, under the 4.5:1 floor for 11.52px/400 text. FAILS IN BOTH MODES — the only finding this run that is not dark-mode-specific. Measured on the settled live page with a compositor that resolves the painted surface by walking every ancestor background (flat #0d0d0d here, no image layer to confound it), then confirmed visually in a full-page screenshot where this is plainly the faintest text on the homepage. Missed by every prior run for a precise reason: the 2026-08-13 scrub measured .latest-meta ONLY under pointer hover, where `.issue-latest:hover .latest-meta` re-declares `color: var(--bg); opacity: .6` against the cream hover bar and clears at 5.23:1. F83 recorded that number and closed the question. The RESTING state — which is what a reader actually sees — was never measured. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: `.latest-meta` 3.36:1 dark / 2.93:1 light on the homepage, and 3.36:1 again on /brand/. Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | .latest-meta re-measured live 2026-08-25: 3.36:1 dark (homepage + /brand/), 2.93:1 light — unchanged from 2026-08-15. Root cause of the non-closure is NOT the fix: it is that the fix never shipped. origin/main is still b64a39b; the F85 commit (55a6d72) sits on LOCAL main, 8 commits ahead of origin, unpushed for 9 days. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live: .latest-meta 5.13:1 dark / 4.67:1 light, opacity 1 (no stacked multiplier). Also 5.13 on /brand/ dark. | 2026-09-28: live: covered by today's sweeps, 0 failures both modes. | 2026-10-05: live: sweep 0 failures on the homepage standfirst in both modes.</t>
         </is>
       </c>
       <c r="I88" s="6" t="inlineStr">
@@ -5107,7 +5107,7 @@
       </c>
       <c r="H89" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-08-15) — `.hero-corner` sets `color: var(--bg); opacity: .5`. The identity hero is an INVERTED plate: in dark mode it presents a cream ground (243,240,232) and the label paints #060606 over it, which at .5 opacity computes 3.71:1 — under the 4.5:1 floor for 11.52px/700 (bold, but well below the 18.66px large-text threshold). Light mode inverts to cream-on-black and clears at 4.91:1, so this is dark-mode-only. Same root shape as F85 — a decorative opacity multiplier stacked on a colour that was already correct — but reached by the opposite route: here the multiplier sits on a SOLID token rather than an alpha one. Surface resolved by walking to the first opaque ancestor (.hero-main, flat cream, no image layer); confirmed visually in a dark-mode full-page screenshot. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: `.hero-corner` 3.71:1 dark on the homepage, and 3.71:1 again on /brand/. Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | .hero-corner re-measured live 2026-08-25: 3.71:1 dark. Unchanged — fix committed locally (55a6d72), never pushed. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live: .identity-hero .hero-corner 5.23:1 dark / 6.74:1 light at opacity .6. | 2026-09-28: live: covered by today's sweeps, 0 failures both modes.</t>
+          <t>ISSUE/High (2026-08-15) — `.hero-corner` sets `color: var(--bg); opacity: .5`. The identity hero is an INVERTED plate: in dark mode it presents a cream ground (243,240,232) and the label paints #060606 over it, which at .5 opacity computes 3.71:1 — under the 4.5:1 floor for 11.52px/700 (bold, but well below the 18.66px large-text threshold). Light mode inverts to cream-on-black and clears at 4.91:1, so this is dark-mode-only. Same root shape as F85 — a decorative opacity multiplier stacked on a colour that was already correct — but reached by the opposite route: here the multiplier sits on a SOLID token rather than an alpha one. Surface resolved by walking to the first opaque ancestor (.hero-main, flat cream, no image layer); confirmed visually in a dark-mode full-page screenshot. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: `.hero-corner` 3.71:1 dark on the homepage, and 3.71:1 again on /brand/. Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | .hero-corner re-measured live 2026-08-25: 3.71:1 dark. Unchanged — fix committed locally (55a6d72), never pushed. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live: .identity-hero .hero-corner 5.23:1 dark / 6.74:1 light at opacity .6. | 2026-09-28: live: covered by today's sweeps, 0 failures both modes. | 2026-10-05: live: sweep 0 failures on the identity hero in both modes.</t>
         </is>
       </c>
       <c r="I89" s="6" t="inlineStr">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="H90" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-08-15) — /brand/ was still rendering `.latest-tag` at 3.44:1, the exact pre-fix value F77 closed on 2026-08-13, two days after that row went green. Cause: the F77 and F83 dark-mode overrides were written into css/home-v2.css. The homepage loads home-augment.css AND home-v2.css; /brand/ loads home-augment.css and never home-v2.css. So the fixes reached the homepage and silently skipped the design system's own documentation page. This is a broken contract, not a cosmetic gap: brand/index.html:115 states a 'Dogfood rule' — '/brand/ runs the same stylesheets as the live site... If a live component breaks, this page breaks too. That is intentional.' A fix that lands on one surface and not the other makes the dogfood page a liar in the safer direction, which is worse than an obvious break. The F77 comment even asserted it 'Covers the .issue-head hook in home-augment.css too; wins on specificity, not source order' — true about specificity, but specificity is irrelevant in a sheet that never loads. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: /brand/ `.latest-tag` 3.44:1 — and /brand/'s loaded-sheet list confirms the cause directly: tokens, shell, plates, home-augment, article, brand.css, with NO home-v2.css. Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | /brand/ re-measured live 2026-08-25: .latest-tag still 3.44:1 (the pre-F77 value), because live /brand/ serves home-augment.css?v=phase32 which does not yet carry the moved override blocks. The move (55a6d72) is committed locally and confirmed present in a fresh dist build; it has never been pushed. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live: /brand/ loads home-augment.css?v=phase34 (not home-v2); .latest-tag 5.17:1 dark / 5.34:1 light, identical to the homepage — dogfood contract holds. | 2026-09-28: carried: /brand/ loads home-augment.css; sweep 0 failures.</t>
+          <t>ISSUE/High (2026-08-15) — /brand/ was still rendering `.latest-tag` at 3.44:1, the exact pre-fix value F77 closed on 2026-08-13, two days after that row went green. Cause: the F77 and F83 dark-mode overrides were written into css/home-v2.css. The homepage loads home-augment.css AND home-v2.css; /brand/ loads home-augment.css and never home-v2.css. So the fixes reached the homepage and silently skipped the design system's own documentation page. This is a broken contract, not a cosmetic gap: brand/index.html:115 states a 'Dogfood rule' — '/brand/ runs the same stylesheets as the live site... If a live component breaks, this page breaks too. That is intentional.' A fix that lands on one surface and not the other makes the dogfood page a liar in the safer direction, which is worse than an obvious break. The F77 comment even asserted it 'Covers the .issue-head hook in home-augment.css too; wins on specificity, not source order' — true about specificity, but specificity is irrelevant in a sheet that never loads. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: /brand/ `.latest-tag` 3.44:1 — and /brand/'s loaded-sheet list confirms the cause directly: tokens, shell, plates, home-augment, article, brand.css, with NO home-v2.css. Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | /brand/ re-measured live 2026-08-25: .latest-tag still 3.44:1 (the pre-F77 value), because live /brand/ serves home-augment.css?v=phase32 which does not yet carry the moved override blocks. The move (55a6d72) is committed locally and confirmed present in a fresh dist build; it has never been pushed. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live: /brand/ loads home-augment.css?v=phase34 (not home-v2); .latest-tag 5.17:1 dark / 5.34:1 light, identical to the homepage — dogfood contract holds. | 2026-09-28: carried: /brand/ loads home-augment.css; sweep 0 failures. | 2026-10-05: live: /brand/ loads home-augment.css?v=phase40 (not home-v2); sweep 0 failures dark.</t>
         </is>
       </c>
       <c r="I90" s="6" t="inlineStr">
@@ -5221,7 +5221,7 @@
       </c>
       <c r="H91" s="6" t="inlineStr">
         <is>
-          <t>N/A — surface retired | ISSUE/Medium (2026-08-15) — `.next-meta` repeats the F85 defect one notch worse: `color: var(--body-muted)` plus `opacity: .65`, computing 2.81:1 in dark against the 4.5:1 floor. Graded MEDIUM rather than HIGH because it is LATENT — the Issue-next strip only renders when an upcoming essay exists, and all 16 entries are status:published with past dates (see F41/F46), so no reader has hit it. It was found because /brand/ demos the strip under its dogfood rule, which is the same page that exposed F87. Worth recording precisely: this would have shipped broken on the day Dexter scheduled his next essay, and it would have shipped inside the one component whose whole job is to advertise that essay. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: `.next-meta` 2.81:1 dark on the /brand/ dogfood demo (still latent on the live homepage — no upcoming essay exists). Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | .next-meta re-measured on the /brand/ demo of the strip 2026-08-25: still 2.81:1 dark. Unchanged — fix committed locally (55a6d72), never pushed. Still latent on the homepage itself: zero ghost:true flags remain in the collection and no upcoming entry exists, so IssueNext does not render. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: marked N/A per the never-delete rule. The `.issue-next` strip this row measured was deleted in e3b4e91 (IssueNext.astro removed, ~200 lines of .issue-next CSS removed from home-v2.css + home-augment.css). Live: zero `.next-meta` in home-v2.css?v=phase36 / home-augment.css?v=phase34, zero `.issue-next` in the homepage DOM, /brand/ shows only the retirement note. Nothing left to measure; F30 carries the regression watch.</t>
+          <t>N/A — surface retired | ISSUE/Medium (2026-08-15) — `.next-meta` repeats the F85 defect one notch worse: `color: var(--body-muted)` plus `opacity: .65`, computing 2.81:1 in dark against the 4.5:1 floor. Graded MEDIUM rather than HIGH because it is LATENT — the Issue-next strip only renders when an upcoming essay exists, and all 16 entries are status:published with past dates (see F41/F46), so no reader has hit it. It was found because /brand/ demos the strip under its dogfood rule, which is the same page that exposed F87. Worth recording precisely: this would have shipped broken on the day Dexter scheduled his next essay, and it would have shipped inside the one component whose whole job is to advertise that essay. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: `.next-meta` 2.81:1 dark on the /brand/ dogfood demo (still latent on the live homepage — no upcoming essay exists). Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | .next-meta re-measured on the /brand/ demo of the strip 2026-08-25: still 2.81:1 dark. Unchanged — fix committed locally (55a6d72), never pushed. Still latent on the homepage itself: zero ghost:true flags remain in the collection and no upcoming entry exists, so IssueNext does not render. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: marked N/A per the never-delete rule. The `.issue-next` strip this row measured was deleted in e3b4e91 (IssueNext.astro removed, ~200 lines of .issue-next CSS removed from home-v2.css + home-augment.css). Live: zero `.next-meta` in home-v2.css?v=phase36 / home-augment.css?v=phase34, zero `.issue-next` in the homepage DOM, /brand/ shows only the retirement note. Nothing left to measure; F30 carries the regression watch. | 2026-10-05: N/A (surface retired, 0 .issue-next).</t>
         </is>
       </c>
       <c r="I91" s="6" t="inlineStr"/>
@@ -5274,7 +5274,7 @@
       </c>
       <c r="H92" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-08-15) — the `·` separators in the 404 eyebrow carry `opacity: .5`, computing 3.61:1. Unlike the homepage's `.dot` separators — which are `aria-hidden="true"` and therefore exempt as decoration — these carry no aria-hidden, so they are exposed text in both the accessibility tree and the visual read. Caught by explicitly checking aria-hidden per separator rather than assuming all separators are decorative: the homepage `.dot` at 4.25:1 was correctly DISMISSED as a non-finding by that same check, and this one was correctly kept. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: `.notfound-eyebrow span.divider` 3.61:1 on /404. Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | /404 span.divider re-measured live 2026-08-25: still 3.61:1 at opacity .5; live serves notfound.css?v=phase10 (the fix bumps it to phase11). Fix committed locally (8c1e6aa), never pushed. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live: /404 .notfound-eyebrow span.divider 7.19:1 dark / 8.95:1 light; still not aria-hidden (exposed text, in scope). | 2026-09-28: live: 404 0 contrast failures.</t>
+          <t>ISSUE/Medium (2026-08-15) — the `·` separators in the 404 eyebrow carry `opacity: .5`, computing 3.61:1. Unlike the homepage's `.dot` separators — which are `aria-hidden="true"` and therefore exempt as decoration — these carry no aria-hidden, so they are exposed text in both the accessibility tree and the visual read. Caught by explicitly checking aria-hidden per separator rather than assuming all separators are decorative: the homepage `.dot` at 4.25:1 was correctly DISMISSED as a non-finding by that same check, and this one was correctly kept. | 2026-08-16 LIVE RE-CHECK: still failing on production — qa/fixes-20260815 is UNMERGED, so yesterday's fix has not shipped. Re-measured on the live page with the same compositor: `.notfound-eyebrow span.divider` 3.61:1 on /404. Value is identical to the 2026-08-15 reading, which confirms the defect is static and the fix is simply undeployed, not regressed. Row stays ISSUE until a live-verified deploy. | /404 span.divider re-measured live 2026-08-25: still 3.61:1 at opacity .5; live serves notfound.css?v=phase10 (the fix bumps it to phase11). Fix committed locally (8c1e6aa), never pushed. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live: /404 .notfound-eyebrow span.divider 7.19:1 dark / 8.95:1 light; still not aria-hidden (exposed text, in scope). | 2026-09-28: live: 404 0 contrast failures. | 2026-10-05: live: 404 divider opacity .7; sweep 0 failures both modes.</t>
         </is>
       </c>
       <c r="I92" s="6" t="inlineStr">
@@ -5331,7 +5331,7 @@
       </c>
       <c r="H93" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Low (2026-08-15) — five /brand/-only text elements measure under AA in dark mode: `.demo-ghost-meta` ('Coming Soon') 2.05:1, `.demo-ghost-date` 2.45:1, `.demo-ghost-title` 2.93:1 (against its 3:1 large-text floor), `.demo-plate-meta` 3.17:1, and the bespoke 'Download Pack' h3 at 2.87:1. Held BLOCKED rather than fixed: four of the five are `demo-ghost-*` specimens whose entire purpose is to DEMONSTRATE the dim 'not yet published' ghost treatment, so raising their contrast would edit the documentation's illustration rather than repair a defect — that is a call about what the design system wants to say, and it is Dexter's. The fifth ('Download Pack') is bespoke brand.css chrome and is a genuine, if low-traffic, AA miss. Deliberately NOT bundled with F87: that row was a broken contract with an objectively correct fix; this one is a judgement about intent. | 2026-08-16 LIVE RE-CHECK: still open and still BLOCKED — unchanged by design. Re-measured on live /brand/: `.demo-ghost-meta` 2.05:1 and `.demo-plate-meta` 3.17:1 both reproduce exactly. The other three named elements (demo-ghost-date, demo-ghost-title, the 'Download Pack' h3) did not surface in today's sweep because this run only measures elements holding their own text node and not inside an aria-hidden subtree; that is a narrower filter than the 2026-08-15 pass used, not evidence they were fixed. Still NEEDS DEXTER on both questions. | Re-confirmed live 2026-08-25, all five values unchanged: .demo-ghost-meta 2.05:1, .demo-ghost-date 2.45:1, .demo-ghost-title 2.93:1 (vs its 3:1 large-text floor), .demo-plate-meta 3.17:1, and the bespoke "Download Pack" h3 2.87:1 (#ff4d4d on the cream panel). Still BLOCKED — still the same two questions for Dexter, now open 10 days. | 2026-08-27 RE-DIAGNOSED, and the premise of this row was wrong. Four of the five are not documentation-intent choices at all — `.demo-ghost-title/-date/-meta` and `.demo-plate-meta` are faithful mirrors of `.plate-ghost` and `.identity-plate` in css/plates.css, carrying the same tokens and the same opacity multipliers. Composited against their real grounds those production rules measure .plate-title 2.92:1 light / 2.84:1 dark (3:1 large-text floor), .teaser-date 2.06/2.37, `.plate-ghost .meta-rail` 1.80/1.97, and `.identity-plate .meta-rail` 4.14/4.09 (4.5:1 floor) — every one under AA. css/plates.css:377-380 carried a comment asserting these values PASSED ("3.1:1 on #f4f4f1", "3.7:1 on #060606"); both figures are wrong and are what kept the defect invisible. The fifth, the /brand/ 'Download Pack' h3, is worse than recorded: it fails in BOTH modes (2.87:1 dark, 3.46:1 light), not just dark. Separately found: the /brand/ identity specimen had drifted — it used var(--ink)/var(--bg), which invert, so in dark mode it rendered a CREAM identity plate while production deliberately holds #0a0a0a. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live: /brand/ demo specimens clear their floors in both modes — .demo-ghost-meta 5.13/4.67, .demo-ghost-date 5.13/4.67, .demo-ghost-title 3.48/3.33 (44.8px, 3:1 floor), .demo-plate-meta 18.11; full-page sweep 793 elements per mode, 0 failures; img-plate bodies flex/flex-end. | 2026-09-28: live: /brand/ 776 elements, 0 failures both modes.</t>
+          <t>ISSUE/Low (2026-08-15) — five /brand/-only text elements measure under AA in dark mode: `.demo-ghost-meta` ('Coming Soon') 2.05:1, `.demo-ghost-date` 2.45:1, `.demo-ghost-title` 2.93:1 (against its 3:1 large-text floor), `.demo-plate-meta` 3.17:1, and the bespoke 'Download Pack' h3 at 2.87:1. Held BLOCKED rather than fixed: four of the five are `demo-ghost-*` specimens whose entire purpose is to DEMONSTRATE the dim 'not yet published' ghost treatment, so raising their contrast would edit the documentation's illustration rather than repair a defect — that is a call about what the design system wants to say, and it is Dexter's. The fifth ('Download Pack') is bespoke brand.css chrome and is a genuine, if low-traffic, AA miss. Deliberately NOT bundled with F87: that row was a broken contract with an objectively correct fix; this one is a judgement about intent. | 2026-08-16 LIVE RE-CHECK: still open and still BLOCKED — unchanged by design. Re-measured on live /brand/: `.demo-ghost-meta` 2.05:1 and `.demo-plate-meta` 3.17:1 both reproduce exactly. The other three named elements (demo-ghost-date, demo-ghost-title, the 'Download Pack' h3) did not surface in today's sweep because this run only measures elements holding their own text node and not inside an aria-hidden subtree; that is a narrower filter than the 2026-08-15 pass used, not evidence they were fixed. Still NEEDS DEXTER on both questions. | Re-confirmed live 2026-08-25, all five values unchanged: .demo-ghost-meta 2.05:1, .demo-ghost-date 2.45:1, .demo-ghost-title 2.93:1 (vs its 3:1 large-text floor), .demo-plate-meta 3.17:1, and the bespoke "Download Pack" h3 2.87:1 (#ff4d4d on the cream panel). Still BLOCKED — still the same two questions for Dexter, now open 10 days. | 2026-08-27 RE-DIAGNOSED, and the premise of this row was wrong. Four of the five are not documentation-intent choices at all — `.demo-ghost-title/-date/-meta` and `.demo-plate-meta` are faithful mirrors of `.plate-ghost` and `.identity-plate` in css/plates.css, carrying the same tokens and the same opacity multipliers. Composited against their real grounds those production rules measure .plate-title 2.92:1 light / 2.84:1 dark (3:1 large-text floor), .teaser-date 2.06/2.37, `.plate-ghost .meta-rail` 1.80/1.97, and `.identity-plate .meta-rail` 4.14/4.09 (4.5:1 floor) — every one under AA. css/plates.css:377-380 carried a comment asserting these values PASSED ("3.1:1 on #f4f4f1", "3.7:1 on #060606"); both figures are wrong and are what kept the defect invisible. The fifth, the /brand/ 'Download Pack' h3, is worse than recorded: it fails in BOTH modes (2.87:1 dark, 3.46:1 light), not just dark. Separately found: the /brand/ identity specimen had drifted — it used var(--ink)/var(--bg), which invert, so in dark mode it rendered a CREAM identity plate while production deliberately holds #0a0a0a. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live: /brand/ demo specimens clear their floors in both modes — .demo-ghost-meta 5.13/4.67, .demo-ghost-date 5.13/4.67, .demo-ghost-title 3.48/3.33 (44.8px, 3:1 floor), .demo-plate-meta 18.11; full-page sweep 793 elements per mode, 0 failures; img-plate bodies flex/flex-end. | 2026-09-28: live: /brand/ 776 elements, 0 failures both modes. | 2026-10-05: live: /brand/ sweep 0 failures dark; light-mode readings are the image-plate artifact only (geometry checked).</t>
         </is>
       </c>
       <c r="I93" s="6" t="inlineStr">
@@ -5388,7 +5388,7 @@
       </c>
       <c r="H94" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-08-16) — /phase0/'s skip link, the first focusable element on the page, computed `color: rgba(243,240,232,.82)` on its own `background: var(--ink)` cream chip: 1.00:1. This is the worst ratio the ledger has recorded and the only finding to date where the text is not merely low-contrast but literally invisible — a sighted keyboard user sees the accent focus ring land on a blank cream box. NOT a colour bug: `--bg` resolves correctly to #060606 at every level of the chain (verified by walking the ancestor chain: A.skip-link / BODY.phase0 / HTML.dark-mode all report #060606). It is a specificity bug. Three rules set colour on this element — `a {color:inherit}` (0,0,1) in tokens.css, `.skip-link {color:var(--bg)}` (0,1,0) in shell.css, and `.phase0 a {color:inherit}` (0,1,1) in phase0.css. The last wins on specificity and hands the chip back the inherited body cream. Scope is exactly one page: /brand/, the other bespoke-CSS surface, carries no blanket `a` rule and measured clean. Missed by every prior run because the skip link sits at left:-999px in its resting state, so a sweep that filters to on-screen elements never measures it — this run caught it by measuring every element with layout geometry regardless of viewport position. | /phase0/ skip link re-measured live 2026-08-25: still rgba(243,240,232,.82) on its own cream chip = 1.00:1, the worst ratio in the ledger and still literally invisible to a sighted keyboard user. Live serves shell.css?v=phase23; the hardened selector ships as phase36. Fix committed locally (79df261), never pushed. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live under a real shift+Tab: /phase0/ skip link is first focusable, rgb(6,6,6) on rgb(243,240,232) = 17.79:1 dark; light rgb(244,244,241) on rgb(5,5,5); 2px #c00 ring. Homepage skip link same, activation lands focus on MAIN#archive. | 2026-09-28: carried: skip-link rule unchanged; home skip link verified under real Tab.</t>
+          <t>ISSUE/High (2026-08-16) — /phase0/'s skip link, the first focusable element on the page, computed `color: rgba(243,240,232,.82)` on its own `background: var(--ink)` cream chip: 1.00:1. This is the worst ratio the ledger has recorded and the only finding to date where the text is not merely low-contrast but literally invisible — a sighted keyboard user sees the accent focus ring land on a blank cream box. NOT a colour bug: `--bg` resolves correctly to #060606 at every level of the chain (verified by walking the ancestor chain: A.skip-link / BODY.phase0 / HTML.dark-mode all report #060606). It is a specificity bug. Three rules set colour on this element — `a {color:inherit}` (0,0,1) in tokens.css, `.skip-link {color:var(--bg)}` (0,1,0) in shell.css, and `.phase0 a {color:inherit}` (0,1,1) in phase0.css. The last wins on specificity and hands the chip back the inherited body cream. Scope is exactly one page: /brand/, the other bespoke-CSS surface, carries no blanket `a` rule and measured clean. Missed by every prior run because the skip link sits at left:-999px in its resting state, so a sweep that filters to on-screen elements never measures it — this run caught it by measuring every element with layout geometry regardless of viewport position. | /phase0/ skip link re-measured live 2026-08-25: still rgba(243,240,232,.82) on its own cream chip = 1.00:1, the worst ratio in the ledger and still literally invisible to a sighted keyboard user. Live serves shell.css?v=phase23; the hardened selector ships as phase36. Fix committed locally (79df261), never pushed. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-25: re-verified live under a real shift+Tab: /phase0/ skip link is first focusable, rgb(6,6,6) on rgb(243,240,232) = 17.79:1 dark; light rgb(244,244,241) on rgb(5,5,5); 2px #c00 ring. Homepage skip link same, activation lands focus on MAIN#archive. | 2026-09-28: carried: skip-link rule unchanged; home skip link verified under real Tab. | 2026-10-05: live: /phase0/ skip link inverted chip rgb(6,6,6) on rgb(243,240,232) in dark; sweep 0 failures both modes.</t>
         </is>
       </c>
       <c r="I94" s="6" t="inlineStr">
@@ -5445,7 +5445,7 @@
       </c>
       <c r="H95" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Low (2026-08-27) — the click handler rewrote the label and the count but never touched the glyph. Live on b64a39b the expanded state reads 'Show Less — showing all ↓': the arrow still points down, i.e. 'more below', while the button's own words say it will collapse. The glyph carries aria-hidden="true" so nothing is exposed to assistive tech — this is a purely visual affordance contradiction, which is why it survived every prior scrub. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-01 re-verified live: .btn-glyph tracks the button state — down-arrow collapsed, up-arrow expanded, and back. | 2026-09-11 re-verified live: glyph tracks state live — ↓ at 7 shown, ↑ at 17 shown, back to ↓; still aria-hidden. | 2026-09-19 re-verified live: View Earlier toggle: 7 shown / aria-expanded false / ↓ → 17 shown / true / ↑ → back to 7 / false. | 2026-09-25: re-verified live: 7 shown / aria-expanded false / ↓ → 17 shown / true / ↑ → back to 7 / false; glyph aria-hidden. | 2026-09-28: live: glyph ↓ collapsed / ↑ expanded tracks the label.</t>
+          <t>ISSUE/Low (2026-08-27) — the click handler rewrote the label and the count but never touched the glyph. Live on b64a39b the expanded state reads 'Show Less — showing all ↓': the arrow still points down, i.e. 'more below', while the button's own words say it will collapse. The glyph carries aria-hidden="true" so nothing is exposed to assistive tech — this is a purely visual affordance contradiction, which is why it survived every prior scrub. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-01 re-verified live: .btn-glyph tracks the button state — down-arrow collapsed, up-arrow expanded, and back. | 2026-09-11 re-verified live: glyph tracks state live — ↓ at 7 shown, ↑ at 17 shown, back to ↓; still aria-hidden. | 2026-09-19 re-verified live: View Earlier toggle: 7 shown / aria-expanded false / ↓ → 17 shown / true / ↑ → back to 7 / false. | 2026-09-25: re-verified live: 7 shown / aria-expanded false / ↓ → 17 shown / true / ↑ → back to 7 / false; glyph aria-hidden. | 2026-09-28: live: glyph ↓ collapsed / ↑ expanded tracks the label. | 2026-10-05: live: glyph ↓ collapsed, ↑ expanded.</t>
         </is>
       </c>
       <c r="I95" s="6" t="inlineStr">
@@ -5502,7 +5502,7 @@
       </c>
       <c r="H96" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-08-27) — both class names are DEAD in production. `Plate.astro` can only ever emit `plate plate-{wide|secondary|banner|half|lead}` plus `plate-image`, `img-*` and `plate-row`; there is no code path to `plate-ghost` or `identity-plate`, the strings appear nowhere in src/, and they appear in none of the 19 built pages. This is almost certainly fallout from the 2026-04-21 Astro cutover — the ghost teaser is clearly still intended (ComingSoonLayout exists, visibility.ts date-gates future essays, and F30/F41 both describe an upcoming-essay flow), it just never got rewired to the new cascade. Two consequences: css/plates.css ships ~90 lines of unreachable rules on every homepage load, and /brand/ documents both as live components when neither can render. Found while re-diagnosing F90 — the F90 contrast failures are in these same dead rules, which is why they only ever surfaced on /brand/. | Dexter chose REWIRE over retire, 2026-08-27. | RESOLVED 2026-08-27 — see p4. | CORRECTION 2026-08-27: this row was closed as 'fixed' while it named TWO orphaned components and only ONE was rewired. `.plate-ghost` has an emitter now; `.identity-plate` still has none — no occurrence anywhere in src/, zero in the 19 built pages. F93 is hereby narrowed to the ghost plate, which is genuinely fixed, and the identity-plate half is split out to F95 so it is not buried under a green row. My closure, my error. | 2026-09-25: static re-check: GhostPlate.astro still emits .plate-ghost; plates.css?v=phase39 carries the rules. Live render still untestable (0 upcoming entries), so no live claim. | 2026-09-28: build-verified via fixture: .plate-ghost renders with .plate-title == fixture title and .teaser-date &lt;time 2027-01-15&gt; == publishedDate.</t>
+          <t>ISSUE/Medium (2026-08-27) — both class names are DEAD in production. `Plate.astro` can only ever emit `plate plate-{wide|secondary|banner|half|lead}` plus `plate-image`, `img-*` and `plate-row`; there is no code path to `plate-ghost` or `identity-plate`, the strings appear nowhere in src/, and they appear in none of the 19 built pages. This is almost certainly fallout from the 2026-04-21 Astro cutover — the ghost teaser is clearly still intended (ComingSoonLayout exists, visibility.ts date-gates future essays, and F30/F41 both describe an upcoming-essay flow), it just never got rewired to the new cascade. Two consequences: css/plates.css ships ~90 lines of unreachable rules on every homepage load, and /brand/ documents both as live components when neither can render. Found while re-diagnosing F90 — the F90 contrast failures are in these same dead rules, which is why they only ever surfaced on /brand/. | Dexter chose REWIRE over retire, 2026-08-27. | RESOLVED 2026-08-27 — see p4. | CORRECTION 2026-08-27: this row was closed as 'fixed' while it named TWO orphaned components and only ONE was rewired. `.plate-ghost` has an emitter now; `.identity-plate` still has none — no occurrence anywhere in src/, zero in the 19 built pages. F93 is hereby narrowed to the ghost plate, which is genuinely fixed, and the identity-plate half is split out to F95 so it is not buried under a green row. My closure, my error. | 2026-09-25: static re-check: GhostPlate.astro still emits .plate-ghost; plates.css?v=phase39 carries the rules. Live render still untestable (0 upcoming entries), so no live claim. | 2026-09-28: build-verified via fixture: .plate-ghost renders with .plate-title == fixture title and .teaser-date &lt;time 2027-01-15&gt; == publishedDate. | 2026-10-05: fixture build: .plate-ghost renders, .plate-title == fixture title, .teaser-date &lt;time 2027-01-15&gt;, no href.</t>
         </is>
       </c>
       <c r="I96" s="6" t="inlineStr">
@@ -5559,7 +5559,7 @@
       </c>
       <c r="H97" s="6" t="inlineStr">
         <is>
-          <t>N/A by decision (2026-08-27) — not a defect. Dexter's call after seeing F93 ship: the ghost plate and the IssueNext strip are two presentations of the same upcoming essay, so with both live the title appeared on the homepage twice. The plate wins. | 2026-09-25: still N/A by decision. Note: the expected column's "component and CSS stay intact" was overtaken the same day by e3b4e91, which deleted IssueNext.astro and its CSS; reversal now means restoring from git (121a621), not a one-line flip. Live: 0 .issue-next in DOM/CSS. | 2026-09-28: build-verified via fixture: ghost plate rendered, .issue-next count 0.</t>
+          <t>N/A by decision (2026-08-27) — not a defect. Dexter's call after seeing F93 ship: the ghost plate and the IssueNext strip are two presentations of the same upcoming essay, so with both live the title appeared on the homepage twice. The plate wins. | 2026-09-25: still N/A by decision. Note: the expected column's "component and CSS stay intact" was overtaken the same day by e3b4e91, which deleted IssueNext.astro and its CSS; reversal now means restoring from git (121a621), not a one-line flip. Live: 0 .issue-next in DOM/CSS. | 2026-09-28: build-verified via fixture: ghost plate rendered, .issue-next count 0. | 2026-10-05: fixture build: ghost plate shown, 0 .issue-next.</t>
         </is>
       </c>
       <c r="I97" s="6" t="inlineStr"/>
@@ -5612,7 +5612,7 @@
       </c>
       <c r="H98" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-08-27) — SPLIT FROM F93, WHICH I CLOSED TOO BROADLY. F93 named two orphaned components; Dexter asked for the ghost plate to be rewired and it was, but `.identity-plate` was never in scope and is still dead. Re-verified today: the string appears nowhere in src/ and in none of the 19 built pages, because Plate.astro can only emit plate-{wide|secondary|banner|half|lead} plus plate-image/img-*/plate-row. css/plates.css ships ~85 lines of unreachable rules on every homepage load, and /brand/ documents the plate as live. Note this is NOT the same thing as `.identity-hero`, which does render on the homepage and is fine (F21). Contrast is not at issue — F90 already lifted `.identity-plate .meta-rail` to 5.77/5.63 — this is purely reachability. | RESOLVED 2026-08-28 — Dexter chose retire. See p4. | 2026-09-26 re-verified: css/plates.css carries zero live .identity-plate rules (only the retirement comment at :270) and brand/index.html documents no .identity-plate specimen; the homepage's identity surface is IdentityHero via src/pages/index.astro — retirement holds. | 2026-09-28: carried: source unchanged.</t>
+          <t>ISSUE/Medium (2026-08-27) — SPLIT FROM F93, WHICH I CLOSED TOO BROADLY. F93 named two orphaned components; Dexter asked for the ghost plate to be rewired and it was, but `.identity-plate` was never in scope and is still dead. Re-verified today: the string appears nowhere in src/ and in none of the 19 built pages, because Plate.astro can only emit plate-{wide|secondary|banner|half|lead} plus plate-image/img-*/plate-row. css/plates.css ships ~85 lines of unreachable rules on every homepage load, and /brand/ documents the plate as live. Note this is NOT the same thing as `.identity-hero`, which does render on the homepage and is fine (F21). Contrast is not at issue — F90 already lifted `.identity-plate .meta-rail` to 5.77/5.63 — this is purely reachability. | RESOLVED 2026-08-28 — Dexter chose retire. See p4. | 2026-09-26 re-verified: css/plates.css carries zero live .identity-plate rules (only the retirement comment at :270) and brand/index.html documents no .identity-plate specimen; the homepage's identity surface is IdentityHero via src/pages/index.astro — retirement holds. | 2026-09-28: carried: source unchanged. | 2026-10-05: repo: plates.css carries only the retirement comment; 0 .identity-plate live.</t>
         </is>
       </c>
       <c r="I98" s="6" t="inlineStr">
@@ -5669,7 +5669,7 @@
       </c>
       <c r="H99" s="6" t="inlineStr">
         <is>
-          <t>PASS (2026-08-31, live on 13b631c then 83c2137) — POST-gate half verified live end to end: article 200 with 55 paragraphs and zero coming-soon markers; present in sitemap-0.xml, feed.xml and the homepage cascade (latest strip, lead plate, 'Week of August 31, 2026'); 'Send Someone Else' renders 0 .article-nav-ghost, i.e. the ghost treatment retired itself on go-live exactly as designed. OG plate 1200x630 (1.905), reads VOL 17 matching the essay's own number, title clears Anton's caps on the .92 leading from 9301d61. Metadata complete (description, og:title/image/image:alt/type, twitter:summary_large_image, canonical). Redate to Aug 31 propagated to every surface: JSON-LD datePublished 2026-08-31T12:00:00-05:00, Atom &lt;published&gt; 2026-08-31T17:00:00Z, homepage &lt;time datetime="2026-08-31"&gt;, zero 'Aug 30' anywhere live. Contrast 87 elements / 0 failures in BOTH modes (dark floor 5.13:1, light 4.67:1). Single h1, h1-&gt;h2 with no skipped level, skip link takes first Tab with a visible ring, 0 unnamed interactive elements, 0 console errors. || PRE-gate half NOT verified in production — see F93/F94: the release sat unpushed from Aug 29 until after the Aug 30 noon gate, so the Coming-Soon route never rendered on the live site for this essay. | 2026-09-01 re-verified live: VOL 17 present and correct across article (200), homepage lead plate, feed (17/17), sitemap and OG plate; article:published_time 2026-08-31 matches the homepage plate's &lt;time datetime&gt;. | 2026-09-26 re-verified live: /words/the-weight-of-my-no/ renders the full ArticleLayout (no 'Coming Soon', no noindex), sits in feed.xml (17 entries), sitemap-0.xml (21 locs) and the homepage cascade; 'Send Someone Else' carries a real rel=next .article-nav-next link to it, no ghost. | 2026-09-28: live: the-weight-of-my-no in cascade (lead), feed and sitemap.</t>
+          <t>PASS (2026-08-31, live on 13b631c then 83c2137) — POST-gate half verified live end to end: article 200 with 55 paragraphs and zero coming-soon markers; present in sitemap-0.xml, feed.xml and the homepage cascade (latest strip, lead plate, 'Week of August 31, 2026'); 'Send Someone Else' renders 0 .article-nav-ghost, i.e. the ghost treatment retired itself on go-live exactly as designed. OG plate 1200x630 (1.905), reads VOL 17 matching the essay's own number, title clears Anton's caps on the .92 leading from 9301d61. Metadata complete (description, og:title/image/image:alt/type, twitter:summary_large_image, canonical). Redate to Aug 31 propagated to every surface: JSON-LD datePublished 2026-08-31T12:00:00-05:00, Atom &lt;published&gt; 2026-08-31T17:00:00Z, homepage &lt;time datetime="2026-08-31"&gt;, zero 'Aug 30' anywhere live. Contrast 87 elements / 0 failures in BOTH modes (dark floor 5.13:1, light 4.67:1). Single h1, h1-&gt;h2 with no skipped level, skip link takes first Tab with a visible ring, 0 unnamed interactive elements, 0 console errors. || PRE-gate half NOT verified in production — see F93/F94: the release sat unpushed from Aug 29 until after the Aug 30 noon gate, so the Coming-Soon route never rendered on the live site for this essay. | 2026-09-01 re-verified live: VOL 17 present and correct across article (200), homepage lead plate, feed (17/17), sitemap and OG plate; article:published_time 2026-08-31 matches the homepage plate's &lt;time datetime&gt;. | 2026-09-26 re-verified live: /words/the-weight-of-my-no/ renders the full ArticleLayout (no 'Coming Soon', no noindex), sits in feed.xml (17 entries), sitemap-0.xml (21 locs) and the homepage cascade; 'Send Someone Else' carries a real rel=next .article-nav-next link to it, no ghost. | 2026-09-28: live: the-weight-of-my-no in cascade (lead), feed and sitemap. | 2026-10-05: live: the-weight-of-my-no full article, in feed, sitemap and cascade (lead).</t>
         </is>
       </c>
       <c r="I99" s="6" t="inlineStr"/>
@@ -5714,7 +5714,7 @@
       </c>
       <c r="H100" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-08-31) — .article-eyebrow shipped flex-wrap: nowrap with no mobile override, so the rail runs off the frame on every article. Measured LIVE at 375px on /words/the-weight-of-my-no/ (6 chips: 2 lanes + 2 tags + date + read-time): scrollWidth 406 vs clientWidth 362 = 105px overflow; .article-read sits at left:418 against a 375px viewport, i.e. '8 min' is 100% invisible and 'Aug 31, 2026' is 92% clipped. Control /words/send-someone-else/ (5 chips) overflows 39px and loses 2px of '16 min', confirming this is site-wide and pre-existing rather than introduced by VOL 17 — VOL 17 is simply the worst case, being the first 6-chip essay. Because body/.page-shell are overflow-x: clip there is no scrollbar and no gesture that reaches the clipped text. Survived every prior scrub because source-only inspection cannot see it: the CSS is valid, the defect only exists once the flex row is laid out under 760px. | 2026-09-06 re-verified live: holds live - eyebrow wraps at 375px with zero overflow. | 2026-09-11 re-verified live: 375px /words/the-weight-of-my-no/: .article-eyebrow computes flex-wrap: wrap, all six chips inside the frame (rightmost 331px), documentElement.scrollWidth == clientWidth == 375. | 2026-09-19 re-verified live: 375px /words/the-weight-of-my-no/: .article-eyebrow flex-wrap: wrap, rightmost chip at 331px, scrollWidth == clientWidth == 375. | 2026-09-26 re-verified live at 375x812: .article-eyebrow is flex-wrap: wrap and 0 children overflow the viewport on /about/ and all 17 articles; no document-level horizontal overflow on any of the 18. | 2026-09-28: live at 390px: .article-eyebrow wraps inside the frame (right edge 353px of 390), 0 overflow.</t>
+          <t>ISSUE/High (2026-08-31) — .article-eyebrow shipped flex-wrap: nowrap with no mobile override, so the rail runs off the frame on every article. Measured LIVE at 375px on /words/the-weight-of-my-no/ (6 chips: 2 lanes + 2 tags + date + read-time): scrollWidth 406 vs clientWidth 362 = 105px overflow; .article-read sits at left:418 against a 375px viewport, i.e. '8 min' is 100% invisible and 'Aug 31, 2026' is 92% clipped. Control /words/send-someone-else/ (5 chips) overflows 39px and loses 2px of '16 min', confirming this is site-wide and pre-existing rather than introduced by VOL 17 — VOL 17 is simply the worst case, being the first 6-chip essay. Because body/.page-shell are overflow-x: clip there is no scrollbar and no gesture that reaches the clipped text. Survived every prior scrub because source-only inspection cannot see it: the CSS is valid, the defect only exists once the flex row is laid out under 760px. | 2026-09-06 re-verified live: holds live - eyebrow wraps at 375px with zero overflow. | 2026-09-11 re-verified live: 375px /words/the-weight-of-my-no/: .article-eyebrow computes flex-wrap: wrap, all six chips inside the frame (rightmost 331px), documentElement.scrollWidth == clientWidth == 375. | 2026-09-19 re-verified live: 375px /words/the-weight-of-my-no/: .article-eyebrow flex-wrap: wrap, rightmost chip at 331px, scrollWidth == clientWidth == 375. | 2026-09-26 re-verified live at 375x812: .article-eyebrow is flex-wrap: wrap and 0 children overflow the viewport on /about/ and all 17 articles; no document-level horizontal overflow on any of the 18. | 2026-09-28: live at 390px: .article-eyebrow wraps inside the frame (right edge 353px of 390), 0 overflow. | 2026-10-05: live: .article-eyebrow flex-wrap: wrap; 375px article has 0 overflowing elements.</t>
         </is>
       </c>
       <c r="I100" s="6" t="inlineStr">
@@ -5771,7 +5771,7 @@
       </c>
       <c r="H101" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-09-02) — `.skip-link` had NO :focus-visible rule anywhere in the loaded cascade. Enumerated every rule matching /skip-link/ across all loaded sheets on live: exactly two hits, both in shell.css (the (0,2,0) :link/:visited base chip from F91, and .skip-link:focus for positioning) — neither carries an outline. Measured under a REAL Tab press on the live homepage with the chip focused: outline `rgb(153,200,255) auto 1px` — Chrome's UA default — while every sibling control measured the same way paints `rgb(204,0,0) solid 2px` (.brand-block, .mode-toggle, a.plate, .issue-standfirst, .hero-link, .sm-submit all confirmed this run). Confirmed identical on /about/ (shared shell.css, skipFocusRule:false). NOT a WCAG 2.4.7 failure — the UA ring is visible, which is exactly why five months of contrast-led sweeps never surfaced it — but a design-token break on the first element a keyboard user ever focuses. Same defect class as F76 (.sm-submit, closed 2026-08-10); this is a distinct element that rule never covered, not a regression of it. | 2026-09-06 re-verified live: still open ON LIVE, as expected - the fix is on this branch and unmerged. Live skip link focuses with the Chrome default ring (outline rgb(153,200,255) auto 1px) instead of the site's red --focus-ring. Closes on merge. | 2026-09-11 re-verified live: .skip-link:focus-visible rule present in shell.css?v=phase38 alongside .mode-toggle/.brand-block/.footer-strip a; measured live as outline rgb(204,0,0) solid 2px under a real Tab. | 2026-09-19 re-verified live: .skip-link measured under a real shift+Tab: outline rgb(204,0,0) solid 2px. | 2026-09-26 re-verified live under a REAL shift+Tab on /words/the-stone/: .skip-link matches :focus-visible and paints solid 2px rgb(204,0,0), offset 2px; forward Tab continues to .brand-block and .mode-toggle, both 2px #c00. Skip-link activation (el.click) sets #article and the target exists. | 2026-09-28: live: skip link :focus-visible 2px solid #c00 under real Tab.</t>
+          <t>ISSUE/Medium (2026-09-02) — `.skip-link` had NO :focus-visible rule anywhere in the loaded cascade. Enumerated every rule matching /skip-link/ across all loaded sheets on live: exactly two hits, both in shell.css (the (0,2,0) :link/:visited base chip from F91, and .skip-link:focus for positioning) — neither carries an outline. Measured under a REAL Tab press on the live homepage with the chip focused: outline `rgb(153,200,255) auto 1px` — Chrome's UA default — while every sibling control measured the same way paints `rgb(204,0,0) solid 2px` (.brand-block, .mode-toggle, a.plate, .issue-standfirst, .hero-link, .sm-submit all confirmed this run). Confirmed identical on /about/ (shared shell.css, skipFocusRule:false). NOT a WCAG 2.4.7 failure — the UA ring is visible, which is exactly why five months of contrast-led sweeps never surfaced it — but a design-token break on the first element a keyboard user ever focuses. Same defect class as F76 (.sm-submit, closed 2026-08-10); this is a distinct element that rule never covered, not a regression of it. | 2026-09-06 re-verified live: still open ON LIVE, as expected - the fix is on this branch and unmerged. Live skip link focuses with the Chrome default ring (outline rgb(153,200,255) auto 1px) instead of the site's red --focus-ring. Closes on merge. | 2026-09-11 re-verified live: .skip-link:focus-visible rule present in shell.css?v=phase38 alongside .mode-toggle/.brand-block/.footer-strip a; measured live as outline rgb(204,0,0) solid 2px under a real Tab. | 2026-09-19 re-verified live: .skip-link measured under a real shift+Tab: outline rgb(204,0,0) solid 2px. | 2026-09-26 re-verified live under a REAL shift+Tab on /words/the-stone/: .skip-link matches :focus-visible and paints solid 2px rgb(204,0,0), offset 2px; forward Tab continues to .brand-block and .mode-toggle, both 2px #c00. Skip-link activation (el.click) sets #article and the target exists. | 2026-09-28: live: skip link :focus-visible 2px solid #c00 under real Tab. | 2026-10-05: live: real Tab focus on .skip-link paints 2px #c00 outline, 2px offset.</t>
         </is>
       </c>
       <c r="I101" s="6" t="inlineStr">
@@ -5828,7 +5828,7 @@
       </c>
       <c r="H102" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-09-02) — /brand/ was pinning `article.css?v=phase24` while the three src/ references sat at phase37, live-confirmed by reading document.styleSheets on both pages: /brand/ loaded article.css?v=phase24, /words/the-stone/ loaded article.css?v=phase37. article.css moved phase24 -&gt; phase37 in 558aa07 (the F97 eyebrow wrap, merged as f8d7702 on 2026-08-31); that commit bumped three references and missed the fourth. Effect: /css/* is immutable/1y, so any reader who had loaded /brand/ before that bump keeps the pre-F97 sheet on the design-system page for up to a year, while every article page serves the fixed one — the documentation surface silently disagreeing with the site it documents. Same contract as F87 (closed 2026-08-27), different mechanism: F87 was the fix landing in a sheet /brand/ does not load; this is /brand/ loading the right sheet at a stale key. Root cause is structural: the passthrough references sit outside src/, so both the bump sweep and DESIGN-SYSTEM.md's own high-water-mark grep (scoped `src/`) are blind to them — and the doc, written one day earlier in 885930e specifically to codify this rule, itself counted article.css at three references instead of four. | 2026-09-11 re-verified live: /brand/ loads article.css?v=phase37, shell.css?v=phase38, plates.css?v=phase39, brand.css?v=brand10 — the same versions the rest of the site loads. Parity holds. | 2026-09-26 re-verified: every /css/*.css reference across src/, brand/ and phase0/ carries one ?v= per filename (tokens phase24 x7, shell phase38 x7, article phase37 x4, plates phase39 x2, home-augment phase40 x2, home-v2 phase36, notfound phase11, phase0 phase2) — zero parity splits on this branch. | 2026-09-28: repo: one ?v= per sheet across layouts + passthroughs (8 sheets). phase0.js bumped phase2 -&gt; phase3 with today's F53 fix (its only reference).</t>
+          <t>ISSUE/Medium (2026-09-02) — /brand/ was pinning `article.css?v=phase24` while the three src/ references sat at phase37, live-confirmed by reading document.styleSheets on both pages: /brand/ loaded article.css?v=phase24, /words/the-stone/ loaded article.css?v=phase37. article.css moved phase24 -&gt; phase37 in 558aa07 (the F97 eyebrow wrap, merged as f8d7702 on 2026-08-31); that commit bumped three references and missed the fourth. Effect: /css/* is immutable/1y, so any reader who had loaded /brand/ before that bump keeps the pre-F97 sheet on the design-system page for up to a year, while every article page serves the fixed one — the documentation surface silently disagreeing with the site it documents. Same contract as F87 (closed 2026-08-27), different mechanism: F87 was the fix landing in a sheet /brand/ does not load; this is /brand/ loading the right sheet at a stale key. Root cause is structural: the passthrough references sit outside src/, so both the bump sweep and DESIGN-SYSTEM.md's own high-water-mark grep (scoped `src/`) are blind to them — and the doc, written one day earlier in 885930e specifically to codify this rule, itself counted article.css at three references instead of four. | 2026-09-11 re-verified live: /brand/ loads article.css?v=phase37, shell.css?v=phase38, plates.css?v=phase39, brand.css?v=brand10 — the same versions the rest of the site loads. Parity holds. | 2026-09-26 re-verified: every /css/*.css reference across src/, brand/ and phase0/ carries one ?v= per filename (tokens phase24 x7, shell phase38 x7, article phase37 x4, plates phase39 x2, home-augment phase40 x2, home-v2 phase36, notfound phase11, phase0 phase2) — zero parity splits on this branch. | 2026-09-28: repo: one ?v= per sheet across layouts + passthroughs (8 sheets). phase0.js bumped phase2 -&gt; phase3 with today's F53 fix (its only reference). | 2026-10-05: repo: cache-bust parity holds for all 8 sheets across src/, brand/ and phase0/.</t>
         </is>
       </c>
       <c r="I102" s="6" t="inlineStr">
@@ -5885,7 +5885,7 @@
       </c>
       <c r="H103" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-09-05) — `.demo-plate-body` had `flex: 1` but no `display: flex`, so the `justify-content: flex-end` written for `.demo-plate.img-plate .demo-plate-body` was inert and every white specimen title rendered at the TOP of its plate (measured live: titleTopFrac 0.11, titleBotFrac 0.24-0.38 on all five). The `::after` overlay is `linear-gradient(to top, rgba(0,0,0,.78), rgba(0,0,0,.08) 55%, rgba(0,0,0,.14))` — near-opaque at the bottom, ~.12 alpha at the title's actual position — so the titles sat over the LIGHT end of the concrete texture instead of the dark end. Pixel-measured (headless Chrome 1280px, real CSS, glyph-free sample strip inside the plate at the title's own y-band): the `concrete` specimens' title band runs rgb(98)-rgb(160), giving white-on-lightest 2.61:1 and white-on-median 3.03:1 against a 3:1 large-text floor (25.6px bold Anton). `lines` measured 4.12:1 and `noise` 18.1:1 at the same position, so the failure is texture-dependent — concrete is the light one — but all five were in the wrong band. Not caught by earlier sweeps because a computed-style probe walks the ancestor `background-color` chain straight through both pseudo-elements and reports the page ground (1.06:1) for every one of them, which reads exactly like the known `.plate-image` measurement artifact and was dismissed as such. It is not that artifact: on `.plate-image` the title genuinely sits in the .78 band; here the mirror had lost the rule that puts it there. Same contract as F87/F90 — /brand/ failing to dogfood — third distinct mechanism: F87 was the fix landing in a sheet /brand/ does not load, F99 was /brand/ loading the right sheet at a stale key, this is /brand/ loading the right sheet at the right key with a rule the production component has and the specimen does not. | 2026-09-11 re-verified live: all five .demo-plate.img-plate .demo-plate-body report display:flex / justify-content:flex-end; titles bottom-anchored at topFrac 0.52–0.79. Fix holds. | 2026-09-19 re-verified live: all five /brand/ .demo-plate.img-plate .demo-plate-body compute display:flex / justify-content:flex-end. | 2026-09-26 re-verified live on /brand/: all 5 .img-plate .demo-plate-body are display:flex + justify-content:flex-end, titles sit at 0.69-0.82 of plate height, ::after scrim present (to top .78 -&gt; .26 55% -&gt; ...). | 2026-09-28: live: .demo-plate-body flex / flex-end.</t>
+          <t>ISSUE/Medium (2026-09-05) — `.demo-plate-body` had `flex: 1` but no `display: flex`, so the `justify-content: flex-end` written for `.demo-plate.img-plate .demo-plate-body` was inert and every white specimen title rendered at the TOP of its plate (measured live: titleTopFrac 0.11, titleBotFrac 0.24-0.38 on all five). The `::after` overlay is `linear-gradient(to top, rgba(0,0,0,.78), rgba(0,0,0,.08) 55%, rgba(0,0,0,.14))` — near-opaque at the bottom, ~.12 alpha at the title's actual position — so the titles sat over the LIGHT end of the concrete texture instead of the dark end. Pixel-measured (headless Chrome 1280px, real CSS, glyph-free sample strip inside the plate at the title's own y-band): the `concrete` specimens' title band runs rgb(98)-rgb(160), giving white-on-lightest 2.61:1 and white-on-median 3.03:1 against a 3:1 large-text floor (25.6px bold Anton). `lines` measured 4.12:1 and `noise` 18.1:1 at the same position, so the failure is texture-dependent — concrete is the light one — but all five were in the wrong band. Not caught by earlier sweeps because a computed-style probe walks the ancestor `background-color` chain straight through both pseudo-elements and reports the page ground (1.06:1) for every one of them, which reads exactly like the known `.plate-image` measurement artifact and was dismissed as such. It is not that artifact: on `.plate-image` the title genuinely sits in the .78 band; here the mirror had lost the rule that puts it there. Same contract as F87/F90 — /brand/ failing to dogfood — third distinct mechanism: F87 was the fix landing in a sheet /brand/ does not load, F99 was /brand/ loading the right sheet at a stale key, this is /brand/ loading the right sheet at the right key with a rule the production component has and the specimen does not. | 2026-09-11 re-verified live: all five .demo-plate.img-plate .demo-plate-body report display:flex / justify-content:flex-end; titles bottom-anchored at topFrac 0.52–0.79. Fix holds. | 2026-09-19 re-verified live: all five /brand/ .demo-plate.img-plate .demo-plate-body compute display:flex / justify-content:flex-end. | 2026-09-26 re-verified live on /brand/: all 5 .img-plate .demo-plate-body are display:flex + justify-content:flex-end, titles sit at 0.69-0.82 of plate height, ::after scrim present (to top .78 -&gt; .26 55% -&gt; ...). | 2026-09-28: live: .demo-plate-body flex / flex-end. | 2026-10-05: live: .demo-plate-body display flex / justify-content flex-end.</t>
         </is>
       </c>
       <c r="I103" s="6" t="inlineStr">
@@ -5942,7 +5942,7 @@
       </c>
       <c r="H104" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-09-06) — the scrim is `linear-gradient(to top, rgba(0,0,0,.78), rgba(0,0,0,.08) 55%, rgba(0,0,0,.14))`: .78 black at the bottom, but only .08–.14 across the top ~45%. That is sound while every title fits inside the bottom band, which is what `justify-content: flex-end` assumes. It does not hold for a three-line Anton title: 'Show Me Your Glory' is 165px tall in a 283px plate, so flex-end has no free space left to give and the first line starts 7% from the top. On `.img-concrete`, whose texture opens on a #c7c7c7 band, the white cap-height rows of 'SHOW' sit on a measured rgb(158,158,158) — 2.68:1 against a 3:1 large-text floor. 'The Theology of Staying on the Call' fails the same way at 2.92:1. Six of the eight live image plates pass (img-lines worst 3.69:1, img-noise worst 12.27:1), so this is texture-and-title-length dependent, not universal. MEASUREMENT: rasterised the homepage in headless Chrome at 1280 wide with the Earlier section unhidden, then sampled a glyph-free 12px strip inside each plate at each glyph row and took the row median — the computed-style probe reports 1.06:1 for all eight, which is the known .plate-image artifact and is why nine months of sweeps saw nothing. This is the second time that artifact has hidden a real defect (F100 was the first) and the first time it hid one in PRODUCTION rather than on /brand/. | 2026-09-11 re-verified live: plates.css?v=phase39 serving the .26/.34 scrim stops; .plate-image .plate-body display:flex / justify-content:flex-end on every image plate. 'Show Me Your Glory' (the three-line title that opened this row) sits at topFrac 0.067 where the scrim is ~.33 alpha — white on ~134 grey = ~3.6:1 against the 3:1 large-text floor. Fix holds. | 2026-09-26 re-verified live: 3 visible homepage .plate-image plates carry the 3-stop scrim (.78 -&gt; .26 @55% -&gt; .34 top); rasterised with headless system Chrome at 1280px and sampled glyph-free strips beside each title line — medians 3.95:1 (Show Me Your Glory, top line on the concrete band) to 11.73:1, all clear of the 3:1 large-text floor. | 2026-09-28: live: every .plate-image ::after = linear-gradient(to top, .78, .26 55%, .34) — the F101 scrim.</t>
+          <t>ISSUE/High (2026-09-06) — the scrim is `linear-gradient(to top, rgba(0,0,0,.78), rgba(0,0,0,.08) 55%, rgba(0,0,0,.14))`: .78 black at the bottom, but only .08–.14 across the top ~45%. That is sound while every title fits inside the bottom band, which is what `justify-content: flex-end` assumes. It does not hold for a three-line Anton title: 'Show Me Your Glory' is 165px tall in a 283px plate, so flex-end has no free space left to give and the first line starts 7% from the top. On `.img-concrete`, whose texture opens on a #c7c7c7 band, the white cap-height rows of 'SHOW' sit on a measured rgb(158,158,158) — 2.68:1 against a 3:1 large-text floor. 'The Theology of Staying on the Call' fails the same way at 2.92:1. Six of the eight live image plates pass (img-lines worst 3.69:1, img-noise worst 12.27:1), so this is texture-and-title-length dependent, not universal. MEASUREMENT: rasterised the homepage in headless Chrome at 1280 wide with the Earlier section unhidden, then sampled a glyph-free 12px strip inside each plate at each glyph row and took the row median — the computed-style probe reports 1.06:1 for all eight, which is the known .plate-image artifact and is why nine months of sweeps saw nothing. This is the second time that artifact has hidden a real defect (F100 was the first) and the first time it hid one in PRODUCTION rather than on /brand/. | 2026-09-11 re-verified live: plates.css?v=phase39 serving the .26/.34 scrim stops; .plate-image .plate-body display:flex / justify-content:flex-end on every image plate. 'Show Me Your Glory' (the three-line title that opened this row) sits at topFrac 0.067 where the scrim is ~.33 alpha — white on ~134 grey = ~3.6:1 against the 3:1 large-text floor. Fix holds. | 2026-09-26 re-verified live: 3 visible homepage .plate-image plates carry the 3-stop scrim (.78 -&gt; .26 @55% -&gt; .34 top); rasterised with headless system Chrome at 1280px and sampled glyph-free strips beside each title line — medians 3.95:1 (Show Me Your Glory, top line on the concrete band) to 11.73:1, all clear of the 3:1 large-text floor. | 2026-09-28: live: every .plate-image ::after = linear-gradient(to top, .78, .26 55%, .34) — the F101 scrim. | 2026-10-05: live: /brand/ scrim gradient carries the F101 values (.26 at 55%, .34 top); titles in the bottom band.</t>
         </is>
       </c>
       <c r="I104" s="6" t="inlineStr">
@@ -5999,7 +5999,7 @@
       </c>
       <c r="H105" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Low (2026-09-11) — the comment's choice 1 reads 'The linked call-to-action for the same essay is the IssueNext strip below the archive, which is what carries "Notify me →" to the coming-soon page.' That strip was deleted on 2026-08-27 in e3b4e91 under F94, along with 202 lines of its CSS. F94's own p4 already recorded the consequence — 'the upcoming essay's coming-soon page now has ZERO inbound links from the homepage' — but the component that states the trade-off was never updated, so the file explains a bargain whose other half is gone. No behavioural defect: the plate renders correctly and the row is graded Low because it only misleads a reader of the source. Found by grepping src/ for IssueNext after confirming the live homepage and both shipped sheets are clean of it (the three CSS mentions F94 catalogued are comments; this is a fourth mention F94 missed). | 2026-09-26 re-verified: GhostPlate.astro:16-24 records the IssueNext strip as retired 2026-08-27 (e3b4e91) [F94] and says where the decision lives — no dependency on a shipping component. | 2026-09-28: carried: GhostPlate comment unchanged.</t>
+          <t>ISSUE/Low (2026-09-11) — the comment's choice 1 reads 'The linked call-to-action for the same essay is the IssueNext strip below the archive, which is what carries "Notify me →" to the coming-soon page.' That strip was deleted on 2026-08-27 in e3b4e91 under F94, along with 202 lines of its CSS. F94's own p4 already recorded the consequence — 'the upcoming essay's coming-soon page now has ZERO inbound links from the homepage' — but the component that states the trade-off was never updated, so the file explains a bargain whose other half is gone. No behavioural defect: the plate renders correctly and the row is graded Low because it only misleads a reader of the source. Found by grepping src/ for IssueNext after confirming the live homepage and both shipped sheets are clean of it (the three CSS mentions F94 catalogued are comments; this is a fourth mention F94 missed). | 2026-09-26 re-verified: GhostPlate.astro:16-24 records the IssueNext strip as retired 2026-08-27 (e3b4e91) [F94] and says where the decision lives — no dependency on a shipping component. | 2026-09-28: carried: GhostPlate comment unchanged. | 2026-10-05: repo: GhostPlate.astro comment records IssueNext as retired.</t>
         </is>
       </c>
       <c r="I105" s="6" t="inlineStr">
@@ -6056,7 +6056,7 @@
       </c>
       <c r="H106" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Low (2026-09-11) — three references to the `.issue-next` strip survived its retirement (e3b4e91, 2026-08-27, F94): the homepage route description listed 'Issue-next ghost CTA' as part of the cascade; PAGES TO CRAWL told the crawler to follow article links from 'the homepage cascade or Issue-next ghost'; and §8 CONTENT COLLECTION INTEGRITY prescribed 'Issue-next ghost CTA's `.next-title` matches the referenced upcoming article's `&lt;title&gt;`'. The §8 line is the one that matters: `.next-title` cannot exist on any page the loop can reach, so that check can only ever be silently skipped — or, worse, reported as run. Graded Low because no site surface is affected and the two descriptive lines are merely stale; it is filed rather than fixed-in-passing because the operating prompt is what every future run executes. | 2026-09-26 re-verified: audit/QA-OS.md names .issue-next / .next-title only as retired (lines 103, 276-277, citing F94); no live check targets them. | 2026-09-28: carried: QA-OS.md unchanged.</t>
+          <t>ISSUE/Low (2026-09-11) — three references to the `.issue-next` strip survived its retirement (e3b4e91, 2026-08-27, F94): the homepage route description listed 'Issue-next ghost CTA' as part of the cascade; PAGES TO CRAWL told the crawler to follow article links from 'the homepage cascade or Issue-next ghost'; and §8 CONTENT COLLECTION INTEGRITY prescribed 'Issue-next ghost CTA's `.next-title` matches the referenced upcoming article's `&lt;title&gt;`'. The §8 line is the one that matters: `.next-title` cannot exist on any page the loop can reach, so that check can only ever be silently skipped — or, worse, reported as run. Graded Low because no site surface is affected and the two descriptive lines are merely stale; it is filed rather than fixed-in-passing because the operating prompt is what every future run executes. | 2026-09-26 re-verified: audit/QA-OS.md names .issue-next / .next-title only as retired (lines 103, 276-277, citing F94); no live check targets them. | 2026-09-28: carried: QA-OS.md unchanged. | 2026-10-05: repo: QA-OS.md names .issue-next only as retired [F94].</t>
         </is>
       </c>
       <c r="I106" s="6" t="inlineStr">
@@ -6113,7 +6113,7 @@
       </c>
       <c r="H107" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Low (2026-09-18) — §3 read 'Verify `--accent` usage on section-head h2, reading-progress bars, pull-quote borders.' Measured live on /words/the-weight-of-my-no/ in dark mode: `.reading-progress` background rgb(243,240,232) (--ink) and `.pull-quote` borders rgba(243,240,232,.82) (--border). Both are deliberate: the progress bar was recoloured from --accent to --ink in 68b0c1d (2026-04-10) with a comment at css/article.css:873 explaining the red bar competed with the masthead, and DESIGN-SYSTEM.md §4 lists pull-quote top/bottom borders as ordinary content borders while naming the .callout left border as the accent one. The check predates nothing — QA-OS was written 2026-08-07, four months after the recolour — so it has been either silently skipped or passed on assumption every run. Same class as F103: a dead check in the operating prompt. Graded Low: no site surface affected. | 2026-09-26 re-verified: QA-OS.md §3 (line 171-175) names section-head h2 + .callout as the accent's homes and records the reading-progress bar and pull-quote borders as by-design. Live spot-check agrees: /brand/ .section-head h2 = rgb(204,0,0), /words/the-stone/ .callout border-left = solid rgb(204,0,0). | 2026-09-28: carried: QA-OS.md unchanged.</t>
+          <t>ISSUE/Low (2026-09-18) — §3 read 'Verify `--accent` usage on section-head h2, reading-progress bars, pull-quote borders.' Measured live on /words/the-weight-of-my-no/ in dark mode: `.reading-progress` background rgb(243,240,232) (--ink) and `.pull-quote` borders rgba(243,240,232,.82) (--border). Both are deliberate: the progress bar was recoloured from --accent to --ink in 68b0c1d (2026-04-10) with a comment at css/article.css:873 explaining the red bar competed with the masthead, and DESIGN-SYSTEM.md §4 lists pull-quote top/bottom borders as ordinary content borders while naming the .callout left border as the accent one. The check predates nothing — QA-OS was written 2026-08-07, four months after the recolour — so it has been either silently skipped or passed on assumption every run. Same class as F103: a dead check in the operating prompt. Graded Low: no site surface affected. | 2026-09-26 re-verified: QA-OS.md §3 (line 171-175) names section-head h2 + .callout as the accent's homes and records the reading-progress bar and pull-quote borders as by-design. Live spot-check agrees: /brand/ .section-head h2 = rgb(204,0,0), /words/the-stone/ .callout border-left = solid rgb(204,0,0). | 2026-09-28: carried: QA-OS.md unchanged. | 2026-10-05: repo: §3 unchanged — accent homes + by-design exclusions intact.</t>
         </is>
       </c>
       <c r="I107" s="6" t="inlineStr">
@@ -6170,7 +6170,7 @@
       </c>
       <c r="H108" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-09-18) — every page (/, /about/, /brand/, /phase0/, /404, all /words/) carries a Netlify-injected `&lt;script async id="netlify-rum-container" src="/.netlify/scripts/rum"&gt;` with a CWV token for deploy 6aad063. The script beacons to https://ingesteer.services-prod.nsvcs.net/rum_collection, which the site's own CSP (`connect-src 'self'`, commented in netlify.toml as 'no analytics/beacons allowed') refuses. Result, reproduced on the homepage and on /words/the-weight-of-my-no/: two CSP violation errors plus an 'Uncaught (in promise) TypeError: Failed to fetch' from /.netlify/scripts/rum:1:11100. No reader-visible breakage — but it is a console error on every page view, and whatever Netlify observability panel this feeds is receiving nothing. The script was already present on 2026-09-11 (F102's p4 notes it in the live-vs-dist diff) while that run logged zero console errors, so either the beacon only fires on page hide / navigation (consistent with it arriving on navigate here) or the collector moved off-origin since; NEW to the ledger either way. Graded HIGH per the console-error rule. | 2026-09-19: still live, as expected — the connect-src fix sits on the unmerged qa/fixes-20260918 (carried into qa/fixes-20260919). Re-observed on /words/the-weight-of-my-no/: two connect-src violations against https://ingesteer.services-prod.nsvcs.net/rum_collection plus an uncaught 'Failed to fetch' from /.netlify/scripts/rum. Live CSP still reads connect-src 'self'. Not a regression; closes on merge. | 2026-09-28: live: 0 site console errors across 9 routes; RUM loads with no CSP violation.</t>
+          <t>ISSUE/High (2026-09-18) — every page (/, /about/, /brand/, /phase0/, /404, all /words/) carries a Netlify-injected `&lt;script async id="netlify-rum-container" src="/.netlify/scripts/rum"&gt;` with a CWV token for deploy 6aad063. The script beacons to https://ingesteer.services-prod.nsvcs.net/rum_collection, which the site's own CSP (`connect-src 'self'`, commented in netlify.toml as 'no analytics/beacons allowed') refuses. Result, reproduced on the homepage and on /words/the-weight-of-my-no/: two CSP violation errors plus an 'Uncaught (in promise) TypeError: Failed to fetch' from /.netlify/scripts/rum:1:11100. No reader-visible breakage — but it is a console error on every page view, and whatever Netlify observability panel this feeds is receiving nothing. The script was already present on 2026-09-11 (F102's p4 notes it in the live-vs-dist diff) while that run logged zero console errors, so either the beacon only fires on page hide / navigation (consistent with it arriving on navigate here) or the collector moved off-origin since; NEW to the ledger either way. Graded HIGH per the console-error rule. | 2026-09-19: still live, as expected — the connect-src fix sits on the unmerged qa/fixes-20260918 (carried into qa/fixes-20260919). Re-observed on /words/the-weight-of-my-no/: two connect-src violations against https://ingesteer.services-prod.nsvcs.net/rum_collection plus an uncaught 'Failed to fetch' from /.netlify/scripts/rum. Live CSP still reads connect-src 'self'. Not a regression; closes on merge. | 2026-09-28: live: 0 site console errors across 9 routes; RUM loads with no CSP violation. | 2026-10-05: live: 0 console errors on home/article/about/404/phase0/brand; RUM collector allowed in connect-src.</t>
         </is>
       </c>
       <c r="I108" s="6" t="inlineStr">
@@ -6227,7 +6227,7 @@
       </c>
       <c r="H109" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Low (2026-09-18) — index.astro:205 renders `&lt;RowHead label="This Week" variant="lead" /&gt;` unconditionally for the newest published essay; nothing compares the lead's publishedDate to the build date. Live today (Fri 2026-09-18) the row reads '01 This Week' over The Weight of My No, published 2026-08-31 — 18 days old. It read the same over Send Someone Else through most of August, when that essay was up to 57 days old. The daily rebuild (F73) would make a date-derived label accurate every morning at no cost. Filed Low: nothing breaks and it is not an a11y or SEO defect, but it is a false recency claim in the most prominent label on the page. | 2026-09-19: still live, as expected — homepage lead row head reads '01 THIS WEEK' over The Weight of My No (2026-08-31, now 19 days old); the 'Latest' fix sits on the unmerged qa/fixes-20260918. Closes on merge. | 2026-09-28: live: lead row label 'Latest'.</t>
+          <t>ISSUE/Low (2026-09-18) — index.astro:205 renders `&lt;RowHead label="This Week" variant="lead" /&gt;` unconditionally for the newest published essay; nothing compares the lead's publishedDate to the build date. Live today (Fri 2026-09-18) the row reads '01 This Week' over The Weight of My No, published 2026-08-31 — 18 days old. It read the same over Send Someone Else through most of August, when that essay was up to 57 days old. The daily rebuild (F73) would make a date-derived label accurate every morning at no cost. Filed Low: nothing breaks and it is not an a11y or SEO defect, but it is a false recency claim in the most prominent label on the page. | 2026-09-19: still live, as expected — homepage lead row head reads '01 THIS WEEK' over The Weight of My No (2026-08-31, now 19 days old); the 'Latest' fix sits on the unmerged qa/fixes-20260918. Closes on merge. | 2026-09-28: live: lead row label 'Latest'. | 2026-10-05: repo + live: lead row head reads "Latest".</t>
         </is>
       </c>
       <c r="I109" s="6" t="inlineStr">
@@ -6284,7 +6284,7 @@
       </c>
       <c r="H110" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Low (2026-09-22) — §9 named no method for F57, so this run tested it with a burst chained onto the subscribe smoke test: 8 POSTs returned 8 x 200 and no 429 (one returned HTTP 000, an instance churn tell), which reads as a dead limiter. A clean sequential re-run returned exactly 5 x 400 then 5 x 429; a parallel re-run returned 10 x 400 and no 429. The limiter is correct; the prompt lacked the method, and the false reading cost two test cycles. Same class as F103/F104. | 2026-09-27 re-verified against the file: QA-OS.md §9 still carries the sequential 10-POST method (5 x 400 then 5 x 429) and the MEASUREMENT ANTIPATTERNS fan-out entry. | 2026-09-28: carried: QA-OS.md §9 unchanged; method used today (see F57).</t>
+          <t>ISSUE/Low (2026-09-22) — §9 named no method for F57, so this run tested it with a burst chained onto the subscribe smoke test: 8 POSTs returned 8 x 200 and no 429 (one returned HTTP 000, an instance churn tell), which reads as a dead limiter. A clean sequential re-run returned exactly 5 x 400 then 5 x 429; a parallel re-run returned 10 x 400 and no 429. The limiter is correct; the prompt lacked the method, and the false reading cost two test cycles. Same class as F103/F104. | 2026-09-27 re-verified against the file: QA-OS.md §9 still carries the sequential 10-POST method (5 x 400 then 5 x 429) and the MEASUREMENT ANTIPATTERNS fan-out entry. | 2026-09-28: carried: QA-OS.md §9 unchanged; method used today (see F57). | 2026-10-05: repo: §9 method intact; today's run followed it (5 x 400 then 5 x 429).</t>
         </is>
       </c>
       <c r="I110" s="6" t="inlineStr">
@@ -6341,7 +6341,7 @@
       </c>
       <c r="H111" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/High (2026-09-24) — .rail-cta's base rule is background: var(--ink); color: var(--bg), and a.plate-lead:hover .rail-cta swaps only the background to var(--accent). In light mode that is cream on #c00 (#f4f4f1, ~5.2:1, passes). In dark mode --bg is #060606, so the hovered chip renders near-black 'READ →' on #c00 at 3.44:1 at 12px/700, under the 4.5:1 floor (WCAG 1.4.3). Measured under a REAL pointer hover after a 3s settle (a.plate-lead:hover true; computed rgb(6,6,6) on rgb(204,0,0)) and confirmed on screenshot. It is the same defect class F83 closed for .latest-cta and .hero-link.primary on 2026-08-13; F83's scope note said only those two controls invert onto the fill, which missed this third one. Present since the lead plate shipped (d1f8e7e, 2026-04-21), so NEW to the ledger, not a regression. /brand/ renders .plate-lead and loads home-augment.css, so it carries the same defect. | 2026-09-25: still present LIVE — live home-augment.css is phase34 without the rule; fix sits on the unmerged stacked branch (now qa/fixes-20260925). Awaiting Dexter's merge; not re-counted as new. | 2026-09-28: still present LIVE — real pointer hover, dark mode, 3s settle: .rail-cta rgb(6,6,6) on rgb(204,0,0) = 3.44:1 (screenshot). A 1s read caught the chip mid-transition on --ink; re-measured before concluding. Awaiting Dexter's merge; not re-counted as new. | 2026-09-29: still present LIVE — real pointer hover, dark mode (real toggle click, 2s settle), 3s hover settle: .rail-cta rgb(6,6,6) on rgb(204,0,0) = 3.44:1 (screenshot). Awaiting Dexter's merge; not re-counted as new.</t>
+          <t>ISSUE/High (2026-09-24) — .rail-cta's base rule is background: var(--ink); color: var(--bg), and a.plate-lead:hover .rail-cta swaps only the background to var(--accent). In light mode that is cream on #c00 (#f4f4f1, ~5.2:1, passes). In dark mode --bg is #060606, so the hovered chip renders near-black 'READ →' on #c00 at 3.44:1 at 12px/700, under the 4.5:1 floor (WCAG 1.4.3). Measured under a REAL pointer hover after a 3s settle (a.plate-lead:hover true; computed rgb(6,6,6) on rgb(204,0,0)) and confirmed on screenshot. It is the same defect class F83 closed for .latest-cta and .hero-link.primary on 2026-08-13; F83's scope note said only those two controls invert onto the fill, which missed this third one. Present since the lead plate shipped (d1f8e7e, 2026-04-21), so NEW to the ledger, not a regression. /brand/ renders .plate-lead and loads home-augment.css, so it carries the same defect. | 2026-09-25: still present LIVE — live home-augment.css is phase34 without the rule; fix sits on the unmerged stacked branch (now qa/fixes-20260925). Awaiting Dexter's merge; not re-counted as new. | 2026-09-28: still present LIVE — real pointer hover, dark mode, 3s settle: .rail-cta rgb(6,6,6) on rgb(204,0,0) = 3.44:1 (screenshot). A 1s read caught the chip mid-transition on --ink; re-measured before concluding. Awaiting Dexter's merge; not re-counted as new. | 2026-09-29: still present LIVE — real pointer hover, dark mode (real toggle click, 2s settle), 3s hover settle: .rail-cta rgb(6,6,6) on rgb(204,0,0) = 3.44:1 (screenshot). Awaiting Dexter's merge; not re-counted as new. | 2026-10-05: live: real pointer hover in dark mode; with transitions neutralised via insertRule, .rail-cta = rgb(243,240,232) on rgb(204,0,0) = 5.17:1. The first unneutralised read (1.00:1) was the hidden-pane transition freeze — now in QA-OS antipatterns.</t>
         </is>
       </c>
       <c r="I111" s="6" t="inlineStr">
@@ -6360,8 +6360,65 @@
         </is>
       </c>
     </row>
+    <row r="112">
+      <c r="A112" s="4" t="inlineStr">
+        <is>
+          <t>F109</t>
+        </is>
+      </c>
+      <c r="B112" s="4" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="C112" s="4" t="inlineStr">
+        <is>
+          <t>Backward-nav stitch completeness across the essay chain (prev mirrors next)</t>
+        </is>
+      </c>
+      <c r="D112" s="4" t="inlineStr">
+        <is>
+          <t>As a reader working backward through the essays, I want "Previous Essay" (and rel=prev) to take me to the essay published just before this one, so I never skip pieces.</t>
+        </is>
+      </c>
+      <c r="E112" s="4" t="inlineStr">
+        <is>
+          <t>Every entry except the chronologically oldest published essay carries prev{slug,title} == its chronological predecessor, and the title matches that entry's title frontmatter. Mirror of F81 (forward). Violation = the reader silently skips essays going backward and rel=prev points at the wrong page.</t>
+        </is>
+      </c>
+      <c r="F112" s="4" t="inlineStr">
+        <is>
+          <t>src/content/words/*.mdx (prev frontmatter), src/layouts/ArticleLayout.astro:123,195-198</t>
+        </is>
+      </c>
+      <c r="G112" s="6" t="inlineStr">
+        <is>
+          <t>Cataloged 2026-10-05 (full-regression chain audit)</t>
+        </is>
+      </c>
+      <c r="H112" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE/Medium (2026-10-05) — /words/send-someone-else/ (Jul 5) had prev: "some" (May 22), so its "Previous Essay" card and &lt;link rel="prev"&gt; skipped four essays: Not the Same as Alive, Music That Raised Me, Outsourced Faith, Show Me Your Glory. The forward chain was fine (show-me-your-glory -&gt; send-someone-else). The mistake was there when the essay was added in d38ffba (2026-07-02); outsourced-faith (Jun 14) was already live then. The F81 forward stitch (d539b0f) fixed the other direction only. A repo audit of all 17 prev links found this one mismatch.</t>
+        </is>
+      </c>
+      <c r="I112" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J112" s="4" t="inlineStr">
+        <is>
+          <t>FIX (qa/fixes-20261005 c0479c8): src/content/words/send-someone-else.mdx prev -&gt; {slug: "show-me-your-glory", title: "Show Me Your Glory"}. Nav frontmatter only; no copy touched (the F81 precedent). The stale next.ghost: true is left alone: nextLive already neutralises it (F41).</t>
+        </is>
+      </c>
+      <c r="K112" s="6" t="inlineStr">
+        <is>
+          <t>PASS (verified against build) — 2026-10-05. npm run build passes (20 pages); dist send-someone-else emits &lt;link rel="prev" href=".../show-me-your-glory/"&gt; and a "Previous Essay: Show Me Your Glory" card. Whole-chain walk of dist: 17/17 prev and next match chronological order, 0 mismatches. Goes live-verified on the first scrub after the merge.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:K111"/>
+  <autoFilter ref="A3:K112"/>
   <mergeCells count="2">
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A1:K1"/>
@@ -6431,7 +6488,7 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9">
@@ -6468,7 +6525,7 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -6478,7 +6535,7 @@
         </is>
       </c>
       <c r="B15" s="10" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16">
@@ -6494,7 +6551,7 @@
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>Total features: 108</t>
+          <t>Total features: 109</t>
         </is>
       </c>
     </row>

</xml_diff>